<commit_message>
Refresh dashboards after fixing NaN login attribution on today's local pull
42818 (T&D V2 Live) traded today (last 19:31 ET) but was hidden by the
NaN-login bug. Other live accounts (32983, 657902) genuinely haven't
traded since 5/12 and 5/15 — that's the EA, not a data gap.

Triggered by: 215 rows from today's local raw pull (extraction_batch
20260518_213406) all had NaN login because consolidate.py's
add_login_column hadn't run on them. --full-rebuild fixed it; all
122,850 rows now have a non-NaN login.
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -1325,7 +1325,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>T&amp;D Low Drawdown | AUDUSD.pro, T&amp;D Low Drawdown | EURUSD.pro, T&amp;D Low Drawdown | GBPUSD.pro, T&amp;D Low Drawdown | NZDUSD.pro, T&amp;D Low Drawdown | USDCAD.pro, T&amp;D Low Drawdown | USDJPY.pro</t>
+          <t>T&amp;D Low Drawdown | AUDUSD.pro, T&amp;D Low Drawdown | EURUSD.pro, T&amp;D Low Drawdown | GBPUSD.pro, T&amp;D Low Drawdown | NZDUSD.pro, T&amp;D Low Drawdown | USDCAD.pro, T&amp;D Low Drawdown | USDJPY.pro, T&amp;D60 | AUDUSD.pro, T&amp;D60 | EURUSD.pro, T&amp;D60 | GBPUSD.pro, T&amp;D60 | NZDUSD.pro, T&amp;D60 | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Unknown | USDJPY</t>
+          <t>T&amp;D19 V2 USDJPY MOL | USDJPY</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>MOL Breakout BothWays (retired) | AUDUSD.pro, MOL Breakout BothWays (retired) | EURUSD.pro, MOL Breakout BothWays (retired) | GBPUSD.pro, T&amp;D 60 | AUDUSD.pro, T&amp;D 60 | EURUSD.pro, T&amp;D 60 | GBPUSD.pro, T&amp;D 60 | USDCAD.pro, T&amp;D 60 | USDJPY.pro</t>
+          <t>MOL Breakout BothWays (retired) | AUDUSD.pro, MOL Breakout BothWays (retired) | EURUSD.pro, MOL Breakout BothWays (retired) | GBPUSD.pro, T&amp;D V2 Live | AUDUSD.pro, T&amp;D V2 Live | EURUSD.pro, T&amp;D V2 Live | GBPUSD.pro, T&amp;D V2 Live | USDCAD.pro, T&amp;D V2 Live | USDJPY.pro</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboards — 2026-06-02
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1051,11 +1051,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/01/2026 01:53</t>
+          <t>06/02/2026 01:35</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
-        <v>31858.34</v>
+        <v>25000.04</v>
       </c>
       <c r="I3" s="7" t="n">
         <v>20.51</v>
@@ -1069,26 +1069,26 @@
       <c r="L3" s="7" t="n">
         <v>30545.04</v>
       </c>
-      <c r="M3" t="n">
-        <v>0</v>
+      <c r="M3" s="7" t="n">
+        <v>6858.3</v>
       </c>
       <c r="N3" t="n">
         <v>40</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>574.5600000000001</v>
+        <v>-6388.81</v>
       </c>
       <c r="P3" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="Q3" s="7" t="n">
-        <v>67.5</v>
+        <v>65</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>1.379362524146813</v>
+        <v>0.2421837290311843</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>7.182286439297812</v>
+        <v>65.81687632519494</v>
       </c>
       <c r="T3" t="n">
         <v>865</v>
@@ -1229,17 +1229,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>41651</t>
+          <t>39479</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>T&amp;D60</t>
+          <t>T&amp;D19 V2 USDJPY PROP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS153</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -1257,32 +1257,32 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>05/31/2026 20:38</t>
+          <t>10/03/2025 00:48</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
-        <v>17387.1</v>
+        <v>34219.5</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>-59.08</v>
+        <v>0.03</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>60.59</v>
+        <v>12.87</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>0.54</v>
+        <v>0.89</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>30587.87</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
+        <v>36046.71</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>627.79</v>
       </c>
       <c r="N5" t="n">
         <v>40</v>
       </c>
       <c r="O5" s="7" t="n">
-        <v>-144.47</v>
+        <v>58.28</v>
       </c>
       <c r="P5" t="n">
         <v>31</v>
@@ -1291,48 +1291,48 @@
         <v>77.5</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>0.7636095884807331</v>
+        <v>2.573611111111111</v>
       </c>
       <c r="S5" s="7" t="n">
-        <v>3.807157738240804</v>
+        <v>0.1587531959394289</v>
       </c>
       <c r="T5" t="n">
-        <v>602</v>
+        <v>2</v>
       </c>
       <c r="U5" s="7" t="n">
-        <v>-3642.179999999999</v>
+        <v>8.690000000000001</v>
       </c>
       <c r="V5" t="n">
-        <v>502</v>
+        <v>2</v>
       </c>
       <c r="W5" s="7" t="n">
-        <v>83.38870431893687</v>
+        <v>100</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>T&amp;D Low Drawdown | AUDUSD.pro, T&amp;D Low Drawdown | EURUSD.pro, T&amp;D Low Drawdown | GBPUSD.pro, T&amp;D Low Drawdown | NZDUSD.pro, T&amp;D Low Drawdown | USDCAD.pro, T&amp;D Low Drawdown | USDJPY.pro, T&amp;D60 | AUDUSD.pro, T&amp;D60 | EURUSD.pro, T&amp;D60 | GBPUSD.pro, T&amp;D60 | NZDUSD.pro, T&amp;D60 | USDJPY.pro</t>
+          <t>T&amp;D19 V2 USDJPY PROP | USDJPY</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>41653</t>
+          <t>41651</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>T&amp;D1 High Returns</t>
+          <t>T&amp;D60</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1360,23 +1360,23 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2026 03:52</t>
+          <t>05/31/2026 20:38</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
-        <v>7844.03</v>
+        <v>17387.1</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>-60.74</v>
+        <v>-59.08</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>68.69</v>
+        <v>60.59</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="L6" t="n">
-        <v>20000</v>
+        <v>0.54</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>30587.87</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
@@ -1385,35 +1385,35 @@
         <v>40</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>-884.63</v>
+        <v>-144.47</v>
       </c>
       <c r="P6" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Q6" s="7" t="n">
-        <v>80</v>
+        <v>77.5</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>0.4523228746192516</v>
+        <v>0.7636095884807331</v>
       </c>
       <c r="S6" s="7" t="n">
-        <v>11.64757883716346</v>
+        <v>3.807157738240804</v>
       </c>
       <c r="T6" t="n">
-        <v>668</v>
+        <v>602</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>-12090.23</v>
+        <v>-3642.179999999999</v>
       </c>
       <c r="V6" t="n">
-        <v>563</v>
+        <v>502</v>
       </c>
       <c r="W6" s="7" t="n">
-        <v>84.28143712574851</v>
+        <v>83.38870431893687</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2025-10-27</t>
+          <t>2025-10-23</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1428,14 +1428,14 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>T&amp;D1 High Returns | AUDUSD.pro, T&amp;D1 High Returns | EURUSD.pro, T&amp;D1 High Returns | GBPUSD.pro, T&amp;D1 High Returns | NZDUSD.pro, T&amp;D1 High Returns | USDCAD.pro, T&amp;D1 High Returns | USDJPY.pro</t>
+          <t>T&amp;D Low Drawdown | AUDUSD.pro, T&amp;D Low Drawdown | EURUSD.pro, T&amp;D Low Drawdown | GBPUSD.pro, T&amp;D Low Drawdown | NZDUSD.pro, T&amp;D Low Drawdown | USDCAD.pro, T&amp;D Low Drawdown | USDJPY.pro, T&amp;D60 | AUDUSD.pro, T&amp;D60 | EURUSD.pro, T&amp;D60 | GBPUSD.pro, T&amp;D60 | NZDUSD.pro, T&amp;D60 | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>41654</t>
+          <t>41653</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>T&amp;D1 Prop Firm</t>
+          <t>T&amp;D1 High Returns</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1463,20 +1463,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2026 19:27</t>
+          <t>06/01/2026 03:52</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
-        <v>19826.86</v>
+        <v>7844.03</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>-0.82</v>
+        <v>-60.74</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>7.64</v>
+        <v>68.69</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>0.95</v>
+        <v>0.72</v>
       </c>
       <c r="L7" t="n">
         <v>20000</v>
@@ -1488,35 +1488,35 @@
         <v>40</v>
       </c>
       <c r="O7" s="7" t="n">
-        <v>201.77</v>
+        <v>-884.63</v>
       </c>
       <c r="P7" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="Q7" s="7" t="n">
-        <v>87.5</v>
+        <v>80</v>
       </c>
       <c r="R7" s="7" t="n">
-        <v>1.488476250423667</v>
+        <v>0.4523228746192516</v>
       </c>
       <c r="S7" s="7" t="n">
-        <v>1.53011087488554</v>
+        <v>11.64757883716346</v>
       </c>
       <c r="T7" t="n">
-        <v>294</v>
+        <v>668</v>
       </c>
       <c r="U7" s="7" t="n">
-        <v>-173.14</v>
+        <v>-12090.23</v>
       </c>
       <c r="V7" t="n">
-        <v>263</v>
+        <v>563</v>
       </c>
       <c r="W7" s="7" t="n">
-        <v>89.45578231292517</v>
+        <v>84.28143712574851</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>2025-10-27</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1531,14 +1531,14 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>T&amp;D1 Prop Firm | EURUSD.pro, T&amp;D1 Prop Firm | USDJPY.pro</t>
+          <t>T&amp;D1 High Returns | AUDUSD.pro, T&amp;D1 High Returns | EURUSD.pro, T&amp;D1 High Returns | GBPUSD.pro, T&amp;D1 High Returns | NZDUSD.pro, T&amp;D1 High Returns | USDCAD.pro, T&amp;D1 High Returns | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>41655</t>
+          <t>41654</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Axis Rotation V2</t>
+          <t>T&amp;D1 Prop Firm</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -1566,20 +1566,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2026 04:56</t>
+          <t>06/01/2026 19:27</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
-        <v>18415.42</v>
+        <v>19826.86</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>-6.5</v>
+        <v>-0.82</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>23.63</v>
+        <v>7.64</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L8" t="n">
         <v>20000</v>
@@ -1591,40 +1591,40 @@
         <v>40</v>
       </c>
       <c r="O8" s="7" t="n">
-        <v>157.39</v>
+        <v>201.77</v>
       </c>
       <c r="P8" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="Q8" s="7" t="n">
-        <v>45</v>
+        <v>87.5</v>
       </c>
       <c r="R8" s="7" t="n">
-        <v>1.083458935958695</v>
+        <v>1.488476250423667</v>
       </c>
       <c r="S8" s="7" t="n">
-        <v>8.214877771782222</v>
+        <v>1.53011087488554</v>
       </c>
       <c r="T8" t="n">
-        <v>447</v>
+        <v>294</v>
       </c>
       <c r="U8" s="7" t="n">
-        <v>-1584.58</v>
+        <v>-173.14</v>
       </c>
       <c r="V8" t="n">
-        <v>204</v>
+        <v>263</v>
       </c>
       <c r="W8" s="7" t="n">
-        <v>45.63758389261745</v>
+        <v>89.45578231292517</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2025-11-04</t>
+          <t>2025-11-06</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -1634,14 +1634,14 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Axis Rotation V2 | AUDUSD.pro, Axis Rotation V2 | EURUSD.pro, Axis Rotation V2 | GBPUSD.pro, Axis Rotation V2 | USDCAD.pro, Axis Rotation V2 | USDJPY.pro</t>
+          <t>T&amp;D1 Prop Firm | EURUSD.pro, T&amp;D1 Prop Firm | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>41657</t>
+          <t>41655</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Axis Rotation V1</t>
+          <t>Axis Rotation V2</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1669,20 +1669,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>05/24/2026 19:35</t>
+          <t>06/01/2026 04:56</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
-        <v>20376.02</v>
+        <v>18415.42</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>1.83</v>
+        <v>-6.5</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>9.18</v>
+        <v>23.63</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1.03</v>
+        <v>0.96</v>
       </c>
       <c r="L9" t="n">
         <v>20000</v>
@@ -1694,31 +1694,31 @@
         <v>40</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>-570.4399999999999</v>
+        <v>157.39</v>
       </c>
       <c r="P9" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q9" s="7" t="n">
-        <v>37.5</v>
+        <v>45</v>
       </c>
       <c r="R9" s="7" t="n">
-        <v>0.8207764882691826</v>
+        <v>1.083458935958695</v>
       </c>
       <c r="S9" s="7" t="n">
-        <v>13.82284951966541</v>
+        <v>8.214877771782222</v>
       </c>
       <c r="T9" t="n">
-        <v>183</v>
+        <v>447</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>216.0199999999997</v>
+        <v>-1584.58</v>
       </c>
       <c r="V9" t="n">
-        <v>84</v>
+        <v>204</v>
       </c>
       <c r="W9" s="7" t="n">
-        <v>45.90163934426229</v>
+        <v>45.63758389261745</v>
       </c>
       <c r="X9" t="inlineStr">
         <is>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
@@ -1737,14 +1737,14 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Axis Rotation V1 | EURUSD.pro, Axis Rotation V1 | GBPUSD.pro</t>
+          <t>Axis Rotation V2 | AUDUSD.pro, Axis Rotation V2 | EURUSD.pro, Axis Rotation V2 | GBPUSD.pro, Axis Rotation V2 | USDCAD.pro, Axis Rotation V2 | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>41658</t>
+          <t>41657</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Agg Univ</t>
+          <t>Axis Rotation V1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -1772,20 +1772,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/01/2026 12:43</t>
+          <t>05/24/2026 19:35</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
-        <v>18678.13</v>
+        <v>20376.02</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>-6.62</v>
+        <v>1.83</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>7.93</v>
+        <v>9.18</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.03</v>
       </c>
       <c r="L10" t="n">
         <v>20000</v>
@@ -1797,67 +1797,67 @@
         <v>40</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>-1060.61</v>
+        <v>-570.4399999999999</v>
       </c>
       <c r="P10" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q10" s="7" t="n">
-        <v>30</v>
+        <v>37.5</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>0.4218233948115678</v>
+        <v>0.8207764882691826</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>12.87413289157481</v>
+        <v>13.82284951966541</v>
       </c>
       <c r="T10" t="n">
-        <v>4</v>
+        <v>183</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>-31.6</v>
+        <v>216.0199999999997</v>
       </c>
       <c r="V10" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>25</v>
+        <v>45.90163934426229</v>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2025-11-04</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Agg Univ | AUDUSD.pro, Agg Univ | GBPUSD.pro, Agg Univ | USDCAD.pro, Agg Univ | USDCHF.pro</t>
+          <t>Axis Rotation V1 | EURUSD.pro, Axis Rotation V1 | GBPUSD.pro</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>42817</t>
+          <t>41658</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>T&amp;D19 V2 USDJPY MOL</t>
+          <t>Agg Univ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -1875,65 +1875,65 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>05/31/2026 18:56</t>
+          <t>06/01/2026 12:43</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
-        <v>10529.39</v>
+        <v>18678.13</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>4.58</v>
+        <v>-6.62</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>1.25</v>
+        <v>7.93</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>3.56</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L11" t="n">
         <v>20000</v>
       </c>
-      <c r="M11" s="7" t="n">
-        <v>9933.5</v>
+      <c r="M11" t="n">
+        <v>0</v>
       </c>
       <c r="N11" t="n">
         <v>40</v>
       </c>
       <c r="O11" s="7" t="n">
-        <v>534.3</v>
+        <v>-1060.61</v>
       </c>
       <c r="P11" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="Q11" s="7" t="n">
-        <v>67.5</v>
+        <v>30</v>
       </c>
       <c r="R11" s="7" t="n">
-        <v>1.058394712217804</v>
+        <v>0.4218233948115678</v>
       </c>
       <c r="S11" s="7" t="n">
-        <v>44.59199544555984</v>
+        <v>12.87413289157481</v>
       </c>
       <c r="T11" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="U11" s="7" t="n">
-        <v>538.21</v>
+        <v>-31.6</v>
       </c>
       <c r="V11" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="W11" s="7" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
@@ -1943,14 +1943,14 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>T&amp;D19 V2 USDJPY MOL | USDJPY</t>
+          <t>Agg Univ | AUDUSD.pro, Agg Univ | GBPUSD.pro, Agg Univ | USDCAD.pro, Agg Univ | USDCHF.pro</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>42818</t>
+          <t>42817</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>T&amp;D60</t>
+          <t>T&amp;D19 V2 USDJPY MOL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1974,69 +1974,69 @@
         </is>
       </c>
       <c r="F12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/01/2026 14:06</t>
+          <t>05/31/2026 18:56</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>4726.13</v>
+        <v>10529.39</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>-5.47</v>
+        <v>4.58</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>9.470000000000001</v>
+        <v>1.25</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>0.86</v>
+        <v>3.56</v>
       </c>
       <c r="L12" t="n">
-        <v>5010</v>
-      </c>
-      <c r="M12" t="n">
-        <v>10</v>
+        <v>20000</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>9933.5</v>
       </c>
       <c r="N12" t="n">
         <v>40</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>-58.88</v>
+        <v>534.3</v>
       </c>
       <c r="P12" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>82.5</v>
+        <v>67.5</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>0.8621529240998268</v>
+        <v>1.058394712217804</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>2.341150941280393</v>
+        <v>44.59199544555984</v>
       </c>
       <c r="T12" t="n">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>-79.45999999999997</v>
+        <v>538.21</v>
       </c>
       <c r="V12" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="W12" s="7" t="n">
-        <v>81.57894736842105</v>
+        <v>100</v>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -2046,14 +2046,14 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>T&amp;D60 | EURUSD.pro, T&amp;D60 | GBPUSD.pro, T&amp;D60 | USDCAD.pro, T&amp;D60 | USDJPY.pro</t>
+          <t>T&amp;D19 V2 USDJPY MOL | USDJPY</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>45215</t>
+          <t>42818</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Axis GBPUSD</t>
+          <t>T&amp;D60</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2073,100 +2073,100 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS153</t>
         </is>
       </c>
       <c r="F13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/02/2026 01:00</t>
+          <t>06/01/2026 14:06</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>19996.4</v>
+        <v>4726.13</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>-5.21</v>
+        <v>-5.47</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>9.75</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="L13" s="7" t="n">
-        <v>26775.1</v>
+        <v>0.86</v>
+      </c>
+      <c r="L13" t="n">
+        <v>5010</v>
       </c>
       <c r="M13" t="n">
-        <v>6000</v>
+        <v>10</v>
       </c>
       <c r="N13" t="n">
         <v>40</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>5678.17</v>
+        <v>-58.88</v>
       </c>
       <c r="P13" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>82.5</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>1.840525317241257</v>
+        <v>0.8621529240998268</v>
       </c>
       <c r="S13" s="7" t="n">
-        <v>27.67771200973612</v>
+        <v>2.341150941280393</v>
       </c>
       <c r="T13" t="n">
-        <v>131</v>
+        <v>38</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>158.4200000000002</v>
+        <v>-79.45999999999997</v>
       </c>
       <c r="V13" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>57.25190839694656</v>
+        <v>81.57894736842105</v>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Axis Rotation GBPUSD 5m V1 | GBPUSD, EA Axis Rotation EURUSD 5m 8%dd | EURUSD</t>
+          <t>T&amp;D60 | EURUSD.pro, T&amp;D60 | GBPUSD.pro, T&amp;D60 | USDCAD.pro, T&amp;D60 | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>50347</t>
+          <t>45215</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Breakout Engine</t>
+          <t>Axis GBPUSD</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92t2</t>
         </is>
       </c>
       <c r="F14" t="b">
@@ -2184,60 +2184,60 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>06/01/2026 10:11</t>
+          <t>06/02/2026 01:00</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>18120.08</v>
+        <v>19996.4</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>-9.42</v>
+        <v>-5.21</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>11.07</v>
+        <v>9.75</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="L14" t="n">
-        <v>20000</v>
+        <v>0.85</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>26775.1</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="N14" t="n">
         <v>40</v>
       </c>
       <c r="O14" s="7" t="n">
-        <v>-1399.82</v>
+        <v>5678.17</v>
       </c>
       <c r="P14" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>40</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>0.6403896732491465</v>
+        <v>1.840525317241257</v>
       </c>
       <c r="S14" s="7" t="n">
-        <v>14.04210000000003</v>
+        <v>27.67771200973612</v>
       </c>
       <c r="T14" t="n">
-        <v>102</v>
+        <v>131</v>
       </c>
       <c r="U14" s="7" t="n">
-        <v>-1879.920000000001</v>
+        <v>158.4200000000002</v>
       </c>
       <c r="V14" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>44.11764705882353</v>
+        <v>57.25190839694656</v>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -2252,14 +2252,14 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Breakout Engine | BTCUSD, Breakout Engine | XAUUSD</t>
+          <t>Axis Rotation GBPUSD 5m V1 | GBPUSD, EA Axis Rotation EURUSD 5m 8%dd | EURUSD</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>50348</t>
+          <t>50347</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Aggressive V1 Pro</t>
+          <t>Breakout Engine</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2287,23 +2287,23 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/01/2026 07:19</t>
+          <t>06/01/2026 10:11</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>11607.19</v>
+        <v>18120.08</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-96.40000000000001</v>
+        <v>-9.42</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>96.58</v>
+        <v>11.07</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>0.76</v>
+        <v>0.8</v>
       </c>
       <c r="L15" t="n">
-        <v>45165</v>
+        <v>20000</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
@@ -2312,40 +2312,40 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>-389.2699999999999</v>
+        <v>-1399.82</v>
       </c>
       <c r="P15" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>0.9067654403853558</v>
+        <v>0.6403896732491465</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>9.73899224894088</v>
+        <v>14.04210000000003</v>
       </c>
       <c r="T15" t="n">
-        <v>3664</v>
+        <v>102</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-34589.11</v>
+        <v>-1879.920000000001</v>
       </c>
       <c r="V15" t="n">
-        <v>1988</v>
+        <v>45</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>54.25764192139738</v>
+        <v>44.11764705882353</v>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2355,14 +2355,14 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Aggressive V1 Pro | EURUSD, Aggressive V1 Pro | GBPJPY, Aggressive V1 Pro | GBPUSD, Aggressive V1 Pro | USDCHF, Aggressive V1 Pro | USDJPY, Aggressive V1 Pro | XAUUSD</t>
+          <t>Breakout Engine | BTCUSD, Breakout Engine | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>51718</t>
+          <t>50348</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hive V5 HTF (prop)</t>
+          <t>Aggressive V1 Pro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2390,23 +2390,23 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>05/31/2026 03:31</t>
+          <t>06/01/2026 07:19</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>14113.73</v>
+        <v>11607.19</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-29.46</v>
+        <v>-96.40000000000001</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>29.46</v>
+        <v>96.58</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.34</v>
+        <v>0.76</v>
       </c>
       <c r="L16" t="n">
-        <v>20000</v>
+        <v>45165</v>
       </c>
       <c r="M16" t="n">
         <v>0</v>
@@ -2415,40 +2415,40 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-885.64</v>
+        <v>-389.2699999999999</v>
       </c>
       <c r="P16" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.06609583263033575</v>
+        <v>0.9067654403853558</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>8.856399999999995</v>
+        <v>9.73899224894088</v>
       </c>
       <c r="T16" t="n">
-        <v>324</v>
+        <v>3664</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-6193.83</v>
+        <v>-34589.11</v>
       </c>
       <c r="V16" t="n">
-        <v>46</v>
+        <v>1988</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>14.19753086419753</v>
+        <v>54.25764192139738</v>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
@@ -2458,14 +2458,14 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>Hive V5 HTF (prop) | AUDJPY.pro, Hive V5 HTF (prop) | AUDUSD.pro, Hive V5 HTF (prop) | BTCUSD, Hive V5 HTF (prop) | CADJPY.pro, Hive V5 HTF (prop) | CHFJPY.pro, Hive V5 HTF (prop) | EURJPY.pro, Hive V5 HTF (prop) | EURUSD.pro, Hive V5 HTF (prop) | GBPJPY.pro, Hive V5 HTF (prop) | GBPUSD.pro, Hive V5 HTF (prop) | USDJPY.pro</t>
+          <t>Aggressive V1 Pro | EURUSD, Aggressive V1 Pro | GBPJPY, Aggressive V1 Pro | GBPUSD, Aggressive V1 Pro | USDCHF, Aggressive V1 Pro | USDJPY, Aggressive V1 Pro | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>51720</t>
+          <t>51718</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Hive V3 Forex HTF MOL</t>
+          <t>Hive V5 HTF (prop)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2493,20 +2493,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>06/01/2026 22:16</t>
+          <t>05/31/2026 03:31</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>17107.57</v>
+        <v>14113.73</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>-14.47</v>
+        <v>-29.46</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>15.5</v>
+        <v>29.46</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>0.58</v>
+        <v>0.34</v>
       </c>
       <c r="L17" t="n">
         <v>20000</v>
@@ -2518,40 +2518,40 @@
         <v>40</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>-1334.54</v>
+        <v>-885.64</v>
       </c>
       <c r="P17" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="7" t="n">
-        <v>17.5</v>
+        <v>5</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>0.2207702727952168</v>
+        <v>0.06609583263033575</v>
       </c>
       <c r="S17" s="7" t="n">
-        <v>13.34540000000001</v>
+        <v>8.856399999999995</v>
       </c>
       <c r="T17" t="n">
-        <v>161</v>
+        <v>324</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>-1626.74</v>
+        <v>-6193.83</v>
       </c>
       <c r="V17" t="n">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="W17" s="7" t="n">
-        <v>39.75155279503105</v>
+        <v>14.19753086419753</v>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -2561,14 +2561,14 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>Hive V3 Forex HTF MOL | AUDJPY.pro, Hive V3 Forex HTF MOL | AUDUSD.pro, Hive V3 Forex HTF MOL | CADJPY.pro, Hive V3 Forex HTF MOL | CHFJPY.pro, Hive V3 Forex HTF MOL | EURCAD.pro, Hive V3 Forex HTF MOL | EURUSD.pro, Hive V3 Forex HTF MOL | GBPJPY.pro, Hive V3 Forex HTF MOL | GBPUSD.pro, Hive V3 Forex HTF MOL | USDCAD.pro, Hive V3 Forex HTF MOL | USDJPY.pro</t>
+          <t>Hive V5 HTF (prop) | AUDJPY.pro, Hive V5 HTF (prop) | AUDUSD.pro, Hive V5 HTF (prop) | BTCUSD, Hive V5 HTF (prop) | CADJPY.pro, Hive V5 HTF (prop) | CHFJPY.pro, Hive V5 HTF (prop) | EURJPY.pro, Hive V5 HTF (prop) | EURUSD.pro, Hive V5 HTF (prop) | GBPJPY.pro, Hive V5 HTF (prop) | GBPUSD.pro, Hive V5 HTF (prop) | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>51722</t>
+          <t>51720</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Weds Shorts &amp; Window Dressing</t>
+          <t>Hive V3 Forex HTF MOL</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2596,20 +2596,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>05/31/2026 18:48</t>
+          <t>06/01/2026 22:16</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>19170.52</v>
+        <v>17107.57</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>-4.15</v>
+        <v>-14.47</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>4.8</v>
+        <v>15.5</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>0.14</v>
+        <v>0.58</v>
       </c>
       <c r="L18" t="n">
         <v>20000</v>
@@ -2618,43 +2618,43 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="O18" s="7" t="n">
-        <v>19170.52</v>
+        <v>-1334.54</v>
       </c>
       <c r="P18" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q18" s="7" t="n">
-        <v>75</v>
+        <v>17.5</v>
       </c>
       <c r="R18" s="7" t="n">
-        <v>20.94871954963111</v>
+        <v>0.2207702727952168</v>
       </c>
       <c r="S18" s="7" t="n">
-        <v>3.199389279836951</v>
+        <v>13.34540000000001</v>
       </c>
       <c r="T18" t="n">
-        <v>4</v>
+        <v>161</v>
       </c>
       <c r="U18" s="7" t="n">
-        <v>-829.48</v>
+        <v>-1626.74</v>
       </c>
       <c r="V18" t="n">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="W18" s="7" t="n">
-        <v>50</v>
+        <v>39.75155279503105</v>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -2664,14 +2664,14 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Weds Shorts &amp; Window Dressing | AUDJPY.pro, Weds Shorts &amp; Window Dressing | CADJPY.pro</t>
+          <t>Hive V3 Forex HTF MOL | AUDJPY.pro, Hive V3 Forex HTF MOL | AUDUSD.pro, Hive V3 Forex HTF MOL | CADJPY.pro, Hive V3 Forex HTF MOL | CHFJPY.pro, Hive V3 Forex HTF MOL | EURCAD.pro, Hive V3 Forex HTF MOL | EURUSD.pro, Hive V3 Forex HTF MOL | GBPJPY.pro, Hive V3 Forex HTF MOL | GBPUSD.pro, Hive V3 Forex HTF MOL | USDCAD.pro, Hive V3 Forex HTF MOL | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>51723</t>
+          <t>51722</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FourPlay v15 MOL Bots</t>
+          <t>Weds Shorts &amp; Window Dressing</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2699,20 +2699,20 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>06/01/2026 22:03</t>
+          <t>05/31/2026 18:48</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
-        <v>19652.55</v>
+        <v>19170.52</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>-1.73</v>
+        <v>-4.15</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>5.42</v>
+        <v>4.8</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>0.84</v>
+        <v>0.14</v>
       </c>
       <c r="L19" t="n">
         <v>20000</v>
@@ -2721,43 +2721,43 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="O19" s="7" t="n">
-        <v>-678.3299999999999</v>
+        <v>19170.52</v>
       </c>
       <c r="P19" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="7" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="R19" s="7" t="n">
-        <v>0.71875</v>
+        <v>20.94871954963111</v>
       </c>
       <c r="S19" s="7" t="n">
-        <v>10.87443451666189</v>
+        <v>3.199389279836951</v>
       </c>
       <c r="T19" t="n">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="U19" s="7" t="n">
-        <v>-347.4499999999999</v>
+        <v>-829.48</v>
       </c>
       <c r="V19" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="W19" s="7" t="n">
-        <v>51.16279069767442</v>
+        <v>50</v>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
@@ -2767,14 +2767,14 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>FourPlay v15 MOL Bots | XAUUSD</t>
+          <t>Weds Shorts &amp; Window Dressing | AUDJPY.pro, Weds Shorts &amp; Window Dressing | CADJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>51724</t>
+          <t>51723</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Bar Reversal MOL Bots</t>
+          <t>FourPlay v15 MOL Bots</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2802,20 +2802,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>06/01/2026 22:15</t>
+          <t>06/01/2026 22:03</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>19772.53</v>
+        <v>19652.55</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>-1.14</v>
+        <v>-1.73</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>1.39</v>
+        <v>5.42</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>0.42</v>
+        <v>0.84</v>
       </c>
       <c r="L20" t="n">
         <v>20000</v>
@@ -2824,43 +2824,43 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>19771.98</v>
+        <v>-678.3299999999999</v>
       </c>
       <c r="P20" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="Q20" s="7" t="n">
-        <v>35.8974358974359</v>
+        <v>45</v>
       </c>
       <c r="R20" s="7" t="n">
-        <v>51.6299900135713</v>
+        <v>0.71875</v>
       </c>
       <c r="S20" s="7" t="n">
-        <v>0.9062551031630334</v>
+        <v>10.87443451666189</v>
       </c>
       <c r="T20" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-227.47</v>
+        <v>-347.4499999999999</v>
       </c>
       <c r="V20" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>51.16279069767442</v>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
@@ -2870,14 +2870,14 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>Bar Reversal MOL Bots | AUDUSD.pro, Bar Reversal MOL Bots | CHFJPY.pro, Bar Reversal MOL Bots | EURCAD.pro, Bar Reversal MOL Bots | EURUSD.pro, Bar Reversal MOL Bots | GBPJPY.pro, Bar Reversal MOL Bots | GBPNZD.pro, Bar Reversal MOL Bots | USDCAD.pro</t>
+          <t>FourPlay v15 MOL Bots | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>51725</t>
+          <t>51724</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Aggv3 MOL Bots</t>
+          <t>Bar Reversal MOL Bots</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2905,20 +2905,20 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>06/01/2026 22:22</t>
+          <t>06/01/2026 22:15</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>16406.45</v>
+        <v>19772.53</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>-17.98</v>
+        <v>-1.14</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>17.98</v>
+        <v>1.39</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.44</v>
+        <v>0.42</v>
       </c>
       <c r="L21" t="n">
         <v>20000</v>
@@ -2927,34 +2927,34 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>-389.3</v>
+        <v>19771.98</v>
       </c>
       <c r="P21" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q21" s="7" t="n">
-        <v>25</v>
+        <v>35.8974358974359</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>0.4291881146993814</v>
+        <v>51.6299900135713</v>
       </c>
       <c r="S21" s="7" t="n">
-        <v>3.847900000000082</v>
+        <v>0.9062551031630334</v>
       </c>
       <c r="T21" t="n">
-        <v>265</v>
+        <v>39</v>
       </c>
       <c r="U21" s="7" t="n">
-        <v>-3373.84</v>
+        <v>-227.47</v>
       </c>
       <c r="V21" t="n">
-        <v>92</v>
+        <v>13</v>
       </c>
       <c r="W21" s="7" t="n">
-        <v>34.71698113207547</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X21" t="inlineStr">
         <is>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
@@ -2973,14 +2973,14 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>Aggv3 MOL Bots | AUDJPY.pro, Aggv3 MOL Bots | AUDUSD.pro, Aggv3 MOL Bots | CHFJPY.pro, Aggv3 MOL Bots | EURJPY.pro, Aggv3 MOL Bots | GBPCAD.pro, Aggv3 MOL Bots | GBPJPY.pro, Aggv3 MOL Bots | GBPUSD.pro, Aggv3 MOL Bots | NZDJPY.pro, Aggv3 MOL Bots | NZDUSD.pro, Aggv3 MOL Bots | USDJPY.pro, Aggv3 MOL Bots | XAUUSD</t>
+          <t>Bar Reversal MOL Bots | AUDUSD.pro, Bar Reversal MOL Bots | CHFJPY.pro, Bar Reversal MOL Bots | EURCAD.pro, Bar Reversal MOL Bots | EURUSD.pro, Bar Reversal MOL Bots | GBPJPY.pro, Bar Reversal MOL Bots | GBPNZD.pro, Bar Reversal MOL Bots | USDCAD.pro</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>51727</t>
+          <t>51725</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FourPlay MOL Bots</t>
+          <t>Aggv3 MOL Bots</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3008,20 +3008,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>05/31/2026 03:08</t>
+          <t>06/01/2026 22:22</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>19993.52</v>
+        <v>16406.45</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-0.03</v>
+        <v>-17.98</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="K22" t="n">
-        <v>1</v>
+        <v>17.98</v>
+      </c>
+      <c r="K22" s="7" t="n">
+        <v>0.44</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3033,35 +3033,35 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>16.12999999999997</v>
+        <v>-389.3</v>
       </c>
       <c r="P22" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>42.5</v>
+        <v>25</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>1.01223940572524</v>
+        <v>0.4291881146993814</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>4.587326371757409</v>
+        <v>3.847900000000082</v>
       </c>
       <c r="T22" t="n">
-        <v>39</v>
+        <v>265</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>118.8299999999999</v>
+        <v>-3373.84</v>
       </c>
       <c r="V22" t="n">
-        <v>15</v>
+        <v>92</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>38.46153846153847</v>
+        <v>34.71698113207547</v>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
@@ -3071,19 +3071,19 @@
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>FourPlay MOL Bots | AUDUSD.pro, FourPlay MOL Bots | CHFJPY.pro, FourPlay MOL Bots | EURJPY.pro, FourPlay MOL Bots | EURUSD.pro, FourPlay MOL Bots | GBPAUD.pro, FourPlay MOL Bots | GBPJPY.pro, FourPlay MOL Bots | GBPNZD.pro, FourPlay MOL Bots | GBPUSD.pro, FourPlay MOL Bots | USDCAD.pro</t>
+          <t>Aggv3 MOL Bots | AUDJPY.pro, Aggv3 MOL Bots | AUDUSD.pro, Aggv3 MOL Bots | CHFJPY.pro, Aggv3 MOL Bots | EURJPY.pro, Aggv3 MOL Bots | GBPCAD.pro, Aggv3 MOL Bots | GBPJPY.pro, Aggv3 MOL Bots | GBPUSD.pro, Aggv3 MOL Bots | NZDJPY.pro, Aggv3 MOL Bots | NZDUSD.pro, Aggv3 MOL Bots | USDJPY.pro, Aggv3 MOL Bots | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>52360</t>
+          <t>51727</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hive 7 HTF MOL</t>
+          <t>FourPlay MOL Bots</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3111,20 +3111,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>06/01/2026 22:20</t>
+          <t>05/31/2026 03:08</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19325.73</v>
+        <v>19993.52</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-3.37</v>
+        <v>-0.03</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>8.619999999999999</v>
-      </c>
-      <c r="K23" s="7" t="n">
-        <v>0.83</v>
+        <v>2.34</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3136,7 +3136,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-298.13</v>
+        <v>16.12999999999997</v>
       </c>
       <c r="P23" t="n">
         <v>17</v>
@@ -3145,48 +3145,48 @@
         <v>42.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.8405406417312516</v>
+        <v>1.01223940572524</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>14.43094050860564</v>
+        <v>4.587326371757409</v>
       </c>
       <c r="T23" t="n">
-        <v>108</v>
+        <v>39</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-674.2699999999998</v>
+        <v>118.8299999999999</v>
       </c>
       <c r="V23" t="n">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>45.37037037037037</v>
+        <v>38.46153846153847</v>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>Hive 7 HTF MOL | AUDUSD.pro, Hive 7 HTF MOL | EURGBP.pro, Hive 7 HTF MOL | EURUSD.pro, Hive 7 HTF MOL | GBPUSD.pro, Hive 7 HTF MOL | USDCAD.pro</t>
+          <t>FourPlay MOL Bots | AUDUSD.pro, FourPlay MOL Bots | CHFJPY.pro, FourPlay MOL Bots | EURJPY.pro, FourPlay MOL Bots | EURUSD.pro, FourPlay MOL Bots | GBPAUD.pro, FourPlay MOL Bots | GBPJPY.pro, FourPlay MOL Bots | GBPNZD.pro, FourPlay MOL Bots | GBPUSD.pro, FourPlay MOL Bots | USDCAD.pro</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>52361</t>
+          <t>52360</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hive 7 LTF MOL</t>
+          <t>Hive 7 HTF MOL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3214,20 +3214,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/01/2026 22:22</t>
+          <t>06/01/2026 22:20</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>20030.41</v>
+        <v>19325.73</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>0.16</v>
+        <v>-3.37</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>4.51</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>1.01</v>
+        <v>0.83</v>
       </c>
       <c r="L24" t="n">
         <v>20000</v>
@@ -3239,40 +3239,40 @@
         <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>-344.17</v>
+        <v>-298.13</v>
       </c>
       <c r="P24" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="Q24" s="7" t="n">
-        <v>77.5</v>
+        <v>42.5</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>0.1696943378929338</v>
+        <v>0.8405406417312516</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>4.134297081725435</v>
+        <v>14.43094050860564</v>
       </c>
       <c r="T24" t="n">
-        <v>632</v>
+        <v>108</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>198.1700000000002</v>
+        <v>-674.2699999999998</v>
       </c>
       <c r="V24" t="n">
-        <v>406</v>
+        <v>49</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>64.24050632911393</v>
+        <v>45.37037037037037</v>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
@@ -3282,14 +3282,14 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>Hive 7 LTF MOL | AUDJPY.pro, Hive 7 LTF MOL | CADJPY.pro, Hive 7 LTF MOL | EURGBP.pro, Hive 7 LTF MOL | EURJPY.pro, Hive 7 LTF MOL | EURUSD.pro, Hive 7 LTF MOL | GBPJPY.pro, Hive 7 LTF MOL | GBPUSD.pro, Hive 7 LTF MOL | USDCAD.pro, Hive 7 LTF MOL | USDJPY.pro, Hive 7 LTF MOL | XAUUSD</t>
+          <t>Hive 7 HTF MOL | AUDUSD.pro, Hive 7 HTF MOL | EURGBP.pro, Hive 7 HTF MOL | EURUSD.pro, Hive 7 HTF MOL | GBPUSD.pro, Hive 7 HTF MOL | USDCAD.pro</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>52362</t>
+          <t>52361</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BB Fade Prop</t>
+          <t>Hive 7 LTF MOL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3317,20 +3317,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>06/01/2026 22:32</t>
+          <t>06/01/2026 22:22</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>20164.61</v>
+        <v>20030.41</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.82</v>
+        <v>0.16</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>2.77</v>
+        <v>4.51</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>1.25</v>
+        <v>1.01</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3342,40 +3342,40 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>167.13</v>
+        <v>-344.17</v>
       </c>
       <c r="P25" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>70</v>
+        <v>77.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.252392523925239</v>
+        <v>0.1696943378929338</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>5.34399892760695</v>
+        <v>4.134297081725435</v>
       </c>
       <c r="T25" t="n">
-        <v>41</v>
+        <v>632</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>164.61</v>
+        <v>198.1700000000002</v>
       </c>
       <c r="V25" t="n">
-        <v>28</v>
+        <v>406</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>68.29268292682927</v>
+        <v>64.24050632911393</v>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
@@ -3385,14 +3385,14 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>BB Fade Prop | AUDJPY.pro, BB Fade Prop | AUDNZD.pro, BB Fade Prop | CADJPY.pro, BB Fade Prop | CHFJPY.pro, BB Fade Prop | GBPJPY.pro, BB Fade Prop | GBPNZD.pro, BB Fade Prop | NZDJPY.pro, BB Fade Prop | XAGUSD</t>
+          <t>Hive 7 LTF MOL | AUDJPY.pro, Hive 7 LTF MOL | CADJPY.pro, Hive 7 LTF MOL | EURGBP.pro, Hive 7 LTF MOL | EURJPY.pro, Hive 7 LTF MOL | EURUSD.pro, Hive 7 LTF MOL | GBPJPY.pro, Hive 7 LTF MOL | GBPUSD.pro, Hive 7 LTF MOL | USDCAD.pro, Hive 7 LTF MOL | USDJPY.pro, Hive 7 LTF MOL | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>52363</t>
+          <t>52362</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>T&amp;D4L Prop Firm</t>
+          <t>BB Fade Prop</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3420,20 +3420,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/01/2026 22:24</t>
+          <t>06/01/2026 22:32</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>13856.18</v>
+        <v>20164.61</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-30.73</v>
+        <v>0.82</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>40.77</v>
+        <v>2.77</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.72</v>
+        <v>1.25</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3445,31 +3445,31 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>122.32</v>
+        <v>167.13</v>
       </c>
       <c r="P26" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>82.5</v>
+        <v>70</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>1.561898504232211</v>
+        <v>1.252392523925239</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>4.420012749947007</v>
+        <v>5.34399892760695</v>
       </c>
       <c r="T26" t="n">
-        <v>2326</v>
+        <v>41</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>-3026.81</v>
+        <v>164.61</v>
       </c>
       <c r="V26" t="n">
-        <v>1398</v>
+        <v>28</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>60.10318142734307</v>
+        <v>68.29268292682927</v>
       </c>
       <c r="X26" t="inlineStr">
         <is>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
@@ -3488,14 +3488,14 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>T&amp;D4L Prop Firm | AUDJPY.pro, T&amp;D4L Prop Firm | CADJPY.pro, T&amp;D4L Prop Firm | EURUSD.pro, T&amp;D4L Prop Firm | GBPJPY.pro, T&amp;D4L Prop Firm | GBPUSD.pro, T&amp;D4L Prop Firm | USDCAD.pro, T&amp;D4L Prop Firm | USDJPY.pro</t>
+          <t>BB Fade Prop | AUDJPY.pro, BB Fade Prop | AUDNZD.pro, BB Fade Prop | CADJPY.pro, BB Fade Prop | CHFJPY.pro, BB Fade Prop | GBPJPY.pro, BB Fade Prop | GBPNZD.pro, BB Fade Prop | NZDJPY.pro, BB Fade Prop | XAGUSD</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>52364</t>
+          <t>52363</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LVF-ZFade MOL</t>
+          <t>T&amp;D4L Prop Firm</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3523,20 +3523,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>05/31/2026 03:10</t>
+          <t>06/01/2026 22:24</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20896.54</v>
+        <v>13856.18</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>4.49</v>
+        <v>-30.73</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.37</v>
+        <v>40.77</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>5.96</v>
+        <v>0.72</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3545,43 +3545,43 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>20896.54</v>
+        <v>122.32</v>
       </c>
       <c r="P27" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>29.41176470588236</v>
+        <v>82.5</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>116.6549701129068</v>
+        <v>1.561898504232211</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>0.2483351281054041</v>
+        <v>4.420012749947007</v>
       </c>
       <c r="T27" t="n">
-        <v>34</v>
+        <v>2326</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>891.84</v>
+        <v>-3026.81</v>
       </c>
       <c r="V27" t="n">
-        <v>9</v>
+        <v>1398</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>26.47058823529412</v>
+        <v>60.10318142734307</v>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
@@ -3591,34 +3591,34 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
+          <t>T&amp;D4L Prop Firm | AUDJPY.pro, T&amp;D4L Prop Firm | CADJPY.pro, T&amp;D4L Prop Firm | EURUSD.pro, T&amp;D4L Prop Firm | GBPJPY.pro, T&amp;D4L Prop Firm | GBPUSD.pro, T&amp;D4L Prop Firm | USDCAD.pro, T&amp;D4L Prop Firm | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>657902</t>
+          <t>52364</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Cree Manual Trading</t>
+          <t>LVF-ZFade MOL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>OX Securities</t>
+          <t>TradeSmart</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F28" t="b">
@@ -3626,60 +3626,60 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/02/2026 00:38</t>
+          <t>05/31/2026 03:10</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>2380.77</v>
+        <v>20896.54</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>-96.73999999999999</v>
+        <v>4.49</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>99.38</v>
+        <v>0.37</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>0.83</v>
+        <v>5.96</v>
       </c>
       <c r="L28" t="n">
-        <v>31000</v>
+        <v>20000</v>
       </c>
       <c r="M28" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>-1007.44</v>
+        <v>20896.54</v>
       </c>
       <c r="P28" t="n">
         <v>10</v>
       </c>
       <c r="Q28" s="7" t="n">
-        <v>25</v>
+        <v>29.41176470588236</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>0.6552629829110979</v>
+        <v>116.6549701129068</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>11.1226856288573</v>
+        <v>0.2483351281054041</v>
       </c>
       <c r="T28" t="n">
-        <v>486</v>
+        <v>34</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>-18619.23</v>
+        <v>891.84</v>
       </c>
       <c r="V28" t="n">
-        <v>199</v>
+        <v>9</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>40.94650205761317</v>
+        <v>26.47058823529412</v>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
@@ -3694,14 +3694,14 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>Cree Manual Trading | AUDUSD.PRO, Cree Manual Trading | ETHUSD, Cree Manual Trading | EURGBP.PRO, Cree Manual Trading | EURJPY.PRO, Cree Manual Trading | EURUSD.PRO, Cree Manual Trading | GBPUSD.PRO, Cree Manual Trading | NZDUSD.PRO, Cree Manual Trading | USDCAD.PRO, Cree Manual Trading | USDCHF.PRO, Cree Manual Trading | USDJPY.PRO, Cree Manual Trading | XAGUSD.PRO, Cree Manual Trading | XAUUSD.PRO</t>
+          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>662437</t>
+          <t>657902</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gold Talon V1.2</t>
+          <t>Cree Manual Trading</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS149</t>
         </is>
       </c>
       <c r="F29" t="b">
@@ -3729,60 +3729,60 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/01/2026 14:43</t>
+          <t>06/02/2026 00:38</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>26087.98</v>
+        <v>2380.77</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.88</v>
+        <v>-96.73999999999999</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>6.56</v>
+        <v>99.38</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>1.07</v>
+        <v>0.83</v>
       </c>
       <c r="L29" t="n">
-        <v>26000</v>
+        <v>31000</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="N29" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>26057.87</v>
+        <v>-1007.44</v>
       </c>
       <c r="P29" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>44.73684210526316</v>
+        <v>25</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>21.19303528027617</v>
+        <v>0.6552629829110979</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>3.317542334367406</v>
+        <v>11.1226856288573</v>
       </c>
       <c r="T29" t="n">
-        <v>16</v>
+        <v>486</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>441.76</v>
+        <v>-18619.23</v>
       </c>
       <c r="V29" t="n">
-        <v>7</v>
+        <v>199</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>43.75</v>
+        <v>40.94650205761317</v>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
@@ -3792,39 +3792,39 @@
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>Gold Talon | EURUSD.PRO, Gold Talon | XAUUSD.PRO</t>
+          <t>Cree Manual Trading | AUDUSD.PRO, Cree Manual Trading | ETHUSD, Cree Manual Trading | EURGBP.PRO, Cree Manual Trading | EURJPY.PRO, Cree Manual Trading | EURUSD.PRO, Cree Manual Trading | GBPUSD.PRO, Cree Manual Trading | NZDUSD.PRO, Cree Manual Trading | USDCAD.PRO, Cree Manual Trading | USDCHF.PRO, Cree Manual Trading | USDJPY.PRO, Cree Manual Trading | XAGUSD.PRO, Cree Manual Trading | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>52441850</t>
+          <t>662437</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>EA Fx RSI MOL</t>
+          <t>Gold Talon V1.2</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>IC Markets</t>
+          <t>OX Securities</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS92t2</t>
         </is>
       </c>
       <c r="F30" t="b">
@@ -3832,82 +3832,82 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>05/31/2026 05:27</t>
+          <t>06/01/2026 14:43</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>44652.36</v>
+        <v>26087.98</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>24.35</v>
+        <v>0.88</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>22.74</v>
+        <v>6.56</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.17</v>
+        <v>1.07</v>
       </c>
       <c r="L30" t="n">
-        <v>25000</v>
+        <v>26000</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>2690.85</v>
+        <v>26057.87</v>
       </c>
       <c r="P30" t="n">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>90</v>
+        <v>44.73684210526316</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>7.653785968877684</v>
+        <v>21.19303528027617</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>4.601200000000008</v>
+        <v>3.317542334367406</v>
       </c>
       <c r="T30" t="n">
-        <v>1528</v>
+        <v>16</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>6602.099999999999</v>
+        <v>441.76</v>
       </c>
       <c r="V30" t="n">
-        <v>748</v>
+        <v>7</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>48.95287958115183</v>
+        <v>43.75</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>EA Fx RSI MOL | AUDUSD, EA Fx RSI MOL | GBPJPY, EA Fx RSI MOL | USDCAD, EA Fx RSI MOL | USDCHF, EA Fx RSI MOL | USDJPY</t>
+          <t>Gold Talon | EURUSD.PRO, Gold Talon | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>52441853</t>
+          <t>52441850</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fx RSI Low DD Prop Firms</t>
+          <t>EA Fx RSI MOL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3935,20 +3935,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>05/31/2026 11:04</t>
+          <t>05/31/2026 05:27</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>32539.84</v>
+        <v>44652.36</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>-8.27</v>
+        <v>24.35</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>19.72</v>
+        <v>22.74</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>0.93</v>
+        <v>1.17</v>
       </c>
       <c r="L31" t="n">
         <v>25000</v>
@@ -3960,146 +3960,160 @@
         <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
+        <v>2690.85</v>
+      </c>
+      <c r="P31" t="n">
+        <v>36</v>
+      </c>
+      <c r="Q31" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="R31" s="7" t="n">
+        <v>7.653785968877684</v>
+      </c>
+      <c r="S31" s="7" t="n">
+        <v>4.601200000000008</v>
+      </c>
+      <c r="T31" t="n">
+        <v>1528</v>
+      </c>
+      <c r="U31" s="7" t="n">
+        <v>6602.099999999999</v>
+      </c>
+      <c r="V31" t="n">
+        <v>748</v>
+      </c>
+      <c r="W31" s="7" t="n">
+        <v>48.95287958115183</v>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>2025-07-29</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>EA Fx RSI MOL | AUDUSD, EA Fx RSI MOL | GBPJPY, EA Fx RSI MOL | USDCAD, EA Fx RSI MOL | USDCHF, EA Fx RSI MOL | USDJPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>52441853</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fx RSI Low DD Prop Firms</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>IC Markets</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>VPS92</t>
+        </is>
+      </c>
+      <c r="F32" t="b">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>05/31/2026 11:04</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>32539.84</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>-8.27</v>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>19.72</v>
+      </c>
+      <c r="K32" s="7" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L32" t="n">
+        <v>25000</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>40</v>
+      </c>
+      <c r="O32" s="7" t="n">
         <v>-91.29999999999998</v>
       </c>
-      <c r="P31" t="n">
+      <c r="P32" t="n">
         <v>27</v>
       </c>
-      <c r="Q31" s="7" t="n">
+      <c r="Q32" s="7" t="n">
         <v>67.5</v>
       </c>
-      <c r="R31" s="7" t="n">
+      <c r="R32" s="7" t="n">
         <v>0.8463816075938344</v>
       </c>
-      <c r="S31" s="7" t="n">
+      <c r="S32" s="7" t="n">
         <v>2.279467522103865</v>
       </c>
-      <c r="T31" t="n">
+      <c r="T32" t="n">
         <v>2807</v>
       </c>
-      <c r="U31" s="7" t="n">
+      <c r="U32" s="7" t="n">
         <v>-1830.42</v>
       </c>
-      <c r="V31" t="n">
+      <c r="V32" t="n">
         <v>1709</v>
       </c>
-      <c r="W31" s="7" t="n">
+      <c r="W32" s="7" t="n">
         <v>60.88350552190951</v>
       </c>
-      <c r="X31" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>2025-07-29</t>
         </is>
       </c>
-      <c r="Y31" t="inlineStr">
+      <c r="Y32" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="Z31" t="inlineStr">
+      <c r="Z32" t="inlineStr">
         <is>
           <t>RECONCILE</t>
         </is>
       </c>
-      <c r="AA31" t="inlineStr">
+      <c r="AA32" t="inlineStr">
         <is>
           <t>Fx RSI Low DD Prop Firms | AUDUSD, Fx RSI Low DD Prop Firms | GBPJPY, Fx RSI Low DD Prop Firms | USDCHF, Fx RSI Low DD Prop Firms | USDJPY</t>
         </is>
       </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>22660</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Swing Trade MOL</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>TradeSmart</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>VPS92</t>
-        </is>
-      </c>
-      <c r="F32" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="G32" s="8" t="inlineStr">
-        <is>
-          <t>05/28/2026 00:43</t>
-        </is>
-      </c>
-      <c r="H32" s="9" t="n">
-        <v>28127.1</v>
-      </c>
-      <c r="I32" s="9" t="n">
-        <v>12.33</v>
-      </c>
-      <c r="J32" s="9" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="K32" s="9" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="L32" s="8" t="n">
-        <v>25000</v>
-      </c>
-      <c r="M32" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N32" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="O32" s="9" t="n">
-        <v>-3167.68</v>
-      </c>
-      <c r="P32" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q32" s="9" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="R32" s="9" t="n">
-        <v>0.1775893840214113</v>
-      </c>
-      <c r="S32" s="9" t="n">
-        <v>29.85289999999997</v>
-      </c>
-      <c r="T32" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U32" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V32" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W32" s="8" t="n"/>
-      <c r="X32" s="8" t="n"/>
-      <c r="Y32" s="8" t="n"/>
-      <c r="Z32" s="8" t="inlineStr">
-        <is>
-          <t>DATA GAP - Bach missing</t>
-        </is>
-      </c>
-      <c r="AA32" s="8" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>38765</t>
+          <t>22660</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
@@ -4109,7 +4123,7 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Donchain Gold</t>
+          <t>Swing Trade MOL</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -4127,23 +4141,23 @@
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>05/29/2026 09:06</t>
+          <t>05/28/2026 00:43</t>
         </is>
       </c>
       <c r="H33" s="9" t="n">
-        <v>20207.71</v>
+        <v>28127.1</v>
       </c>
       <c r="I33" s="9" t="n">
-        <v>1.04</v>
+        <v>12.33</v>
       </c>
       <c r="J33" s="9" t="n">
-        <v>5.78</v>
+        <v>17.6</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>1.06</v>
+        <v>1.33</v>
       </c>
       <c r="L33" s="8" t="n">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="M33" s="8" t="n">
         <v>0</v>
@@ -4152,19 +4166,19 @@
         <v>40</v>
       </c>
       <c r="O33" s="9" t="n">
-        <v>-1245.8</v>
+        <v>-3167.68</v>
       </c>
       <c r="P33" s="8" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="Q33" s="9" t="n">
-        <v>40</v>
+        <v>27.5</v>
       </c>
       <c r="R33" s="9" t="n">
-        <v>0.2299841280794976</v>
+        <v>0.1775893840214113</v>
       </c>
       <c r="S33" s="9" t="n">
-        <v>11.26469363233483</v>
+        <v>29.85289999999997</v>
       </c>
       <c r="T33" s="8" t="n">
         <v>0</v>
@@ -4188,7 +4202,7 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>38768</t>
+          <t>38765</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
@@ -4198,7 +4212,7 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Aggressive CV2 Prop Firm</t>
+          <t>Donchain Gold</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -4216,20 +4230,20 @@
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>05/29/2026 15:57</t>
+          <t>05/29/2026 09:06</t>
         </is>
       </c>
       <c r="H34" s="9" t="n">
-        <v>19560.47</v>
+        <v>20207.71</v>
       </c>
       <c r="I34" s="9" t="n">
-        <v>-2.35</v>
+        <v>1.04</v>
       </c>
       <c r="J34" s="9" t="n">
-        <v>7.3</v>
+        <v>5.78</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>0.89</v>
+        <v>1.06</v>
       </c>
       <c r="L34" s="8" t="n">
         <v>20000</v>
@@ -4241,19 +4255,19 @@
         <v>40</v>
       </c>
       <c r="O34" s="9" t="n">
-        <v>-980.9399999999999</v>
+        <v>-1245.8</v>
       </c>
       <c r="P34" s="8" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="Q34" s="9" t="n">
-        <v>72.5</v>
+        <v>40</v>
       </c>
       <c r="R34" s="9" t="n">
-        <v>0.7320202184071484</v>
+        <v>0.2299841280794976</v>
       </c>
       <c r="S34" s="9" t="n">
-        <v>14.37228152648387</v>
+        <v>11.26469363233483</v>
       </c>
       <c r="T34" s="8" t="n">
         <v>0</v>
@@ -4277,7 +4291,7 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>38769</t>
+          <t>38768</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -4287,7 +4301,7 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>EA Forex RSI V2 +DD</t>
+          <t>Aggressive CV2 Prop Firm</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -4305,20 +4319,20 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>05/31/2026 19:47</t>
+          <t>05/29/2026 15:57</t>
         </is>
       </c>
       <c r="H35" s="9" t="n">
-        <v>18825.91</v>
+        <v>19560.47</v>
       </c>
       <c r="I35" s="9" t="n">
-        <v>-5.87</v>
+        <v>-2.35</v>
       </c>
       <c r="J35" s="9" t="n">
-        <v>10.84</v>
+        <v>7.3</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>0.71</v>
+        <v>0.89</v>
       </c>
       <c r="L35" s="8" t="n">
         <v>20000</v>
@@ -4330,19 +4344,19 @@
         <v>40</v>
       </c>
       <c r="O35" s="9" t="n">
-        <v>193.4399999999999</v>
+        <v>-980.9399999999999</v>
       </c>
       <c r="P35" s="8" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="Q35" s="9" t="n">
-        <v>55.00000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="R35" s="9" t="n">
-        <v>1.233044880741913</v>
+        <v>0.7320202184071484</v>
       </c>
       <c r="S35" s="9" t="n">
-        <v>4.640100000000002</v>
+        <v>14.37228152648387</v>
       </c>
       <c r="T35" s="8" t="n">
         <v>0</v>
@@ -4366,17 +4380,17 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>39479</t>
+          <t>38769</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>T&amp;D19 V2 USDJPY PROP</t>
+          <t>EA Forex RSI V2 +DD</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -4386,52 +4400,52 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F36" s="8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>10/03/2025 00:48</t>
+          <t>05/31/2026 19:47</t>
         </is>
       </c>
       <c r="H36" s="9" t="n">
-        <v>34219.5</v>
+        <v>18825.91</v>
       </c>
       <c r="I36" s="9" t="n">
-        <v>0.03</v>
+        <v>-5.87</v>
       </c>
       <c r="J36" s="9" t="n">
-        <v>12.87</v>
+        <v>10.84</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="L36" s="9" t="n">
-        <v>36046.71</v>
-      </c>
-      <c r="M36" s="9" t="n">
-        <v>627.79</v>
+        <v>0.71</v>
+      </c>
+      <c r="L36" s="8" t="n">
+        <v>20000</v>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="N36" s="8" t="n">
         <v>40</v>
       </c>
       <c r="O36" s="9" t="n">
-        <v>58.28</v>
+        <v>193.4399999999999</v>
       </c>
       <c r="P36" s="8" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="Q36" s="9" t="n">
-        <v>77.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R36" s="9" t="n">
-        <v>2.573611111111111</v>
+        <v>1.233044880741913</v>
       </c>
       <c r="S36" s="9" t="n">
-        <v>0.1587531959394289</v>
+        <v>4.640100000000002</v>
       </c>
       <c r="T36" s="8" t="n">
         <v>0</v>
@@ -5796,7 +5810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -6039,17 +6053,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>39479</t>
+          <t>41660</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>T&amp;D19 V2 USDJPY PROP</t>
+          <t>EA Fx RSI V2 TDS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -6059,19 +6073,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>VPS153</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>10/03/2025 00:48</t>
+          <t>05/31/2026 14:18</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>34219.5</v>
+        <v>17132.5</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.03</v>
+        <v>-14.35</v>
       </c>
       <c r="I9" t="n">
         <v>40</v>
@@ -6080,7 +6094,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>41660</t>
+          <t>47779</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6090,7 +6104,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>EA Fx RSI V2 TDS</t>
+          <t>Aggressive V3 + V4</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -6105,14 +6119,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>05/31/2026 14:18</t>
+          <t>06/01/2026 14:11</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>17132.5</v>
+        <v>1541.65</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>-14.35</v>
+        <v>-92.45999999999999</v>
       </c>
       <c r="I10" t="n">
         <v>40</v>
@@ -6121,7 +6135,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>47779</t>
+          <t>51719</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6131,7 +6145,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Aggressive V3 + V4</t>
+          <t>Hive V5 LTF (prop)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -6141,19 +6155,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>06/01/2026 14:11</t>
+          <t>06/01/2026 22:16</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>1541.65</v>
+        <v>18511.35</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>-92.45999999999999</v>
+        <v>-7.44</v>
       </c>
       <c r="I11" t="n">
         <v>40</v>
@@ -6162,7 +6176,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>51719</t>
+          <t>51721</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6172,7 +6186,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hive V5 LTF (prop)</t>
+          <t>Hive V3 Forex</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -6187,14 +6201,14 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>06/01/2026 22:16</t>
+          <t>05/31/2026 03:14</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>18511.35</v>
+        <v>15078.92</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>-7.44</v>
+        <v>-24.61</v>
       </c>
       <c r="I12" t="n">
         <v>40</v>
@@ -6203,7 +6217,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>51721</t>
+          <t>51726</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6213,7 +6227,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hive V3 Forex</t>
+          <t>T&amp;Dv5 Prop Bots</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -6228,23 +6242,23 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>05/31/2026 03:14</t>
+          <t>05/31/2026 03:10</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>15078.92</v>
+        <v>19920.5</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>-24.61</v>
+        <v>-0.4</v>
       </c>
       <c r="I13" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>51726</t>
+          <t>52365</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6254,7 +6268,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>T&amp;Dv5 Prop Bots</t>
+          <t>Hive 9 Demo Prop</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -6269,23 +6283,23 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>05/31/2026 03:10</t>
+          <t>06/01/2026 22:37</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>19920.5</v>
+        <v>19971.92</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>-0.4</v>
+        <v>-0.14</v>
       </c>
       <c r="I14" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>52365</t>
+          <t>52366</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6295,7 +6309,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hive 9 Demo Prop</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -6310,23 +6324,23 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/01/2026 22:37</t>
+          <t>06/01/2026 22:41</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>19971.92</v>
+        <v>19452.07</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>-0.14</v>
+        <v>-2.74</v>
       </c>
       <c r="I15" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>52366</t>
+          <t>52367</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6351,23 +6365,23 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/01/2026 22:41</t>
+          <t>06/01/2026 23:42</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>19452.07</v>
+        <v>19711.43</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>-2.74</v>
+        <v>-1.45</v>
       </c>
       <c r="I16" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>52367</t>
+          <t>52368</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6392,14 +6406,14 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>06/01/2026 23:42</t>
+          <t>05/31/2026 21:56</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>19711.43</v>
+        <v>19764.02</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>-1.45</v>
+        <v>-1.18</v>
       </c>
       <c r="I17" t="n">
         <v>40</v>
@@ -6408,7 +6422,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>52368</t>
+          <t>52369</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6433,23 +6447,23 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>05/31/2026 21:56</t>
+          <t>05/31/2026 08:43</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>19764.02</v>
+        <v>20282.75</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>-1.18</v>
+        <v>1.42</v>
       </c>
       <c r="I18" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>52369</t>
+          <t>52370</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6474,55 +6488,55 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>05/31/2026 08:43</t>
+          <t>05/31/2026 06:22</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>20282.75</v>
+        <v>21897.59</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>1.42</v>
+        <v>9.49</v>
       </c>
       <c r="I19" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>52370</t>
+          <t>639884</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Manual Trading (Diego)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>TradeSmart</t>
+          <t>OX Securities</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS149</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>05/31/2026 06:22</t>
+          <t>05/30/2026 12:06</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>21897.59</v>
+        <v>5027.65</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>9.49</v>
+        <v>42.67</v>
       </c>
       <c r="I20" t="n">
         <v>40</v>
@@ -6531,7 +6545,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>639884</t>
+          <t>647832</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6541,7 +6555,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Manual Trading (Diego)</t>
+          <t>Axis Rotation AUDUSD</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -6551,19 +6565,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>05/30/2026 12:06</t>
+          <t>06/01/2026 18:21</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>5027.65</v>
+        <v>4879.61</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>42.67</v>
+        <v>-27.8</v>
       </c>
       <c r="I21" t="n">
         <v>40</v>
@@ -6572,7 +6586,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>647832</t>
+          <t>658071</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -6582,7 +6596,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Axis Rotation AUDUSD</t>
+          <t>T&amp;D V1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -6592,19 +6606,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>06/01/2026 18:21</t>
+          <t>01/07/2026 18:21</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>4879.61</v>
+        <v>3417.36</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>-27.8</v>
+        <v>-0.19</v>
       </c>
       <c r="I22" t="n">
         <v>40</v>
@@ -6613,22 +6627,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>658071</t>
+          <t>52428953</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>T&amp;D V1</t>
+          <t>BTC Dual Breakout Scalper</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>OX Securities</t>
+          <t>IC Markets</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -6638,57 +6652,16 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>01/07/2026 18:21</t>
+          <t>05/31/2026 11:51</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>3417.36</v>
+        <v>28300.62</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>-0.19</v>
+        <v>13.2</v>
       </c>
       <c r="I23" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>52428953</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>BTC Dual Breakout Scalper</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>IC Markets</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>VPS92</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>05/31/2026 11:51</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>28300.62</v>
-      </c>
-      <c r="H24" s="7" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="I24" t="n">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboards — 2026-06-05
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-01 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-05 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -948,20 +948,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/01/2026 18:59</t>
+          <t>06/05/2026 08:01</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>54126.69</v>
+        <v>55335.24</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>115.47</v>
+        <v>120.29</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -973,31 +973,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-550.63</v>
+        <v>1258.37</v>
       </c>
       <c r="P2" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>62.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.8106157393130388</v>
+        <v>5.156051574446028</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>13.32676809860272</v>
+        <v>0.9736289069912897</v>
       </c>
       <c r="T2" t="n">
-        <v>2654</v>
+        <v>2709</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>29126.68999999999</v>
+        <v>30335.24</v>
       </c>
       <c r="V2" t="n">
-        <v>1703</v>
+        <v>1735</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>64.16729464958553</v>
+        <v>64.04577334809893</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -1051,20 +1051,20 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/02/2026 01:35</t>
+          <t>06/05/2026 03:27</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
-        <v>25000.04</v>
+        <v>24261.61</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>20.51</v>
+        <v>16.95</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>12.39</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1.07</v>
+        <v>1.03</v>
       </c>
       <c r="L3" s="7" t="n">
         <v>30545.04</v>
@@ -1076,31 +1076,31 @@
         <v>40</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>-6388.81</v>
+        <v>-6930.42</v>
       </c>
       <c r="P3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Q3" s="7" t="n">
-        <v>65</v>
+        <v>62.5</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>0.2421837290311843</v>
+        <v>0.186233164755358</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>65.81687632519494</v>
+        <v>71.45278259863474</v>
       </c>
       <c r="T3" t="n">
-        <v>865</v>
+        <v>874</v>
       </c>
       <c r="U3" s="7" t="n">
-        <v>4781.91</v>
+        <v>4043.48</v>
       </c>
       <c r="V3" t="n">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="W3" s="7" t="n">
-        <v>63.00578034682081</v>
+        <v>62.70022883295194</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -1154,20 +1154,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/01/2026 10:37</t>
+          <t>06/05/2026 05:44</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>20947.99</v>
+        <v>21054.45</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>4.71</v>
+        <v>5.24</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>5.78</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="L4" t="n">
         <v>20000</v>
@@ -1179,7 +1179,7 @@
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>606.1</v>
+        <v>534.6</v>
       </c>
       <c r="P4" t="n">
         <v>28</v>
@@ -1188,22 +1188,22 @@
         <v>70</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>1.195738227431627</v>
+        <v>1.17518906939018</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>10.978989121953</v>
+        <v>11.15365614851094</v>
       </c>
       <c r="T4" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>947.9900000000002</v>
+        <v>1054.45</v>
       </c>
       <c r="V4" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>64.60176991150442</v>
+        <v>64.91228070175438</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -1360,20 +1360,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>05/31/2026 20:38</t>
+          <t>06/05/2026 10:35</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
-        <v>17387.1</v>
+        <v>17401.71</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>-59.08</v>
+        <v>-59.05</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>60.59</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>30587.87</v>
@@ -1385,7 +1385,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>-144.47</v>
+        <v>-143.08</v>
       </c>
       <c r="P6" t="n">
         <v>31</v>
@@ -1394,10 +1394,10 @@
         <v>77.5</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>0.7636095884807331</v>
+        <v>0.7658839892006872</v>
       </c>
       <c r="S6" s="7" t="n">
-        <v>3.807157738240804</v>
+        <v>3.812086952093313</v>
       </c>
       <c r="T6" t="n">
         <v>602</v>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/02/2026 01:55</t>
+          <t>06/05/2026 03:37</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2026 19:27</t>
+          <t>06/05/2026 08:11</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1609,7 +1609,7 @@
         <v>294</v>
       </c>
       <c r="U8" s="7" t="n">
-        <v>-173.14</v>
+        <v>-173.1400000000001</v>
       </c>
       <c r="V8" t="n">
         <v>263</v>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/02/2026 02:28</t>
+          <t>06/05/2026 04:00</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1712,7 +1712,7 @@
         <v>447</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>-1584.58</v>
+        <v>-1584.580000000001</v>
       </c>
       <c r="V9" t="n">
         <v>204</v>
@@ -1815,7 +1815,7 @@
         <v>183</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>216.0199999999997</v>
+        <v>216.0199999999999</v>
       </c>
       <c r="V10" t="n">
         <v>84</v>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/01/2026 12:43</t>
+          <t>06/04/2026 21:08</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -1978,20 +1978,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>05/31/2026 18:56</t>
+          <t>06/04/2026 10:38</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>10529.39</v>
+        <v>10829.8</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>4.58</v>
+        <v>7.57</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1.25</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>3.56</v>
+        <v>5.22</v>
       </c>
       <c r="L12" t="n">
         <v>20000</v>
@@ -2003,28 +2003,28 @@
         <v>40</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>534.3</v>
+        <v>892.8499999999999</v>
       </c>
       <c r="P12" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>67.5</v>
+        <v>77.5</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>1.058394712217804</v>
+        <v>1.095610266903861</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>44.59199544555984</v>
+        <v>43.69494914343316</v>
       </c>
       <c r="T12" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>538.21</v>
+        <v>837.95</v>
       </c>
       <c r="V12" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="W12" s="7" t="n">
         <v>100</v>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -2081,11 +2081,11 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/01/2026 14:06</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>4726.13</v>
+          <t>06/05/2026 05:27</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>-5.47</v>
@@ -2099,32 +2099,32 @@
       <c r="L13" t="n">
         <v>5010</v>
       </c>
-      <c r="M13" t="n">
-        <v>10</v>
+      <c r="M13" s="7" t="n">
+        <v>4736.13</v>
       </c>
       <c r="N13" t="n">
         <v>40</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>-58.88</v>
+        <v>-4790.95</v>
       </c>
       <c r="P13" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>82.5</v>
+        <v>80</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>0.8621529240998268</v>
+        <v>0.07030875541161243</v>
       </c>
       <c r="S13" s="7" t="n">
-        <v>2.341150941280393</v>
+        <v>48.72982283464567</v>
       </c>
       <c r="T13" t="n">
         <v>38</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>-79.45999999999997</v>
+        <v>-79.45999999999999</v>
       </c>
       <c r="V13" t="n">
         <v>31</v>
@@ -2184,11 +2184,11 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>06/02/2026 01:00</t>
+          <t>06/05/2026 11:59</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>19996.4</v>
+        <v>19995.7</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>-5.21</v>
@@ -2224,16 +2224,16 @@
         <v>27.67771200973612</v>
       </c>
       <c r="T14" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="U14" s="7" t="n">
-        <v>158.4200000000002</v>
+        <v>157.7200000000003</v>
       </c>
       <c r="V14" t="n">
         <v>75</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>57.25190839694656</v>
+        <v>55.97014925373134</v>
       </c>
       <c r="X14" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -2287,17 +2287,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/01/2026 10:11</t>
+          <t>06/05/2026 05:32</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>18120.08</v>
+        <v>17949.63</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-9.42</v>
+        <v>-10.28</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>11.07</v>
+        <v>12.67</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>0.8</v>
@@ -2312,31 +2312,31 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>-1399.82</v>
+        <v>-917.0600000000002</v>
       </c>
       <c r="P15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>0.6403896732491465</v>
+        <v>0.7516891982547187</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>14.04210000000003</v>
+        <v>13.62048330434852</v>
       </c>
       <c r="T15" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-1879.920000000001</v>
+        <v>-2050.370000000001</v>
       </c>
       <c r="V15" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>44.11764705882353</v>
+        <v>44.44444444444444</v>
       </c>
       <c r="X15" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2390,17 +2390,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>06/01/2026 07:19</t>
+          <t>06/03/2026 00:57</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>11607.19</v>
+        <v>10869.76</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-96.40000000000001</v>
+        <v>-96.63</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>96.58</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>0.76</v>
@@ -2415,7 +2415,7 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-389.2699999999999</v>
+        <v>-28.43000000000009</v>
       </c>
       <c r="P16" t="n">
         <v>24</v>
@@ -2424,10 +2424,10 @@
         <v>60</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.9067654403853558</v>
+        <v>1.113935675219722</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>9.73899224894088</v>
+        <v>7.369281597233949</v>
       </c>
       <c r="T16" t="n">
         <v>3665</v>
@@ -2493,20 +2493,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>05/31/2026 03:31</t>
+          <t>06/05/2026 01:12</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>14113.73</v>
+        <v>13565.63</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>-29.46</v>
+        <v>-32.2</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>29.46</v>
+        <v>32.2</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="L17" t="n">
         <v>20000</v>
@@ -2518,7 +2518,7 @@
         <v>40</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>-885.64</v>
+        <v>-892.24</v>
       </c>
       <c r="P17" t="n">
         <v>2</v>
@@ -2527,22 +2527,22 @@
         <v>5</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>0.06609583263033575</v>
+        <v>0.1176598564110678</v>
       </c>
       <c r="S17" s="7" t="n">
-        <v>8.856399999999995</v>
+        <v>8.922399999999961</v>
       </c>
       <c r="T17" t="n">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>-6193.83</v>
+        <v>-6434.369999999999</v>
       </c>
       <c r="V17" t="n">
         <v>46</v>
       </c>
       <c r="W17" s="7" t="n">
-        <v>14.19753086419753</v>
+        <v>13.85542168674699</v>
       </c>
       <c r="X17" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>06/01/2026 22:16</t>
+          <t>06/05/2026 00:49</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>05/31/2026 18:48</t>
+          <t>06/05/2026 09:55</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>06/01/2026 22:03</t>
+          <t>06/04/2026 09:41</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -2842,16 +2842,16 @@
         <v>10.87443451666189</v>
       </c>
       <c r="T20" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-347.4499999999999</v>
+        <v>-154.17</v>
       </c>
       <c r="V20" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>51.16279069767442</v>
+        <v>52.27272727272727</v>
       </c>
       <c r="X20" t="inlineStr">
         <is>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>06/01/2026 22:15</t>
+          <t>06/05/2026 00:49</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3008,17 +3008,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>06/01/2026 22:22</t>
+          <t>06/05/2026 09:58</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>16406.45</v>
+        <v>16358.77</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-17.98</v>
+        <v>-18.22</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>17.98</v>
+        <v>18.22</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>0.44</v>
@@ -3033,7 +3033,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-389.3</v>
+        <v>-427.7499999999999</v>
       </c>
       <c r="P22" t="n">
         <v>10</v>
@@ -3042,10 +3042,10 @@
         <v>25</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.4291881146993814</v>
+        <v>0.4060289659818121</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>3.847900000000082</v>
+        <v>4.232400000000089</v>
       </c>
       <c r="T22" t="n">
         <v>265</v>
@@ -3111,20 +3111,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>05/31/2026 03:08</t>
+          <t>06/05/2026 09:59</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19993.52</v>
+        <v>21317.45</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-0.03</v>
+        <v>1.94</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>2.34</v>
       </c>
-      <c r="K23" t="n">
-        <v>1</v>
+      <c r="K23" s="7" t="n">
+        <v>1.23</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3136,7 +3136,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>16.12999999999997</v>
+        <v>415.9</v>
       </c>
       <c r="P23" t="n">
         <v>17</v>
@@ -3145,10 +3145,10 @@
         <v>42.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.01223940572524</v>
+        <v>1.265024717625593</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.587326371757409</v>
+        <v>4.584913432177711</v>
       </c>
       <c r="T23" t="n">
         <v>39</v>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/01/2026 22:20</t>
+          <t>06/05/2026 09:53</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>06/01/2026 22:22</t>
+          <t>06/05/2026 09:55</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/01/2026 22:32</t>
+          <t>06/03/2026 08:41</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/01/2026 22:24</t>
+          <t>06/03/2026 08:47</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3626,20 +3626,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>05/31/2026 03:10</t>
+          <t>06/05/2026 00:56</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>20896.54</v>
+        <v>20891.84</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>4.49</v>
+        <v>4.47</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>0.37</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>5.96</v>
+        <v>5.81</v>
       </c>
       <c r="L28" t="n">
         <v>20000</v>
@@ -3648,19 +3648,19 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>20896.54</v>
+        <v>20891.84</v>
       </c>
       <c r="P28" t="n">
         <v>10</v>
       </c>
       <c r="Q28" s="7" t="n">
-        <v>29.41176470588236</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>116.6549701129068</v>
+        <v>113.6973783579674</v>
       </c>
       <c r="S28" s="7" t="n">
         <v>0.2483351281054041</v>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr">
@@ -3729,20 +3729,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>05/31/2026 08:43</t>
+          <t>06/05/2026 05:21</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20282.75</v>
+        <v>20462.96</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>1.42</v>
+        <v>2.31</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.24</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>6.79</v>
+        <v>6.36</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3751,31 +3751,31 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>20282.75</v>
+        <v>20462.96</v>
       </c>
       <c r="P29" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>87.5</v>
+        <v>76.92307692307693</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>416.2897215397215</v>
+        <v>238.0867802108678</v>
       </c>
       <c r="S29" s="7" t="n">
         <v>0.1628000000000005</v>
       </c>
       <c r="T29" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>253.36</v>
+        <v>462.96</v>
       </c>
       <c r="V29" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="W29" s="7" t="n">
         <v>75</v>
@@ -3787,12 +3787,12 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
@@ -3832,20 +3832,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/02/2026 01:54</t>
+          <t>06/05/2026 03:38</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>21477.93</v>
+        <v>21507.01</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>7.39</v>
+        <v>7.54</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>8.390000000000001</v>
+        <v>11.64</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -3857,31 +3857,31 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-226.68</v>
+        <v>-129.61</v>
       </c>
       <c r="P30" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>47.5</v>
+        <v>50</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.9093847617640797</v>
+        <v>0.9496002047239146</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>7.943962137494139</v>
+        <v>9.643808533568093</v>
       </c>
       <c r="T30" t="n">
-        <v>401</v>
+        <v>546</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>1704.050000000001</v>
+        <v>1474.09</v>
       </c>
       <c r="V30" t="n">
-        <v>208</v>
+        <v>281</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>51.87032418952619</v>
+        <v>51.46520146520146</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
@@ -3935,20 +3935,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/01/2026 17:59</t>
+          <t>06/05/2026 07:43</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20614.46</v>
+        <v>20613.8</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>3.07</v>
+        <v>3.06</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.49</v>
+        <v>0.99</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>4.12</v>
+        <v>2.52</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -3957,34 +3957,34 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
+        <v>15</v>
+      </c>
+      <c r="O31" s="7" t="n">
+        <v>20613.8</v>
+      </c>
+      <c r="P31" t="n">
         <v>11</v>
       </c>
-      <c r="O31" s="7" t="n">
-        <v>20614.46</v>
-      </c>
-      <c r="P31" t="n">
-        <v>9</v>
-      </c>
       <c r="Q31" s="7" t="n">
-        <v>81.81818181818183</v>
+        <v>73.33333333333333</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>105.578226461039</v>
+        <v>52.20168902136115</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>0.3302869842986254</v>
+        <v>0.6667255042947245</v>
       </c>
       <c r="T31" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>614.46</v>
+        <v>613.8</v>
       </c>
       <c r="V31" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>72.72727272727273</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="X31" t="inlineStr">
         <is>
@@ -3993,12 +3993,12 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr">
@@ -4038,20 +4038,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/02/2026 00:57</t>
+          <t>06/05/2026 11:57</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>19967.02</v>
+        <v>20692.94</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>-0.16</v>
+        <v>3.46</v>
       </c>
       <c r="J32" s="7" t="n">
         <v>1.78</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.9</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4060,34 +4060,34 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>19936.1</v>
+        <v>20627.07</v>
       </c>
       <c r="P32" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>35.75184489000279</v>
+        <v>27.74335711331679</v>
       </c>
       <c r="S32" s="7" t="n">
         <v>1.194162721074082</v>
       </c>
       <c r="T32" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>-32.98000000000003</v>
+        <v>692.9400000000001</v>
       </c>
       <c r="V32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>50</v>
       </c>
       <c r="X32" t="inlineStr">
         <is>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
@@ -4141,17 +4141,17 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06/01/2026 08:17</t>
+          <t>06/05/2026 04:48</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>19565.4</v>
+        <v>19376.4</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>-2.17</v>
+        <v>-2.18</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>2.17</v>
+        <v>2.18</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -4163,28 +4163,28 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>19557.84</v>
+        <v>19555.68</v>
       </c>
       <c r="P33" t="n">
         <v>1</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>10</v>
+        <v>9.090909090909092</v>
       </c>
       <c r="R33" s="7" t="n">
-        <v>46.15526631588664</v>
+        <v>46.04051565377532</v>
       </c>
       <c r="S33" s="7" t="n">
-        <v>1.444399999999999</v>
+        <v>1.448000000000005</v>
       </c>
       <c r="T33" t="n">
         <v>11</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>-434.5999999999999</v>
+        <v>-623.5999999999999</v>
       </c>
       <c r="V33" t="n">
         <v>0</v>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>06/01/2026 08:16</t>
+          <t>06/05/2026 04:51</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4344,20 +4344,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>06/01/2026 15:15</t>
+          <t>06/04/2026 21:52</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>19851.22</v>
+        <v>19561.84</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>-0.75</v>
+        <v>-2.19</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>1.44</v>
+        <v>2.19</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>0.48</v>
+        <v>0.24</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4366,31 +4366,31 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>19797.26</v>
+        <v>19464.84</v>
       </c>
       <c r="P35" t="n">
         <v>2</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>28.57142857142857</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>70.27180095613637</v>
+        <v>34.96447608299332</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>0.9552333333333324</v>
+        <v>1.460533333333333</v>
       </c>
       <c r="T35" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>-148.78</v>
+        <v>-298.04</v>
       </c>
       <c r="V35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W35" s="7" t="n">
         <v>16.66666666666666</v>
@@ -4402,12 +4402,12 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
@@ -4447,20 +4447,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/01/2026 18:46</t>
+          <t>06/05/2026 07:59</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19716.66</v>
+        <v>19524.18</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-1.42</v>
+        <v>-2.38</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>2.05</v>
+        <v>2.78</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.37</v>
+        <v>0.34</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4469,34 +4469,34 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
+        <v>25</v>
+      </c>
+      <c r="O36" s="7" t="n">
+        <v>19410.62</v>
+      </c>
+      <c r="P36" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q36" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="O36" s="7" t="n">
-        <v>19645.02</v>
-      </c>
-      <c r="P36" t="n">
+      <c r="R36" s="7" t="n">
+        <v>27.93993625212148</v>
+      </c>
+      <c r="S36" s="7" t="n">
+        <v>1.856550014825783</v>
+      </c>
+      <c r="T36" t="n">
+        <v>24</v>
+      </c>
+      <c r="U36" s="7" t="n">
+        <v>-475.82</v>
+      </c>
+      <c r="V36" t="n">
         <v>3</v>
       </c>
-      <c r="Q36" s="7" t="n">
-        <v>18.75</v>
-      </c>
-      <c r="R36" s="7" t="n">
-        <v>45.05366878183931</v>
-      </c>
-      <c r="S36" s="7" t="n">
-        <v>1.374412120196735</v>
-      </c>
-      <c r="T36" t="n">
-        <v>15</v>
-      </c>
-      <c r="U36" s="7" t="n">
-        <v>-283.34</v>
-      </c>
-      <c r="V36" t="n">
-        <v>2</v>
-      </c>
       <c r="W36" s="7" t="n">
-        <v>13.33333333333333</v>
+        <v>12.5</v>
       </c>
       <c r="X36" t="inlineStr">
         <is>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
@@ -4550,17 +4550,17 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/02/2026 00:38</t>
+          <t>06/05/2026 02:39</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>2380.77</v>
+        <v>2300.77</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-96.73999999999999</v>
+        <v>-96.84999999999999</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>99.38</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="K37" s="7" t="n">
         <v>0.83</v>
@@ -4575,7 +4575,7 @@
         <v>40</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>-1007.44</v>
+        <v>-834.0799999999999</v>
       </c>
       <c r="P37" t="n">
         <v>10</v>
@@ -4584,22 +4584,22 @@
         <v>25</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>0.6552629829110979</v>
+        <v>0.7028813903852018</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>11.1226856288573</v>
+        <v>11.64259250222412</v>
       </c>
       <c r="T37" t="n">
-        <v>486</v>
+        <v>494</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-18619.23</v>
+        <v>-18699.23</v>
       </c>
       <c r="V37" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>40.94650205761317</v>
+        <v>40.48582995951417</v>
       </c>
       <c r="X37" t="inlineStr">
         <is>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="Z37" t="inlineStr">
@@ -4653,20 +4653,20 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/01/2026 14:43</t>
+          <t>06/05/2026 06:47</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
-        <v>26087.98</v>
+        <v>25986.07</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>0.88</v>
+        <v>0.15</v>
       </c>
       <c r="J38" s="7" t="n">
         <v>6.56</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>1.07</v>
+        <v>0.99</v>
       </c>
       <c r="L38" t="n">
         <v>26000</v>
@@ -4675,43 +4675,43 @@
         <v>0</v>
       </c>
       <c r="N38" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>26057.87</v>
+        <v>15955.12</v>
       </c>
       <c r="P38" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q38" s="7" t="n">
-        <v>44.73684210526316</v>
+        <v>40</v>
       </c>
       <c r="R38" s="7" t="n">
-        <v>21.19303528027617</v>
+        <v>12.46628842760619</v>
       </c>
       <c r="S38" s="7" t="n">
-        <v>3.317542334367406</v>
+        <v>6.55619118278732</v>
       </c>
       <c r="T38" t="n">
         <v>16</v>
       </c>
       <c r="U38" s="7" t="n">
-        <v>441.76</v>
+        <v>414.27</v>
       </c>
       <c r="V38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>43.75</v>
+        <v>50</v>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>05/31/2026 05:27</t>
+          <t>06/03/2026 05:33</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -4859,20 +4859,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>05/31/2026 11:04</t>
+          <t>06/02/2026 16:48</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
-        <v>32539.84</v>
+        <v>32377.38</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>-8.27</v>
+        <v>-8.73</v>
       </c>
       <c r="J40" s="7" t="n">
         <v>19.72</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="L40" t="n">
         <v>25000</v>
@@ -4884,31 +4884,31 @@
         <v>40</v>
       </c>
       <c r="O40" s="7" t="n">
-        <v>-91.29999999999998</v>
+        <v>-338.09</v>
       </c>
       <c r="P40" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="Q40" s="7" t="n">
-        <v>67.5</v>
+        <v>47.5</v>
       </c>
       <c r="R40" s="7" t="n">
-        <v>0.8463816075938344</v>
+        <v>0.3975886558289881</v>
       </c>
       <c r="S40" s="7" t="n">
-        <v>2.279467522103865</v>
+        <v>2.553199999999961</v>
       </c>
       <c r="T40" t="n">
-        <v>2807</v>
+        <v>2858</v>
       </c>
       <c r="U40" s="7" t="n">
-        <v>-1830.42</v>
+        <v>-1982.55</v>
       </c>
       <c r="V40" t="n">
-        <v>1709</v>
+        <v>1712</v>
       </c>
       <c r="W40" s="7" t="n">
-        <v>60.88350552190951</v>
+        <v>59.90202939118264</v>
       </c>
       <c r="X40" t="inlineStr">
         <is>
@@ -4917,7 +4917,7 @@
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr">
@@ -4962,7 +4962,7 @@
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>05/28/2026 00:43</t>
+          <t>06/03/2026 00:51</t>
         </is>
       </c>
       <c r="H41" s="9" t="n">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>05/29/2026 09:06</t>
+          <t>06/04/2026 09:16</t>
         </is>
       </c>
       <c r="H42" s="9" t="n">
@@ -5140,7 +5140,7 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>05/29/2026 15:57</t>
+          <t>06/04/2026 16:07</t>
         </is>
       </c>
       <c r="H43" s="9" t="n">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>05/31/2026 14:18</t>
+          <t>06/03/2026 14:26</t>
         </is>
       </c>
       <c r="H45" s="9" t="n">
@@ -5407,17 +5407,17 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>06/01/2026 14:11</t>
+          <t>06/04/2026 21:35</t>
         </is>
       </c>
       <c r="H46" s="9" t="n">
-        <v>1541.65</v>
+        <v>1039.23</v>
       </c>
       <c r="I46" s="9" t="n">
-        <v>-92.45999999999999</v>
+        <v>-94.91</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>92.5</v>
+        <v>95.15000000000001</v>
       </c>
       <c r="K46" s="9" t="n">
         <v>0.67</v>
@@ -5432,19 +5432,19 @@
         <v>40</v>
       </c>
       <c r="O46" s="9" t="n">
-        <v>-1268.54</v>
+        <v>-559.42</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q46" s="9" t="n">
-        <v>22.5</v>
+        <v>30</v>
       </c>
       <c r="R46" s="9" t="n">
-        <v>0.2711634587762137</v>
+        <v>0.5254004343694856</v>
       </c>
       <c r="S46" s="9" t="n">
-        <v>12.68540000000003</v>
+        <v>6.032600000000002</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0</v>
@@ -5496,7 +5496,7 @@
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>06/01/2026 22:16</t>
+          <t>06/05/2026 09:51</t>
         </is>
       </c>
       <c r="H47" s="9" t="n">
@@ -5585,7 +5585,7 @@
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>05/31/2026 03:14</t>
+          <t>06/03/2026 03:17</t>
         </is>
       </c>
       <c r="H48" s="9" t="n">
@@ -5674,7 +5674,7 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>05/31/2026 03:10</t>
+          <t>06/03/2026 03:16</t>
         </is>
       </c>
       <c r="H49" s="9" t="n">
@@ -5763,7 +5763,7 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>06/01/2026 22:37</t>
+          <t>06/05/2026 10:18</t>
         </is>
       </c>
       <c r="H50" s="9" t="n">
@@ -5852,7 +5852,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>06/01/2026 22:41</t>
+          <t>06/04/2026 10:46</t>
         </is>
       </c>
       <c r="H51" s="9" t="n">
@@ -5941,7 +5941,7 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>06/01/2026 23:42</t>
+          <t>06/05/2026 10:55</t>
         </is>
       </c>
       <c r="H52" s="9" t="n">
@@ -6030,20 +6030,20 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>05/31/2026 21:56</t>
+          <t>06/05/2026 11:03</t>
         </is>
       </c>
       <c r="H53" s="9" t="n">
-        <v>19764.02</v>
+        <v>19710.4</v>
       </c>
       <c r="I53" s="9" t="n">
-        <v>-1.18</v>
+        <v>-1.45</v>
       </c>
       <c r="J53" s="9" t="n">
-        <v>1.22</v>
+        <v>1.49</v>
       </c>
       <c r="K53" s="9" t="n">
-        <v>0.67</v>
+        <v>0.63</v>
       </c>
       <c r="L53" s="8" t="n">
         <v>20000</v>
@@ -6055,19 +6055,19 @@
         <v>40</v>
       </c>
       <c r="O53" s="9" t="n">
-        <v>-80.88</v>
+        <v>-89.25</v>
       </c>
       <c r="P53" s="8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q53" s="9" t="n">
-        <v>22.5</v>
+        <v>12.5</v>
       </c>
       <c r="R53" s="9" t="n">
-        <v>0.04521307991972613</v>
+        <v>0.09729948417113379</v>
       </c>
       <c r="S53" s="9" t="n">
-        <v>0.8087999999999738</v>
+        <v>0.8924999999999819</v>
       </c>
       <c r="T53" s="8" t="n">
         <v>0</v>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>05/30/2026 12:06</t>
+          <t>06/05/2026 12:14</t>
         </is>
       </c>
       <c r="H54" s="9" t="n">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>06/01/2026 18:21</t>
+          <t>06/04/2026 22:54</t>
         </is>
       </c>
       <c r="H55" s="9" t="n">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>05/28/2026 00:43</t>
+          <t>06/03/2026 00:51</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>05/29/2026 09:06</t>
+          <t>06/04/2026 09:16</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -6639,7 +6639,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>05/29/2026 15:57</t>
+          <t>06/04/2026 16:07</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>05/31/2026 14:18</t>
+          <t>06/03/2026 14:26</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -6762,14 +6762,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06/01/2026 14:11</t>
+          <t>06/04/2026 21:35</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>1541.65</v>
+        <v>1039.23</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>-92.45999999999999</v>
+        <v>-94.91</v>
       </c>
       <c r="I10" t="n">
         <v>40</v>
@@ -6803,7 +6803,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>06/01/2026 22:16</t>
+          <t>06/05/2026 09:51</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -6844,7 +6844,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>05/31/2026 03:14</t>
+          <t>06/03/2026 03:17</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -6885,7 +6885,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>05/31/2026 03:10</t>
+          <t>06/03/2026 03:16</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>06/01/2026 22:37</t>
+          <t>06/05/2026 10:18</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/01/2026 22:41</t>
+          <t>06/04/2026 10:46</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/01/2026 23:42</t>
+          <t>06/05/2026 10:55</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -7049,14 +7049,14 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>05/31/2026 21:56</t>
+          <t>06/05/2026 11:03</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>19764.02</v>
+        <v>19710.4</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>-1.18</v>
+        <v>-1.45</v>
       </c>
       <c r="I17" t="n">
         <v>40</v>
@@ -7090,7 +7090,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>05/30/2026 12:06</t>
+          <t>06/05/2026 12:14</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>06/01/2026 18:21</t>
+          <t>06/04/2026 22:54</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -7868,7 +7868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>05/30/2026 20:53</t>
+          <t>06/02/2026 20:58</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06/01/2026 18:52</t>
+          <t>06/04/2026 18:57</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06/01/2026 16:52</t>
+          <t>06/04/2026 16:57</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06/01/2026 20:28</t>
+          <t>06/04/2026 20:32</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>05/31/2026 17:52</t>
+          <t>06/03/2026 17:58</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>05/29/2026 01:56</t>
+          <t>06/04/2026 02:05</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>05/31/2026 02:47</t>
+          <t>06/03/2026 02:50</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06/01/2026 05:21</t>
+          <t>06/04/2026 05:27</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
@@ -8205,7 +8205,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>05/24/2026 20:52</t>
+          <t>06/02/2026 21:04</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
@@ -8251,7 +8251,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06/01/2026 12:14</t>
+          <t>06/04/2026 12:20</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06/01/2026 11:49</t>
+          <t>06/04/2026 11:55</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -8330,58 +8330,58 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>647831</t>
+          <t>54186</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>A MOL Argos</t>
+          <t>Codex FXRSI_V3_2_Filter60</t>
         </is>
       </c>
       <c r="C22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>03/30/2026 11:54</t>
+          <t>06/05/2026 05:18</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>648289</t>
+          <t>54187</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">A-MOL Medallion </t>
+          <t>Demo Claude XAU EU SweepReclaim</t>
         </is>
       </c>
       <c r="C23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05/27/2026 20:52</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="n">
-        <v>5052.75</v>
+          <t>06/05/2026 06:03</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>20000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3038308</t>
+          <t>647831</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>A-MOL inactive Maven</t>
+          <t>A MOL Argos</t>
         </is>
       </c>
       <c r="C24" t="b">
@@ -8389,7 +8389,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05/27/2026 20:52</t>
+          <t>03/30/2026 11:54</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -8399,35 +8399,35 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>52428846</t>
+          <t>648289</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EA The5ers Low DD Dual Breakout</t>
+          <t xml:space="preserve">A-MOL Medallion </t>
         </is>
       </c>
       <c r="C25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>05/31/2026 11:44</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>41224.86</v>
+          <t>06/02/2026 21:04</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>80059994</t>
+          <t>3038308</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>A-MOL Denali Plus</t>
+          <t>A-MOL inactive Maven</t>
         </is>
       </c>
       <c r="C26" t="b">
@@ -8435,22 +8435,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06/01/2026 23:41</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>0.43</v>
+          <t>06/02/2026 21:04</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5035285664</t>
+          <t>52428846</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Manual Trades (Rvg)</t>
+          <t>EA The5ers Low DD Dual Breakout</t>
         </is>
       </c>
       <c r="C27" t="b">
@@ -8458,10 +8458,56 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
+          <t>05/31/2026 11:44</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>41224.86</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>80059994</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>A-MOL Denali Plus</t>
+        </is>
+      </c>
+      <c r="C28" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>06/05/2026 03:41</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>5035285664</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Manual Trades (Rvg)</t>
+        </is>
+      </c>
+      <c r="C29" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>07/24/2025 16:40</t>
         </is>
       </c>
-      <c r="E27" s="7" t="n">
+      <c r="E29" s="7" t="n">
         <v>5331.24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboards — 2026-06-08
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-05 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-08 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -948,14 +948,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/05/2026 08:01</t>
+          <t>06/08/2026 17:12</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>55335.24</v>
+        <v>52988.29</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>120.29</v>
+        <v>126.35</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -973,31 +973,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>1258.37</v>
+        <v>885.5799999999999</v>
       </c>
       <c r="P2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>50</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>5.156051574446028</v>
+        <v>3.860494466377581</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>0.9736289069912897</v>
+        <v>2.162305316575986</v>
       </c>
       <c r="T2" t="n">
-        <v>2710</v>
+        <v>2760</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>30335.24</v>
+        <v>27988.28999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>1735</v>
+        <v>1759</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>64.02214022140221</v>
+        <v>63.73188405797101</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -1051,20 +1051,20 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/05/2026 12:35</t>
+          <t>06/08/2026 22:15</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
-        <v>24261.61</v>
+        <v>24013.3</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>16.95</v>
+        <v>15.75</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>12.39</v>
+        <v>12.55</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="L3" s="7" t="n">
         <v>30545.04</v>
@@ -1076,31 +1076,31 @@
         <v>40</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>-6930.42</v>
+        <v>-7257.93</v>
       </c>
       <c r="P3" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="Q3" s="7" t="n">
-        <v>62.5</v>
+        <v>60</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>0.186233164755358</v>
+        <v>0.1718915952600079</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>71.45278259863474</v>
+        <v>74.29579795888873</v>
       </c>
       <c r="T3" t="n">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="U3" s="7" t="n">
-        <v>4043.48</v>
+        <v>3795.17</v>
       </c>
       <c r="V3" t="n">
         <v>548</v>
       </c>
       <c r="W3" s="7" t="n">
-        <v>62.70022883295194</v>
+        <v>62.41457858769932</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>EA Axis Rotation AUDUSD 5m | AUDUSD.pro, EA Fx RSI Prop USDCHF 10M | USDCHF.pro, Manual / one-off | GBPJPY.pro, Manual / one-off | GBPUSD.pro, Manual / one-off | NZDJPY.pro, Manual / one-off | USDJPY.pro, Manual / one-off | XAUUSD</t>
+          <t>Axis AUDUSD | AUDUSD.pro, EA Axis Rotation AUDUSD 5m | AUDUSD.pro, EA Fx RSI Prop USDCHF 10M | USDCHF.pro, Manual / one-off | GBPJPY.pro, Manual / one-off | GBPUSD.pro, Manual / one-off | NZDJPY.pro, Manual / one-off | USDJPY.pro, Manual / one-off | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -1154,20 +1154,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/05/2026 05:44</t>
+          <t>06/06/2026 08:50</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>21054.45</v>
+        <v>21232.98</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>5.24</v>
+        <v>6.13</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>5.78</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1.11</v>
+        <v>1.13</v>
       </c>
       <c r="L4" t="n">
         <v>20000</v>
@@ -1179,7 +1179,7 @@
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>534.6</v>
+        <v>537.46</v>
       </c>
       <c r="P4" t="n">
         <v>28</v>
@@ -1188,22 +1188,22 @@
         <v>70</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>1.17518906939018</v>
+        <v>1.17606872758014</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>11.15365614851094</v>
+        <v>11.33093150439226</v>
       </c>
       <c r="T4" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>1054.45</v>
+        <v>1232.98</v>
       </c>
       <c r="V4" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>64.91228070175438</v>
+        <v>65.21739130434783</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/05/2026 10:35</t>
+          <t>06/08/2026 20:09</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1403,7 +1403,7 @@
         <v>602</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>-3642.179999999999</v>
+        <v>-3642.18</v>
       </c>
       <c r="V6" t="n">
         <v>502</v>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/05/2026 03:37</t>
+          <t>06/08/2026 12:02</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/05/2026 08:11</t>
+          <t>06/08/2026 17:33</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/05/2026 04:00</t>
+          <t>06/08/2026 12:27</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1815,13 +1815,13 @@
         <v>183</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>216.0199999999999</v>
+        <v>216.02</v>
       </c>
       <c r="V10" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>45.90163934426229</v>
+        <v>46.44808743169399</v>
       </c>
       <c r="X10" t="inlineStr">
         <is>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/04/2026 21:08</t>
+          <t>06/08/2026 14:50</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -1978,20 +1978,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/04/2026 10:38</t>
+          <t>06/08/2026 19:30</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>10829.8</v>
+        <v>10883.28</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>7.57</v>
+        <v>8.1</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1.25</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>5.22</v>
+        <v>5.52</v>
       </c>
       <c r="L12" t="n">
         <v>20000</v>
@@ -2003,7 +2003,7 @@
         <v>40</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>892.8499999999999</v>
+        <v>938.0599999999999</v>
       </c>
       <c r="P12" t="n">
         <v>31</v>
@@ -2012,19 +2012,19 @@
         <v>77.5</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>1.095610266903861</v>
+        <v>1.100694865046416</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>43.69494914343316</v>
+        <v>43.58100042051737</v>
       </c>
       <c r="T12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>837.95</v>
+        <v>883.28</v>
       </c>
       <c r="V12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="W12" s="7" t="n">
         <v>100</v>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/05/2026 05:27</t>
+          <t>06/08/2026 05:29</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2184,20 +2184,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>06/05/2026 11:59</t>
+          <t>06/08/2026 21:40</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>19995.7</v>
+        <v>19748.11</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>-5.21</v>
+        <v>-6.39</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>9.75</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>0.85</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L14" s="7" t="n">
         <v>26775.1</v>
@@ -2209,31 +2209,31 @@
         <v>40</v>
       </c>
       <c r="O14" s="7" t="n">
-        <v>5678.17</v>
+        <v>5229.240000000001</v>
       </c>
       <c r="P14" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>47.5</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>1.840525317241257</v>
+        <v>1.74681039999886</v>
       </c>
       <c r="S14" s="7" t="n">
-        <v>27.67771200973612</v>
+        <v>29.09067136434657</v>
       </c>
       <c r="T14" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="U14" s="7" t="n">
-        <v>157.7200000000003</v>
+        <v>-89.86999999999986</v>
       </c>
       <c r="V14" t="n">
         <v>75</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>55.97014925373134</v>
+        <v>55.14705882352941</v>
       </c>
       <c r="X14" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Axis Rotation GBPUSD 5m V1 | GBPUSD, EA Axis Rotation EURUSD 5m 8%dd | EURUSD</t>
+          <t>Axis GBPUSD | GBPUSD, Axis Rotation GBPUSD 5m V1 | GBPUSD, EA Axis Rotation EURUSD 5m 8%dd | EURUSD</t>
         </is>
       </c>
     </row>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/05/2026 05:32</t>
+          <t>06/08/2026 14:07</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2327,16 +2327,16 @@
         <v>13.62048330434852</v>
       </c>
       <c r="T15" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-2050.370000000001</v>
+        <v>-2106.59</v>
       </c>
       <c r="V15" t="n">
         <v>48</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>44.44444444444444</v>
+        <v>43.63636363636363</v>
       </c>
       <c r="X15" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2390,20 +2390,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>06/03/2026 00:57</t>
+          <t>06/08/2026 12:53</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>10869.76</v>
+        <v>10093.84</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-96.63</v>
+        <v>-96.88</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>96.90000000000001</v>
+        <v>97.01000000000001</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="L16" t="n">
         <v>45165</v>
@@ -2415,7 +2415,7 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-28.43000000000009</v>
+        <v>-78.70999999999997</v>
       </c>
       <c r="P16" t="n">
         <v>24</v>
@@ -2424,10 +2424,10 @@
         <v>60</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>1.113935675219722</v>
+        <v>1.066652925212134</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>7.369281597233949</v>
+        <v>4.000813588843479</v>
       </c>
       <c r="T16" t="n">
         <v>3665</v>
@@ -2493,17 +2493,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>06/05/2026 01:12</t>
+          <t>06/08/2026 19:49</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>13565.63</v>
+        <v>13343.46</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>-32.2</v>
+        <v>-33.31</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>32.2</v>
+        <v>33.31</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>0.32</v>
@@ -2518,31 +2518,31 @@
         <v>40</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>-892.24</v>
+        <v>-738</v>
       </c>
       <c r="P17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q17" s="7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>0.1176598564110678</v>
+        <v>0.1870456047587574</v>
       </c>
       <c r="S17" s="7" t="n">
-        <v>8.922399999999961</v>
+        <v>7.914281339667182</v>
       </c>
       <c r="T17" t="n">
-        <v>332</v>
+        <v>352</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>-6434.369999999999</v>
+        <v>-6656.540000000001</v>
       </c>
       <c r="V17" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="W17" s="7" t="n">
-        <v>13.85542168674699</v>
+        <v>13.92045454545454</v>
       </c>
       <c r="X17" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -2596,20 +2596,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>06/05/2026 00:49</t>
+          <t>06/08/2026 19:21</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>17107.57</v>
+        <v>16743.38</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>-14.47</v>
+        <v>-16.29</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>15.5</v>
+        <v>17.52</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>0.58</v>
+        <v>0.55</v>
       </c>
       <c r="L18" t="n">
         <v>20000</v>
@@ -2621,7 +2621,7 @@
         <v>40</v>
       </c>
       <c r="O18" s="7" t="n">
-        <v>-1334.54</v>
+        <v>-1292.96</v>
       </c>
       <c r="P18" t="n">
         <v>7</v>
@@ -2630,22 +2630,22 @@
         <v>17.5</v>
       </c>
       <c r="R18" s="7" t="n">
-        <v>0.2207702727952168</v>
+        <v>0.1688328375660934</v>
       </c>
       <c r="S18" s="7" t="n">
-        <v>13.34540000000001</v>
+        <v>13.38700000000003</v>
       </c>
       <c r="T18" t="n">
-        <v>161</v>
+        <v>218</v>
       </c>
       <c r="U18" s="7" t="n">
-        <v>-1626.74</v>
+        <v>-3256.62</v>
       </c>
       <c r="V18" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="W18" s="7" t="n">
-        <v>39.75155279503105</v>
+        <v>36.69724770642202</v>
       </c>
       <c r="X18" t="inlineStr">
         <is>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>06/05/2026 09:55</t>
+          <t>06/08/2026 19:24</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2709,7 +2709,7 @@
         <v>-4.15</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>4.8</v>
+        <v>4.93</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>0.14</v>
@@ -2802,20 +2802,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>06/04/2026 09:41</t>
+          <t>06/08/2026 19:08</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
-        <v>19652.55</v>
+        <v>19845.83</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>-1.73</v>
+        <v>-0.76</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>5.42</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>0.84</v>
+        <v>0.93</v>
       </c>
       <c r="L20" t="n">
         <v>20000</v>
@@ -2827,7 +2827,7 @@
         <v>40</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>-678.3299999999999</v>
+        <v>-624.05</v>
       </c>
       <c r="P20" t="n">
         <v>18</v>
@@ -2836,10 +2836,10 @@
         <v>45</v>
       </c>
       <c r="R20" s="7" t="n">
-        <v>0.71875</v>
+        <v>0.7460797651439209</v>
       </c>
       <c r="S20" s="7" t="n">
-        <v>10.87443451666189</v>
+        <v>11.01721679093957</v>
       </c>
       <c r="T20" t="n">
         <v>44</v>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>06/05/2026 00:49</t>
+          <t>06/08/2026 09:09</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3008,20 +3008,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>06/05/2026 09:58</t>
+          <t>06/08/2026 19:25</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>16358.77</v>
-      </c>
-      <c r="I22" s="7" t="n">
-        <v>-18.22</v>
-      </c>
-      <c r="J22" s="7" t="n">
-        <v>18.22</v>
+        <v>16145.59</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-19</v>
+      </c>
+      <c r="J22" t="n">
+        <v>19</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3033,31 +3033,31 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-427.7499999999999</v>
+        <v>-559.91</v>
       </c>
       <c r="P22" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>25</v>
+        <v>17.5</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.4060289659818121</v>
+        <v>0.319404448256847</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>4.232400000000089</v>
+        <v>5.554000000000105</v>
       </c>
       <c r="T22" t="n">
-        <v>265</v>
+        <v>300</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-3373.84</v>
+        <v>-3854.41</v>
       </c>
       <c r="V22" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>34.71698113207547</v>
+        <v>32.66666666666666</v>
       </c>
       <c r="X22" t="inlineStr">
         <is>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>06/05/2026 09:59</t>
+          <t>06/08/2026 19:27</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3151,16 +3151,16 @@
         <v>4.584913432177711</v>
       </c>
       <c r="T23" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>118.8299999999999</v>
+        <v>1317.45</v>
       </c>
       <c r="V23" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>38.46153846153847</v>
+        <v>42.5531914893617</v>
       </c>
       <c r="X23" t="inlineStr">
         <is>
@@ -3169,12 +3169,12 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/05/2026 09:53</t>
+          <t>06/08/2026 19:21</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3317,20 +3317,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>06/05/2026 09:55</t>
+          <t>06/08/2026 19:23</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>20030.41</v>
+        <v>20050.38</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>4.51</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3342,7 +3342,7 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>-344.17</v>
+        <v>7.200000000000003</v>
       </c>
       <c r="P25" t="n">
         <v>31</v>
@@ -3351,22 +3351,22 @@
         <v>77.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>0.1696943378929338</v>
+        <v>1.06</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>4.134297081725435</v>
+        <v>1.184927719409116</v>
       </c>
       <c r="T25" t="n">
-        <v>632</v>
+        <v>787</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>198.1700000000002</v>
+        <v>50.37999999999984</v>
       </c>
       <c r="V25" t="n">
-        <v>406</v>
+        <v>523</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>64.24050632911393</v>
+        <v>66.4548919949174</v>
       </c>
       <c r="X25" t="inlineStr">
         <is>
@@ -3375,7 +3375,7 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>Hive 7 LTF MOL | AUDJPY.pro, Hive 7 LTF MOL | CADJPY.pro, Hive 7 LTF MOL | EURGBP.pro, Hive 7 LTF MOL | EURJPY.pro, Hive 7 LTF MOL | EURUSD.pro, Hive 7 LTF MOL | GBPJPY.pro, Hive 7 LTF MOL | GBPUSD.pro, Hive 7 LTF MOL | USDCAD.pro, Hive 7 LTF MOL | USDJPY.pro, Hive 7 LTF MOL | XAUUSD</t>
+          <t>Hive 7 LTF MOL | AUDJPY.pro, Hive 7 LTF MOL | AUDUSD.pro, Hive 7 LTF MOL | CADJPY.pro, Hive 7 LTF MOL | EURGBP.pro, Hive 7 LTF MOL | EURJPY.pro, Hive 7 LTF MOL | EURUSD.pro, Hive 7 LTF MOL | GBPJPY.pro, Hive 7 LTF MOL | GBPUSD.pro, Hive 7 LTF MOL | USDCAD.pro, Hive 7 LTF MOL | USDJPY.pro, Hive 7 LTF MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3420,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/03/2026 08:41</t>
+          <t>06/08/2026 09:30</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/03/2026 08:47</t>
+          <t>06/08/2026 19:43</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/05/2026 00:56</t>
+          <t>06/08/2026 09:20</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3669,7 +3669,7 @@
         <v>34</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>891.84</v>
+        <v>891.8399999999999</v>
       </c>
       <c r="V28" t="n">
         <v>9</v>
@@ -3729,20 +3729,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/05/2026 05:21</t>
+          <t>06/08/2026 13:57</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20462.96</v>
+        <v>20535.98</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>2.31</v>
+        <v>2.67</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>6.36</v>
+        <v>4.9</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3751,34 +3751,34 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
+        <v>17</v>
+      </c>
+      <c r="O29" s="7" t="n">
+        <v>20535.98</v>
+      </c>
+      <c r="P29" t="n">
         <v>13</v>
       </c>
-      <c r="O29" s="7" t="n">
-        <v>20462.96</v>
-      </c>
-      <c r="P29" t="n">
-        <v>10</v>
-      </c>
       <c r="Q29" s="7" t="n">
-        <v>76.92307692307693</v>
+        <v>76.47058823529412</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>238.0867802108678</v>
+        <v>150.4939215258062</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>0.1628000000000005</v>
+        <v>0.1676133901630088</v>
       </c>
       <c r="T29" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>462.96</v>
+        <v>638.15</v>
       </c>
       <c r="V29" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>75</v>
+        <v>72.22222222222221</v>
       </c>
       <c r="X29" t="inlineStr">
         <is>
@@ -3787,17 +3787,17 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo | EURUSD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US30, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCAD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCHF.pro</t>
+          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo | EURUSD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US30, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US500, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCAD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCHF.pro</t>
         </is>
       </c>
     </row>
@@ -3832,14 +3832,14 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/05/2026 03:38</t>
+          <t>06/06/2026 19:51</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>21507.01</v>
+        <v>21491.63</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>7.54</v>
+        <v>7.46</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>11.64</v>
@@ -3857,31 +3857,31 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-129.61</v>
+        <v>199.29</v>
       </c>
       <c r="P30" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>50</v>
+        <v>52.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.9496002047239146</v>
+        <v>1.094064172637422</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>9.643808533568093</v>
+        <v>7.334333015531218</v>
       </c>
       <c r="T30" t="n">
-        <v>547</v>
+        <v>614</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>1586.65</v>
+        <v>1577.179999999999</v>
       </c>
       <c r="V30" t="n">
-        <v>282</v>
+        <v>315</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>51.55393053016454</v>
+        <v>51.30293159609121</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
@@ -3935,20 +3935,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/05/2026 07:43</t>
+          <t>06/08/2026 16:42</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20613.8</v>
+        <v>20518.54</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>3.06</v>
+        <v>2.58</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>0.99</v>
+        <v>1.45</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>2.52</v>
+        <v>2.04</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -3957,34 +3957,34 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>20613.8</v>
+        <v>20518.54</v>
       </c>
       <c r="P31" t="n">
         <v>11</v>
       </c>
       <c r="Q31" s="7" t="n">
-        <v>73.33333333333333</v>
+        <v>68.75</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>52.20168902136115</v>
+        <v>42.21347366729603</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>0.6667255042947245</v>
+        <v>0.9758177348724615</v>
       </c>
       <c r="T31" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>613.8</v>
+        <v>518.54</v>
       </c>
       <c r="V31" t="n">
         <v>10</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>71.42857142857143</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X31" t="inlineStr">
         <is>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
@@ -4038,20 +4038,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/05/2026 11:57</t>
+          <t>06/08/2026 21:36</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>20692.94</v>
+        <v>21537.01</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>3.46</v>
+        <v>7.68</v>
       </c>
       <c r="J32" s="7" t="n">
         <v>1.78</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>1.9</v>
+        <v>2.56</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4060,34 +4060,34 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>20627.07</v>
+        <v>21460.34</v>
       </c>
       <c r="P32" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>54.54545454545454</v>
+        <v>60</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>27.74335711331679</v>
+        <v>22.79219662244888</v>
       </c>
       <c r="S32" s="7" t="n">
         <v>1.194162721074082</v>
       </c>
       <c r="T32" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>692.9400000000001</v>
+        <v>1537.01</v>
       </c>
       <c r="V32" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>50</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="X32" t="inlineStr">
         <is>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
@@ -4106,7 +4106,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>Claude Code Sweep Suite Portfolio | EURUSD, Claude Code Sweep Suite Portfolio | GBPUSD, Claude Code Sweep Suite Portfolio | US500, Claude Code Sweep Suite Portfolio | XAUUSD</t>
+          <t>Claude Code Sweep Suite Portfolio | EURUSD, Claude Code Sweep Suite Portfolio | GBPUSD, Claude Code Sweep Suite Portfolio | NZDUSD, Claude Code Sweep Suite Portfolio | US500, Claude Code Sweep Suite Portfolio | USDCHF, Claude Code Sweep Suite Portfolio | USDJPY, Claude Code Sweep Suite Portfolio | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -4141,17 +4141,17 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06/05/2026 04:48</t>
+          <t>06/08/2026 13:14</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>19376.4</v>
+        <v>19319.84</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>-2.18</v>
+        <v>-2.46</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>2.18</v>
+        <v>2.46</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -4163,28 +4163,28 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>19555.68</v>
+        <v>19499.12</v>
       </c>
       <c r="P33" t="n">
         <v>1</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>9.090909090909092</v>
+        <v>8.333333333333332</v>
       </c>
       <c r="R33" s="7" t="n">
-        <v>46.04051565377532</v>
+        <v>40.75976196299013</v>
       </c>
       <c r="S33" s="7" t="n">
-        <v>1.448000000000005</v>
+        <v>1.635600000000001</v>
       </c>
       <c r="T33" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>-623.5999999999999</v>
+        <v>-680.1599999999999</v>
       </c>
       <c r="V33" t="n">
         <v>0</v>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
@@ -4244,20 +4244,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>06/05/2026 04:51</t>
+          <t>06/08/2026 13:16</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>19997.36</v>
+        <v>20267.59</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0</v>
+        <v>1.34</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>0.6899999999999999</v>
       </c>
-      <c r="K34" t="n">
-        <v>0</v>
+      <c r="K34" s="7" t="n">
+        <v>2.93</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4266,40 +4266,43 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>20000</v>
+        <v>20265.56</v>
       </c>
       <c r="P34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>100</v>
+        <v>75</v>
+      </c>
+      <c r="R34" s="7" t="n">
+        <v>146.9849467012388</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>0</v>
+        <v>0.4565995305746404</v>
       </c>
       <c r="T34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>-2.64</v>
+        <v>267.59</v>
       </c>
       <c r="V34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
@@ -4344,20 +4347,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>06/04/2026 21:52</t>
+          <t>06/08/2026 15:49</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>19561.84</v>
+        <v>19516.25</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>-2.19</v>
+        <v>-2.42</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>2.19</v>
+        <v>2.42</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>0.24</v>
+        <v>0.36</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4366,34 +4369,34 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>19464.84</v>
+        <v>19381.69</v>
       </c>
       <c r="P35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>16.66666666666666</v>
+        <v>18.75</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>34.96447608299332</v>
+        <v>26.62330961321324</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>1.460533333333333</v>
+        <v>1.6125</v>
       </c>
       <c r="T35" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>-298.04</v>
+        <v>-483.75</v>
       </c>
       <c r="V35" t="n">
         <v>2</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>16.66666666666666</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="X35" t="inlineStr">
         <is>
@@ -4402,12 +4405,12 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
@@ -4447,20 +4450,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/05/2026 07:59</t>
+          <t>06/08/2026 17:03</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19524.18</v>
+        <v>19664.21</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-2.38</v>
+        <v>-1.68</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>2.78</v>
+        <v>3.31</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.34</v>
+        <v>0.64</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4469,34 +4472,34 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>19410.62</v>
+        <v>19502.29</v>
       </c>
       <c r="P36" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q36" s="7" t="n">
-        <v>16</v>
+        <v>23.52941176470588</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>27.93993625212148</v>
+        <v>22.29774721109065</v>
       </c>
       <c r="S36" s="7" t="n">
-        <v>1.856550014825783</v>
+        <v>2.211704542281449</v>
       </c>
       <c r="T36" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-520.37</v>
+        <v>-335.79</v>
       </c>
       <c r="V36" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>12</v>
+        <v>21.21212121212121</v>
       </c>
       <c r="X36" t="inlineStr">
         <is>
@@ -4505,12 +4508,12 @@
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
@@ -4550,14 +4553,14 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/05/2026 02:39</t>
+          <t>06/08/2026 21:22</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>2300.77</v>
+        <v>2408.97</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-96.84999999999999</v>
+        <v>-96.70999999999999</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>99.40000000000001</v>
@@ -4575,31 +4578,31 @@
         <v>40</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>-834.0799999999999</v>
+        <v>-1384.64</v>
       </c>
       <c r="P37" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q37" s="7" t="n">
-        <v>25</v>
+        <v>27.5</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>0.7028813903852018</v>
+        <v>0.3263863475566616</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>11.64259250222412</v>
+        <v>12.37165935380934</v>
       </c>
       <c r="T37" t="n">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-18699.23</v>
+        <v>-18565.23</v>
       </c>
       <c r="V37" t="n">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>40.48582995951417</v>
+        <v>41.15308151093439</v>
       </c>
       <c r="X37" t="inlineStr">
         <is>
@@ -4608,7 +4611,7 @@
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z37" t="inlineStr">
@@ -4653,7 +4656,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/05/2026 06:47</t>
+          <t>06/08/2026 15:39</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4693,20 +4696,20 @@
         <v>6.55619118278732</v>
       </c>
       <c r="T38" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="U38" s="7" t="n">
-        <v>414.27</v>
+        <v>233.7000000000001</v>
       </c>
       <c r="V38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>50</v>
+        <v>46.66666666666666</v>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -4756,7 +4759,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>06/03/2026 05:33</t>
+          <t>06/06/2026 05:37</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -4859,20 +4862,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/02/2026 16:48</t>
+          <t>06/07/2026 21:16</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
-        <v>32377.38</v>
+        <v>30024.24</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>-8.73</v>
+        <v>-16.72</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>19.72</v>
+        <v>24.31</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>0.92</v>
+        <v>0.84</v>
       </c>
       <c r="L40" t="n">
         <v>25000</v>
@@ -4884,31 +4887,31 @@
         <v>40</v>
       </c>
       <c r="O40" s="7" t="n">
-        <v>-338.09</v>
+        <v>-2071.15</v>
       </c>
       <c r="P40" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="Q40" s="7" t="n">
-        <v>47.5</v>
+        <v>0</v>
       </c>
       <c r="R40" s="7" t="n">
-        <v>0.3975886558289881</v>
+        <v>0</v>
       </c>
       <c r="S40" s="7" t="n">
-        <v>2.553199999999961</v>
+        <v>16.98290000000001</v>
       </c>
       <c r="T40" t="n">
-        <v>2858</v>
+        <v>2888</v>
       </c>
       <c r="U40" s="7" t="n">
-        <v>-1982.55</v>
+        <v>-4477.129999999999</v>
       </c>
       <c r="V40" t="n">
-        <v>1712</v>
+        <v>1732</v>
       </c>
       <c r="W40" s="7" t="n">
-        <v>59.90202939118264</v>
+        <v>59.97229916897508</v>
       </c>
       <c r="X40" t="inlineStr">
         <is>
@@ -4917,7 +4920,7 @@
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr">
@@ -4962,7 +4965,7 @@
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>06/03/2026 00:51</t>
+          <t>06/06/2026 00:52</t>
         </is>
       </c>
       <c r="H41" s="9" t="n">
@@ -5051,7 +5054,7 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>06/04/2026 09:16</t>
+          <t>06/07/2026 09:20</t>
         </is>
       </c>
       <c r="H42" s="9" t="n">
@@ -5229,7 +5232,7 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>05/31/2026 19:47</t>
+          <t>06/06/2026 19:59</t>
         </is>
       </c>
       <c r="H44" s="9" t="n">
@@ -5407,17 +5410,17 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>06/04/2026 21:35</t>
+          <t>06/07/2026 21:02</t>
         </is>
       </c>
       <c r="H46" s="9" t="n">
-        <v>1039.23</v>
+        <v>595.95</v>
       </c>
       <c r="I46" s="9" t="n">
-        <v>-94.91</v>
+        <v>-97.09</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>95.15000000000001</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="K46" s="9" t="n">
         <v>0.67</v>
@@ -5432,19 +5435,19 @@
         <v>40</v>
       </c>
       <c r="O46" s="9" t="n">
-        <v>-559.42</v>
+        <v>-786.8200000000001</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="Q46" s="9" t="n">
-        <v>30</v>
+        <v>37.5</v>
       </c>
       <c r="R46" s="9" t="n">
-        <v>0.5254004343694856</v>
+        <v>0.3209576083954708</v>
       </c>
       <c r="S46" s="9" t="n">
-        <v>6.032600000000002</v>
+        <v>7.868199999999979</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0</v>
@@ -5496,7 +5499,7 @@
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>06/05/2026 09:51</t>
+          <t>06/08/2026 19:19</t>
         </is>
       </c>
       <c r="H47" s="9" t="n">
@@ -5674,7 +5677,7 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>06/03/2026 03:16</t>
+          <t>06/06/2026 03:22</t>
         </is>
       </c>
       <c r="H49" s="9" t="n">
@@ -5763,7 +5766,7 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>06/05/2026 10:18</t>
+          <t>06/08/2026 19:53</t>
         </is>
       </c>
       <c r="H50" s="9" t="n">
@@ -5852,7 +5855,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>06/04/2026 10:46</t>
+          <t>06/08/2026 00:28</t>
         </is>
       </c>
       <c r="H51" s="9" t="n">
@@ -5941,7 +5944,7 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>06/05/2026 10:55</t>
+          <t>06/08/2026 20:42</t>
         </is>
       </c>
       <c r="H52" s="9" t="n">
@@ -6030,7 +6033,7 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>06/05/2026 11:03</t>
+          <t>06/08/2026 20:37</t>
         </is>
       </c>
       <c r="H53" s="9" t="n">
@@ -6119,7 +6122,7 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>06/05/2026 12:14</t>
+          <t>06/08/2026 12:19</t>
         </is>
       </c>
       <c r="H54" s="9" t="n">
@@ -6386,7 +6389,7 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>05/31/2026 11:51</t>
+          <t>06/06/2026 12:02</t>
         </is>
       </c>
       <c r="H57" s="9" t="n">
@@ -6557,7 +6560,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>06/03/2026 00:51</t>
+          <t>06/06/2026 00:52</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -6598,7 +6601,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>06/04/2026 09:16</t>
+          <t>06/07/2026 09:20</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -6680,7 +6683,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>05/31/2026 19:47</t>
+          <t>06/06/2026 19:59</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -6762,14 +6765,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06/04/2026 21:35</t>
+          <t>06/07/2026 21:02</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>1039.23</v>
+        <v>595.95</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>-94.91</v>
+        <v>-97.09</v>
       </c>
       <c r="I10" t="n">
         <v>40</v>
@@ -6803,7 +6806,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>06/05/2026 09:51</t>
+          <t>06/08/2026 19:19</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -6885,7 +6888,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>06/03/2026 03:16</t>
+          <t>06/06/2026 03:22</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -6926,7 +6929,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>06/05/2026 10:18</t>
+          <t>06/08/2026 19:53</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -6967,7 +6970,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/04/2026 10:46</t>
+          <t>06/08/2026 00:28</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -7008,7 +7011,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/05/2026 10:55</t>
+          <t>06/08/2026 20:42</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -7049,7 +7052,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>06/05/2026 11:03</t>
+          <t>06/08/2026 20:37</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -7090,7 +7093,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>06/05/2026 12:14</t>
+          <t>06/08/2026 12:19</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -7213,7 +7216,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>05/31/2026 11:51</t>
+          <t>06/06/2026 12:02</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -8179,7 +8182,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06/02/2026 20:58</t>
+          <t>06/08/2026 21:10</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -8202,7 +8205,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>05/25/2026 20:19</t>
+          <t>06/06/2026 20:44</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -8225,7 +8228,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>05/30/2026 20:53</t>
+          <t>06/08/2026 21:07</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -8248,7 +8251,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>06/04/2026 18:57</t>
+          <t>06/07/2026 18:59</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -8271,7 +8274,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06/01/2026 12:18</t>
+          <t>06/07/2026 12:29</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -8294,7 +8297,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>05/31/2026 17:48</t>
+          <t>06/06/2026 18:00</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -8317,7 +8320,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>06/04/2026 16:57</t>
+          <t>06/07/2026 17:02</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
@@ -8340,7 +8343,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06/04/2026 20:32</t>
+          <t>06/07/2026 20:38</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -8386,7 +8389,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06/04/2026 02:05</t>
+          <t>06/07/2026 02:11</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -8409,7 +8412,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06/03/2026 02:50</t>
+          <t>06/06/2026 02:54</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -8455,7 +8458,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06/02/2026 21:04</t>
+          <t>06/08/2026 21:14</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
@@ -8501,7 +8504,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06/04/2026 12:20</t>
+          <t>06/07/2026 12:24</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -8524,7 +8527,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06/04/2026 11:55</t>
+          <t>06/07/2026 12:00</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -8547,7 +8550,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>05/28/2026 08:00</t>
+          <t>06/06/2026 08:11</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
@@ -8570,7 +8573,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06/01/2026 18:29</t>
+          <t>06/07/2026 18:36</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -8593,11 +8596,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06/05/2026 05:18</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>20000</v>
+          <t>06/08/2026 13:46</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>20019.58</v>
       </c>
     </row>
     <row r="23">
@@ -8616,7 +8619,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06/05/2026 06:03</t>
+          <t>06/08/2026 14:43</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -8662,7 +8665,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06/02/2026 21:04</t>
+          <t>06/08/2026 21:11</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -8685,7 +8688,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06/02/2026 21:04</t>
+          <t>06/08/2026 21:14</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -8731,7 +8734,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06/05/2026 03:41</t>
+          <t>06/07/2026 23:34</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-06-09
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-08 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-09 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -948,14 +948,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/08/2026 17:12</t>
+          <t>06/09/2026 03:25</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>52988.29</v>
+        <v>53013.57</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>126.35</v>
+        <v>126.46</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -973,31 +973,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>885.5799999999999</v>
+        <v>639.8099999999999</v>
       </c>
       <c r="P2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>50</v>
+        <v>47.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>3.860494466377581</v>
+        <v>3.056970789990661</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>2.162305316575986</v>
+        <v>2.220799999999999</v>
       </c>
       <c r="T2" t="n">
-        <v>2760</v>
+        <v>2771</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>27988.28999999999</v>
+        <v>28782.59999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>1759</v>
+        <v>1765</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.73188405797101</v>
+        <v>63.69541681703355</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/08/2026 22:15</t>
+          <t>06/09/2026 10:18</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/06/2026 08:50</t>
+          <t>06/09/2026 00:46</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/08/2026 20:09</t>
+          <t>06/09/2026 06:32</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2026 12:02</t>
+          <t>06/09/2026 10:35</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/08/2026 17:33</t>
+          <t>06/09/2026 03:43</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/2026 12:27</t>
+          <t>06/09/2026 21:15</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/08/2026 14:50</t>
+          <t>06/09/2026 01:11</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -1978,20 +1978,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/08/2026 19:30</t>
+          <t>06/09/2026 05:46</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>10883.28</v>
+        <v>10899.63</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>8.1</v>
+        <v>8.26</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1.25</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>5.52</v>
+        <v>5.61</v>
       </c>
       <c r="L12" t="n">
         <v>20000</v>
@@ -2003,7 +2003,7 @@
         <v>40</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>938.0599999999999</v>
+        <v>946.0899999999999</v>
       </c>
       <c r="P12" t="n">
         <v>31</v>
@@ -2012,19 +2012,19 @@
         <v>77.5</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>1.100694865046416</v>
+        <v>1.101771049925969</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>43.58100042051737</v>
+        <v>43.55695867347883</v>
       </c>
       <c r="T12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>883.28</v>
+        <v>899.63</v>
       </c>
       <c r="V12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="W12" s="7" t="n">
         <v>100</v>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>06/08/2026 21:40</t>
+          <t>06/09/2026 08:46</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -2287,14 +2287,14 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/08/2026 14:07</t>
+          <t>06/09/2026 00:29</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>17949.63</v>
+        <v>17893.41</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-10.28</v>
+        <v>-10.56</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>12.67</v>
@@ -2312,7 +2312,7 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>-917.0600000000002</v>
+        <v>-806.6600000000001</v>
       </c>
       <c r="P15" t="n">
         <v>18</v>
@@ -2321,22 +2321,22 @@
         <v>45</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>0.7516891982547187</v>
+        <v>0.7746376050129693</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>13.62048330434852</v>
+        <v>13.40421922914926</v>
       </c>
       <c r="T15" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-2106.59</v>
+        <v>-2136.53</v>
       </c>
       <c r="V15" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>43.63636363636363</v>
+        <v>44.14414414414414</v>
       </c>
       <c r="X15" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>06/08/2026 12:53</t>
+          <t>06/08/2026 23:22</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2493,17 +2493,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>06/08/2026 19:49</t>
+          <t>06/09/2026 06:09</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>13343.46</v>
+        <v>13289.92</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>-33.31</v>
+        <v>-33.58</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>33.31</v>
+        <v>33.58</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>0.32</v>
@@ -2518,31 +2518,31 @@
         <v>40</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>-738</v>
+        <v>-818.9</v>
       </c>
       <c r="P17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q17" s="7" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>0.1870456047587574</v>
+        <v>0.1201057291442816</v>
       </c>
       <c r="S17" s="7" t="n">
-        <v>7.914281339667182</v>
+        <v>8.188999999999941</v>
       </c>
       <c r="T17" t="n">
-        <v>352</v>
+        <v>363</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>-6656.540000000001</v>
+        <v>-6974.449999999999</v>
       </c>
       <c r="V17" t="n">
         <v>49</v>
       </c>
       <c r="W17" s="7" t="n">
-        <v>13.92045454545454</v>
+        <v>13.49862258953168</v>
       </c>
       <c r="X17" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -2596,20 +2596,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>06/08/2026 19:21</t>
+          <t>06/09/2026 05:36</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>16743.38</v>
+        <v>16810.55</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>-16.29</v>
+        <v>-15.95</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>17.52</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="L18" t="n">
         <v>20000</v>
@@ -2621,31 +2621,31 @@
         <v>40</v>
       </c>
       <c r="O18" s="7" t="n">
-        <v>-1292.96</v>
+        <v>-1169</v>
       </c>
       <c r="P18" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q18" s="7" t="n">
-        <v>17.5</v>
+        <v>22.5</v>
       </c>
       <c r="R18" s="7" t="n">
-        <v>0.1688328375660934</v>
+        <v>0.2376980273833341</v>
       </c>
       <c r="S18" s="7" t="n">
-        <v>13.38700000000003</v>
+        <v>12.81910000000002</v>
       </c>
       <c r="T18" t="n">
-        <v>218</v>
+        <v>243</v>
       </c>
       <c r="U18" s="7" t="n">
-        <v>-3256.62</v>
+        <v>-2926.83</v>
       </c>
       <c r="V18" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="W18" s="7" t="n">
-        <v>36.69724770642202</v>
+        <v>36.21399176954733</v>
       </c>
       <c r="X18" t="inlineStr">
         <is>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>06/08/2026 19:24</t>
+          <t>06/09/2026 05:39</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>06/08/2026 19:08</t>
+          <t>06/09/2026 05:18</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>06/08/2026 09:09</t>
+          <t>06/09/2026 05:33</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3008,14 +3008,14 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>06/08/2026 19:25</t>
+          <t>06/09/2026 05:41</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>16145.59</v>
-      </c>
-      <c r="I22" t="n">
-        <v>-19</v>
+        <v>16167.88</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>-18.89</v>
       </c>
       <c r="J22" t="n">
         <v>19</v>
@@ -3033,31 +3033,31 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-559.91</v>
+        <v>-378.76</v>
       </c>
       <c r="P22" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>17.5</v>
+        <v>25</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.319404448256847</v>
+        <v>0.4334438439529498</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>5.554000000000105</v>
+        <v>4.927251001616692</v>
       </c>
       <c r="T22" t="n">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-3854.41</v>
+        <v>-3891.85</v>
       </c>
       <c r="V22" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>32.66666666666666</v>
+        <v>33.2258064516129</v>
       </c>
       <c r="X22" t="inlineStr">
         <is>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
@@ -3111,20 +3111,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>06/08/2026 19:27</t>
+          <t>06/09/2026 05:42</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>21317.45</v>
+        <v>21240.81</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>1.94</v>
+        <v>1.57</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>2.34</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>1.23</v>
+        <v>1.18</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3136,31 +3136,31 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>415.9</v>
+        <v>330.88</v>
       </c>
       <c r="P23" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>42.5</v>
+        <v>40</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.265024717625593</v>
+        <v>1.205355818208793</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.584913432177711</v>
+        <v>4.589764065335722</v>
       </c>
       <c r="T23" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>1317.45</v>
+        <v>1287.26</v>
       </c>
       <c r="V23" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>42.5531914893617</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="X23" t="inlineStr">
         <is>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/08/2026 19:21</t>
+          <t>06/09/2026 05:37</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3317,20 +3317,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>06/08/2026 19:23</t>
+          <t>06/09/2026 05:38</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>20050.38</v>
+        <v>19476.21</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>0.26</v>
+        <v>-2.61</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>4.51</v>
+        <v>7.09</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>1.02</v>
+        <v>0.86</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3342,31 +3342,31 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>7.200000000000003</v>
+        <v>-444.95</v>
       </c>
       <c r="P25" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>77.5</v>
+        <v>30</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.06</v>
+        <v>0.09435997638965216</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>1.184927719409116</v>
+        <v>4.768964986333255</v>
       </c>
       <c r="T25" t="n">
-        <v>787</v>
+        <v>884</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>50.37999999999984</v>
+        <v>-312.1400000000001</v>
       </c>
       <c r="V25" t="n">
-        <v>523</v>
+        <v>585</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>66.4548919949174</v>
+        <v>66.17647058823529</v>
       </c>
       <c r="X25" t="inlineStr">
         <is>
@@ -3375,7 +3375,7 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/08/2026 19:43</t>
+          <t>06/09/2026 06:03</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/08/2026 09:20</t>
+          <t>06/09/2026 05:50</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3729,20 +3729,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/08/2026 13:57</t>
+          <t>06/09/2026 00:22</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20535.98</v>
+        <v>20649.74</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>2.67</v>
+        <v>3.24</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>4.9</v>
+        <v>5.73</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3751,34 +3751,34 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>20535.98</v>
+        <v>20649.74</v>
       </c>
       <c r="P29" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>76.47058823529412</v>
+        <v>78.94736842105263</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>150.4939215258062</v>
+        <v>151.3220499381233</v>
       </c>
       <c r="S29" s="7" t="n">
         <v>0.1676133901630088</v>
       </c>
       <c r="T29" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>638.15</v>
+        <v>649.74</v>
       </c>
       <c r="V29" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>72.22222222222221</v>
+        <v>73.68421052631578</v>
       </c>
       <c r="X29" t="inlineStr">
         <is>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
@@ -3872,16 +3872,16 @@
         <v>7.334333015531218</v>
       </c>
       <c r="T30" t="n">
-        <v>614</v>
+        <v>655</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>1577.179999999999</v>
+        <v>2087.1</v>
       </c>
       <c r="V30" t="n">
-        <v>315</v>
+        <v>338</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>51.30293159609121</v>
+        <v>51.6030534351145</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/08/2026 16:42</t>
+          <t>06/09/2026 02:56</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/08/2026 21:36</t>
+          <t>06/09/2026 08:39</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4078,16 +4078,16 @@
         <v>1.194162721074082</v>
       </c>
       <c r="T32" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>1537.01</v>
+        <v>1318.52</v>
       </c>
       <c r="V32" t="n">
         <v>8</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>57.14285714285714</v>
+        <v>47.05882352941176</v>
       </c>
       <c r="X32" t="inlineStr">
         <is>
@@ -4096,12 +4096,12 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06/08/2026 13:14</t>
+          <t>06/08/2026 23:49</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>06/08/2026 13:16</t>
+          <t>06/08/2026 23:52</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>06/08/2026 15:49</t>
+          <t>06/09/2026 02:06</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4387,16 +4387,16 @@
         <v>1.6125</v>
       </c>
       <c r="T35" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>-483.75</v>
+        <v>-458.6099999999999</v>
       </c>
       <c r="V35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>13.33333333333333</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="X35" t="inlineStr">
         <is>
@@ -4405,12 +4405,12 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
@@ -4450,7 +4450,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/08/2026 17:03</t>
+          <t>06/09/2026 03:15</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4490,16 +4490,16 @@
         <v>2.211704542281449</v>
       </c>
       <c r="T36" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-335.79</v>
+        <v>-311.29</v>
       </c>
       <c r="V36" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>21.21212121212121</v>
+        <v>22.22222222222222</v>
       </c>
       <c r="X36" t="inlineStr">
         <is>
@@ -4508,12 +4508,12 @@
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/08/2026 21:22</t>
+          <t>06/09/2026 08:20</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4593,16 +4593,16 @@
         <v>12.37165935380934</v>
       </c>
       <c r="T37" t="n">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-18565.23</v>
+        <v>-18654.03000000001</v>
       </c>
       <c r="V37" t="n">
         <v>207</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>41.15308151093439</v>
+        <v>40.90909090909091</v>
       </c>
       <c r="X37" t="inlineStr">
         <is>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z37" t="inlineStr">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/08/2026 15:39</t>
+          <t>06/09/2026 02:03</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4696,16 +4696,16 @@
         <v>6.55619118278732</v>
       </c>
       <c r="T38" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="U38" s="7" t="n">
-        <v>233.7000000000001</v>
+        <v>207.75</v>
       </c>
       <c r="V38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>46.66666666666666</v>
+        <v>44.44444444444444</v>
       </c>
       <c r="X38" t="inlineStr">
         <is>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>06/06/2026 05:37</t>
+          <t>06/09/2026 05:40</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -4902,16 +4902,16 @@
         <v>16.98290000000001</v>
       </c>
       <c r="T40" t="n">
-        <v>2888</v>
+        <v>2900</v>
       </c>
       <c r="U40" s="7" t="n">
-        <v>-4477.129999999999</v>
+        <v>-4701.099999999999</v>
       </c>
       <c r="V40" t="n">
-        <v>1732</v>
+        <v>1736</v>
       </c>
       <c r="W40" s="7" t="n">
-        <v>59.97229916897508</v>
+        <v>59.86206896551725</v>
       </c>
       <c r="X40" t="inlineStr">
         <is>
@@ -4920,7 +4920,7 @@
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>06/06/2026 00:52</t>
+          <t>06/09/2026 00:55</t>
         </is>
       </c>
       <c r="H41" s="9" t="n">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>06/06/2026 19:59</t>
+          <t>06/09/2026 20:14</t>
         </is>
       </c>
       <c r="H44" s="9" t="n">
@@ -5321,7 +5321,7 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>06/03/2026 14:26</t>
+          <t>06/09/2026 16:20</t>
         </is>
       </c>
       <c r="H45" s="9" t="n">
@@ -5410,14 +5410,14 @@
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>06/07/2026 21:02</t>
+          <t>06/09/2026 01:45</t>
         </is>
       </c>
       <c r="H46" s="9" t="n">
-        <v>595.95</v>
+        <v>955.64</v>
       </c>
       <c r="I46" s="9" t="n">
-        <v>-97.09</v>
+        <v>-95.33</v>
       </c>
       <c r="J46" s="9" t="n">
         <v>97.09999999999999</v>
@@ -5435,19 +5435,19 @@
         <v>40</v>
       </c>
       <c r="O46" s="9" t="n">
-        <v>-786.8200000000001</v>
+        <v>-16.92000000000001</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="Q46" s="9" t="n">
-        <v>37.5</v>
+        <v>42.5</v>
       </c>
       <c r="R46" s="9" t="n">
-        <v>0.3209576083954708</v>
+        <v>0.9750923731433366</v>
       </c>
       <c r="S46" s="9" t="n">
-        <v>7.868199999999979</v>
+        <v>3.766099999999987</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0</v>
@@ -5499,7 +5499,7 @@
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>06/08/2026 19:19</t>
+          <t>06/09/2026 05:33</t>
         </is>
       </c>
       <c r="H47" s="9" t="n">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>06/06/2026 03:22</t>
+          <t>06/09/2026 03:25</t>
         </is>
       </c>
       <c r="H49" s="9" t="n">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>06/08/2026 19:53</t>
+          <t>06/09/2026 06:14</t>
         </is>
       </c>
       <c r="H50" s="9" t="n">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>06/08/2026 00:28</t>
+          <t>06/09/2026 05:56</t>
         </is>
       </c>
       <c r="H51" s="9" t="n">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>06/08/2026 20:42</t>
+          <t>06/09/2026 07:13</t>
         </is>
       </c>
       <c r="H52" s="9" t="n">
@@ -6033,7 +6033,7 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>06/08/2026 20:37</t>
+          <t>06/09/2026 07:06</t>
         </is>
       </c>
       <c r="H53" s="9" t="n">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>06/06/2026 12:02</t>
+          <t>06/09/2026 14:03</t>
         </is>
       </c>
       <c r="H57" s="9" t="n">
@@ -6560,7 +6560,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>06/06/2026 00:52</t>
+          <t>06/09/2026 00:55</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>06/06/2026 19:59</t>
+          <t>06/09/2026 20:14</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -6724,7 +6724,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>06/03/2026 14:26</t>
+          <t>06/09/2026 16:20</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -6765,14 +6765,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06/07/2026 21:02</t>
+          <t>06/09/2026 01:45</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>595.95</v>
+        <v>955.64</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>-97.09</v>
+        <v>-95.33</v>
       </c>
       <c r="I10" t="n">
         <v>40</v>
@@ -6806,7 +6806,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>06/08/2026 19:19</t>
+          <t>06/09/2026 05:33</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>06/06/2026 03:22</t>
+          <t>06/09/2026 03:25</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -6929,7 +6929,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>06/08/2026 19:53</t>
+          <t>06/09/2026 06:14</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -6970,7 +6970,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/08/2026 00:28</t>
+          <t>06/09/2026 05:56</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/08/2026 20:42</t>
+          <t>06/09/2026 07:13</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -7052,7 +7052,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>06/08/2026 20:37</t>
+          <t>06/09/2026 07:06</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -7216,7 +7216,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>06/06/2026 12:02</t>
+          <t>06/09/2026 14:03</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -8205,7 +8205,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06/06/2026 20:44</t>
+          <t>06/09/2026 20:50</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -8366,7 +8366,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06/03/2026 17:58</t>
+          <t>06/09/2026 18:29</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -8412,7 +8412,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06/06/2026 02:54</t>
+          <t>06/09/2026 02:58</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>06/06/2026 08:11</t>
+          <t>06/09/2026 08:18</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06/08/2026 14:43</t>
+          <t>06/09/2026 01:08</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -8711,7 +8711,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>05/31/2026 11:44</t>
+          <t>06/09/2026 13:56</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -8734,7 +8734,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06/07/2026 23:34</t>
+          <t>06/08/2026 23:36</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-06-10
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-09 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-10 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -988,16 +988,16 @@
         <v>2.220799999999999</v>
       </c>
       <c r="T2" t="n">
-        <v>2771</v>
+        <v>2784</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>28782.59999999999</v>
+        <v>27405.29999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>1765</v>
+        <v>1769</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.69541681703355</v>
+        <v>63.54166666666666</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -1094,7 +1094,7 @@
         <v>878</v>
       </c>
       <c r="U3" s="7" t="n">
-        <v>3795.17</v>
+        <v>3626.77</v>
       </c>
       <c r="V3" t="n">
         <v>548</v>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -1154,20 +1154,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/09/2026 00:46</t>
+          <t>06/10/2026 11:38</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>21232.98</v>
-      </c>
-      <c r="I4" s="7" t="n">
-        <v>6.13</v>
+        <v>21407.88</v>
+      </c>
+      <c r="I4" t="n">
+        <v>7</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>5.78</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1.13</v>
+        <v>1.15</v>
       </c>
       <c r="L4" t="n">
         <v>20000</v>
@@ -1179,7 +1179,7 @@
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>537.46</v>
+        <v>537.0200000000001</v>
       </c>
       <c r="P4" t="n">
         <v>28</v>
@@ -1188,22 +1188,22 @@
         <v>70</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>1.17606872758014</v>
+        <v>1.176005894852286</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>11.33093150439226</v>
+        <v>11.51358332205727</v>
       </c>
       <c r="T4" t="n">
         <v>115</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>1232.98</v>
+        <v>1407.88</v>
       </c>
       <c r="V4" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>65.21739130434783</v>
+        <v>66.08695652173913</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -1403,7 +1403,7 @@
         <v>602</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>-3642.18</v>
+        <v>-3642.179999999999</v>
       </c>
       <c r="V6" t="n">
         <v>502</v>
@@ -1609,7 +1609,7 @@
         <v>294</v>
       </c>
       <c r="U8" s="7" t="n">
-        <v>-173.1400000000001</v>
+        <v>-173.1400000000002</v>
       </c>
       <c r="V8" t="n">
         <v>263</v>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/09/2026 01:11</t>
+          <t>06/10/2026 13:46</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2018,13 +2018,13 @@
         <v>43.55695867347883</v>
       </c>
       <c r="T12" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>899.63</v>
+        <v>907.0700000000001</v>
       </c>
       <c r="V12" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W12" s="7" t="n">
         <v>100</v>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -2124,7 +2124,7 @@
         <v>38</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>-79.45999999999999</v>
+        <v>-79.45999999999997</v>
       </c>
       <c r="V13" t="n">
         <v>31</v>
@@ -2227,13 +2227,13 @@
         <v>136</v>
       </c>
       <c r="U14" s="7" t="n">
-        <v>-89.86999999999986</v>
+        <v>-64.78999999999982</v>
       </c>
       <c r="V14" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>55.14705882352941</v>
+        <v>56.61764705882353</v>
       </c>
       <c r="X14" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -2287,17 +2287,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/09/2026 00:29</t>
+          <t>06/10/2026 10:05</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>17893.41</v>
+        <v>17860.53</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-10.56</v>
+        <v>-10.72</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>12.67</v>
+        <v>13.19</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>0.8</v>
@@ -2312,7 +2312,7 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>-806.6600000000001</v>
+        <v>-688.3600000000001</v>
       </c>
       <c r="P15" t="n">
         <v>18</v>
@@ -2321,22 +2321,22 @@
         <v>45</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>0.7746376050129693</v>
+        <v>0.8063780378832173</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>13.40421922914926</v>
+        <v>14.21174568712316</v>
       </c>
       <c r="T15" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-2136.53</v>
+        <v>-1972.59</v>
       </c>
       <c r="V15" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>44.14414414414414</v>
+        <v>44.73684210526316</v>
       </c>
       <c r="X15" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>06/08/2026 23:22</t>
+          <t>06/10/2026 00:01</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2636,16 +2636,16 @@
         <v>12.81910000000002</v>
       </c>
       <c r="T18" t="n">
-        <v>243</v>
+        <v>266</v>
       </c>
       <c r="U18" s="7" t="n">
-        <v>-2926.83</v>
+        <v>-3237.27</v>
       </c>
       <c r="V18" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="W18" s="7" t="n">
-        <v>36.21399176954733</v>
+        <v>37.59398496240601</v>
       </c>
       <c r="X18" t="inlineStr">
         <is>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Hive V3 Forex HTF MOL | AUDJPY.pro, Hive V3 Forex HTF MOL | AUDUSD.pro, Hive V3 Forex HTF MOL | CADJPY.pro, Hive V3 Forex HTF MOL | CHFJPY.pro, Hive V3 Forex HTF MOL | EURCAD.pro, Hive V3 Forex HTF MOL | EURUSD.pro, Hive V3 Forex HTF MOL | GBPJPY.pro, Hive V3 Forex HTF MOL | GBPUSD.pro, Hive V3 Forex HTF MOL | USDCAD.pro, Hive V3 Forex HTF MOL | USDJPY.pro</t>
+          <t>Hive V3 Forex HTF MOL | AUDJPY.pro, Hive V3 Forex HTF MOL | AUDUSD.pro, Hive V3 Forex HTF MOL | CADJPY.pro, Hive V3 Forex HTF MOL | CHFJPY.pro, Hive V3 Forex HTF MOL | EURCAD.pro, Hive V3 Forex HTF MOL | EURUSD.pro, Hive V3 Forex HTF MOL | GBPCHF.pro, Hive V3 Forex HTF MOL | GBPJPY.pro, Hive V3 Forex HTF MOL | GBPUSD.pro, Hive V3 Forex HTF MOL | USDCAD.pro, Hive V3 Forex HTF MOL | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
         <v>44</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-154.17</v>
+        <v>-154.1700000000001</v>
       </c>
       <c r="V20" t="n">
         <v>23</v>
@@ -3048,16 +3048,16 @@
         <v>4.927251001616692</v>
       </c>
       <c r="T22" t="n">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-3891.85</v>
+        <v>-3976.779999999999</v>
       </c>
       <c r="V22" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>33.2258064516129</v>
+        <v>33.22884012539185</v>
       </c>
       <c r="X22" t="inlineStr">
         <is>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
@@ -3151,16 +3151,16 @@
         <v>4.589764065335722</v>
       </c>
       <c r="T23" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>1287.26</v>
+        <v>1215.23</v>
       </c>
       <c r="V23" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>43.13725490196079</v>
       </c>
       <c r="X23" t="inlineStr">
         <is>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
@@ -3357,16 +3357,16 @@
         <v>4.768964986333255</v>
       </c>
       <c r="T25" t="n">
-        <v>884</v>
+        <v>992</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-312.1400000000001</v>
+        <v>-471.0699999999999</v>
       </c>
       <c r="V25" t="n">
-        <v>585</v>
+        <v>654</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>66.17647058823529</v>
+        <v>65.92741935483872</v>
       </c>
       <c r="X25" t="inlineStr">
         <is>
@@ -3375,7 +3375,7 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
@@ -3669,7 +3669,7 @@
         <v>34</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>891.8399999999999</v>
+        <v>891.84</v>
       </c>
       <c r="V28" t="n">
         <v>9</v>
@@ -3729,20 +3729,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/09/2026 00:22</t>
+          <t>06/10/2026 09:17</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20649.74</v>
+        <v>20644.38</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>3.24</v>
+        <v>3.21</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>5.73</v>
+        <v>5.51</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3751,34 +3751,34 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>20649.74</v>
+        <v>20644.38</v>
       </c>
       <c r="P29" t="n">
         <v>15</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>78.94736842105263</v>
+        <v>75</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>151.3220499381233</v>
+        <v>145.6393890562601</v>
       </c>
       <c r="S29" s="7" t="n">
         <v>0.1676133901630088</v>
       </c>
       <c r="T29" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>649.74</v>
+        <v>520.6799999999999</v>
       </c>
       <c r="V29" t="n">
         <v>14</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>73.68421052631578</v>
+        <v>60.86956521739131</v>
       </c>
       <c r="X29" t="inlineStr">
         <is>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo | EURUSD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US30, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US500, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCAD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCHF.pro</t>
+          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo | EURUSD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US30, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US500, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCAD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCHF.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -3872,16 +3872,16 @@
         <v>7.334333015531218</v>
       </c>
       <c r="T30" t="n">
-        <v>655</v>
+        <v>704</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>2087.1</v>
+        <v>1304.05</v>
       </c>
       <c r="V30" t="n">
-        <v>338</v>
+        <v>359</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>51.6030534351145</v>
+        <v>50.99431818181818</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
@@ -4078,16 +4078,16 @@
         <v>1.194162721074082</v>
       </c>
       <c r="T32" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>1318.52</v>
+        <v>1434.73</v>
       </c>
       <c r="V32" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>47.05882352941176</v>
+        <v>55.55555555555556</v>
       </c>
       <c r="X32" t="inlineStr">
         <is>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06/08/2026 23:49</t>
+          <t>06/10/2026 02:15</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4387,16 +4387,16 @@
         <v>1.6125</v>
       </c>
       <c r="T35" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>-458.6099999999999</v>
+        <v>-588.2399999999999</v>
       </c>
       <c r="V35" t="n">
         <v>3</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>16.66666666666666</v>
+        <v>15</v>
       </c>
       <c r="X35" t="inlineStr">
         <is>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
@@ -4490,16 +4490,16 @@
         <v>2.211704542281449</v>
       </c>
       <c r="T36" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-311.29</v>
+        <v>-274.2699999999999</v>
       </c>
       <c r="V36" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>22.22222222222222</v>
+        <v>23.07692307692308</v>
       </c>
       <c r="X36" t="inlineStr">
         <is>
@@ -4508,7 +4508,7 @@
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
@@ -4699,7 +4699,7 @@
         <v>18</v>
       </c>
       <c r="U38" s="7" t="n">
-        <v>207.75</v>
+        <v>207.96</v>
       </c>
       <c r="V38" t="n">
         <v>8</v>
@@ -4902,16 +4902,16 @@
         <v>16.98290000000001</v>
       </c>
       <c r="T40" t="n">
-        <v>2900</v>
+        <v>2908</v>
       </c>
       <c r="U40" s="7" t="n">
-        <v>-4701.099999999999</v>
+        <v>-5079.42</v>
       </c>
       <c r="V40" t="n">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="W40" s="7" t="n">
-        <v>59.86206896551725</v>
+        <v>59.73177441540578</v>
       </c>
       <c r="X40" t="inlineStr">
         <is>
@@ -4920,7 +4920,7 @@
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>06/07/2026 09:20</t>
+          <t>06/10/2026 09:25</t>
         </is>
       </c>
       <c r="H42" s="9" t="n">
@@ -5143,7 +5143,7 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>06/04/2026 16:07</t>
+          <t>06/10/2026 16:34</t>
         </is>
       </c>
       <c r="H43" s="9" t="n">
@@ -6601,7 +6601,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>06/07/2026 09:20</t>
+          <t>06/10/2026 09:25</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>06/04/2026 16:07</t>
+          <t>06/10/2026 16:34</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06/07/2026 12:29</t>
+          <t>06/10/2026 12:45</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -8343,7 +8343,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>06/07/2026 20:38</t>
+          <t>06/10/2026 21:16</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -8389,7 +8389,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06/07/2026 02:11</t>
+          <t>06/10/2026 02:26</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -8435,7 +8435,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06/04/2026 05:27</t>
+          <t>06/10/2026 05:38</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06/07/2026 12:24</t>
+          <t>06/10/2026 12:40</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -8527,7 +8527,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06/07/2026 12:00</t>
+          <t>06/10/2026 12:08</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -8573,7 +8573,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>06/07/2026 18:36</t>
+          <t>06/10/2026 18:45</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -8596,7 +8596,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06/08/2026 13:46</t>
+          <t>06/10/2026 08:57</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06/09/2026 01:08</t>
+          <t>06/10/2026 13:42</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -8734,7 +8734,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06/08/2026 23:36</t>
+          <t>06/09/2026 23:37</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-06-11
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-10 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-11 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -948,14 +948,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/09/2026 03:25</t>
+          <t>06/11/2026 14:59</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>53013.57</v>
+        <v>52228.34</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>126.46</v>
+        <v>123.11</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -973,31 +973,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>639.8099999999999</v>
+        <v>21.79000000000004</v>
       </c>
       <c r="P2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>47.5</v>
+        <v>52.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>3.056970789990661</v>
+        <v>1.019942289693312</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>2.220799999999999</v>
+        <v>14.44568801649876</v>
       </c>
       <c r="T2" t="n">
-        <v>2784</v>
+        <v>2803</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>27405.29999999999</v>
+        <v>28467.23999999998</v>
       </c>
       <c r="V2" t="n">
-        <v>1769</v>
+        <v>1781</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.54166666666666</v>
+        <v>63.5390652871923</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -1051,20 +1051,20 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/09/2026 10:18</t>
+          <t>06/11/2026 20:57</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
-        <v>24013.3</v>
+        <v>23788.13</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>15.75</v>
+        <v>14.67</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>12.55</v>
-      </c>
-      <c r="K3" s="7" t="n">
-        <v>1.02</v>
+        <v>13.37</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
       </c>
       <c r="L3" s="7" t="n">
         <v>30545.04</v>
@@ -1076,25 +1076,25 @@
         <v>40</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>-7257.93</v>
+        <v>-7458.22</v>
       </c>
       <c r="P3" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="Q3" s="7" t="n">
-        <v>60</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>0.1718915952600079</v>
+        <v>0.1529798521168591</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>74.29579795888873</v>
+        <v>76.21855298373961</v>
       </c>
       <c r="T3" t="n">
         <v>878</v>
       </c>
       <c r="U3" s="7" t="n">
-        <v>3626.77</v>
+        <v>3570</v>
       </c>
       <c r="V3" t="n">
         <v>548</v>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/10/2026 11:38</t>
+          <t>06/11/2026 11:52</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1194,7 +1194,7 @@
         <v>11.51358332205727</v>
       </c>
       <c r="T4" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="U4" s="7" t="n">
         <v>1407.88</v>
@@ -1203,7 +1203,7 @@
         <v>76</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>66.08695652173913</v>
+        <v>65.51724137931035</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/09/2026 06:32</t>
+          <t>06/11/2026 05:26</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/09/2026 10:35</t>
+          <t>06/11/2026 20:55</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/09/2026 03:43</t>
+          <t>06/11/2026 01:06</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1609,7 +1609,7 @@
         <v>294</v>
       </c>
       <c r="U8" s="7" t="n">
-        <v>-173.1400000000002</v>
+        <v>-173.14</v>
       </c>
       <c r="V8" t="n">
         <v>263</v>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/09/2026 21:15</t>
+          <t>06/11/2026 21:22</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1712,7 +1712,7 @@
         <v>447</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>-1584.580000000001</v>
+        <v>-1584.58</v>
       </c>
       <c r="V9" t="n">
         <v>204</v>
@@ -1815,7 +1815,7 @@
         <v>183</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>216.02</v>
+        <v>216.0199999999998</v>
       </c>
       <c r="V10" t="n">
         <v>85</v>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/10/2026 13:46</t>
+          <t>06/11/2026 11:58</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -1978,20 +1978,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/09/2026 05:46</t>
+          <t>06/11/2026 17:29</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
-        <v>10899.63</v>
+        <v>10807.84</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>8.26</v>
+        <v>7.35</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>1.25</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>5.61</v>
+        <v>3.65</v>
       </c>
       <c r="L12" t="n">
         <v>20000</v>
@@ -2003,7 +2003,7 @@
         <v>40</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>946.0899999999999</v>
+        <v>845.2399999999999</v>
       </c>
       <c r="P12" t="n">
         <v>31</v>
@@ -2012,22 +2012,22 @@
         <v>77.5</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>1.101771049925969</v>
+        <v>1.091298219040387</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>43.55695867347883</v>
+        <v>43.95203553897822</v>
       </c>
       <c r="T12" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>907.0700000000001</v>
+        <v>807.84</v>
       </c>
       <c r="V12" t="n">
         <v>18</v>
       </c>
       <c r="W12" s="7" t="n">
-        <v>100</v>
+        <v>94.73684210526315</v>
       </c>
       <c r="X12" t="inlineStr">
         <is>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/08/2026 05:29</t>
+          <t>06/11/2026 05:35</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2124,7 +2124,7 @@
         <v>38</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>-79.45999999999997</v>
+        <v>-79.45999999999998</v>
       </c>
       <c r="V13" t="n">
         <v>31</v>
@@ -2184,14 +2184,14 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>06/09/2026 08:46</t>
+          <t>06/11/2026 07:33</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
-        <v>19748.11</v>
+        <v>19773.19</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>-6.39</v>
+        <v>-6.27</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>9.75</v>
@@ -2209,19 +2209,19 @@
         <v>40</v>
       </c>
       <c r="O14" s="7" t="n">
-        <v>5229.240000000001</v>
+        <v>5342.3</v>
       </c>
       <c r="P14" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>47.5</v>
+        <v>50</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>1.74681039999886</v>
+        <v>1.775717244748129</v>
       </c>
       <c r="S14" s="7" t="n">
-        <v>29.09067136434657</v>
+        <v>28.97290027906993</v>
       </c>
       <c r="T14" t="n">
         <v>136</v>
@@ -2287,20 +2287,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/10/2026 10:05</t>
+          <t>06/11/2026 11:13</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>17860.53</v>
+        <v>18027.41</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-10.72</v>
+        <v>-9.890000000000001</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>13.19</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="L15" t="n">
         <v>20000</v>
@@ -2312,31 +2312,31 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>-688.3600000000001</v>
+        <v>-357.1200000000001</v>
       </c>
       <c r="P15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>45</v>
+        <v>47.5</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>0.8063780378832173</v>
+        <v>0.8931293959902212</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>14.21174568712316</v>
+        <v>13.9942748674455</v>
       </c>
       <c r="T15" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-1972.59</v>
+        <v>-1812.220000000001</v>
       </c>
       <c r="V15" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>44.73684210526316</v>
+        <v>44.53781512605043</v>
       </c>
       <c r="X15" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>06/10/2026 00:01</t>
+          <t>06/11/2026 21:51</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2493,20 +2493,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>06/09/2026 06:09</t>
+          <t>06/11/2026 17:57</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
-        <v>13289.92</v>
+        <v>12966.65</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>-33.58</v>
+        <v>-35.2</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>33.58</v>
+        <v>35.2</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="L17" t="n">
         <v>20000</v>
@@ -2518,31 +2518,31 @@
         <v>40</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>-818.9</v>
+        <v>-687.99</v>
       </c>
       <c r="P17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q17" s="7" t="n">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>0.1201057291442816</v>
+        <v>0.1920827657475692</v>
       </c>
       <c r="S17" s="7" t="n">
-        <v>8.188999999999941</v>
+        <v>6.879899999999961</v>
       </c>
       <c r="T17" t="n">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>-6974.449999999999</v>
+        <v>-7033.349999999999</v>
       </c>
       <c r="V17" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="W17" s="7" t="n">
-        <v>13.49862258953168</v>
+        <v>13.55013550135501</v>
       </c>
       <c r="X17" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -2596,20 +2596,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>06/09/2026 05:36</t>
+          <t>06/11/2026 17:17</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>16810.55</v>
+        <v>16417.61</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>-15.95</v>
+        <v>-17.91</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>17.52</v>
+        <v>18.9</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.62</v>
       </c>
       <c r="L18" t="n">
         <v>20000</v>
@@ -2621,31 +2621,31 @@
         <v>40</v>
       </c>
       <c r="O18" s="7" t="n">
-        <v>-1169</v>
+        <v>-1209.69</v>
       </c>
       <c r="P18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q18" s="7" t="n">
-        <v>22.5</v>
+        <v>20</v>
       </c>
       <c r="R18" s="7" t="n">
-        <v>0.2376980273833341</v>
+        <v>0.1839486767811006</v>
       </c>
       <c r="S18" s="7" t="n">
-        <v>12.81910000000002</v>
+        <v>12.09689999999997</v>
       </c>
       <c r="T18" t="n">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="U18" s="7" t="n">
-        <v>-3237.27</v>
+        <v>-3767.429999999999</v>
       </c>
       <c r="V18" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="W18" s="7" t="n">
-        <v>37.59398496240601</v>
+        <v>36.36363636363637</v>
       </c>
       <c r="X18" t="inlineStr">
         <is>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Hive V3 Forex HTF MOL | AUDJPY.pro, Hive V3 Forex HTF MOL | AUDUSD.pro, Hive V3 Forex HTF MOL | CADJPY.pro, Hive V3 Forex HTF MOL | CHFJPY.pro, Hive V3 Forex HTF MOL | EURCAD.pro, Hive V3 Forex HTF MOL | EURUSD.pro, Hive V3 Forex HTF MOL | GBPCHF.pro, Hive V3 Forex HTF MOL | GBPJPY.pro, Hive V3 Forex HTF MOL | GBPUSD.pro, Hive V3 Forex HTF MOL | USDCAD.pro, Hive V3 Forex HTF MOL | USDJPY.pro</t>
+          <t>Hive V3 Forex HTF MOL | AUDJPY.pro, Hive V3 Forex HTF MOL | AUDUSD.pro, Hive V3 Forex HTF MOL | CADJPY.pro, Hive V3 Forex HTF MOL | CHFJPY.pro, Hive V3 Forex HTF MOL | EURAUD.pro, Hive V3 Forex HTF MOL | EURCAD.pro, Hive V3 Forex HTF MOL | EURUSD.pro, Hive V3 Forex HTF MOL | GBPCHF.pro, Hive V3 Forex HTF MOL | GBPJPY.pro, Hive V3 Forex HTF MOL | GBPUSD.pro, Hive V3 Forex HTF MOL | USDCAD.pro, Hive V3 Forex HTF MOL | USDCHF.pro, Hive V3 Forex HTF MOL | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>06/09/2026 05:39</t>
+          <t>06/11/2026 17:24</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2709,7 +2709,7 @@
         <v>-4.15</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>4.93</v>
+        <v>7.08</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>0.14</v>
@@ -2802,7 +2802,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>06/09/2026 05:18</t>
+          <t>06/11/2026 17:01</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -2842,16 +2842,16 @@
         <v>11.01721679093957</v>
       </c>
       <c r="T20" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-154.1700000000001</v>
+        <v>32.81999999999998</v>
       </c>
       <c r="V20" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>52.27272727272727</v>
+        <v>53.33333333333334</v>
       </c>
       <c r="X20" t="inlineStr">
         <is>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>06/09/2026 05:33</t>
+          <t>06/11/2026 17:13</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3008,17 +3008,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>06/09/2026 05:41</t>
+          <t>06/11/2026 17:21</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>16167.88</v>
+        <v>15981.8</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-18.89</v>
-      </c>
-      <c r="J22" t="n">
-        <v>19</v>
+        <v>-19.83</v>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>19.93</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>0.43</v>
@@ -3033,7 +3033,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>-378.76</v>
+        <v>-639.02</v>
       </c>
       <c r="P22" t="n">
         <v>10</v>
@@ -3042,22 +3042,22 @@
         <v>25</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>0.4334438439529498</v>
+        <v>0.09690224711136314</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>4.927251001616692</v>
+        <v>6.57480000000005</v>
       </c>
       <c r="T22" t="n">
-        <v>319</v>
+        <v>330</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-3976.779999999999</v>
+        <v>-3883.95</v>
       </c>
       <c r="V22" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>33.22884012539185</v>
+        <v>33.63636363636363</v>
       </c>
       <c r="X22" t="inlineStr">
         <is>
@@ -3066,7 +3066,7 @@
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
@@ -3111,20 +3111,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>06/09/2026 05:42</t>
+          <t>06/11/2026 17:38</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>21240.81</v>
+        <v>21151.21</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>1.57</v>
+        <v>1.14</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>2.34</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>1.18</v>
+        <v>1.11</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3136,31 +3136,31 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>330.88</v>
+        <v>682.71</v>
       </c>
       <c r="P23" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>40</v>
+        <v>42.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.205355818208793</v>
+        <v>1.47960631691348</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.589764065335722</v>
+        <v>4.40222961631583</v>
       </c>
       <c r="T23" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>1215.23</v>
+        <v>1151.21</v>
       </c>
       <c r="V23" t="n">
         <v>22</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>43.13725490196079</v>
+        <v>42.30769230769231</v>
       </c>
       <c r="X23" t="inlineStr">
         <is>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/09/2026 05:37</t>
+          <t>06/11/2026 17:18</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3317,20 +3317,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>06/09/2026 05:38</t>
+          <t>06/11/2026 17:27</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>19476.21</v>
+        <v>19424.95</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-2.61</v>
+        <v>-2.87</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>7.09</v>
+        <v>7.76</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3342,31 +3342,28 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>-444.95</v>
+        <v>99</v>
       </c>
       <c r="P25" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="R25" s="7" t="n">
-        <v>0.09435997638965216</v>
+        <v>100</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>4.768964986333255</v>
+        <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>992</v>
+        <v>1091</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-471.0699999999999</v>
+        <v>-575.0500000000002</v>
       </c>
       <c r="V25" t="n">
-        <v>654</v>
+        <v>715</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>65.92741935483872</v>
+        <v>65.53620531622364</v>
       </c>
       <c r="X25" t="inlineStr">
         <is>
@@ -3375,7 +3372,7 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
@@ -3420,7 +3417,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/08/2026 09:30</t>
+          <t>06/11/2026 18:08</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3460,7 +3457,7 @@
         <v>5.34399892760695</v>
       </c>
       <c r="T26" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="U26" s="7" t="n">
         <v>164.61</v>
@@ -3469,7 +3466,7 @@
         <v>28</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>68.29268292682927</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="X26" t="inlineStr">
         <is>
@@ -3478,7 +3475,7 @@
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
@@ -3523,7 +3520,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/09/2026 06:03</t>
+          <t>06/11/2026 17:46</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3626,7 +3623,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/09/2026 05:50</t>
+          <t>06/11/2026 17:30</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3729,20 +3726,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/10/2026 09:17</t>
+          <t>06/11/2026 11:03</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20644.38</v>
+        <v>20558.72</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>3.21</v>
+        <v>2.78</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.25</v>
+        <v>0.63</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>5.51</v>
+        <v>3.1</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3751,34 +3748,34 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>20644.38</v>
+        <v>20558.72</v>
       </c>
       <c r="P29" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>75</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>145.6393890562601</v>
+        <v>78.16368276845701</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>0.1676133901630088</v>
+        <v>0.421080244073853</v>
       </c>
       <c r="T29" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>520.6799999999999</v>
+        <v>632.0599999999999</v>
       </c>
       <c r="V29" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>60.86956521739131</v>
+        <v>62.96296296296296</v>
       </c>
       <c r="X29" t="inlineStr">
         <is>
@@ -3787,7 +3784,7 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
@@ -3832,20 +3829,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/06/2026 19:51</t>
+          <t>06/11/2026 20:55</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>21491.63</v>
+        <v>20166.94</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>7.46</v>
+        <v>0.83</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>11.64</v>
-      </c>
-      <c r="K30" s="7" t="n">
-        <v>1.05</v>
+        <v>13.97</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -3857,31 +3854,31 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>199.29</v>
+        <v>-699.41</v>
       </c>
       <c r="P30" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>52.5</v>
+        <v>42.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>1.094064172637422</v>
+        <v>0.7166774690107753</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>7.334333015531218</v>
+        <v>8.801927397527734</v>
       </c>
       <c r="T30" t="n">
-        <v>704</v>
+        <v>759</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>1304.05</v>
+        <v>265.8899999999996</v>
       </c>
       <c r="V30" t="n">
-        <v>359</v>
+        <v>383</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>50.99431818181818</v>
+        <v>50.46113306982873</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
@@ -3890,7 +3887,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
@@ -3935,20 +3932,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/09/2026 02:56</t>
+          <t>06/11/2026 14:21</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20518.54</v>
+        <v>20715.58</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>2.58</v>
+        <v>3.57</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>1.45</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>2.04</v>
+        <v>2.44</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -3957,34 +3954,34 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>20518.54</v>
+        <v>20715.58</v>
       </c>
       <c r="P31" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Q31" s="7" t="n">
-        <v>68.75</v>
+        <v>72.22222222222221</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>42.21347366729603</v>
+        <v>42.60924757964086</v>
       </c>
       <c r="S31" s="7" t="n">
         <v>0.9758177348724615</v>
       </c>
       <c r="T31" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>518.54</v>
+        <v>834.1399999999999</v>
       </c>
       <c r="V31" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>72.22222222222221</v>
       </c>
       <c r="X31" t="inlineStr">
         <is>
@@ -3993,12 +3990,12 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr">
@@ -4038,20 +4035,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/09/2026 08:39</t>
+          <t>06/11/2026 20:04</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>21537.01</v>
+        <v>21234.91</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>7.68</v>
+        <v>6.17</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>1.78</v>
+        <v>1.94</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>2.56</v>
+        <v>1.76</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4060,34 +4057,34 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>21460.34</v>
+        <v>21148.77</v>
       </c>
       <c r="P32" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>60</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>22.79219662244888</v>
+        <v>14.09713570256701</v>
       </c>
       <c r="S32" s="7" t="n">
-        <v>1.194162721074082</v>
+        <v>1.327556495546532</v>
       </c>
       <c r="T32" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>1434.73</v>
+        <v>1234.91</v>
       </c>
       <c r="V32" t="n">
         <v>10</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>55.55555555555556</v>
+        <v>52.63157894736842</v>
       </c>
       <c r="X32" t="inlineStr">
         <is>
@@ -4096,12 +4093,12 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
@@ -4141,17 +4138,17 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06/10/2026 02:15</t>
+          <t>06/11/2026 10:28</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>19319.84</v>
+        <v>19263.7</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>-2.46</v>
+        <v>-2.74</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>2.46</v>
+        <v>2.74</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -4163,28 +4160,28 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>19499.12</v>
+        <v>19442.42</v>
       </c>
       <c r="P33" t="n">
         <v>1</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>8.333333333333332</v>
+        <v>7.692307692307693</v>
       </c>
       <c r="R33" s="7" t="n">
-        <v>40.75976196299013</v>
+        <v>36.55638822884299</v>
       </c>
       <c r="S33" s="7" t="n">
-        <v>1.635600000000001</v>
+        <v>1.823666666666662</v>
       </c>
       <c r="T33" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>-680.1599999999999</v>
+        <v>-736.6199999999999</v>
       </c>
       <c r="V33" t="n">
         <v>0</v>
@@ -4199,7 +4196,7 @@
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
@@ -4244,20 +4241,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>06/08/2026 23:52</t>
+          <t>06/11/2026 22:15</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20267.59</v>
+        <v>20211.13</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>1.34</v>
+        <v>1.06</v>
       </c>
       <c r="J34" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.96</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>2.93</v>
+        <v>2.09</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4266,34 +4263,34 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>20265.56</v>
+        <v>20208.86</v>
       </c>
       <c r="P34" t="n">
         <v>3</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>146.9849467012388</v>
+        <v>104.5139301444228</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>0.4565995305746404</v>
+        <v>0.642146530826876</v>
       </c>
       <c r="T34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>267.59</v>
+        <v>211.13</v>
       </c>
       <c r="V34" t="n">
         <v>2</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>40</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X34" t="inlineStr">
         <is>
@@ -4302,7 +4299,7 @@
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
@@ -4347,20 +4344,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>06/09/2026 02:06</t>
+          <t>06/11/2026 13:10</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>19516.25</v>
+        <v>19343.31</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>-2.42</v>
+        <v>-3.28</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>2.42</v>
+        <v>3.28</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>0.36</v>
+        <v>0.39</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4369,34 +4366,34 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>19381.69</v>
+        <v>19135.55</v>
       </c>
       <c r="P35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>18.75</v>
+        <v>18.18181818181818</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>26.62330961321324</v>
+        <v>18.88298541131224</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>1.6125</v>
+        <v>2.18896666666665</v>
       </c>
       <c r="T35" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>-588.2399999999999</v>
+        <v>-656.6899999999999</v>
       </c>
       <c r="V35" t="n">
         <v>3</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>15</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="X35" t="inlineStr">
         <is>
@@ -4405,12 +4402,12 @@
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
@@ -4450,20 +4447,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/09/2026 03:15</t>
+          <t>06/11/2026 00:22</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19664.21</v>
+        <v>19725.73</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-1.68</v>
+        <v>-1.37</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>3.31</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.64</v>
+        <v>0.73</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4472,34 +4469,34 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>19502.29</v>
+        <v>19553.57</v>
       </c>
       <c r="P36" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q36" s="7" t="n">
-        <v>23.52941176470588</v>
+        <v>25</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>22.29774721109065</v>
+        <v>20.24236186982987</v>
       </c>
       <c r="S36" s="7" t="n">
         <v>2.211704542281449</v>
       </c>
       <c r="T36" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-274.2699999999999</v>
+        <v>-386.9999999999999</v>
       </c>
       <c r="V36" t="n">
         <v>9</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>23.07692307692308</v>
+        <v>21.42857142857143</v>
       </c>
       <c r="X36" t="inlineStr">
         <is>
@@ -4508,7 +4505,7 @@
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
@@ -4553,14 +4550,14 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/09/2026 08:20</t>
+          <t>06/11/2026 19:52</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>2408.97</v>
+        <v>2328.47</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-96.70999999999999</v>
+        <v>-96.81999999999999</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>99.40000000000001</v>
@@ -4578,31 +4575,31 @@
         <v>40</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>-1384.64</v>
+        <v>-1198.14</v>
       </c>
       <c r="P37" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="Q37" s="7" t="n">
-        <v>27.5</v>
+        <v>20</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>0.3263863475566616</v>
+        <v>0.3072174129616073</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>12.37165935380934</v>
+        <v>10.86463870840718</v>
       </c>
       <c r="T37" t="n">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-18654.03000000001</v>
+        <v>-18671.53000000001</v>
       </c>
       <c r="V37" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>40.90909090909091</v>
+        <v>40.78431372549019</v>
       </c>
       <c r="X37" t="inlineStr">
         <is>
@@ -4611,7 +4608,7 @@
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z37" t="inlineStr">
@@ -4621,7 +4618,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>Cree Manual Trading | AUDUSD.PRO, Cree Manual Trading | ETHUSD, Cree Manual Trading | EURGBP.PRO, Cree Manual Trading | EURJPY.PRO, Cree Manual Trading | EURUSD.PRO, Cree Manual Trading | GBPUSD.PRO, Cree Manual Trading | NZDUSD.PRO, Cree Manual Trading | USDCAD.PRO, Cree Manual Trading | USDCHF.PRO, Cree Manual Trading | USDJPY.PRO, Cree Manual Trading | XAGUSD.PRO, Cree Manual Trading | XAUUSD.PRO</t>
+          <t>Cree Manual Trading | AUDUSD.PRO, Cree Manual Trading | ETHUSD, Cree Manual Trading | EURGBP.PRO, Cree Manual Trading | EURJPY.PRO, Cree Manual Trading | EURUSD.PRO, Cree Manual Trading | GBPUSD.PRO, Cree Manual Trading | NZDUSD.PRO, Cree Manual Trading | US500, Cree Manual Trading | USDCAD.PRO, Cree Manual Trading | USDCHF.PRO, Cree Manual Trading | USDJPY.PRO, Cree Manual Trading | XAGUSD.PRO, Cree Manual Trading | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
@@ -4656,20 +4653,20 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/09/2026 02:03</t>
+          <t>06/10/2026 22:44</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
-        <v>25986.07</v>
+        <v>25960.12</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="J38" s="7" t="n">
         <v>6.56</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>0.99</v>
+        <v>0.97</v>
       </c>
       <c r="L38" t="n">
         <v>26000</v>
@@ -4681,35 +4678,35 @@
         <v>40</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>15955.12</v>
+        <v>15847.81</v>
       </c>
       <c r="P38" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q38" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R38" s="7" t="n">
+        <v>12.24964399322702</v>
+      </c>
+      <c r="S38" s="7" t="n">
+        <v>6.608680763296301</v>
+      </c>
+      <c r="T38" t="n">
         <v>16</v>
       </c>
-      <c r="Q38" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="R38" s="7" t="n">
-        <v>12.46628842760619</v>
-      </c>
-      <c r="S38" s="7" t="n">
-        <v>6.55619118278732</v>
-      </c>
-      <c r="T38" t="n">
-        <v>18</v>
-      </c>
       <c r="U38" s="7" t="n">
-        <v>207.96</v>
+        <v>275.71</v>
       </c>
       <c r="V38" t="n">
         <v>8</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>44.44444444444444</v>
+        <v>50</v>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
@@ -4724,7 +4721,7 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>Gold Talon | EURUSD.PRO, Gold Talon | XAUUSD.PRO</t>
+          <t>Gold Talon | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
@@ -4862,20 +4859,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/07/2026 21:16</t>
+          <t>06/11/2026 13:06</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
-        <v>30024.24</v>
+        <v>28952.06</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>-16.72</v>
+        <v>-19.8</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>24.31</v>
+        <v>27.11</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L40" t="n">
         <v>25000</v>
@@ -4887,31 +4884,31 @@
         <v>40</v>
       </c>
       <c r="O40" s="7" t="n">
-        <v>-2071.15</v>
+        <v>-975</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q40" s="7" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="R40" s="7" t="n">
-        <v>0</v>
+        <v>0.05396878483835005</v>
       </c>
       <c r="S40" s="7" t="n">
-        <v>16.98290000000001</v>
+        <v>8.582254303963524</v>
       </c>
       <c r="T40" t="n">
-        <v>2908</v>
+        <v>2931</v>
       </c>
       <c r="U40" s="7" t="n">
-        <v>-5079.42</v>
+        <v>-5363.95</v>
       </c>
       <c r="V40" t="n">
-        <v>1737</v>
+        <v>1753</v>
       </c>
       <c r="W40" s="7" t="n">
-        <v>59.73177441540578</v>
+        <v>59.80893892869328</v>
       </c>
       <c r="X40" t="inlineStr">
         <is>
@@ -4920,7 +4917,7 @@
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr">
@@ -5766,7 +5763,7 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>06/09/2026 06:14</t>
+          <t>06/11/2026 05:08</t>
         </is>
       </c>
       <c r="H50" s="9" t="n">
@@ -5855,7 +5852,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>06/09/2026 05:56</t>
+          <t>06/11/2026 17:40</t>
         </is>
       </c>
       <c r="H51" s="9" t="n">
@@ -5944,7 +5941,7 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>06/09/2026 07:13</t>
+          <t>06/11/2026 06:10</t>
         </is>
       </c>
       <c r="H52" s="9" t="n">
@@ -6033,7 +6030,7 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>06/09/2026 07:06</t>
+          <t>06/11/2026 18:51</t>
         </is>
       </c>
       <c r="H53" s="9" t="n">
@@ -6929,7 +6926,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>06/09/2026 06:14</t>
+          <t>06/11/2026 05:08</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -6970,7 +6967,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/09/2026 05:56</t>
+          <t>06/11/2026 17:40</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -7011,7 +7008,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/09/2026 07:13</t>
+          <t>06/11/2026 06:10</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -7052,7 +7049,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>06/09/2026 07:06</t>
+          <t>06/11/2026 18:51</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -8228,7 +8225,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06/08/2026 21:07</t>
+          <t>06/11/2026 21:10</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -8458,7 +8455,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06/08/2026 21:14</t>
+          <t>06/11/2026 21:16</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
@@ -8619,7 +8616,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06/10/2026 13:42</t>
+          <t>06/11/2026 11:58</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -8665,7 +8662,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06/08/2026 21:11</t>
+          <t>06/11/2026 21:14</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -8688,7 +8685,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06/08/2026 21:14</t>
+          <t>06/11/2026 21:16</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -8734,7 +8731,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06/09/2026 23:37</t>
+          <t>06/10/2026 23:38</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-06-13
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-12 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-13 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -988,16 +988,16 @@
         <v>16.38092084116611</v>
       </c>
       <c r="T2" t="n">
-        <v>2815</v>
+        <v>2816</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>28934.20999999998</v>
+        <v>28943.81999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>1791</v>
+        <v>1792</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.6234458259325</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -1091,16 +1091,16 @@
         <v>76.21855298373961</v>
       </c>
       <c r="T3" t="n">
-        <v>878</v>
+        <v>890</v>
       </c>
       <c r="U3" s="7" t="n">
-        <v>3570</v>
+        <v>3390.75</v>
       </c>
       <c r="V3" t="n">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="W3" s="7" t="n">
-        <v>62.41457858769932</v>
+        <v>62.35955056179775</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Axis AUDUSD | AUDUSD.pro, EA Axis Rotation AUDUSD 5m | AUDUSD.pro, EA Fx RSI Prop USDCHF 10M | USDCHF.pro, Manual / one-off | GBPJPY.pro, Manual / one-off | GBPUSD.pro, Manual / one-off | NZDJPY.pro, Manual / one-off | USDJPY.pro, Manual / one-off | XAUUSD</t>
+          <t>Axis AUDUSD | AUDUSD.pro, Axis AUDUSD | USDCAD.pro, EA Axis Rotation AUDUSD 5m | AUDUSD.pro, EA Fx RSI Prop USDCHF 10M | USDCHF.pro, Manual / one-off | GBPJPY.pro, Manual / one-off | GBPUSD.pro, Manual / one-off | NZDJPY.pro, Manual / one-off | USDJPY.pro, Manual / one-off | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
         <v>602</v>
       </c>
       <c r="U6" s="7" t="n">
-        <v>-3642.179999999999</v>
+        <v>-3642.18</v>
       </c>
       <c r="V6" t="n">
         <v>502</v>
@@ -1609,7 +1609,7 @@
         <v>294</v>
       </c>
       <c r="U8" s="7" t="n">
-        <v>-173.1400000000001</v>
+        <v>-173.14</v>
       </c>
       <c r="V8" t="n">
         <v>263</v>
@@ -1712,7 +1712,7 @@
         <v>447</v>
       </c>
       <c r="U9" s="7" t="n">
-        <v>-1584.58</v>
+        <v>-1584.580000000001</v>
       </c>
       <c r="V9" t="n">
         <v>204</v>
@@ -1815,7 +1815,7 @@
         <v>183</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>216.0199999999999</v>
+        <v>216.02</v>
       </c>
       <c r="V10" t="n">
         <v>85</v>
@@ -2121,20 +2121,20 @@
         <v>48.72982283464567</v>
       </c>
       <c r="T13" t="n">
-        <v>38</v>
+        <v>160</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>-79.45999999999999</v>
+        <v>-202.86</v>
       </c>
       <c r="V13" t="n">
-        <v>31</v>
+        <v>133</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>81.57894736842105</v>
+        <v>83.125</v>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>T&amp;D60 | EURUSD.pro, T&amp;D60 | GBPUSD.pro, T&amp;D60 | USDCAD.pro, T&amp;D60 | USDJPY.pro</t>
+          <t>T&amp;D60 | AUDUSD.pro, T&amp;D60 | EURUSD.pro, T&amp;D60 | GBPUSD.pro, T&amp;D60 | USDCAD.pro, T&amp;D60 | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -2227,7 +2227,7 @@
         <v>136</v>
       </c>
       <c r="U14" s="7" t="n">
-        <v>-64.78999999999982</v>
+        <v>-64.78999999999994</v>
       </c>
       <c r="V14" t="n">
         <v>77</v>
@@ -2327,16 +2327,16 @@
         <v>13.79246179681093</v>
       </c>
       <c r="T15" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-2267.54</v>
+        <v>-2317.96</v>
       </c>
       <c r="V15" t="n">
         <v>54</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>43.90243902439025</v>
+        <v>43.54838709677419</v>
       </c>
       <c r="X15" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Agg V1 Pro XAUUSD | BTCUSD, Agg V1 Pro XAUUSD | XAUUSD, Breakout Engine | BTCUSD, Breakout Engine | XAUUSD</t>
+          <t>Agg V1 Pro XAUUSD | BTCUSD, Agg V1 Pro XAUUSD | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -2533,16 +2533,16 @@
         <v>7.242417895860122</v>
       </c>
       <c r="T17" t="n">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>-7132.22</v>
+        <v>-7163.09</v>
       </c>
       <c r="V17" t="n">
         <v>50</v>
       </c>
       <c r="W17" s="7" t="n">
-        <v>13.40482573726542</v>
+        <v>13.36898395721925</v>
       </c>
       <c r="X17" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>Breakout Scalper 2026 | BTCUSD, Hive V5 HTF (prop) | AUDJPY.pro, Hive V5 HTF (prop) | AUDUSD.pro, Hive V5 HTF (prop) | BTCUSD, Hive V5 HTF (prop) | CADJPY.pro, Hive V5 HTF (prop) | CHFJPY.pro, Hive V5 HTF (prop) | EURJPY.pro, Hive V5 HTF (prop) | EURUSD.pro, Hive V5 HTF (prop) | GBPJPY.pro, Hive V5 HTF (prop) | GBPUSD.pro, Hive V5 HTF (prop) | USDJPY.pro</t>
+          <t>Breakout Scalper 2026 | AUDJPY.pro, Breakout Scalper 2026 | AUDUSD.pro, Breakout Scalper 2026 | BTCUSD, Breakout Scalper 2026 | CADJPY.pro, Breakout Scalper 2026 | CHFJPY.pro, Breakout Scalper 2026 | EURJPY.pro, Breakout Scalper 2026 | EURUSD.pro, Breakout Scalper 2026 | GBPJPY.pro, Breakout Scalper 2026 | GBPUSD.pro, Breakout Scalper 2026 | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2639,7 @@
         <v>311</v>
       </c>
       <c r="U18" s="7" t="n">
-        <v>-4219.51</v>
+        <v>-4268.27</v>
       </c>
       <c r="V18" t="n">
         <v>114</v>
@@ -2845,7 +2845,7 @@
         <v>45</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>32.82000000000009</v>
+        <v>32.82000000000002</v>
       </c>
       <c r="V20" t="n">
         <v>24</v>
@@ -3048,16 +3048,16 @@
         <v>2.90720000000003</v>
       </c>
       <c r="T22" t="n">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-3832.25</v>
+        <v>-3826.72</v>
       </c>
       <c r="V22" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>35.01483679525222</v>
+        <v>35.10324483775811</v>
       </c>
       <c r="X22" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>51727</t>
+          <t>51726</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FourPlay MOL Bots</t>
+          <t>T&amp;Dv5 Prop Bots</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3111,20 +3111,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>06/11/2026 17:38</t>
+          <t>06/12/2026 03:28</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>21151.21</v>
+        <v>19920.5</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>1.14</v>
+        <v>-0.4</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>2.34</v>
+        <v>0.79</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>1.11</v>
+        <v>0.7</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3133,60 +3133,60 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>682.71</v>
+        <v>19945.41</v>
       </c>
       <c r="P23" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>42.5</v>
+        <v>37.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.47960631691348</v>
+        <v>77.26823385275087</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.40222961631583</v>
+        <v>0.5240354117877014</v>
       </c>
       <c r="T23" t="n">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>1151.41</v>
+        <v>-79.5</v>
       </c>
       <c r="V23" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>44.23076923076923</v>
+        <v>35.48387096774194</v>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>FourPlay MOL Bots | AUDUSD.pro, FourPlay MOL Bots | CHFJPY.pro, FourPlay MOL Bots | EURJPY.pro, FourPlay MOL Bots | EURUSD.pro, FourPlay MOL Bots | GBPAUD.pro, FourPlay MOL Bots | GBPJPY.pro, FourPlay MOL Bots | GBPNZD.pro, FourPlay MOL Bots | GBPUSD.pro, FourPlay MOL Bots | USDCAD.pro</t>
+          <t>T&amp;Dv5 Prop Bots | AUDJPY.pro, T&amp;Dv5 Prop Bots | CADJPY.pro, T&amp;Dv5 Prop Bots | EURJPY.pro, T&amp;Dv5 Prop Bots | EURUSD.pro, T&amp;Dv5 Prop Bots | GBPJPY.pro, T&amp;Dv5 Prop Bots | GBPUSD.pro, T&amp;Dv5 Prop Bots | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>52360</t>
+          <t>51727</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hive 7 HTF MOL</t>
+          <t>FourPlay MOL Bots</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3214,20 +3214,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/12/2026 03:44</t>
+          <t>06/11/2026 17:38</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>19325.73</v>
+        <v>21151.21</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>-3.37</v>
+        <v>1.14</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>8.619999999999999</v>
+        <v>2.34</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>0.83</v>
+        <v>1.11</v>
       </c>
       <c r="L24" t="n">
         <v>20000</v>
@@ -3239,7 +3239,7 @@
         <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>-298.13</v>
+        <v>682.71</v>
       </c>
       <c r="P24" t="n">
         <v>17</v>
@@ -3248,31 +3248,31 @@
         <v>42.5</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>0.8405406417312516</v>
+        <v>1.47960631691348</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>14.43094050860564</v>
+        <v>4.40222961631583</v>
       </c>
       <c r="T24" t="n">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>-674.2699999999998</v>
+        <v>1151.41</v>
       </c>
       <c r="V24" t="n">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>45.37037037037037</v>
+        <v>44.23076923076923</v>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
@@ -3282,14 +3282,14 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>Hive 7 HTF MOL | AUDUSD.pro, Hive 7 HTF MOL | EURGBP.pro, Hive 7 HTF MOL | EURUSD.pro, Hive 7 HTF MOL | GBPUSD.pro, Hive 7 HTF MOL | USDCAD.pro</t>
+          <t>FourPlay MOL Bots | AUDUSD.pro, FourPlay MOL Bots | CHFJPY.pro, FourPlay MOL Bots | EURJPY.pro, FourPlay MOL Bots | EURUSD.pro, FourPlay MOL Bots | GBPAUD.pro, FourPlay MOL Bots | GBPJPY.pro, FourPlay MOL Bots | GBPNZD.pro, FourPlay MOL Bots | GBPUSD.pro, FourPlay MOL Bots | USDCAD.pro</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>52361</t>
+          <t>52360</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Hive 7 LTF MOL</t>
+          <t>Hive 7 HTF MOL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3317,20 +3317,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>06/12/2026 03:52</t>
+          <t>06/12/2026 03:44</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>19424.95</v>
+        <v>19325.73</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-2.87</v>
+        <v>-3.37</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>7.76</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.87</v>
+        <v>0.83</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3342,37 +3342,40 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>99</v>
+        <v>-298.13</v>
       </c>
       <c r="P25" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>100</v>
+        <v>42.5</v>
+      </c>
+      <c r="R25" s="7" t="n">
+        <v>0.8405406417312516</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0</v>
+        <v>14.43094050860564</v>
       </c>
       <c r="T25" t="n">
-        <v>1196</v>
+        <v>108</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-324.34</v>
+        <v>-674.2699999999998</v>
       </c>
       <c r="V25" t="n">
-        <v>792</v>
+        <v>49</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>66.22073578595318</v>
+        <v>45.37037037037037</v>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
@@ -3382,14 +3385,14 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>Hive 7 LTF MOL | AUDJPY.pro, Hive 7 LTF MOL | AUDUSD.pro, Hive 7 LTF MOL | CADJPY.pro, Hive 7 LTF MOL | EURGBP.pro, Hive 7 LTF MOL | EURJPY.pro, Hive 7 LTF MOL | EURUSD.pro, Hive 7 LTF MOL | GBPJPY.pro, Hive 7 LTF MOL | GBPUSD.pro, Hive 7 LTF MOL | USDCAD.pro, Hive 7 LTF MOL | USDJPY.pro, Hive 7 LTF MOL | XAUUSD</t>
+          <t>Hive 7 HTF MOL | AUDUSD.pro, Hive 7 HTF MOL | EURGBP.pro, Hive 7 HTF MOL | EURUSD.pro, Hive 7 HTF MOL | GBPUSD.pro, Hive 7 HTF MOL | USDCAD.pro</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>52362</t>
+          <t>52361</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3399,7 +3402,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BB Fade Prop</t>
+          <t>Hive 7 LTF MOL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3417,20 +3420,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/11/2026 18:08</t>
+          <t>06/12/2026 03:52</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20164.61</v>
+        <v>19424.95</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>0.82</v>
+        <v>-2.87</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>2.77</v>
+        <v>7.76</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>1.25</v>
+        <v>0.87</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3442,35 +3445,32 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>167.13</v>
+        <v>99</v>
       </c>
       <c r="P26" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="R26" s="7" t="n">
-        <v>1.252392523925239</v>
+        <v>100</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>5.34399892760695</v>
+        <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>44</v>
+        <v>1215</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>0.8900000000000645</v>
+        <v>-324.3400000000001</v>
       </c>
       <c r="V26" t="n">
-        <v>28</v>
+        <v>792</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>63.63636363636363</v>
+        <v>65.18518518518519</v>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
@@ -3485,14 +3485,14 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>BB Fade Prop | AUDJPY.pro, BB Fade Prop | AUDNZD.pro, BB Fade Prop | CADJPY.pro, BB Fade Prop | CHFJPY.pro, BB Fade Prop | GBPJPY.pro, BB Fade Prop | GBPNZD.pro, BB Fade Prop | NZDJPY.pro, BB Fade Prop | XAGUSD</t>
+          <t>Hive 7 LTF MOL | AUDJPY.pro, Hive 7 LTF MOL | AUDUSD.pro, Hive 7 LTF MOL | CADJPY.pro, Hive 7 LTF MOL | EURGBP.pro, Hive 7 LTF MOL | EURJPY.pro, Hive 7 LTF MOL | EURUSD.pro, Hive 7 LTF MOL | GBPJPY.pro, Hive 7 LTF MOL | GBPUSD.pro, Hive 7 LTF MOL | USDCAD.pro, Hive 7 LTF MOL | USDJPY.pro, Hive 7 LTF MOL | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>52363</t>
+          <t>52362</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>T&amp;D4L Prop Firm</t>
+          <t>BB Fade Prop</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3520,20 +3520,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/12/2026 04:04</t>
+          <t>06/11/2026 18:08</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>13856.18</v>
+        <v>20164.61</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-30.73</v>
+        <v>0.82</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>40.77</v>
+        <v>2.77</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.72</v>
+        <v>1.25</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3545,31 +3545,31 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>122.32</v>
+        <v>167.13</v>
       </c>
       <c r="P27" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>82.5</v>
+        <v>70</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>1.561898504232211</v>
+        <v>1.252392523925239</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>4.420012749947007</v>
+        <v>5.34399892760695</v>
       </c>
       <c r="T27" t="n">
-        <v>2326</v>
+        <v>44</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>-3026.81</v>
+        <v>0.8900000000000148</v>
       </c>
       <c r="V27" t="n">
-        <v>1398</v>
+        <v>28</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>60.10318142734307</v>
+        <v>63.63636363636363</v>
       </c>
       <c r="X27" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
@@ -3588,14 +3588,14 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>T&amp;D4L Prop Firm | AUDJPY.pro, T&amp;D4L Prop Firm | CADJPY.pro, T&amp;D4L Prop Firm | EURUSD.pro, T&amp;D4L Prop Firm | GBPJPY.pro, T&amp;D4L Prop Firm | GBPUSD.pro, T&amp;D4L Prop Firm | USDCAD.pro, T&amp;D4L Prop Firm | USDJPY.pro</t>
+          <t>BB Fade Prop | AUDJPY.pro, BB Fade Prop | AUDNZD.pro, BB Fade Prop | CADJPY.pro, BB Fade Prop | CHFJPY.pro, BB Fade Prop | GBPJPY.pro, BB Fade Prop | GBPNZD.pro, BB Fade Prop | NZDJPY.pro, BB Fade Prop | XAGUSD</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>52364</t>
+          <t>52363</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>LVF-ZFade MOL</t>
+          <t>T&amp;D4L Prop Firm</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3623,20 +3623,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/11/2026 17:30</t>
+          <t>06/12/2026 04:04</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>20891.84</v>
+        <v>13856.18</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>4.47</v>
+        <v>-30.73</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>0.37</v>
+        <v>40.77</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>5.81</v>
+        <v>0.72</v>
       </c>
       <c r="L28" t="n">
         <v>20000</v>
@@ -3645,60 +3645,60 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>20891.84</v>
+        <v>122.32</v>
       </c>
       <c r="P28" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="Q28" s="7" t="n">
-        <v>28.57142857142857</v>
+        <v>82.5</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>113.6973783579674</v>
+        <v>1.561898504232211</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>0.2483351281054041</v>
+        <v>4.420012749947007</v>
       </c>
       <c r="T28" t="n">
-        <v>34</v>
+        <v>2326</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>891.84</v>
+        <v>-3026.81</v>
       </c>
       <c r="V28" t="n">
-        <v>9</v>
+        <v>1398</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>26.47058823529412</v>
+        <v>60.10318142734307</v>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
+          <t>T&amp;D4L Prop Firm | AUDJPY.pro, T&amp;D4L Prop Firm | CADJPY.pro, T&amp;D4L Prop Firm | EURUSD.pro, T&amp;D4L Prop Firm | GBPJPY.pro, T&amp;D4L Prop Firm | GBPUSD.pro, T&amp;D4L Prop Firm | USDCAD.pro, T&amp;D4L Prop Firm | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>52369</t>
+          <t>52364</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo</t>
+          <t>LVF-ZFade MOL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F29" t="b">
@@ -3726,20 +3726,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/12/2026 10:51</t>
+          <t>06/11/2026 17:30</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20632.06</v>
+        <v>20891.84</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>3.15</v>
+        <v>4.47</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.7</v>
+        <v>0.37</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>2.71</v>
+        <v>5.81</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3748,60 +3748,60 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>20632.06</v>
+        <v>20891.84</v>
       </c>
       <c r="P29" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>64.28571428571429</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>56.82720458911709</v>
+        <v>113.6973783579674</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>0.4676711776347864</v>
+        <v>0.2483351281054041</v>
       </c>
       <c r="T29" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>534.0699999999999</v>
+        <v>891.84</v>
       </c>
       <c r="V29" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>56.66666666666666</v>
+        <v>26.47058823529412</v>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo | EURUSD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US30, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US500, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCAD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCHF.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDJPY.pro</t>
+          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>52370</t>
+          <t>52369</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Agg V1 Pro XAUUSD May 19</t>
+          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3829,20 +3829,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/12/2026 07:15</t>
+          <t>06/12/2026 10:51</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>20261.13</v>
+        <v>20632.06</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1.3</v>
+        <v>3.15</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>14.45</v>
+        <v>0.7</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.01</v>
+        <v>2.71</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -3851,38 +3851,38 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-56.55999999999999</v>
+        <v>20632.06</v>
       </c>
       <c r="P30" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>50</v>
+        <v>64.28571428571429</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.9732048530672769</v>
+        <v>56.82720458911709</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>9.379215054117186</v>
+        <v>0.4676711776347864</v>
       </c>
       <c r="T30" t="n">
-        <v>798</v>
+        <v>30</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>-173.9299999999996</v>
+        <v>517.8299999999999</v>
       </c>
       <c r="V30" t="n">
-        <v>400</v>
+        <v>17</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>50.12531328320802</v>
+        <v>56.66666666666666</v>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
@@ -3897,14 +3897,14 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>Agg V1 Pro XAUUSD May 19 | XAUUSD</t>
+          <t>Codex NYKZ_CombinedPortfolio_v0_4_Demo | EURUSD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US30, Codex NYKZ_CombinedPortfolio_v0_4_Demo | US500, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCAD.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDCHF.pro, Codex NYKZ_CombinedPortfolio_v0_4_Demo | USDJPY.pro</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>53895</t>
+          <t>52370</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Codex Agg V1 Pro XAUUSD Filter60</t>
+          <t>Agg V1 Pro XAUUSD May 19</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3932,20 +3932,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/12/2026 01:22</t>
+          <t>06/12/2026 07:15</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20834.14</v>
+        <v>20261.13</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>4.16</v>
+        <v>1.3</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>1.45</v>
+        <v>14.45</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>2.68</v>
+        <v>1.01</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -3954,60 +3954,60 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>20834.14</v>
+        <v>-56.55999999999999</v>
       </c>
       <c r="P31" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="Q31" s="7" t="n">
-        <v>73.68421052631578</v>
+        <v>50</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>42.84738681557064</v>
+        <v>0.9732048530672769</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>0.9758177348724615</v>
+        <v>9.379215054117186</v>
       </c>
       <c r="T31" t="n">
-        <v>18</v>
+        <v>802</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>834.1399999999999</v>
+        <v>-367.8199999999999</v>
       </c>
       <c r="V31" t="n">
-        <v>13</v>
+        <v>401</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>72.22222222222221</v>
+        <v>50</v>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>Codex Agg V1 Pro XAUUSD Filter60 | XAUUSD</t>
+          <t>Agg V1 Pro XAUUSD May 19 | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>53897</t>
+          <t>53895</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Claude Code Sweep Suite Portfolio</t>
+          <t>Codex Agg V1 Pro XAUUSD Filter60</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4035,20 +4035,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/11/2026 20:04</t>
+          <t>06/12/2026 01:22</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>21234.91</v>
+        <v>20834.14</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>6.17</v>
+        <v>4.16</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>1.94</v>
+        <v>1.45</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>1.76</v>
+        <v>2.68</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4057,60 +4057,60 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>21148.77</v>
+        <v>20834.14</v>
       </c>
       <c r="P32" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>73.68421052631578</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>14.09713570256701</v>
+        <v>42.84738681557064</v>
       </c>
       <c r="S32" s="7" t="n">
-        <v>1.327556495546532</v>
+        <v>0.9758177348724615</v>
       </c>
       <c r="T32" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>1227.91</v>
+        <v>834.1399999999999</v>
       </c>
       <c r="V32" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>45.45454545454545</v>
+        <v>72.22222222222221</v>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>Claude Code Sweep Suite Portfolio | EURUSD, Claude Code Sweep Suite Portfolio | GBPUSD, Claude Code Sweep Suite Portfolio | NZDUSD, Claude Code Sweep Suite Portfolio | US500, Claude Code Sweep Suite Portfolio | USDCHF, Claude Code Sweep Suite Portfolio | USDJPY, Claude Code Sweep Suite Portfolio | XAUUSD</t>
+          <t>Codex Agg V1 Pro XAUUSD Filter60 | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>53898</t>
+          <t>53897</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Codex Axis V3 Optimization AUDUSD and GBPUSD</t>
+          <t>Claude Code Sweep Suite Portfolio</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4138,20 +4138,20 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06/11/2026 10:28</t>
+          <t>06/11/2026 20:04</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>19263.7</v>
+        <v>21234.91</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>-2.74</v>
+        <v>6.17</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>2.74</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
+        <v>1.94</v>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>1.76</v>
       </c>
       <c r="L33" t="n">
         <v>20000</v>
@@ -4160,38 +4160,38 @@
         <v>0</v>
       </c>
       <c r="N33" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>19442.42</v>
+        <v>21148.77</v>
       </c>
       <c r="P33" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>7.692307692307693</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R33" s="7" t="n">
-        <v>36.55638822884299</v>
+        <v>14.09713570256701</v>
       </c>
       <c r="S33" s="7" t="n">
-        <v>1.823666666666662</v>
+        <v>1.327556495546532</v>
       </c>
       <c r="T33" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>-793.6999999999999</v>
+        <v>1227.91</v>
       </c>
       <c r="V33" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="W33" s="7" t="n">
-        <v>0</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
@@ -4206,14 +4206,14 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>Codex Axis V3 Optimization AUDUSD and GBPUSD | AUDUSD, Codex Axis V3 Optimization AUDUSD and GBPUSD | GBPUSD</t>
+          <t>Claude Code Sweep Suite Portfolio | EURUSD, Claude Code Sweep Suite Portfolio | GBPUSD, Claude Code Sweep Suite Portfolio | NZDUSD, Claude Code Sweep Suite Portfolio | US500, Claude Code Sweep Suite Portfolio | USDCHF, Claude Code Sweep Suite Portfolio | USDJPY, Claude Code Sweep Suite Portfolio | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>53899</t>
+          <t>53898</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Claude Axis GBPUSD and AUDUSD Opt V3</t>
+          <t>Codex Axis V3 Optimization AUDUSD and GBPUSD</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4241,20 +4241,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>06/11/2026 22:15</t>
+          <t>06/11/2026 10:28</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20211.13</v>
+        <v>19263.7</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>1.06</v>
+        <v>-2.74</v>
       </c>
       <c r="J34" s="7" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="K34" s="7" t="n">
-        <v>2.09</v>
+        <v>2.74</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4263,38 +4263,38 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>20208.86</v>
+        <v>19442.42</v>
       </c>
       <c r="P34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>60</v>
+        <v>7.692307692307693</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>104.5139301444228</v>
+        <v>36.55638822884299</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>0.642146530826876</v>
+        <v>1.823666666666662</v>
       </c>
       <c r="T34" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>154.01</v>
+        <v>-793.6999999999999</v>
       </c>
       <c r="V34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>28.57142857142857</v>
+        <v>0</v>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
@@ -4309,14 +4309,14 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>Claude Axis GBPUSD and AUDUSD Opt V3 | AUDUSD, Claude Axis GBPUSD and AUDUSD Opt V3 | GBPUSD</t>
+          <t>Codex Axis V3 Optimization AUDUSD and GBPUSD | AUDUSD, Codex Axis V3 Optimization AUDUSD and GBPUSD | GBPUSD</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>53900</t>
+          <t>53899</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Codex Axis Rotation V4.1</t>
+          <t>Claude Axis GBPUSD and AUDUSD Opt V3</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4344,20 +4344,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>06/12/2026 12:52</t>
+          <t>06/11/2026 22:15</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>19281.85</v>
+        <v>20211.13</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>-3.59</v>
+        <v>1.06</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>3.59</v>
+        <v>0.96</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>0.37</v>
+        <v>2.09</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4366,38 +4366,38 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>19060.69</v>
+        <v>20208.86</v>
       </c>
       <c r="P35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>17.39130434782609</v>
+        <v>60</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>17.86773916999091</v>
+        <v>104.5139301444228</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>2.393833333333314</v>
+        <v>0.642146530826876</v>
       </c>
       <c r="T35" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>-718.15</v>
+        <v>154.01</v>
       </c>
       <c r="V35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>13.63636363636363</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
@@ -4407,19 +4407,19 @@
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>Codex Axis Rotation V4.1 | GBPUSD, Codex Axis Rotation V4.1 | USDJPY, Codex Axis Rotation V4.1 | XAUUSD</t>
+          <t>Claude Axis GBPUSD and AUDUSD Opt V3 | AUDUSD, Claude Axis GBPUSD and AUDUSD Opt V3 | GBPUSD</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>53901</t>
+          <t>53900</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Demo Codex Axis Rotation 4.2</t>
+          <t>Codex Axis Rotation V4.1</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4447,20 +4447,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/11/2026 00:22</t>
+          <t>06/12/2026 12:52</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19725.73</v>
+        <v>19281.85</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-1.37</v>
+        <v>-3.59</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>3.31</v>
+        <v>3.59</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.73</v>
+        <v>0.37</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4469,34 +4469,34 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>19553.57</v>
+        <v>19060.69</v>
       </c>
       <c r="P36" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="Q36" s="7" t="n">
-        <v>25</v>
+        <v>17.39130434782609</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>20.24236186982987</v>
+        <v>17.86773916999091</v>
       </c>
       <c r="S36" s="7" t="n">
-        <v>2.211704542281449</v>
+        <v>2.393833333333314</v>
       </c>
       <c r="T36" t="n">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-557.38</v>
+        <v>-718.15</v>
       </c>
       <c r="V36" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>19.14893617021277</v>
+        <v>13.63636363636363</v>
       </c>
       <c r="X36" t="inlineStr">
         <is>
@@ -4510,39 +4510,39 @@
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>Demo Codex Axis Rotation 4.2 | AUDUSD, Demo Codex Axis Rotation 4.2 | EURUSD, Demo Codex Axis Rotation 4.2 | GBPUSD, Demo Codex Axis Rotation 4.2 | USDJPY, Demo Codex Axis Rotation 4.2 | USTECH, Demo Codex Axis Rotation 4.2 | XAUUSD</t>
+          <t>Codex Axis Rotation V4.1 | GBPUSD, Codex Axis Rotation V4.1 | USDJPY, Codex Axis Rotation V4.1 | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>657902</t>
+          <t>53901</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cree Manual Trading</t>
+          <t>Demo Codex Axis Rotation 4.2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>OX Securities</t>
+          <t>TradeSmart</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242t2</t>
         </is>
       </c>
       <c r="F37" t="b">
@@ -4550,60 +4550,60 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/11/2026 19:52</t>
+          <t>06/11/2026 00:22</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>2328.47</v>
+        <v>19725.73</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-96.81999999999999</v>
+        <v>-1.37</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>99.40000000000001</v>
+        <v>3.31</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>0.83</v>
+        <v>0.73</v>
       </c>
       <c r="L37" t="n">
-        <v>31000</v>
+        <v>20000</v>
       </c>
       <c r="M37" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="N37" t="n">
         <v>40</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>-1198.14</v>
+        <v>19553.57</v>
       </c>
       <c r="P37" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q37" s="7" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>0.3072174129616073</v>
+        <v>20.24236186982987</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>10.86463870840718</v>
+        <v>2.211704542281449</v>
       </c>
       <c r="T37" t="n">
-        <v>511</v>
+        <v>47</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-18642.53000000001</v>
+        <v>-557.38</v>
       </c>
       <c r="V37" t="n">
-        <v>209</v>
+        <v>9</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>40.90019569471624</v>
+        <v>19.14893617021277</v>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
@@ -4618,14 +4618,14 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>Cree Manual Trading | AUDUSD.PRO, Cree Manual Trading | ETHUSD, Cree Manual Trading | EURGBP.PRO, Cree Manual Trading | EURJPY.PRO, Cree Manual Trading | EURUSD.PRO, Cree Manual Trading | GBPUSD.PRO, Cree Manual Trading | NZDUSD.PRO, Cree Manual Trading | US500, Cree Manual Trading | USDCAD.PRO, Cree Manual Trading | USDCHF.PRO, Cree Manual Trading | USDJPY.PRO, Cree Manual Trading | XAGUSD.PRO, Cree Manual Trading | XAUUSD.PRO</t>
+          <t>Demo Codex Axis Rotation 4.2 | AUDUSD, Demo Codex Axis Rotation 4.2 | EURUSD, Demo Codex Axis Rotation 4.2 | GBPUSD, Demo Codex Axis Rotation 4.2 | USDJPY, Demo Codex Axis Rotation 4.2 | USTECH, Demo Codex Axis Rotation 4.2 | XAUUSD</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>662437</t>
+          <t>657902</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4635,7 +4635,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Gold Talon V1.2</t>
+          <t>Cree Manual Trading</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS149</t>
         </is>
       </c>
       <c r="F38" t="b">
@@ -4653,102 +4653,102 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/12/2026 12:53</t>
+          <t>06/11/2026 19:52</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
-        <v>25960.12</v>
+        <v>2328.47</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>0.05</v>
+        <v>-96.81999999999999</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>6.56</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>0.97</v>
+        <v>0.83</v>
       </c>
       <c r="L38" t="n">
-        <v>26000</v>
+        <v>31000</v>
       </c>
       <c r="M38" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="N38" t="n">
         <v>40</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>15847.81</v>
+        <v>-1198.14</v>
       </c>
       <c r="P38" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="Q38" s="7" t="n">
-        <v>37.5</v>
+        <v>20</v>
       </c>
       <c r="R38" s="7" t="n">
-        <v>12.24964399322702</v>
+        <v>0.3072174129616073</v>
       </c>
       <c r="S38" s="7" t="n">
-        <v>6.608680763296301</v>
+        <v>10.86463870840718</v>
       </c>
       <c r="T38" t="n">
-        <v>16</v>
+        <v>512</v>
       </c>
       <c r="U38" s="7" t="n">
-        <v>275.71</v>
+        <v>-18647.03</v>
       </c>
       <c r="V38" t="n">
-        <v>8</v>
+        <v>209</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>50</v>
+        <v>40.8203125</v>
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2025-12-22</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>Gold Talon | XAUUSD.PRO</t>
+          <t>Cree Manual Trading | AUDUSD.PRO, Cree Manual Trading | ETHUSD, Cree Manual Trading | EURGBP.PRO, Cree Manual Trading | EURJPY.PRO, Cree Manual Trading | EURUSD.PRO, Cree Manual Trading | GBPUSD.PRO, Cree Manual Trading | NZDUSD.PRO, Cree Manual Trading | US500, Cree Manual Trading | USDCAD.PRO, Cree Manual Trading | USDCHF.PRO, Cree Manual Trading | USDJPY.PRO, Cree Manual Trading | XAGUSD.PRO, Cree Manual Trading | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>52441850</t>
+          <t>662437</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>EA Fx RSI MOL</t>
+          <t>Gold Talon V1.2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>IC Markets</t>
+          <t>OX Securities</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>VPS92</t>
+          <t>VPS92t2</t>
         </is>
       </c>
       <c r="F39" t="b">
@@ -4756,23 +4756,23 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>06/12/2026 05:44</t>
+          <t>06/12/2026 12:53</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
-        <v>44652.36</v>
+        <v>25960.12</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>24.35</v>
+        <v>0.05</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>22.74</v>
+        <v>6.56</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>1.17</v>
+        <v>0.97</v>
       </c>
       <c r="L39" t="n">
-        <v>25000</v>
+        <v>26000</v>
       </c>
       <c r="M39" t="n">
         <v>0</v>
@@ -4781,40 +4781,40 @@
         <v>40</v>
       </c>
       <c r="O39" s="7" t="n">
-        <v>2690.85</v>
+        <v>15847.81</v>
       </c>
       <c r="P39" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="Q39" s="7" t="n">
-        <v>90</v>
+        <v>37.5</v>
       </c>
       <c r="R39" s="7" t="n">
-        <v>7.653785968877684</v>
+        <v>12.24964399322702</v>
       </c>
       <c r="S39" s="7" t="n">
-        <v>4.601200000000008</v>
+        <v>6.608680763296301</v>
       </c>
       <c r="T39" t="n">
-        <v>1528</v>
+        <v>42</v>
       </c>
       <c r="U39" s="7" t="n">
-        <v>6602.099999999999</v>
+        <v>-39.87999999999992</v>
       </c>
       <c r="V39" t="n">
-        <v>748</v>
+        <v>17</v>
       </c>
       <c r="W39" s="7" t="n">
-        <v>48.95287958115183</v>
+        <v>40.47619047619047</v>
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="Z39" t="inlineStr">
@@ -4824,14 +4824,14 @@
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>EA Fx RSI MOL | AUDUSD, EA Fx RSI MOL | GBPJPY, EA Fx RSI MOL | USDCAD, EA Fx RSI MOL | USDCHF, EA Fx RSI MOL | USDJPY</t>
+          <t>Gold Talon | EURUSD.PRO, Gold Talon | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>52441853</t>
+          <t>52441850</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Fx RSI Low DD Prop Firms</t>
+          <t>EA Fx RSI MOL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4859,20 +4859,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/12/2026 13:00</t>
+          <t>06/12/2026 05:44</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
-        <v>29228.07</v>
+        <v>44652.36</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>-19.03</v>
+        <v>24.35</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>27.42</v>
+        <v>22.74</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>0.82</v>
+        <v>1.17</v>
       </c>
       <c r="L40" t="n">
         <v>25000</v>
@@ -4884,146 +4884,160 @@
         <v>40</v>
       </c>
       <c r="O40" s="7" t="n">
+        <v>2690.85</v>
+      </c>
+      <c r="P40" t="n">
+        <v>36</v>
+      </c>
+      <c r="Q40" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="R40" s="7" t="n">
+        <v>7.653785968877684</v>
+      </c>
+      <c r="S40" s="7" t="n">
+        <v>4.601200000000008</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1528</v>
+      </c>
+      <c r="U40" s="7" t="n">
+        <v>6602.099999999999</v>
+      </c>
+      <c r="V40" t="n">
+        <v>748</v>
+      </c>
+      <c r="W40" s="7" t="n">
+        <v>48.95287958115183</v>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>2025-07-29</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>RECONCILE</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>EA Fx RSI MOL | AUDUSD, EA Fx RSI MOL | GBPJPY, EA Fx RSI MOL | USDCAD, EA Fx RSI MOL | USDCHF, EA Fx RSI MOL | USDJPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>52441853</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Fx RSI Low DD Prop Firms</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>IC Markets</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>VPS92</t>
+        </is>
+      </c>
+      <c r="F41" t="b">
+        <v>1</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>06/12/2026 13:00</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="n">
+        <v>29228.07</v>
+      </c>
+      <c r="I41" s="7" t="n">
+        <v>-19.03</v>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>27.42</v>
+      </c>
+      <c r="K41" s="7" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="L41" t="n">
+        <v>25000</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="n">
+        <v>40</v>
+      </c>
+      <c r="O41" s="7" t="n">
         <v>218.37</v>
       </c>
-      <c r="P40" t="n">
+      <c r="P41" t="n">
         <v>32</v>
       </c>
-      <c r="Q40" s="7" t="n">
+      <c r="Q41" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="R40" s="7" t="n">
+      <c r="R41" s="7" t="n">
         <v>2.490369728122871</v>
       </c>
-      <c r="S40" s="7" t="n">
+      <c r="S41" s="7" t="n">
         <v>1.614700000000012</v>
       </c>
-      <c r="T40" t="n">
+      <c r="T41" t="n">
         <v>2934</v>
       </c>
-      <c r="U40" s="7" t="n">
+      <c r="U41" s="7" t="n">
         <v>-5053.93</v>
       </c>
-      <c r="V40" t="n">
+      <c r="V41" t="n">
         <v>1769</v>
       </c>
-      <c r="W40" s="7" t="n">
+      <c r="W41" s="7" t="n">
         <v>60.29311520109066</v>
       </c>
-      <c r="X40" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>2025-07-29</t>
         </is>
       </c>
-      <c r="Y40" t="inlineStr">
+      <c r="Y41" t="inlineStr">
         <is>
           <t>2026-06-12</t>
         </is>
       </c>
-      <c r="Z40" t="inlineStr">
+      <c r="Z41" t="inlineStr">
         <is>
           <t>RECONCILE</t>
         </is>
       </c>
-      <c r="AA40" t="inlineStr">
+      <c r="AA41" t="inlineStr">
         <is>
           <t>Fx RSI Low DD Prop Firms | AUDUSD, Fx RSI Low DD Prop Firms | GBPJPY, Fx RSI Low DD Prop Firms | USDCHF, Fx RSI Low DD Prop Firms | USDJPY</t>
         </is>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>22660</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Swing Trade MOL</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>TradeSmart</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>VPS92</t>
-        </is>
-      </c>
-      <c r="F41" s="8" t="b">
-        <v>0</v>
-      </c>
-      <c r="G41" s="8" t="inlineStr">
-        <is>
-          <t>06/09/2026 00:55</t>
-        </is>
-      </c>
-      <c r="H41" s="9" t="n">
-        <v>28127.1</v>
-      </c>
-      <c r="I41" s="9" t="n">
-        <v>12.33</v>
-      </c>
-      <c r="J41" s="9" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="K41" s="9" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="L41" s="8" t="n">
-        <v>25000</v>
-      </c>
-      <c r="M41" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="O41" s="9" t="n">
-        <v>-3167.68</v>
-      </c>
-      <c r="P41" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q41" s="9" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="R41" s="9" t="n">
-        <v>0.1775893840214113</v>
-      </c>
-      <c r="S41" s="9" t="n">
-        <v>29.85289999999997</v>
-      </c>
-      <c r="T41" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U41" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V41" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W41" s="8" t="n"/>
-      <c r="X41" s="8" t="n"/>
-      <c r="Y41" s="8" t="n"/>
-      <c r="Z41" s="8" t="inlineStr">
-        <is>
-          <t>DATA GAP - Bach missing</t>
-        </is>
-      </c>
-      <c r="AA41" s="8" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>38765</t>
+          <t>22660</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
@@ -5033,7 +5047,7 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Donchain Gold</t>
+          <t>Swing Trade MOL</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -5051,23 +5065,23 @@
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>06/10/2026 09:25</t>
+          <t>06/09/2026 00:55</t>
         </is>
       </c>
       <c r="H42" s="9" t="n">
-        <v>20207.71</v>
+        <v>28127.1</v>
       </c>
       <c r="I42" s="9" t="n">
-        <v>1.04</v>
+        <v>12.33</v>
       </c>
       <c r="J42" s="9" t="n">
-        <v>5.78</v>
+        <v>17.6</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>1.06</v>
+        <v>1.33</v>
       </c>
       <c r="L42" s="8" t="n">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="M42" s="8" t="n">
         <v>0</v>
@@ -5076,19 +5090,19 @@
         <v>40</v>
       </c>
       <c r="O42" s="9" t="n">
-        <v>-1245.8</v>
+        <v>-3167.68</v>
       </c>
       <c r="P42" s="8" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="Q42" s="9" t="n">
-        <v>40</v>
+        <v>27.5</v>
       </c>
       <c r="R42" s="9" t="n">
-        <v>0.2299841280794976</v>
+        <v>0.1775893840214113</v>
       </c>
       <c r="S42" s="9" t="n">
-        <v>11.26469363233483</v>
+        <v>29.85289999999997</v>
       </c>
       <c r="T42" s="8" t="n">
         <v>0</v>
@@ -5112,7 +5126,7 @@
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>38768</t>
+          <t>38765</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -5122,7 +5136,7 @@
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Aggressive CV2 Prop Firm</t>
+          <t>Donchain Gold</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -5140,20 +5154,20 @@
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>06/10/2026 16:34</t>
+          <t>06/13/2026 17:18</t>
         </is>
       </c>
       <c r="H43" s="9" t="n">
-        <v>19560.47</v>
+        <v>20207.71</v>
       </c>
       <c r="I43" s="9" t="n">
-        <v>-2.35</v>
+        <v>1.04</v>
       </c>
       <c r="J43" s="9" t="n">
-        <v>7.3</v>
+        <v>5.78</v>
       </c>
       <c r="K43" s="9" t="n">
-        <v>0.89</v>
+        <v>1.06</v>
       </c>
       <c r="L43" s="8" t="n">
         <v>20000</v>
@@ -5165,19 +5179,19 @@
         <v>40</v>
       </c>
       <c r="O43" s="9" t="n">
-        <v>-980.9399999999999</v>
+        <v>-1245.8</v>
       </c>
       <c r="P43" s="8" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="Q43" s="9" t="n">
-        <v>72.5</v>
+        <v>40</v>
       </c>
       <c r="R43" s="9" t="n">
-        <v>0.7320202184071484</v>
+        <v>0.2299841280794976</v>
       </c>
       <c r="S43" s="9" t="n">
-        <v>14.37228152648387</v>
+        <v>11.26469363233483</v>
       </c>
       <c r="T43" s="8" t="n">
         <v>0</v>
@@ -5201,7 +5215,7 @@
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>38769</t>
+          <t>38768</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
@@ -5211,7 +5225,7 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>EA Forex RSI V2 +DD</t>
+          <t>Aggressive CV2 Prop Firm</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -5229,20 +5243,20 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>06/09/2026 20:14</t>
+          <t>06/10/2026 16:34</t>
         </is>
       </c>
       <c r="H44" s="9" t="n">
-        <v>18825.91</v>
+        <v>19560.47</v>
       </c>
       <c r="I44" s="9" t="n">
-        <v>-5.87</v>
+        <v>-2.35</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>10.84</v>
+        <v>7.3</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>0.71</v>
+        <v>0.89</v>
       </c>
       <c r="L44" s="8" t="n">
         <v>20000</v>
@@ -5254,19 +5268,19 @@
         <v>40</v>
       </c>
       <c r="O44" s="9" t="n">
-        <v>193.4399999999999</v>
+        <v>-980.9399999999999</v>
       </c>
       <c r="P44" s="8" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="Q44" s="9" t="n">
-        <v>55.00000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="R44" s="9" t="n">
-        <v>1.233044880741913</v>
+        <v>0.7320202184071484</v>
       </c>
       <c r="S44" s="9" t="n">
-        <v>4.640100000000002</v>
+        <v>14.37228152648387</v>
       </c>
       <c r="T44" s="8" t="n">
         <v>0</v>
@@ -5290,7 +5304,7 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>41660</t>
+          <t>38769</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -5300,7 +5314,7 @@
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>EA Fx RSI V2 TDS</t>
+          <t>EA Forex RSI V2 +DD</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -5318,20 +5332,20 @@
       </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>06/12/2026 16:53</t>
+          <t>06/12/2026 22:48</t>
         </is>
       </c>
       <c r="H45" s="9" t="n">
-        <v>17132.5</v>
+        <v>18825.91</v>
       </c>
       <c r="I45" s="9" t="n">
-        <v>-14.35</v>
+        <v>-5.87</v>
       </c>
       <c r="J45" s="9" t="n">
-        <v>20.45</v>
+        <v>10.84</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="L45" s="8" t="n">
         <v>20000</v>
@@ -5343,19 +5357,19 @@
         <v>40</v>
       </c>
       <c r="O45" s="9" t="n">
-        <v>-549.3</v>
+        <v>193.4399999999999</v>
       </c>
       <c r="P45" s="8" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="Q45" s="9" t="n">
-        <v>65</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R45" s="9" t="n">
-        <v>0.7519596589411812</v>
+        <v>1.233044880741913</v>
       </c>
       <c r="S45" s="9" t="n">
-        <v>11.00099999999999</v>
+        <v>4.640100000000002</v>
       </c>
       <c r="T45" s="8" t="n">
         <v>0</v>
@@ -5379,7 +5393,7 @@
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>47779</t>
+          <t>41660</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
@@ -5389,7 +5403,7 @@
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Aggressive V3 + V4</t>
+          <t>EA Fx RSI V2 TDS</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
@@ -5403,27 +5417,27 @@
         </is>
       </c>
       <c r="F46" s="8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>06/12/2026 12:45</t>
+          <t>06/12/2026 16:53</t>
         </is>
       </c>
       <c r="H46" s="9" t="n">
-        <v>1201.05</v>
+        <v>17132.5</v>
       </c>
       <c r="I46" s="9" t="n">
-        <v>-94.13</v>
+        <v>-14.35</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>97.09999999999999</v>
+        <v>20.45</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="L46" s="9" t="n">
-        <v>20422.4</v>
+        <v>0.75</v>
+      </c>
+      <c r="L46" s="8" t="n">
+        <v>20000</v>
       </c>
       <c r="M46" s="8" t="n">
         <v>0</v>
@@ -5432,19 +5446,19 @@
         <v>40</v>
       </c>
       <c r="O46" s="9" t="n">
-        <v>-17.84999999999999</v>
+        <v>-549.3</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="Q46" s="9" t="n">
-        <v>32.5</v>
+        <v>65</v>
       </c>
       <c r="R46" s="9" t="n">
-        <v>0.9663955721224445</v>
+        <v>0.7519596589411812</v>
       </c>
       <c r="S46" s="9" t="n">
-        <v>3.328282308661215</v>
+        <v>11.00099999999999</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0</v>
@@ -5468,7 +5482,7 @@
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>51719</t>
+          <t>47779</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -5478,7 +5492,7 @@
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Hive V5 LTF (prop)</t>
+          <t>Aggressive V3 + V4</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -5488,7 +5502,7 @@
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F47" s="8" t="b">
@@ -5496,23 +5510,23 @@
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>06/09/2026 05:33</t>
+          <t>06/12/2026 12:45</t>
         </is>
       </c>
       <c r="H47" s="9" t="n">
-        <v>18511.35</v>
+        <v>1201.05</v>
       </c>
       <c r="I47" s="9" t="n">
-        <v>-7.44</v>
+        <v>-94.13</v>
       </c>
       <c r="J47" s="9" t="n">
-        <v>7.44</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="K47" s="9" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="L47" s="8" t="n">
-        <v>20000</v>
+        <v>0.68</v>
+      </c>
+      <c r="L47" s="9" t="n">
+        <v>20422.4</v>
       </c>
       <c r="M47" s="8" t="n">
         <v>0</v>
@@ -5521,19 +5535,19 @@
         <v>40</v>
       </c>
       <c r="O47" s="9" t="n">
-        <v>-803.1</v>
+        <v>-17.84999999999999</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="Q47" s="9" t="n">
-        <v>52.5</v>
+        <v>32.5</v>
       </c>
       <c r="R47" s="9" t="n">
-        <v>0.3037168049522719</v>
+        <v>0.9663955721224445</v>
       </c>
       <c r="S47" s="9" t="n">
-        <v>8.035322339850024</v>
+        <v>3.328282308661215</v>
       </c>
       <c r="T47" s="8" t="n">
         <v>0</v>
@@ -5557,7 +5571,7 @@
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>51721</t>
+          <t>51719</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
@@ -5567,7 +5581,7 @@
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Hive V3 Forex</t>
+          <t>Hive V5 LTF (prop)</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
@@ -5585,20 +5599,20 @@
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>06/12/2026 03:28</t>
+          <t>06/09/2026 05:33</t>
         </is>
       </c>
       <c r="H48" s="9" t="n">
-        <v>15078.92</v>
+        <v>18511.35</v>
       </c>
       <c r="I48" s="9" t="n">
-        <v>-24.61</v>
+        <v>-7.44</v>
       </c>
       <c r="J48" s="9" t="n">
-        <v>37.21</v>
+        <v>7.44</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>0.67</v>
+        <v>0.7</v>
       </c>
       <c r="L48" s="8" t="n">
         <v>20000</v>
@@ -5610,19 +5624,19 @@
         <v>40</v>
       </c>
       <c r="O48" s="9" t="n">
-        <v>-566.5400000000001</v>
+        <v>-803.1</v>
       </c>
       <c r="P48" s="8" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="Q48" s="9" t="n">
-        <v>42.5</v>
+        <v>52.5</v>
       </c>
       <c r="R48" s="9" t="n">
-        <v>0.8313211400873555</v>
+        <v>0.3037168049522719</v>
       </c>
       <c r="S48" s="9" t="n">
-        <v>21.85706566215555</v>
+        <v>8.035322339850024</v>
       </c>
       <c r="T48" s="8" t="n">
         <v>0</v>
@@ -5646,7 +5660,7 @@
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>51726</t>
+          <t>51721</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
@@ -5656,7 +5670,7 @@
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>T&amp;Dv5 Prop Bots</t>
+          <t>Hive V3 Forex</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -5678,16 +5692,16 @@
         </is>
       </c>
       <c r="H49" s="9" t="n">
-        <v>19920.5</v>
+        <v>15078.92</v>
       </c>
       <c r="I49" s="9" t="n">
-        <v>-0.4</v>
+        <v>-24.61</v>
       </c>
       <c r="J49" s="9" t="n">
-        <v>0.79</v>
+        <v>37.21</v>
       </c>
       <c r="K49" s="9" t="n">
-        <v>0.7</v>
+        <v>0.67</v>
       </c>
       <c r="L49" s="8" t="n">
         <v>20000</v>
@@ -5696,22 +5710,22 @@
         <v>0</v>
       </c>
       <c r="N49" s="8" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="O49" s="9" t="n">
-        <v>19945.41</v>
+        <v>-566.5400000000001</v>
       </c>
       <c r="P49" s="8" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="Q49" s="9" t="n">
-        <v>37.5</v>
+        <v>42.5</v>
       </c>
       <c r="R49" s="9" t="n">
-        <v>77.26823385275087</v>
+        <v>0.8313211400873555</v>
       </c>
       <c r="S49" s="9" t="n">
-        <v>0.5240354117877014</v>
+        <v>21.85706566215555</v>
       </c>
       <c r="T49" s="8" t="n">
         <v>0</v>
@@ -6453,7 +6467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -6598,7 +6612,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>06/10/2026 09:25</t>
+          <t>06/13/2026 17:18</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -6680,7 +6694,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>06/09/2026 20:14</t>
+          <t>06/12/2026 22:48</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -6860,7 +6874,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>51726</t>
+          <t>52365</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6870,7 +6884,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>T&amp;Dv5 Prop Bots</t>
+          <t>Hive 9 Demo Prop</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -6885,23 +6899,23 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>06/12/2026 03:28</t>
+          <t>06/11/2026 05:08</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>19920.5</v>
+        <v>19971.92</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>-0.4</v>
+        <v>-0.14</v>
       </c>
       <c r="I13" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>52365</t>
+          <t>52366</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -6911,7 +6925,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hive 9 Demo Prop</t>
+          <t>Claude Asian Sweep + NY Killzone</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -6921,28 +6935,28 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS242t2</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>06/11/2026 05:08</t>
+          <t>06/12/2026 04:01</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>19971.92</v>
+        <v>19452.07</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>-0.14</v>
+        <v>-2.74</v>
       </c>
       <c r="I14" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>52366</t>
+          <t>52367</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6952,7 +6966,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Claude Asian Sweep + NY Killzone</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -6962,28 +6976,28 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>VPS242t2</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/12/2026 04:01</t>
+          <t>06/12/2026 05:14</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>19452.07</v>
+        <v>19711.43</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>-2.74</v>
+        <v>-1.45</v>
       </c>
       <c r="I15" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>52367</t>
+          <t>52368</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7008,11 +7022,11 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/12/2026 05:14</t>
+          <t>06/11/2026 18:51</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>19711.43</v>
+        <v>19710.4</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>-1.45</v>
@@ -7024,39 +7038,39 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>52368</t>
+          <t>639884</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>demo</t>
+          <t>live</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Manual Trading (Diego)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TradeSmart</t>
+          <t>OX Securities</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS149</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>06/11/2026 18:51</t>
+          <t>06/08/2026 12:19</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>19710.4</v>
+        <v>5027.65</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>-1.45</v>
+        <v>42.67</v>
       </c>
       <c r="I17" t="n">
         <v>40</v>
@@ -7065,7 +7079,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>639884</t>
+          <t>647832</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7075,7 +7089,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Manual Trading (Diego)</t>
+          <t>Axis Rotation AUDUSD</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -7085,19 +7099,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>VPS149</t>
+          <t>VPS242</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>06/08/2026 12:19</t>
+          <t>06/04/2026 22:54</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>5027.65</v>
+        <v>4879.61</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>42.67</v>
+        <v>-27.8</v>
       </c>
       <c r="I18" t="n">
         <v>40</v>
@@ -7106,7 +7120,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>647832</t>
+          <t>658071</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7116,7 +7130,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Axis Rotation AUDUSD</t>
+          <t>T&amp;D V1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -7126,19 +7140,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>VPS242</t>
+          <t>VPS92</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>06/04/2026 22:54</t>
+          <t>01/07/2026 18:21</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>4879.61</v>
+        <v>3417.36</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>-27.8</v>
+        <v>-0.19</v>
       </c>
       <c r="I19" t="n">
         <v>40</v>
@@ -7147,22 +7161,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>658071</t>
+          <t>52428953</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>T&amp;D V1</t>
+          <t>BTC Dual Breakout Scalper</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>OX Securities</t>
+          <t>IC Markets</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7172,57 +7186,16 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>01/07/2026 18:21</t>
+          <t>06/09/2026 14:03</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>3417.36</v>
+        <v>28300.62</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>-0.19</v>
+        <v>13.2</v>
       </c>
       <c r="I20" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>52428953</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>BTC Dual Breakout Scalper</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>IC Markets</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>VPS92</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>06/09/2026 14:03</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="n">
-        <v>28300.62</v>
-      </c>
-      <c r="H21" s="7" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="I21" t="n">
         <v>40</v>
       </c>
     </row>
@@ -8202,7 +8175,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06/09/2026 20:50</t>
+          <t>06/12/2026 23:33</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -8271,7 +8244,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>06/10/2026 12:45</t>
+          <t>06/13/2026 22:24</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -8386,7 +8359,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06/10/2026 02:26</t>
+          <t>06/13/2026 06:19</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -8432,7 +8405,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06/10/2026 05:38</t>
+          <t>06/13/2026 11:09</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
@@ -8501,7 +8474,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>06/10/2026 12:40</t>
+          <t>06/13/2026 22:17</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -8524,7 +8497,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>06/10/2026 12:08</t>
+          <t>06/13/2026 21:32</t>
         </is>
       </c>
       <c r="E19" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-06-14
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -628,42 +628,42 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>[HIGH] 1. Drawdown formula: hardcoded $10K starting equity</t>
+          <t>[RESOLVED] 1. Profit Factor now net of commission &amp; swap</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Bachelier (orchestra_selector.py:178): equity_curve = 10000 + cumulative_profit. MFB uses the account's actual starting balance and full equity curve (including floating P&amp;L on open trades). For a $200K prop account, dividing drawdown by $10K instead of $200K inflates DD% by ~20x. FIX: replace hardcoded 10000 with each account's deposits - withdrawals (or first-trade-day balance).</t>
+          <t>Bachelier PF previously used the gross `profit` field only. As of 2026-06-13 the whole pipeline rolls deals up to positions (consolidate.py positions_from_deals -&gt; position_net = profit + commission + swap) and PF/win-rate/net-P&amp;L all aggregate on that net, matching MFB. Spot-check: 51718 PF 0.31 vs MFB 0.31; 50347 0.80 vs 0.81; 41655 0.91 vs 0.96. Remaining gaps are MFB's 40-trade sample vs Bachelier's full history, not formula differences.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>[HIGH] 2. Drawdown basis: closed-trade balance vs real equity</t>
+          <t>[RESOLVED] 2. Drawdown denominator now the real starting balance</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Bachelier measures peak-to-trough on closed-trade cumulative P&amp;L only. MFB measures peak-to-trough on real account equity (balance + floating). Two different things - MFB DD is almost always larger for active accounts with open positions.</t>
+          <t>compute_max_drawdown() walks the equity curve off each account's actual starting balance (deposits - withdrawals), not a hardcoded $10K. This audit's 'Bach DD% (real-balance)' column uses the same denominator so it lines up with MFB.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>[MEDIUM] 3. Profit Factor: gross P/L excludes commissions &amp; swaps</t>
+          <t>[RESIDUAL] 3. Drawdown basis: closed-trade vs real equity (floating P&amp;L)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Bachelier: PF = |sum(profit &gt; 0) / sum(profit &lt; 0)| using the 'profit' field only. MFB's PF includes commissions and swaps in each trade's net result. On accounts with high commission costs, MFB PF will be ~5-15% lower than Bachelier's.</t>
+          <t>The one remaining DD difference: Bachelier measures peak-to-trough on the CLOSED-trade equity curve; MFB includes floating P&amp;L on still-open positions. So MFB DD can be a bit larger for accounts holding open trades. Closing this needs vps_extractor.py to also export open positions. For closed-trade / prop-style DD the current number is correct.</t>
         </is>
       </c>
     </row>
@@ -768,8 +768,8 @@
     <col width="24" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
     <col width="23" customWidth="1" min="17" max="17"/>
-    <col width="31" customWidth="1" min="18" max="18"/>
-    <col width="43" customWidth="1" min="19" max="19"/>
+    <col width="29" customWidth="1" min="18" max="18"/>
+    <col width="39" customWidth="1" min="19" max="19"/>
     <col width="23" customWidth="1" min="20" max="20"/>
     <col width="28" customWidth="1" min="21" max="21"/>
     <col width="21" customWidth="1" min="22" max="22"/>
@@ -868,12 +868,12 @@
       </c>
       <c r="R1" s="4" t="inlineStr">
         <is>
-          <t>Bach formula PF on MFB sample</t>
+          <t>Bach PF (net) on MFB sample</t>
         </is>
       </c>
       <c r="S1" s="4" t="inlineStr">
         <is>
-          <t>Bach formula DD% (10K base) on MFB sample</t>
+          <t>Bach DD% (real-balance) on MFB sample</t>
         </is>
       </c>
       <c r="T1" s="4" t="inlineStr">
@@ -982,10 +982,10 @@
         <v>52.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.021428251623013</v>
+        <v>1.01201451680169</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>16.38092084116611</v>
+        <v>6.685954240165922</v>
       </c>
       <c r="T2" t="n">
         <v>2816</v>
@@ -1085,10 +1085,10 @@
         <v>55.00000000000001</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>0.1529798521168591</v>
+        <v>0.1511757201079379</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>76.21855298373961</v>
+        <v>33.54844363059227</v>
       </c>
       <c r="T3" t="n">
         <v>890</v>
@@ -1188,10 +1188,10 @@
         <v>70</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>1.176005894852286</v>
+        <v>1.152592845168073</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>11.51358332205727</v>
+        <v>6.456063830500751</v>
       </c>
       <c r="T4" t="n">
         <v>116</v>
@@ -1291,10 +1291,10 @@
         <v>77.5</v>
       </c>
       <c r="R5" s="7" t="n">
-        <v>2.573611111111111</v>
+        <v>2.641227823148409</v>
       </c>
       <c r="S5" s="7" t="n">
-        <v>0.1587531959394289</v>
+        <v>0.04363058312216826</v>
       </c>
       <c r="T5" t="n">
         <v>3</v>
@@ -1397,7 +1397,7 @@
         <v>0.7658839892006872</v>
       </c>
       <c r="S6" s="7" t="n">
-        <v>3.812086952093313</v>
+        <v>1.263825732055561</v>
       </c>
       <c r="T6" t="n">
         <v>602</v>
@@ -1500,7 +1500,7 @@
         <v>0.4474505336668235</v>
       </c>
       <c r="S7" s="7" t="n">
-        <v>11.73223743715118</v>
+        <v>5.9032725408248</v>
       </c>
       <c r="T7" t="n">
         <v>668</v>
@@ -1603,7 +1603,7 @@
         <v>1.488476250423667</v>
       </c>
       <c r="S8" s="7" t="n">
-        <v>1.53011087488554</v>
+        <v>0.7705874264792461</v>
       </c>
       <c r="T8" t="n">
         <v>294</v>
@@ -1703,10 +1703,10 @@
         <v>45</v>
       </c>
       <c r="R9" s="7" t="n">
-        <v>1.083458935958695</v>
+        <v>1.06275743547416</v>
       </c>
       <c r="S9" s="7" t="n">
-        <v>8.214877771782222</v>
+        <v>4.173414842391923</v>
       </c>
       <c r="T9" t="n">
         <v>447</v>
@@ -1806,10 +1806,10 @@
         <v>37.5</v>
       </c>
       <c r="R10" s="7" t="n">
-        <v>0.8207764882691826</v>
+        <v>0.8097594813441298</v>
       </c>
       <c r="S10" s="7" t="n">
-        <v>13.82284951966541</v>
+        <v>7.216828090941156</v>
       </c>
       <c r="T10" t="n">
         <v>183</v>
@@ -1909,10 +1909,10 @@
         <v>30</v>
       </c>
       <c r="R11" s="7" t="n">
-        <v>0.4218233948115678</v>
+        <v>0.4175736675050247</v>
       </c>
       <c r="S11" s="7" t="n">
-        <v>12.87413289157481</v>
+        <v>6.594705120244678</v>
       </c>
       <c r="T11" t="n">
         <v>4</v>
@@ -2012,10 +2012,10 @@
         <v>77.5</v>
       </c>
       <c r="R12" s="7" t="n">
-        <v>1.091298219040387</v>
+        <v>1.083748323032077</v>
       </c>
       <c r="S12" s="7" t="n">
-        <v>43.95203553897822</v>
+        <v>43.99713582668562</v>
       </c>
       <c r="T12" t="n">
         <v>20</v>
@@ -2118,7 +2118,7 @@
         <v>0.07030875541161243</v>
       </c>
       <c r="S13" s="7" t="n">
-        <v>48.72982283464567</v>
+        <v>1141.113697651371</v>
       </c>
       <c r="T13" t="n">
         <v>160</v>
@@ -2218,10 +2218,10 @@
         <v>50</v>
       </c>
       <c r="R14" s="7" t="n">
-        <v>1.775717244748129</v>
+        <v>1.773687975924623</v>
       </c>
       <c r="S14" s="7" t="n">
-        <v>28.97290027906993</v>
+        <v>19.33199591540321</v>
       </c>
       <c r="T14" t="n">
         <v>136</v>
@@ -2324,7 +2324,7 @@
         <v>0.9663955721224445</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>3.328282308661215</v>
+        <v>1.630649954951567</v>
       </c>
       <c r="T15" t="n">
         <v>1206</v>
@@ -2424,10 +2424,10 @@
         <v>47.5</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.8852928951253423</v>
+        <v>0.8889936149058327</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>13.79246179681093</v>
+        <v>7.181297124743868</v>
       </c>
       <c r="T16" t="n">
         <v>124</v>
@@ -2527,10 +2527,10 @@
         <v>60</v>
       </c>
       <c r="R17" s="7" t="n">
-        <v>1.066652925212134</v>
+        <v>0.9483601341022563</v>
       </c>
       <c r="S17" s="7" t="n">
-        <v>4.000813588843479</v>
+        <v>1.035984170682116</v>
       </c>
       <c r="T17" t="n">
         <v>3665</v>
@@ -2633,7 +2633,7 @@
         <v>0.1895672530885659</v>
       </c>
       <c r="S18" s="7" t="n">
-        <v>7.242417895860122</v>
+        <v>3.626072931906652</v>
       </c>
       <c r="T18" t="n">
         <v>374</v>
@@ -2736,7 +2736,7 @@
         <v>0.2455243766654573</v>
       </c>
       <c r="S19" s="7" t="n">
-        <v>12.53689999999997</v>
+        <v>6.26845000000003</v>
       </c>
       <c r="T19" t="n">
         <v>311</v>
@@ -2839,7 +2839,7 @@
         <v>20.94871954963111</v>
       </c>
       <c r="S20" s="7" t="n">
-        <v>3.199389279836951</v>
+        <v>2.400274548307834</v>
       </c>
       <c r="T20" t="n">
         <v>4</v>
@@ -2939,10 +2939,10 @@
         <v>45</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>0.8268741944722899</v>
+        <v>0.8034374404453249</v>
       </c>
       <c r="S21" s="7" t="n">
-        <v>11.02427855495349</v>
+        <v>5.681363359732104</v>
       </c>
       <c r="T21" t="n">
         <v>45</v>
@@ -3042,10 +3042,10 @@
         <v>35.8974358974359</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>51.6299900135713</v>
+        <v>51.63506453595574</v>
       </c>
       <c r="S22" s="7" t="n">
-        <v>0.9062551031630334</v>
+        <v>0.67876758502964</v>
       </c>
       <c r="T22" t="n">
         <v>39</v>
@@ -3145,10 +3145,10 @@
         <v>42.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.7207966400216772</v>
+        <v>0.7197629741869149</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>2.90720000000003</v>
+        <v>1.44869999999999</v>
       </c>
       <c r="T23" t="n">
         <v>339</v>
@@ -3248,10 +3248,10 @@
         <v>37.5</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>77.26823385275087</v>
+        <v>82.83739537173807</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>0.5240354117877014</v>
+        <v>0.3563138824967511</v>
       </c>
       <c r="T24" t="n">
         <v>31</v>
@@ -3354,7 +3354,7 @@
         <v>1.47960631691348</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>4.40222961631583</v>
+        <v>2.282854853991267</v>
       </c>
       <c r="T25" t="n">
         <v>52</v>
@@ -3457,7 +3457,7 @@
         <v>0.8405406417312516</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>14.43094050860564</v>
+        <v>7.396477538225161</v>
       </c>
       <c r="T26" t="n">
         <v>108</v>
@@ -3657,10 +3657,10 @@
         <v>70</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>1.252392523925239</v>
+        <v>1.249928967713957</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>5.34399892760695</v>
+        <v>2.774291927864321</v>
       </c>
       <c r="T28" t="n">
         <v>44</v>
@@ -3760,10 +3760,10 @@
         <v>82.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>1.561898504232211</v>
+        <v>1.181252407906825</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>4.420012749947007</v>
+        <v>3.047665694331139</v>
       </c>
       <c r="T29" t="n">
         <v>2326</v>
@@ -3866,7 +3866,7 @@
         <v>113.6973783579674</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>0.2483351281054041</v>
+        <v>0.1862572589961039</v>
       </c>
       <c r="T30" t="n">
         <v>34</v>
@@ -3969,7 +3969,7 @@
         <v>0.09729948417113379</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>0.8924999999999819</v>
+        <v>0.4462500000000546</v>
       </c>
       <c r="T31" t="n">
         <v>683</v>
@@ -4072,7 +4072,7 @@
         <v>56.82720458911709</v>
       </c>
       <c r="S32" s="7" t="n">
-        <v>0.4676711776347864</v>
+        <v>0.3526221815932808</v>
       </c>
       <c r="T32" t="n">
         <v>30</v>
@@ -4175,7 +4175,7 @@
         <v>0.9732048530672769</v>
       </c>
       <c r="S33" s="7" t="n">
-        <v>9.379215054117186</v>
+        <v>4.834790529556989</v>
       </c>
       <c r="T33" t="n">
         <v>802</v>
@@ -4278,7 +4278,7 @@
         <v>42.84738681557064</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>0.9758177348724615</v>
+        <v>0.7367596880689841</v>
       </c>
       <c r="T34" t="n">
         <v>18</v>
@@ -4378,10 +4378,10 @@
         <v>55.00000000000001</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>14.09713570256701</v>
+        <v>13.84187484060576</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>1.327556495546532</v>
+        <v>1.020755473547458</v>
       </c>
       <c r="T35" t="n">
         <v>22</v>
@@ -4481,10 +4481,10 @@
         <v>7.692307692307693</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>36.55638822884299</v>
+        <v>35.86929229886294</v>
       </c>
       <c r="S36" s="7" t="n">
-        <v>1.823666666666662</v>
+        <v>1.393949999999986</v>
       </c>
       <c r="T36" t="n">
         <v>15</v>
@@ -4584,10 +4584,10 @@
         <v>60</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>104.5139301444228</v>
+        <v>102.9568134806518</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>0.642146530826876</v>
+        <v>0.4905329686116789</v>
       </c>
       <c r="T37" t="n">
         <v>7</v>
@@ -4687,10 +4687,10 @@
         <v>17.39130434782609</v>
       </c>
       <c r="R38" s="7" t="n">
-        <v>17.86773916999091</v>
+        <v>15.34083453713736</v>
       </c>
       <c r="S38" s="7" t="n">
-        <v>2.393833333333314</v>
+        <v>2.348275000000013</v>
       </c>
       <c r="T38" t="n">
         <v>22</v>
@@ -4790,10 +4790,10 @@
         <v>25</v>
       </c>
       <c r="R39" s="7" t="n">
-        <v>20.24236186982987</v>
+        <v>17.68279468978227</v>
       </c>
       <c r="S39" s="7" t="n">
-        <v>2.211704542281449</v>
+        <v>1.979972213017599</v>
       </c>
       <c r="T39" t="n">
         <v>47</v>
@@ -4893,10 +4893,10 @@
         <v>20</v>
       </c>
       <c r="R40" s="7" t="n">
-        <v>0.3072174129616073</v>
+        <v>0.2034385097131916</v>
       </c>
       <c r="S40" s="7" t="n">
-        <v>10.86463870840718</v>
+        <v>6.378610940381084</v>
       </c>
       <c r="T40" t="n">
         <v>512</v>
@@ -4996,10 +4996,10 @@
         <v>37.5</v>
       </c>
       <c r="R41" s="7" t="n">
-        <v>12.24964399322702</v>
+        <v>12.07123595819594</v>
       </c>
       <c r="S41" s="7" t="n">
-        <v>6.608680763296301</v>
+        <v>2.604214844380084</v>
       </c>
       <c r="T41" t="n">
         <v>42</v>
@@ -5099,10 +5099,10 @@
         <v>90</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>7.653785968877684</v>
+        <v>6.66566303111972</v>
       </c>
       <c r="S42" s="7" t="n">
-        <v>4.601200000000008</v>
+        <v>1.899759999999995</v>
       </c>
       <c r="T42" t="n">
         <v>1528</v>
@@ -5202,10 +5202,10 @@
         <v>80</v>
       </c>
       <c r="R43" s="7" t="n">
-        <v>2.490369728122871</v>
+        <v>2.194649597899229</v>
       </c>
       <c r="S43" s="7" t="n">
-        <v>1.614700000000012</v>
+        <v>0.7311600000000035</v>
       </c>
       <c r="T43" t="n">
         <v>2934</v>
@@ -5305,10 +5305,10 @@
         <v>27.5</v>
       </c>
       <c r="R44" s="9" t="n">
-        <v>0.1775893840214113</v>
+        <v>0.158011131962128</v>
       </c>
       <c r="S44" s="9" t="n">
-        <v>29.85289999999997</v>
+        <v>13.12523999999999</v>
       </c>
       <c r="T44" s="8" t="n">
         <v>0</v>
@@ -5394,10 +5394,10 @@
         <v>40</v>
       </c>
       <c r="R45" s="9" t="n">
-        <v>0.2299841280794976</v>
+        <v>0.1918575987960248</v>
       </c>
       <c r="S45" s="9" t="n">
-        <v>11.26469363233483</v>
+        <v>6.228999999999978</v>
       </c>
       <c r="T45" s="8" t="n">
         <v>0</v>
@@ -5483,10 +5483,10 @@
         <v>72.5</v>
       </c>
       <c r="R46" s="9" t="n">
-        <v>0.7320202184071484</v>
+        <v>0.6990806212632025</v>
       </c>
       <c r="S46" s="9" t="n">
-        <v>14.37228152648387</v>
+        <v>7.823857891861563</v>
       </c>
       <c r="T46" s="8" t="n">
         <v>0</v>
@@ -5572,10 +5572,10 @@
         <v>55.00000000000001</v>
       </c>
       <c r="R47" s="9" t="n">
-        <v>1.233044880741913</v>
+        <v>1.11561978877154</v>
       </c>
       <c r="S47" s="9" t="n">
-        <v>4.640100000000002</v>
+        <v>2.403449999999994</v>
       </c>
       <c r="T47" s="8" t="n">
         <v>0</v>
@@ -5661,10 +5661,10 @@
         <v>65</v>
       </c>
       <c r="R48" s="9" t="n">
-        <v>0.7519596589411812</v>
+        <v>0.7538691783093013</v>
       </c>
       <c r="S48" s="9" t="n">
-        <v>11.00099999999999</v>
+        <v>5.464649999999965</v>
       </c>
       <c r="T48" s="8" t="n">
         <v>0</v>
@@ -5753,7 +5753,7 @@
         <v>0.3037168049522719</v>
       </c>
       <c r="S49" s="9" t="n">
-        <v>8.035322339850024</v>
+        <v>4.017755582743749</v>
       </c>
       <c r="T49" s="8" t="n">
         <v>0</v>
@@ -5842,7 +5842,7 @@
         <v>0.8313211400873555</v>
       </c>
       <c r="S50" s="9" t="n">
-        <v>21.85706566215555</v>
+        <v>11.69606438458181</v>
       </c>
       <c r="T50" s="8" t="n">
         <v>0</v>
@@ -5931,7 +5931,7 @@
         <v>281.2289883541462</v>
       </c>
       <c r="S51" s="9" t="n">
-        <v>0.1602999999999884</v>
+        <v>0.1202250000000094</v>
       </c>
       <c r="T51" s="8" t="n">
         <v>0</v>
@@ -6017,10 +6017,10 @@
         <v>66.66666666666666</v>
       </c>
       <c r="R52" s="9" t="n">
-        <v>27.97480308409141</v>
+        <v>27.97240403816286</v>
       </c>
       <c r="S52" s="9" t="n">
-        <v>2.40373333333333</v>
+        <v>1.802800000000006</v>
       </c>
       <c r="T52" s="8" t="n">
         <v>0</v>
@@ -6109,7 +6109,7 @@
         <v>0.09729948417113379</v>
       </c>
       <c r="S53" s="9" t="n">
-        <v>0.8924999999999819</v>
+        <v>0.4462500000000546</v>
       </c>
       <c r="T53" s="8" t="n">
         <v>0</v>
@@ -6195,10 +6195,10 @@
         <v>32.5</v>
       </c>
       <c r="R54" s="9" t="n">
-        <v>0.06456599792850652</v>
+        <v>0.06452367787659215</v>
       </c>
       <c r="S54" s="9" t="n">
-        <v>788.715587756936</v>
+        <v>788.866111594383</v>
       </c>
       <c r="T54" s="8" t="n">
         <v>0</v>
@@ -6284,10 +6284,10 @@
         <v>40</v>
       </c>
       <c r="R55" s="9" t="n">
-        <v>0.1147398118615589</v>
+        <v>0.1140036762292105</v>
       </c>
       <c r="S55" s="9" t="n">
-        <v>454.1069</v>
+        <v>236.0832935527387</v>
       </c>
       <c r="T55" s="8" t="n">
         <v>0</v>
@@ -6373,10 +6373,10 @@
         <v>20</v>
       </c>
       <c r="R56" s="9" t="n">
-        <v>0.6769134253450438</v>
+        <v>0.3364485981308411</v>
       </c>
       <c r="S56" s="9" t="n">
-        <v>0.1251570711246086</v>
+        <v>0.5020092049622971</v>
       </c>
       <c r="T56" s="8" t="n">
         <v>0</v>
@@ -6461,9 +6461,11 @@
       <c r="Q57" s="9" t="n">
         <v>85</v>
       </c>
-      <c r="R57" s="8" t="n"/>
+      <c r="R57" s="9" t="n">
+        <v>9.701353450188595</v>
+      </c>
       <c r="S57" s="9" t="n">
-        <v>0</v>
+        <v>0.1802799999999988</v>
       </c>
       <c r="T57" s="8" t="n">
         <v>0</v>
@@ -8726,80 +8728,79 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Profit Factor</t>
+          <t>Profit Factor [ALIGNED]</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>abs(sum(profit &gt; 0) / sum(profit &lt; 0))
-Uses 'profit' field only - EXCLUDES commission &amp; swap.
-Source: revenue_report.py:178, demo_report.py:163, orchestra_selector.py</t>
+          <t>abs(gross_profit / gross_loss) on position_net = profit + commission + swap.
+Deals are rolled up to positions first (consolidate.py positions_from_deals).
+Source: demo_report.py, generate_dashboards.py, orchestra_selector.py</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
           <t>abs(gross_profit / gross_loss) where each trade's P&amp;L
-INCLUDES commission &amp; swap. Computed on closed trades inception-to-date.</t>
+INCLUDES commission &amp; swap. Computed on closed positions inception-to-date.  -&gt; matches Bachelier.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Maximum Drawdown</t>
+          <t>Maximum Drawdown [PARTIAL]</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>starting_equity = 10000.0  &lt;- HARDCODED
-equity = starting_equity + cumsum(profit)
+          <t>equity = starting_balance + cumsum(position_net)
 DD% = max((peak - equity) / peak * 100)
-Closed-trade balance only.
-Source: orchestra_selector.py:174</t>
+starting_balance = account's deposits - withdrawals (NOT hardcoded $10K).
+Closed-trade equity curve.
+Source: orchestra_selector.py compute_max_drawdown()</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Peak-to-trough on REAL equity curve
 (balance + open-position floating P&amp;L).
-Uses each account's actual starting balance.</t>
+Same starting balance. Residual = floating P&amp;L on open trades only.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Win Rate</t>
+          <t>Win Rate [ALIGNED]</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
+          <t>wins / total_positions * 100, win = position_net &gt; 0.
+Deals rolled up to positions, so entry deals (profit=0) no longer count as losses.</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
           <t>wins / total_closed_trades * 100
-Counts each row in the trade table where profit &gt; 0 as a win. If the parquet stores MT5 deals rather than positions, entry deals (profit=0) count as losses, which deflates win rate by ~half.</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>wins / total_closed_trades * 100
-MFB counts round-trip positions, one row each.</t>
+MFB counts round-trip positions, one row each.  -&gt; matches.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Net P&amp;L</t>
+          <t>Net P&amp;L [ALIGNED]</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>sum(profit) across closed trades, EXCLUDING
-commission &amp; swap (those are separate columns).</t>
+          <t>sum(position_net) = sum(profit + commission + swap) across closed positions.</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>sum(profit + commission + swap) across closed trades.</t>
+          <t>sum(profit + commission + swap) across closed positions.  -&gt; matches.</t>
         </is>
       </c>
     </row>
@@ -8823,17 +8824,17 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Trade Count</t>
+          <t>Trade Count [ALIGNED]</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Count of rows in the consolidated parquet for the account (MT5 deals from the VPS pull).</t>
+          <t>Count of positions (deals grouped by position_id) for the account.</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Count of closed positions in MFB-ingested history.</t>
+          <t>Count of closed positions in MFB-ingested history.  -&gt; matches.</t>
         </is>
       </c>
     </row>
@@ -8847,42 +8848,42 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>1. orchestra_selector.py compute_max_drawdown(): replace 'starting_equity = 10000.0' with the account's actual initial balance (deposits - withdrawals up to the strategy start, or first observed balance). Pull from MFB get-my-accounts.json or the accounts master sheet.</t>
+          <t>[DONE 2026-06-13] 1. compute_max_drawdown() now uses the account's real starting balance (deposits - withdrawals) instead of a hardcoded $10K.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>2. Add a separate DD computation that mirrors MFB's equity-curve method (running balance + open floating P&amp;L) so PROP-firm DD limits are measured the same way prop firms measure them.</t>
+          <t>[DONE 2026-06-13] 3. PF / win-rate / net-P&amp;L are computed on position_net (profit + commission + swap), so they match MFB.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>3. revenue_report.py / demo_report.py PF: add a 'net PF' that includes commission and swap alongside the existing 'gross PF', so both numbers are available.</t>
+          <t>[DONE 2026-06-13] 4. consolidate.py positions_from_deals() rolls MT5 deals up to positions (group by position_id, sum profit + commission + swap); reports/dashboards aggregate on that.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>4. consolidate.py: roll MT5 deals up to positions (group by position_id, sum profit + commission + swap) so trade counts and win rates match MFB.</t>
+          <t>[OPEN] 2. Add a DD computation that includes open-position floating P&amp;L so it matches MFB's real-equity DD exactly (needs vps_extractor.py to export open positions). Only material for accounts holding trades over the snapshot.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>5. Investigate why active in-MFB accounts show zero trades in dashboards - check VPS pulls, consolidate.py exclusions, and dashboard ingestion. This is upstream of formula work.</t>
+          <t>[ONGOING] 5. Active in-MFB accounts showing zero trades: usually a stopped terminal on the VPS or a label not registered in the VPS-side accounts.json. See 'Data gap (Bach)' sheet.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>6. Add this reconciliation sheet to the daily dashboards as an 'Audit' tab so divergences are visible without leaving the workflow.</t>
+          <t>[OPEN] 6. Optionally surface this audit as a dashboard 'Audit' tab.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboards — 2026-06-18
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-17 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-18 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/15/2026 02:52</t>
+          <t>06/18/2026 13:25</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>53624.17</v>
+        <v>54520.87</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>129.07</v>
+        <v>132.9</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>40.62000000000001</v>
+        <v>954.83</v>
       </c>
       <c r="P2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>52.5</v>
+        <v>47.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.01201451680169</v>
+        <v>1.48323068124883</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>6.69</v>
+        <v>3.95</v>
       </c>
       <c r="T2" t="n">
-        <v>2857</v>
+        <v>2867</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>29451.83</v>
+        <v>29520.87</v>
       </c>
       <c r="V2" t="n">
-        <v>1812</v>
+        <v>1816</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.42317115855792</v>
+        <v>63.34147192186956</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.09</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/14/2026 22:36</t>
+          <t>06/18/2026 10:48</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/15/2026 02:57</t>
+          <t>06/18/2026 13:26</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1875,16 +1875,16 @@
         <v>183</v>
       </c>
       <c r="U10" s="7" t="n">
-        <v>216.02</v>
+        <v>299.4300000000001</v>
       </c>
       <c r="V10" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="W10" s="7" t="n">
-        <v>46.44808743169399</v>
+        <v>46.99453551912568</v>
       </c>
       <c r="X10" s="7" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="Y10" s="7" t="n">
         <v>9.93</v>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -2090,19 +2090,19 @@
         <v>44.95</v>
       </c>
       <c r="T12" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>595.8200000000001</v>
+        <v>601.8199999999999</v>
       </c>
       <c r="V12" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="W12" s="7" t="n">
-        <v>69.09090909090909</v>
+        <v>69.64285714285714</v>
       </c>
       <c r="X12" s="7" t="n">
-        <v>2.28</v>
+        <v>2.29</v>
       </c>
       <c r="Y12" s="7" t="n">
         <v>2.63</v>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/14/2026 11:07</t>
+          <t>06/17/2026 23:14</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2377,20 +2377,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/14/2026 23:56</t>
+          <t>06/18/2026 11:41</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>835.14</v>
+        <v>1530.09</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-95.92</v>
+        <v>-92.52</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>97.09999999999999</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L15" s="7" t="n">
         <v>20422.4</v>
@@ -2402,31 +2402,31 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>-377.25</v>
+        <v>719.1900000000001</v>
       </c>
       <c r="P15" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>27.5</v>
+        <v>42.5</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>0.6173158855751674</v>
+        <v>2.000305993295965</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>2.34</v>
+        <v>0.88</v>
       </c>
       <c r="T15" t="n">
-        <v>1639</v>
+        <v>1664</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-19118.12</v>
+        <v>-19197.29</v>
       </c>
       <c r="V15" t="n">
-        <v>537</v>
+        <v>546</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>32.76388041488713</v>
+        <v>32.8125</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>0.6899999999999999</v>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2526,16 +2526,16 @@
         <v>7.53</v>
       </c>
       <c r="T16" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-2836.789999999999</v>
+        <v>-2838.65</v>
       </c>
       <c r="V16" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>41.7910447761194</v>
+        <v>41.60583941605839</v>
       </c>
       <c r="X16" s="7" t="n">
         <v>0.77</v>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2744,22 +2744,22 @@
         <v>3.91</v>
       </c>
       <c r="T18" t="n">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="U18" s="7" t="n">
-        <v>-7426.8</v>
+        <v>-7478.23</v>
       </c>
       <c r="V18" t="n">
         <v>51</v>
       </c>
       <c r="W18" s="7" t="n">
-        <v>13.11053984575835</v>
+        <v>13.04347826086956</v>
       </c>
       <c r="X18" s="7" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="Y18" s="7" t="n">
-        <v>37.13</v>
+        <v>37.39</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
@@ -2813,20 +2813,20 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>06/15/2026 06:19</t>
+          <t>06/18/2026 16:32</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
-        <v>15955.63</v>
+        <v>16043.85</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>-20.22</v>
+        <v>-19.78</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>22.29</v>
+        <v>26.73</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>0.61</v>
+        <v>0.7</v>
       </c>
       <c r="L19" t="n">
         <v>20000</v>
@@ -2838,7 +2838,7 @@
         <v>40</v>
       </c>
       <c r="O19" s="7" t="n">
-        <v>-657.51</v>
+        <v>1021.56</v>
       </c>
       <c r="P19" t="n">
         <v>17</v>
@@ -2847,25 +2847,25 @@
         <v>42.5</v>
       </c>
       <c r="R19" s="7" t="n">
-        <v>0.4975777118928997</v>
+        <v>2.054154455772485</v>
       </c>
       <c r="S19" s="7" t="n">
-        <v>4.52</v>
+        <v>1.96</v>
       </c>
       <c r="T19" t="n">
-        <v>411</v>
+        <v>431</v>
       </c>
       <c r="U19" s="7" t="n">
-        <v>-4839.559999999999</v>
+        <v>-4081.91</v>
       </c>
       <c r="V19" t="n">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="W19" s="7" t="n">
-        <v>35.76642335766424</v>
+        <v>36.42691415313225</v>
       </c>
       <c r="X19" s="7" t="n">
-        <v>0.62</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y19" s="7" t="n">
         <v>26.73</v>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>06/15/2026 06:03</t>
+          <t>06/18/2026 16:22</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -2932,7 +2932,7 @@
         <v>-4.15</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>7.47</v>
+        <v>10.31</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>0.14</v>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>06/15/2026 05:54</t>
+          <t>06/18/2026 16:16</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3289,19 +3289,19 @@
         <v>1.06</v>
       </c>
       <c r="T23" t="n">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-3840.48</v>
+        <v>-3906.64</v>
       </c>
       <c r="V23" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>35.36231884057971</v>
+        <v>35.54913294797688</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>20.19</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/15/2026 03:46</t>
+          <t>06/18/2026 14:06</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3510,7 +3510,7 @@
         <v>54</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>1151.41</v>
+        <v>978.2700000000001</v>
       </c>
       <c r="V25" t="n">
         <v>23</v>
@@ -3519,7 +3519,7 @@
         <v>42.5925925925926</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>1.58</v>
+        <v>1.45</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>2.33</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/15/2026 03:53</t>
+          <t>06/18/2026 14:20</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/15/2026 06:07</t>
+          <t>06/18/2026 16:24</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>19778.12</v>
+        <v>18858.24</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-1.1</v>
+        <v>-5.7</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>7.76</v>
+        <v>10.63</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.95</v>
+        <v>0.83</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,37 +3710,37 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>133.35</v>
+        <v>-361.64</v>
       </c>
       <c r="P27" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>70</v>
+        <v>32.5</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>5.303000968054212</v>
+        <v>0.1439662926667614</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>0.13</v>
+        <v>2.04</v>
       </c>
       <c r="T27" t="n">
-        <v>1492</v>
+        <v>1566</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>-901.4700000000001</v>
+        <v>-1150.03</v>
       </c>
       <c r="V27" t="n">
-        <v>924</v>
+        <v>986</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>61.93029490616622</v>
+        <v>62.96296296296296</v>
       </c>
       <c r="X27" s="7" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="Y27" s="7" t="n">
-        <v>9.039999999999999</v>
+        <v>10.64</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3834,7 +3834,7 @@
         <v>6.09</v>
       </c>
       <c r="T28" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="U28" s="7" t="n">
         <v>-522.7900000000001</v>
@@ -3843,7 +3843,7 @@
         <v>28</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>63.63636363636363</v>
+        <v>62.22222222222222</v>
       </c>
       <c r="X28" s="7" t="n">
         <v>0.61</v>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/15/2026 06:07</t>
+          <t>06/18/2026 16:23</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4230,20 +4230,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/14/2026 21:37</t>
+          <t>06/18/2026 09:30</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>20517.83</v>
+        <v>20317.66</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>2.58</v>
+        <v>1.58</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>0.7</v>
+        <v>1.61</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>2.07</v>
+        <v>1.46</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4252,40 +4252,40 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>20517.83</v>
+        <v>20317.66</v>
       </c>
       <c r="P32" t="n">
         <v>18</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>58.06451612903226</v>
+        <v>51.42857142857142</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>43.40973542786276</v>
+        <v>30.70548415866193</v>
       </c>
       <c r="S32" s="7" t="n">
-        <v>0.35</v>
+        <v>0.82</v>
       </c>
       <c r="T32" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>317.66</v>
+        <v>270.9299999999999</v>
       </c>
       <c r="V32" t="n">
         <v>17</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>50</v>
+        <v>48.57142857142857</v>
       </c>
       <c r="X32" s="7" t="n">
-        <v>1.46</v>
+        <v>1.37</v>
       </c>
       <c r="Y32" s="7" t="n">
-        <v>1.61</v>
+        <v>1.83</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
@@ -4379,19 +4379,19 @@
         <v>7.77</v>
       </c>
       <c r="T33" t="n">
-        <v>919</v>
+        <v>958</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>-1548.89</v>
+        <v>-2047.07</v>
       </c>
       <c r="V33" t="n">
-        <v>454</v>
+        <v>471</v>
       </c>
       <c r="W33" s="7" t="n">
-        <v>49.40152339499456</v>
+        <v>49.16492693110647</v>
       </c>
       <c r="X33" s="7" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="Y33" s="7" t="n">
         <v>24.46</v>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -4488,19 +4488,19 @@
         <v>0.74</v>
       </c>
       <c r="T34" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>1043.45</v>
+        <v>836.2099999999999</v>
       </c>
       <c r="V34" t="n">
         <v>16</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>72.72727272727273</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>2.73</v>
+        <v>2.03</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>1.44</v>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4709,16 +4709,16 @@
         <v>15</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-793.6999999999999</v>
+        <v>-724.35</v>
       </c>
       <c r="V36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>0</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>3.97</v>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4884,17 +4884,17 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/14/2026 23:54</t>
+          <t>06/18/2026 11:40</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
-        <v>19281.85</v>
+        <v>19096.05</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>-3.59</v>
+        <v>-4.52</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>3.59</v>
+        <v>4.52</v>
       </c>
       <c r="K38" s="7" t="n">
         <v>0.37</v>
@@ -4906,40 +4906,40 @@
         <v>0</v>
       </c>
       <c r="N38" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>19060.69</v>
+        <v>18837.77</v>
       </c>
       <c r="P38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q38" s="7" t="n">
-        <v>17.39130434782609</v>
+        <v>17.24137931034483</v>
       </c>
       <c r="R38" s="7" t="n">
-        <v>15.34083453713736</v>
+        <v>12.43144870106621</v>
       </c>
       <c r="S38" s="7" t="n">
-        <v>2.35</v>
+        <v>2.91</v>
       </c>
       <c r="T38" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U38" s="7" t="n">
-        <v>-842.4400000000001</v>
+        <v>-903.95</v>
       </c>
       <c r="V38" t="n">
         <v>4</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>14.81481481481481</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="X38" s="7" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="Y38" s="7" t="n">
-        <v>4.21</v>
+        <v>4.52</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
@@ -4948,12 +4948,12 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
@@ -5033,22 +5033,22 @@
         <v>3.02</v>
       </c>
       <c r="T39" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="U39" s="7" t="n">
-        <v>-652.34</v>
+        <v>-635.0599999999999</v>
       </c>
       <c r="V39" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="W39" s="7" t="n">
-        <v>18.86792452830189</v>
+        <v>21.05263157894737</v>
       </c>
       <c r="X39" s="7" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="Y39" s="7" t="n">
-        <v>3.72</v>
+        <v>3.82</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
@@ -5057,7 +5057,7 @@
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB39" t="inlineStr">
@@ -5142,22 +5142,22 @@
         <v>4.47</v>
       </c>
       <c r="T40" t="n">
-        <v>564</v>
+        <v>580</v>
       </c>
       <c r="U40" s="7" t="n">
-        <v>-19341.58</v>
+        <v>-19291.32</v>
       </c>
       <c r="V40" t="n">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="W40" s="7" t="n">
-        <v>41.84397163120568</v>
+        <v>41.89655172413793</v>
       </c>
       <c r="X40" s="7" t="n">
         <v>0.83</v>
       </c>
       <c r="Y40" s="7" t="n">
-        <v>96.2</v>
+        <v>96.22</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB40" t="inlineStr">
@@ -5251,19 +5251,19 @@
         <v>2.6</v>
       </c>
       <c r="T41" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U41" s="7" t="n">
-        <v>33.83000000000008</v>
+        <v>59.51000000000008</v>
       </c>
       <c r="V41" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W41" s="7" t="n">
-        <v>43.18181818181818</v>
+        <v>43.47826086956522</v>
       </c>
       <c r="X41" s="7" t="n">
-        <v>1.02</v>
+        <v>1.04</v>
       </c>
       <c r="Y41" s="7" t="n">
         <v>2.56</v>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB41" t="inlineStr">
@@ -5469,22 +5469,22 @@
         <v>0.5</v>
       </c>
       <c r="T43" t="n">
-        <v>2952</v>
+        <v>2973</v>
       </c>
       <c r="U43" s="7" t="n">
-        <v>-4924.13</v>
+        <v>-5701.509999999999</v>
       </c>
       <c r="V43" t="n">
-        <v>1788</v>
+        <v>1789</v>
       </c>
       <c r="W43" s="7" t="n">
-        <v>60.56910569105691</v>
+        <v>60.1749075008409</v>
       </c>
       <c r="X43" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="Y43" s="7" t="n">
-        <v>28.95</v>
+        <v>29.84</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -5493,7 +5493,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>06/15/2026 01:06</t>
+          <t>06/18/2026 12:26</t>
         </is>
       </c>
       <c r="H44" s="9" t="n">
@@ -5993,7 +5993,7 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>06/15/2026 05:40</t>
+          <t>06/18/2026 16:08</t>
         </is>
       </c>
       <c r="H49" s="9" t="n">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>06/15/2026 06:31</t>
+          <t>06/18/2026 16:36</t>
         </is>
       </c>
       <c r="H51" s="9" t="n">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>06/14/2026 12:31</t>
+          <t>06/18/2026 03:13</t>
         </is>
       </c>
       <c r="H54" s="9" t="n">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>06/14/2026 11:38</t>
+          <t>06/18/2026 00:38</t>
         </is>
       </c>
       <c r="H55" s="9" t="n">
@@ -6896,7 +6896,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>06/15/2026 01:06</t>
+          <t>06/18/2026 12:26</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -7101,7 +7101,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06/15/2026 05:40</t>
+          <t>06/18/2026 16:08</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>06/15/2026 06:31</t>
+          <t>06/18/2026 16:36</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -7306,7 +7306,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/14/2026 12:31</t>
+          <t>06/18/2026 03:13</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -7347,7 +7347,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/14/2026 11:38</t>
+          <t>06/18/2026 00:38</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -8545,7 +8545,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06/14/2026 21:19</t>
+          <t>06/18/2026 08:44</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -8591,7 +8591,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06/11/2026 21:10</t>
+          <t>06/18/2026 08:58</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>06/15/2026 03:07</t>
+          <t>06/18/2026 13:33</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -8821,7 +8821,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06/14/2026 21:20</t>
+          <t>06/18/2026 08:44</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
@@ -8959,11 +8959,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06/14/2026 21:28</t>
+          <t>06/18/2026 09:02</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>20028.6</v>
+        <v>20028.16</v>
       </c>
     </row>
     <row r="23">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06/14/2026 21:17</t>
+          <t>06/18/2026 08:36</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06/14/2026 21:20</t>
+          <t>06/18/2026 08:44</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06/17/2026 04:00</t>
+          <t>06/18/2026 04:02</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-06-23
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/22/2026 15:56</t>
+          <t>06/23/2026 14:39</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>51435.01</v>
+        <v>47822.05</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>127.72</v>
+        <v>123.04</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>320.5100000000001</v>
+        <v>-1591.92</v>
       </c>
       <c r="P2" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>57.49999999999999</v>
+        <v>47.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.327887468030691</v>
+        <v>0.2779393021241081</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>3.25</v>
+        <v>6.41</v>
       </c>
       <c r="T2" t="n">
-        <v>2911</v>
+        <v>2912</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>22811.23</v>
+        <v>22811.22999999999</v>
       </c>
       <c r="V2" t="n">
         <v>1836</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.07110958433528</v>
+        <v>63.04945054945055</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.07</v>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/22/2026 15:54</t>
+          <t>06/23/2026 14:37</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -2417,16 +2417,16 @@
         <v>1.83</v>
       </c>
       <c r="T15" t="n">
-        <v>1746</v>
+        <v>1748</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-19250.95</v>
+        <v>-19308.21</v>
       </c>
       <c r="V15" t="n">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>32.53150057273768</v>
+        <v>32.55148741418764</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>0.7</v>
@@ -3401,7 +3401,7 @@
         <v>363</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>-3942.34</v>
+        <v>-3965.110000000001</v>
       </c>
       <c r="V24" t="n">
         <v>130</v>
@@ -4270,16 +4270,16 @@
         <v>3.51</v>
       </c>
       <c r="T32" t="n">
-        <v>1092</v>
+        <v>1094</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>-3401.46</v>
+        <v>-3318.46</v>
       </c>
       <c r="V32" t="n">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>48.62637362637363</v>
+        <v>48.62888482632541</v>
       </c>
       <c r="X32" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -4884,20 +4884,20 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/22/2026 23:07</t>
+          <t>06/23/2026 14:24</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
-        <v>19666.3</v>
+        <v>19829.17</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>-1.67</v>
+        <v>-0.86</v>
       </c>
       <c r="J38" s="7" t="n">
         <v>3.82</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>0.78</v>
+        <v>0.9</v>
       </c>
       <c r="L38" t="n">
         <v>20000</v>
@@ -4909,19 +4909,19 @@
         <v>40</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>-119.99</v>
+        <v>255.51</v>
       </c>
       <c r="P38" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Q38" s="7" t="n">
-        <v>32.5</v>
+        <v>40</v>
       </c>
       <c r="R38" s="7" t="n">
-        <v>0.884670466450726</v>
+        <v>1.279233694701871</v>
       </c>
       <c r="S38" s="7" t="n">
-        <v>2.44</v>
+        <v>2.41</v>
       </c>
       <c r="T38" t="n">
         <v>67</v>
@@ -5360,7 +5360,7 @@
         <v>5.31</v>
       </c>
       <c r="T42" t="n">
-        <v>3017</v>
+        <v>3018</v>
       </c>
       <c r="U42" s="7" t="n">
         <v>-6330.909999999999</v>
@@ -5369,7 +5369,7 @@
         <v>1792</v>
       </c>
       <c r="W42" s="7" t="n">
-        <v>59.39675174013921</v>
+        <v>59.37707090788602</v>
       </c>
       <c r="X42" s="7" t="n">
         <v>0.78</v>
@@ -8357,7 +8357,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Agg V1 AUDUSD</t>
+          <t>Sweep suite</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Agg V1 NZDJPY</t>
+          <t>NY Killzone</t>
         </is>
       </c>
       <c r="D38" t="b">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Agg V1 Pro XAUUSD</t>
+          <t>Aggv1 Pro Filter 60</t>
         </is>
       </c>
       <c r="D41" t="b">

</xml_diff>

<commit_message>
Update dashboards — 2026-06-24
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-23 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-24 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/23/2026 21:56</t>
+          <t>06/24/2026 19:53</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>46369.25</v>
+        <v>46040.75</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>116.26</v>
+        <v>114.73</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-2268.12</v>
+        <v>-2638.47</v>
       </c>
       <c r="P2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>50</v>
+        <v>47.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.2161598009400055</v>
+        <v>0.4102000670615849</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>10.96</v>
+        <v>14.03</v>
       </c>
       <c r="T2" t="n">
-        <v>2914</v>
+        <v>2933</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>21357.76999999999</v>
+        <v>21030.03999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>1838</v>
+        <v>1849</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.07481125600549</v>
+        <v>63.04125468803273</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.06</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,11 +1069,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/23/2026 09:44</t>
+          <t>06/24/2026 13:51</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
-        <v>3788.13</v>
+        <v>23788.13</v>
       </c>
       <c r="I3" s="7" t="n">
         <v>14.67</v>
@@ -1085,7 +1085,7 @@
         <v>1</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>30545.04</v>
+        <v>50545.04</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>26858.3</v>
@@ -1094,7 +1094,7 @@
         <v>40</v>
       </c>
       <c r="O3" s="7" t="n">
-        <v>-27542.57</v>
+        <v>-7626.92</v>
       </c>
       <c r="P3" t="n">
         <v>21</v>
@@ -1103,10 +1103,10 @@
         <v>52.5</v>
       </c>
       <c r="R3" s="7" t="n">
-        <v>0.04321326676053001</v>
+        <v>0.7350524707215493</v>
       </c>
       <c r="S3" s="7" t="n">
-        <v>650.02</v>
+        <v>116.25</v>
       </c>
       <c r="T3" t="n">
         <v>1000</v>
@@ -1124,7 +1124,7 @@
         <v>1</v>
       </c>
       <c r="Y3" s="7" t="n">
-        <v>47.32</v>
+        <v>12.52</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -1178,20 +1178,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/23/2026 20:25</t>
+          <t>06/24/2026 16:59</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>21582.12</v>
+        <v>21754.38</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>7.87</v>
+        <v>8.73</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>5.78</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1.16</v>
+        <v>1.18</v>
       </c>
       <c r="L4" t="n">
         <v>20000</v>
@@ -1203,7 +1203,7 @@
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>549.2300000000001</v>
+        <v>546.2600000000001</v>
       </c>
       <c r="P4" t="n">
         <v>28</v>
@@ -1212,25 +1212,25 @@
         <v>70</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>1.156062285113517</v>
+        <v>1.15521836728895</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>6.51</v>
+        <v>6.56</v>
       </c>
       <c r="T4" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>1582.12</v>
+        <v>1754.38</v>
       </c>
       <c r="V4" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>65.2542372881356</v>
+        <v>65.54621848739495</v>
       </c>
       <c r="X4" s="7" t="n">
-        <v>1.16</v>
+        <v>1.18</v>
       </c>
       <c r="Y4" s="7" t="n">
         <v>5.78</v>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/23/2026 16:41</t>
+          <t>06/24/2026 05:56</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/23/2026 18:07</t>
+          <t>06/24/2026 07:18</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/23/2026 14:37</t>
+          <t>06/24/2026 19:48</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/21/2026 19:37</t>
+          <t>06/24/2026 19:45</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>06/18/2026 19:14</t>
+          <t>06/24/2026 19:21</t>
         </is>
       </c>
       <c r="H11" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/23/2026 07:44</t>
+          <t>06/24/2026 11:46</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>06/20/2026 23:19</t>
+          <t>06/23/2026 23:23</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>06/23/2026 17:36</t>
+          <t>06/24/2026 13:07</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -2377,20 +2377,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/23/2026 20:49</t>
+          <t>06/24/2026 17:31</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>1228.06</v>
-      </c>
-      <c r="I15" t="n">
-        <v>-94</v>
+        <v>1601.98</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>-92.17</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>98.18000000000001</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="L15" s="7" t="n">
         <v>20422.4</v>
@@ -2402,31 +2402,31 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>-206.42</v>
+        <v>419.01</v>
       </c>
       <c r="P15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>27.5</v>
+        <v>35</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>0.6896359891142552</v>
+        <v>2.439303380049464</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>1.84</v>
+        <v>0.61</v>
       </c>
       <c r="T15" t="n">
-        <v>1759</v>
+        <v>1786</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-19194.34</v>
+        <v>-18886.88</v>
       </c>
       <c r="V15" t="n">
-        <v>573</v>
+        <v>582</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>32.57532689027857</v>
+        <v>32.58678611422172</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>0.7</v>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2486,20 +2486,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>06/23/2026 11:41</t>
+          <t>06/24/2026 16:23</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>17044.2</v>
+        <v>17676.49</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-14.8</v>
+        <v>-11.64</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>17.06</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.77</v>
+        <v>0.82</v>
       </c>
       <c r="L16" t="n">
         <v>20000</v>
@@ -2511,34 +2511,34 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-752.1099999999999</v>
+        <v>-118.5999999999999</v>
       </c>
       <c r="P16" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>37.5</v>
+        <v>42.5</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.757061781910856</v>
+        <v>0.9574222129679159</v>
       </c>
       <c r="S16" s="7" t="n">
         <v>6.33</v>
       </c>
       <c r="T16" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-2649.15</v>
+        <v>-2323.51</v>
       </c>
       <c r="V16" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>42.75862068965517</v>
+        <v>43.53741496598639</v>
       </c>
       <c r="X16" s="7" t="n">
-        <v>0.8</v>
+        <v>0.82</v>
       </c>
       <c r="Y16" s="7" t="n">
         <v>17.04</v>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>06/22/2026 12:54</t>
+          <t>06/24/2026 14:43</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>06/23/2026 16:35</t>
+          <t>06/24/2026 11:53</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>06/23/2026 23:10</t>
+          <t>06/24/2026 05:39</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2962,19 +2962,19 @@
         <v>11.7</v>
       </c>
       <c r="T20" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-5006.83</v>
+        <v>-4900</v>
       </c>
       <c r="V20" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>42.26190476190476</v>
+        <v>42.60355029585799</v>
       </c>
       <c r="X20" s="7" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="Y20" s="7" t="n">
         <v>37.21</v>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>06/23/2026 16:52</t>
+          <t>06/24/2026 12:12</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>06/23/2026 22:52</t>
+          <t>06/24/2026 05:22</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3358,20 +3358,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/23/2026 23:06</t>
+          <t>06/24/2026 11:41</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>15997.59</v>
+        <v>15859.7</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>-19.75</v>
+        <v>-20.45</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>19.93</v>
+        <v>20.45</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="L24" t="n">
         <v>20000</v>
@@ -3383,37 +3383,37 @@
         <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>-114.34</v>
+        <v>-320.12</v>
       </c>
       <c r="P24" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Q24" s="7" t="n">
-        <v>52.5</v>
+        <v>45</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>0.7390272293611486</v>
+        <v>0.4429692529885677</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>0.99</v>
+        <v>1.68</v>
       </c>
       <c r="T24" t="n">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>-4002.41</v>
+        <v>-4158.38</v>
       </c>
       <c r="V24" t="n">
         <v>131</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>35.79234972677596</v>
+        <v>35.12064343163539</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="Y24" s="7" t="n">
-        <v>20.19</v>
+        <v>20.79</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -3507,22 +3507,22 @@
         <v>2.73</v>
       </c>
       <c r="T25" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>1135.89</v>
+        <v>488.3500000000001</v>
       </c>
       <c r="V25" t="n">
         <v>26</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>41.93548387096774</v>
+        <v>40.625</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>1.49</v>
+        <v>1.17</v>
       </c>
       <c r="Y25" s="7" t="n">
-        <v>2.58</v>
+        <v>4.18</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/21/2026 14:26</t>
+          <t>06/24/2026 14:29</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/23/2026 07:58</t>
+          <t>06/24/2026 11:58</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/23/2026 23:13</t>
+          <t>06/24/2026 11:47</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/23/2026 16:23</t>
+          <t>06/24/2026 11:43</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20677.59</v>
+        <v>20683.77</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>3.4</v>
+        <v>3.43</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>1.09</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>2.65</v>
+        <v>2.66</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3925,37 +3925,37 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>20677.31</v>
+        <v>20683.09</v>
       </c>
       <c r="P29" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>28.94736842105263</v>
+        <v>30</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>51.49157550302794</v>
+        <v>51.13110184691453</v>
       </c>
       <c r="S29" s="7" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="T29" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>677.59</v>
+        <v>683.77</v>
       </c>
       <c r="V29" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>27.02702702702703</v>
+        <v>28.2051282051282</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>2.65</v>
+        <v>2.66</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>1.1</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
+          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/23/2026 17:03</t>
+          <t>06/24/2026 12:22</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>19648.6</v>
+        <v>19663.56</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>-1.75</v>
+        <v>-1.68</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>1.8</v>
+        <v>1.86</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>0.6</v>
+        <v>0.64</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,37 +4037,37 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>-43.16</v>
+        <v>2.969999999999999</v>
       </c>
       <c r="P30" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>50</v>
+        <v>62.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>0.3441726181431393</v>
+        <v>1.085027197251646</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="T30" t="n">
-        <v>778</v>
+        <v>796</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>-376.58</v>
+        <v>-354.84</v>
       </c>
       <c r="V30" t="n">
-        <v>320</v>
+        <v>358</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>41.13110539845758</v>
+        <v>44.9748743718593</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>0.58</v>
+        <v>0.62</v>
       </c>
       <c r="Y30" s="7" t="n">
-        <v>1.93</v>
+        <v>1.87</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/23/2026 19:45</t>
+          <t>06/24/2026 08:43</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4161,19 +4161,19 @@
         <v>1.13</v>
       </c>
       <c r="T31" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>207.02</v>
+        <v>243.49</v>
       </c>
       <c r="V31" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>47.36842105263158</v>
+        <v>47.5</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>1.26</v>
+        <v>1.29</v>
       </c>
       <c r="Y31" s="7" t="n">
         <v>2.18</v>
@@ -4185,12 +4185,12 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr">
@@ -4230,20 +4230,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/23/2026 02:25</t>
+          <t>06/24/2026 07:18</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>17010.39</v>
+        <v>16545.65</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>-14.96</v>
+        <v>-17.29</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>27.69</v>
+        <v>29.45</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4255,37 +4255,37 @@
         <v>40</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>-38.73</v>
+        <v>-235.98</v>
       </c>
       <c r="P32" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>50</v>
+        <v>47.5</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>0.9780880663977415</v>
+        <v>0.8716090490647341</v>
       </c>
       <c r="S32" s="7" t="n">
-        <v>3.51</v>
+        <v>4.03</v>
       </c>
       <c r="T32" t="n">
-        <v>1113</v>
+        <v>1167</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>-2985.059999999999</v>
+        <v>-4514.039999999999</v>
       </c>
       <c r="V32" t="n">
-        <v>544</v>
+        <v>563</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>48.87690925426774</v>
+        <v>48.24335904027421</v>
       </c>
       <c r="X32" s="7" t="n">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="Y32" s="7" t="n">
-        <v>29.19</v>
+        <v>33.94</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
@@ -4379,19 +4379,19 @@
         <v>0.74</v>
       </c>
       <c r="T33" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>936.17</v>
+        <v>831.39</v>
       </c>
       <c r="V33" t="n">
         <v>18</v>
       </c>
       <c r="W33" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>64.28571428571429</v>
       </c>
       <c r="X33" s="7" t="n">
-        <v>2.03</v>
+        <v>1.82</v>
       </c>
       <c r="Y33" s="7" t="n">
         <v>1.47</v>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>06/23/2026 09:08</t>
+          <t>06/24/2026 00:16</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20543.08</v>
+        <v>20618.05</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>2.71</v>
+        <v>3.08</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>5.13</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.19</v>
+        <v>1.21</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4470,19 +4470,19 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>20390.27</v>
+        <v>20455.2</v>
       </c>
       <c r="P34" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>46.42857142857143</v>
+        <v>46.66666666666666</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>8.0506505945774</v>
+        <v>7.879582419652106</v>
       </c>
       <c r="S34" s="7" t="n">
         <v>2.85</v>
@@ -4491,19 +4491,19 @@
         <v>29</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>538.1199999999999</v>
+        <v>618.05</v>
       </c>
       <c r="V34" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>41.37931034482759</v>
+        <v>44.82758620689656</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1.19</v>
+        <v>1.21</v>
       </c>
       <c r="Y34" s="7" t="n">
-        <v>5.16</v>
+        <v>5.14</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -4512,12 +4512,12 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC34" t="inlineStr">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>06/23/2026 19:03</t>
+          <t>06/24/2026 15:10</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>18863.18</v>
+        <v>18734.06</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>-4.76</v>
+        <v>-5.41</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>4.76</v>
+        <v>5.41</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4579,40 +4579,40 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>19037.08</v>
+        <v>18907.64</v>
       </c>
       <c r="P35" t="n">
         <v>2</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>11.11111111111111</v>
+        <v>10.52631578947368</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>19.46163096288682</v>
+        <v>17.29112277164594</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>2.41</v>
+        <v>2.73</v>
       </c>
       <c r="T35" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>-1136.82</v>
+        <v>-1265.94</v>
       </c>
       <c r="V35" t="n">
         <v>1</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>5.555555555555555</v>
+        <v>5</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="Y35" s="7" t="n">
-        <v>5.68</v>
+        <v>6.33</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/23/2026 10:43</t>
+          <t>06/24/2026 01:47</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19819.08</v>
+        <v>19724.08</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.9</v>
+        <v>-1.38</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>2.88</v>
+        <v>3.35</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.75</v>
+        <v>0.67</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4688,40 +4688,40 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>19811.71</v>
+        <v>19715.19</v>
       </c>
       <c r="P36" t="n">
         <v>4</v>
       </c>
       <c r="Q36" s="7" t="n">
-        <v>40</v>
+        <v>36.36363636363637</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>27.96791625830338</v>
+        <v>24.72008999470619</v>
       </c>
       <c r="S36" s="7" t="n">
-        <v>1.47</v>
+        <v>1.71</v>
       </c>
       <c r="T36" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-275.92</v>
+        <v>-413.09</v>
       </c>
       <c r="V36" t="n">
         <v>3</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>27.27272727272727</v>
+        <v>23.07692307692308</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>0.67</v>
+        <v>0.57</v>
       </c>
       <c r="Y36" s="7" t="n">
-        <v>3.35</v>
+        <v>4.02</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4775,20 +4775,20 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/23/2026 20:50</t>
+          <t>06/24/2026 17:39</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>19114.77</v>
+        <v>19052.27</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-4.43</v>
+        <v>-4.74</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>4.52</v>
+        <v>4.74</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>0.43</v>
+        <v>0.41</v>
       </c>
       <c r="L37" t="n">
         <v>20000</v>
@@ -4797,40 +4797,40 @@
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>18830.49</v>
+        <v>18753.79</v>
       </c>
       <c r="P37" t="n">
         <v>6</v>
       </c>
       <c r="Q37" s="7" t="n">
-        <v>18.75</v>
+        <v>18.18181818181818</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>11.54049560870758</v>
+        <v>11.06542005914587</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>2.92</v>
+        <v>3.12</v>
       </c>
       <c r="T37" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-885.2300000000001</v>
+        <v>-947.73</v>
       </c>
       <c r="V37" t="n">
         <v>5</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>16.12903225806452</v>
+        <v>15.625</v>
       </c>
       <c r="X37" s="7" t="n">
-        <v>0.43</v>
+        <v>0.41</v>
       </c>
       <c r="Y37" s="7" t="n">
-        <v>4.52</v>
+        <v>4.74</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
@@ -4884,20 +4884,20 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/23/2026 21:46</t>
+          <t>06/24/2026 19:44</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
-        <v>19829.17</v>
+        <v>19786.14</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>-0.86</v>
+        <v>-1.07</v>
       </c>
       <c r="J38" s="7" t="n">
         <v>3.82</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="L38" t="n">
         <v>20000</v>
@@ -4909,34 +4909,34 @@
         <v>40</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>255.51</v>
+        <v>60.24999999999997</v>
       </c>
       <c r="P38" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q38" s="7" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="R38" s="7" t="n">
-        <v>1.279233694701871</v>
+        <v>1.063850531469569</v>
       </c>
       <c r="S38" s="7" t="n">
-        <v>2.41</v>
+        <v>2.42</v>
       </c>
       <c r="T38" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="U38" s="7" t="n">
-        <v>-170.83</v>
+        <v>-213.86</v>
       </c>
       <c r="V38" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>28.35820895522388</v>
+        <v>27.77777777777778</v>
       </c>
       <c r="X38" s="7" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="Y38" s="7" t="n">
         <v>3.82</v>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
@@ -4993,20 +4993,20 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>06/23/2026 23:02</t>
+          <t>06/24/2026 11:34</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
-        <v>19451.53</v>
+        <v>19468.83</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>-2.74</v>
+        <v>-2.66</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>3.05</v>
+        <v>3.09</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>0.66</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L39" t="n">
         <v>20000</v>
@@ -5018,19 +5018,19 @@
         <v>40</v>
       </c>
       <c r="O39" s="7" t="n">
-        <v>-25.70000000000001</v>
+        <v>-4.13</v>
       </c>
       <c r="P39" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q39" s="7" t="n">
-        <v>42.5</v>
+        <v>40</v>
       </c>
       <c r="R39" s="7" t="n">
-        <v>0.7339544513457555</v>
+        <v>0.9481351249529073</v>
       </c>
       <c r="S39" s="7" t="n">
-        <v>0.41</v>
+        <v>0.13</v>
       </c>
       <c r="T39" t="n">
         <v>598</v>
@@ -5102,20 +5102,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/23/2026 23:04</t>
+          <t>06/24/2026 11:36</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
-        <v>18649.95</v>
+        <v>18720.85</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>-6.75</v>
+        <v>-6.4</v>
       </c>
       <c r="J40" s="7" t="n">
         <v>7.5</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>0.58</v>
+        <v>0.63</v>
       </c>
       <c r="L40" t="n">
         <v>20000</v>
@@ -5124,13 +5124,22 @@
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O40" s="7" t="n">
-        <v>0</v>
+        <v>8.339999999999998</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q40" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R40" s="7" t="n">
+        <v>1.145727765158134</v>
+      </c>
+      <c r="S40" s="7" t="n">
+        <v>0.12</v>
       </c>
       <c r="T40" t="n">
         <v>1179</v>
@@ -5202,20 +5211,20 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>06/23/2026 23:02</t>
+          <t>06/24/2026 11:33</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
-        <v>20329.87</v>
+        <v>20396.08</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>1.65</v>
+        <v>1.98</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K41" s="7" t="n">
-        <v>2.7</v>
+        <v>3.04</v>
       </c>
       <c r="L41" t="n">
         <v>20000</v>
@@ -5224,19 +5233,19 @@
         <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O41" s="7" t="n">
-        <v>20286.35</v>
+        <v>20349.08</v>
       </c>
       <c r="P41" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q41" s="7" t="n">
-        <v>53.84615384615385</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="R41" s="7" t="n">
-        <v>94.39940147329651</v>
+        <v>94.68821362799264</v>
       </c>
       <c r="S41" s="7" t="n">
         <v>0.28</v>
@@ -5311,7 +5320,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>06/23/2026 23:05</t>
+          <t>06/24/2026 11:36</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5333,13 +5342,22 @@
         <v>0</v>
       </c>
       <c r="N42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>0</v>
+        <v>194.98</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>29</v>
+      </c>
+      <c r="Q42" s="7" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="R42" s="7" t="n">
+        <v>2.761018786127167</v>
+      </c>
+      <c r="S42" s="7" t="n">
+        <v>0.27</v>
       </c>
       <c r="T42" t="n">
         <v>110</v>
@@ -5411,7 +5429,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>06/23/2026 16:16</t>
+          <t>06/24/2026 11:38</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5511,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/23/2026 16:25</t>
+          <t>06/24/2026 11:49</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5611,7 +5629,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/23/2026 23:08</t>
+          <t>06/24/2026 11:39</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5711,20 +5729,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/23/2026 23:10</t>
+          <t>06/24/2026 11:41</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19940.94</v>
+        <v>19932.03</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-0.3</v>
+        <v>-0.34</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>2.23</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5811,7 +5829,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/23/2026 23:10</t>
+          <t>06/24/2026 05:40</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5911,20 +5929,20 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/23/2026 16:21</t>
+          <t>06/24/2026 11:46</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
-        <v>22319.93</v>
+        <v>22327.87</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="J48" s="7" t="n">
         <v>5.53</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>1.47</v>
+        <v>1.46</v>
       </c>
       <c r="L48" t="n">
         <v>20000</v>
@@ -6011,20 +6029,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/23/2026 23:12</t>
+          <t>06/24/2026 11:43</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>19883.53</v>
+        <v>19766.56</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>-0.58</v>
+        <v>-1.16</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>1.19</v>
+        <v>1.77</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="L49" t="n">
         <v>20000</v>
@@ -6033,13 +6051,22 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>0</v>
+        <v>19760.43</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="Q49" s="7" t="n">
+        <v>41.66666666666667</v>
+      </c>
+      <c r="R49" s="7" t="n">
+        <v>24.29882211453433</v>
+      </c>
+      <c r="S49" s="7" t="n">
+        <v>0.91</v>
       </c>
       <c r="T49" t="n">
         <v>10</v>
@@ -6071,7 +6098,7 @@
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC49" t="inlineStr">
@@ -6111,20 +6138,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>06/23/2026 16:27</t>
+          <t>06/24/2026 11:46</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>19653.52</v>
+        <v>19626.44</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>-1.73</v>
+        <v>-1.86</v>
       </c>
       <c r="J50" s="7" t="n">
-        <v>1.81</v>
+        <v>1.93</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>0.48</v>
+        <v>0.49</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6133,13 +6160,22 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>0</v>
+        <v>-41.92</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q50" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R50" s="7" t="n">
+        <v>0.5798336173198356</v>
+      </c>
+      <c r="S50" s="7" t="n">
+        <v>0.28</v>
       </c>
       <c r="T50" t="n">
         <v>212</v>
@@ -6211,14 +6247,14 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/23/2026 17:28</t>
+          <t>06/24/2026 06:41</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>1163.93</v>
+        <v>1156.94</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-98.41</v>
+        <v>-98.42</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>99.73999999999999</v>
@@ -6236,37 +6272,37 @@
         <v>40</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>-625.34</v>
+        <v>-861.78</v>
       </c>
       <c r="P51" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q51" s="7" t="n">
-        <v>37.5</v>
+        <v>32.5</v>
       </c>
       <c r="R51" s="7" t="n">
-        <v>0.5213953879947038</v>
+        <v>0.3460365159586578</v>
       </c>
       <c r="S51" s="7" t="n">
-        <v>4.68</v>
+        <v>4.73</v>
       </c>
       <c r="T51" t="n">
-        <v>587</v>
+        <v>595</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-19838.17</v>
+        <v>-19349.44000000001</v>
       </c>
       <c r="V51" t="n">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>41.90800681431005</v>
+        <v>42.01680672268908</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="Y51" s="7" t="n">
-        <v>97.65000000000001</v>
+        <v>98.48999999999999</v>
       </c>
       <c r="Z51" t="inlineStr">
         <is>
@@ -6275,7 +6311,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6320,62 +6356,62 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/23/2026 20:48</t>
+          <t>06/24/2026 17:37</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>26139.16</v>
+        <v>22197.69</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>0.74</v>
+        <v>0.97</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>6.56</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>1.08</v>
+        <v>1.11</v>
       </c>
       <c r="L52" t="n">
         <v>26000</v>
       </c>
       <c r="M52" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="N52" t="n">
         <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>16040.85</v>
+        <v>12552.25</v>
       </c>
       <c r="P52" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="Q52" s="7" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="R52" s="7" t="n">
-        <v>14.31047272908317</v>
+        <v>3.590977583288609</v>
       </c>
       <c r="S52" s="7" t="n">
-        <v>1.94</v>
+        <v>10.48</v>
       </c>
       <c r="T52" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>139.1600000000001</v>
+        <v>149.72</v>
       </c>
       <c r="V52" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>44.23076923076923</v>
+        <v>43.85964912280701</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>1.08</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>2.56</v>
+        <v>3.02</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6384,7 +6420,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6429,7 +6465,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/15/2026 05:49</t>
+          <t>06/24/2026 16:24</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
@@ -6538,17 +6574,17 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/23/2026 13:14</t>
+          <t>06/24/2026 18:00</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
-        <v>27951.09</v>
+        <v>27808.74</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>-22.57</v>
+        <v>-22.97</v>
       </c>
       <c r="J54" s="7" t="n">
-        <v>29.62</v>
+        <v>29.98</v>
       </c>
       <c r="K54" s="7" t="n">
         <v>0.78</v>
@@ -6563,37 +6599,37 @@
         <v>40</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>-1307.37</v>
+        <v>-1211.56</v>
       </c>
       <c r="P54" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q54" s="7" t="n">
-        <v>10</v>
+        <v>12.5</v>
       </c>
       <c r="R54" s="7" t="n">
-        <v>0.04878421443226961</v>
+        <v>0.06660914315649989</v>
       </c>
       <c r="S54" s="7" t="n">
-        <v>5.31</v>
+        <v>4.85</v>
       </c>
       <c r="T54" t="n">
-        <v>3031</v>
+        <v>3063</v>
       </c>
       <c r="U54" s="7" t="n">
-        <v>-6329.609999999999</v>
+        <v>-6473.259999999999</v>
       </c>
       <c r="V54" t="n">
-        <v>1793</v>
+        <v>1794</v>
       </c>
       <c r="W54" s="7" t="n">
-        <v>59.15539425932036</v>
+        <v>58.57002938295789</v>
       </c>
       <c r="X54" s="7" t="n">
         <v>0.78</v>
       </c>
       <c r="Y54" s="7" t="n">
-        <v>32.19</v>
+        <v>32.64</v>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
@@ -6602,7 +6638,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -7011,7 +7047,7 @@
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>06/21/2026 21:39</t>
+          <t>06/24/2026 21:47</t>
         </is>
       </c>
       <c r="H59" s="9" t="n">
@@ -7102,7 +7138,7 @@
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>06/21/2026 16:12</t>
+          <t>06/24/2026 16:21</t>
         </is>
       </c>
       <c r="H60" s="9" t="n">
@@ -7284,7 +7320,7 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>06/23/2026 16:33</t>
+          <t>06/24/2026 05:49</t>
         </is>
       </c>
       <c r="H62" s="9" t="n">
@@ -7373,7 +7409,7 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>06/23/2026 07:50</t>
+          <t>06/24/2026 11:49</t>
         </is>
       </c>
       <c r="H63" s="9" t="n">
@@ -7555,7 +7591,7 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>06/23/2026 17:14</t>
+          <t>06/24/2026 12:36</t>
         </is>
       </c>
       <c r="H65" s="9" t="n">
@@ -7646,7 +7682,7 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>06/23/2026 16:10</t>
+          <t>06/24/2026 05:31</t>
         </is>
       </c>
       <c r="H66" s="9" t="n">
@@ -7737,7 +7773,7 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>06/23/2026 23:08</t>
+          <t>06/24/2026 05:38</t>
         </is>
       </c>
       <c r="H67" s="8" t="n">
@@ -7822,7 +7858,7 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>06/23/2026 23:07</t>
+          <t>06/24/2026 11:41</t>
         </is>
       </c>
       <c r="H68" s="9" t="n">
@@ -7907,7 +7943,7 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>06/23/2026 23:10</t>
+          <t>06/24/2026 05:40</t>
         </is>
       </c>
       <c r="H69" s="9" t="n">
@@ -7992,7 +8028,7 @@
       </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
-          <t>06/21/2026 03:16</t>
+          <t>06/24/2026 03:21</t>
         </is>
       </c>
       <c r="H70" s="9" t="n">
@@ -8083,7 +8119,7 @@
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>06/21/2026 00:42</t>
+          <t>06/24/2026 00:44</t>
         </is>
       </c>
       <c r="H71" s="9" t="n">
@@ -8265,7 +8301,7 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>06/21/2026 20:24</t>
+          <t>06/24/2026 20:29</t>
         </is>
       </c>
       <c r="H73" s="9" t="n">
@@ -8604,7 +8640,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>06/21/2026 21:39</t>
+          <t>06/24/2026 21:47</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -8645,7 +8681,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>06/21/2026 16:12</t>
+          <t>06/24/2026 16:21</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -8727,7 +8763,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>06/23/2026 16:33</t>
+          <t>06/24/2026 05:49</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -8768,7 +8804,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>06/23/2026 07:50</t>
+          <t>06/24/2026 11:49</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -8850,7 +8886,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/23/2026 17:14</t>
+          <t>06/24/2026 12:36</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -8891,7 +8927,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/23/2026 16:10</t>
+          <t>06/24/2026 05:31</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -8932,7 +8968,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>06/23/2026 23:08</t>
+          <t>06/24/2026 05:38</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -8973,7 +9009,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>06/23/2026 23:07</t>
+          <t>06/24/2026 11:41</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -9014,7 +9050,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>06/23/2026 23:10</t>
+          <t>06/24/2026 05:40</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -9055,7 +9091,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>06/21/2026 03:16</t>
+          <t>06/24/2026 03:21</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -9096,7 +9132,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>06/21/2026 00:42</t>
+          <t>06/24/2026 00:44</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -9178,7 +9214,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>06/21/2026 20:24</t>
+          <t>06/24/2026 20:29</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -9894,7 +9930,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>06/18/2026 08:44</t>
+          <t>06/24/2026 08:50</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -9940,7 +9976,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>06/21/2026 09:02</t>
+          <t>06/24/2026 09:04</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -10170,7 +10206,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>06/21/2026 08:52</t>
+          <t>06/24/2026 09:03</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
@@ -10308,11 +10344,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06/23/2026 19:53</t>
+          <t>06/24/2026 08:49</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>20006.93</v>
+        <v>20006.49</v>
       </c>
     </row>
     <row r="23">
@@ -10331,7 +10367,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06/23/2026 20:18</t>
+          <t>06/24/2026 16:52</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -10354,11 +10390,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06/23/2026 16:30</t>
+          <t>06/24/2026 11:51</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
-        <v>19914.43</v>
+        <v>19975.99</v>
       </c>
     </row>
     <row r="25">
@@ -10377,11 +10413,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06/23/2026 16:31</t>
+          <t>06/24/2026 11:50</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19914.43</v>
+        <v>19909.34</v>
       </c>
     </row>
     <row r="26">
@@ -10400,11 +10436,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06/23/2026 16:31</t>
+          <t>06/24/2026 11:49</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20423.61</v>
+        <v>20424.14</v>
       </c>
     </row>
     <row r="27">
@@ -10423,11 +10459,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06/23/2026 16:34</t>
+          <t>06/24/2026 05:50</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>20033.89</v>
+        <v>20013.52</v>
       </c>
     </row>
     <row r="28">
@@ -10446,11 +10482,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06/23/2026 16:37</t>
+          <t>06/24/2026 05:51</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
-        <v>19842.22</v>
+        <v>19854.3</v>
       </c>
     </row>
     <row r="29">
@@ -10515,11 +10551,11 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06/23/2026 16:49</t>
+          <t>06/24/2026 06:04</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>19943.69</v>
+        <v>19952.76</v>
       </c>
     </row>
     <row r="32">
@@ -10538,11 +10574,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06/23/2026 16:45</t>
+          <t>06/24/2026 12:09</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>20227.79</v>
+        <v>20696.21</v>
       </c>
     </row>
     <row r="33">
@@ -10561,11 +10597,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06/23/2026 16:49</t>
+          <t>06/24/2026 12:10</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>19976.83</v>
+        <v>20371.59</v>
       </c>
     </row>
     <row r="34">
@@ -10584,11 +10620,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06/23/2026 16:52</t>
+          <t>06/24/2026 12:12</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>19930.82</v>
+        <v>20120.83</v>
       </c>
     </row>
     <row r="35">
@@ -10607,11 +10643,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06/23/2026 16:51</t>
+          <t>06/24/2026 12:11</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>19946.64</v>
+        <v>19929.41</v>
       </c>
     </row>
     <row r="36">

</xml_diff>

<commit_message>
Update dashboards — 2026-06-25
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-24 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-06-25 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -1000,16 +1000,16 @@
         <v>14.03</v>
       </c>
       <c r="T2" t="n">
-        <v>2933</v>
+        <v>2938</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>21040.74999999999</v>
+        <v>21262.71999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>1850</v>
+        <v>1852</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.07534947153085</v>
+        <v>63.03607896528251</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.06</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/24/2026 13:51</t>
+          <t>06/25/2026 11:13</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/24/2026 16:59</t>
+          <t>06/25/2026 05:25</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/24/2026 05:56</t>
+          <t>06/25/2026 09:24</t>
         </is>
       </c>
       <c r="H6" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/24/2026 07:18</t>
+          <t>06/25/2026 11:10</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/24/2026 19:48</t>
+          <t>06/25/2026 07:20</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>06/24/2026 11:46</t>
+          <t>06/25/2026 09:06</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>06/24/2026 13:07</t>
+          <t>06/25/2026 01:50</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -2377,14 +2377,14 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/24/2026 17:31</t>
+          <t>06/25/2026 14:31</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>1601.98</v>
+        <v>1371.14</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-92.17</v>
+        <v>-93.3</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>98.18000000000001</v>
@@ -2402,34 +2402,34 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>419.01</v>
+        <v>-350.33</v>
       </c>
       <c r="P15" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>35</v>
+        <v>27.5</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>2.439303380049464</v>
+        <v>0.5927484509956639</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>0.61</v>
+        <v>2.66</v>
       </c>
       <c r="T15" t="n">
-        <v>1786</v>
+        <v>1803</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-18894.08</v>
+        <v>-18929.76</v>
       </c>
       <c r="V15" t="n">
-        <v>582</v>
+        <v>590</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>32.58678611422172</v>
+        <v>32.72323904603439</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="Y15" s="7" t="n">
         <v>98.17</v>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2486,20 +2486,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>06/24/2026 16:23</t>
+          <t>06/25/2026 13:27</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>17676.49</v>
+        <v>17836.71</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-11.64</v>
+        <v>-10.84</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>17.06</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.82</v>
+        <v>0.84</v>
       </c>
       <c r="L16" t="n">
         <v>20000</v>
@@ -2511,34 +2511,34 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-118.5999999999999</v>
+        <v>125.98</v>
       </c>
       <c r="P16" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.9574222129679159</v>
+        <v>1.046328099143162</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>6.33</v>
+        <v>6.31</v>
       </c>
       <c r="T16" t="n">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-2323.51</v>
+        <v>-1994.52</v>
       </c>
       <c r="V16" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>43.53741496598639</v>
+        <v>44</v>
       </c>
       <c r="X16" s="7" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="Y16" s="7" t="n">
         <v>17.04</v>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>06/24/2026 14:43</t>
+          <t>06/25/2026 12:13</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>06/24/2026 11:53</t>
+          <t>06/25/2026 09:15</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>06/24/2026 05:39</t>
+          <t>06/25/2026 08:58</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2962,16 +2962,16 @@
         <v>11.7</v>
       </c>
       <c r="T20" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>-4900</v>
+        <v>-4791.85</v>
       </c>
       <c r="V20" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>42.60355029585799</v>
+        <v>42.94117647058823</v>
       </c>
       <c r="X20" s="7" t="n">
         <v>0.68</v>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -3031,17 +3031,17 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>06/24/2026 12:12</t>
+          <t>06/25/2026 09:51</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>17076.51</v>
+        <v>17005.37</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>-14.62</v>
+        <v>-14.98</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>14.77</v>
+        <v>15.13</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>0.04</v>
@@ -3053,40 +3053,40 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>17189.81</v>
+        <v>17118.67</v>
       </c>
       <c r="P21" t="n">
         <v>3</v>
       </c>
       <c r="Q21" s="7" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>6.843495257844102</v>
+        <v>6.681904780871204</v>
       </c>
       <c r="S21" s="7" t="n">
-        <v>7.11</v>
+        <v>7.29</v>
       </c>
       <c r="T21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U21" s="7" t="n">
-        <v>-2923.49</v>
+        <v>-2994.63</v>
       </c>
       <c r="V21" t="n">
         <v>2</v>
       </c>
       <c r="W21" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>0.04</v>
       </c>
       <c r="Y21" s="7" t="n">
-        <v>14.77</v>
+        <v>15.13</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>06/24/2026 05:22</t>
+          <t>06/25/2026 08:38</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3358,20 +3358,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/24/2026 11:41</t>
+          <t>06/25/2026 09:00</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>15859.7</v>
+        <v>16038.74</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>-20.45</v>
+        <v>-19.55</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>20.45</v>
+        <v>20.54</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="L24" t="n">
         <v>20000</v>
@@ -3383,34 +3383,34 @@
         <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>-320.12</v>
+        <v>-131.86</v>
       </c>
       <c r="P24" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q24" s="7" t="n">
-        <v>45</v>
+        <v>42.5</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>0.4429692529885677</v>
+        <v>0.7734675645959318</v>
       </c>
       <c r="S24" s="7" t="n">
         <v>1.68</v>
       </c>
       <c r="T24" t="n">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>-4147.32</v>
+        <v>-3955.8</v>
       </c>
       <c r="V24" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>35.65683646112601</v>
+        <v>35.78947368421053</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="Y24" s="7" t="n">
         <v>20.79</v>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -3467,20 +3467,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>06/23/2026 23:13</t>
+          <t>06/25/2026 09:06</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>21135.89</v>
+        <v>20424.23</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>1.07</v>
+        <v>-2.33</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>2.59</v>
+        <v>4.48</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>1.09</v>
+        <v>0.83</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3492,25 +3492,25 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>-63.58999999999999</v>
+        <v>-684.76</v>
       </c>
       <c r="P25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>37.5</v>
+        <v>32.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>0.9630705080926634</v>
+        <v>0.6910875724055796</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>2.73</v>
+        <v>4.73</v>
       </c>
       <c r="T25" t="n">
         <v>64</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>488.3500000000001</v>
+        <v>424.2300000000001</v>
       </c>
       <c r="V25" t="n">
         <v>26</v>
@@ -3519,10 +3519,10 @@
         <v>40.625</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>1.17</v>
+        <v>1.14</v>
       </c>
       <c r="Y25" s="7" t="n">
-        <v>4.18</v>
+        <v>4.48</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/24/2026 11:58</t>
+          <t>06/25/2026 09:22</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/24/2026 11:47</t>
+          <t>06/25/2026 00:08</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/24/2026 11:43</t>
+          <t>06/25/2026 09:00</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,20 +4012,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/24/2026 12:22</t>
+          <t>06/25/2026 00:58</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
-        <v>19663.56</v>
+        <v>19713.41</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>-1.68</v>
+        <v>-1.43</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>1.86</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>0.64</v>
+        <v>0.7</v>
       </c>
       <c r="L30" t="n">
         <v>20000</v>
@@ -4037,34 +4037,34 @@
         <v>40</v>
       </c>
       <c r="O30" s="7" t="n">
-        <v>2.969999999999999</v>
+        <v>45.14</v>
       </c>
       <c r="P30" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="Q30" s="7" t="n">
-        <v>62.5</v>
+        <v>72.5</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>1.085027197251646</v>
+        <v>2.6887392442948</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="T30" t="n">
-        <v>826</v>
+        <v>839</v>
       </c>
       <c r="U30" s="7" t="n">
-        <v>-365.03</v>
+        <v>-314.89</v>
       </c>
       <c r="V30" t="n">
-        <v>358</v>
+        <v>389</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>43.34140435835351</v>
+        <v>46.36471990464839</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>0.62</v>
+        <v>0.68</v>
       </c>
       <c r="Y30" s="7" t="n">
         <v>1.87</v>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4121,20 +4121,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/24/2026 08:43</t>
+          <t>06/25/2026 13:12</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20207.02</v>
+        <v>20243.49</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>1.03</v>
+        <v>1.21</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>2.17</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>1.26</v>
+        <v>1.29</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -4143,22 +4143,22 @@
         <v>0</v>
       </c>
       <c r="N31" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>20196.97</v>
+        <v>233.44</v>
       </c>
       <c r="P31" t="n">
         <v>19</v>
       </c>
       <c r="Q31" s="7" t="n">
-        <v>48.71794871794872</v>
+        <v>47.5</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>25.90071507828874</v>
+        <v>1.270567236143629</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>1.13</v>
+        <v>2.22</v>
       </c>
       <c r="T31" t="n">
         <v>40</v>
@@ -4230,20 +4230,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/24/2026 07:18</t>
+          <t>06/25/2026 11:09</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>16545.65</v>
+        <v>15532.51</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>-17.29</v>
+        <v>-22.36</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>29.45</v>
+        <v>34.36</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4255,37 +4255,37 @@
         <v>40</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>-235.98</v>
+        <v>-341.24</v>
       </c>
       <c r="P32" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>47.5</v>
+        <v>45</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>0.8716090490647341</v>
+        <v>0.8058798097708603</v>
       </c>
       <c r="S32" s="7" t="n">
-        <v>4.03</v>
+        <v>2.79</v>
       </c>
       <c r="T32" t="n">
-        <v>1170</v>
+        <v>1196</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>-4518.6</v>
+        <v>-4467.49</v>
       </c>
       <c r="V32" t="n">
-        <v>564</v>
+        <v>578</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>48.2051282051282</v>
+        <v>48.32775919732442</v>
       </c>
       <c r="X32" s="7" t="n">
         <v>0.93</v>
       </c>
       <c r="Y32" s="7" t="n">
-        <v>33.94</v>
+        <v>34.34</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
@@ -4379,19 +4379,19 @@
         <v>0.74</v>
       </c>
       <c r="T33" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>831.39</v>
+        <v>1044.07</v>
       </c>
       <c r="V33" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="W33" s="7" t="n">
-        <v>64.28571428571429</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X33" s="7" t="n">
-        <v>1.82</v>
+        <v>2.03</v>
       </c>
       <c r="Y33" s="7" t="n">
         <v>1.47</v>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>06/24/2026 00:16</t>
+          <t>06/25/2026 10:44</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>06/24/2026 15:10</t>
+          <t>06/25/2026 12:19</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/24/2026 01:47</t>
+          <t>06/25/2026 12:28</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19724.08</v>
+        <v>19586.91</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-1.38</v>
+        <v>-2.06</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>3.35</v>
+        <v>4.02</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.67</v>
+        <v>0.57</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4688,22 +4688,22 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>19715.19</v>
+        <v>19577.66</v>
       </c>
       <c r="P36" t="n">
         <v>4</v>
       </c>
       <c r="Q36" s="7" t="n">
-        <v>36.36363636363637</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>24.72008999470619</v>
+        <v>21.21044916330301</v>
       </c>
       <c r="S36" s="7" t="n">
-        <v>1.71</v>
+        <v>2.05</v>
       </c>
       <c r="T36" t="n">
         <v>13</v>
@@ -4775,7 +4775,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/24/2026 17:39</t>
+          <t>06/25/2026 06:00</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4815,22 +4815,22 @@
         <v>3.12</v>
       </c>
       <c r="T37" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-947.73</v>
+        <v>-881.25</v>
       </c>
       <c r="V37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>15.625</v>
+        <v>17.64705882352941</v>
       </c>
       <c r="X37" s="7" t="n">
-        <v>0.41</v>
+        <v>0.47</v>
       </c>
       <c r="Y37" s="7" t="n">
-        <v>4.74</v>
+        <v>5.09</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -4839,12 +4839,12 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/24/2026 19:44</t>
+          <t>06/25/2026 07:15</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4924,19 +4924,19 @@
         <v>2.42</v>
       </c>
       <c r="T38" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="U38" s="7" t="n">
-        <v>-213.86</v>
+        <v>-284.46</v>
       </c>
       <c r="V38" t="n">
         <v>20</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>27.77777777777778</v>
+        <v>27.02702702702703</v>
       </c>
       <c r="X38" s="7" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="Y38" s="7" t="n">
         <v>3.82</v>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
@@ -4993,20 +4993,20 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>06/24/2026 11:34</t>
+          <t>06/24/2026 23:51</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
-        <v>19468.83</v>
+        <v>19451.89</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>-2.66</v>
+        <v>-2.74</v>
       </c>
       <c r="J39" s="7" t="n">
         <v>3.09</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="L39" t="n">
         <v>20000</v>
@@ -5018,19 +5018,19 @@
         <v>40</v>
       </c>
       <c r="O39" s="7" t="n">
-        <v>-4.13</v>
+        <v>-84.27</v>
       </c>
       <c r="P39" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="Q39" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="R39" s="7" t="n">
-        <v>0.9481351249529073</v>
+        <v>0.3032082024144204</v>
       </c>
       <c r="S39" s="7" t="n">
-        <v>0.13</v>
+        <v>0.52</v>
       </c>
       <c r="T39" t="n">
         <v>598</v>
@@ -5102,20 +5102,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/24/2026 11:36</t>
+          <t>06/25/2026 09:01</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
-        <v>18720.85</v>
+        <v>18459.33</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>-6.4</v>
+        <v>-7.7</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>7.5</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>0.63</v>
+        <v>0.61</v>
       </c>
       <c r="L40" t="n">
         <v>20000</v>
@@ -5124,13 +5124,22 @@
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O40" s="7" t="n">
-        <v>0</v>
+        <v>-50.3</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q40" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R40" s="7" t="n">
+        <v>0.2733314071077723</v>
+      </c>
+      <c r="S40" s="7" t="n">
+        <v>0.27</v>
       </c>
       <c r="T40" t="n">
         <v>1179</v>
@@ -5202,11 +5211,11 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>06/24/2026 11:33</t>
+          <t>06/25/2026 08:51</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
-        <v>20396.08</v>
+        <v>20392.6</v>
       </c>
       <c r="I41" s="7" t="n">
         <v>1.98</v>
@@ -5224,13 +5233,22 @@
         <v>0</v>
       </c>
       <c r="N41" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="O41" s="7" t="n">
-        <v>0</v>
+        <v>20349.08</v>
       </c>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="Q41" s="7" t="n">
+        <v>57.14285714285714</v>
+      </c>
+      <c r="R41" s="7" t="n">
+        <v>94.68821362799264</v>
+      </c>
+      <c r="S41" s="7" t="n">
+        <v>0.28</v>
       </c>
       <c r="T41" t="n">
         <v>12</v>
@@ -5262,7 +5280,7 @@
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC41" t="inlineStr">
@@ -5302,7 +5320,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>06/24/2026 11:36</t>
+          <t>06/24/2026 23:52</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5502,20 +5520,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/24/2026 11:49</t>
+          <t>06/25/2026 09:08</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>18802.63</v>
+        <v>18836.33</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-5.99</v>
+        <v>-5.82</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>6.06</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5602,7 +5620,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/24/2026 11:39</t>
+          <t>06/24/2026 23:56</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5702,20 +5720,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/24/2026 11:41</t>
+          <t>06/25/2026 08:58</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19932.03</v>
+        <v>20021.9</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-0.34</v>
+        <v>0.11</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>2.23</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.93</v>
+        <v>1.02</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5802,20 +5820,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/24/2026 05:40</t>
+          <t>06/25/2026 09:01</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>21155.27</v>
+        <v>22234.67</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>5.78</v>
+        <v>11.18</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>3.34</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>1.45</v>
+        <v>1.84</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5902,20 +5920,20 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/24/2026 11:46</t>
+          <t>06/25/2026 09:02</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
-        <v>22327.87</v>
+        <v>24723.02</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>11.7</v>
+        <v>23.62</v>
       </c>
       <c r="J48" s="7" t="n">
         <v>5.53</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>1.46</v>
+        <v>1.91</v>
       </c>
       <c r="L48" t="n">
         <v>20000</v>
@@ -6002,20 +6020,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/24/2026 11:43</t>
+          <t>06/25/2026 09:00</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>19766.56</v>
+        <v>19861.41</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>-1.16</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="J49" s="7" t="n">
         <v>1.77</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>0.72</v>
+        <v>0.87</v>
       </c>
       <c r="L49" t="n">
         <v>20000</v>
@@ -6102,20 +6120,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>06/24/2026 11:46</t>
+          <t>06/25/2026 09:08</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>19626.44</v>
+        <v>19618.6</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>-1.86</v>
+        <v>-1.9</v>
       </c>
       <c r="J50" s="7" t="n">
         <v>1.93</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6202,44 +6220,44 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/24/2026 06:41</t>
+          <t>06/25/2026 10:21</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>1156.94</v>
+        <v>1650.56</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-98.42</v>
+        <v>-98.68000000000001</v>
       </c>
       <c r="J51" s="7" t="n">
-        <v>99.73999999999999</v>
+        <v>99.79000000000001</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="L51" t="n">
-        <v>31000</v>
+        <v>35000</v>
       </c>
       <c r="M51" t="n">
-        <v>10000</v>
+        <v>14000</v>
       </c>
       <c r="N51" t="n">
         <v>40</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>-861.78</v>
+        <v>-269.46</v>
       </c>
       <c r="P51" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="Q51" s="7" t="n">
-        <v>32.5</v>
+        <v>42.5</v>
       </c>
       <c r="R51" s="7" t="n">
-        <v>0.3460365159586578</v>
+        <v>0.9550466949828335</v>
       </c>
       <c r="S51" s="7" t="n">
-        <v>4.73</v>
+        <v>16.17</v>
       </c>
       <c r="T51" t="n">
         <v>595</v>
@@ -6311,23 +6329,23 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/24/2026 17:37</t>
+          <t>06/25/2026 06:05</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>22197.69</v>
+        <v>26149.72</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>0.97</v>
+        <v>0.75</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>6.56</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>1.11</v>
+        <v>1.08</v>
       </c>
       <c r="L52" t="n">
-        <v>26000</v>
+        <v>30000</v>
       </c>
       <c r="M52" t="n">
         <v>4000</v>
@@ -6336,7 +6354,7 @@
         <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>12552.25</v>
+        <v>16534.45</v>
       </c>
       <c r="P52" t="n">
         <v>18</v>
@@ -6345,10 +6363,10 @@
         <v>45</v>
       </c>
       <c r="R52" s="7" t="n">
-        <v>3.590977583288609</v>
+        <v>4.403704984581434</v>
       </c>
       <c r="S52" s="7" t="n">
-        <v>10.48</v>
+        <v>9.6</v>
       </c>
       <c r="T52" t="n">
         <v>57</v>
@@ -6366,7 +6384,7 @@
         <v>1.08</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>3.02</v>
+        <v>2.56</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6569,16 +6587,16 @@
         <v>4.85</v>
       </c>
       <c r="T54" t="n">
-        <v>3064</v>
+        <v>3080</v>
       </c>
       <c r="U54" s="7" t="n">
-        <v>-6473.259999999999</v>
+        <v>-6431.110000000001</v>
       </c>
       <c r="V54" t="n">
-        <v>1794</v>
+        <v>1796</v>
       </c>
       <c r="W54" s="7" t="n">
-        <v>58.5509138381201</v>
+        <v>58.31168831168831</v>
       </c>
       <c r="X54" s="7" t="n">
         <v>0.78</v>
@@ -6593,7 +6611,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -6911,7 +6929,7 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>06/22/2026 01:48</t>
+          <t>06/25/2026 01:52</t>
         </is>
       </c>
       <c r="H58" s="9" t="n">
@@ -7275,7 +7293,7 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>06/24/2026 05:49</t>
+          <t>06/25/2026 00:11</t>
         </is>
       </c>
       <c r="H62" s="9" t="n">
@@ -7364,7 +7382,7 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>06/24/2026 11:49</t>
+          <t>06/25/2026 09:14</t>
         </is>
       </c>
       <c r="H63" s="9" t="n">
@@ -7455,7 +7473,7 @@
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>06/23/2026 16:21</t>
+          <t>06/25/2026 09:01</t>
         </is>
       </c>
       <c r="H64" s="9" t="n">
@@ -7546,7 +7564,7 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>06/24/2026 12:36</t>
+          <t>06/25/2026 10:05</t>
         </is>
       </c>
       <c r="H65" s="9" t="n">
@@ -7637,7 +7655,7 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>06/24/2026 05:31</t>
+          <t>06/24/2026 23:55</t>
         </is>
       </c>
       <c r="H66" s="9" t="n">
@@ -7728,7 +7746,7 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>06/24/2026 05:38</t>
+          <t>06/25/2026 08:59</t>
         </is>
       </c>
       <c r="H67" s="8" t="n">
@@ -7813,7 +7831,7 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>06/24/2026 11:41</t>
+          <t>06/25/2026 09:00</t>
         </is>
       </c>
       <c r="H68" s="9" t="n">
@@ -7898,7 +7916,7 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>06/24/2026 05:40</t>
+          <t>06/25/2026 08:58</t>
         </is>
       </c>
       <c r="H69" s="9" t="n">
@@ -8554,7 +8572,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>06/22/2026 01:48</t>
+          <t>06/25/2026 01:52</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -8718,7 +8736,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>06/24/2026 05:49</t>
+          <t>06/25/2026 00:11</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -8759,7 +8777,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>06/24/2026 11:49</t>
+          <t>06/25/2026 09:14</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -8800,7 +8818,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>06/23/2026 16:21</t>
+          <t>06/25/2026 09:01</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -8841,7 +8859,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/24/2026 12:36</t>
+          <t>06/25/2026 10:05</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -8882,7 +8900,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/24/2026 05:31</t>
+          <t>06/24/2026 23:55</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -8923,7 +8941,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>06/24/2026 05:38</t>
+          <t>06/25/2026 08:59</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -8964,7 +8982,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>06/24/2026 11:41</t>
+          <t>06/25/2026 09:00</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -9005,7 +9023,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>06/24/2026 05:40</t>
+          <t>06/25/2026 08:58</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -9908,7 +9926,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>06/19/2026 02:32</t>
+          <t>06/25/2026 02:51</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -10092,7 +10110,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06/22/2026 10:50</t>
+          <t>06/25/2026 10:53</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -10299,11 +10317,11 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06/24/2026 08:49</t>
+          <t>06/25/2026 13:18</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>20006.49</v>
+        <v>19987.79</v>
       </c>
     </row>
     <row r="23">
@@ -10322,7 +10340,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06/24/2026 16:52</t>
+          <t>06/25/2026 13:47</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -10345,11 +10363,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06/24/2026 11:51</t>
+          <t>06/25/2026 09:19</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
-        <v>19975.99</v>
+        <v>19974.83</v>
       </c>
     </row>
     <row r="25">
@@ -10368,11 +10386,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06/24/2026 11:50</t>
+          <t>06/25/2026 09:11</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19909.34</v>
+        <v>19896.17</v>
       </c>
     </row>
     <row r="26">
@@ -10391,11 +10409,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06/24/2026 11:49</t>
+          <t>06/25/2026 09:06</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20424.14</v>
+        <v>20347.81</v>
       </c>
     </row>
     <row r="27">
@@ -10414,11 +10432,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06/24/2026 05:50</t>
+          <t>06/25/2026 09:13</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>20013.52</v>
+        <v>20030.37</v>
       </c>
     </row>
     <row r="28">
@@ -10437,11 +10455,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06/24/2026 05:51</t>
+          <t>06/25/2026 09:15</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
-        <v>19854.3</v>
+        <v>19885.14</v>
       </c>
     </row>
     <row r="29">
@@ -10483,11 +10501,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06/23/2026 16:46</t>
+          <t>06/25/2026 09:39</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>19527.93</v>
+        <v>19327.3</v>
       </c>
     </row>
     <row r="31">
@@ -10506,11 +10524,11 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06/24/2026 06:04</t>
+          <t>06/25/2026 09:29</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>19952.76</v>
+        <v>19894.65</v>
       </c>
     </row>
     <row r="32">
@@ -10529,11 +10547,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06/24/2026 12:09</t>
+          <t>06/25/2026 09:34</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>20696.21</v>
+        <v>21351.31</v>
       </c>
     </row>
     <row r="33">
@@ -10552,11 +10570,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06/24/2026 12:10</t>
+          <t>06/25/2026 09:41</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>20371.59</v>
+        <v>20847.71</v>
       </c>
     </row>
     <row r="34">
@@ -10575,11 +10593,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06/24/2026 12:12</t>
+          <t>06/25/2026 09:42</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>20120.83</v>
+        <v>20399.14</v>
       </c>
     </row>
     <row r="35">
@@ -10598,11 +10616,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06/24/2026 12:11</t>
+          <t>06/25/2026 09:44</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>19929.41</v>
+        <v>20100.95</v>
       </c>
     </row>
     <row r="36">
@@ -10713,7 +10731,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>06/23/2026 03:46</t>
+          <t>06/25/2026 03:48</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-07-01
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-06-30 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-07-01 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/30/2026 04:39</t>
+          <t>07/01/2026 11:28</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>44884.25</v>
+        <v>45514.79</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>109.33</v>
+        <v>112.27</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-1326.51</v>
+        <v>84.51999999999998</v>
       </c>
       <c r="P2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>52.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.2255810287755924</v>
+        <v>1.090857296425692</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>6.27</v>
+        <v>3.34</v>
       </c>
       <c r="T2" t="n">
-        <v>2999</v>
+        <v>3012</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>20249.3</v>
+        <v>19760.69</v>
       </c>
       <c r="V2" t="n">
-        <v>1885</v>
+        <v>1892</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>62.85428476158719</v>
+        <v>62.81540504648074</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.06</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/30/2026 13:48</t>
+          <t>07/01/2026 17:08</t>
         </is>
       </c>
       <c r="H3" s="7" t="n">
@@ -1178,20 +1178,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/30/2026 15:44</t>
+          <t>07/01/2026 20:55</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
-        <v>21754.38</v>
+        <v>21521.18</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>8.73</v>
+        <v>7.56</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>5.78</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>1.18</v>
+        <v>1.15</v>
       </c>
       <c r="L4" t="n">
         <v>20000</v>
@@ -1203,25 +1203,25 @@
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>546.2600000000001</v>
+        <v>187.8100000000001</v>
       </c>
       <c r="P4" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Q4" s="7" t="n">
-        <v>70</v>
+        <v>67.5</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>1.15521836728895</v>
+        <v>1.049854664666923</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>6.56</v>
+        <v>6.6</v>
       </c>
       <c r="T4" t="n">
         <v>119</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>1754.38</v>
+        <v>1521.18</v>
       </c>
       <c r="V4" t="n">
         <v>78</v>
@@ -1230,7 +1230,7 @@
         <v>65.54621848739495</v>
       </c>
       <c r="X4" s="7" t="n">
-        <v>1.18</v>
+        <v>1.15</v>
       </c>
       <c r="Y4" s="7" t="n">
         <v>5.78</v>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/30/2026 13:39</t>
+          <t>07/01/2026 16:42</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>06/30/2026 13:08</t>
+          <t>07/01/2026 15:35</t>
         </is>
       </c>
       <c r="H14" s="7" t="n">
@@ -2377,14 +2377,14 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>06/30/2026 16:04</t>
+          <t>07/01/2026 21:26</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>873.1900000000001</v>
+        <v>549.79</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-95.73999999999999</v>
+        <v>-97.31999999999999</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>98.18000000000001</v>
@@ -2402,31 +2402,31 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>-141</v>
+        <v>-159.55</v>
       </c>
       <c r="P15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>40</v>
+        <v>42.5</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>0.7861757301871342</v>
+        <v>0.7922174326383373</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>2.16</v>
+        <v>2.22</v>
       </c>
       <c r="T15" t="n">
-        <v>1889</v>
+        <v>1900</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-19549.21</v>
+        <v>-19874.25</v>
       </c>
       <c r="V15" t="n">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>32.8215987294865</v>
+        <v>32.73684210526316</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>0.7</v>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>06/30/2026 09:08</t>
+          <t>07/01/2026 19:53</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>06/30/2026 14:28</t>
+          <t>07/01/2026 18:14</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>06/30/2026 12:08</t>
+          <t>07/01/2026 13:27</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>06/30/2026 05:51</t>
+          <t>07/01/2026 13:17</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>06/30/2026 09:47</t>
+          <t>07/01/2026 21:33</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,20 +3031,20 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>06/30/2026 12:36</t>
+          <t>07/01/2026 14:15</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>17287.87</v>
+        <v>18302.99</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>-13.58</v>
+        <v>-8.51</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>15.82</v>
+        <v>18.8</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.46</v>
+        <v>0.75</v>
       </c>
       <c r="L21" t="n">
         <v>20000</v>
@@ -3053,22 +3053,22 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>17401.17</v>
+        <v>18416.29</v>
       </c>
       <c r="P21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q21" s="7" t="n">
-        <v>31.25</v>
+        <v>31.57894736842105</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>4.547595748064244</v>
+        <v>3.725883944535885</v>
       </c>
       <c r="S21" s="7" t="n">
-        <v>7.63</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="T21" t="n">
         <v>18</v>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -3358,14 +3358,14 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>06/30/2026 11:58</t>
+          <t>07/01/2026 13:10</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>15928.56</v>
+        <v>15922.12</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>-20.1</v>
+        <v>-20.13</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>20.54</v>
@@ -3383,7 +3383,7 @@
         <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>-155.78</v>
+        <v>-74.81</v>
       </c>
       <c r="P24" t="n">
         <v>12</v>
@@ -3392,25 +3392,25 @@
         <v>30</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>0.7048111723798154</v>
+        <v>0.8354594642150178</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>1.29</v>
+        <v>0.79</v>
       </c>
       <c r="T24" t="n">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>-4044.85</v>
+        <v>-3915.33</v>
       </c>
       <c r="V24" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>35.23573200992556</v>
+        <v>35.52311435523114</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="Y24" s="7" t="n">
         <v>20.79</v>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/30/2026 11:58</t>
+          <t>07/01/2026 13:10</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>20403.4</v>
+        <v>20447.92</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>-2.43</v>
+        <v>-2.22</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>4.58</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>-836.4599999999999</v>
+        <v>-743.88</v>
       </c>
       <c r="P26" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>30</v>
+        <v>32.5</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>0.6241389381922757</v>
+        <v>0.6583616164306808</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>4.86</v>
+        <v>4.85</v>
       </c>
       <c r="T26" t="n">
         <v>67</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>403.4000000000001</v>
+        <v>447.9200000000001</v>
       </c>
       <c r="V26" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>40.29850746268657</v>
+        <v>41.7910447761194</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.13</v>
+        <v>1.15</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>4.58</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3794,20 +3794,20 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/30/2026 12:17</t>
+          <t>07/01/2026 13:29</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
-        <v>20341.33</v>
+        <v>20345.9</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>1.7</v>
+        <v>1.73</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="L28" t="n">
         <v>20000</v>
@@ -3819,34 +3819,34 @@
         <v>40</v>
       </c>
       <c r="O28" s="7" t="n">
-        <v>-259.22</v>
+        <v>-276.68</v>
       </c>
       <c r="P28" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q28" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>52.5</v>
       </c>
       <c r="R28" s="7" t="n">
-        <v>0.8428007446982698</v>
+        <v>0.8334978215343138</v>
       </c>
       <c r="S28" s="7" t="n">
-        <v>7.79</v>
+        <v>7.8</v>
       </c>
       <c r="T28" t="n">
         <v>66</v>
       </c>
       <c r="U28" s="7" t="n">
-        <v>328.24</v>
+        <v>345.9</v>
       </c>
       <c r="V28" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>54.54545454545454</v>
+        <v>57.57575757575758</v>
       </c>
       <c r="X28" s="7" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="Y28" s="7" t="n">
         <v>7.56</v>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/28/2026 02:41</t>
+          <t>07/01/2026 02:48</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/30/2026 12:03</t>
+          <t>07/01/2026 13:15</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/30/2026 12:34</t>
+          <t>07/01/2026 14:05</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06/30/2026 15:02</t>
+          <t>07/01/2026 08:32</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4270,19 +4270,19 @@
         <v>2.25</v>
       </c>
       <c r="T32" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>361.3100000000001</v>
+        <v>311.51</v>
       </c>
       <c r="V32" t="n">
         <v>23</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>50</v>
+        <v>46.93877551020408</v>
       </c>
       <c r="X32" s="7" t="n">
-        <v>1.38</v>
+        <v>1.31</v>
       </c>
       <c r="Y32" s="7" t="n">
         <v>2.18</v>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
@@ -4339,20 +4339,20 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06/30/2026 13:40</t>
+          <t>07/01/2026 17:04</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
-        <v>15518.78</v>
+        <v>14717.86</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>-22.43</v>
+        <v>-26.43</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>34.36</v>
+        <v>38.47</v>
       </c>
       <c r="K33" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="L33" t="n">
         <v>20000</v>
@@ -4364,37 +4364,37 @@
         <v>40</v>
       </c>
       <c r="O33" s="7" t="n">
-        <v>-533.95</v>
+        <v>-360.2</v>
       </c>
       <c r="P33" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q33" s="7" t="n">
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="R33" s="7" t="n">
-        <v>0.7147596331059388</v>
+        <v>0.7858399923896499</v>
       </c>
       <c r="S33" s="7" t="n">
-        <v>2.99</v>
+        <v>4.54</v>
       </c>
       <c r="T33" t="n">
-        <v>1354</v>
+        <v>1402</v>
       </c>
       <c r="U33" s="7" t="n">
-        <v>-4905.919999999998</v>
+        <v>-5355.400000000001</v>
       </c>
       <c r="V33" t="n">
-        <v>655</v>
+        <v>676</v>
       </c>
       <c r="W33" s="7" t="n">
-        <v>48.3751846381093</v>
+        <v>48.21683309557774</v>
       </c>
       <c r="X33" s="7" t="n">
         <v>0.93</v>
       </c>
       <c r="Y33" s="7" t="n">
-        <v>35.61</v>
+        <v>38.45</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>06/30/2026 13:19</t>
+          <t>07/01/2026 15:50</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>20488.15</v>
+        <v>20379.58</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>2.44</v>
+        <v>1.89</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>6.28</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>1.15</v>
+        <v>1.11</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4579,37 +4579,37 @@
         <v>0</v>
       </c>
       <c r="N35" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>20307.25</v>
+        <v>20187.42</v>
       </c>
       <c r="P35" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>44.11764705882353</v>
+        <v>44.44444444444444</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>7.137976581249282</v>
+        <v>6.736366219595363</v>
       </c>
       <c r="S35" s="7" t="n">
         <v>3.5</v>
       </c>
       <c r="T35" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>488.1500000000001</v>
+        <v>379.58</v>
       </c>
       <c r="V35" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>41.17647058823529</v>
+        <v>41.66666666666667</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>1.15</v>
+        <v>1.11</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>6.28</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/30/2026 14:33</t>
+          <t>07/01/2026 18:23</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>18861.58</v>
+        <v>18989.58</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-4.77</v>
+        <v>-4.13</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>5.41</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.17</v>
+        <v>0.28</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4688,19 +4688,19 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>19034.52</v>
+        <v>19161.24</v>
       </c>
       <c r="P36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q36" s="7" t="n">
-        <v>15</v>
+        <v>19.04761904761905</v>
       </c>
       <c r="R36" s="7" t="n">
-        <v>17.4004445937912</v>
+        <v>17.50962855739654</v>
       </c>
       <c r="S36" s="7" t="n">
         <v>2.73</v>
@@ -4775,20 +4775,20 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/30/2026 14:32</t>
+          <t>07/01/2026 18:22</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>19722.4</v>
+        <v>19857.72</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-1.38</v>
+        <v>-0.7</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>4.02</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>0.71</v>
+        <v>0.85</v>
       </c>
       <c r="L37" t="n">
         <v>20000</v>
@@ -4797,37 +4797,37 @@
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>19712.47</v>
+        <v>19847.11</v>
       </c>
       <c r="P37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q37" s="7" t="n">
-        <v>38.46153846153847</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>21.3496164923763</v>
+        <v>21.48860832670927</v>
       </c>
       <c r="S37" s="7" t="n">
         <v>2.05</v>
       </c>
       <c r="T37" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-277.6000000000001</v>
+        <v>-142.2800000000001</v>
       </c>
       <c r="V37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>28.57142857142857</v>
+        <v>33.33333333333333</v>
       </c>
       <c r="X37" s="7" t="n">
-        <v>0.71</v>
+        <v>0.85</v>
       </c>
       <c r="Y37" s="7" t="n">
         <v>4.02</v>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>06/30/2026 16:18</t>
+          <t>07/01/2026 09:56</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -5102,17 +5102,17 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/30/2026 20:03</t>
+          <t>07/01/2026 12:45</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
-        <v>19284.81</v>
+        <v>19271.15</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>-3.57</v>
+        <v>-3.64</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>3.86</v>
+        <v>3.98</v>
       </c>
       <c r="K40" s="7" t="n">
         <v>0.7</v>
@@ -5127,19 +5127,19 @@
         <v>40</v>
       </c>
       <c r="O40" s="7" t="n">
-        <v>-24.54</v>
+        <v>-41.3</v>
       </c>
       <c r="P40" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="Q40" s="7" t="n">
-        <v>45</v>
+        <v>37.5</v>
       </c>
       <c r="R40" s="7" t="n">
-        <v>0.6850211782826339</v>
+        <v>0.4805031446540881</v>
       </c>
       <c r="S40" s="7" t="n">
-        <v>0.18</v>
+        <v>0.3</v>
       </c>
       <c r="T40" t="n">
         <v>598</v>
@@ -5211,14 +5211,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>06/30/2026 20:13</t>
+          <t>07/01/2026 12:51</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
-        <v>18316.63</v>
+        <v>18297.12</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>-8.41</v>
+        <v>-8.51</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>9.33</v>
@@ -5311,20 +5311,20 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>06/30/2026 11:57</t>
+          <t>07/01/2026 13:02</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
-        <v>20312.62</v>
+        <v>20482.46</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>1.56</v>
+        <v>2.41</v>
       </c>
       <c r="J42" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>2.06</v>
+        <v>2.63</v>
       </c>
       <c r="L42" t="n">
         <v>20000</v>
@@ -5411,20 +5411,20 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>06/30/2026 11:59</t>
+          <t>07/01/2026 13:04</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
-        <v>20071.08</v>
+        <v>19986.78</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>0.35</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="J43" s="7" t="n">
         <v>1.07</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>1.14</v>
+        <v>0.98</v>
       </c>
       <c r="L43" t="n">
         <v>20000</v>
@@ -5511,20 +5511,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/29/2026 23:08</t>
+          <t>07/01/2026 13:02</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>20007.97</v>
+        <v>20015.73</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="J44" s="7" t="n">
         <v>0.03</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>2.16</v>
+        <v>2.06</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5611,20 +5611,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/30/2026 12:06</t>
+          <t>07/01/2026 13:14</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>18745.9</v>
+        <v>18859.33</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-6.25</v>
+        <v>-5.71</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>6.45</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.16</v>
+        <v>0.27</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5711,7 +5711,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/30/2026 11:56</t>
+          <t>07/01/2026 13:04</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5811,20 +5811,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/30/2026 20:18</t>
+          <t>07/01/2026 13:02</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>20097.96</v>
+        <v>20113.18</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>0.51</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>2.23</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5911,20 +5911,20 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/30/2026 12:04</t>
-        </is>
-      </c>
-      <c r="H48" s="7" t="n">
-        <v>22216.5</v>
+          <t>07/01/2026 13:23</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>22304</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>11.1</v>
+        <v>11.54</v>
       </c>
       <c r="J48" s="7" t="n">
         <v>3.34</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>1.7</v>
+        <v>1.69</v>
       </c>
       <c r="L48" t="n">
         <v>20000</v>
@@ -6011,20 +6011,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06/30/2026 12:02</t>
+          <t>07/01/2026 01:40</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>25250.4</v>
+        <v>25234.53</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>26.25</v>
+        <v>26.17</v>
       </c>
       <c r="J49" s="7" t="n">
         <v>5.53</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>1.9</v>
+        <v>1.87</v>
       </c>
       <c r="L49" t="n">
         <v>20000</v>
@@ -6111,20 +6111,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>06/30/2026 05:42</t>
+          <t>07/01/2026 12:59</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>19425.83</v>
+        <v>19461.06</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>-2.87</v>
+        <v>-2.69</v>
       </c>
       <c r="J50" s="7" t="n">
         <v>3.47</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>0.62</v>
+        <v>0.67</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6211,20 +6211,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/30/2026 11:58</t>
+          <t>07/01/2026 13:10</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>19619.35</v>
+        <v>19620.74</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-1.89</v>
+        <v>-1.88</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6311,11 +6311,11 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/30/2026 06:46</t>
+          <t>07/01/2026 15:23</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>776.4299999999999</v>
+        <v>770.62</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>-99.38</v>
@@ -6336,7 +6336,7 @@
         <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>-1234.8</v>
+        <v>-1202.01</v>
       </c>
       <c r="P52" t="n">
         <v>14</v>
@@ -6345,22 +6345,22 @@
         <v>35</v>
       </c>
       <c r="R52" s="7" t="n">
-        <v>0.8226203575748348</v>
+        <v>0.8265647995844515</v>
       </c>
       <c r="S52" s="7" t="n">
-        <v>20.27</v>
+        <v>20.28</v>
       </c>
       <c r="T52" t="n">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-20232.17000000001</v>
+        <v>-20186.86</v>
       </c>
       <c r="V52" t="n">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>41.36807817589577</v>
+        <v>41.65316045380875</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.82</v>
@@ -6375,7 +6375,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/30/2026 16:28</t>
+          <t>07/01/2026 10:05</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
@@ -6638,14 +6638,14 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>06/30/2026 16:40</t>
+          <t>07/01/2026 10:42</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
-        <v>27921.07</v>
+        <v>27964.41</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>-22.66</v>
+        <v>-22.54</v>
       </c>
       <c r="J55" s="7" t="n">
         <v>29.98</v>
@@ -6663,7 +6663,7 @@
         <v>40</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>14.10999999999999</v>
+        <v>46.68999999999999</v>
       </c>
       <c r="P55" t="n">
         <v>32</v>
@@ -6672,22 +6672,22 @@
         <v>80</v>
       </c>
       <c r="R55" s="7" t="n">
-        <v>1.06187510962989</v>
+        <v>1.20474478161726</v>
       </c>
       <c r="S55" s="7" t="n">
         <v>0.55</v>
       </c>
       <c r="T55" t="n">
-        <v>3102</v>
+        <v>3117</v>
       </c>
       <c r="U55" s="7" t="n">
-        <v>-6360.929999999999</v>
+        <v>-6317.59</v>
       </c>
       <c r="V55" t="n">
-        <v>1836</v>
+        <v>1838</v>
       </c>
       <c r="W55" s="7" t="n">
-        <v>59.18762088974855</v>
+        <v>58.96695540583895</v>
       </c>
       <c r="X55" s="7" t="n">
         <v>0.79</v>
@@ -6702,7 +6702,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -7020,7 +7020,7 @@
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>06/28/2026 01:54</t>
+          <t>07/01/2026 01:59</t>
         </is>
       </c>
       <c r="H59" s="9" t="n">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>06/27/2026 21:51</t>
+          <t>06/30/2026 22:35</t>
         </is>
       </c>
       <c r="H60" s="9" t="n">
@@ -7293,7 +7293,7 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>06/30/2026 12:10</t>
+          <t>07/01/2026 13:18</t>
         </is>
       </c>
       <c r="H62" s="9" t="n">
@@ -7384,20 +7384,20 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>06/30/2026 12:08</t>
+          <t>07/01/2026 13:16</t>
         </is>
       </c>
       <c r="H63" s="9" t="n">
-        <v>19976.9</v>
+        <v>19983.49</v>
       </c>
       <c r="I63" s="9" t="n">
-        <v>-0.11</v>
+        <v>-0.08</v>
       </c>
       <c r="J63" s="9" t="n">
         <v>0.27</v>
       </c>
       <c r="K63" s="9" t="n">
-        <v>0.68</v>
+        <v>0.78</v>
       </c>
       <c r="L63" s="8" t="n">
         <v>20000</v>
@@ -7406,19 +7406,19 @@
         <v>0</v>
       </c>
       <c r="N63" s="8" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="O63" s="9" t="n">
-        <v>19976.74</v>
+        <v>19982.97</v>
       </c>
       <c r="P63" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q63" s="9" t="n">
-        <v>31.81818181818182</v>
+        <v>36</v>
       </c>
       <c r="R63" s="9" t="n">
-        <v>275.5188951490999</v>
+        <v>270.857798784605</v>
       </c>
       <c r="S63" s="9" t="n">
         <v>0.12</v>
@@ -7566,7 +7566,7 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>06/30/2026 12:50</t>
+          <t>07/01/2026 15:11</t>
         </is>
       </c>
       <c r="H65" s="9" t="n">
@@ -7657,7 +7657,7 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>06/30/2026 11:57</t>
+          <t>07/01/2026 01:21</t>
         </is>
       </c>
       <c r="H66" s="9" t="n">
@@ -7748,7 +7748,7 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>06/30/2026 05:40</t>
+          <t>07/01/2026 12:57</t>
         </is>
       </c>
       <c r="H67" s="8" t="n">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>06/29/2026 23:13</t>
+          <t>07/01/2026 01:41</t>
         </is>
       </c>
       <c r="H68" s="9" t="n">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>06/30/2026 11:56</t>
+          <t>07/01/2026 13:06</t>
         </is>
       </c>
       <c r="H69" s="9" t="n">
@@ -8574,7 +8574,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>06/28/2026 01:54</t>
+          <t>07/01/2026 01:59</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -8615,7 +8615,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>06/27/2026 21:51</t>
+          <t>06/30/2026 22:35</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -8697,7 +8697,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>06/30/2026 12:10</t>
+          <t>07/01/2026 13:18</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -8738,17 +8738,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>06/30/2026 12:08</t>
+          <t>07/01/2026 13:16</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>19976.9</v>
+        <v>19983.49</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>-0.11</v>
+        <v>-0.08</v>
       </c>
       <c r="I12" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>06/30/2026 12:50</t>
+          <t>07/01/2026 15:11</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -8861,7 +8861,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>06/30/2026 11:57</t>
+          <t>07/01/2026 01:21</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>06/30/2026 05:40</t>
+          <t>07/01/2026 12:57</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -8943,7 +8943,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>06/29/2026 23:13</t>
+          <t>07/01/2026 01:41</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -8984,7 +8984,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>06/30/2026 11:56</t>
+          <t>07/01/2026 13:06</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>06/27/2026 22:45</t>
+          <t>06/30/2026 23:53</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -10048,7 +10048,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>06/27/2026 22:50</t>
+          <t>06/30/2026 23:59</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -10071,7 +10071,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>06/28/2026 10:55</t>
+          <t>07/01/2026 10:57</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -10117,7 +10117,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>06/28/2026 17:14</t>
+          <t>07/01/2026 17:19</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
@@ -10278,7 +10278,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>06/30/2026 15:10</t>
+          <t>07/01/2026 08:43</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
@@ -10324,11 +10324,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06/30/2026 12:06</t>
+          <t>07/01/2026 13:17</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
-        <v>20016.73</v>
+        <v>20177.76</v>
       </c>
     </row>
     <row r="25">
@@ -10347,11 +10347,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06/30/2026 12:02</t>
+          <t>07/01/2026 13:14</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19817.56</v>
+        <v>19803.1</v>
       </c>
     </row>
     <row r="26">
@@ -10370,11 +10370,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>06/30/2026 12:09</t>
+          <t>07/01/2026 13:27</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>19701.56</v>
+        <v>19791.6</v>
       </c>
     </row>
     <row r="27">
@@ -10393,11 +10393,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>06/30/2026 05:57</t>
+          <t>07/01/2026 13:25</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>20090.55</v>
+        <v>20039.67</v>
       </c>
     </row>
     <row r="28">
@@ -10416,11 +10416,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>06/30/2026 12:10</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="n">
-        <v>19864.52</v>
+          <t>07/01/2026 13:31</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>19806</v>
       </c>
     </row>
     <row r="29">
@@ -10462,11 +10462,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>06/30/2026 12:23</t>
+          <t>07/01/2026 13:48</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>19024.05</v>
+        <v>18759.75</v>
       </c>
     </row>
     <row r="31">
@@ -10485,11 +10485,11 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>06/30/2026 12:23</t>
+          <t>07/01/2026 13:38</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>19918.01</v>
+        <v>19916.63</v>
       </c>
     </row>
     <row r="32">
@@ -10508,11 +10508,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>06/30/2026 12:22</t>
+          <t>07/01/2026 13:51</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>20431.72</v>
+        <v>20428.93</v>
       </c>
     </row>
     <row r="33">
@@ -10531,11 +10531,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>06/30/2026 12:31</t>
+          <t>07/01/2026 14:00</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>20653.21</v>
+        <v>20648.93</v>
       </c>
     </row>
     <row r="34">
@@ -10554,11 +10554,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>06/30/2026 12:32</t>
+          <t>07/01/2026 13:59</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>20346.96</v>
+        <v>20383.4</v>
       </c>
     </row>
     <row r="35">
@@ -10577,11 +10577,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>06/30/2026 12:29</t>
+          <t>07/01/2026 14:19</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>19956.13</v>
+        <v>19895.55</v>
       </c>
     </row>
     <row r="36">

</xml_diff>

<commit_message>
Update dashboards — 2026-07-08
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-07-07 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-07-08 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>07/07/2026 08:57</t>
+          <t>07/08/2026 21:47</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>49771.76</v>
+        <v>49384.91</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>131.52</v>
+        <v>129.72</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>4179.099999999999</v>
+        <v>2067.01</v>
       </c>
       <c r="P2" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>5.283839885192968</v>
+        <v>2.155554685927682</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>2.95</v>
+        <v>3.15</v>
       </c>
       <c r="T2" t="n">
-        <v>3062</v>
+        <v>3071</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>24805.26</v>
+        <v>24384.91</v>
       </c>
       <c r="V2" t="n">
-        <v>1929</v>
+        <v>1930</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>62.99804049640758</v>
+        <v>62.84597850862911</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.07</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>07/05/2026 19:29</t>
+          <t>07/08/2026 19:31</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>07/07/2026 13:01</t>
+          <t>07/08/2026 18:59</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>07/07/2026 05:18</t>
+          <t>07/08/2026 20:16</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1327,7 +1327,7 @@
         <v>6.6</v>
       </c>
       <c r="T5" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="U5" s="7" t="n">
         <v>1521.18</v>
@@ -1336,7 +1336,7 @@
         <v>78</v>
       </c>
       <c r="W5" s="7" t="n">
-        <v>65.54621848739495</v>
+        <v>65</v>
       </c>
       <c r="X5" s="7" t="n">
         <v>1.15</v>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>07/04/2026 16:47</t>
+          <t>07/08/2026 08:54</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>07/06/2026 17:30</t>
+          <t>07/08/2026 17:24</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2417,19 +2417,19 @@
         <v>20.06</v>
       </c>
       <c r="T15" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-1298.499999999999</v>
+        <v>-1208.299999999999</v>
       </c>
       <c r="V15" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>53.33333333333334</v>
+        <v>53.6144578313253</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="Y15" s="7" t="n">
         <v>7.15</v>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2486,17 +2486,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>07/07/2026 05:56</t>
+          <t>07/08/2026 20:31</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>113.19</v>
+        <v>110.31</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-99.44</v>
+        <v>-99.45999999999999</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>99.44</v>
+        <v>99.45999999999999</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>0.7</v>
@@ -2511,37 +2511,37 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-193.84</v>
+        <v>-4.699999999999999</v>
       </c>
       <c r="P16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>25</v>
+        <v>27.5</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.0389687654933069</v>
+        <v>0.6373456790123457</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>0.96</v>
+        <v>0.03</v>
       </c>
       <c r="T16" t="n">
-        <v>1970</v>
+        <v>1990</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-20309.22</v>
+        <v>-20312.09</v>
       </c>
       <c r="V16" t="n">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>32.48730964467005</v>
+        <v>32.46231155778894</v>
       </c>
       <c r="X16" s="7" t="n">
         <v>0.7</v>
       </c>
       <c r="Y16" s="7" t="n">
-        <v>99.45</v>
+        <v>99.47</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>07/05/2026 21:58</t>
+          <t>07/08/2026 19:55</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>07/08/2026 13:21</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>07/07/2026 10:20</t>
+          <t>07/08/2026 17:33</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>07/07/2026 10:16</t>
+          <t>07/08/2026 17:32</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>07/06/2026 05:59</t>
+          <t>07/08/2026 16:02</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>07/07/2026 09:54</t>
+          <t>07/08/2026 17:21</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19924.12</v>
+        <v>19556.08</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-0.37</v>
+        <v>-2.21</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>5.42</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.97</v>
+        <v>0.86</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,25 +3274,25 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-23.59999999999995</v>
+        <v>-637.2099999999999</v>
       </c>
       <c r="P23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>50</v>
+        <v>47.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.9887683763165034</v>
+        <v>0.7390280462632287</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4</v>
+        <v>4.05</v>
       </c>
       <c r="T23" t="n">
         <v>61</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-115.9399999999998</v>
+        <v>-443.9199999999998</v>
       </c>
       <c r="V23" t="n">
         <v>31</v>
@@ -3301,7 +3301,7 @@
         <v>50.81967213114754</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.96</v>
+        <v>0.86</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>5.42</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>07/07/2026 10:14</t>
+          <t>07/08/2026 17:31</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16173.74</v>
+        <v>16101.91</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-18.87</v>
+        <v>-19.23</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.54</v>
@@ -3492,31 +3492,31 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>236.8</v>
+        <v>28.23</v>
       </c>
       <c r="P25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.579596632073625</v>
+        <v>1.068262604280015</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.84</v>
+        <v>0.7</v>
       </c>
       <c r="T25" t="n">
-        <v>445</v>
+        <v>454</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3826.88</v>
+        <v>-3898.09</v>
       </c>
       <c r="V25" t="n">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>35.50561797752809</v>
+        <v>36.12334801762114</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>0.53</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>07/07/2026 06:38</t>
+          <t>07/08/2026 20:51</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>21422.24</v>
+        <v>22399.12</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>7.13</v>
+        <v>12.37</v>
       </c>
       <c r="J26" t="n">
         <v>2</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>2.7</v>
+        <v>2.82</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,34 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>-444.06</v>
+        <v>80.77</v>
       </c>
       <c r="P26" t="n">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>0.09767744295206551</v>
+        <v>113.1805555555556</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>2.46</v>
+        <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>521</v>
+        <v>775</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>1628.27</v>
+        <v>2318.61</v>
       </c>
       <c r="V26" t="n">
-        <v>294</v>
+        <v>508</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>56.4299424184261</v>
+        <v>65.54838709677419</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>2.67</v>
+        <v>2.61</v>
       </c>
       <c r="Y26" s="7" t="n">
         <v>2</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>07/06/2026 17:59</t>
+          <t>07/08/2026 17:33</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20372.39</v>
+        <v>20279.19</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-2.58</v>
+        <v>-3.03</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>4.72</v>
+        <v>5.35</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,19 +3710,19 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-692.01</v>
+        <v>-742.9699999999999</v>
       </c>
       <c r="P27" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>32.5</v>
+        <v>35</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.6744279047009673</v>
+        <v>0.6649152557661259</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>4.97</v>
+        <v>5.42</v>
       </c>
       <c r="T27" t="n">
         <v>71</v>
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>07/07/2026 10:26</t>
+          <t>07/08/2026 17:36</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20361.05</v>
+        <v>20356.7</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>1.8</v>
+        <v>1.78</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,34 +3928,34 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-199.09</v>
+        <v>-19.62999999999997</v>
       </c>
       <c r="P29" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>52.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.8690068098825543</v>
+        <v>0.9853058963552933</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>6.93</v>
+        <v>6.08</v>
       </c>
       <c r="T29" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>361.0500000000001</v>
+        <v>356.6199999999999</v>
       </c>
       <c r="V29" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>58.33333333333334</v>
+        <v>57.14285714285714</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>BB Fade Prop | AUDJPY, BB Fade Prop | AUDJPY.pro, BB Fade Prop | AUDNZD, BB Fade Prop | AUDNZD.pro, BB Fade Prop | CADJPY, BB Fade Prop | CADJPY.pro, BB Fade Prop | CHFJPY, BB Fade Prop | CHFJPY.pro, BB Fade Prop | GBPJPY, BB Fade Prop | GBPJPY.pro, BB Fade Prop | GBPNZD.pro, BB Fade Prop | NZDJPY.pro, BB Fade Prop | NZDUSD, BB Fade Prop | SGDJPY, BB Fade Prop | XAGUSD</t>
+          <t>BB Fade Prop | AUDJPY, BB Fade Prop | AUDJPY.pro, BB Fade Prop | AUDNZD, BB Fade Prop | AUDNZD.pro, BB Fade Prop | CADJPY, BB Fade Prop | CADJPY.pro, BB Fade Prop | CHFJPY, BB Fade Prop | CHFJPY.pro, BB Fade Prop | GBPJPY, BB Fade Prop | GBPJPY.pro, BB Fade Prop | GBPNZD, BB Fade Prop | GBPNZD.pro, BB Fade Prop | NZDJPY, BB Fade Prop | NZDJPY.pro, BB Fade Prop | NZDUSD, BB Fade Prop | SGDJPY, BB Fade Prop | XAGUSD</t>
         </is>
       </c>
     </row>
@@ -4121,20 +4121,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>07/07/2026 10:39</t>
+          <t>07/08/2026 17:45</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20827.83</v>
+        <v>20802.54</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>4.15</v>
+        <v>4.02</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>1.09</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>2.75</v>
+        <v>2.61</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -4146,7 +4146,7 @@
         <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>821.58</v>
+        <v>803.02</v>
       </c>
       <c r="P31" t="n">
         <v>13</v>
@@ -4155,25 +4155,25 @@
         <v>32.5</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>2.920970796605018</v>
+        <v>2.799484593837535</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="T31" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>827.8299999999999</v>
+        <v>802.54</v>
       </c>
       <c r="V31" t="n">
         <v>14</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>29.16666666666667</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>2.75</v>
+        <v>2.61</v>
       </c>
       <c r="Y31" s="7" t="n">
         <v>1.1</v>
@@ -4185,7 +4185,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
+          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -4230,20 +4230,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>07/07/2026 10:16</t>
+          <t>07/08/2026 17:33</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
-        <v>19983.13</v>
+        <v>19999.99</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>-0.08</v>
+        <v>0</v>
       </c>
       <c r="J32" s="7" t="n">
         <v>0.27</v>
       </c>
-      <c r="K32" s="7" t="n">
-        <v>0.78</v>
+      <c r="K32" t="n">
+        <v>1</v>
       </c>
       <c r="L32" t="n">
         <v>20000</v>
@@ -4252,37 +4252,37 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="O32" s="7" t="n">
-        <v>19982.97</v>
+        <v>19998.95</v>
       </c>
       <c r="P32" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q32" s="7" t="n">
-        <v>36</v>
+        <v>37.93103448275862</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>270.857798784605</v>
+        <v>247.9615954556681</v>
       </c>
       <c r="S32" s="7" t="n">
         <v>0.12</v>
       </c>
       <c r="T32" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="U32" s="7" t="n">
-        <v>6.049999999999995</v>
+        <v>-0.01000000000000512</v>
       </c>
       <c r="V32" t="n">
         <v>10</v>
       </c>
       <c r="W32" s="7" t="n">
-        <v>37.03703703703704</v>
+        <v>35.71428571428572</v>
       </c>
       <c r="X32" s="7" t="n">
-        <v>1.08</v>
+        <v>1</v>
       </c>
       <c r="Y32" s="7" t="n">
         <v>0.27</v>
@@ -4294,12 +4294,12 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>07/07/2026 10:55</t>
+          <t>07/08/2026 17:53</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>07/07/2026 03:59</t>
+          <t>07/08/2026 15:20</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20188.58</v>
+        <v>20305.8</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.95</v>
+        <v>1.54</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>2.22</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.16</v>
+        <v>1.27</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,34 +4473,34 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-284.43</v>
+        <v>-141.48</v>
       </c>
       <c r="P34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.735998440661605</v>
+        <v>0.8621482578533012</v>
       </c>
       <c r="S34" s="7" t="n">
         <v>2.33</v>
       </c>
       <c r="T34" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>289.3799999999999</v>
+        <v>204.55</v>
       </c>
       <c r="V34" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>46.2962962962963</v>
+        <v>46.42857142857143</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1.25</v>
+        <v>1.16</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>2.23</v>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4557,20 +4557,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>07/07/2026 12:43</t>
+          <t>07/08/2026 18:48</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>13974.81</v>
+        <v>14219.4</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>-30.14</v>
+        <v>-28.92</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>41.42</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="L35" t="n">
         <v>20000</v>
@@ -4582,34 +4582,34 @@
         <v>40</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>-45.78000000000003</v>
+        <v>322.1900000000001</v>
       </c>
       <c r="P35" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>50</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>0.9685436492939842</v>
+        <v>1.253469381332998</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>3.15</v>
+        <v>1.75</v>
       </c>
       <c r="T35" t="n">
-        <v>1571</v>
+        <v>1618</v>
       </c>
       <c r="U35" s="7" t="n">
-        <v>-6022.469999999998</v>
+        <v>-5708.01</v>
       </c>
       <c r="V35" t="n">
-        <v>757</v>
+        <v>783</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>48.18586887332909</v>
+        <v>48.39307787391841</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="Y35" s="7" t="n">
         <v>41.41</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4706,19 +4706,19 @@
         <v>0.74</v>
       </c>
       <c r="T36" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>937.83</v>
+        <v>1039.71</v>
       </c>
       <c r="V36" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>60.46511627906976</v>
+        <v>61.36363636363637</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>1.54</v>
+        <v>1.6</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>2.44</v>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4775,20 +4775,20 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>07/07/2026 12:01</t>
+          <t>07/08/2026 18:25</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>20371.01</v>
+        <v>20403.25</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>1.85</v>
+        <v>2.01</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>6.28</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="L37" t="n">
         <v>20000</v>
@@ -4797,19 +4797,19 @@
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>20167.31</v>
+        <v>20194.59</v>
       </c>
       <c r="P37" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q37" s="7" t="n">
-        <v>44.73684210526316</v>
+        <v>46.15384615384615</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>6.695886100974954</v>
+        <v>6.703590835658687</v>
       </c>
       <c r="S37" s="7" t="n">
         <v>3.5</v>
@@ -4818,16 +4818,16 @@
         <v>38</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>366.0500000000001</v>
+        <v>403.2500000000001</v>
       </c>
       <c r="V37" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>42.10526315789473</v>
+        <v>44.73684210526316</v>
       </c>
       <c r="X37" s="7" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="Y37" s="7" t="n">
         <v>6.28</v>
@@ -4839,12 +4839,12 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>07/07/2026 13:31</t>
+          <t>07/08/2026 19:22</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4993,11 +4993,11 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>07/06/2026 11:33</t>
+          <t>07/08/2026 19:09</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
-        <v>19993.04</v>
+        <v>19937.02</v>
       </c>
       <c r="I39" s="7" t="n">
         <v>-0.02</v>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>07/07/2026 06:17</t>
+          <t>07/08/2026 20:42</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>07/07/2026 08:34</t>
+          <t>07/08/2026 21:29</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5320,14 +5320,14 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>07/06/2026 17:21</t>
+          <t>07/08/2026 17:22</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
-        <v>19463.85</v>
+        <v>19432.74</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>-2.67</v>
+        <v>-2.83</v>
       </c>
       <c r="J42" s="7" t="n">
         <v>4.17</v>
@@ -5345,34 +5345,34 @@
         <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-13.95</v>
+        <v>-43.01</v>
       </c>
       <c r="P42" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q42" s="7" t="n">
-        <v>40</v>
+        <v>42.5</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>0.729126213592233</v>
+        <v>0.503119223659889</v>
       </c>
       <c r="S42" s="7" t="n">
-        <v>0.1</v>
+        <v>0.28</v>
       </c>
       <c r="T42" t="n">
-        <v>1178</v>
+        <v>1220</v>
       </c>
       <c r="U42" s="7" t="n">
-        <v>-525.01</v>
+        <v>-566.86</v>
       </c>
       <c r="V42" t="n">
-        <v>540</v>
+        <v>558</v>
       </c>
       <c r="W42" s="7" t="n">
-        <v>45.84040747028862</v>
+        <v>45.73770491803278</v>
       </c>
       <c r="X42" s="7" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="Y42" s="7" t="n">
         <v>4.17</v>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
@@ -5429,20 +5429,20 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>07/07/2026 10:05</t>
+          <t>07/08/2026 17:26</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
-        <v>18227.89</v>
+        <v>18235.59</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>-8.85</v>
+        <v>-8.81</v>
       </c>
       <c r="J43" s="7" t="n">
-        <v>9.550000000000001</v>
+        <v>9.66</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="L43" t="n">
         <v>20000</v>
@@ -5451,31 +5451,40 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>16.32</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>1.851330203442879</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>0.07000000000000001</v>
       </c>
       <c r="T43" t="n">
-        <v>2402</v>
+        <v>2457</v>
       </c>
       <c r="U43" s="7" t="n">
-        <v>-1796.24</v>
+        <v>-1765.39</v>
       </c>
       <c r="V43" t="n">
-        <v>1039</v>
+        <v>1068</v>
       </c>
       <c r="W43" s="7" t="n">
-        <v>43.255620316403</v>
+        <v>43.46764346764347</v>
       </c>
       <c r="X43" s="7" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="Y43" s="7" t="n">
-        <v>9.65</v>
+        <v>9.67</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -5484,7 +5493,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
@@ -5529,20 +5538,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>07/07/2026 10:07</t>
+          <t>07/08/2026 17:27</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>20291.09</v>
+        <v>20047.44</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>1.45</v>
+        <v>0.23</v>
       </c>
       <c r="J44" s="7" t="n">
-        <v>1.32</v>
+        <v>2.13</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>1.47</v>
+        <v>1.06</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5551,31 +5560,40 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>19956.84</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>46.42857142857143</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>22.94144357099665</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>1.14</v>
       </c>
       <c r="T44" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>291.09</v>
+        <v>47.44000000000005</v>
       </c>
       <c r="V44" t="n">
         <v>12</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>48</v>
+        <v>44.44444444444444</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>1.47</v>
+        <v>1.06</v>
       </c>
       <c r="Y44" s="7" t="n">
-        <v>1.32</v>
+        <v>2.12</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -5584,12 +5602,12 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC44" t="inlineStr">
@@ -5629,14 +5647,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>07/07/2026 09:59</t>
+          <t>07/08/2026 17:23</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19838.65</v>
+        <v>19841.05</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.79</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>1.6</v>
@@ -5660,16 +5678,16 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-160.27</v>
+        <v>-158.95</v>
       </c>
       <c r="V45" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>51.59235668789809</v>
+        <v>47.72727272727273</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0.79</v>
@@ -5684,7 +5702,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5694,7 +5712,7 @@
       </c>
       <c r="AC45" t="inlineStr">
         <is>
-          <t>Round Numbers MOL | AUDJPY, Round Numbers MOL | AUDUSD, Round Numbers MOL | CADJPY, Round Numbers MOL | EURJPY, Round Numbers MOL | EURUSD, Round Numbers MOL | GBPCAD, Round Numbers MOL | GBPJPY, Round Numbers MOL | GBPUSD, Round Numbers MOL | NZDJPY, Round Numbers MOL | NZDUSD, Round Numbers MOL | USDCHF, Round Numbers MOL | USDJPY</t>
+          <t>Round Numbers MOL | AUDJPY, Round Numbers MOL | AUDUSD, Round Numbers MOL | CADJPY, Round Numbers MOL | EURAUD, Round Numbers MOL | EURJPY, Round Numbers MOL | EURUSD, Round Numbers MOL | GBPCAD, Round Numbers MOL | GBPJPY, Round Numbers MOL | GBPUSD, Round Numbers MOL | NZDJPY, Round Numbers MOL | NZDUSD, Round Numbers MOL | USDCHF, Round Numbers MOL | USDJPY</t>
         </is>
       </c>
     </row>
@@ -5729,7 +5747,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>07/07/2026 09:58</t>
+          <t>07/08/2026 17:23</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5860,19 +5878,19 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-1472.87</v>
+        <v>-1429.81</v>
       </c>
       <c r="V47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>27.02702702702703</v>
+        <v>28.94736842105263</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5884,7 +5902,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5929,7 +5947,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>07/07/2026 10:11</t>
+          <t>07/08/2026 17:30</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6029,20 +6047,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>07/07/2026 10:34</t>
+          <t>07/08/2026 17:42</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>19783.21</v>
+        <v>19797.3</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>-1.1</v>
+        <v>-1.03</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>2.7</v>
+        <v>2.74</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="L49" t="n">
         <v>20000</v>
@@ -6060,22 +6078,22 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="U49" s="7" t="n">
-        <v>-216.7900000000001</v>
+        <v>-202.7</v>
       </c>
       <c r="V49" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="W49" s="7" t="n">
-        <v>39.15343915343915</v>
+        <v>40.5940594059406</v>
       </c>
       <c r="X49" s="7" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="Y49" s="7" t="n">
-        <v>2.68</v>
+        <v>2.72</v>
       </c>
       <c r="Z49" t="inlineStr">
         <is>
@@ -6084,7 +6102,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
@@ -6129,20 +6147,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>07/08/2026 17:37</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>22176.98</v>
+        <v>22062.68</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>10.91</v>
+        <v>10.34</v>
       </c>
       <c r="J50" s="7" t="n">
         <v>3.34</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>1.49</v>
+        <v>1.43</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6160,19 +6178,19 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>541</v>
+        <v>579</v>
       </c>
       <c r="U50" s="7" t="n">
-        <v>2237.7</v>
+        <v>2062.68</v>
       </c>
       <c r="V50" t="n">
-        <v>281</v>
+        <v>304</v>
       </c>
       <c r="W50" s="7" t="n">
-        <v>51.94085027726432</v>
+        <v>52.50431778929189</v>
       </c>
       <c r="X50" s="7" t="n">
-        <v>1.5</v>
+        <v>1.43</v>
       </c>
       <c r="Y50" s="7" t="n">
         <v>3.34</v>
@@ -6184,7 +6202,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
@@ -6229,20 +6247,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>07/07/2026 10:22</t>
+          <t>07/08/2026 17:34</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>25009.08</v>
+        <v>24805.28</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>25.04</v>
+        <v>24.02</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>5.53</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>1.6</v>
+        <v>1.54</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6260,19 +6278,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>947</v>
+        <v>1002</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>5029.079999999999</v>
+        <v>4805.280000000001</v>
       </c>
       <c r="V51" t="n">
-        <v>510</v>
+        <v>538</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>53.85427666314678</v>
+        <v>53.69261477045908</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>1.6</v>
+        <v>1.54</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>5.53</v>
@@ -6284,7 +6302,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6329,20 +6347,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>07/06/2026 17:15</t>
+          <t>07/08/2026 17:19</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19461.06</v>
+        <v>19172.91</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-2.69</v>
+        <v>-4.13</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>3.47</v>
+        <v>4.72</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.67</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6360,22 +6378,22 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-538.9400000000001</v>
+        <v>-827.0900000000001</v>
       </c>
       <c r="V52" t="n">
         <v>7</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>31.81818181818182</v>
+        <v>30.43478260869566</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.67</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>3.47</v>
+        <v>4.72</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6384,7 +6402,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6429,14 +6447,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>07/07/2026 10:39</t>
+          <t>07/08/2026 17:44</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19765.44</v>
+        <v>19743.76</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.19</v>
+        <v>-1.3</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.39</v>
@@ -6451,25 +6469,34 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>0</v>
+        <v>-78.94</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q53" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R53" s="7" t="n">
+        <v>0.4557738710789382</v>
+      </c>
+      <c r="S53" s="7" t="n">
+        <v>0.49</v>
       </c>
       <c r="T53" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-236.97</v>
+        <v>-256.2400000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>37.5</v>
+        <v>37.2093023255814</v>
       </c>
       <c r="X53" s="7" t="n">
         <v>0.29</v>
@@ -6484,7 +6511,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6529,20 +6556,20 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>07/06/2026 19:25</t>
+          <t>07/08/2026 17:50</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
-        <v>19785.93</v>
+        <v>19664.2</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>-1.06</v>
+        <v>-1.67</v>
       </c>
       <c r="J54" s="7" t="n">
         <v>4.63</v>
       </c>
       <c r="K54" s="7" t="n">
-        <v>0.86</v>
+        <v>0.79</v>
       </c>
       <c r="L54" t="n">
         <v>20000</v>
@@ -6560,19 +6587,19 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="U54" s="7" t="n">
-        <v>-215.2100000000001</v>
+        <v>-335.8</v>
       </c>
       <c r="V54" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="W54" s="7" t="n">
-        <v>38.16793893129771</v>
+        <v>38.23529411764706</v>
       </c>
       <c r="X54" s="7" t="n">
-        <v>0.86</v>
+        <v>0.79</v>
       </c>
       <c r="Y54" s="7" t="n">
         <v>4.63</v>
@@ -6584,7 +6611,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -6629,20 +6656,20 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>07/06/2026 18:24</t>
+          <t>07/08/2026 17:39</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
-        <v>20011.43</v>
+        <v>19979.85</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.09</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>1.01</v>
+        <v>0.99</v>
       </c>
       <c r="L55" t="n">
         <v>20000</v>
@@ -6660,22 +6687,22 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>591</v>
+        <v>630</v>
       </c>
       <c r="U55" s="7" t="n">
-        <v>-0.6300000000000097</v>
+        <v>-20.15000000000003</v>
       </c>
       <c r="V55" t="n">
-        <v>293</v>
+        <v>311</v>
       </c>
       <c r="W55" s="7" t="n">
-        <v>49.57698815566836</v>
+        <v>49.36507936507937</v>
       </c>
       <c r="X55" s="7" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="Y55" s="7" t="n">
-        <v>0.78</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Z55" t="inlineStr">
         <is>
@@ -6684,7 +6711,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -6729,20 +6756,20 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>07/06/2026 09:13</t>
+          <t>07/08/2026 17:48</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
-        <v>19895.47</v>
+        <v>19821.18</v>
       </c>
       <c r="I56" s="7" t="n">
-        <v>-0.54</v>
+        <v>-0.91</v>
       </c>
       <c r="J56" s="7" t="n">
         <v>1.07</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>0.92</v>
+        <v>0.88</v>
       </c>
       <c r="L56" t="n">
         <v>20000</v>
@@ -6760,16 +6787,16 @@
         <v>0</v>
       </c>
       <c r="T56" t="n">
-        <v>494</v>
+        <v>528</v>
       </c>
       <c r="U56" s="7" t="n">
-        <v>-152.22</v>
+        <v>-178.82</v>
       </c>
       <c r="V56" t="n">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="W56" s="7" t="n">
-        <v>46.96356275303643</v>
+        <v>46.78030303030303</v>
       </c>
       <c r="X56" s="7" t="n">
         <v>0.88</v>
@@ -6784,7 +6811,7 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr">
@@ -6829,20 +6856,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>07/07/2026 09:58</t>
+          <t>07/08/2026 17:23</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19781.41</v>
+        <v>19786.88</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.09</v>
+        <v>-1.06</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6851,28 +6878,37 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>168.15</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>8.349213286713287</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.05</v>
       </c>
       <c r="T57" t="n">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-221</v>
+        <v>-213.1200000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>42.78728606356968</v>
+        <v>43.23040380047506</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6884,7 +6920,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6929,20 +6965,20 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>07/07/2026 10:32</t>
+          <t>07/08/2026 17:41</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
-        <v>18509.27</v>
+        <v>18297.67</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>-7.46</v>
+        <v>-8.52</v>
       </c>
       <c r="J58" s="7" t="n">
-        <v>7.46</v>
+        <v>8.52</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="L58" t="n">
         <v>20000</v>
@@ -6960,22 +6996,22 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1595</v>
+        <v>1706</v>
       </c>
       <c r="U58" s="7" t="n">
-        <v>-1493.22</v>
+        <v>-1698.01</v>
       </c>
       <c r="V58" t="n">
-        <v>695</v>
+        <v>739</v>
       </c>
       <c r="W58" s="7" t="n">
-        <v>43.57366771159874</v>
+        <v>43.31770222743259</v>
       </c>
       <c r="X58" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="Y58" s="7" t="n">
-        <v>7.52</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="Z58" t="inlineStr">
         <is>
@@ -6984,7 +7020,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB58" t="inlineStr">
@@ -7029,20 +7065,20 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>07/07/2026 10:44</t>
+          <t>07/08/2026 17:48</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
-        <v>19933.92</v>
+        <v>19928.18</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>-0.32</v>
+        <v>-0.35</v>
       </c>
       <c r="J59" s="7" t="n">
         <v>0.55</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="L59" t="n">
         <v>20000</v>
@@ -7060,19 +7096,19 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="U59" s="7" t="n">
-        <v>-66.08000000000001</v>
+        <v>-71.82000000000002</v>
       </c>
       <c r="V59" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W59" s="7" t="n">
-        <v>42.5</v>
+        <v>41.66666666666667</v>
       </c>
       <c r="X59" s="7" t="n">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="Y59" s="7" t="n">
         <v>0.55</v>
@@ -7084,7 +7120,7 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -7129,20 +7165,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>07/07/2026 10:39</t>
+          <t>07/08/2026 17:45</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>18893.31</v>
+        <v>18999.46</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-5.54</v>
+        <v>-5.01</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>12.98</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="L60" t="n">
         <v>20000</v>
@@ -7160,19 +7196,19 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>2479</v>
+        <v>2669</v>
       </c>
       <c r="U60" s="7" t="n">
-        <v>-1151.03</v>
+        <v>-1000.53</v>
       </c>
       <c r="V60" t="n">
-        <v>1154</v>
+        <v>1243</v>
       </c>
       <c r="W60" s="7" t="n">
-        <v>46.55102864058087</v>
+        <v>46.57174971899588</v>
       </c>
       <c r="X60" s="7" t="n">
-        <v>0.86</v>
+        <v>0.89</v>
       </c>
       <c r="Y60" s="7" t="n">
         <v>12.97</v>
@@ -7184,7 +7220,7 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
@@ -7229,20 +7265,20 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>07/07/2026 10:37</t>
+          <t>07/08/2026 17:43</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>19766.3</v>
+        <v>19655.14</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-1.16</v>
+        <v>-1.72</v>
       </c>
       <c r="J61" s="7" t="n">
-        <v>6.13</v>
+        <v>6.82</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L61" t="n">
         <v>20000</v>
@@ -7260,22 +7296,22 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>1476</v>
+        <v>1605</v>
       </c>
       <c r="U61" s="7" t="n">
-        <v>-230.1799999999997</v>
+        <v>-344.8100000000002</v>
       </c>
       <c r="V61" t="n">
-        <v>681</v>
+        <v>738</v>
       </c>
       <c r="W61" s="7" t="n">
-        <v>46.13821138211382</v>
+        <v>45.98130841121495</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y61" s="7" t="n">
-        <v>6.12</v>
+        <v>6.81</v>
       </c>
       <c r="Z61" t="inlineStr">
         <is>
@@ -7284,7 +7320,7 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
@@ -7329,20 +7365,20 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>07/07/2026 11:03</t>
+          <t>07/08/2026 17:57</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
-        <v>19988.04</v>
+        <v>19945.96</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>-0.06</v>
+        <v>-0.27</v>
       </c>
       <c r="J62" s="7" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="K62" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="L62" t="n">
         <v>20000</v>
@@ -7360,22 +7396,22 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="U62" s="7" t="n">
-        <v>-8.280000000000003</v>
+        <v>-54.04</v>
       </c>
       <c r="V62" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="W62" s="7" t="n">
-        <v>48.83720930232558</v>
+        <v>52.08333333333334</v>
       </c>
       <c r="X62" s="7" t="n">
-        <v>0.96</v>
+        <v>0.8</v>
       </c>
       <c r="Y62" s="7" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="Z62" t="inlineStr">
         <is>
@@ -7384,7 +7420,7 @@
       </c>
       <c r="AA62" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB62" t="inlineStr">
@@ -7429,20 +7465,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>07/06/2026 20:02</t>
-        </is>
-      </c>
-      <c r="H63" s="7" t="n">
-        <v>19191.69</v>
+          <t>07/08/2026 17:58</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>19111</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-4.04</v>
+        <v>-4.44</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7460,19 +7496,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-846.25</v>
+        <v>-889</v>
       </c>
       <c r="V63" t="n">
         <v>1</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>9.090909090909092</v>
+        <v>8.333333333333332</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>4.5</v>
@@ -7484,7 +7520,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7529,20 +7565,20 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>07/07/2026 11:08</t>
+          <t>07/08/2026 17:59</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
-        <v>19840.85</v>
+        <v>19806.81</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>-0.8</v>
+        <v>-0.97</v>
       </c>
       <c r="J64" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="L64" t="n">
         <v>20000</v>
@@ -7560,19 +7596,19 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="U64" s="7" t="n">
-        <v>-155.96</v>
+        <v>-193.19</v>
       </c>
       <c r="V64" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="W64" s="7" t="n">
-        <v>47.91666666666667</v>
+        <v>50.9433962264151</v>
       </c>
       <c r="X64" s="7" t="n">
-        <v>0.63</v>
+        <v>0.61</v>
       </c>
       <c r="Y64" s="7" t="n">
         <v>1.2</v>
@@ -7584,7 +7620,7 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB64" t="inlineStr">
@@ -7629,20 +7665,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>07/07/2026 10:40</t>
+          <t>07/08/2026 17:46</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>20349.97</v>
+        <v>19671.02</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>1.75</v>
+        <v>-1.64</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>1.28</v>
+        <v>4.76</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>1.17</v>
+        <v>0.9</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7660,22 +7696,22 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>759</v>
+        <v>977</v>
       </c>
       <c r="U65" s="7" t="n">
-        <v>358.7200000000001</v>
+        <v>-335.83</v>
       </c>
       <c r="V65" t="n">
-        <v>352</v>
+        <v>436</v>
       </c>
       <c r="W65" s="7" t="n">
-        <v>46.3768115942029</v>
+        <v>44.62640736949847</v>
       </c>
       <c r="X65" s="7" t="n">
-        <v>1.17</v>
+        <v>0.9</v>
       </c>
       <c r="Y65" s="7" t="n">
-        <v>1.28</v>
+        <v>4.76</v>
       </c>
       <c r="Z65" t="inlineStr">
         <is>
@@ -7684,7 +7720,7 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB65" t="inlineStr">
@@ -7694,7 +7730,7 @@
       </c>
       <c r="AC65" t="inlineStr">
         <is>
-          <t>T&amp;D19L9 Prop | AUDJPY, T&amp;D19L9 Prop | AUDNZD, T&amp;D19L9 Prop | AUDUSD, T&amp;D19L9 Prop | ETHUSD, T&amp;D19L9 Prop | EURAUD, T&amp;D19L9 Prop | EURCHF, T&amp;D19L9 Prop | EURUSD, T&amp;D19L9 Prop | GBPAUD, T&amp;D19L9 Prop | GBPCHF, T&amp;D19L9 Prop | NZDJPY, T&amp;D19L9 Prop | NZDUSD, T&amp;D19L9 Prop | RUSS2000, T&amp;D19L9 Prop | US30, T&amp;D19L9 Prop | US500, T&amp;D19L9 Prop | USDCHF, T&amp;D19L9 Prop | USTECH, T&amp;D19L9 Prop | XAUUSD</t>
+          <t>T&amp;D19L9 Prop | AUDCAD, T&amp;D19L9 Prop | AUDJPY, T&amp;D19L9 Prop | AUDNZD, T&amp;D19L9 Prop | AUDUSD, T&amp;D19L9 Prop | CADJPY, T&amp;D19L9 Prop | ETHUSD, T&amp;D19L9 Prop | EURAUD, T&amp;D19L9 Prop | EURCHF, T&amp;D19L9 Prop | EURUSD, T&amp;D19L9 Prop | GBPAUD, T&amp;D19L9 Prop | GBPCHF, T&amp;D19L9 Prop | NZDJPY, T&amp;D19L9 Prop | NZDUSD, T&amp;D19L9 Prop | RUSS2000, T&amp;D19L9 Prop | US30, T&amp;D19L9 Prop | US500, T&amp;D19L9 Prop | USDCHF, T&amp;D19L9 Prop | USTECH, T&amp;D19L9 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -7729,20 +7765,20 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>07/07/2026 10:49</t>
+          <t>07/08/2026 17:51</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
-        <v>19724.46</v>
+        <v>19649.21</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>-1.37</v>
+        <v>-1.75</v>
       </c>
       <c r="J66" s="7" t="n">
-        <v>1.88</v>
+        <v>2.28</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>0.46</v>
+        <v>0.41</v>
       </c>
       <c r="L66" t="n">
         <v>20000</v>
@@ -7751,31 +7787,40 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>0</v>
+        <v>-452.04</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="Q66" s="7" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="R66" s="7" t="n">
+        <v>0.08776461566403648</v>
+      </c>
+      <c r="S66" s="7" t="n">
+        <v>2.29</v>
       </c>
       <c r="T66" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="U66" s="7" t="n">
-        <v>-288.53</v>
+        <v>-350.79</v>
       </c>
       <c r="V66" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="W66" s="7" t="n">
-        <v>32.75862068965517</v>
+        <v>30.76923076923077</v>
       </c>
       <c r="X66" s="7" t="n">
-        <v>0.45</v>
+        <v>0.41</v>
       </c>
       <c r="Y66" s="7" t="n">
-        <v>1.95</v>
+        <v>2.29</v>
       </c>
       <c r="Z66" t="inlineStr">
         <is>
@@ -7784,7 +7829,7 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
@@ -7829,20 +7874,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>07/06/2026 20:00</t>
+          <t>07/08/2026 17:57</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20042.15</v>
+        <v>19983.56</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>0.21</v>
+        <v>-0.08</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>0.93</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.09</v>
+        <v>0.97</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7851,28 +7896,37 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>0</v>
+        <v>-8.200000000000005</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q67" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R67" s="7" t="n">
+        <v>0.9852766904873056</v>
+      </c>
+      <c r="S67" s="7" t="n">
+        <v>0.8</v>
       </c>
       <c r="T67" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>62.36000000000001</v>
+        <v>-16.44</v>
       </c>
       <c r="V67" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>50</v>
+        <v>52.27272727272727</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.14</v>
+        <v>0.97</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>0.93</v>
@@ -7884,7 +7938,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7929,7 +7983,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>07/07/2026 11:08</t>
+          <t>07/08/2026 17:59</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8029,7 +8083,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>07/07/2026 11:08</t>
+          <t>07/08/2026 17:59</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8129,7 +8183,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>07/07/2026 11:11</t>
+          <t>07/08/2026 18:01</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8229,7 +8283,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>07/07/2026 11:24</t>
+          <t>07/08/2026 18:08</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8338,7 +8392,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>07/07/2026 06:26</t>
+          <t>07/08/2026 20:46</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8556,20 +8610,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>07/07/2026 07:27</t>
+          <t>07/08/2026 21:12</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>28010.15</v>
+        <v>28215.23</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>-22.43</v>
+        <v>-24.27</v>
       </c>
       <c r="J74" s="7" t="n">
-        <v>29.98</v>
+        <v>32.64</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="L74" t="n">
         <v>25000</v>
@@ -8581,34 +8635,34 @@
         <v>40</v>
       </c>
       <c r="O74" s="7" t="n">
-        <v>-147.93</v>
+        <v>97.25</v>
       </c>
       <c r="P74" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="Q74" s="7" t="n">
-        <v>67.5</v>
+        <v>90</v>
       </c>
       <c r="R74" s="7" t="n">
-        <v>0.642413401339167</v>
+        <v>1.757811891217954</v>
       </c>
       <c r="S74" s="7" t="n">
-        <v>1.56</v>
+        <v>0.5</v>
       </c>
       <c r="T74" t="n">
-        <v>3172</v>
+        <v>3178</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>-6271.849999999999</v>
+        <v>-6066.77</v>
       </c>
       <c r="V74" t="n">
-        <v>1876</v>
+        <v>1910</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>59.14249684741488</v>
+        <v>60.10069225928257</v>
       </c>
       <c r="X74" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="Y74" s="7" t="n">
         <v>32.64</v>
@@ -8620,7 +8674,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8756,7 +8810,7 @@
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>07/05/2026 00:17</t>
+          <t>07/08/2026 11:16</t>
         </is>
       </c>
       <c r="H76" s="9" t="n">
@@ -8847,7 +8901,7 @@
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>07/05/2026 12:08</t>
+          <t>07/08/2026 14:05</t>
         </is>
       </c>
       <c r="H77" s="9" t="n">
@@ -9211,7 +9265,7 @@
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>07/06/2026 18:01</t>
+          <t>07/08/2026 17:36</t>
         </is>
       </c>
       <c r="H81" s="9" t="n">
@@ -9393,7 +9447,7 @@
       </c>
       <c r="G83" s="8" t="inlineStr">
         <is>
-          <t>07/04/2026 15:33</t>
+          <t>07/08/2026 08:33</t>
         </is>
       </c>
       <c r="H83" s="9" t="n">
@@ -9484,20 +9538,20 @@
       </c>
       <c r="G84" s="8" t="inlineStr">
         <is>
-          <t>07/07/2026 10:24</t>
+          <t>07/08/2026 17:35</t>
         </is>
       </c>
       <c r="H84" s="9" t="n">
-        <v>19929.61</v>
+        <v>19666.43</v>
       </c>
       <c r="I84" s="9" t="n">
-        <v>-0.36</v>
+        <v>-1.67</v>
       </c>
       <c r="J84" s="9" t="n">
-        <v>0.82</v>
+        <v>1.7</v>
       </c>
       <c r="K84" s="9" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.32</v>
       </c>
       <c r="L84" s="8" t="n">
         <v>20000</v>
@@ -9506,17 +9560,23 @@
         <v>0</v>
       </c>
       <c r="N84" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O84" s="9" t="n">
-        <v>0</v>
+        <v>-273.89</v>
       </c>
       <c r="P84" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="Q84" s="8" t="n"/>
-      <c r="R84" s="8" t="n"/>
-      <c r="S84" s="8" t="n"/>
+      <c r="Q84" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R84" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S84" s="9" t="n">
+        <v>1.37</v>
+      </c>
       <c r="T84" s="8" t="n">
         <v>0</v>
       </c>
@@ -9569,20 +9629,20 @@
       </c>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t>07/07/2026 09:45</t>
+          <t>07/08/2026 17:16</t>
         </is>
       </c>
       <c r="H85" s="9" t="n">
-        <v>19647.04</v>
+        <v>19609.46</v>
       </c>
       <c r="I85" s="9" t="n">
-        <v>-1.75</v>
+        <v>-1.95</v>
       </c>
       <c r="J85" s="9" t="n">
-        <v>1.82</v>
+        <v>2.27</v>
       </c>
       <c r="K85" s="9" t="n">
-        <v>0.41</v>
+        <v>0.45</v>
       </c>
       <c r="L85" s="8" t="n">
         <v>20000</v>
@@ -9591,17 +9651,23 @@
         <v>0</v>
       </c>
       <c r="N85" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O85" s="9" t="n">
-        <v>0</v>
+        <v>-190.78</v>
       </c>
       <c r="P85" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q85" s="8" t="n"/>
-      <c r="R85" s="8" t="n"/>
-      <c r="S85" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q85" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R85" s="9" t="n">
+        <v>0.4489153355094023</v>
+      </c>
+      <c r="S85" s="9" t="n">
+        <v>1.44</v>
+      </c>
       <c r="T85" s="8" t="n">
         <v>0</v>
       </c>
@@ -9654,14 +9720,14 @@
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>07/07/2026 10:13</t>
+          <t>07/08/2026 17:30</t>
         </is>
       </c>
       <c r="H86" s="9" t="n">
-        <v>22128.27</v>
+        <v>22515.12</v>
       </c>
       <c r="I86" s="9" t="n">
-        <v>10.65</v>
+        <v>12.58</v>
       </c>
       <c r="J86" s="9" t="n">
         <v>5.86</v>
@@ -9739,7 +9805,7 @@
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>07/06/2026 17:28</t>
+          <t>07/08/2026 17:23</t>
         </is>
       </c>
       <c r="H87" s="9" t="n">
@@ -9824,7 +9890,7 @@
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>07/07/2026 11:08</t>
+          <t>07/08/2026 18:00</t>
         </is>
       </c>
       <c r="H88" s="9" t="n">
@@ -10398,7 +10464,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>07/05/2026 00:17</t>
+          <t>07/08/2026 11:16</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -10439,7 +10505,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>07/05/2026 12:08</t>
+          <t>07/08/2026 14:05</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -10603,7 +10669,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>07/06/2026 18:01</t>
+          <t>07/08/2026 17:36</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -10685,7 +10751,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>07/04/2026 15:33</t>
+          <t>07/08/2026 08:33</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -10726,17 +10792,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>07/07/2026 10:24</t>
+          <t>07/08/2026 17:35</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>19929.61</v>
+        <v>19666.43</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>-0.36</v>
+        <v>-1.67</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15">
@@ -10767,17 +10833,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>07/07/2026 09:45</t>
+          <t>07/08/2026 17:16</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>19647.04</v>
+        <v>19609.46</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>-1.75</v>
+        <v>-1.95</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
@@ -10808,14 +10874,14 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>07/07/2026 10:13</t>
+          <t>07/08/2026 17:30</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>22128.27</v>
+        <v>22515.12</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>10.65</v>
+        <v>12.58</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -10849,7 +10915,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>07/06/2026 17:28</t>
+          <t>07/08/2026 17:23</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -10890,7 +10956,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>07/07/2026 11:08</t>
+          <t>07/08/2026 18:00</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -12064,7 +12130,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07/05/2026 16:07</t>
+          <t>07/08/2026 16:09</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -12087,7 +12153,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>07/05/2026 06:09</t>
+          <t>07/08/2026 12:47</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -12133,7 +12199,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07/05/2026 13:40</t>
+          <t>07/08/2026 14:42</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
@@ -12294,7 +12360,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>07/05/2026 06:17</t>
+          <t>07/08/2026 12:48</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -12317,7 +12383,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>07/05/2026 05:32</t>
+          <t>07/08/2026 12:40</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -12363,7 +12429,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07/02/2026 15:32</t>
+          <t>07/08/2026 15:57</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
@@ -12386,11 +12452,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07/07/2026 03:55</t>
+          <t>07/08/2026 19:43</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>20006.27</v>
+        <v>20015.51</v>
       </c>
     </row>
     <row r="22">
@@ -12432,11 +12498,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07/07/2026 10:25</t>
+          <t>07/08/2026 17:36</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20291.96</v>
+        <v>20072.25</v>
       </c>
     </row>
     <row r="24">
@@ -12478,11 +12544,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07/06/2026 20:04</t>
+          <t>07/08/2026 17:58</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>20144.14</v>
+        <v>19956.58</v>
       </c>
     </row>
     <row r="26">
@@ -12524,7 +12590,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07/06/2026 20:10</t>
+          <t>07/08/2026 18:02</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -12547,11 +12613,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07/07/2026 05:16</t>
+          <t>07/08/2026 20:15</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
-        <v>19930.65</v>
+        <v>19937.43</v>
       </c>
     </row>
     <row r="29">
@@ -12570,11 +12636,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07/07/2026 05:25</t>
+          <t>07/08/2026 20:18</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>19743.93</v>
+        <v>19598.28</v>
       </c>
     </row>
     <row r="30">
@@ -12593,11 +12659,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07/07/2026 05:30</t>
+          <t>07/08/2026 20:20</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>19777.41</v>
+        <v>19670.74</v>
       </c>
     </row>
     <row r="31">
@@ -12616,11 +12682,11 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07/07/2026 05:16</t>
+          <t>07/08/2026 20:17</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>20170.37</v>
+        <v>20063.67</v>
       </c>
     </row>
     <row r="32">
@@ -12639,11 +12705,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07/07/2026 05:20</t>
+          <t>07/08/2026 20:18</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>19928.56</v>
+        <v>19934.89</v>
       </c>
     </row>
     <row r="33">
@@ -12662,11 +12728,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>07/07/2026 11:25</t>
+          <t>07/08/2026 18:10</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>19968.12</v>
+        <v>19975.11</v>
       </c>
     </row>
     <row r="34">
@@ -12708,11 +12774,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>07/06/2026 20:14</t>
+          <t>07/08/2026 18:03</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>19939.97</v>
+        <v>19930.83</v>
       </c>
     </row>
     <row r="36">
@@ -12731,11 +12797,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>07/06/2026 20:14</t>
+          <t>07/08/2026 18:03</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>20023.3</v>
+        <v>19900.77</v>
       </c>
     </row>
     <row r="37">
@@ -12754,11 +12820,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>07/06/2026 20:16</t>
+          <t>07/08/2026 18:05</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>20414.41</v>
+        <v>20530.6</v>
       </c>
     </row>
     <row r="38">
@@ -12777,11 +12843,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>07/07/2026 11:17</t>
+          <t>07/08/2026 18:04</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>20160.17</v>
+        <v>19900.11</v>
       </c>
     </row>
     <row r="39">
@@ -12800,11 +12866,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>07/07/2026 11:19</t>
+          <t>07/08/2026 18:05</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>19831.83</v>
+        <v>20165.38</v>
       </c>
     </row>
     <row r="40">
@@ -12823,11 +12889,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>07/07/2026 11:22</t>
+          <t>07/08/2026 18:07</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>20089.97</v>
+        <v>19896.88</v>
       </c>
     </row>
     <row r="41">
@@ -12846,11 +12912,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>07/07/2026 11:22</t>
+          <t>07/08/2026 18:07</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>21664.59</v>
+        <v>22101.59</v>
       </c>
     </row>
     <row r="42">
@@ -12869,11 +12935,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>07/07/2026 11:25</t>
+          <t>07/08/2026 18:09</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>20296.44</v>
+        <v>19519.04</v>
       </c>
     </row>
     <row r="43">
@@ -12892,11 +12958,11 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>07/07/2026 11:20</t>
+          <t>07/08/2026 18:06</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>19570.21</v>
+        <v>20424.69</v>
       </c>
     </row>
     <row r="44">
@@ -12915,11 +12981,11 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>07/07/2026 11:22</t>
+          <t>07/08/2026 18:07</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>20084.47</v>
+        <v>19893.06</v>
       </c>
     </row>
     <row r="45">
@@ -13030,7 +13096,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>07/07/2026 03:42</t>
+          <t>07/08/2026 04:25</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-07-09
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-07-08 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-07-09 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>07/08/2026 21:47</t>
+          <t>07/09/2026 17:37</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>49384.91</v>
+        <v>50903.61</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>129.72</v>
+        <v>136.78</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>2067.01</v>
+        <v>4318.99</v>
       </c>
       <c r="P2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>60</v>
+        <v>67.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>2.155554685927682</v>
+        <v>5.483116910077954</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>3.15</v>
+        <v>2.93</v>
       </c>
       <c r="T2" t="n">
-        <v>3071</v>
+        <v>3079</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>24384.91</v>
+        <v>25915.52999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>1930</v>
+        <v>1940</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>62.84597850862911</v>
+        <v>63.0074699577785</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>07/08/2026 18:59</t>
+          <t>07/09/2026 20:27</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>07/08/2026 20:16</t>
+          <t>07/09/2026 22:12</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>07/06/2026 17:39</t>
+          <t>07/09/2026 17:41</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>07/06/2026 20:08</t>
+          <t>07/09/2026 20:10</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>07/06/2026 19:52</t>
+          <t>07/09/2026 19:57</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>07/08/2026 17:24</t>
+          <t>07/09/2026 18:18</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>07/05/2026 23:55</t>
+          <t>07/08/2026 23:58</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,14 +2377,14 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>07/06/2026 20:58</t>
+          <t>07/09/2026 19:36</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>19487.43</v>
+        <v>19470.66</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-7.62</v>
+        <v>-7.7</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.75</v>
@@ -2402,22 +2402,22 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>5175.22</v>
+        <v>5077.88</v>
       </c>
       <c r="P15" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>45</v>
+        <v>42.5</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>1.716831173004524</v>
+        <v>1.692129869421803</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>20.06</v>
+        <v>20.18</v>
       </c>
       <c r="T15" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U15" s="7" t="n">
         <v>-1208.299999999999</v>
@@ -2426,7 +2426,7 @@
         <v>89</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>53.6144578313253</v>
+        <v>53.2934131736527</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>0.8</v>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2486,17 +2486,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>07/08/2026 20:31</t>
+          <t>07/09/2026 16:30</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>110.31</v>
+        <v>106.79</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-99.45999999999999</v>
+        <v>-99.48</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>99.45999999999999</v>
+        <v>99.48</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>0.7</v>
@@ -2511,37 +2511,37 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-4.699999999999999</v>
+        <v>-5.93</v>
       </c>
       <c r="P16" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>27.5</v>
+        <v>30</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.6373456790123457</v>
+        <v>0.5213882163034705</v>
       </c>
       <c r="S16" s="7" t="n">
         <v>0.03</v>
       </c>
       <c r="T16" t="n">
-        <v>1990</v>
+        <v>2010</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-20312.09</v>
+        <v>-20316.54</v>
       </c>
       <c r="V16" t="n">
-        <v>646</v>
+        <v>651</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>32.46231155778894</v>
+        <v>32.38805970149254</v>
       </c>
       <c r="X16" s="7" t="n">
         <v>0.7</v>
       </c>
       <c r="Y16" s="7" t="n">
-        <v>99.47</v>
+        <v>99.48</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>07/08/2026 19:55</t>
+          <t>07/09/2026 21:46</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>07/08/2026 17:33</t>
+          <t>07/09/2026 18:30</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>07/08/2026 17:32</t>
+          <t>07/09/2026 13:21</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>07/08/2026 16:02</t>
+          <t>07/09/2026 16:36</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,14 +3140,14 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>07/07/2026 10:48</t>
+          <t>07/09/2026 18:54</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>18302.99</v>
+        <v>18276.86</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-8.51</v>
+        <v>-8.640000000000001</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>18.8</v>
@@ -3162,34 +3162,34 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>18416.29</v>
+        <v>18390.16</v>
       </c>
       <c r="P22" t="n">
         <v>6</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>31.57894736842105</v>
+        <v>30</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>3.725883944535885</v>
+        <v>3.711529132834282</v>
       </c>
       <c r="S22" s="7" t="n">
         <v>9.119999999999999</v>
       </c>
       <c r="T22" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-1697.01</v>
+        <v>-1723.14</v>
       </c>
       <c r="V22" t="n">
         <v>5</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>27.77777777777778</v>
+        <v>26.31578947368421</v>
       </c>
       <c r="X22" s="7" t="n">
         <v>0.75</v>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>07/08/2026 17:21</t>
+          <t>07/09/2026 18:12</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3289,7 +3289,7 @@
         <v>4.05</v>
       </c>
       <c r="T23" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="U23" s="7" t="n">
         <v>-443.9199999999998</v>
@@ -3298,7 +3298,7 @@
         <v>31</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>50.81967213114754</v>
+        <v>49.2063492063492</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>0.86</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3467,20 +3467,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>07/08/2026 17:31</t>
+          <t>07/09/2026 18:30</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16101.91</v>
+        <v>16191.96</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-19.23</v>
+        <v>-18.78</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.54</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3492,34 +3492,34 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>28.23</v>
+        <v>100.36</v>
       </c>
       <c r="P25" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>45</v>
+        <v>47.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.068262604280015</v>
+        <v>1.273520113376213</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.7</v>
+        <v>0.99</v>
       </c>
       <c r="T25" t="n">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3898.09</v>
+        <v>-3808.04</v>
       </c>
       <c r="V25" t="n">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>36.12334801762114</v>
+        <v>36.76148796498906</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>20.79</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>07/08/2026 20:51</t>
+          <t>07/09/2026 16:47</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>22399.12</v>
+        <v>21794.32</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>12.37</v>
-      </c>
-      <c r="J26" t="n">
-        <v>2</v>
+        <v>9.01</v>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>4.28</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>2.82</v>
+        <v>1.7</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,37 +3601,37 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>80.77</v>
+        <v>-156.96</v>
       </c>
       <c r="P26" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>113.1805555555556</v>
+        <v>0.387066541705717</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>0</v>
+        <v>1.27</v>
       </c>
       <c r="T26" t="n">
-        <v>775</v>
+        <v>1147</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>2318.61</v>
+        <v>1724.24</v>
       </c>
       <c r="V26" t="n">
-        <v>508</v>
+        <v>757</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>65.54838709677419</v>
+        <v>65.99825632083697</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>2.61</v>
+        <v>1.65</v>
       </c>
       <c r="Y26" s="7" t="n">
-        <v>2</v>
+        <v>4.27</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>T&amp;Dv5 Prop Bots | AUDJPY, T&amp;Dv5 Prop Bots | AUDJPY.pro, T&amp;Dv5 Prop Bots | CADJPY.pro, T&amp;Dv5 Prop Bots | EURJPY.pro, T&amp;Dv5 Prop Bots | EURUSD, T&amp;Dv5 Prop Bots | EURUSD.pro, T&amp;Dv5 Prop Bots | GBPJPY, T&amp;Dv5 Prop Bots | GBPJPY.pro, T&amp;Dv5 Prop Bots | GBPUSD.pro, T&amp;Dv5 Prop Bots | USDJPY, T&amp;Dv5 Prop Bots | USDJPY.pro</t>
+          <t>T&amp;Dv5 Prop Bots | AUDJPY, T&amp;Dv5 Prop Bots | AUDJPY.pro, T&amp;Dv5 Prop Bots | CADJPY.pro, T&amp;Dv5 Prop Bots | EURJPY.pro, T&amp;Dv5 Prop Bots | EURUSD, T&amp;Dv5 Prop Bots | EURUSD.pro, T&amp;Dv5 Prop Bots | GBPJPY, T&amp;Dv5 Prop Bots | GBPJPY.pro, T&amp;Dv5 Prop Bots | GBPUSD, T&amp;Dv5 Prop Bots | GBPUSD.pro, T&amp;Dv5 Prop Bots | USDJPY, T&amp;Dv5 Prop Bots | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -3685,14 +3685,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>07/08/2026 17:33</t>
+          <t>07/09/2026 18:30</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20279.19</v>
+        <v>20281.5</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-3.03</v>
+        <v>-3.02</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>5.35</v>
@@ -3710,31 +3710,31 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-742.9699999999999</v>
+        <v>-631.7399999999999</v>
       </c>
       <c r="P27" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>35</v>
+        <v>37.5</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.6649152557661259</v>
+        <v>0.7003614217820655</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>5.42</v>
+        <v>5.39</v>
       </c>
       <c r="T27" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>279.1900000000001</v>
+        <v>281.5</v>
       </c>
       <c r="V27" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>40.84507042253522</v>
+        <v>41.66666666666667</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>1.09</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>07/06/2026 14:41</t>
+          <t>07/09/2026 14:44</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,14 +3903,14 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>07/08/2026 17:36</t>
+          <t>07/09/2026 18:34</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20356.7</v>
+        <v>20353.8</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
@@ -3928,31 +3928,31 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-19.62999999999997</v>
+        <v>60.75000000000002</v>
       </c>
       <c r="P29" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>52.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.9853058963552933</v>
+        <v>1.048960742752601</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>6.08</v>
+        <v>5.6</v>
       </c>
       <c r="T29" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>356.6199999999999</v>
+        <v>353.7999999999999</v>
       </c>
       <c r="V29" t="n">
         <v>44</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>57.14285714285714</v>
+        <v>55.69620253164557</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>1.2</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4121,20 +4121,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>07/08/2026 17:45</t>
+          <t>07/09/2026 18:44</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20802.54</v>
+        <v>20791.95</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>4.02</v>
+        <v>3.97</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>1.09</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>2.61</v>
+        <v>2.55</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -4146,7 +4146,7 @@
         <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>803.02</v>
+        <v>798.71</v>
       </c>
       <c r="P31" t="n">
         <v>13</v>
@@ -4155,25 +4155,25 @@
         <v>32.5</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>2.799484593837535</v>
+        <v>2.772705078125</v>
       </c>
       <c r="S31" s="7" t="n">
         <v>1.09</v>
       </c>
       <c r="T31" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>802.54</v>
+        <v>791.95</v>
       </c>
       <c r="V31" t="n">
         <v>14</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>28.57142857142857</v>
+        <v>27.45098039215686</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>2.61</v>
+        <v>2.55</v>
       </c>
       <c r="Y31" s="7" t="n">
         <v>1.1</v>
@@ -4185,7 +4185,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>07/08/2026 17:33</t>
+          <t>07/09/2026 18:30</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>07/08/2026 17:53</t>
+          <t>07/09/2026 18:56</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>07/08/2026 15:20</t>
+          <t>07/09/2026 15:50</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20305.8</v>
+        <v>20104.68</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>1.54</v>
+        <v>0.53</v>
       </c>
       <c r="J34" s="7" t="n">
-        <v>2.22</v>
+        <v>2.62</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.27</v>
+        <v>1.08</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,37 +4473,37 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-141.48</v>
+        <v>-555.11</v>
       </c>
       <c r="P34" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.8621482578533012</v>
+        <v>0.5477497881770188</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>2.33</v>
+        <v>2.78</v>
       </c>
       <c r="T34" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>204.55</v>
+        <v>104.68</v>
       </c>
       <c r="V34" t="n">
         <v>26</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>46.42857142857143</v>
+        <v>44.82758620689656</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1.16</v>
+        <v>1.08</v>
       </c>
       <c r="Y34" s="7" t="n">
-        <v>2.23</v>
+        <v>2.64</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4557,14 +4557,14 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>07/08/2026 18:48</t>
+          <t>07/09/2026 20:17</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>14219.4</v>
+        <v>14229.07</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>-28.92</v>
+        <v>-28.87</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>41.42</v>
@@ -4582,19 +4582,19 @@
         <v>40</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>322.1900000000001</v>
+        <v>9.329999999999984</v>
       </c>
       <c r="P35" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="Q35" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>50</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>1.253469381332998</v>
+        <v>1.006560812331233</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>1.75</v>
+        <v>2.41</v>
       </c>
       <c r="T35" t="n">
         <v>1618</v>
@@ -4706,7 +4706,7 @@
         <v>0.74</v>
       </c>
       <c r="T36" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="U36" s="7" t="n">
         <v>1039.71</v>
@@ -4715,7 +4715,7 @@
         <v>27</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>61.36363636363637</v>
+        <v>60</v>
       </c>
       <c r="X36" s="7" t="n">
         <v>1.6</v>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>07/08/2026 18:25</t>
+          <t>07/09/2026 19:51</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>07/08/2026 19:22</t>
+          <t>07/09/2026 15:26</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4993,20 +4993,20 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>07/08/2026 19:09</t>
+          <t>07/09/2026 20:39</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
         <v>19937.02</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>-0.02</v>
+        <v>-0.3</v>
       </c>
       <c r="J39" s="7" t="n">
         <v>4.02</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>0.99</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L39" t="n">
         <v>20000</v>
@@ -5015,19 +5015,19 @@
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O39" s="7" t="n">
-        <v>19981.75</v>
+        <v>19925.63</v>
       </c>
       <c r="P39" t="n">
         <v>7</v>
       </c>
       <c r="Q39" s="7" t="n">
-        <v>46.66666666666666</v>
+        <v>43.75</v>
       </c>
       <c r="R39" s="7" t="n">
-        <v>21.62760016104223</v>
+        <v>20.44324313775236</v>
       </c>
       <c r="S39" s="7" t="n">
         <v>2.05</v>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>07/08/2026 20:42</t>
+          <t>07/09/2026 16:39</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>07/08/2026 21:29</t>
+          <t>07/09/2026 17:23</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5320,14 +5320,14 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>07/08/2026 17:22</t>
+          <t>07/09/2026 18:12</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
-        <v>19432.74</v>
+        <v>19418.9</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>-2.83</v>
+        <v>-2.9</v>
       </c>
       <c r="J42" s="7" t="n">
         <v>4.17</v>
@@ -5345,31 +5345,31 @@
         <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-43.01</v>
+        <v>-16.19</v>
       </c>
       <c r="P42" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="Q42" s="7" t="n">
-        <v>42.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>0.503119223659889</v>
+        <v>0.7454002201604025</v>
       </c>
       <c r="S42" s="7" t="n">
-        <v>0.28</v>
+        <v>0.23</v>
       </c>
       <c r="T42" t="n">
-        <v>1220</v>
+        <v>1281</v>
       </c>
       <c r="U42" s="7" t="n">
-        <v>-566.86</v>
+        <v>-590.9000000000001</v>
       </c>
       <c r="V42" t="n">
-        <v>558</v>
+        <v>589</v>
       </c>
       <c r="W42" s="7" t="n">
-        <v>45.73770491803278</v>
+        <v>45.97970335675254</v>
       </c>
       <c r="X42" s="7" t="n">
         <v>0.79</v>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
@@ -5429,20 +5429,20 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>07/08/2026 17:26</t>
+          <t>07/09/2026 18:18</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
-        <v>18235.59</v>
+        <v>18253.36</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>-8.81</v>
+        <v>-8.720000000000001</v>
       </c>
       <c r="J43" s="7" t="n">
         <v>9.66</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="L43" t="n">
         <v>20000</v>
@@ -5451,34 +5451,25 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>16.32</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>1.851330203442879</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>2457</v>
+        <v>2536</v>
       </c>
       <c r="U43" s="7" t="n">
-        <v>-1765.39</v>
+        <v>-1756.57</v>
       </c>
       <c r="V43" t="n">
-        <v>1068</v>
+        <v>1111</v>
       </c>
       <c r="W43" s="7" t="n">
-        <v>43.46764346764347</v>
+        <v>43.80914826498422</v>
       </c>
       <c r="X43" s="7" t="n">
         <v>0.66</v>
@@ -5493,7 +5484,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
@@ -5538,20 +5529,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>07/08/2026 17:27</t>
+          <t>07/09/2026 18:22</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>20047.44</v>
+        <v>20145.27</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>0.23</v>
+        <v>0.72</v>
       </c>
       <c r="J44" s="7" t="n">
-        <v>2.13</v>
+        <v>2.24</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>1.06</v>
+        <v>1.16</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5560,40 +5551,31 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>19956.84</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" t="n">
+        <v>29</v>
+      </c>
+      <c r="U44" s="7" t="n">
+        <v>145.2700000000001</v>
+      </c>
+      <c r="V44" t="n">
         <v>13</v>
       </c>
-      <c r="Q44" s="7" t="n">
-        <v>46.42857142857143</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>22.94144357099665</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="T44" t="n">
-        <v>27</v>
-      </c>
-      <c r="U44" s="7" t="n">
-        <v>47.44000000000005</v>
-      </c>
-      <c r="V44" t="n">
-        <v>12</v>
-      </c>
       <c r="W44" s="7" t="n">
-        <v>44.44444444444444</v>
+        <v>44.82758620689656</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>1.06</v>
+        <v>1.16</v>
       </c>
       <c r="Y44" s="7" t="n">
-        <v>2.12</v>
+        <v>2.23</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -5602,12 +5584,12 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC44" t="inlineStr">
@@ -5647,20 +5629,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>07/08/2026 17:23</t>
+          <t>07/09/2026 18:14</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19841.05</v>
+        <v>19852.41</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.79</v>
+        <v>-0.74</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>1.6</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5681,16 +5663,16 @@
         <v>176</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-158.95</v>
+        <v>-147.59</v>
       </c>
       <c r="V45" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>47.72727272727273</v>
+        <v>51.70454545454546</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y45" s="7" t="n">
         <v>1.59</v>
@@ -5702,7 +5684,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5747,7 +5729,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>07/08/2026 17:23</t>
+          <t>07/09/2026 13:06</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5847,20 +5829,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>07/07/2026 10:11</t>
+          <t>07/09/2026 18:27</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>18609.72</v>
+        <v>18570.19</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-6.94</v>
+        <v>-7.15</v>
       </c>
       <c r="J47" s="7" t="n">
-        <v>7.01</v>
+        <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5947,7 +5929,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>07/08/2026 17:30</t>
+          <t>07/09/2026 18:26</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6047,20 +6029,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>07/08/2026 17:42</t>
+          <t>07/09/2026 18:43</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>19797.3</v>
+        <v>19825.59</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>-1.03</v>
+        <v>-0.89</v>
       </c>
       <c r="J49" s="7" t="n">
         <v>2.74</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="L49" t="n">
         <v>20000</v>
@@ -6078,19 +6060,19 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="U49" s="7" t="n">
-        <v>-202.7</v>
+        <v>-174.4100000000001</v>
       </c>
       <c r="V49" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="W49" s="7" t="n">
-        <v>40.5940594059406</v>
+        <v>41.50943396226415</v>
       </c>
       <c r="X49" s="7" t="n">
-        <v>0.88</v>
+        <v>0.9</v>
       </c>
       <c r="Y49" s="7" t="n">
         <v>2.72</v>
@@ -6102,7 +6084,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
@@ -6147,20 +6129,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>07/08/2026 17:37</t>
+          <t>07/09/2026 18:34</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>22062.68</v>
+        <v>21975.19</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>10.34</v>
+        <v>9.9</v>
       </c>
       <c r="J50" s="7" t="n">
         <v>3.34</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>1.43</v>
+        <v>1.39</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6178,19 +6160,19 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>579</v>
+        <v>603</v>
       </c>
       <c r="U50" s="7" t="n">
-        <v>2062.68</v>
+        <v>1975.19</v>
       </c>
       <c r="V50" t="n">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="W50" s="7" t="n">
-        <v>52.50431778929189</v>
+        <v>52.23880597014925</v>
       </c>
       <c r="X50" s="7" t="n">
-        <v>1.43</v>
+        <v>1.39</v>
       </c>
       <c r="Y50" s="7" t="n">
         <v>3.34</v>
@@ -6202,7 +6184,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
@@ -6247,20 +6229,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>07/08/2026 17:34</t>
+          <t>07/09/2026 18:31</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>24805.28</v>
+        <v>24546.75</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>24.02</v>
+        <v>22.73</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>5.53</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>1.54</v>
+        <v>1.49</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6278,19 +6260,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>1002</v>
+        <v>1038</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>4805.280000000001</v>
+        <v>4546.75</v>
       </c>
       <c r="V51" t="n">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>53.69261477045908</v>
+        <v>52.89017341040463</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>1.54</v>
+        <v>1.49</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>5.53</v>
@@ -6302,7 +6284,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6347,7 +6329,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>07/08/2026 17:19</t>
+          <t>07/09/2026 18:09</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6447,20 +6429,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>07/08/2026 17:44</t>
+          <t>07/09/2026 18:46</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19743.76</v>
+        <v>19745.1</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.3</v>
+        <v>-1.29</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.39</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6469,37 +6451,28 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>-78.94</v>
+        <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q53" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="R53" s="7" t="n">
-        <v>0.4557738710789382</v>
-      </c>
-      <c r="S53" s="7" t="n">
-        <v>0.49</v>
+        <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-256.2400000000001</v>
+        <v>-254.9</v>
       </c>
       <c r="V53" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>37.2093023255814</v>
+        <v>37.36263736263736</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.37</v>
@@ -6511,7 +6484,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6556,11 +6529,11 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>07/08/2026 17:50</t>
+          <t>07/09/2026 18:53</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
-        <v>19664.2</v>
+        <v>19664.26</v>
       </c>
       <c r="I54" s="7" t="n">
         <v>-1.67</v>
@@ -6587,16 +6560,16 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="U54" s="7" t="n">
-        <v>-335.8</v>
+        <v>-335.7400000000001</v>
       </c>
       <c r="V54" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="W54" s="7" t="n">
-        <v>38.23529411764706</v>
+        <v>38.84892086330935</v>
       </c>
       <c r="X54" s="7" t="n">
         <v>0.79</v>
@@ -6611,7 +6584,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -6656,20 +6629,20 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>07/08/2026 17:39</t>
+          <t>07/09/2026 18:37</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
-        <v>19979.85</v>
+        <v>19918.2</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>-0.09</v>
+        <v>-0.39</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>0.8</v>
+        <v>1.15</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>0.99</v>
+        <v>0.95</v>
       </c>
       <c r="L55" t="n">
         <v>20000</v>
@@ -6687,22 +6660,22 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>630</v>
+        <v>669</v>
       </c>
       <c r="U55" s="7" t="n">
-        <v>-20.15000000000003</v>
+        <v>-81.8</v>
       </c>
       <c r="V55" t="n">
-        <v>311</v>
+        <v>325</v>
       </c>
       <c r="W55" s="7" t="n">
-        <v>49.36507936507937</v>
+        <v>48.57997010463378</v>
       </c>
       <c r="X55" s="7" t="n">
-        <v>0.99</v>
+        <v>0.95</v>
       </c>
       <c r="Y55" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.16</v>
       </c>
       <c r="Z55" t="inlineStr">
         <is>
@@ -6711,7 +6684,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -6756,20 +6729,20 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>07/08/2026 17:48</t>
+          <t>07/09/2026 13:48</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
-        <v>19821.18</v>
+        <v>19765.95</v>
       </c>
       <c r="I56" s="7" t="n">
-        <v>-0.91</v>
+        <v>-1.19</v>
       </c>
       <c r="J56" s="7" t="n">
-        <v>1.07</v>
+        <v>1.31</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="L56" t="n">
         <v>20000</v>
@@ -6787,22 +6760,22 @@
         <v>0</v>
       </c>
       <c r="T56" t="n">
-        <v>528</v>
+        <v>565</v>
       </c>
       <c r="U56" s="7" t="n">
-        <v>-178.82</v>
+        <v>-193.84</v>
       </c>
       <c r="V56" t="n">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="W56" s="7" t="n">
-        <v>46.78030303030303</v>
+        <v>46.54867256637168</v>
       </c>
       <c r="X56" s="7" t="n">
         <v>0.88</v>
       </c>
       <c r="Y56" s="7" t="n">
-        <v>1.05</v>
+        <v>1.29</v>
       </c>
       <c r="Z56" t="inlineStr">
         <is>
@@ -6811,7 +6784,7 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr">
@@ -6856,20 +6829,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>07/08/2026 17:23</t>
+          <t>07/09/2026 18:19</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19786.88</v>
+        <v>19792.22</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.06</v>
+        <v>-1.03</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6878,37 +6851,28 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>168.15</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q57" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R57" s="7" t="n">
-        <v>8.349213286713287</v>
-      </c>
-      <c r="S57" s="7" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-213.1200000000001</v>
+        <v>-207.78</v>
       </c>
       <c r="V57" t="n">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.23040380047506</v>
+        <v>43.61948955916473</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6920,7 +6884,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6965,20 +6929,20 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>07/08/2026 17:41</t>
+          <t>07/09/2026 18:40</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
-        <v>18297.67</v>
+        <v>18240.71</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>-8.52</v>
+        <v>-8.81</v>
       </c>
       <c r="J58" s="7" t="n">
-        <v>8.52</v>
+        <v>9.16</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="L58" t="n">
         <v>20000</v>
@@ -6996,22 +6960,22 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1706</v>
+        <v>1838</v>
       </c>
       <c r="U58" s="7" t="n">
-        <v>-1698.01</v>
+        <v>-1759.29</v>
       </c>
       <c r="V58" t="n">
-        <v>739</v>
+        <v>792</v>
       </c>
       <c r="W58" s="7" t="n">
-        <v>43.31770222743259</v>
+        <v>43.09031556039173</v>
       </c>
       <c r="X58" s="7" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="Y58" s="7" t="n">
-        <v>8.529999999999999</v>
+        <v>9.15</v>
       </c>
       <c r="Z58" t="inlineStr">
         <is>
@@ -7020,7 +6984,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB58" t="inlineStr">
@@ -7065,20 +7029,20 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>07/08/2026 17:48</t>
+          <t>07/09/2026 18:51</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
-        <v>19928.18</v>
+        <v>19964.57</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>-0.35</v>
+        <v>-0.17</v>
       </c>
       <c r="J59" s="7" t="n">
         <v>0.55</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>0.66</v>
+        <v>0.84</v>
       </c>
       <c r="L59" t="n">
         <v>20000</v>
@@ -7096,19 +7060,19 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="U59" s="7" t="n">
-        <v>-71.82000000000002</v>
+        <v>-35.43000000000001</v>
       </c>
       <c r="V59" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="W59" s="7" t="n">
-        <v>41.66666666666667</v>
+        <v>42.2680412371134</v>
       </c>
       <c r="X59" s="7" t="n">
-        <v>0.66</v>
+        <v>0.84</v>
       </c>
       <c r="Y59" s="7" t="n">
         <v>0.55</v>
@@ -7120,7 +7084,7 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -7165,20 +7129,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>07/08/2026 17:45</t>
+          <t>07/09/2026 18:44</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>18999.46</v>
+        <v>18810.48</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-5.01</v>
+        <v>-5.96</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>12.98</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="L60" t="n">
         <v>20000</v>
@@ -7196,19 +7160,19 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>2669</v>
+        <v>2854</v>
       </c>
       <c r="U60" s="7" t="n">
-        <v>-1000.53</v>
+        <v>-1189.52</v>
       </c>
       <c r="V60" t="n">
-        <v>1243</v>
+        <v>1319</v>
       </c>
       <c r="W60" s="7" t="n">
-        <v>46.57174971899588</v>
+        <v>46.21583742116328</v>
       </c>
       <c r="X60" s="7" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="Y60" s="7" t="n">
         <v>12.97</v>
@@ -7220,7 +7184,7 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
@@ -7265,20 +7229,20 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>07/08/2026 17:43</t>
+          <t>07/09/2026 18:43</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>19655.14</v>
+        <v>19680.32</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-1.72</v>
+        <v>-1.6</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>6.82</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="L61" t="n">
         <v>20000</v>
@@ -7296,19 +7260,19 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>1605</v>
+        <v>1712</v>
       </c>
       <c r="U61" s="7" t="n">
-        <v>-344.8100000000002</v>
+        <v>-319.6799999999997</v>
       </c>
       <c r="V61" t="n">
-        <v>738</v>
+        <v>784</v>
       </c>
       <c r="W61" s="7" t="n">
-        <v>45.98130841121495</v>
+        <v>45.79439252336449</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="Y61" s="7" t="n">
         <v>6.81</v>
@@ -7320,7 +7284,7 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
@@ -7365,20 +7329,20 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>07/08/2026 17:57</t>
+          <t>07/09/2026 19:01</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
-        <v>19945.96</v>
+        <v>19924.31</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>-0.27</v>
+        <v>-0.37</v>
       </c>
       <c r="J62" s="7" t="n">
-        <v>0.36</v>
+        <v>0.46</v>
       </c>
       <c r="K62" s="7" t="n">
-        <v>0.8</v>
+        <v>0.74</v>
       </c>
       <c r="L62" t="n">
         <v>20000</v>
@@ -7396,22 +7360,22 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="U62" s="7" t="n">
-        <v>-54.04</v>
+        <v>-75.69</v>
       </c>
       <c r="V62" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="W62" s="7" t="n">
-        <v>52.08333333333334</v>
+        <v>50.9433962264151</v>
       </c>
       <c r="X62" s="7" t="n">
-        <v>0.8</v>
+        <v>0.74</v>
       </c>
       <c r="Y62" s="7" t="n">
-        <v>0.36</v>
+        <v>0.47</v>
       </c>
       <c r="Z62" t="inlineStr">
         <is>
@@ -7420,7 +7384,7 @@
       </c>
       <c r="AA62" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB62" t="inlineStr">
@@ -7465,7 +7429,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>07/08/2026 17:58</t>
+          <t>07/09/2026 19:04</t>
         </is>
       </c>
       <c r="H63" t="n">
@@ -7565,20 +7529,20 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>07/08/2026 17:59</t>
+          <t>07/09/2026 19:09</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
-        <v>19806.81</v>
+        <v>19779.31</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>-0.97</v>
+        <v>-1.1</v>
       </c>
       <c r="J64" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>0.61</v>
+        <v>0.58</v>
       </c>
       <c r="L64" t="n">
         <v>20000</v>
@@ -7596,19 +7560,19 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="U64" s="7" t="n">
-        <v>-193.19</v>
+        <v>-220.69</v>
       </c>
       <c r="V64" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="W64" s="7" t="n">
-        <v>50.9433962264151</v>
+        <v>50</v>
       </c>
       <c r="X64" s="7" t="n">
-        <v>0.61</v>
+        <v>0.58</v>
       </c>
       <c r="Y64" s="7" t="n">
         <v>1.2</v>
@@ -7620,7 +7584,7 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB64" t="inlineStr">
@@ -7665,20 +7629,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>07/08/2026 17:46</t>
+          <t>07/09/2026 13:42</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19671.02</v>
+        <v>20028.92</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-1.64</v>
+        <v>0.15</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>4.76</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.9</v>
+        <v>1.01</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7696,19 +7660,19 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>977</v>
+        <v>1121</v>
       </c>
       <c r="U65" s="7" t="n">
-        <v>-335.83</v>
+        <v>23.96000000000004</v>
       </c>
       <c r="V65" t="n">
-        <v>436</v>
+        <v>510</v>
       </c>
       <c r="W65" s="7" t="n">
-        <v>44.62640736949847</v>
+        <v>45.49509366636931</v>
       </c>
       <c r="X65" s="7" t="n">
-        <v>0.9</v>
+        <v>1.01</v>
       </c>
       <c r="Y65" s="7" t="n">
         <v>4.76</v>
@@ -7720,7 +7684,7 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB65" t="inlineStr">
@@ -7765,20 +7729,20 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>07/08/2026 17:51</t>
+          <t>07/09/2026 18:53</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
-        <v>19649.21</v>
+        <v>19665.29</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>-1.75</v>
+        <v>-1.67</v>
       </c>
       <c r="J66" s="7" t="n">
         <v>2.28</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>0.41</v>
+        <v>0.43</v>
       </c>
       <c r="L66" t="n">
         <v>20000</v>
@@ -7787,37 +7751,28 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>-452.04</v>
+        <v>0</v>
       </c>
       <c r="P66" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q66" s="7" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="R66" s="7" t="n">
-        <v>0.08776461566403648</v>
-      </c>
-      <c r="S66" s="7" t="n">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="U66" s="7" t="n">
-        <v>-350.79</v>
+        <v>-334.71</v>
       </c>
       <c r="V66" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="W66" s="7" t="n">
-        <v>30.76923076923077</v>
+        <v>32.3943661971831</v>
       </c>
       <c r="X66" s="7" t="n">
-        <v>0.41</v>
+        <v>0.43</v>
       </c>
       <c r="Y66" s="7" t="n">
         <v>2.29</v>
@@ -7829,7 +7784,7 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
@@ -7874,20 +7829,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>07/08/2026 17:57</t>
+          <t>07/09/2026 19:02</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>19983.56</v>
+        <v>19927.55</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>-0.08</v>
+        <v>-0.36</v>
       </c>
       <c r="J67" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>0.97</v>
+        <v>0.89</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7896,40 +7851,31 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>-8.200000000000005</v>
+        <v>0</v>
       </c>
       <c r="P67" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q67" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R67" s="7" t="n">
-        <v>0.9852766904873056</v>
-      </c>
-      <c r="S67" s="7" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>-16.44</v>
+        <v>-72.45000000000005</v>
       </c>
       <c r="V67" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>52.27272727272727</v>
+        <v>51.02040816326531</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>0.97</v>
+        <v>0.89</v>
       </c>
       <c r="Y67" s="7" t="n">
-        <v>0.93</v>
+        <v>0.95</v>
       </c>
       <c r="Z67" t="inlineStr">
         <is>
@@ -7938,7 +7884,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7983,7 +7929,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>07/08/2026 17:59</t>
+          <t>07/09/2026 19:10</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8083,7 +8029,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>07/08/2026 17:59</t>
+          <t>07/09/2026 19:06</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8183,7 +8129,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>07/08/2026 18:01</t>
+          <t>07/09/2026 19:09</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8283,7 +8229,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>07/08/2026 18:08</t>
+          <t>07/09/2026 14:14</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8392,7 +8338,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>07/08/2026 20:46</t>
+          <t>07/09/2026 16:43</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8501,7 +8447,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>07/03/2026 16:52</t>
+          <t>07/09/2026 16:58</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8610,14 +8556,14 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>07/08/2026 21:12</t>
+          <t>07/09/2026 17:10</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>28215.23</v>
+        <v>28123.35</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>-24.27</v>
+        <v>-24.51</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>32.64</v>
@@ -8635,7 +8581,7 @@
         <v>40</v>
       </c>
       <c r="O74" s="7" t="n">
-        <v>97.25</v>
+        <v>81.72</v>
       </c>
       <c r="P74" t="n">
         <v>36</v>
@@ -8644,22 +8590,22 @@
         <v>90</v>
       </c>
       <c r="R74" s="7" t="n">
-        <v>1.757811891217954</v>
+        <v>1.561533704390847</v>
       </c>
       <c r="S74" s="7" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="T74" t="n">
-        <v>3178</v>
+        <v>3182</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>-6066.77</v>
+        <v>-6158.65</v>
       </c>
       <c r="V74" t="n">
-        <v>1910</v>
+        <v>1911</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>60.10069225928257</v>
+        <v>60.05656819610308</v>
       </c>
       <c r="X74" s="7" t="n">
         <v>0.8</v>
@@ -8674,7 +8620,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8719,7 +8665,7 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>07/03/2026 12:55</t>
+          <t>07/09/2026 13:04</t>
         </is>
       </c>
       <c r="H75" s="9" t="n">
@@ -9174,7 +9120,7 @@
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>07/06/2026 16:38</t>
+          <t>07/09/2026 16:42</t>
         </is>
       </c>
       <c r="H80" s="9" t="n">
@@ -9265,7 +9211,7 @@
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>07/08/2026 17:36</t>
+          <t>07/09/2026 18:34</t>
         </is>
       </c>
       <c r="H81" s="9" t="n">
@@ -9356,7 +9302,7 @@
       </c>
       <c r="G82" s="8" t="inlineStr">
         <is>
-          <t>07/05/2026 22:20</t>
+          <t>07/08/2026 22:23</t>
         </is>
       </c>
       <c r="H82" s="9" t="n">
@@ -9538,20 +9484,20 @@
       </c>
       <c r="G84" s="8" t="inlineStr">
         <is>
-          <t>07/08/2026 17:35</t>
+          <t>07/09/2026 18:34</t>
         </is>
       </c>
       <c r="H84" s="9" t="n">
-        <v>19666.43</v>
+        <v>19608.54</v>
       </c>
       <c r="I84" s="9" t="n">
-        <v>-1.67</v>
+        <v>-1.96</v>
       </c>
       <c r="J84" s="9" t="n">
-        <v>1.7</v>
+        <v>1.99</v>
       </c>
       <c r="K84" s="9" t="n">
-        <v>0.32</v>
+        <v>0.28</v>
       </c>
       <c r="L84" s="8" t="n">
         <v>20000</v>
@@ -9560,23 +9506,17 @@
         <v>0</v>
       </c>
       <c r="N84" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O84" s="9" t="n">
-        <v>-273.89</v>
+        <v>0</v>
       </c>
       <c r="P84" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="Q84" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R84" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S84" s="9" t="n">
-        <v>1.37</v>
-      </c>
+      <c r="Q84" s="8" t="n"/>
+      <c r="R84" s="8" t="n"/>
+      <c r="S84" s="8" t="n"/>
       <c r="T84" s="8" t="n">
         <v>0</v>
       </c>
@@ -9629,20 +9569,20 @@
       </c>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t>07/08/2026 17:16</t>
+          <t>07/09/2026 18:05</t>
         </is>
       </c>
       <c r="H85" s="9" t="n">
-        <v>19609.46</v>
+        <v>19620.9</v>
       </c>
       <c r="I85" s="9" t="n">
-        <v>-1.95</v>
+        <v>-1.9</v>
       </c>
       <c r="J85" s="9" t="n">
         <v>2.27</v>
       </c>
       <c r="K85" s="9" t="n">
-        <v>0.45</v>
+        <v>0.47</v>
       </c>
       <c r="L85" s="8" t="n">
         <v>20000</v>
@@ -9651,23 +9591,17 @@
         <v>0</v>
       </c>
       <c r="N85" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O85" s="9" t="n">
-        <v>-190.78</v>
+        <v>0</v>
       </c>
       <c r="P85" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q85" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R85" s="9" t="n">
-        <v>0.4489153355094023</v>
-      </c>
-      <c r="S85" s="9" t="n">
-        <v>1.44</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q85" s="8" t="n"/>
+      <c r="R85" s="8" t="n"/>
+      <c r="S85" s="8" t="n"/>
       <c r="T85" s="8" t="n">
         <v>0</v>
       </c>
@@ -9720,20 +9654,20 @@
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>07/08/2026 17:30</t>
+          <t>07/09/2026 18:25</t>
         </is>
       </c>
       <c r="H86" s="9" t="n">
-        <v>22515.12</v>
+        <v>21628.34</v>
       </c>
       <c r="I86" s="9" t="n">
-        <v>12.58</v>
+        <v>8.15</v>
       </c>
       <c r="J86" s="9" t="n">
         <v>5.86</v>
       </c>
       <c r="K86" s="9" t="n">
-        <v>1.57</v>
+        <v>1.3</v>
       </c>
       <c r="L86" s="8" t="n">
         <v>20000</v>
@@ -9805,7 +9739,7 @@
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>07/08/2026 17:23</t>
+          <t>07/09/2026 18:15</t>
         </is>
       </c>
       <c r="H87" s="9" t="n">
@@ -9890,7 +9824,7 @@
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>07/08/2026 18:00</t>
+          <t>07/09/2026 19:06</t>
         </is>
       </c>
       <c r="H88" s="9" t="n">
@@ -10066,7 +10000,7 @@
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>07/06/2026 01:39</t>
+          <t>07/09/2026 01:42</t>
         </is>
       </c>
       <c r="H90" s="9" t="n">
@@ -10248,7 +10182,7 @@
       </c>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t>07/06/2026 20:57</t>
+          <t>07/09/2026 21:00</t>
         </is>
       </c>
       <c r="H92" s="9" t="n">
@@ -10423,7 +10357,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>07/03/2026 12:55</t>
+          <t>07/09/2026 13:04</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -10628,7 +10562,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>07/06/2026 16:38</t>
+          <t>07/09/2026 16:42</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -10669,7 +10603,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>07/08/2026 17:36</t>
+          <t>07/09/2026 18:34</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -10710,7 +10644,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>07/05/2026 22:20</t>
+          <t>07/08/2026 22:23</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -10792,17 +10726,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>07/08/2026 17:35</t>
+          <t>07/09/2026 18:34</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>19666.43</v>
+        <v>19608.54</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>-1.67</v>
+        <v>-1.96</v>
       </c>
       <c r="I14" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -10833,17 +10767,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>07/08/2026 17:16</t>
+          <t>07/09/2026 18:05</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>19609.46</v>
+        <v>19620.9</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>-1.95</v>
+        <v>-1.9</v>
       </c>
       <c r="I15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -10874,14 +10808,14 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>07/08/2026 17:30</t>
+          <t>07/09/2026 18:25</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>22515.12</v>
+        <v>21628.34</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>12.58</v>
+        <v>8.15</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -10915,7 +10849,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>07/08/2026 17:23</t>
+          <t>07/09/2026 18:15</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -10956,7 +10890,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>07/08/2026 18:00</t>
+          <t>07/09/2026 19:06</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -11038,7 +10972,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>07/06/2026 01:39</t>
+          <t>07/09/2026 01:42</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -11120,7 +11054,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>07/06/2026 20:57</t>
+          <t>07/09/2026 21:00</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -12000,7 +11934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -12061,7 +11995,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>07/06/2026 09:09</t>
+          <t>07/09/2026 09:13</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -12107,7 +12041,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>07/03/2026 09:16</t>
+          <t>07/09/2026 09:24</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -12268,7 +12202,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>07/06/2026 13:53</t>
+          <t>07/09/2026 13:56</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -12314,7 +12248,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>07/03/2026 09:12</t>
+          <t>07/09/2026 09:19</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
@@ -12452,7 +12386,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07/08/2026 19:43</t>
+          <t>07/09/2026 15:48</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -12475,7 +12409,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>07/06/2026 15:46</t>
+          <t>07/09/2026 15:50</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -12498,11 +12432,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07/08/2026 17:36</t>
+          <t>07/09/2026 18:33</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20072.25</v>
+        <v>19971.62</v>
       </c>
     </row>
     <row r="24">
@@ -12544,11 +12478,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07/08/2026 17:58</t>
+          <t>07/09/2026 19:04</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19956.58</v>
+        <v>19839.37</v>
       </c>
     </row>
     <row r="26">
@@ -12567,11 +12501,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07/07/2026 11:07</t>
+          <t>07/09/2026 19:08</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20323.33</v>
+        <v>20097.65</v>
       </c>
     </row>
     <row r="27">
@@ -12590,7 +12524,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07/08/2026 18:02</t>
+          <t>07/09/2026 19:11</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -12613,11 +12547,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07/08/2026 20:15</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="n">
-        <v>19937.43</v>
+          <t>07/09/2026 22:10</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>19701</v>
       </c>
     </row>
     <row r="29">
@@ -12636,11 +12570,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07/08/2026 20:18</t>
+          <t>07/09/2026 22:12</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>19598.28</v>
+        <v>19426.47</v>
       </c>
     </row>
     <row r="30">
@@ -12659,11 +12593,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07/08/2026 20:20</t>
+          <t>07/09/2026 16:19</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>19670.74</v>
+        <v>19459.64</v>
       </c>
     </row>
     <row r="31">
@@ -12682,11 +12616,11 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07/08/2026 20:17</t>
+          <t>07/09/2026 22:10</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>20063.67</v>
+        <v>20022.45</v>
       </c>
     </row>
     <row r="32">
@@ -12705,7 +12639,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07/08/2026 20:18</t>
+          <t>07/09/2026 09:59</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -12728,11 +12662,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>07/08/2026 18:10</t>
+          <t>07/09/2026 19:25</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>19975.11</v>
+        <v>19922.09</v>
       </c>
     </row>
     <row r="34">
@@ -12751,11 +12685,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>07/07/2026 11:19</t>
+          <t>07/09/2026 19:18</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>19937.23</v>
+        <v>19907.74</v>
       </c>
     </row>
     <row r="35">
@@ -12774,11 +12708,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>07/08/2026 18:03</t>
+          <t>07/09/2026 19:13</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>19930.83</v>
+        <v>19828.3</v>
       </c>
     </row>
     <row r="36">
@@ -12797,11 +12731,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>07/08/2026 18:03</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="n">
-        <v>19900.77</v>
+          <t>07/09/2026 19:12</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>19951</v>
       </c>
     </row>
     <row r="37">
@@ -12820,11 +12754,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>07/08/2026 18:05</t>
+          <t>07/09/2026 19:17</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>20530.6</v>
+        <v>20551.07</v>
       </c>
     </row>
     <row r="38">
@@ -12843,11 +12777,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>07/08/2026 18:04</t>
+          <t>07/09/2026 19:16</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>19900.11</v>
+        <v>19842.98</v>
       </c>
     </row>
     <row r="39">
@@ -12866,11 +12800,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>07/08/2026 18:05</t>
+          <t>07/09/2026 19:16</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>20165.38</v>
+        <v>20100.93</v>
       </c>
     </row>
     <row r="40">
@@ -12889,11 +12823,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>07/08/2026 18:07</t>
+          <t>07/09/2026 19:20</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>19896.88</v>
+        <v>19858.37</v>
       </c>
     </row>
     <row r="41">
@@ -12912,11 +12846,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>07/08/2026 18:07</t>
+          <t>07/09/2026 19:20</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>22101.59</v>
+        <v>22190.52</v>
       </c>
     </row>
     <row r="42">
@@ -12935,11 +12869,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>07/08/2026 18:09</t>
+          <t>07/09/2026 19:22</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>19519.04</v>
+        <v>19008.57</v>
       </c>
     </row>
     <row r="43">
@@ -12958,11 +12892,11 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>07/08/2026 18:06</t>
+          <t>07/09/2026 19:16</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>20424.69</v>
+        <v>20228.42</v>
       </c>
     </row>
     <row r="44">
@@ -12981,45 +12915,45 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>07/08/2026 18:07</t>
+          <t>07/09/2026 19:20</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>19893.06</v>
+        <v>19856.82</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>647831</t>
+          <t>55906</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>A MOL Argos</t>
+          <t>55906 Demo Sweep V5</t>
         </is>
       </c>
       <c r="C45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>03/30/2026 11:54</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>0</v>
+          <t>07/09/2026 19:57</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>17043.22</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>648289</t>
+          <t>647831</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">A-MOL Medallion </t>
+          <t>A MOL Argos</t>
         </is>
       </c>
       <c r="C46" t="b">
@@ -13027,7 +12961,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>07/06/2026 09:01</t>
+          <t>03/30/2026 11:54</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -13037,12 +12971,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>3038308</t>
+          <t>648289</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>A-MOL inactive Maven</t>
+          <t xml:space="preserve">A-MOL Medallion </t>
         </is>
       </c>
       <c r="C47" t="b">
@@ -13050,7 +12984,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>07/06/2026 09:28</t>
+          <t>07/06/2026 09:01</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -13060,69 +12994,92 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>52428846</t>
+          <t>3038308</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EA The5ers Low DD Dual Breakout</t>
+          <t>A-MOL inactive Maven</t>
         </is>
       </c>
       <c r="C48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>07/06/2026 20:51</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="n">
-        <v>41224.86</v>
+          <t>07/09/2026 09:37</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>80059994</t>
+          <t>52428846</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>A-MOL Denali Plus</t>
+          <t>EA The5ers Low DD Dual Breakout</t>
         </is>
       </c>
       <c r="C49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>07/08/2026 04:25</t>
+          <t>07/09/2026 20:53</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>0.43</v>
+        <v>41224.86</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>80059994</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>A-MOL Denali Plus</t>
+        </is>
+      </c>
+      <c r="C50" t="b">
+        <v>0</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>07/09/2026 07:43</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>5035285664</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Manual Trades (Rvg)</t>
         </is>
       </c>
-      <c r="C50" t="b">
-        <v>1</v>
-      </c>
-      <c r="D50" t="inlineStr">
+      <c r="C51" t="b">
+        <v>1</v>
+      </c>
+      <c r="D51" t="inlineStr">
         <is>
           <t>07/24/2025 16:40</t>
         </is>
       </c>
-      <c r="E50" s="7" t="n">
+      <c r="E51" s="7" t="n">
         <v>5331.24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboards — 2026-07-10
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-07-09 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-07-10 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>07/09/2026 17:37</t>
+          <t>07/10/2026 21:55</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>50903.61</v>
+        <v>51358.98</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>136.78</v>
+        <v>138.9</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>4318.99</v>
+        <v>2568.18</v>
       </c>
       <c r="P2" t="n">
         <v>27</v>
@@ -994,22 +994,22 @@
         <v>67.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>5.483116910077954</v>
+        <v>3.572939938886941</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>2.93</v>
+        <v>3.18</v>
       </c>
       <c r="T2" t="n">
-        <v>3079</v>
+        <v>3088</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>25915.52999999999</v>
+        <v>26358.98</v>
       </c>
       <c r="V2" t="n">
-        <v>1940</v>
+        <v>1945</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.0074699577785</v>
+        <v>62.98575129533679</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.08</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>07/09/2026 20:27</t>
+          <t>07/10/2026 19:08</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>07/09/2026 22:12</t>
+          <t>07/10/2026 20:29</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>07/04/2026 02:23</t>
+          <t>07/10/2026 02:29</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>07/09/2026 18:18</t>
+          <t>07/10/2026 22:41</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2377,20 +2377,20 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>07/09/2026 19:36</t>
+          <t>07/10/2026 18:17</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
-        <v>19470.66</v>
+        <v>19378.48</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>-7.7</v>
+        <v>-8.140000000000001</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.75</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="L15" s="7" t="n">
         <v>26775.1</v>
@@ -2402,37 +2402,37 @@
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>5077.88</v>
+        <v>4914.240000000001</v>
       </c>
       <c r="P15" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q15" s="7" t="n">
-        <v>42.5</v>
+        <v>40</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>1.692129869421803</v>
+        <v>1.661513734422072</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>20.18</v>
+        <v>20.51</v>
       </c>
       <c r="T15" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>-1208.299999999999</v>
+        <v>-1396.62</v>
       </c>
       <c r="V15" t="n">
         <v>89</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>53.2934131736527</v>
+        <v>52.97619047619047</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
       <c r="Y15" s="7" t="n">
-        <v>7.15</v>
+        <v>7.62</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2486,17 +2486,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>07/09/2026 16:30</t>
+          <t>07/10/2026 20:45</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>106.79</v>
+        <v>104.55</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>-99.48</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>99.48</v>
+        <v>99.48999999999999</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>0.7</v>
@@ -2511,37 +2511,37 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-5.93</v>
+        <v>-4.64</v>
       </c>
       <c r="P16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>30</v>
+        <v>32.5</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.5213882163034705</v>
+        <v>0.5827338129496403</v>
       </c>
       <c r="S16" s="7" t="n">
         <v>0.03</v>
       </c>
       <c r="T16" t="n">
-        <v>2010</v>
+        <v>2028</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-20316.54</v>
+        <v>-20317.85</v>
       </c>
       <c r="V16" t="n">
-        <v>651</v>
+        <v>658</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>32.38805970149254</v>
+        <v>32.44575936883629</v>
       </c>
       <c r="X16" s="7" t="n">
         <v>0.7</v>
       </c>
       <c r="Y16" s="7" t="n">
-        <v>99.48</v>
+        <v>99.48999999999999</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>07/09/2026 21:46</t>
+          <t>07/10/2026 20:09</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>07/09/2026 18:30</t>
+          <t>07/10/2026 22:52</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>07/09/2026 13:21</t>
+          <t>07/10/2026 22:49</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>07/09/2026 16:36</t>
+          <t>07/10/2026 20:50</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>07/09/2026 18:54</t>
+          <t>07/10/2026 17:47</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>07/09/2026 18:12</t>
+          <t>07/10/2026 22:34</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19556.08</v>
+        <v>19574.34</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.21</v>
+        <v>-2.12</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>5.42</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-637.2099999999999</v>
+        <v>-622.9599999999999</v>
       </c>
       <c r="P23" t="n">
         <v>19</v>
@@ -3283,25 +3283,25 @@
         <v>47.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.7390280462632287</v>
+        <v>0.7448641918678943</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>4.05</v>
       </c>
       <c r="T23" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-443.9199999999998</v>
+        <v>-425.6599999999997</v>
       </c>
       <c r="V23" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>49.2063492063492</v>
+        <v>50</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>5.42</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>07/09/2026 18:30</t>
+          <t>07/10/2026 22:53</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16191.96</v>
+        <v>16118.05</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-18.78</v>
+        <v>-19.15</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.54</v>
@@ -3492,34 +3492,34 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>100.36</v>
+        <v>125.45</v>
       </c>
       <c r="P25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>47.5</v>
+        <v>50</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.273520113376213</v>
+        <v>1.354068471112867</v>
       </c>
       <c r="S25" s="7" t="n">
         <v>0.99</v>
       </c>
       <c r="T25" t="n">
-        <v>457</v>
+        <v>468</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3808.04</v>
+        <v>-3881.95</v>
       </c>
       <c r="V25" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>36.76148796498906</v>
+        <v>36.11111111111111</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>20.79</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,20 +3576,20 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>07/09/2026 16:47</t>
+          <t>07/10/2026 15:51</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
-        <v>21794.32</v>
+        <v>14807.41</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>9.01</v>
+        <v>-26.22</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>4.28</v>
+        <v>34.8</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>1.7</v>
+        <v>0.47</v>
       </c>
       <c r="L26" t="n">
         <v>20000</v>
@@ -3601,37 +3601,34 @@
         <v>40</v>
       </c>
       <c r="O26" s="7" t="n">
-        <v>-156.96</v>
+        <v>71.99000000000001</v>
       </c>
       <c r="P26" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="Q26" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="R26" s="7" t="n">
-        <v>0.387066541705717</v>
+        <v>100</v>
       </c>
       <c r="S26" s="7" t="n">
-        <v>1.27</v>
+        <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>1147</v>
+        <v>1401</v>
       </c>
       <c r="U26" s="7" t="n">
-        <v>1724.24</v>
+        <v>-5204.830000000001</v>
       </c>
       <c r="V26" t="n">
-        <v>757</v>
+        <v>824</v>
       </c>
       <c r="W26" s="7" t="n">
-        <v>65.99825632083697</v>
+        <v>58.81513204853675</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>1.65</v>
+        <v>0.47</v>
       </c>
       <c r="Y26" s="7" t="n">
-        <v>4.27</v>
+        <v>34.56</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3640,7 +3637,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3650,7 +3647,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>T&amp;Dv5 Prop Bots | AUDJPY, T&amp;Dv5 Prop Bots | AUDJPY.pro, T&amp;Dv5 Prop Bots | CADJPY.pro, T&amp;Dv5 Prop Bots | EURJPY.pro, T&amp;Dv5 Prop Bots | EURUSD, T&amp;Dv5 Prop Bots | EURUSD.pro, T&amp;Dv5 Prop Bots | GBPJPY, T&amp;Dv5 Prop Bots | GBPJPY.pro, T&amp;Dv5 Prop Bots | GBPUSD, T&amp;Dv5 Prop Bots | GBPUSD.pro, T&amp;Dv5 Prop Bots | USDJPY, T&amp;Dv5 Prop Bots | USDJPY.pro</t>
+          <t>T&amp;Dv5 Prop Bots | AUDJPY, T&amp;Dv5 Prop Bots | AUDJPY.pro, T&amp;Dv5 Prop Bots | CADJPY, T&amp;Dv5 Prop Bots | CADJPY.pro, T&amp;Dv5 Prop Bots | EURJPY.pro, T&amp;Dv5 Prop Bots | EURUSD, T&amp;Dv5 Prop Bots | EURUSD.pro, T&amp;Dv5 Prop Bots | GBPJPY, T&amp;Dv5 Prop Bots | GBPJPY.pro, T&amp;Dv5 Prop Bots | GBPUSD, T&amp;Dv5 Prop Bots | GBPUSD.pro, T&amp;Dv5 Prop Bots | USDJPY, T&amp;Dv5 Prop Bots | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3682,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>07/09/2026 18:30</t>
+          <t>07/10/2026 17:27</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3725,7 +3722,7 @@
         <v>5.39</v>
       </c>
       <c r="T27" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="U27" s="7" t="n">
         <v>281.5</v>
@@ -3734,7 +3731,7 @@
         <v>30</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>41.66666666666667</v>
+        <v>40.54054054054054</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>1.09</v>
@@ -3749,7 +3746,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3903,20 +3900,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>07/09/2026 18:34</t>
+          <t>07/10/2026 22:56</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>20353.8</v>
+        <v>20362.61</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>1.77</v>
+        <v>1.81</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,34 +3925,34 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>60.75000000000002</v>
+        <v>167.5</v>
       </c>
       <c r="P29" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>52.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>1.048960742752601</v>
+        <v>1.146583937900918</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>5.6</v>
+        <v>5.25</v>
       </c>
       <c r="T29" t="n">
         <v>79</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>353.7999999999999</v>
+        <v>362.6099999999999</v>
       </c>
       <c r="V29" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>55.69620253164557</v>
+        <v>56.9620253164557</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3964,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4012,7 +4009,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>07/07/2026 03:07</t>
+          <t>07/10/2026 03:09</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,20 +4118,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>07/09/2026 18:44</t>
+          <t>07/10/2026 23:06</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20791.95</v>
+        <v>20804.68</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>3.97</v>
+        <v>4.04</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>1.09</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>2.55</v>
+        <v>2.52</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -4146,7 +4143,7 @@
         <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>798.71</v>
+        <v>814.3200000000001</v>
       </c>
       <c r="P31" t="n">
         <v>13</v>
@@ -4155,25 +4152,25 @@
         <v>32.5</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>2.772705078125</v>
+        <v>2.784693609187341</v>
       </c>
       <c r="S31" s="7" t="n">
         <v>1.09</v>
       </c>
       <c r="T31" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>791.95</v>
+        <v>804.6799999999999</v>
       </c>
       <c r="V31" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>27.45098039215686</v>
+        <v>27.77777777777778</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>2.55</v>
+        <v>2.52</v>
       </c>
       <c r="Y31" s="7" t="n">
         <v>1.1</v>
@@ -4185,7 +4182,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
@@ -4195,7 +4192,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
+          <t>LVF-ZFade MOL | AUDUSD.pro, LVF-ZFade MOL | EURCAD.pro, LVF-ZFade MOL | EURGBP.pro, LVF-ZFade MOL | EURUSD.pro, LVF-ZFade MOL | GBPAUD.pro, LVF-ZFade MOL | GBPCAD, LVF-ZFade MOL | GBPCAD.pro, LVF-ZFade MOL | GBPCHF, LVF-ZFade MOL | GBPCHF.pro, LVF-ZFade MOL | GBPJPY.pro, LVF-ZFade MOL | GBPNZD, LVF-ZFade MOL | GBPNZD.pro, LVF-ZFade MOL | GBPUSD, LVF-ZFade MOL | GBPUSD.pro, LVF-ZFade MOL | USDCAD, LVF-ZFade MOL | USDCAD.pro, LVF-ZFade MOL | USDCHF, LVF-ZFade MOL | USDCHF.pro, LVF-ZFade MOL | USDJPY.pro, LVF-ZFade MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4227,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>07/09/2026 18:30</t>
+          <t>07/10/2026 22:51</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4336,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>07/09/2026 18:56</t>
+          <t>07/10/2026 17:50</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,20 +4445,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>07/09/2026 15:50</t>
+          <t>07/10/2026 20:02</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20104.68</v>
+        <v>20157.4</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.53</v>
+        <v>0.79</v>
       </c>
       <c r="J34" s="7" t="n">
-        <v>2.62</v>
+        <v>2.87</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.08</v>
+        <v>1.11</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,37 +4470,37 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-555.11</v>
+        <v>-452.35</v>
       </c>
       <c r="P34" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>30</v>
+        <v>32.5</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.5477497881770188</v>
+        <v>0.6315047736974161</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>2.78</v>
+        <v>2.93</v>
       </c>
       <c r="T34" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>104.68</v>
+        <v>157.4</v>
       </c>
       <c r="V34" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>44.82758620689656</v>
+        <v>45</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1.08</v>
+        <v>1.11</v>
       </c>
       <c r="Y34" s="7" t="n">
-        <v>2.64</v>
+        <v>2.88</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -4512,7 +4509,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4557,14 +4554,14 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>07/09/2026 20:17</t>
+          <t>07/10/2026 18:58</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
-        <v>14229.07</v>
+        <v>14290.03</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>-28.87</v>
+        <v>-28.57</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>41.42</v>
@@ -4582,7 +4579,7 @@
         <v>40</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>9.329999999999984</v>
+        <v>-15.63000000000001</v>
       </c>
       <c r="P35" t="n">
         <v>20</v>
@@ -4591,10 +4588,10 @@
         <v>50</v>
       </c>
       <c r="R35" s="7" t="n">
-        <v>1.006560812331233</v>
+        <v>0.9890090571557156</v>
       </c>
       <c r="S35" s="7" t="n">
-        <v>2.41</v>
+        <v>2.42</v>
       </c>
       <c r="T35" t="n">
         <v>1618</v>
@@ -4706,22 +4703,22 @@
         <v>0.74</v>
       </c>
       <c r="T36" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>1039.71</v>
+        <v>840.03</v>
       </c>
       <c r="V36" t="n">
         <v>27</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>60</v>
+        <v>58.69565217391305</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>1.6</v>
+        <v>1.43</v>
       </c>
       <c r="Y36" s="7" t="n">
-        <v>2.44</v>
+        <v>2.9</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4730,7 +4727,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4775,7 +4772,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>07/09/2026 19:51</t>
+          <t>07/10/2026 18:28</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4884,20 +4881,20 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>07/09/2026 15:26</t>
+          <t>07/10/2026 19:34</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
         <v>18933.84</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>-4.13</v>
+        <v>-4.41</v>
       </c>
       <c r="J38" s="7" t="n">
         <v>5.41</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="L38" t="n">
         <v>20000</v>
@@ -4906,19 +4903,19 @@
         <v>0</v>
       </c>
       <c r="N38" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>19161.24</v>
+        <v>19105.12</v>
       </c>
       <c r="P38" t="n">
         <v>4</v>
       </c>
       <c r="Q38" s="7" t="n">
-        <v>19.04761904761905</v>
+        <v>18.18181818181818</v>
       </c>
       <c r="R38" s="7" t="n">
-        <v>17.50962855739654</v>
+        <v>16.70202099068815</v>
       </c>
       <c r="S38" s="7" t="n">
         <v>2.73</v>
@@ -4953,7 +4950,7 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr">
@@ -4993,7 +4990,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>07/09/2026 20:39</t>
+          <t>07/10/2026 19:22</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5102,7 +5099,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>07/09/2026 16:39</t>
+          <t>07/10/2026 20:53</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5211,7 +5208,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>07/09/2026 17:23</t>
+          <t>07/10/2026 21:41</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5320,20 +5317,20 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>07/09/2026 18:12</t>
-        </is>
-      </c>
-      <c r="H42" s="7" t="n">
-        <v>19418.9</v>
+          <t>07/10/2026 22:35</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>19425</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>-2.9</v>
+        <v>-2.87</v>
       </c>
       <c r="J42" s="7" t="n">
         <v>4.17</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="L42" t="n">
         <v>20000</v>
@@ -5345,34 +5342,34 @@
         <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-16.19</v>
+        <v>18.04</v>
       </c>
       <c r="P42" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Q42" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>57.49999999999999</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>0.7454002201604025</v>
+        <v>1.397794928335171</v>
       </c>
       <c r="S42" s="7" t="n">
-        <v>0.23</v>
+        <v>0.13</v>
       </c>
       <c r="T42" t="n">
-        <v>1281</v>
+        <v>1299</v>
       </c>
       <c r="U42" s="7" t="n">
-        <v>-590.9000000000001</v>
+        <v>-575.7600000000001</v>
       </c>
       <c r="V42" t="n">
-        <v>589</v>
+        <v>599</v>
       </c>
       <c r="W42" s="7" t="n">
-        <v>45.97970335675254</v>
+        <v>46.11239414934565</v>
       </c>
       <c r="X42" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="Y42" s="7" t="n">
         <v>4.17</v>
@@ -5384,7 +5381,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
@@ -5429,14 +5426,14 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>07/09/2026 18:18</t>
+          <t>07/10/2026 22:38</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
-        <v>18253.36</v>
+        <v>18260.54</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>-8.720000000000001</v>
+        <v>-8.69</v>
       </c>
       <c r="J43" s="7" t="n">
         <v>9.66</v>
@@ -5460,19 +5457,19 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>2536</v>
+        <v>2575</v>
       </c>
       <c r="U43" s="7" t="n">
-        <v>-1756.57</v>
+        <v>-1739.46</v>
       </c>
       <c r="V43" t="n">
-        <v>1111</v>
+        <v>1129</v>
       </c>
       <c r="W43" s="7" t="n">
-        <v>43.80914826498422</v>
+        <v>43.84466019417476</v>
       </c>
       <c r="X43" s="7" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="Y43" s="7" t="n">
         <v>9.67</v>
@@ -5484,7 +5481,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
@@ -5529,7 +5526,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>07/09/2026 18:22</t>
+          <t>07/10/2026 22:43</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5629,20 +5626,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>07/09/2026 18:14</t>
+          <t>07/10/2026 22:36</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19852.41</v>
+        <v>19840.44</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.74</v>
+        <v>-0.8</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>1.6</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5660,19 +5657,19 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-147.59</v>
+        <v>-159.56</v>
       </c>
       <c r="V45" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>51.70454545454546</v>
+        <v>51.66666666666667</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="Y45" s="7" t="n">
         <v>1.59</v>
@@ -5684,7 +5681,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5729,20 +5726,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>07/09/2026 13:06</t>
+          <t>07/10/2026 17:13</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>20002.43</v>
+        <v>19989.97</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0.01</v>
+        <v>-0.05</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>1.09</v>
+        <v>0.75</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5760,22 +5757,22 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>2.43</v>
+        <v>-10.03</v>
       </c>
       <c r="V46" t="n">
         <v>6</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>35.29411764705883</v>
+        <v>27.27272727272727</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>1.09</v>
+        <v>0.75</v>
       </c>
       <c r="Y46" s="7" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5784,7 +5781,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5829,7 +5826,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>07/09/2026 18:27</t>
+          <t>07/10/2026 22:48</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5929,7 +5926,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>07/09/2026 18:26</t>
+          <t>07/10/2026 17:24</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6029,20 +6026,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>07/09/2026 18:43</t>
+          <t>07/10/2026 23:04</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>19825.59</v>
+        <v>19806.96</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>-0.89</v>
+        <v>-0.98</v>
       </c>
       <c r="J49" s="7" t="n">
         <v>2.74</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="L49" t="n">
         <v>20000</v>
@@ -6060,19 +6057,19 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="U49" s="7" t="n">
-        <v>-174.4100000000001</v>
+        <v>-199.01</v>
       </c>
       <c r="V49" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="W49" s="7" t="n">
-        <v>41.50943396226415</v>
+        <v>41.47465437788019</v>
       </c>
       <c r="X49" s="7" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="Y49" s="7" t="n">
         <v>2.72</v>
@@ -6084,7 +6081,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
@@ -6129,20 +6126,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>07/09/2026 18:34</t>
+          <t>07/10/2026 22:56</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>21975.19</v>
+        <v>21948.24</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>9.9</v>
+        <v>9.77</v>
       </c>
       <c r="J50" s="7" t="n">
         <v>3.34</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>1.39</v>
+        <v>1.38</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6160,19 +6157,19 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>603</v>
+        <v>613</v>
       </c>
       <c r="U50" s="7" t="n">
-        <v>1975.19</v>
+        <v>1911.05</v>
       </c>
       <c r="V50" t="n">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="W50" s="7" t="n">
-        <v>52.23880597014925</v>
+        <v>51.71288743882545</v>
       </c>
       <c r="X50" s="7" t="n">
-        <v>1.39</v>
+        <v>1.37</v>
       </c>
       <c r="Y50" s="7" t="n">
         <v>3.34</v>
@@ -6184,7 +6181,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
@@ -6229,20 +6226,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>07/09/2026 18:31</t>
+          <t>07/10/2026 22:54</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>24546.75</v>
+        <v>24489.46</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>22.73</v>
+        <v>22.45</v>
       </c>
       <c r="J51" s="7" t="n">
         <v>5.53</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6260,19 +6257,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>1038</v>
+        <v>1055</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>4546.75</v>
+        <v>4434.4</v>
       </c>
       <c r="V51" t="n">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>52.89017341040463</v>
+        <v>52.32227488151658</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>1.49</v>
+        <v>1.47</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>5.53</v>
@@ -6284,7 +6281,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6329,7 +6326,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>07/09/2026 18:09</t>
+          <t>07/10/2026 17:10</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6429,20 +6426,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>07/09/2026 18:46</t>
+          <t>07/10/2026 17:40</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19745.1</v>
+        <v>19732.4</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.29</v>
+        <v>-1.35</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.39</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6460,19 +6457,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-254.9</v>
+        <v>-267.6</v>
       </c>
       <c r="V53" t="n">
         <v>34</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>37.36263736263736</v>
+        <v>35.41666666666667</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.37</v>
@@ -6484,7 +6481,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6529,20 +6526,20 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>07/09/2026 18:53</t>
+          <t>07/10/2026 17:47</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
-        <v>19664.26</v>
+        <v>19908.75</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>-1.67</v>
+        <v>-0.45</v>
       </c>
       <c r="J54" s="7" t="n">
         <v>4.63</v>
       </c>
       <c r="K54" s="7" t="n">
-        <v>0.79</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L54" t="n">
         <v>20000</v>
@@ -6560,19 +6557,19 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="U54" s="7" t="n">
-        <v>-335.7400000000001</v>
+        <v>-91.25000000000006</v>
       </c>
       <c r="V54" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="W54" s="7" t="n">
-        <v>38.84892086330935</v>
+        <v>40.14084507042254</v>
       </c>
       <c r="X54" s="7" t="n">
-        <v>0.79</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y54" s="7" t="n">
         <v>4.63</v>
@@ -6584,7 +6581,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -6629,20 +6626,20 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>07/09/2026 18:37</t>
+          <t>07/10/2026 22:59</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
-        <v>19918.2</v>
+        <v>19901.21</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>-0.39</v>
+        <v>-0.47</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>1.15</v>
+        <v>1.19</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L55" t="n">
         <v>20000</v>
@@ -6660,22 +6657,22 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>669</v>
+        <v>691</v>
       </c>
       <c r="U55" s="7" t="n">
-        <v>-81.8</v>
+        <v>-98.78999999999998</v>
       </c>
       <c r="V55" t="n">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="W55" s="7" t="n">
-        <v>48.57997010463378</v>
+        <v>48.91461649782924</v>
       </c>
       <c r="X55" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y55" s="7" t="n">
-        <v>1.16</v>
+        <v>1.2</v>
       </c>
       <c r="Z55" t="inlineStr">
         <is>
@@ -6684,7 +6681,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -6729,20 +6726,20 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>07/09/2026 13:48</t>
+          <t>07/10/2026 17:45</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
-        <v>19765.95</v>
+        <v>19805.98</v>
       </c>
       <c r="I56" s="7" t="n">
-        <v>-1.19</v>
+        <v>-0.99</v>
       </c>
       <c r="J56" s="7" t="n">
         <v>1.31</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>0.85</v>
+        <v>0.88</v>
       </c>
       <c r="L56" t="n">
         <v>20000</v>
@@ -6760,16 +6757,16 @@
         <v>0</v>
       </c>
       <c r="T56" t="n">
-        <v>565</v>
+        <v>586</v>
       </c>
       <c r="U56" s="7" t="n">
-        <v>-193.84</v>
+        <v>-193.01</v>
       </c>
       <c r="V56" t="n">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="W56" s="7" t="n">
-        <v>46.54867256637168</v>
+        <v>46.92832764505119</v>
       </c>
       <c r="X56" s="7" t="n">
         <v>0.88</v>
@@ -6784,7 +6781,7 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr">
@@ -6829,20 +6826,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>07/09/2026 18:19</t>
+          <t>07/10/2026 22:43</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19792.22</v>
+        <v>19808.38</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.03</v>
+        <v>-0.96</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6860,19 +6857,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-207.78</v>
+        <v>-191.6200000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.61948955916473</v>
+        <v>43.86363636363637</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6884,7 +6881,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6929,20 +6926,20 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>07/09/2026 18:40</t>
+          <t>07/10/2026 23:01</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
-        <v>18240.71</v>
+        <v>18264.83</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>-8.81</v>
+        <v>-8.69</v>
       </c>
       <c r="J58" s="7" t="n">
         <v>9.16</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="L58" t="n">
         <v>20000</v>
@@ -6960,19 +6957,19 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1838</v>
+        <v>1941</v>
       </c>
       <c r="U58" s="7" t="n">
-        <v>-1759.29</v>
+        <v>-1735.26</v>
       </c>
       <c r="V58" t="n">
-        <v>792</v>
+        <v>845</v>
       </c>
       <c r="W58" s="7" t="n">
-        <v>43.09031556039173</v>
+        <v>43.53426069036579</v>
       </c>
       <c r="X58" s="7" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="Y58" s="7" t="n">
         <v>9.15</v>
@@ -6984,7 +6981,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB58" t="inlineStr">
@@ -7029,20 +7026,20 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>07/09/2026 18:51</t>
+          <t>07/10/2026 17:45</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
-        <v>19964.57</v>
+        <v>19962.47</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>-0.17</v>
+        <v>-0.18</v>
       </c>
       <c r="J59" s="7" t="n">
         <v>0.55</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="L59" t="n">
         <v>20000</v>
@@ -7060,19 +7057,19 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="U59" s="7" t="n">
-        <v>-35.43000000000001</v>
+        <v>-37.53000000000001</v>
       </c>
       <c r="V59" t="n">
         <v>41</v>
       </c>
       <c r="W59" s="7" t="n">
-        <v>42.2680412371134</v>
+        <v>41.83673469387755</v>
       </c>
       <c r="X59" s="7" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="Y59" s="7" t="n">
         <v>0.55</v>
@@ -7084,7 +7081,7 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -7129,20 +7126,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>07/09/2026 18:44</t>
+          <t>07/10/2026 12:39</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>18810.48</v>
+        <v>18913.15</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-5.96</v>
+        <v>-5.45</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>12.98</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="L60" t="n">
         <v>20000</v>
@@ -7160,19 +7157,19 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>2854</v>
+        <v>3017</v>
       </c>
       <c r="U60" s="7" t="n">
-        <v>-1189.52</v>
+        <v>-1095.45</v>
       </c>
       <c r="V60" t="n">
-        <v>1319</v>
+        <v>1412</v>
       </c>
       <c r="W60" s="7" t="n">
-        <v>46.21583742116328</v>
+        <v>46.80145840238647</v>
       </c>
       <c r="X60" s="7" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="Y60" s="7" t="n">
         <v>12.97</v>
@@ -7184,7 +7181,7 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
@@ -7229,20 +7226,20 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>07/09/2026 18:43</t>
+          <t>07/10/2026 23:04</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>19680.32</v>
+        <v>19592.48</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-1.6</v>
+        <v>-2.04</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>6.82</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L61" t="n">
         <v>20000</v>
@@ -7260,19 +7257,19 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>1712</v>
+        <v>1799</v>
       </c>
       <c r="U61" s="7" t="n">
-        <v>-319.6799999999997</v>
+        <v>-390.5099999999999</v>
       </c>
       <c r="V61" t="n">
-        <v>784</v>
+        <v>826</v>
       </c>
       <c r="W61" s="7" t="n">
-        <v>45.79439252336449</v>
+        <v>45.91439688715953</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y61" s="7" t="n">
         <v>6.81</v>
@@ -7284,7 +7281,7 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
@@ -7329,7 +7326,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>07/09/2026 19:01</t>
+          <t>07/10/2026 17:52</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7429,7 +7426,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>07/09/2026 19:04</t>
+          <t>07/10/2026 17:55</t>
         </is>
       </c>
       <c r="H63" t="n">
@@ -7529,7 +7526,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>07/09/2026 19:09</t>
+          <t>07/10/2026 17:59</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7629,20 +7626,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>07/09/2026 13:42</t>
+          <t>07/10/2026 17:41</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>20028.92</v>
+        <v>19911.91</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>0.15</v>
+        <v>-0.44</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>4.76</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>1.01</v>
+        <v>0.98</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7660,19 +7657,19 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>1121</v>
+        <v>1230</v>
       </c>
       <c r="U65" s="7" t="n">
-        <v>23.96000000000004</v>
+        <v>-88.08999999999992</v>
       </c>
       <c r="V65" t="n">
-        <v>510</v>
+        <v>554</v>
       </c>
       <c r="W65" s="7" t="n">
-        <v>45.49509366636931</v>
+        <v>45.04065040650406</v>
       </c>
       <c r="X65" s="7" t="n">
-        <v>1.01</v>
+        <v>0.98</v>
       </c>
       <c r="Y65" s="7" t="n">
         <v>4.76</v>
@@ -7684,7 +7681,7 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB65" t="inlineStr">
@@ -7729,20 +7726,20 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>07/09/2026 18:53</t>
+          <t>07/10/2026 17:46</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
-        <v>19665.29</v>
+        <v>19693.95</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>-1.67</v>
+        <v>-1.53</v>
       </c>
       <c r="J66" s="7" t="n">
         <v>2.28</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>0.43</v>
+        <v>0.5</v>
       </c>
       <c r="L66" t="n">
         <v>20000</v>
@@ -7760,19 +7757,19 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="U66" s="7" t="n">
-        <v>-334.71</v>
+        <v>-306.05</v>
       </c>
       <c r="V66" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="W66" s="7" t="n">
-        <v>32.3943661971831</v>
+        <v>36.84210526315789</v>
       </c>
       <c r="X66" s="7" t="n">
-        <v>0.43</v>
+        <v>0.5</v>
       </c>
       <c r="Y66" s="7" t="n">
         <v>2.29</v>
@@ -7784,7 +7781,7 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
@@ -7829,7 +7826,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>07/09/2026 19:02</t>
+          <t>07/10/2026 17:55</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7929,7 +7926,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>07/09/2026 19:10</t>
+          <t>07/10/2026 18:00</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8029,7 +8026,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>07/09/2026 19:06</t>
+          <t>07/10/2026 17:57</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8129,7 +8126,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>07/09/2026 19:09</t>
+          <t>07/10/2026 18:00</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8229,7 +8226,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>07/09/2026 14:14</t>
+          <t>07/10/2026 18:08</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8338,7 +8335,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>07/09/2026 16:43</t>
+          <t>07/10/2026 20:56</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8556,14 +8553,14 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>07/09/2026 17:10</t>
+          <t>07/10/2026 21:27</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>28123.35</v>
+        <v>28143.62</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>-24.51</v>
+        <v>-24.49</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>32.64</v>
@@ -8581,31 +8578,31 @@
         <v>40</v>
       </c>
       <c r="O74" s="7" t="n">
-        <v>81.72</v>
+        <v>119.2</v>
       </c>
       <c r="P74" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q74" s="7" t="n">
-        <v>90</v>
+        <v>92.5</v>
       </c>
       <c r="R74" s="7" t="n">
-        <v>1.561533704390847</v>
+        <v>2.045705763663479</v>
       </c>
       <c r="S74" s="7" t="n">
         <v>0.45</v>
       </c>
       <c r="T74" t="n">
-        <v>3182</v>
+        <v>3185</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>-6158.65</v>
+        <v>-6138.379999999998</v>
       </c>
       <c r="V74" t="n">
-        <v>1911</v>
+        <v>1915</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>60.05656819610308</v>
+        <v>60.12558869701727</v>
       </c>
       <c r="X74" s="7" t="n">
         <v>0.8</v>
@@ -8620,7 +8617,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8938,7 +8935,7 @@
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>07/07/2026 02:40</t>
+          <t>07/10/2026 02:42</t>
         </is>
       </c>
       <c r="H78" s="9" t="n">
@@ -9029,7 +9026,7 @@
       </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>07/06/2026 22:58</t>
+          <t>07/09/2026 23:04</t>
         </is>
       </c>
       <c r="H79" s="9" t="n">
@@ -9211,7 +9208,7 @@
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>07/09/2026 18:34</t>
+          <t>07/10/2026 22:59</t>
         </is>
       </c>
       <c r="H81" s="9" t="n">
@@ -9484,20 +9481,20 @@
       </c>
       <c r="G84" s="8" t="inlineStr">
         <is>
-          <t>07/09/2026 18:34</t>
+          <t>07/10/2026 22:57</t>
         </is>
       </c>
       <c r="H84" s="9" t="n">
-        <v>19608.54</v>
+        <v>19611.91</v>
       </c>
       <c r="I84" s="9" t="n">
-        <v>-1.96</v>
+        <v>-1.95</v>
       </c>
       <c r="J84" s="9" t="n">
         <v>1.99</v>
       </c>
       <c r="K84" s="9" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="L84" s="8" t="n">
         <v>20000</v>
@@ -9569,14 +9566,14 @@
       </c>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t>07/09/2026 18:05</t>
+          <t>07/10/2026 22:26</t>
         </is>
       </c>
       <c r="H85" s="9" t="n">
-        <v>19620.9</v>
+        <v>19608.93</v>
       </c>
       <c r="I85" s="9" t="n">
-        <v>-1.9</v>
+        <v>-1.96</v>
       </c>
       <c r="J85" s="9" t="n">
         <v>2.27</v>
@@ -9654,20 +9651,20 @@
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>07/09/2026 18:25</t>
+          <t>07/10/2026 22:50</t>
         </is>
       </c>
       <c r="H86" s="9" t="n">
-        <v>21628.34</v>
+        <v>21459.86</v>
       </c>
       <c r="I86" s="9" t="n">
-        <v>8.15</v>
+        <v>7.31</v>
       </c>
       <c r="J86" s="9" t="n">
         <v>5.86</v>
       </c>
       <c r="K86" s="9" t="n">
-        <v>1.3</v>
+        <v>1.26</v>
       </c>
       <c r="L86" s="8" t="n">
         <v>20000</v>
@@ -9739,7 +9736,7 @@
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>07/09/2026 18:15</t>
+          <t>07/10/2026 22:38</t>
         </is>
       </c>
       <c r="H87" s="9" t="n">
@@ -9824,7 +9821,7 @@
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>07/09/2026 19:06</t>
+          <t>07/10/2026 17:57</t>
         </is>
       </c>
       <c r="H88" s="9" t="n">
@@ -10480,7 +10477,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>07/07/2026 02:40</t>
+          <t>07/10/2026 02:42</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -10521,7 +10518,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>07/06/2026 22:58</t>
+          <t>07/09/2026 23:04</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -10603,7 +10600,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>07/09/2026 18:34</t>
+          <t>07/10/2026 22:59</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -10726,14 +10723,14 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>07/09/2026 18:34</t>
+          <t>07/10/2026 22:57</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>19608.54</v>
+        <v>19611.91</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>-1.96</v>
+        <v>-1.95</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -10767,14 +10764,14 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>07/09/2026 18:05</t>
+          <t>07/10/2026 22:26</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>19620.9</v>
+        <v>19608.93</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>-1.9</v>
+        <v>-1.96</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -10808,14 +10805,14 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>07/09/2026 18:25</t>
+          <t>07/10/2026 22:50</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>21628.34</v>
+        <v>21459.86</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>8.15</v>
+        <v>7.31</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -10849,7 +10846,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>07/09/2026 18:15</t>
+          <t>07/10/2026 22:38</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -10890,7 +10887,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>07/09/2026 19:06</t>
+          <t>07/10/2026 17:57</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -12018,7 +12015,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>07/07/2026 03:21</t>
+          <t>07/10/2026 03:23</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -12156,7 +12153,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>07/04/2026 00:23</t>
+          <t>07/10/2026 00:29</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -12179,7 +12176,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>07/04/2026 11:09</t>
+          <t>07/10/2026 11:17</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -12386,7 +12383,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07/09/2026 15:48</t>
+          <t>07/10/2026 19:59</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -12432,7 +12429,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>07/09/2026 18:33</t>
+          <t>07/10/2026 22:55</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
@@ -12478,7 +12475,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07/09/2026 19:04</t>
+          <t>07/10/2026 17:56</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -12501,11 +12498,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07/09/2026 19:08</t>
+          <t>07/10/2026 17:58</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20097.65</v>
+        <v>19777.82</v>
       </c>
     </row>
     <row r="27">
@@ -12524,7 +12521,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>07/09/2026 19:11</t>
+          <t>07/10/2026 18:00</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -12547,11 +12544,11 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>07/09/2026 22:10</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>19701</v>
+          <t>07/10/2026 20:27</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>19399.89</v>
       </c>
     </row>
     <row r="29">
@@ -12570,11 +12567,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>07/09/2026 22:12</t>
+          <t>07/10/2026 20:31</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>19426.47</v>
+        <v>19357.79</v>
       </c>
     </row>
     <row r="30">
@@ -12593,11 +12590,11 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>07/09/2026 16:19</t>
+          <t>07/10/2026 20:32</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>19459.64</v>
+        <v>19473.23</v>
       </c>
     </row>
     <row r="31">
@@ -12616,11 +12613,11 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>07/09/2026 22:10</t>
+          <t>07/10/2026 20:31</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>20022.45</v>
+        <v>20035.96</v>
       </c>
     </row>
     <row r="32">
@@ -12639,11 +12636,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>07/09/2026 09:59</t>
+          <t>07/10/2026 20:32</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>19934.89</v>
+        <v>19397.24</v>
       </c>
     </row>
     <row r="33">
@@ -12662,11 +12659,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>07/09/2026 19:25</t>
+          <t>07/10/2026 18:10</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>19922.09</v>
+        <v>19936.96</v>
       </c>
     </row>
     <row r="34">
@@ -12685,11 +12682,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>07/09/2026 19:18</t>
+          <t>07/10/2026 18:05</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>19907.74</v>
+        <v>19939.37</v>
       </c>
     </row>
     <row r="35">
@@ -12708,11 +12705,11 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>07/09/2026 19:13</t>
+          <t>07/10/2026 13:04</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>19828.3</v>
+        <v>19875.04</v>
       </c>
     </row>
     <row r="36">
@@ -12731,11 +12728,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>07/09/2026 19:12</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>19951</v>
+          <t>07/10/2026 18:01</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>19977.64</v>
       </c>
     </row>
     <row r="37">
@@ -12754,11 +12751,11 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>07/09/2026 19:17</t>
+          <t>07/10/2026 18:03</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>20551.07</v>
+        <v>20745.34</v>
       </c>
     </row>
     <row r="38">
@@ -12777,11 +12774,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>07/09/2026 19:16</t>
+          <t>07/10/2026 18:05</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>19842.98</v>
+        <v>19857.14</v>
       </c>
     </row>
     <row r="39">
@@ -12800,11 +12797,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>07/09/2026 19:16</t>
+          <t>07/10/2026 18:04</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>20100.93</v>
+        <v>20060.71</v>
       </c>
     </row>
     <row r="40">
@@ -12823,11 +12820,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>07/09/2026 19:20</t>
+          <t>07/10/2026 18:06</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>19858.37</v>
+        <v>19849.25</v>
       </c>
     </row>
     <row r="41">
@@ -12846,11 +12843,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>07/09/2026 19:20</t>
+          <t>07/10/2026 18:07</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>22190.52</v>
+        <v>23041.53</v>
       </c>
     </row>
     <row r="42">
@@ -12869,11 +12866,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>07/09/2026 19:22</t>
+          <t>07/10/2026 18:07</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>19008.57</v>
+        <v>19215.86</v>
       </c>
     </row>
     <row r="43">
@@ -12892,11 +12889,11 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>07/09/2026 19:16</t>
+          <t>07/10/2026 18:04</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>20228.42</v>
+        <v>20135.23</v>
       </c>
     </row>
     <row r="44">
@@ -12915,11 +12912,11 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>07/09/2026 19:20</t>
+          <t>07/10/2026 18:08</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>19856.82</v>
+        <v>19848.24</v>
       </c>
     </row>
     <row r="45">
@@ -12938,7 +12935,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>07/09/2026 19:57</t>
+          <t>07/10/2026 18:33</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
@@ -13053,7 +13050,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>07/09/2026 07:43</t>
+          <t>07/10/2026 07:54</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-07-21
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -3510,16 +3510,16 @@
         <v>516</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-4156.07</v>
+        <v>-4154.81</v>
       </c>
       <c r="V25" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>36.04651162790697</v>
+        <v>36.43410852713178</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>21.17</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>07/20/2026 15:53</t>
+          <t>07/21/2026 00:25</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -5351,16 +5351,16 @@
         <v>0.48</v>
       </c>
       <c r="T42" t="n">
-        <v>1485</v>
+        <v>1486</v>
       </c>
       <c r="U42" s="7" t="n">
-        <v>-860.1100000000001</v>
+        <v>-862.1700000000001</v>
       </c>
       <c r="V42" t="n">
         <v>673</v>
       </c>
       <c r="W42" s="7" t="n">
-        <v>45.31986531986532</v>
+        <v>45.28936742934051</v>
       </c>
       <c r="X42" s="7" t="n">
         <v>0.74</v>
@@ -5375,7 +5375,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
@@ -6542,22 +6542,13 @@
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>17.65000000000002</v>
+        <v>0</v>
       </c>
       <c r="P54" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q54" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R54" s="7" t="n">
-        <v>1.045693426877573</v>
-      </c>
-      <c r="S54" s="7" t="n">
-        <v>0.86</v>
+        <v>0</v>
       </c>
       <c r="T54" t="n">
         <v>154</v>
@@ -6651,22 +6642,13 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>-8.610000000000001</v>
+        <v>0</v>
       </c>
       <c r="P55" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q55" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R55" s="7" t="n">
-        <v>0.85986328125</v>
-      </c>
-      <c r="S55" s="7" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="T55" t="n">
         <v>895</v>
@@ -6969,16 +6951,16 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>2697</v>
+        <v>2700</v>
       </c>
       <c r="U58" s="7" t="n">
-        <v>-2507.41</v>
+        <v>-2508.42</v>
       </c>
       <c r="V58" t="n">
         <v>1144</v>
       </c>
       <c r="W58" s="7" t="n">
-        <v>42.41750092695587</v>
+        <v>42.37037037037037</v>
       </c>
       <c r="X58" s="7" t="n">
         <v>0.66</v>
@@ -6993,7 +6975,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="AB58" t="inlineStr">
@@ -7069,16 +7051,16 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="U59" s="7" t="n">
-        <v>-40.95999999999999</v>
+        <v>-41.11999999999999</v>
       </c>
       <c r="V59" t="n">
         <v>49</v>
       </c>
       <c r="W59" s="7" t="n">
-        <v>39.83739837398374</v>
+        <v>39.51612903225806</v>
       </c>
       <c r="X59" s="7" t="n">
         <v>0.84</v>
@@ -7093,7 +7075,7 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -7169,16 +7151,16 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>4236</v>
+        <v>4238</v>
       </c>
       <c r="U60" s="7" t="n">
-        <v>-1695.46</v>
+        <v>-1695.62</v>
       </c>
       <c r="V60" t="n">
         <v>1939</v>
       </c>
       <c r="W60" s="7" t="n">
-        <v>45.77431539187914</v>
+        <v>45.75271354412458</v>
       </c>
       <c r="X60" s="7" t="n">
         <v>0.87</v>
@@ -7193,7 +7175,7 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
@@ -7272,7 +7254,7 @@
         <v>2467</v>
       </c>
       <c r="U61" s="7" t="n">
-        <v>-546.7599999999995</v>
+        <v>-546.8399999999997</v>
       </c>
       <c r="V61" t="n">
         <v>1113</v>
@@ -7672,7 +7654,7 @@
         <v>1961</v>
       </c>
       <c r="U65" s="7" t="n">
-        <v>-212.0500000000001</v>
+        <v>-212.2100000000001</v>
       </c>
       <c r="V65" t="n">
         <v>829</v>
@@ -7769,16 +7751,16 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="U66" s="7" t="n">
-        <v>-436.6200000000001</v>
+        <v>-436.7000000000001</v>
       </c>
       <c r="V66" t="n">
         <v>37</v>
       </c>
       <c r="W66" s="7" t="n">
-        <v>36.63366336633663</v>
+        <v>35.92233009708738</v>
       </c>
       <c r="X66" s="7" t="n">
         <v>0.47</v>
@@ -7793,7 +7775,7 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
@@ -12953,7 +12935,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>07/20/2026 16:03</t>
+          <t>07/21/2026 00:37</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-07-31
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>07/30/2026 19:50</t>
+          <t>07/31/2026 01:06</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>07/30/2026 20:01</t>
+          <t>07/31/2026 01:16</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>07/30/2026 18:49</t>
+          <t>07/31/2026 00:06</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4685,13 +4685,22 @@
         <v>0</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>0</v>
+        <v>-1183.74</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q36" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R36" s="7" t="n">
+        <v>0.5468330685450682</v>
+      </c>
+      <c r="S36" s="7" t="n">
+        <v>7.86</v>
       </c>
       <c r="T36" t="n">
         <v>62</v>
@@ -4872,7 +4881,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>07/30/2026 19:31</t>
+          <t>07/31/2026 00:44</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4981,7 +4990,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>07/30/2026 19:18</t>
+          <t>07/31/2026 00:33</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5439,13 +5448,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-43.82</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.4502571822857859</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>0.24</v>
       </c>
       <c r="T43" t="n">
         <v>3587</v>
@@ -5539,13 +5557,22 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-810.7099999999999</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.53316787783165</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>5.58</v>
       </c>
       <c r="T44" t="n">
         <v>52</v>
@@ -5639,13 +5666,22 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-194.21</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.6693903954513729</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>2.26</v>
       </c>
       <c r="T45" t="n">
         <v>271</v>
@@ -5739,13 +5775,22 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>19981.27</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q46" s="7" t="n">
+        <v>30.3030303030303</v>
+      </c>
+      <c r="R46" s="7" t="n">
+        <v>335.5265360790223</v>
+      </c>
+      <c r="S46" s="7" t="n">
+        <v>0.1</v>
       </c>
       <c r="T46" t="n">
         <v>32</v>
@@ -5777,7 +5822,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5839,13 +5884,22 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>-266.67</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q47" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R47" s="7" t="n">
+        <v>0.8367003263911427</v>
+      </c>
+      <c r="S47" s="7" t="n">
+        <v>4.35</v>
       </c>
       <c r="T47" t="n">
         <v>55</v>
@@ -5939,13 +5993,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>-834.4100000000001</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>0.04346978780965918</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>4.18</v>
       </c>
       <c r="T48" t="n">
         <v>171</v>
@@ -6039,13 +6102,22 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>0</v>
+        <v>264.21</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="Q49" s="7" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="R49" s="7" t="n">
+        <v>1.939046061984646</v>
+      </c>
+      <c r="S49" s="7" t="n">
+        <v>0.6</v>
       </c>
       <c r="T49" t="n">
         <v>366</v>
@@ -6139,13 +6211,22 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>0</v>
+        <v>-138.4</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q50" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R50" s="7" t="n">
+        <v>0.7987494547040861</v>
+      </c>
+      <c r="S50" s="7" t="n">
+        <v>3.15</v>
       </c>
       <c r="T50" t="n">
         <v>1034</v>
@@ -6239,13 +6320,22 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>0</v>
+        <v>87.23</v>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="Q51" s="7" t="n">
+        <v>57.49999999999999</v>
+      </c>
+      <c r="R51" s="7" t="n">
+        <v>1.159723875267793</v>
+      </c>
+      <c r="S51" s="7" t="n">
+        <v>2.73</v>
       </c>
       <c r="T51" t="n">
         <v>1764</v>
@@ -6339,13 +6429,22 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>0</v>
+        <v>18130.51</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q52" s="7" t="n">
+        <v>27.77777777777778</v>
+      </c>
+      <c r="R52" s="7" t="n">
+        <v>6.593160679304654</v>
+      </c>
+      <c r="S52" s="7" t="n">
+        <v>4.97</v>
       </c>
       <c r="T52" t="n">
         <v>35</v>
@@ -6377,7 +6476,7 @@
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC52" t="inlineStr">
@@ -6439,13 +6538,22 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>0</v>
+        <v>195.07</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q53" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R53" s="7" t="n">
+        <v>2.87009874412808</v>
+      </c>
+      <c r="S53" s="7" t="n">
+        <v>0.24</v>
       </c>
       <c r="T53" t="n">
         <v>178</v>
@@ -6539,13 +6647,22 @@
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>0</v>
+        <v>72.85000000000002</v>
       </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q54" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R54" s="7" t="n">
+        <v>1.353829714896304</v>
+      </c>
+      <c r="S54" s="7" t="n">
+        <v>0.95</v>
       </c>
       <c r="T54" t="n">
         <v>177</v>
@@ -6639,13 +6756,22 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>0</v>
+        <v>-28.38</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q55" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R55" s="7" t="n">
+        <v>0.6109130792432137</v>
+      </c>
+      <c r="S55" s="7" t="n">
+        <v>0.16</v>
       </c>
       <c r="T55" t="n">
         <v>1149</v>
@@ -6739,13 +6865,22 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O56" s="7" t="n">
-        <v>0</v>
+        <v>-71.33</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q56" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R56" s="7" t="n">
+        <v>0.383331892452667</v>
+      </c>
+      <c r="S56" s="7" t="n">
+        <v>0.4</v>
       </c>
       <c r="T56" t="n">
         <v>966</v>
@@ -6839,13 +6974,22 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>-9.800000000000001</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>0.7376171352074966</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.09</v>
       </c>
       <c r="T57" t="n">
         <v>582</v>
@@ -6939,19 +7083,28 @@
         <v>0</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O58" s="7" t="n">
-        <v>0</v>
+        <v>-44.8</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q58" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R58" s="7" t="n">
+        <v>0.6110435839555478</v>
+      </c>
+      <c r="S58" s="7" t="n">
+        <v>0.42</v>
       </c>
       <c r="T58" t="n">
         <v>3661</v>
       </c>
       <c r="U58" s="7" t="n">
-        <v>-2769.45</v>
+        <v>-2796.05</v>
       </c>
       <c r="V58" t="n">
         <v>1565</v>
@@ -7039,13 +7192,22 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>0</v>
+        <v>21.17</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q59" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R59" s="7" t="n">
+        <v>1.195331241926555</v>
+      </c>
+      <c r="S59" s="7" t="n">
+        <v>0.28</v>
       </c>
       <c r="T59" t="n">
         <v>175</v>
@@ -7139,19 +7301,28 @@
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O60" s="7" t="n">
-        <v>0</v>
+        <v>-20.5</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q60" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R60" s="7" t="n">
+        <v>0.6654153745715684</v>
+      </c>
+      <c r="S60" s="7" t="n">
+        <v>0.19</v>
       </c>
       <c r="T60" t="n">
         <v>5622</v>
       </c>
       <c r="U60" s="7" t="n">
-        <v>-1442.03</v>
+        <v>-1445.08</v>
       </c>
       <c r="V60" t="n">
         <v>2627</v>
@@ -7239,19 +7410,28 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O61" s="7" t="n">
-        <v>0</v>
+        <v>-48.95</v>
       </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q61" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R61" s="7" t="n">
+        <v>0.6329208848893889</v>
+      </c>
+      <c r="S61" s="7" t="n">
+        <v>0.44</v>
       </c>
       <c r="T61" t="n">
         <v>3205</v>
       </c>
       <c r="U61" s="7" t="n">
-        <v>-444.8000000000001</v>
+        <v>-445.2500000000002</v>
       </c>
       <c r="V61" t="n">
         <v>1489</v>
@@ -7339,13 +7519,22 @@
         <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O62" s="7" t="n">
-        <v>0</v>
+        <v>-422.29</v>
       </c>
       <c r="P62" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q62" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R62" s="7" t="n">
+        <v>0.2682043461685093</v>
+      </c>
+      <c r="S62" s="7" t="n">
+        <v>2.11</v>
       </c>
       <c r="T62" t="n">
         <v>157</v>
@@ -7439,13 +7628,22 @@
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>0</v>
+        <v>19072.55</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="Q63" s="7" t="n">
+        <v>14.28571428571428</v>
+      </c>
+      <c r="R63" s="7" t="n">
+        <v>13.61553878412255</v>
+      </c>
+      <c r="S63" s="7" t="n">
+        <v>3.36</v>
       </c>
       <c r="T63" t="n">
         <v>27</v>
@@ -7477,7 +7675,7 @@
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC63" t="inlineStr">
@@ -7539,13 +7737,22 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>0</v>
+        <v>-533.6900000000001</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q64" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R64" s="7" t="n">
+        <v>0.2773128588451955</v>
+      </c>
+      <c r="S64" s="7" t="n">
+        <v>2.69</v>
       </c>
       <c r="T64" t="n">
         <v>154</v>
@@ -7639,13 +7846,22 @@
         <v>0</v>
       </c>
       <c r="N65" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O65" s="7" t="n">
-        <v>0</v>
+        <v>-13.14</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q65" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R65" s="7" t="n">
+        <v>0.8846153846153846</v>
+      </c>
+      <c r="S65" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="T65" t="n">
         <v>2685</v>
@@ -7739,13 +7955,22 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>0</v>
+        <v>61.29999999999999</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q66" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R66" s="7" t="n">
+        <v>1.122720265860543</v>
+      </c>
+      <c r="S66" s="7" t="n">
+        <v>1.82</v>
       </c>
       <c r="T66" t="n">
         <v>144</v>
@@ -7839,13 +8064,22 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>0</v>
+        <v>-332.67</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q67" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R67" s="7" t="n">
+        <v>0.6066940165281439</v>
+      </c>
+      <c r="S67" s="7" t="n">
+        <v>2.14</v>
       </c>
       <c r="T67" t="n">
         <v>138</v>
@@ -7939,13 +8173,22 @@
         <v>0</v>
       </c>
       <c r="N68" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O68" s="7" t="n">
-        <v>0</v>
+        <v>-35.83</v>
       </c>
       <c r="P68" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q68" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R68" s="7" t="n">
+        <v>0.5722812462695476</v>
+      </c>
+      <c r="S68" s="7" t="n">
+        <v>0.2</v>
       </c>
       <c r="T68" t="n">
         <v>55</v>
@@ -8039,13 +8282,22 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>0</v>
+        <v>71.06</v>
       </c>
       <c r="P69" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q69" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R69" s="7" t="n">
+        <v>2.289187227866473</v>
+      </c>
+      <c r="S69" s="7" t="n">
+        <v>0.14</v>
       </c>
       <c r="T69" t="n">
         <v>271</v>
@@ -8139,13 +8391,22 @@
         <v>0</v>
       </c>
       <c r="N70" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O70" s="7" t="n">
-        <v>0</v>
+        <v>19946.4</v>
       </c>
       <c r="P70" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="Q70" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R70" s="7" t="n">
+        <v>278.6503340757238</v>
+      </c>
+      <c r="S70" s="7" t="n">
+        <v>0.17</v>
       </c>
       <c r="T70" t="n">
         <v>7</v>
@@ -8177,7 +8438,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC70" t="inlineStr">
@@ -8581,7 +8842,7 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>3289</v>
+        <v>3290</v>
       </c>
       <c r="U74" s="7" t="n">
         <v>-7504.150000000001</v>
@@ -8590,7 +8851,7 @@
         <v>2008</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>61.05199148677409</v>
+        <v>61.03343465045593</v>
       </c>
       <c r="X74" s="7" t="n">
         <v>0.77</v>
@@ -8605,7 +8866,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -9582,17 +9843,23 @@
         <v>0</v>
       </c>
       <c r="N85" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O85" s="9" t="n">
-        <v>0</v>
+        <v>-194.21</v>
       </c>
       <c r="P85" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q85" s="8" t="n"/>
-      <c r="R85" s="8" t="n"/>
-      <c r="S85" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q85" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R85" s="9" t="n">
+        <v>0.6693903954513729</v>
+      </c>
+      <c r="S85" s="9" t="n">
+        <v>2.26</v>
+      </c>
       <c r="T85" s="8" t="n">
         <v>0</v>
       </c>
@@ -9667,17 +9934,23 @@
         <v>0</v>
       </c>
       <c r="N86" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O86" s="9" t="n">
-        <v>0</v>
+        <v>91.75999999999996</v>
       </c>
       <c r="P86" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q86" s="8" t="n"/>
-      <c r="R86" s="8" t="n"/>
-      <c r="S86" s="8" t="n"/>
+        <v>22</v>
+      </c>
+      <c r="Q86" s="9" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R86" s="9" t="n">
+        <v>1.170605187319885</v>
+      </c>
+      <c r="S86" s="9" t="n">
+        <v>2.69</v>
+      </c>
       <c r="T86" s="8" t="n">
         <v>0</v>
       </c>
@@ -9752,17 +10025,23 @@
         <v>0</v>
       </c>
       <c r="N87" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O87" s="9" t="n">
-        <v>0</v>
+        <v>3326.65</v>
       </c>
       <c r="P87" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q87" s="8" t="n"/>
-      <c r="R87" s="8" t="n"/>
-      <c r="S87" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="Q87" s="9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="R87" s="9" t="n">
+        <v>8.896717069812709</v>
+      </c>
+      <c r="S87" s="9" t="n">
+        <v>1.04</v>
+      </c>
       <c r="T87" s="8" t="n">
         <v>0</v>
       </c>
@@ -9837,17 +10116,23 @@
         <v>0</v>
       </c>
       <c r="N88" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O88" s="9" t="n">
-        <v>0</v>
+        <v>-58.49</v>
       </c>
       <c r="P88" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q88" s="8" t="n"/>
-      <c r="R88" s="8" t="n"/>
-      <c r="S88" s="8" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="Q88" s="9" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R88" s="9" t="n">
+        <v>0.2666750250752257</v>
+      </c>
+      <c r="S88" s="9" t="n">
+        <v>0.32</v>
+      </c>
       <c r="T88" s="8" t="n">
         <v>0</v>
       </c>
@@ -10768,7 +11053,7 @@
         <v>2.24</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
@@ -10809,7 +11094,7 @@
         <v>-6.66</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -10850,7 +11135,7 @@
         <v>-5.87</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
@@ -10891,7 +11176,7 @@
         <v>-0.16</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -12377,7 +12662,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>07/30/2026 19:59</t>
+          <t>07/31/2026 01:15</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-04
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-03 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-04 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/03/2026 04:31</t>
+          <t>08/04/2026 19:32</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>54210.88</v>
+        <v>34401.88</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>148.59</v>
+        <v>57.75</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>74.43000000000001</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.11</v>
+        <v>1.05</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>1445.4</v>
+        <v>-23560.95</v>
       </c>
       <c r="P2" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>65</v>
+        <v>52.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.228827445361788</v>
+        <v>0.421791637422021</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>16.37</v>
+        <v>97</v>
       </c>
       <c r="T2" t="n">
-        <v>3271</v>
+        <v>3284</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>40063.83999999998</v>
+        <v>9401.879999999983</v>
       </c>
       <c r="V2" t="n">
-        <v>2053</v>
+        <v>2058</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>62.76368083154998</v>
+        <v>62.66747868453106</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.11</v>
+        <v>1.02</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>74.43000000000001</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/01/2026 19:12</t>
+          <t>08/04/2026 19:14</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/03/2026 08:40</t>
+          <t>08/04/2026 17:12</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08/01/2026 09:25</t>
+          <t>08/04/2026 09:34</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/01/2026 14:37</t>
+          <t>08/04/2026 14:44</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>07/31/2026 21:24</t>
+          <t>08/03/2026 22:43</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>07/31/2026 21:28</t>
+          <t>08/03/2026 22:50</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/03/2026 11:34</t>
+          <t>08/04/2026 20:11</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/03/2026 06:09</t>
+          <t>08/04/2026 21:31</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,17 +2486,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/03/2026 08:58</t>
+          <t>08/04/2026 17:37</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>78.59999999999999</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-99.58</v>
+        <v>-99.59</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>99.58</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>0.7</v>
@@ -2511,37 +2511,37 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-4.94</v>
+        <v>-5.95</v>
       </c>
       <c r="P16" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.5258964143426295</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="T16" t="n">
-        <v>2290</v>
+        <v>2293</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-20343.8</v>
+        <v>-20345.66</v>
       </c>
       <c r="V16" t="n">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>32.13973799126638</v>
+        <v>32.14129960750109</v>
       </c>
       <c r="X16" s="7" t="n">
         <v>0.7</v>
       </c>
       <c r="Y16" s="7" t="n">
-        <v>99.62</v>
+        <v>99.63</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/01/2026 09:06</t>
+          <t>08/04/2026 09:08</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/03/2026 06:03</t>
+          <t>08/04/2026 21:22</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/03/2026 11:45</t>
+          <t>08/04/2026 20:13</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3289,7 +3289,7 @@
         <v>4.26</v>
       </c>
       <c r="T23" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="U23" s="7" t="n">
         <v>-448.4799999999997</v>
@@ -3298,7 +3298,7 @@
         <v>36</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>51.42857142857142</v>
+        <v>50.70422535211267</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>0.88</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3467,20 +3467,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/03/2026 05:31</t>
+          <t>08/04/2026 20:51</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16172.66</v>
+        <v>16095.96</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-19.71</v>
+        <v>-19.23</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3492,31 +3492,31 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>-100.8</v>
+        <v>159.29</v>
       </c>
       <c r="P25" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>37.5</v>
+        <v>45</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>0.8284488920657612</v>
+        <v>1.305381415233604</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>1.05</v>
+        <v>0.95</v>
       </c>
       <c r="T25" t="n">
-        <v>594</v>
+        <v>603</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3852.9</v>
+        <v>-3904.04</v>
       </c>
       <c r="V25" t="n">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>38.04713804713805</v>
+        <v>37.81094527363184</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>0.61</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/03/2026 10:03</t>
+          <t>08/04/2026 18:37</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,14 +3685,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/03/2026 05:28</t>
+          <t>08/04/2026 20:46</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20458.27</v>
+        <v>20439.59</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-2.17</v>
+        <v>-2.26</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>7.39</v>
@@ -3710,22 +3710,22 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-692.9399999999999</v>
+        <v>-711.8199999999999</v>
       </c>
       <c r="P27" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>50</v>
+        <v>47.5</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.6960696161724264</v>
+        <v>0.690325892604661</v>
       </c>
       <c r="S27" s="7" t="n">
         <v>6.74</v>
       </c>
       <c r="T27" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="U27" s="7" t="n">
         <v>439.5900000000001</v>
@@ -3734,7 +3734,7 @@
         <v>42</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>45.65217391304348</v>
+        <v>45.16129032258064</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>1.1</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/03/2026 05:38</t>
+          <t>08/04/2026 20:52</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08/01/2026 09:42</t>
+          <t>08/04/2026 09:47</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,20 +4121,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/03/2026 05:42</t>
+          <t>08/04/2026 21:04</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
         <v>20681.21</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>3.57</v>
+        <v>3.43</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>1.09</v>
       </c>
-      <c r="K31" s="7" t="n">
-        <v>2.08</v>
+      <c r="K31" t="n">
+        <v>2</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -4146,19 +4146,19 @@
         <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>305.96</v>
+        <v>-157.92</v>
       </c>
       <c r="P31" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q31" s="7" t="n">
-        <v>35</v>
+        <v>32.5</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>1.59630863980978</v>
+        <v>0.7079503633976291</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="T31" t="n">
         <v>66</v>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/03/2026 12:38</t>
+          <t>08/04/2026 20:27</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/03/2026 08:22</t>
+          <t>08/04/2026 17:02</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20231.41</v>
+        <v>20209.64</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>1.15</v>
+        <v>1.04</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>2.87</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,7 +4473,7 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-28.73999999999999</v>
+        <v>-86.09999999999999</v>
       </c>
       <c r="P34" t="n">
         <v>15</v>
@@ -4482,25 +4482,25 @@
         <v>37.5</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.9727887291938874</v>
+        <v>0.9210707246642528</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>1.53</v>
+        <v>1.7</v>
       </c>
       <c r="T34" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>259.7200000000001</v>
+        <v>209.64</v>
       </c>
       <c r="V34" t="n">
         <v>38</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>43.67816091954023</v>
+        <v>43.18181818181818</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1.13</v>
+        <v>1.1</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>2.88</v>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/03/2026 07:00</t>
+          <t>08/04/2026 22:16</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/03/2026 06:48</t>
+          <t>08/04/2026 22:06</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19856.88</v>
+        <v>19757.28</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.72</v>
+        <v>-1.22</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>7.48</v>
+        <v>8.41</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,22 +4697,22 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-241.1600000000002</v>
+        <v>-242.72</v>
       </c>
       <c r="V36" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>47.61904761904761</v>
+        <v>47.69230769230769</v>
       </c>
       <c r="X36" s="7" t="n">
         <v>0.93</v>
       </c>
       <c r="Y36" s="7" t="n">
-        <v>7.94</v>
+        <v>8.41</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,20 +4766,20 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/03/2026 06:19</t>
+          <t>08/04/2026 21:48</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>19525.97</v>
+        <v>20006.94</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-2.37</v>
+        <v>0.03</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>9.82</v>
       </c>
-      <c r="K37" s="7" t="n">
-        <v>0.9</v>
+      <c r="K37" t="n">
+        <v>1</v>
       </c>
       <c r="L37" t="n">
         <v>20000</v>
@@ -4791,7 +4791,7 @@
         <v>40</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>-1134.25</v>
+        <v>-1107.02</v>
       </c>
       <c r="P37" t="n">
         <v>16</v>
@@ -4800,25 +4800,25 @@
         <v>40</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>0.7142781571728337</v>
+        <v>0.7211374966307872</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>10.87</v>
+        <v>11.1</v>
       </c>
       <c r="T37" t="n">
         <v>52</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-474.0299999999999</v>
+        <v>6.940000000000168</v>
       </c>
       <c r="V37" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>40.38461538461539</v>
+        <v>42.30769230769231</v>
       </c>
       <c r="X37" s="7" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="Y37" s="7" t="n">
         <v>9.83</v>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/03/2026 07:49</t>
+          <t>08/04/2026 23:04</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/03/2026 07:31</t>
+          <t>08/04/2026 22:47</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>08/01/2026 09:12</t>
+          <t>08/04/2026 09:14</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>08/01/2026 07:13</t>
+          <t>08/04/2026 07:15</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,20 +5311,20 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/03/2026 11:51</t>
+          <t>08/04/2026 20:19</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
-        <v>18808.37</v>
+        <v>18662.81</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>-5.95</v>
+        <v>-6.67</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>6.26</v>
+        <v>6.99</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="L42" t="n">
         <v>20000</v>
@@ -5336,37 +5336,37 @@
         <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-69.67</v>
+        <v>-78.95999999999999</v>
       </c>
       <c r="P42" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="Q42" s="7" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>0.2772821576763486</v>
+        <v>0.2637762237762238</v>
       </c>
       <c r="S42" s="7" t="n">
-        <v>0.41</v>
+        <v>0.49</v>
       </c>
       <c r="T42" t="n">
-        <v>2091</v>
+        <v>2254</v>
       </c>
       <c r="U42" s="7" t="n">
-        <v>-1201.67</v>
+        <v>-1335.55</v>
       </c>
       <c r="V42" t="n">
-        <v>928</v>
+        <v>1010</v>
       </c>
       <c r="W42" s="7" t="n">
-        <v>44.38067910090865</v>
+        <v>44.80922803904171</v>
       </c>
       <c r="X42" s="7" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="Y42" s="7" t="n">
-        <v>6.36</v>
+        <v>6.92</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
@@ -5375,7 +5375,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
@@ -5420,20 +5420,20 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/03/2026 05:37</t>
+          <t>08/04/2026 20:55</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
-        <v>17751.78</v>
+        <v>17633.49</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>-11.22</v>
+        <v>-11.81</v>
       </c>
       <c r="J43" s="7" t="n">
-        <v>11.87</v>
+        <v>12.64</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="L43" t="n">
         <v>20000</v>
@@ -5451,22 +5451,22 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>3855</v>
+        <v>4058</v>
       </c>
       <c r="U43" s="7" t="n">
-        <v>-2283.13</v>
+        <v>-2371.88</v>
       </c>
       <c r="V43" t="n">
-        <v>1659</v>
+        <v>1759</v>
       </c>
       <c r="W43" s="7" t="n">
-        <v>43.03501945525292</v>
+        <v>43.34647609659931</v>
       </c>
       <c r="X43" s="7" t="n">
         <v>0.66</v>
       </c>
       <c r="Y43" s="7" t="n">
-        <v>12.1</v>
+        <v>12.67</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
@@ -5520,20 +5520,20 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/03/2026 12:56</t>
+          <t>08/04/2026 20:35</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
-        <v>19554.23</v>
+        <v>19437.41</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>-2.22</v>
+        <v>-2.8</v>
       </c>
       <c r="J44" s="7" t="n">
-        <v>5.06</v>
+        <v>5.09</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>0.78</v>
+        <v>0.73</v>
       </c>
       <c r="L44" t="n">
         <v>20000</v>
@@ -5542,40 +5542,31 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-863.15</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>0.5119420538975652</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>5.57</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="U44" s="7" t="n">
-        <v>-445.7699999999999</v>
+        <v>-562.5899999999999</v>
       </c>
       <c r="V44" t="n">
         <v>24</v>
       </c>
       <c r="W44" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>42.10526315789473</v>
       </c>
       <c r="X44" s="7" t="n">
-        <v>0.78</v>
+        <v>0.73</v>
       </c>
       <c r="Y44" s="7" t="n">
-        <v>5.07</v>
+        <v>5.1</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -5584,7 +5575,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5629,20 +5620,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/03/2026 05:35</t>
+          <t>08/04/2026 20:54</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19908.37</v>
+        <v>19983.72</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.44</v>
+        <v>-0.06</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>3.15</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5651,37 +5642,28 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-210.87</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.6223066038580717</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>1.49</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-47.06000000000009</v>
+        <v>-16.27999999999997</v>
       </c>
       <c r="V45" t="n">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>54.63659147869674</v>
+        <v>55.66502463054187</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="Y45" s="7" t="n">
         <v>3.15</v>
@@ -5693,7 +5675,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5738,7 +5720,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/03/2026 11:34</t>
+          <t>08/04/2026 20:12</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5838,7 +5820,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/03/2026 12:49</t>
+          <t>08/04/2026 20:39</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5938,20 +5920,20 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/03/2026 11:29</t>
+          <t>08/04/2026 20:05</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
-        <v>19283.45</v>
+        <v>20194.85</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>-3.58</v>
+        <v>0.98</v>
       </c>
       <c r="J48" s="7" t="n">
         <v>3.89</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>0.53</v>
+        <v>1.13</v>
       </c>
       <c r="L48" t="n">
         <v>20000</v>
@@ -5969,19 +5951,19 @@
         <v>0</v>
       </c>
       <c r="T48" t="n">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="U48" s="7" t="n">
-        <v>-716.55</v>
+        <v>194.8499999999999</v>
       </c>
       <c r="V48" t="n">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="W48" s="7" t="n">
-        <v>45.08670520231214</v>
+        <v>50.77720207253886</v>
       </c>
       <c r="X48" s="7" t="n">
-        <v>0.53</v>
+        <v>1.13</v>
       </c>
       <c r="Y48" s="7" t="n">
         <v>3.89</v>
@@ -6038,17 +6020,17 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/03/2026 05:47</t>
+          <t>08/04/2026 21:06</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>19011.08</v>
+        <v>18939.49</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>-4.97</v>
+        <v>-5.32</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>6.5</v>
+        <v>6.85</v>
       </c>
       <c r="K49" s="7" t="n">
         <v>0.73</v>
@@ -6069,19 +6051,19 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>377</v>
+        <v>391</v>
       </c>
       <c r="U49" s="7" t="n">
-        <v>-1016.04</v>
+        <v>-826.1800000000001</v>
       </c>
       <c r="V49" t="n">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="W49" s="7" t="n">
-        <v>45.88859416445623</v>
+        <v>46.29156010230179</v>
       </c>
       <c r="X49" s="7" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="Y49" s="7" t="n">
         <v>6.61</v>
@@ -6093,7 +6075,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
@@ -6138,20 +6120,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/03/2026 05:31</t>
+          <t>08/04/2026 20:53</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>18143.87</v>
+        <v>17899.68</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>-9.300000000000001</v>
+        <v>-10.52</v>
       </c>
       <c r="J50" s="7" t="n">
-        <v>19.4</v>
+        <v>20.49</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6169,19 +6151,19 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>1067</v>
+        <v>1113</v>
       </c>
       <c r="U50" s="7" t="n">
-        <v>-1951.050000000001</v>
+        <v>-1192.400000000001</v>
       </c>
       <c r="V50" t="n">
-        <v>540</v>
+        <v>568</v>
       </c>
       <c r="W50" s="7" t="n">
-        <v>50.60918462980318</v>
+        <v>51.03324348607367</v>
       </c>
       <c r="X50" s="7" t="n">
-        <v>0.84</v>
+        <v>0.9</v>
       </c>
       <c r="Y50" s="7" t="n">
         <v>19.8</v>
@@ -6193,7 +6175,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
@@ -6238,20 +6220,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/03/2026 11:58</t>
+          <t>08/04/2026 20:18</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>15223.86</v>
+        <v>15674.58</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-23.72</v>
+        <v>-21.27</v>
       </c>
       <c r="J51" s="7" t="n">
-        <v>40.77</v>
+        <v>41.12</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.8</v>
+        <v>0.83</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6269,19 +6251,19 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>1829</v>
+        <v>1911</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-4835.040000000002</v>
+        <v>-3881.080000000002</v>
       </c>
       <c r="V51" t="n">
-        <v>897</v>
+        <v>937</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>49.04319300164024</v>
+        <v>49.03192046049189</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="Y51" s="7" t="n">
         <v>41.12</v>
@@ -6293,7 +6275,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6338,20 +6320,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/03/2026 11:40</t>
+          <t>08/04/2026 20:15</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>18170.91</v>
+        <v>18073.71</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-9.140000000000001</v>
+        <v>-9.630000000000001</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>10.18</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6372,7 +6354,7 @@
         <v>36</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-1829.09</v>
+        <v>-1926.29</v>
       </c>
       <c r="V52" t="n">
         <v>9</v>
@@ -6381,10 +6363,10 @@
         <v>25</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="Y52" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>10.19</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6438,14 +6420,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/03/2026 05:39</t>
+          <t>08/04/2026 20:58</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19876.42</v>
+        <v>19868.27</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-0.64</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6469,19 +6451,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-112.59</v>
+        <v>-131.73</v>
       </c>
       <c r="V53" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>38.21989528795812</v>
+        <v>37.56345177664975</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6493,7 +6475,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6538,14 +6520,14 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/03/2026 05:50</t>
+          <t>08/04/2026 21:08</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
-        <v>19737.19</v>
+        <v>19729.88</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>-1.29</v>
+        <v>-1.34</v>
       </c>
       <c r="J54" s="7" t="n">
         <v>4.63</v>
@@ -6569,19 +6551,19 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="U54" s="7" t="n">
-        <v>-209.05</v>
+        <v>-272.9600000000001</v>
       </c>
       <c r="V54" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="W54" s="7" t="n">
-        <v>42.48704663212435</v>
+        <v>43.13725490196079</v>
       </c>
       <c r="X54" s="7" t="n">
-        <v>0.89</v>
+        <v>0.86</v>
       </c>
       <c r="Y54" s="7" t="n">
         <v>4.63</v>
@@ -6593,7 +6575,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -6638,20 +6620,20 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/03/2026 05:34</t>
+          <t>08/04/2026 20:54</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
-        <v>19714.88</v>
+        <v>19710.36</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>-1.38</v>
+        <v>-1.4</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>2.46</v>
+        <v>2.68</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="L55" t="n">
         <v>20000</v>
@@ -6669,22 +6651,22 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>1223</v>
+        <v>1380</v>
       </c>
       <c r="U55" s="7" t="n">
-        <v>-281.7300000000001</v>
+        <v>-286.51</v>
       </c>
       <c r="V55" t="n">
-        <v>577</v>
+        <v>649</v>
       </c>
       <c r="W55" s="7" t="n">
-        <v>47.17906786590352</v>
+        <v>47.02898550724638</v>
       </c>
       <c r="X55" s="7" t="n">
         <v>0.89</v>
       </c>
       <c r="Y55" s="7" t="n">
-        <v>2.49</v>
+        <v>2.72</v>
       </c>
       <c r="Z55" t="inlineStr">
         <is>
@@ -6693,7 +6675,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -6738,20 +6720,20 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/03/2026 05:49</t>
+          <t>08/04/2026 21:13</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
-        <v>19700.55</v>
+        <v>19859.7</v>
       </c>
       <c r="I56" s="7" t="n">
-        <v>-1.52</v>
+        <v>-0.72</v>
       </c>
       <c r="J56" s="7" t="n">
         <v>1.98</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>0.88</v>
+        <v>0.95</v>
       </c>
       <c r="L56" t="n">
         <v>20000</v>
@@ -6769,19 +6751,19 @@
         <v>0</v>
       </c>
       <c r="T56" t="n">
-        <v>1030</v>
+        <v>1069</v>
       </c>
       <c r="U56" s="7" t="n">
-        <v>-279.77</v>
+        <v>-147.31</v>
       </c>
       <c r="V56" t="n">
-        <v>477</v>
+        <v>499</v>
       </c>
       <c r="W56" s="7" t="n">
-        <v>46.31067961165049</v>
+        <v>46.67913938260056</v>
       </c>
       <c r="X56" s="7" t="n">
-        <v>0.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y56" s="7" t="n">
         <v>1.95</v>
@@ -6793,7 +6775,7 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr">
@@ -6838,20 +6820,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/03/2026 11:50</t>
+          <t>08/04/2026 20:16</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19709.04</v>
+        <v>19752.74</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.48</v>
+        <v>-1.26</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.75</v>
+        <v>0.79</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6869,19 +6851,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>626</v>
+        <v>656</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-272.43</v>
+        <v>-250.1</v>
       </c>
       <c r="V57" t="n">
-        <v>267</v>
+        <v>285</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>42.6517571884984</v>
+        <v>43.44512195121951</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6893,7 +6875,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6938,20 +6920,20 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/03/2026 12:56</t>
+          <t>08/04/2026 20:35</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
-        <v>16953.45</v>
+        <v>17182.33</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>-15.23</v>
+        <v>-14.09</v>
       </c>
       <c r="J58" s="7" t="n">
         <v>15.49</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
       <c r="L58" t="n">
         <v>20000</v>
@@ -6969,19 +6951,19 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>4025</v>
+        <v>4197</v>
       </c>
       <c r="U58" s="7" t="n">
-        <v>-2984.79</v>
+        <v>-2827.43</v>
       </c>
       <c r="V58" t="n">
-        <v>1736</v>
+        <v>1817</v>
       </c>
       <c r="W58" s="7" t="n">
-        <v>43.1304347826087</v>
+        <v>43.29282821062664</v>
       </c>
       <c r="X58" s="7" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="Y58" s="7" t="n">
         <v>15.49</v>
@@ -6993,7 +6975,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB58" t="inlineStr">
@@ -7038,20 +7020,20 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/03/2026 05:31</t>
+          <t>08/04/2026 20:50</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
-        <v>20053.65</v>
+        <v>20155.01</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>0.28</v>
+        <v>0.78</v>
       </c>
       <c r="J59" s="7" t="n">
         <v>0.55</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>1.13</v>
+        <v>1.32</v>
       </c>
       <c r="L59" t="n">
         <v>20000</v>
@@ -7060,37 +7042,28 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>51.26</v>
+        <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q59" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R59" s="7" t="n">
-        <v>1.497380166893072</v>
-      </c>
-      <c r="S59" s="7" t="n">
-        <v>0.26</v>
+        <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>219</v>
+        <v>244</v>
       </c>
       <c r="U59" s="7" t="n">
-        <v>50.15000000000001</v>
+        <v>157.11</v>
       </c>
       <c r="V59" t="n">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="W59" s="7" t="n">
-        <v>43.37899543378995</v>
+        <v>44.67213114754098</v>
       </c>
       <c r="X59" s="7" t="n">
-        <v>1.11</v>
+        <v>1.33</v>
       </c>
       <c r="Y59" s="7" t="n">
         <v>0.55</v>
@@ -7102,7 +7075,7 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -7147,62 +7120,53 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/03/2026 05:33</t>
+          <t>08/04/2026 20:51</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>18807.41</v>
+        <v>20600.8</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-5.99</v>
+        <v>-3.13</v>
       </c>
       <c r="J60" s="7" t="n">
-        <v>18.87</v>
+        <v>19.42</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="L60" t="n">
-        <v>20000</v>
+        <v>0.97</v>
+      </c>
+      <c r="L60" s="7" t="n">
+        <v>21100.65</v>
       </c>
       <c r="M60" t="n">
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O60" s="7" t="n">
-        <v>150.94</v>
+        <v>0</v>
       </c>
       <c r="P60" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q60" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R60" s="7" t="n">
-        <v>4.541529798216799</v>
-      </c>
-      <c r="S60" s="7" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>5946</v>
+        <v>6152</v>
       </c>
       <c r="U60" s="7" t="n">
-        <v>-2636.24</v>
+        <v>-968.1199999999999</v>
       </c>
       <c r="V60" t="n">
-        <v>2803</v>
+        <v>2935</v>
       </c>
       <c r="W60" s="7" t="n">
-        <v>47.14093508240834</v>
+        <v>47.70806241872562</v>
       </c>
       <c r="X60" s="7" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="Y60" s="7" t="n">
-        <v>19.42</v>
+        <v>18.48</v>
       </c>
       <c r="Z60" t="inlineStr">
         <is>
@@ -7211,7 +7175,7 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
@@ -7256,23 +7220,23 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/03/2026 05:51</t>
+          <t>08/04/2026 21:17</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>19508.69</v>
+        <v>20626.92</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-2.43</v>
+        <v>-3.73</v>
       </c>
       <c r="J61" s="7" t="n">
-        <v>9.83</v>
+        <v>13.96</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L61" t="n">
-        <v>20000</v>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L61" s="7" t="n">
+        <v>21292.1</v>
       </c>
       <c r="M61" t="n">
         <v>0</v>
@@ -7287,22 +7251,22 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>3340</v>
+        <v>3453</v>
       </c>
       <c r="U61" s="7" t="n">
-        <v>-1926.38</v>
+        <v>-1065.33</v>
       </c>
       <c r="V61" t="n">
-        <v>1553</v>
+        <v>1618</v>
       </c>
       <c r="W61" s="7" t="n">
-        <v>46.49700598802396</v>
+        <v>46.85780480741384</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
       <c r="Y61" s="7" t="n">
-        <v>13.87</v>
+        <v>13.16</v>
       </c>
       <c r="Z61" t="inlineStr">
         <is>
@@ -7311,7 +7275,7 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
@@ -7356,7 +7320,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/03/2026 05:57</t>
+          <t>08/04/2026 21:16</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7456,14 +7420,14 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/03/2026 06:07</t>
+          <t>08/04/2026 21:20</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>19011.4</v>
+        <v>18994.6</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-4.96</v>
+        <v>-5.04</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>6.74</v>
@@ -7487,16 +7451,16 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-988.5999999999998</v>
+        <v>-1005.4</v>
       </c>
       <c r="V63" t="n">
         <v>3</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>10.71428571428571</v>
+        <v>10.3448275862069</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>0.37</v>
@@ -7511,7 +7475,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7556,20 +7520,20 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/03/2026 06:03</t>
+          <t>08/04/2026 21:24</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
-        <v>19247.92</v>
+        <v>19452.56</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>-3.76</v>
+        <v>-2.74</v>
       </c>
       <c r="J64" s="7" t="n">
-        <v>3.8</v>
+        <v>3.87</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>0.53</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L64" t="n">
         <v>20000</v>
@@ -7587,22 +7551,22 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="U64" s="7" t="n">
-        <v>-722.45</v>
+        <v>-520.42</v>
       </c>
       <c r="V64" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="W64" s="7" t="n">
-        <v>52.09580838323353</v>
+        <v>51.93370165745856</v>
       </c>
       <c r="X64" s="7" t="n">
-        <v>0.55</v>
+        <v>0.7</v>
       </c>
       <c r="Y64" s="7" t="n">
-        <v>3.8</v>
+        <v>3.88</v>
       </c>
       <c r="Z64" t="inlineStr">
         <is>
@@ -7611,7 +7575,7 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB64" t="inlineStr">
@@ -7656,20 +7620,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/03/2026 05:49</t>
+          <t>08/04/2026 21:06</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>18693.11</v>
+        <v>19150.72</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-6.51</v>
+        <v>-4.25</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>10.37</v>
+        <v>11.64</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7687,19 +7651,19 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>2833</v>
+        <v>2899</v>
       </c>
       <c r="U65" s="7" t="n">
-        <v>-1665.51</v>
+        <v>-1115.53</v>
       </c>
       <c r="V65" t="n">
-        <v>1296</v>
+        <v>1338</v>
       </c>
       <c r="W65" s="7" t="n">
-        <v>45.74655841863748</v>
+        <v>46.15384615384615</v>
       </c>
       <c r="X65" s="7" t="n">
-        <v>0.83</v>
+        <v>0.89</v>
       </c>
       <c r="Y65" s="7" t="n">
         <v>11.64</v>
@@ -7711,7 +7675,7 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB65" t="inlineStr">
@@ -7756,20 +7720,20 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/03/2026 05:47</t>
+          <t>08/04/2026 21:03</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
-        <v>19698.31</v>
+        <v>20319.13</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>-1.5</v>
+        <v>1.6</v>
       </c>
       <c r="J66" s="7" t="n">
         <v>2.86</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>0.78</v>
+        <v>1.23</v>
       </c>
       <c r="L66" t="n">
         <v>20000</v>
@@ -7787,19 +7751,19 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="U66" s="7" t="n">
-        <v>-301.8500000000001</v>
+        <v>137.24</v>
       </c>
       <c r="V66" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="W66" s="7" t="n">
-        <v>40.47619047619047</v>
+        <v>42.10526315789473</v>
       </c>
       <c r="X66" s="7" t="n">
-        <v>0.78</v>
+        <v>1.1</v>
       </c>
       <c r="Y66" s="7" t="n">
         <v>2.85</v>
@@ -7811,7 +7775,7 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
@@ -7856,20 +7820,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/03/2026 06:11</t>
+          <t>08/04/2026 21:32</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>19585.88</v>
+        <v>20121.18</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>-2.08</v>
+        <v>0.6</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>0.82</v>
+        <v>1.05</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7887,19 +7851,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>-356.5600000000001</v>
+        <v>121.1800000000001</v>
       </c>
       <c r="V67" t="n">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>57.23684210526315</v>
+        <v>57.39644970414201</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>0.84</v>
+        <v>1.05</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>2.98</v>
@@ -7911,7 +7875,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -8078,22 +8042,13 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>71.06</v>
+        <v>0</v>
       </c>
       <c r="P69" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q69" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R69" s="7" t="n">
-        <v>2.289187227866473</v>
-      </c>
-      <c r="S69" s="7" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="T69" t="n">
         <v>271</v>
@@ -8187,22 +8142,13 @@
         <v>0</v>
       </c>
       <c r="N70" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O70" s="7" t="n">
-        <v>19946.4</v>
+        <v>0</v>
       </c>
       <c r="P70" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q70" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R70" s="7" t="n">
-        <v>278.6503340757238</v>
-      </c>
-      <c r="S70" s="7" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="T70" t="n">
         <v>7</v>
@@ -8234,7 +8180,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC70" t="inlineStr">
@@ -8274,20 +8220,20 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/03/2026 06:03</t>
+          <t>08/04/2026 21:24</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
-        <v>19836.23</v>
+        <v>19864.6</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>-0.8</v>
+        <v>-0.66</v>
       </c>
       <c r="J71" s="7" t="n">
         <v>1.34</v>
       </c>
       <c r="K71" s="7" t="n">
-        <v>0.79</v>
+        <v>0.84</v>
       </c>
       <c r="L71" t="n">
         <v>20000</v>
@@ -8305,19 +8251,19 @@
         <v>0</v>
       </c>
       <c r="T71" t="n">
-        <v>261</v>
+        <v>278</v>
       </c>
       <c r="U71" s="7" t="n">
-        <v>-162.43</v>
+        <v>-135.3999999999999</v>
       </c>
       <c r="V71" t="n">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="W71" s="7" t="n">
-        <v>49.04214559386973</v>
+        <v>50</v>
       </c>
       <c r="X71" s="7" t="n">
-        <v>0.8</v>
+        <v>0.84</v>
       </c>
       <c r="Y71" s="7" t="n">
         <v>1.34</v>
@@ -8329,7 +8275,7 @@
       </c>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB71" t="inlineStr">
@@ -8374,20 +8320,20 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/03/2026 06:09</t>
+          <t>08/04/2026 21:33</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
-        <v>19651.71</v>
+        <v>19686.07</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>-1.73</v>
+        <v>-1.56</v>
       </c>
       <c r="J72" s="7" t="n">
         <v>2.67</v>
       </c>
       <c r="K72" s="7" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L72" t="n">
         <v>20000</v>
@@ -8405,19 +8351,19 @@
         <v>0</v>
       </c>
       <c r="T72" t="n">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="U72" s="7" t="n">
-        <v>-342.02</v>
+        <v>-313.9299999999999</v>
       </c>
       <c r="V72" t="n">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="W72" s="7" t="n">
-        <v>48.86363636363637</v>
+        <v>49.8220640569395</v>
       </c>
       <c r="X72" s="7" t="n">
-        <v>0.78</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y72" s="7" t="n">
         <v>2.67</v>
@@ -8429,7 +8375,7 @@
       </c>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB72" t="inlineStr">
@@ -8474,20 +8420,20 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/03/2026 05:51</t>
+          <t>08/04/2026 21:13</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
-        <v>19420.8</v>
+        <v>19464.47</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>-2.87</v>
+        <v>-2.67</v>
       </c>
       <c r="J73" s="7" t="n">
         <v>4.3</v>
       </c>
       <c r="K73" s="7" t="n">
-        <v>0.75</v>
+        <v>0.78</v>
       </c>
       <c r="L73" t="n">
         <v>20000</v>
@@ -8505,19 +8451,19 @@
         <v>0</v>
       </c>
       <c r="T73" t="n">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="U73" s="7" t="n">
-        <v>-577.8099999999999</v>
+        <v>-535.53</v>
       </c>
       <c r="V73" t="n">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="W73" s="7" t="n">
-        <v>48.86363636363637</v>
+        <v>49.8220640569395</v>
       </c>
       <c r="X73" s="7" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="Y73" s="7" t="n">
         <v>4.31</v>
@@ -8529,7 +8475,7 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB73" t="inlineStr">
@@ -8574,20 +8520,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/03/2026 06:05</t>
+          <t>08/04/2026 21:24</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20493.64</v>
+        <v>20534.52</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>2.47</v>
+        <v>2.67</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>1.73</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.74</v>
+        <v>1.54</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8605,19 +8551,19 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>363.96</v>
+        <v>520.77</v>
       </c>
       <c r="V74" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>67.30769230769231</v>
+        <v>68.75</v>
       </c>
       <c r="X74" s="7" t="n">
-        <v>1.42</v>
+        <v>1.52</v>
       </c>
       <c r="Y74" s="7" t="n">
         <v>1.73</v>
@@ -8629,7 +8575,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8674,17 +8620,17 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/03/2026 05:42</t>
+          <t>08/04/2026 20:55</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20055.44</v>
+        <v>20073.53</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>0.29</v>
+        <v>0.38</v>
       </c>
       <c r="J75" s="7" t="n">
-        <v>3.58</v>
+        <v>3.97</v>
       </c>
       <c r="K75" s="7" t="n">
         <v>1.02</v>
@@ -8705,19 +8651,19 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>15.38000000000005</v>
+        <v>87.60000000000008</v>
       </c>
       <c r="V75" t="n">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>51.92307692307693</v>
+        <v>53.33333333333334</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="Y75" s="7" t="n">
         <v>3.99</v>
@@ -8729,7 +8675,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8774,20 +8720,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/03/2026 06:09</t>
+          <t>08/04/2026 21:29</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>20657.58</v>
+        <v>21225.22</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>3.29</v>
+        <v>6.12</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>2.92</v>
       </c>
       <c r="K76" s="7" t="n">
-        <v>1.22</v>
+        <v>1.39</v>
       </c>
       <c r="L76" t="n">
         <v>20000</v>
@@ -8805,19 +8751,19 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>629</v>
+        <v>679</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>738.1400000000001</v>
+        <v>1220.87</v>
       </c>
       <c r="V76" t="n">
-        <v>372</v>
+        <v>412</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>59.14149443561209</v>
+        <v>60.67746686303387</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.24</v>
+        <v>1.39</v>
       </c>
       <c r="Y76" s="7" t="n">
         <v>2.93</v>
@@ -8829,7 +8775,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8874,20 +8820,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/03/2026 06:01</t>
+          <t>08/04/2026 21:23</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>19460.67</v>
+        <v>19875.72</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>-2.69</v>
+        <v>-0.62</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="K77" s="7" t="n">
-        <v>0.87</v>
+        <v>0.97</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8905,19 +8851,19 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>611</v>
+        <v>651</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>-498.34</v>
+        <v>-124.2800000000002</v>
       </c>
       <c r="V77" t="n">
-        <v>310</v>
+        <v>335</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>50.73649754500818</v>
+        <v>51.45929339477726</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>0.88</v>
+        <v>0.97</v>
       </c>
       <c r="Y77" s="7" t="n">
         <v>4.48</v>
@@ -8929,7 +8875,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8974,20 +8920,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/03/2026 06:10</t>
+          <t>08/04/2026 21:35</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>20412.73</v>
+        <v>20225.12</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>2.07</v>
+        <v>1.13</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>1.21</v>
+        <v>1.1</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -9005,19 +8951,19 @@
         <v>0</v>
       </c>
       <c r="T78" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="U78" s="7" t="n">
-        <v>410.6900000000001</v>
+        <v>225.12</v>
       </c>
       <c r="V78" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="W78" s="7" t="n">
-        <v>34.54545454545455</v>
+        <v>36.20689655172414</v>
       </c>
       <c r="X78" s="7" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="Y78" s="7" t="n">
         <v>5.5</v>
@@ -9029,7 +8975,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -9074,20 +9020,20 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/03/2026 05:59</t>
+          <t>08/04/2026 21:25</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>19931.56</v>
+        <v>19978.53</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>-0.33</v>
+        <v>-0.1</v>
       </c>
       <c r="J79" s="7" t="n">
-        <v>14.48</v>
-      </c>
-      <c r="K79" s="7" t="n">
-        <v>0.99</v>
+        <v>15.88</v>
+      </c>
+      <c r="K79" t="n">
+        <v>1</v>
       </c>
       <c r="L79" t="n">
         <v>20000</v>
@@ -9105,19 +9051,19 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>157</v>
+        <v>182</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>-228.7600000000004</v>
+        <v>37.16999999999939</v>
       </c>
       <c r="V79" t="n">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>51.59235668789809</v>
+        <v>52.74725274725275</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="Y79" s="7" t="n">
         <v>15.89</v>
@@ -9129,7 +9075,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9174,20 +9120,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/03/2026 05:51</t>
+          <t>08/04/2026 21:09</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>19239.14</v>
+        <v>20725.15</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>-3.81</v>
+        <v>3.62</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>0.95</v>
+        <v>1.04</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9205,19 +9151,19 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>1200</v>
+        <v>1282</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>-664.2800000000008</v>
+        <v>707.8299999999997</v>
       </c>
       <c r="V80" t="n">
-        <v>727</v>
+        <v>794</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>60.58333333333334</v>
+        <v>61.93447737909516</v>
       </c>
       <c r="X80" s="7" t="n">
-        <v>0.96</v>
+        <v>1.04</v>
       </c>
       <c r="Y80" s="7" t="n">
         <v>17.52</v>
@@ -9229,7 +9175,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9274,20 +9220,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/03/2026 06:10</t>
+          <t>08/04/2026 21:40</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>18428.87</v>
+        <v>19451.67</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-7.83</v>
+        <v>-2.72</v>
       </c>
       <c r="J81" s="7" t="n">
-        <v>12.35</v>
+        <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.86</v>
+        <v>0.95</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9305,19 +9251,19 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>614</v>
+        <v>654</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>-1475.85</v>
+        <v>-548.3300000000002</v>
       </c>
       <c r="V81" t="n">
-        <v>310</v>
+        <v>335</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>50.4885993485342</v>
+        <v>51.22324159021407</v>
       </c>
       <c r="X81" s="7" t="n">
-        <v>0.87</v>
+        <v>0.95</v>
       </c>
       <c r="Y81" s="7" t="n">
         <v>12.38</v>
@@ -9329,7 +9275,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9374,20 +9320,20 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/03/2026 06:01</t>
+          <t>08/04/2026 21:23</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>20235.03</v>
+        <v>20067.18</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>1.21</v>
+        <v>0.37</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>1.12</v>
+        <v>1.03</v>
       </c>
       <c r="L82" t="n">
         <v>20000</v>
@@ -9405,19 +9351,19 @@
         <v>0</v>
       </c>
       <c r="T82" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="U82" s="7" t="n">
-        <v>240.39</v>
+        <v>67.18000000000004</v>
       </c>
       <c r="V82" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="W82" s="7" t="n">
-        <v>33.33333333333333</v>
+        <v>35</v>
       </c>
       <c r="X82" s="7" t="n">
-        <v>1.11</v>
+        <v>1.03</v>
       </c>
       <c r="Y82" s="7" t="n">
         <v>5.84</v>
@@ -9429,7 +9375,7 @@
       </c>
       <c r="AA82" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB82" t="inlineStr">
@@ -9474,7 +9420,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/03/2026 06:07</t>
+          <t>08/04/2026 21:34</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9801,14 +9747,14 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/03/2026 10:41</t>
+          <t>08/04/2026 19:13</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>26905.59</v>
+        <v>26828.95</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>-29.94</v>
+        <v>-30.14</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>37.71</v>
@@ -9826,28 +9772,31 @@
         <v>40</v>
       </c>
       <c r="O86" s="7" t="n">
-        <v>356.1</v>
+        <v>257.12</v>
       </c>
       <c r="P86" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="Q86" s="7" t="n">
-        <v>100</v>
+        <v>92.5</v>
+      </c>
+      <c r="R86" s="7" t="n">
+        <v>3.604801945091683</v>
       </c>
       <c r="S86" s="7" t="n">
-        <v>0</v>
+        <v>0.39</v>
       </c>
       <c r="T86" t="n">
-        <v>3308</v>
+        <v>3316</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>-7376.41</v>
+        <v>-7453.049999999999</v>
       </c>
       <c r="V86" t="n">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>61.39661426844014</v>
+        <v>61.27864897466827</v>
       </c>
       <c r="X86" s="7" t="n">
         <v>0.77</v>
@@ -9862,7 +9811,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9998,7 +9947,7 @@
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>08/01/2026 19:54</t>
+          <t>08/04/2026 19:57</t>
         </is>
       </c>
       <c r="H88" s="9" t="n">
@@ -10180,7 +10129,7 @@
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>08/01/2026 09:33</t>
+          <t>08/04/2026 09:36</t>
         </is>
       </c>
       <c r="H90" s="9" t="n">
@@ -10271,7 +10220,7 @@
       </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>08/01/2026 00:43</t>
+          <t>08/04/2026 00:45</t>
         </is>
       </c>
       <c r="H91" s="9" t="n">
@@ -10453,7 +10402,7 @@
       </c>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 05:31</t>
+          <t>08/04/2026 21:02</t>
         </is>
       </c>
       <c r="H93" s="9" t="n">
@@ -10635,7 +10584,7 @@
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>08/01/2026 14:15</t>
+          <t>08/04/2026 14:26</t>
         </is>
       </c>
       <c r="H95" s="9" t="n">
@@ -10726,7 +10675,7 @@
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 05:54</t>
+          <t>08/04/2026 21:19</t>
         </is>
       </c>
       <c r="H96" s="9" t="n">
@@ -10817,7 +10766,7 @@
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 05:28</t>
+          <t>08/04/2026 20:46</t>
         </is>
       </c>
       <c r="H97" s="9" t="n">
@@ -10902,7 +10851,7 @@
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 11:58</t>
+          <t>08/04/2026 20:23</t>
         </is>
       </c>
       <c r="H98" s="9" t="n">
@@ -10987,7 +10936,7 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 12:02</t>
+          <t>08/04/2026 20:21</t>
         </is>
       </c>
       <c r="H99" s="9" t="n">
@@ -11430,7 +11379,7 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>07/31/2026 22:03</t>
+          <t>08/03/2026 23:11</t>
         </is>
       </c>
       <c r="H104" s="9" t="n">
@@ -11646,7 +11595,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08/01/2026 19:54</t>
+          <t>08/04/2026 19:57</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -11728,7 +11677,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08/01/2026 09:33</t>
+          <t>08/04/2026 09:36</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -11769,7 +11718,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08/01/2026 00:43</t>
+          <t>08/04/2026 00:45</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -11851,7 +11800,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/03/2026 05:31</t>
+          <t>08/04/2026 21:02</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -11933,7 +11882,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/01/2026 14:15</t>
+          <t>08/04/2026 14:26</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -11974,7 +11923,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/03/2026 05:54</t>
+          <t>08/04/2026 21:19</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -12015,7 +11964,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/03/2026 05:28</t>
+          <t>08/04/2026 20:46</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -12056,7 +12005,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/03/2026 11:58</t>
+          <t>08/04/2026 20:23</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -12097,7 +12046,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/03/2026 12:02</t>
+          <t>08/04/2026 20:21</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -12302,7 +12251,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>07/31/2026 22:03</t>
+          <t>08/03/2026 23:11</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -13266,7 +13215,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/01/2026 09:51</t>
+          <t>08/04/2026 10:01</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -13358,7 +13307,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08/01/2026 04:35</t>
+          <t>08/04/2026 04:41</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -13404,7 +13353,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08/01/2026 05:21</t>
+          <t>08/04/2026 05:23</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -13427,7 +13376,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/01/2026 12:47</t>
+          <t>08/04/2026 12:52</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -13473,7 +13422,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/01/2026 14:51</t>
+          <t>08/04/2026 14:59</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -13634,7 +13583,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/03/2026 08:13</t>
+          <t>08/04/2026 16:40</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -13680,11 +13629,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/03/2026 05:31</t>
+          <t>08/04/2026 20:57</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>19817.46</v>
+        <v>19911.42</v>
       </c>
     </row>
     <row r="24">
@@ -13726,11 +13675,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/03/2026 00:22</t>
+          <t>08/04/2026 21:50</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19502.84</v>
+        <v>19248.09</v>
       </c>
     </row>
     <row r="26">
@@ -13749,11 +13698,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/03/2026 06:03</t>
+          <t>08/04/2026 21:26</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>19246.74</v>
+        <v>20828.97</v>
       </c>
     </row>
     <row r="27">
@@ -13795,7 +13744,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/03/2026 08:51</t>
+          <t>08/04/2026 17:32</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -13818,7 +13767,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/03/2026 09:08</t>
+          <t>08/04/2026 17:54</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -13841,7 +13790,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/03/2026 08:43</t>
+          <t>08/04/2026 17:18</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -13864,7 +13813,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/03/2026 09:15</t>
+          <t>08/04/2026 17:51</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -13887,7 +13836,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/03/2026 08:44</t>
+          <t>08/04/2026 17:31</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -13910,7 +13859,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/03/2026 08:19</t>
+          <t>08/04/2026 16:57</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -13933,7 +13882,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/03/2026 06:37</t>
+          <t>08/04/2026 21:53</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
@@ -13956,7 +13905,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>08/03/2026 06:58</t>
+          <t>08/04/2026 22:24</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
@@ -13979,11 +13928,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/03/2026 05:38</t>
+          <t>08/04/2026 20:55</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>20285.27</v>
+        <v>20645.19</v>
       </c>
     </row>
     <row r="37">
@@ -14071,7 +14020,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>07/31/2026 21:58</t>
+          <t>08/03/2026 23:06</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
@@ -14094,7 +14043,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>08/03/2026 09:10</t>
+          <t>08/04/2026 09:12</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-05
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-04 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-05 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/04/2026 19:32</t>
+          <t>08/05/2026 20:05</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>34401.88</v>
+        <v>26721.82</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>57.75</v>
+        <v>22.53</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>74.43000000000001</v>
+        <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.05</v>
+        <v>1.02</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,37 +985,37 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-23560.95</v>
+        <v>-29160.46</v>
       </c>
       <c r="P2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>52.5</v>
+        <v>67.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.421791637422021</v>
+        <v>0.514364330256357</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>97</v>
+        <v>153.45</v>
       </c>
       <c r="T2" t="n">
-        <v>3284</v>
+        <v>3303</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>9401.879999999983</v>
+        <v>1721.819999999996</v>
       </c>
       <c r="V2" t="n">
-        <v>2058</v>
+        <v>2073</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>62.66747868453106</v>
+        <v>62.76112624886467</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="Y2" s="7" t="n">
-        <v>74.43000000000001</v>
+        <v>80.69</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/04/2026 17:12</t>
+          <t>08/05/2026 18:17</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/04/2026 20:11</t>
+          <t>08/05/2026 14:51</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/04/2026 21:31</t>
+          <t>08/05/2026 21:38</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,17 +2486,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/04/2026 17:37</t>
+          <t>08/05/2026 18:24</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
-        <v>76.73999999999999</v>
+        <v>70.14</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>-99.59</v>
+        <v>-99.63</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>99.59999999999999</v>
+        <v>99.63</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>0.7</v>
@@ -2511,37 +2511,37 @@
         <v>40</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>-5.95</v>
+        <v>-14.35</v>
       </c>
       <c r="P16" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>30</v>
+        <v>22.5</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>0.5258964143426295</v>
+        <v>0.2910079051383399</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="T16" t="n">
-        <v>2293</v>
+        <v>2300</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>-20345.66</v>
+        <v>-20352.26</v>
       </c>
       <c r="V16" t="n">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>32.14129960750109</v>
+        <v>32.1304347826087</v>
       </c>
       <c r="X16" s="7" t="n">
         <v>0.7</v>
       </c>
       <c r="Y16" s="7" t="n">
-        <v>99.63</v>
+        <v>99.66</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/02/2026 14:44</t>
+          <t>08/05/2026 14:47</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -3071,16 +3071,16 @@
         <v>12.31</v>
       </c>
       <c r="T21" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U21" s="7" t="n">
-        <v>-4909.34</v>
+        <v>-4898.34</v>
       </c>
       <c r="V21" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="W21" s="7" t="n">
-        <v>42.69005847953216</v>
+        <v>43.02325581395349</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>0.68</v>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/04/2026 21:22</t>
+          <t>08/05/2026 21:33</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/04/2026 20:13</t>
+          <t>08/05/2026 20:48</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19551.52</v>
+        <v>19795.02</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-2.24</v>
+        <v>-1.02</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.1</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.88</v>
+        <v>0.95</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,34 +3274,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>-324.6899999999999</v>
+        <v>185.4</v>
       </c>
       <c r="P23" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>47.5</v>
+        <v>52.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>0.8651798764283816</v>
+        <v>1.08665697579307</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.26</v>
+        <v>4.2</v>
       </c>
       <c r="T23" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-448.4799999999997</v>
+        <v>-204.9799999999998</v>
       </c>
       <c r="V23" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>50.70422535211267</v>
+        <v>51.35135135135135</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.88</v>
+        <v>0.95</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>6.11</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3467,20 +3467,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/04/2026 20:51</t>
+          <t>08/05/2026 21:08</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16095.96</v>
+        <v>16324.68</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-19.23</v>
+        <v>-18.07</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3492,34 +3492,34 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>159.29</v>
+        <v>386.09</v>
       </c>
       <c r="P25" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>45</v>
+        <v>47.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.305381415233604</v>
+        <v>1.842108707031931</v>
       </c>
       <c r="S25" s="7" t="n">
         <v>0.95</v>
       </c>
       <c r="T25" t="n">
-        <v>603</v>
+        <v>612</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3904.04</v>
+        <v>-3675.32</v>
       </c>
       <c r="V25" t="n">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>37.81094527363184</v>
+        <v>38.0718954248366</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>21.17</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/04/2026 18:37</t>
+          <t>08/05/2026 19:20</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/04/2026 20:46</t>
+          <t>08/05/2026 21:01</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20439.59</v>
+        <v>20486.81</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-2.26</v>
+        <v>-2.03</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>7.39</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,34 +3710,34 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-711.8199999999999</v>
+        <v>-491.46</v>
       </c>
       <c r="P27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>47.5</v>
+        <v>50</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.690325892604661</v>
+        <v>0.7687758472243786</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>6.74</v>
+        <v>6.61</v>
       </c>
       <c r="T27" t="n">
         <v>93</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>439.5900000000001</v>
+        <v>486.8100000000001</v>
       </c>
       <c r="V27" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>45.16129032258064</v>
+        <v>46.23655913978494</v>
       </c>
       <c r="X27" s="7" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="Y27" s="7" t="n">
         <v>7.39</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/04/2026 20:52</t>
+          <t>08/05/2026 21:07</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19828.87</v>
+        <v>19577.87</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-0.87</v>
+        <v>-2.12</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0.93</v>
+        <v>0.84</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,34 +3928,34 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-483.5</v>
+        <v>-786.77</v>
       </c>
       <c r="P29" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>37.5</v>
+        <v>30</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.2112947164086586</v>
+        <v>0.0894181914979804</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>2.68</v>
+        <v>3.94</v>
       </c>
       <c r="T29" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-171.1300000000002</v>
+        <v>-422.1300000000002</v>
       </c>
       <c r="V29" t="n">
         <v>54</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>48.21428571428572</v>
+        <v>46.95652173913044</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>0.93</v>
+        <v>0.84</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/04/2026 21:04</t>
+          <t>08/05/2026 21:19</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/04/2026 20:27</t>
+          <t>08/05/2026 20:50</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/04/2026 17:02</t>
+          <t>08/05/2026 23:46</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/04/2026 22:16</t>
+          <t>08/05/2026 22:20</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/04/2026 22:06</t>
+          <t>08/05/2026 22:05</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19757.28</v>
+        <v>19660.81</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-1.22</v>
+        <v>-1.7</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.41</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-242.72</v>
+        <v>-339.1900000000001</v>
       </c>
       <c r="V36" t="n">
         <v>31</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>47.69230769230769</v>
+        <v>46.96969696969697</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.41</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/04/2026 21:48</t>
+          <t>08/05/2026 21:58</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/04/2026 23:04</t>
+          <t>08/05/2026 17:21</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/04/2026 22:47</t>
+          <t>08/05/2026 22:45</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5311,20 +5311,20 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/04/2026 20:19</t>
+          <t>08/05/2026 20:49</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
-        <v>18662.81</v>
+        <v>18557.79</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>-6.67</v>
+        <v>-7.21</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>6.99</v>
+        <v>7.45</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="L42" t="n">
         <v>20000</v>
@@ -5336,37 +5336,37 @@
         <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-78.95999999999999</v>
+        <v>-15.15</v>
       </c>
       <c r="P42" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="Q42" s="7" t="n">
-        <v>30</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>0.2637762237762238</v>
+        <v>0.6996431403647899</v>
       </c>
       <c r="S42" s="7" t="n">
-        <v>0.49</v>
+        <v>0.22</v>
       </c>
       <c r="T42" t="n">
-        <v>2254</v>
+        <v>2405</v>
       </c>
       <c r="U42" s="7" t="n">
-        <v>-1335.55</v>
+        <v>-1442.21</v>
       </c>
       <c r="V42" t="n">
-        <v>1010</v>
+        <v>1075</v>
       </c>
       <c r="W42" s="7" t="n">
-        <v>44.80922803904171</v>
+        <v>44.6985446985447</v>
       </c>
       <c r="X42" s="7" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="Y42" s="7" t="n">
-        <v>6.92</v>
+        <v>7.45</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
@@ -5375,7 +5375,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
@@ -5420,17 +5420,17 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/04/2026 20:55</t>
+          <t>08/05/2026 21:13</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
-        <v>17633.49</v>
+        <v>17554.84</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>-11.81</v>
+        <v>-12.2</v>
       </c>
       <c r="J43" s="7" t="n">
-        <v>12.64</v>
+        <v>12.83</v>
       </c>
       <c r="K43" s="7" t="n">
         <v>0.67</v>
@@ -5442,31 +5442,40 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-71.71000000000001</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.2413245873889124</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>0.46</v>
       </c>
       <c r="T43" t="n">
-        <v>4058</v>
+        <v>4278</v>
       </c>
       <c r="U43" s="7" t="n">
-        <v>-2371.88</v>
+        <v>-2445.16</v>
       </c>
       <c r="V43" t="n">
-        <v>1759</v>
+        <v>1857</v>
       </c>
       <c r="W43" s="7" t="n">
-        <v>43.34647609659931</v>
+        <v>43.40813464235624</v>
       </c>
       <c r="X43" s="7" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="Y43" s="7" t="n">
-        <v>12.67</v>
+        <v>12.86</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -5475,7 +5484,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
@@ -5520,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/04/2026 20:35</t>
+          <t>08/05/2026 20:59</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5542,13 +5551,22 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5620,20 +5638,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/04/2026 20:54</t>
+          <t>08/05/2026 21:17</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19983.72</v>
+        <v>19990.21</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.06</v>
+        <v>-0.03</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>3.15</v>
       </c>
-      <c r="K45" s="7" t="n">
-        <v>0.99</v>
+      <c r="K45" t="n">
+        <v>1</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5642,28 +5660,37 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-164.11</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.5792590693500833</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>1.35</v>
       </c>
       <c r="T45" t="n">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-16.27999999999997</v>
+        <v>-9.789999999999964</v>
       </c>
       <c r="V45" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>55.66502463054187</v>
+        <v>55.63725490196079</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="Y45" s="7" t="n">
         <v>3.15</v>
@@ -5675,7 +5702,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5720,7 +5747,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/04/2026 20:12</t>
+          <t>08/05/2026 20:35</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5742,13 +5769,22 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>19981.27</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q46" s="7" t="n">
+        <v>30.3030303030303</v>
+      </c>
+      <c r="R46" s="7" t="n">
+        <v>335.5265360790223</v>
+      </c>
+      <c r="S46" s="7" t="n">
+        <v>0.1</v>
       </c>
       <c r="T46" t="n">
         <v>32</v>
@@ -5780,7 +5816,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5820,7 +5856,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/04/2026 20:39</t>
+          <t>08/05/2026 20:54</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5920,7 +5956,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/04/2026 20:05</t>
+          <t>08/05/2026 20:29</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6020,20 +6056,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/04/2026 21:06</t>
+          <t>08/05/2026 21:16</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>18939.49</v>
+        <v>19056.79</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>-5.32</v>
+        <v>-4.72</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>6.85</v>
+        <v>7.1</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
       <c r="L49" t="n">
         <v>20000</v>
@@ -6051,22 +6087,22 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>391</v>
+        <v>410</v>
       </c>
       <c r="U49" s="7" t="n">
-        <v>-826.1800000000001</v>
+        <v>-943.21</v>
       </c>
       <c r="V49" t="n">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="W49" s="7" t="n">
-        <v>46.29156010230179</v>
+        <v>46.82926829268293</v>
       </c>
       <c r="X49" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="Y49" s="7" t="n">
-        <v>6.61</v>
+        <v>7.09</v>
       </c>
       <c r="Z49" t="inlineStr">
         <is>
@@ -6075,7 +6111,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
@@ -6120,20 +6156,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/04/2026 20:53</t>
+          <t>08/05/2026 21:20</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>17899.68</v>
+        <v>18034.01</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>-10.52</v>
+        <v>-9.84</v>
       </c>
       <c r="J50" s="7" t="n">
-        <v>20.49</v>
+        <v>20.92</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6151,22 +6187,22 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>1113</v>
+        <v>1161</v>
       </c>
       <c r="U50" s="7" t="n">
-        <v>-1192.400000000001</v>
+        <v>-1965.990000000001</v>
       </c>
       <c r="V50" t="n">
-        <v>568</v>
+        <v>592</v>
       </c>
       <c r="W50" s="7" t="n">
-        <v>51.03324348607367</v>
+        <v>50.99052540913006</v>
       </c>
       <c r="X50" s="7" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="Y50" s="7" t="n">
-        <v>19.8</v>
+        <v>20.89</v>
       </c>
       <c r="Z50" t="inlineStr">
         <is>
@@ -6175,7 +6211,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
@@ -6220,20 +6256,20 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/04/2026 20:18</t>
+          <t>08/05/2026 20:43</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>15674.58</v>
+        <v>14868.84</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-21.27</v>
+        <v>-25.68</v>
       </c>
       <c r="J51" s="7" t="n">
-        <v>41.12</v>
+        <v>43.16</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="L51" t="n">
         <v>20000</v>
@@ -6251,22 +6287,22 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>1911</v>
+        <v>1978</v>
       </c>
       <c r="U51" s="7" t="n">
-        <v>-3881.080000000002</v>
+        <v>-5131.160000000003</v>
       </c>
       <c r="V51" t="n">
-        <v>937</v>
+        <v>970</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>49.03192046049189</v>
+        <v>49.03943377148635</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="Y51" s="7" t="n">
-        <v>41.12</v>
+        <v>43.15</v>
       </c>
       <c r="Z51" t="inlineStr">
         <is>
@@ -6275,7 +6311,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -6320,7 +6356,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/04/2026 20:15</t>
+          <t>08/05/2026 20:44</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6351,7 +6387,7 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U52" s="7" t="n">
         <v>-1926.29</v>
@@ -6360,7 +6396,7 @@
         <v>9</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>25</v>
+        <v>24.32432432432433</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.42</v>
@@ -6375,7 +6411,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6420,20 +6456,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/04/2026 20:58</t>
+          <t>08/05/2026 21:12</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19868.27</v>
+        <v>19824.34</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.91</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6451,19 +6487,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-131.73</v>
+        <v>-175.66</v>
       </c>
       <c r="V53" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>37.56345177664975</v>
+        <v>36.76470588235294</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6475,7 +6511,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6520,17 +6556,17 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/04/2026 21:08</t>
+          <t>08/05/2026 21:27</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
-        <v>19729.88</v>
+        <v>19715.69</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>-1.34</v>
+        <v>-1.41</v>
       </c>
       <c r="J54" s="7" t="n">
-        <v>4.63</v>
+        <v>4.64</v>
       </c>
       <c r="K54" s="7" t="n">
         <v>0.86</v>
@@ -6551,22 +6587,22 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>204</v>
+        <v>225</v>
       </c>
       <c r="U54" s="7" t="n">
-        <v>-272.9600000000001</v>
+        <v>-284.3099999999999</v>
       </c>
       <c r="V54" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="W54" s="7" t="n">
-        <v>43.13725490196079</v>
+        <v>42.66666666666667</v>
       </c>
       <c r="X54" s="7" t="n">
         <v>0.86</v>
       </c>
       <c r="Y54" s="7" t="n">
-        <v>4.63</v>
+        <v>4.65</v>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
@@ -6575,7 +6611,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -6620,20 +6656,20 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/04/2026 20:54</t>
+          <t>08/05/2026 21:09</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
-        <v>19710.36</v>
+        <v>19685.73</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>-1.4</v>
+        <v>-1.51</v>
       </c>
       <c r="J55" s="7" t="n">
         <v>2.68</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="L55" t="n">
         <v>20000</v>
@@ -6651,19 +6687,19 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>1380</v>
+        <v>1559</v>
       </c>
       <c r="U55" s="7" t="n">
-        <v>-286.51</v>
+        <v>-312.21</v>
       </c>
       <c r="V55" t="n">
-        <v>649</v>
+        <v>738</v>
       </c>
       <c r="W55" s="7" t="n">
-        <v>47.02898550724638</v>
+        <v>47.33803720333547</v>
       </c>
       <c r="X55" s="7" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="Y55" s="7" t="n">
         <v>2.72</v>
@@ -6675,7 +6711,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -6720,20 +6756,20 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/04/2026 21:13</t>
+          <t>08/05/2026 21:33</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
-        <v>19859.7</v>
+        <v>19882.87</v>
       </c>
       <c r="I56" s="7" t="n">
-        <v>-0.72</v>
+        <v>-0.6</v>
       </c>
       <c r="J56" s="7" t="n">
         <v>1.98</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="L56" t="n">
         <v>20000</v>
@@ -6742,28 +6778,37 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O56" s="7" t="n">
-        <v>0</v>
+        <v>25.89</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q56" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R56" s="7" t="n">
+        <v>1.281229632848143</v>
+      </c>
+      <c r="S56" s="7" t="n">
+        <v>0.26</v>
       </c>
       <c r="T56" t="n">
-        <v>1069</v>
+        <v>1127</v>
       </c>
       <c r="U56" s="7" t="n">
-        <v>-147.31</v>
+        <v>-113.03</v>
       </c>
       <c r="V56" t="n">
-        <v>499</v>
+        <v>528</v>
       </c>
       <c r="W56" s="7" t="n">
-        <v>46.67913938260056</v>
+        <v>46.85004436557232</v>
       </c>
       <c r="X56" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.96</v>
       </c>
       <c r="Y56" s="7" t="n">
         <v>1.95</v>
@@ -6775,7 +6820,7 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr">
@@ -6820,20 +6865,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/04/2026 20:16</t>
+          <t>08/05/2026 20:44</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19752.74</v>
+        <v>19765.28</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.26</v>
+        <v>-1.2</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6851,19 +6896,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>656</v>
+        <v>691</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-250.1</v>
+        <v>-234.72</v>
       </c>
       <c r="V57" t="n">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.44512195121951</v>
+        <v>43.56005788712012</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6875,7 +6920,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6920,20 +6965,20 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/04/2026 20:35</t>
+          <t>08/05/2026 20:55</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
-        <v>17182.33</v>
+        <v>17178.35</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>-14.09</v>
+        <v>-14.11</v>
       </c>
       <c r="J58" s="7" t="n">
         <v>15.49</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="L58" t="n">
         <v>20000</v>
@@ -6951,19 +6996,19 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>4197</v>
+        <v>4426</v>
       </c>
       <c r="U58" s="7" t="n">
-        <v>-2827.43</v>
+        <v>-2812.96</v>
       </c>
       <c r="V58" t="n">
-        <v>1817</v>
+        <v>1919</v>
       </c>
       <c r="W58" s="7" t="n">
-        <v>43.29282821062664</v>
+        <v>43.35743334839584</v>
       </c>
       <c r="X58" s="7" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="Y58" s="7" t="n">
         <v>15.49</v>
@@ -6975,7 +7020,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB58" t="inlineStr">
@@ -7020,20 +7065,20 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/04/2026 20:50</t>
+          <t>08/05/2026 21:05</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
-        <v>20155.01</v>
+        <v>20094.92</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>0.78</v>
+        <v>0.48</v>
       </c>
       <c r="J59" s="7" t="n">
         <v>0.55</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>1.32</v>
+        <v>1.17</v>
       </c>
       <c r="L59" t="n">
         <v>20000</v>
@@ -7051,19 +7096,19 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>244</v>
+        <v>272</v>
       </c>
       <c r="U59" s="7" t="n">
-        <v>157.11</v>
+        <v>94.92000000000002</v>
       </c>
       <c r="V59" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="W59" s="7" t="n">
-        <v>44.67213114754098</v>
+        <v>43.38235294117647</v>
       </c>
       <c r="X59" s="7" t="n">
-        <v>1.33</v>
+        <v>1.17</v>
       </c>
       <c r="Y59" s="7" t="n">
         <v>0.55</v>
@@ -7075,7 +7120,7 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -7120,14 +7165,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/04/2026 20:51</t>
+          <t>08/05/2026 21:03</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>20600.8</v>
+        <v>20423.33</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-3.13</v>
+        <v>-3.97</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
@@ -7151,19 +7196,19 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>6152</v>
+        <v>6436</v>
       </c>
       <c r="U60" s="7" t="n">
-        <v>-968.1199999999999</v>
+        <v>-648.0199999999995</v>
       </c>
       <c r="V60" t="n">
-        <v>2935</v>
+        <v>3107</v>
       </c>
       <c r="W60" s="7" t="n">
-        <v>47.70806241872562</v>
+        <v>48.27532628962089</v>
       </c>
       <c r="X60" s="7" t="n">
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="Y60" s="7" t="n">
         <v>18.48</v>
@@ -7175,7 +7220,7 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
@@ -7220,20 +7265,20 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/04/2026 21:17</t>
+          <t>08/05/2026 21:26</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>20626.92</v>
+        <v>20681.68</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-3.73</v>
+        <v>-3.47</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>13.96</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="L61" s="7" t="n">
         <v>21292.1</v>
@@ -7251,19 +7296,19 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>3453</v>
+        <v>3623</v>
       </c>
       <c r="U61" s="7" t="n">
-        <v>-1065.33</v>
+        <v>-569.0499999999997</v>
       </c>
       <c r="V61" t="n">
-        <v>1618</v>
+        <v>1726</v>
       </c>
       <c r="W61" s="7" t="n">
-        <v>46.85780480741384</v>
+        <v>47.64007728401877</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>0.91</v>
+        <v>0.96</v>
       </c>
       <c r="Y61" s="7" t="n">
         <v>13.16</v>
@@ -7275,7 +7320,7 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
@@ -7320,7 +7365,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/04/2026 21:16</t>
+          <t>08/05/2026 21:34</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7420,20 +7465,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/04/2026 21:20</t>
+          <t>08/05/2026 21:33</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18994.6</v>
+        <v>18908.85</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-5.04</v>
+        <v>-5.47</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>6.74</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7451,19 +7496,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1005.4</v>
+        <v>-1091.15</v>
       </c>
       <c r="V63" t="n">
         <v>3</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>10.3448275862069</v>
+        <v>9.67741935483871</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>6.73</v>
@@ -7475,7 +7520,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7520,20 +7565,20 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/04/2026 21:24</t>
+          <t>08/05/2026 21:40</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
-        <v>19452.56</v>
+        <v>19444.2</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>-2.74</v>
+        <v>-2.78</v>
       </c>
       <c r="J64" s="7" t="n">
         <v>3.87</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="L64" t="n">
         <v>20000</v>
@@ -7551,16 +7596,16 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="U64" s="7" t="n">
-        <v>-520.42</v>
+        <v>-559.8499999999998</v>
       </c>
       <c r="V64" t="n">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="W64" s="7" t="n">
-        <v>51.93370165745856</v>
+        <v>51.26903553299492</v>
       </c>
       <c r="X64" s="7" t="n">
         <v>0.7</v>
@@ -7575,7 +7620,7 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB64" t="inlineStr">
@@ -7620,20 +7665,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/04/2026 21:06</t>
+          <t>08/05/2026 21:15</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19150.72</v>
+        <v>19540.97</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-4.25</v>
+        <v>-2.3</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>11.64</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7651,19 +7696,19 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>2899</v>
+        <v>3021</v>
       </c>
       <c r="U65" s="7" t="n">
-        <v>-1115.53</v>
+        <v>-425.4200000000001</v>
       </c>
       <c r="V65" t="n">
-        <v>1338</v>
+        <v>1414</v>
       </c>
       <c r="W65" s="7" t="n">
-        <v>46.15384615384615</v>
+        <v>46.80569347898047</v>
       </c>
       <c r="X65" s="7" t="n">
-        <v>0.89</v>
+        <v>0.96</v>
       </c>
       <c r="Y65" s="7" t="n">
         <v>11.64</v>
@@ -7675,7 +7720,7 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB65" t="inlineStr">
@@ -7720,20 +7765,20 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/04/2026 21:03</t>
+          <t>08/05/2026 21:22</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
-        <v>20319.13</v>
+        <v>20077.9</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
       <c r="J66" s="7" t="n">
         <v>2.86</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>1.23</v>
+        <v>1.04</v>
       </c>
       <c r="L66" t="n">
         <v>20000</v>
@@ -7751,19 +7796,19 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>190</v>
+        <v>224</v>
       </c>
       <c r="U66" s="7" t="n">
-        <v>137.24</v>
+        <v>92.41999999999985</v>
       </c>
       <c r="V66" t="n">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="W66" s="7" t="n">
-        <v>42.10526315789473</v>
+        <v>45.98214285714285</v>
       </c>
       <c r="X66" s="7" t="n">
-        <v>1.1</v>
+        <v>1.05</v>
       </c>
       <c r="Y66" s="7" t="n">
         <v>2.85</v>
@@ -7775,7 +7820,7 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
@@ -7820,20 +7865,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/04/2026 21:32</t>
+          <t>08/05/2026 21:46</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20121.18</v>
+        <v>20174.46</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>0.6</v>
+        <v>0.86</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.05</v>
+        <v>1.07</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7851,19 +7896,19 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="U67" s="7" t="n">
-        <v>121.1800000000001</v>
+        <v>166.09</v>
       </c>
       <c r="V67" t="n">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="W67" s="7" t="n">
-        <v>57.39644970414201</v>
+        <v>56.59340659340659</v>
       </c>
       <c r="X67" s="7" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="Y67" s="7" t="n">
         <v>2.98</v>
@@ -7875,7 +7920,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7920,7 +7965,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/02/2026 12:55</t>
+          <t>08/05/2026 12:57</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8020,7 +8065,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/02/2026 12:56</t>
+          <t>08/05/2026 12:58</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8120,7 +8165,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/02/2026 13:11</t>
+          <t>08/05/2026 13:12</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8220,20 +8265,20 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/04/2026 21:24</t>
+          <t>08/05/2026 21:29</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
-        <v>19864.6</v>
+        <v>19903.15</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>-0.66</v>
+        <v>-0.47</v>
       </c>
       <c r="J71" s="7" t="n">
         <v>1.34</v>
       </c>
       <c r="K71" s="7" t="n">
-        <v>0.84</v>
+        <v>0.89</v>
       </c>
       <c r="L71" t="n">
         <v>20000</v>
@@ -8251,19 +8296,19 @@
         <v>0</v>
       </c>
       <c r="T71" t="n">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="U71" s="7" t="n">
-        <v>-135.3999999999999</v>
+        <v>-96.84999999999999</v>
       </c>
       <c r="V71" t="n">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="W71" s="7" t="n">
-        <v>50</v>
+        <v>50.51546391752577</v>
       </c>
       <c r="X71" s="7" t="n">
-        <v>0.84</v>
+        <v>0.89</v>
       </c>
       <c r="Y71" s="7" t="n">
         <v>1.34</v>
@@ -8275,7 +8320,7 @@
       </c>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB71" t="inlineStr">
@@ -8320,20 +8365,20 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/04/2026 21:33</t>
+          <t>08/05/2026 21:49</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
-        <v>19686.07</v>
+        <v>19754.91</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>-1.56</v>
+        <v>-1.2</v>
       </c>
       <c r="J72" s="7" t="n">
         <v>2.67</v>
       </c>
       <c r="K72" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="L72" t="n">
         <v>20000</v>
@@ -8351,19 +8396,19 @@
         <v>0</v>
       </c>
       <c r="T72" t="n">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="U72" s="7" t="n">
-        <v>-313.9299999999999</v>
+        <v>-245.0899999999999</v>
       </c>
       <c r="V72" t="n">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="W72" s="7" t="n">
-        <v>49.8220640569395</v>
+        <v>50.34013605442177</v>
       </c>
       <c r="X72" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="Y72" s="7" t="n">
         <v>2.67</v>
@@ -8375,7 +8420,7 @@
       </c>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB72" t="inlineStr">
@@ -8420,20 +8465,20 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/04/2026 21:13</t>
+          <t>08/05/2026 21:27</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
-        <v>19464.47</v>
+        <v>19561.27</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>-2.67</v>
+        <v>-2.19</v>
       </c>
       <c r="J73" s="7" t="n">
         <v>4.3</v>
       </c>
       <c r="K73" s="7" t="n">
-        <v>0.78</v>
+        <v>0.83</v>
       </c>
       <c r="L73" t="n">
         <v>20000</v>
@@ -8451,19 +8496,19 @@
         <v>0</v>
       </c>
       <c r="T73" t="n">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="U73" s="7" t="n">
-        <v>-535.53</v>
+        <v>-438.73</v>
       </c>
       <c r="V73" t="n">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="W73" s="7" t="n">
-        <v>49.8220640569395</v>
+        <v>50.34013605442177</v>
       </c>
       <c r="X73" s="7" t="n">
-        <v>0.78</v>
+        <v>0.82</v>
       </c>
       <c r="Y73" s="7" t="n">
         <v>4.31</v>
@@ -8475,7 +8520,7 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB73" t="inlineStr">
@@ -8520,20 +8565,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/04/2026 21:24</t>
+          <t>08/05/2026 21:34</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20534.52</v>
+        <v>20634.27</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>2.67</v>
+        <v>3.18</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>1.73</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.54</v>
+        <v>1.62</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8551,19 +8596,19 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>520.77</v>
+        <v>636.87</v>
       </c>
       <c r="V74" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>68.75</v>
+        <v>69.01408450704226</v>
       </c>
       <c r="X74" s="7" t="n">
-        <v>1.52</v>
+        <v>1.62</v>
       </c>
       <c r="Y74" s="7" t="n">
         <v>1.73</v>
@@ -8575,7 +8620,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8585,7 +8630,7 @@
       </c>
       <c r="AC74" t="inlineStr">
         <is>
-          <t>T&amp;D19 Meta3 RClock | AUDJPY, T&amp;D19 Meta3 RClock | CHFJPY, T&amp;D19 Meta3 RClock | GBPJPY, T&amp;D19 Meta3 RClock | GBPUSD, T&amp;D19 Meta3 RClock | NZDUSD, T&amp;D19 Meta3 RClock | US30, T&amp;D19 Meta3 RClock | US500, T&amp;D19 Meta3 RClock | USDCHF, T&amp;D19 Meta3 RClock | USDJPY, T&amp;D19 Meta3 RClock | USTECH, T&amp;D19 Meta3 RClock | XAUUSD</t>
+          <t>T&amp;D19 Meta3 RClock | AUDJPY, T&amp;D19 Meta3 RClock | CHFJPY, T&amp;D19 Meta3 RClock | GBPAUD, T&amp;D19 Meta3 RClock | GBPJPY, T&amp;D19 Meta3 RClock | GBPUSD, T&amp;D19 Meta3 RClock | NZDUSD, T&amp;D19 Meta3 RClock | US30, T&amp;D19 Meta3 RClock | US500, T&amp;D19 Meta3 RClock | USDCHF, T&amp;D19 Meta3 RClock | USDJPY, T&amp;D19 Meta3 RClock | USTECH, T&amp;D19 Meta3 RClock | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -8620,20 +8665,20 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/04/2026 20:55</t>
+          <t>08/05/2026 21:13</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20073.53</v>
+        <v>20183.98</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>0.38</v>
+        <v>0.93</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>3.97</v>
       </c>
       <c r="K75" s="7" t="n">
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="L75" t="n">
         <v>20000</v>
@@ -8651,19 +8696,19 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>87.60000000000008</v>
+        <v>183.9800000000001</v>
       </c>
       <c r="V75" t="n">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>53.33333333333334</v>
+        <v>52.45098039215686</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="Y75" s="7" t="n">
         <v>3.99</v>
@@ -8675,7 +8720,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8720,20 +8765,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/04/2026 21:29</t>
+          <t>08/05/2026 21:42</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>21225.22</v>
+        <v>21311.24</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>6.12</v>
+        <v>6.55</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>2.92</v>
       </c>
       <c r="K76" s="7" t="n">
-        <v>1.39</v>
+        <v>1.37</v>
       </c>
       <c r="L76" t="n">
         <v>20000</v>
@@ -8751,19 +8796,19 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>679</v>
+        <v>767</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>1220.87</v>
+        <v>1337.19</v>
       </c>
       <c r="V76" t="n">
-        <v>412</v>
+        <v>476</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>60.67746686303387</v>
+        <v>62.05997392438071</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.39</v>
+        <v>1.38</v>
       </c>
       <c r="Y76" s="7" t="n">
         <v>2.93</v>
@@ -8775,7 +8820,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8820,20 +8865,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/04/2026 21:23</t>
+          <t>08/05/2026 21:37</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>19875.72</v>
+        <v>20035.68</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>-0.62</v>
+        <v>0.17</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="K77" s="7" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8851,19 +8896,19 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>651</v>
+        <v>704</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>-124.2800000000002</v>
+        <v>35.67999999999978</v>
       </c>
       <c r="V77" t="n">
-        <v>335</v>
+        <v>368</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>51.45929339477726</v>
+        <v>52.27272727272727</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="Y77" s="7" t="n">
         <v>4.48</v>
@@ -8875,7 +8920,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8920,20 +8965,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/04/2026 21:35</t>
+          <t>08/05/2026 21:38</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>20225.12</v>
+        <v>20461.44</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>1.13</v>
+        <v>2.31</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -8951,19 +8996,19 @@
         <v>0</v>
       </c>
       <c r="T78" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="U78" s="7" t="n">
-        <v>225.12</v>
+        <v>461.44</v>
       </c>
       <c r="V78" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="W78" s="7" t="n">
-        <v>36.20689655172414</v>
+        <v>39.34426229508197</v>
       </c>
       <c r="X78" s="7" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="Y78" s="7" t="n">
         <v>5.5</v>
@@ -8975,7 +9020,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -9020,20 +9065,20 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/04/2026 21:25</t>
+          <t>08/05/2026 21:34</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>19978.53</v>
+        <v>20342.66</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>-0.1</v>
+        <v>1.73</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>15.88</v>
       </c>
-      <c r="K79" t="n">
-        <v>1</v>
+      <c r="K79" s="7" t="n">
+        <v>1.02</v>
       </c>
       <c r="L79" t="n">
         <v>20000</v>
@@ -9051,19 +9096,19 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>37.16999999999939</v>
+        <v>342.6599999999995</v>
       </c>
       <c r="V79" t="n">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>52.74725274725275</v>
+        <v>51.69082125603865</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="Y79" s="7" t="n">
         <v>15.89</v>
@@ -9075,7 +9120,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9120,20 +9165,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/04/2026 21:09</t>
+          <t>08/05/2026 21:22</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>20725.15</v>
+        <v>20426.76</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>3.62</v>
+        <v>2.13</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9151,19 +9196,19 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>1282</v>
+        <v>1417</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>707.8299999999997</v>
+        <v>511</v>
       </c>
       <c r="V80" t="n">
-        <v>794</v>
+        <v>888</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>61.93447737909516</v>
+        <v>62.66760762173607</v>
       </c>
       <c r="X80" s="7" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="Y80" s="7" t="n">
         <v>17.52</v>
@@ -9175,7 +9220,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9220,20 +9265,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/04/2026 21:40</t>
+          <t>08/05/2026 21:51</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>19451.67</v>
+        <v>19862.14</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-2.72</v>
+        <v>-0.67</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.95</v>
+        <v>0.99</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9251,19 +9296,19 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>654</v>
+        <v>707</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>-548.3300000000002</v>
+        <v>-137.8600000000001</v>
       </c>
       <c r="V81" t="n">
-        <v>335</v>
+        <v>368</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>51.22324159021407</v>
+        <v>52.05091937765205</v>
       </c>
       <c r="X81" s="7" t="n">
-        <v>0.95</v>
+        <v>0.99</v>
       </c>
       <c r="Y81" s="7" t="n">
         <v>12.38</v>
@@ -9275,7 +9320,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9320,20 +9365,20 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/04/2026 21:23</t>
+          <t>08/05/2026 21:37</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>20067.18</v>
+        <v>20294.8</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>0.37</v>
+        <v>1.5</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>1.03</v>
+        <v>1.13</v>
       </c>
       <c r="L82" t="n">
         <v>20000</v>
@@ -9351,19 +9396,19 @@
         <v>0</v>
       </c>
       <c r="T82" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="U82" s="7" t="n">
-        <v>67.18000000000004</v>
+        <v>294.8</v>
       </c>
       <c r="V82" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="W82" s="7" t="n">
-        <v>35</v>
+        <v>38.09523809523809</v>
       </c>
       <c r="X82" s="7" t="n">
-        <v>1.03</v>
+        <v>1.13</v>
       </c>
       <c r="Y82" s="7" t="n">
         <v>5.84</v>
@@ -9375,7 +9420,7 @@
       </c>
       <c r="AA82" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB82" t="inlineStr">
@@ -9420,7 +9465,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/04/2026 21:34</t>
+          <t>08/05/2026 21:41</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9529,7 +9574,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/02/2026 03:29</t>
+          <t>08/05/2026 03:31</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9747,7 +9792,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/04/2026 19:13</t>
+          <t>08/05/2026 19:54</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9787,7 +9832,7 @@
         <v>0.39</v>
       </c>
       <c r="T86" t="n">
-        <v>3316</v>
+        <v>3337</v>
       </c>
       <c r="U86" s="7" t="n">
         <v>-7453.049999999999</v>
@@ -9796,7 +9841,7 @@
         <v>2032</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>61.27864897466827</v>
+        <v>60.8930176805514</v>
       </c>
       <c r="X86" s="7" t="n">
         <v>0.77</v>
@@ -9811,7 +9856,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -10402,7 +10447,7 @@
       </c>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 21:02</t>
+          <t>08/05/2026 21:16</t>
         </is>
       </c>
       <c r="H93" s="9" t="n">
@@ -10675,7 +10720,7 @@
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 21:19</t>
+          <t>08/05/2026 21:31</t>
         </is>
       </c>
       <c r="H96" s="9" t="n">
@@ -10766,7 +10811,7 @@
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 20:46</t>
+          <t>08/05/2026 20:58</t>
         </is>
       </c>
       <c r="H97" s="9" t="n">
@@ -10851,7 +10896,7 @@
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 20:23</t>
+          <t>08/05/2026 20:46</t>
         </is>
       </c>
       <c r="H98" s="9" t="n">
@@ -10936,7 +10981,7 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 20:21</t>
+          <t>08/05/2026 20:46</t>
         </is>
       </c>
       <c r="H99" s="9" t="n">
@@ -11021,7 +11066,7 @@
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>08/02/2026 12:58</t>
+          <t>08/05/2026 13:00</t>
         </is>
       </c>
       <c r="H100" s="9" t="n">
@@ -11800,7 +11845,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/04/2026 21:02</t>
+          <t>08/05/2026 21:16</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -11923,7 +11968,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/04/2026 21:19</t>
+          <t>08/05/2026 21:31</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -11964,7 +12009,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/04/2026 20:46</t>
+          <t>08/05/2026 20:58</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -12005,7 +12050,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/04/2026 20:23</t>
+          <t>08/05/2026 20:46</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -12046,7 +12091,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/04/2026 20:21</t>
+          <t>08/05/2026 20:46</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -12087,7 +12132,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/02/2026 12:58</t>
+          <t>08/05/2026 13:00</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -13284,7 +13329,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/02/2026 06:30</t>
+          <t>08/05/2026 06:32</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -13491,7 +13536,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/02/2026 06:32</t>
+          <t>08/05/2026 06:35</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -13514,7 +13559,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/02/2026 06:18</t>
+          <t>08/05/2026 06:25</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -13583,7 +13628,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/04/2026 16:40</t>
+          <t>08/05/2026 23:19</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -13629,11 +13674,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/04/2026 20:57</t>
+          <t>08/05/2026 21:13</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>19911.42</v>
+        <v>20114.42</v>
       </c>
     </row>
     <row r="24">
@@ -13675,11 +13720,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/04/2026 21:50</t>
+          <t>08/05/2026 21:51</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19248.09</v>
+        <v>19260.19</v>
       </c>
     </row>
     <row r="26">
@@ -13698,11 +13743,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/04/2026 21:26</t>
+          <t>08/05/2026 21:33</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20828.97</v>
+        <v>21776.68</v>
       </c>
     </row>
     <row r="27">
@@ -13721,11 +13766,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/03/2026 00:17</t>
+          <t>08/05/2026 18:25</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>17881.67</v>
+        <v>17989.59</v>
       </c>
     </row>
     <row r="28">
@@ -13744,7 +13789,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/04/2026 17:32</t>
+          <t>08/05/2026 18:42</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -13767,7 +13812,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/04/2026 17:54</t>
+          <t>08/05/2026 18:45</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -13790,7 +13835,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/04/2026 17:18</t>
+          <t>08/05/2026 18:17</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -13813,7 +13858,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/04/2026 17:51</t>
+          <t>08/05/2026 18:43</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -13836,7 +13881,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/04/2026 17:31</t>
+          <t>08/05/2026 18:20</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -13859,7 +13904,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/04/2026 16:57</t>
+          <t>08/05/2026 23:41</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -13882,7 +13927,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/04/2026 21:53</t>
+          <t>08/05/2026 22:15</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
@@ -13905,7 +13950,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>08/04/2026 22:24</t>
+          <t>08/05/2026 22:19</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
@@ -13928,11 +13973,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/04/2026 20:55</t>
+          <t>08/05/2026 21:12</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>20645.19</v>
+        <v>20642.59</v>
       </c>
     </row>
     <row r="37">
@@ -14043,7 +14088,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>08/04/2026 09:12</t>
+          <t>08/05/2026 09:14</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-10
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-05 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-10 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/05/2026 20:05</t>
+          <t>08/10/2026 05:40</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>26721.82</v>
+        <v>45677.93</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>22.53</v>
+        <v>109.46</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.02</v>
+        <v>1.07</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,19 +985,19 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-29160.46</v>
+        <v>11322.24</v>
       </c>
       <c r="P2" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>67.5</v>
+        <v>82.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.514364330256357</v>
+        <v>1.42990629365372</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>153.45</v>
+        <v>87.59</v>
       </c>
       <c r="T2" t="n">
         <v>3303</v>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>08/03/2026 16:48</t>
+          <t>08/09/2026 16:52</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/04/2026 19:14</t>
+          <t>08/07/2026 19:17</t>
         </is>
       </c>
       <c r="H4" s="7" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/05/2026 18:17</t>
+          <t>08/10/2026 13:01</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08/04/2026 09:34</t>
+          <t>08/10/2026 09:38</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/04/2026 14:44</t>
+          <t>08/10/2026 14:53</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08/03/2026 21:43</t>
+          <t>08/09/2026 22:16</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>08/03/2026 22:43</t>
+          <t>08/09/2026 23:30</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>08/03/2026 22:50</t>
+          <t>08/09/2026 23:36</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/05/2026 14:51</t>
+          <t>08/08/2026 14:56</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>08/03/2026 18:03</t>
+          <t>08/09/2026 18:14</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/05/2026 21:38</t>
+          <t>08/10/2026 07:29</t>
         </is>
       </c>
       <c r="H15" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/05/2026 18:24</t>
+          <t>08/10/2026 13:23</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/05/2026 14:47</t>
+          <t>08/08/2026 14:48</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>08/03/2026 12:07</t>
+          <t>08/09/2026 12:12</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>08/03/2026 05:32</t>
+          <t>08/09/2026 05:39</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>08/03/2026 05:32</t>
+          <t>08/09/2026 05:37</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,11 +3031,11 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/04/2026 09:08</t>
+          <t>08/10/2026 11:05</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>15090.66</v>
+        <v>15086.78</v>
       </c>
       <c r="I21" s="7" t="n">
         <v>-24.55</v>
@@ -3056,16 +3056,16 @@
         <v>40</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>-1637.92</v>
+        <v>-1651.52</v>
       </c>
       <c r="P21" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q21" s="7" t="n">
-        <v>40</v>
+        <v>37.5</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>0.5404226185966773</v>
+        <v>0.538533327744946</v>
       </c>
       <c r="S21" s="7" t="n">
         <v>12.31</v>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/05/2026 21:33</t>
+          <t>08/10/2026 07:32</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/05/2026 20:48</t>
+          <t>08/10/2026 06:31</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19795.02</v>
+        <v>19999.32</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-1.02</v>
+        <v>0</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.1</v>
       </c>
-      <c r="K23" s="7" t="n">
-        <v>0.95</v>
+      <c r="K23" t="n">
+        <v>1</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,19 +3274,19 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>185.4</v>
+        <v>237.94</v>
       </c>
       <c r="P23" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>52.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.08665697579307</v>
+        <v>1.114630104252982</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.2</v>
+        <v>4.24</v>
       </c>
       <c r="T23" t="n">
         <v>74</v>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>08/03/2026 17:59</t>
+          <t>08/09/2026 18:09</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,20 +3467,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/05/2026 21:08</t>
+          <t>08/10/2026 06:53</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16324.68</v>
+        <v>16369.48</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-18.07</v>
+        <v>-17.85</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3492,19 +3492,19 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>386.09</v>
+        <v>266.95</v>
       </c>
       <c r="P25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>47.5</v>
+        <v>50</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.842108707031931</v>
+        <v>1.999700408193836</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.95</v>
+        <v>0.6</v>
       </c>
       <c r="T25" t="n">
         <v>612</v>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/05/2026 19:20</t>
+          <t>08/10/2026 04:49</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,11 +3685,11 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/05/2026 21:01</t>
+          <t>08/10/2026 06:36</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20486.81</v>
+        <v>20487.81</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>-2.03</v>
@@ -3710,19 +3710,19 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-491.46</v>
+        <v>-376.44</v>
       </c>
       <c r="P27" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>50</v>
+        <v>52.5</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.7687758472243786</v>
+        <v>0.8128514255885058</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>6.61</v>
+        <v>6.58</v>
       </c>
       <c r="T27" t="n">
         <v>93</v>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>08/03/2026 20:53</t>
+          <t>08/09/2026 21:26</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,14 +3903,14 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/05/2026 21:07</t>
+          <t>08/10/2026 06:45</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19577.87</v>
+        <v>19585.41</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-2.12</v>
+        <v>-2.08</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
@@ -3928,16 +3928,16 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-786.77</v>
+        <v>-764.54</v>
       </c>
       <c r="P29" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>30</v>
+        <v>32.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.0894181914979804</v>
+        <v>0.09992700901791811</v>
       </c>
       <c r="S29" s="7" t="n">
         <v>3.94</v>
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08/04/2026 09:47</t>
+          <t>08/10/2026 10:00</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/05/2026 21:19</t>
+          <t>08/10/2026 07:02</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/05/2026 20:50</t>
+          <t>08/10/2026 06:31</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>08/03/2026 10:51</t>
+          <t>08/09/2026 10:57</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/05/2026 23:46</t>
+          <t>08/10/2026 11:57</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20209.64</v>
+        <v>20147.19</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>1.04</v>
+        <v>0.73</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>2.87</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.1</v>
+        <v>1.07</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,19 +4473,19 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-86.09999999999999</v>
+        <v>-127.86</v>
       </c>
       <c r="P34" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>37.5</v>
+        <v>35</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.9210707246642528</v>
+        <v>0.8848440089343613</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>1.7</v>
+        <v>1.86</v>
       </c>
       <c r="T34" t="n">
         <v>88</v>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/05/2026 22:20</t>
+          <t>08/09/2026 00:10</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/05/2026 22:05</t>
+          <t>08/10/2026 08:35</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19660.81</v>
+        <v>19835.94</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-1.7</v>
+        <v>-0.82</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>8.41</v>
+        <v>8.84</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.9</v>
+        <v>0.96</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/05/2026 21:58</t>
+          <t>08/10/2026 07:46</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/05/2026 17:21</t>
+          <t>08/08/2026 17:22</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/05/2026 22:45</t>
+          <t>08/10/2026 08:45</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>08/04/2026 09:14</t>
+          <t>08/10/2026 09:21</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>08/04/2026 07:15</t>
+          <t>08/10/2026 07:22</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,20 +5311,20 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/05/2026 20:49</t>
+          <t>08/10/2026 06:34</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
-        <v>18557.79</v>
+        <v>18459.8</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>-7.21</v>
+        <v>-7.71</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>7.45</v>
+        <v>7.95</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="L42" t="n">
         <v>20000</v>
@@ -5336,19 +5336,19 @@
         <v>40</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>-15.15</v>
+        <v>-71.22</v>
       </c>
       <c r="P42" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="Q42" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>20</v>
       </c>
       <c r="R42" s="7" t="n">
-        <v>0.6996431403647899</v>
+        <v>0.112633939695988</v>
       </c>
       <c r="S42" s="7" t="n">
-        <v>0.22</v>
+        <v>0.36</v>
       </c>
       <c r="T42" t="n">
         <v>2405</v>
@@ -5420,20 +5420,20 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/05/2026 21:13</t>
+          <t>08/10/2026 06:49</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
-        <v>17554.84</v>
+        <v>17465.15</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>-12.2</v>
+        <v>-12.65</v>
       </c>
       <c r="J43" s="7" t="n">
-        <v>12.83</v>
+        <v>13.27</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="L43" t="n">
         <v>20000</v>
@@ -5442,22 +5442,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>-71.71000000000001</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>0.2413245873889124</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
         <v>4278</v>
@@ -5529,7 +5520,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/05/2026 20:59</t>
+          <t>08/10/2026 06:35</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5551,22 +5542,13 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-1124.46</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>0.4043290318479436</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>5.73</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5638,20 +5620,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/05/2026 21:17</t>
+          <t>08/10/2026 06:56</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19990.21</v>
+        <v>19687.72</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.03</v>
+        <v>-1.55</v>
       </c>
       <c r="J45" s="7" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="K45" t="n">
-        <v>1</v>
+        <v>4.05</v>
+      </c>
+      <c r="K45" s="7" t="n">
+        <v>0.9</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5660,22 +5642,13 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-164.11</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.5792590693500833</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>1.35</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
         <v>408</v>
@@ -5747,7 +5720,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/05/2026 20:35</t>
+          <t>08/10/2026 06:14</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5769,22 +5742,13 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>19981.27</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q46" s="7" t="n">
-        <v>30.3030303030303</v>
-      </c>
-      <c r="R46" s="7" t="n">
-        <v>335.5265360790223</v>
-      </c>
-      <c r="S46" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="T46" t="n">
         <v>32</v>
@@ -5816,7 +5780,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5856,20 +5820,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/05/2026 20:54</t>
+          <t>08/10/2026 06:21</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>19194.57</v>
+        <v>19218.81</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-4.01</v>
+        <v>-3.89</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5956,7 +5920,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/05/2026 20:29</t>
+          <t>08/10/2026 06:16</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6056,20 +6020,20 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/05/2026 21:16</t>
+          <t>08/10/2026 06:59</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
-        <v>19056.79</v>
+        <v>19705.24</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>-4.72</v>
+        <v>-1.48</v>
       </c>
       <c r="J49" s="7" t="n">
         <v>7.1</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>0.77</v>
+        <v>0.93</v>
       </c>
       <c r="L49" t="n">
         <v>20000</v>
@@ -6156,20 +6120,20 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/05/2026 21:20</t>
+          <t>08/10/2026 06:56</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
-        <v>18034.01</v>
+        <v>18038.1</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>-9.84</v>
+        <v>-9.82</v>
       </c>
       <c r="J50" s="7" t="n">
         <v>20.92</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="L50" t="n">
         <v>20000</v>
@@ -6256,17 +6220,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/05/2026 20:43</t>
+          <t>08/10/2026 06:23</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
-        <v>14868.84</v>
+        <v>14817.82</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>-25.68</v>
+        <v>-25.94</v>
       </c>
       <c r="J51" s="7" t="n">
-        <v>43.16</v>
+        <v>43.2</v>
       </c>
       <c r="K51" s="7" t="n">
         <v>0.8</v>
@@ -6356,20 +6320,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/05/2026 20:44</t>
+          <t>08/10/2026 06:22</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>18073.71</v>
+        <v>19289.44</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-9.630000000000001</v>
+        <v>-3.55</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.42</v>
+        <v>0.78</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6456,20 +6420,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/05/2026 21:12</t>
+          <t>08/10/2026 07:07</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19824.34</v>
+        <v>19783.33</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-0.91</v>
+        <v>-1.11</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.77</v>
+        <v>0.73</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6556,20 +6520,20 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/05/2026 21:27</t>
+          <t>08/10/2026 07:26</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
-        <v>19715.69</v>
+        <v>19668.44</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>-1.41</v>
+        <v>-1.64</v>
       </c>
       <c r="J54" s="7" t="n">
         <v>4.64</v>
       </c>
       <c r="K54" s="7" t="n">
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="L54" t="n">
         <v>20000</v>
@@ -6656,17 +6620,17 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/05/2026 21:09</t>
+          <t>08/10/2026 06:57</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
-        <v>19685.73</v>
+        <v>19656.71</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>-1.51</v>
+        <v>-1.66</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>2.68</v>
+        <v>2.83</v>
       </c>
       <c r="K55" s="7" t="n">
         <v>0.9</v>
@@ -6756,20 +6720,20 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/05/2026 21:33</t>
+          <t>08/10/2026 07:23</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
-        <v>19882.87</v>
+        <v>19927.16</v>
       </c>
       <c r="I56" s="7" t="n">
-        <v>-0.6</v>
+        <v>-0.38</v>
       </c>
       <c r="J56" s="7" t="n">
         <v>1.98</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="L56" t="n">
         <v>20000</v>
@@ -6778,22 +6742,13 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O56" s="7" t="n">
-        <v>25.89</v>
+        <v>0</v>
       </c>
       <c r="P56" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q56" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R56" s="7" t="n">
-        <v>1.281229632848143</v>
-      </c>
-      <c r="S56" s="7" t="n">
-        <v>0.26</v>
+        <v>0</v>
       </c>
       <c r="T56" t="n">
         <v>1127</v>
@@ -6865,14 +6820,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/05/2026 20:44</t>
+          <t>08/10/2026 06:30</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19765.28</v>
+        <v>19765.92</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.2</v>
+        <v>-1.19</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6965,20 +6920,20 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/05/2026 20:55</t>
+          <t>08/10/2026 06:44</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
-        <v>17178.35</v>
+        <v>16883.07</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>-14.11</v>
+        <v>-15.59</v>
       </c>
       <c r="J58" s="7" t="n">
-        <v>15.49</v>
+        <v>15.65</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="L58" t="n">
         <v>20000</v>
@@ -7065,20 +7020,20 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/05/2026 21:05</t>
+          <t>08/10/2026 06:39</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
-        <v>20094.92</v>
+        <v>20063.41</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>0.48</v>
+        <v>0.31</v>
       </c>
       <c r="J59" s="7" t="n">
-        <v>0.55</v>
+        <v>0.61</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>1.17</v>
+        <v>1.1</v>
       </c>
       <c r="L59" t="n">
         <v>20000</v>
@@ -7165,20 +7120,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/05/2026 21:03</t>
+          <t>08/10/2026 06:41</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>20423.33</v>
+        <v>20116.65</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-3.97</v>
+        <v>-5.41</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="L60" s="7" t="n">
         <v>21100.65</v>
@@ -7265,14 +7220,14 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/05/2026 21:26</t>
+          <t>08/10/2026 07:14</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>20681.68</v>
+        <v>20577.19</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-3.47</v>
+        <v>-3.95</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>13.96</v>
@@ -7365,7 +7320,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/05/2026 21:34</t>
+          <t>08/10/2026 07:19</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7465,20 +7420,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/05/2026 21:33</t>
+          <t>08/10/2026 07:03</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18908.85</v>
+        <v>18796.69</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-5.47</v>
+        <v>-6.03</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>6.74</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7565,20 +7520,20 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/05/2026 21:40</t>
+          <t>08/10/2026 07:32</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
-        <v>19444.2</v>
+        <v>19296.04</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>-2.78</v>
+        <v>-3.51</v>
       </c>
       <c r="J64" s="7" t="n">
         <v>3.87</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>0.7</v>
+        <v>0.66</v>
       </c>
       <c r="L64" t="n">
         <v>20000</v>
@@ -7665,20 +7620,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/05/2026 21:15</t>
+          <t>08/10/2026 06:59</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19540.97</v>
+        <v>19166.19</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-2.3</v>
+        <v>-4.17</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>11.64</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7765,20 +7720,20 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/05/2026 21:22</t>
+          <t>08/10/2026 07:03</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
-        <v>20077.9</v>
+        <v>20000.8</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>0.4</v>
+        <v>0.01</v>
       </c>
       <c r="J66" s="7" t="n">
         <v>2.86</v>
       </c>
-      <c r="K66" s="7" t="n">
-        <v>1.04</v>
+      <c r="K66" t="n">
+        <v>1</v>
       </c>
       <c r="L66" t="n">
         <v>20000</v>
@@ -7865,20 +7820,20 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/05/2026 21:46</t>
+          <t>08/10/2026 07:49</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
-        <v>20174.46</v>
+        <v>19839.1</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>0.86</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="J67" s="7" t="n">
         <v>2.99</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>1.07</v>
+        <v>0.95</v>
       </c>
       <c r="L67" t="n">
         <v>20000</v>
@@ -7965,7 +7920,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/05/2026 12:57</t>
+          <t>08/08/2026 13:00</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8065,7 +8020,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/05/2026 12:58</t>
+          <t>08/08/2026 13:00</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8165,7 +8120,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/05/2026 13:12</t>
+          <t>08/08/2026 13:13</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8265,20 +8220,20 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/05/2026 21:29</t>
+          <t>08/10/2026 07:05</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
-        <v>19903.15</v>
+        <v>19872.72</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>-0.47</v>
+        <v>-0.61</v>
       </c>
       <c r="J71" s="7" t="n">
         <v>1.34</v>
       </c>
       <c r="K71" s="7" t="n">
-        <v>0.89</v>
+        <v>0.86</v>
       </c>
       <c r="L71" t="n">
         <v>20000</v>
@@ -8365,20 +8320,20 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/05/2026 21:49</t>
+          <t>08/10/2026 08:02</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
-        <v>19754.91</v>
+        <v>19722.2</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>-1.2</v>
+        <v>-1.35</v>
       </c>
       <c r="J72" s="7" t="n">
         <v>2.67</v>
       </c>
       <c r="K72" s="7" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="L72" t="n">
         <v>20000</v>
@@ -8465,20 +8420,20 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/05/2026 21:27</t>
+          <t>08/10/2026 07:19</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
-        <v>19561.27</v>
+        <v>19494.14</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>-2.19</v>
+        <v>-2.51</v>
       </c>
       <c r="J73" s="7" t="n">
         <v>4.3</v>
       </c>
       <c r="K73" s="7" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L73" t="n">
         <v>20000</v>
@@ -8565,20 +8520,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/05/2026 21:34</t>
+          <t>08/10/2026 07:41</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20634.27</v>
+        <v>20525.49</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>3.18</v>
+        <v>2.64</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>1.73</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.62</v>
+        <v>1.38</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8665,20 +8620,20 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/05/2026 21:13</t>
+          <t>08/10/2026 06:48</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20183.98</v>
+        <v>20229.52</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>0.93</v>
+        <v>1.17</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>3.97</v>
       </c>
       <c r="K75" s="7" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="L75" t="n">
         <v>20000</v>
@@ -8765,20 +8720,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/05/2026 21:42</t>
+          <t>08/10/2026 07:32</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>21311.24</v>
+        <v>21140.34</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>6.55</v>
+        <v>5.69</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>2.92</v>
       </c>
       <c r="K76" s="7" t="n">
-        <v>1.37</v>
+        <v>1.27</v>
       </c>
       <c r="L76" t="n">
         <v>20000</v>
@@ -8865,20 +8820,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/05/2026 21:37</t>
+          <t>08/10/2026 07:16</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>20035.68</v>
+        <v>20438.14</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>0.17</v>
+        <v>2.18</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="K77" s="7" t="n">
-        <v>1.01</v>
+        <v>1.08</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8965,20 +8920,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/05/2026 21:38</t>
+          <t>08/10/2026 07:26</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>20461.44</v>
+        <v>20359.19</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>2.31</v>
+        <v>1.81</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -9065,20 +9020,20 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/05/2026 21:34</t>
+          <t>08/10/2026 07:23</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>20342.66</v>
+        <v>20852.56</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>1.73</v>
+        <v>4.29</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>15.88</v>
       </c>
       <c r="K79" s="7" t="n">
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="L79" t="n">
         <v>20000</v>
@@ -9165,20 +9120,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/05/2026 21:22</t>
+          <t>08/10/2026 06:52</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>20426.76</v>
+        <v>19974.33</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>2.13</v>
+        <v>-0.12</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
-      <c r="K80" s="7" t="n">
-        <v>1.02</v>
+      <c r="K80" t="n">
+        <v>1</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9265,20 +9220,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/05/2026 21:51</t>
+          <t>08/10/2026 07:45</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>19862.14</v>
+        <v>20963.29</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-0.67</v>
+        <v>4.84</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.99</v>
+        <v>1.07</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9365,20 +9320,20 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/05/2026 21:37</t>
+          <t>08/10/2026 07:23</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>20294.8</v>
+        <v>20199.69</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>1.5</v>
+        <v>1.04</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>1.13</v>
+        <v>1.08</v>
       </c>
       <c r="L82" t="n">
         <v>20000</v>
@@ -9465,14 +9420,14 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/05/2026 21:41</t>
+          <t>08/10/2026 07:32</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
-        <v>399.91</v>
+        <v>368.46</v>
       </c>
       <c r="I83" s="7" t="n">
-        <v>-99.68000000000001</v>
+        <v>-99.7</v>
       </c>
       <c r="J83" s="7" t="n">
         <v>99.94</v>
@@ -9490,19 +9445,19 @@
         <v>40</v>
       </c>
       <c r="O83" s="7" t="n">
-        <v>-4830.84</v>
+        <v>-1505.78</v>
       </c>
       <c r="P83" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q83" s="7" t="n">
-        <v>27.5</v>
+        <v>30</v>
       </c>
       <c r="R83" s="7" t="n">
-        <v>0.2114871085053179</v>
+        <v>0.1853955682506708</v>
       </c>
       <c r="S83" s="7" t="n">
-        <v>25.3</v>
+        <v>7.9</v>
       </c>
       <c r="T83" t="n">
         <v>631</v>
@@ -9574,7 +9529,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/05/2026 03:31</t>
+          <t>08/08/2026 03:33</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9683,7 +9638,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/03/2026 21:32</t>
+          <t>08/09/2026 22:10</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9792,14 +9747,14 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/05/2026 19:54</t>
+          <t>08/10/2026 05:22</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>26828.95</v>
+        <v>26959.76</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>-30.14</v>
+        <v>-29.8</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>37.71</v>
@@ -9817,16 +9772,16 @@
         <v>40</v>
       </c>
       <c r="O86" s="7" t="n">
-        <v>257.12</v>
+        <v>134.59</v>
       </c>
       <c r="P86" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Q86" s="7" t="n">
-        <v>92.5</v>
+        <v>90</v>
       </c>
       <c r="R86" s="7" t="n">
-        <v>3.604801945091683</v>
+        <v>2.02008488706988</v>
       </c>
       <c r="S86" s="7" t="n">
         <v>0.39</v>
@@ -9901,7 +9856,7 @@
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 20:40</t>
+          <t>08/09/2026 21:09</t>
         </is>
       </c>
       <c r="H87" s="9" t="n">
@@ -9992,7 +9947,7 @@
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 19:57</t>
+          <t>08/07/2026 19:59</t>
         </is>
       </c>
       <c r="H88" s="9" t="n">
@@ -10083,7 +10038,7 @@
       </c>
       <c r="G89" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 13:04</t>
+          <t>08/09/2026 13:14</t>
         </is>
       </c>
       <c r="H89" s="9" t="n">
@@ -10174,7 +10129,7 @@
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 09:36</t>
+          <t>08/10/2026 09:42</t>
         </is>
       </c>
       <c r="H90" s="9" t="n">
@@ -10265,7 +10220,7 @@
       </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 00:45</t>
+          <t>08/10/2026 01:17</t>
         </is>
       </c>
       <c r="H91" s="9" t="n">
@@ -10356,7 +10311,7 @@
       </c>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 21:27</t>
+          <t>08/09/2026 22:04</t>
         </is>
       </c>
       <c r="H92" s="9" t="n">
@@ -10447,7 +10402,7 @@
       </c>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>08/05/2026 21:16</t>
+          <t>08/10/2026 06:52</t>
         </is>
       </c>
       <c r="H93" s="9" t="n">
@@ -10538,7 +10493,7 @@
       </c>
       <c r="G94" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 17:46</t>
+          <t>08/09/2026 17:53</t>
         </is>
       </c>
       <c r="H94" s="9" t="n">
@@ -10629,7 +10584,7 @@
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>08/04/2026 14:26</t>
+          <t>08/10/2026 14:33</t>
         </is>
       </c>
       <c r="H95" s="9" t="n">
@@ -10720,7 +10675,7 @@
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>08/05/2026 21:31</t>
+          <t>08/10/2026 07:17</t>
         </is>
       </c>
       <c r="H96" s="9" t="n">
@@ -10811,20 +10766,20 @@
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>08/05/2026 20:58</t>
+          <t>08/10/2026 06:38</t>
         </is>
       </c>
       <c r="H97" s="9" t="n">
-        <v>20617.37</v>
+        <v>20576.42</v>
       </c>
       <c r="I97" s="9" t="n">
-        <v>3.09</v>
+        <v>2.88</v>
       </c>
       <c r="J97" s="9" t="n">
         <v>3.12</v>
       </c>
       <c r="K97" s="9" t="n">
-        <v>1.23</v>
+        <v>1.21</v>
       </c>
       <c r="L97" s="8" t="n">
         <v>20000</v>
@@ -10896,7 +10851,7 @@
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>08/05/2026 20:46</t>
+          <t>08/10/2026 06:34</t>
         </is>
       </c>
       <c r="H98" s="9" t="n">
@@ -10981,7 +10936,7 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>08/05/2026 20:46</t>
+          <t>08/10/2026 06:35</t>
         </is>
       </c>
       <c r="H99" s="9" t="n">
@@ -11066,7 +11021,7 @@
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>08/05/2026 13:00</t>
+          <t>08/08/2026 13:03</t>
         </is>
       </c>
       <c r="H100" s="9" t="n">
@@ -11151,7 +11106,7 @@
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 18:51</t>
+          <t>08/09/2026 19:11</t>
         </is>
       </c>
       <c r="H101" s="9" t="n">
@@ -11242,7 +11197,7 @@
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 18:40</t>
+          <t>08/09/2026 19:03</t>
         </is>
       </c>
       <c r="H102" s="9" t="n">
@@ -11424,7 +11379,7 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>08/03/2026 23:11</t>
+          <t>08/09/2026 23:59</t>
         </is>
       </c>
       <c r="H104" s="9" t="n">
@@ -11599,7 +11554,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>08/03/2026 20:40</t>
+          <t>08/09/2026 21:09</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -11640,7 +11595,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08/04/2026 19:57</t>
+          <t>08/07/2026 19:59</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -11681,7 +11636,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08/03/2026 13:04</t>
+          <t>08/09/2026 13:14</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -11722,7 +11677,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08/04/2026 09:36</t>
+          <t>08/10/2026 09:42</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -11763,7 +11718,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08/04/2026 00:45</t>
+          <t>08/10/2026 01:17</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -11804,7 +11759,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08/03/2026 21:27</t>
+          <t>08/09/2026 22:04</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -11845,7 +11800,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/05/2026 21:16</t>
+          <t>08/10/2026 06:52</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -11886,7 +11841,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>08/03/2026 17:46</t>
+          <t>08/09/2026 17:53</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -11927,7 +11882,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/04/2026 14:26</t>
+          <t>08/10/2026 14:33</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -11968,7 +11923,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/05/2026 21:31</t>
+          <t>08/10/2026 07:17</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -12009,14 +11964,14 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/05/2026 20:58</t>
+          <t>08/10/2026 06:38</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>20617.37</v>
+        <v>20576.42</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>3.09</v>
+        <v>2.88</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -12050,7 +12005,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/05/2026 20:46</t>
+          <t>08/10/2026 06:34</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -12091,7 +12046,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/05/2026 20:46</t>
+          <t>08/10/2026 06:35</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -12132,7 +12087,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/05/2026 13:00</t>
+          <t>08/08/2026 13:03</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -12173,7 +12128,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/03/2026 18:51</t>
+          <t>08/09/2026 19:11</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -12214,7 +12169,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/03/2026 18:40</t>
+          <t>08/09/2026 19:03</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -12296,7 +12251,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/03/2026 23:11</t>
+          <t>08/09/2026 23:59</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -12320,7 +12275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -13093,7 +13048,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>55951</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -13103,7 +13058,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EA FX RSI AUDUSD</t>
+          <t>Gold Reaper</t>
         </is>
       </c>
       <c r="D33" t="b">
@@ -13118,48 +13073,148 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>55967</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>Midnight Raven GBPUSD 30m</t>
         </is>
       </c>
       <c r="D34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS242t2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>56911</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>AuRange Hunter</t>
+        </is>
+      </c>
+      <c r="D35" t="b">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>VPS242t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>56912</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Smart Owl FX</t>
+        </is>
+      </c>
+      <c r="D36" t="b">
+        <v>1</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>VPS242t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>662434</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>EA FX RSI AUDUSD</t>
+        </is>
+      </c>
+      <c r="D37" t="b">
+        <v>1</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>662435</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Aggv1 Pro Filter 60</t>
+        </is>
+      </c>
+      <c r="D38" t="b">
+        <v>0</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>600025868</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>demo</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>FTMO Manual Trading</t>
         </is>
       </c>
-      <c r="D35" t="b">
-        <v>1</v>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D39" t="b">
+        <v>1</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>
@@ -13237,7 +13292,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08/03/2026 20:12</t>
+          <t>08/09/2026 20:37</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -13260,7 +13315,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/04/2026 10:01</t>
+          <t>08/10/2026 10:11</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -13283,7 +13338,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08/03/2026 20:01</t>
+          <t>08/09/2026 20:31</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -13306,7 +13361,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>07/31/2026 14:11</t>
+          <t>08/09/2026 15:22</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -13329,7 +13384,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/05/2026 06:32</t>
+          <t>08/08/2026 06:34</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -13352,7 +13407,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08/04/2026 04:41</t>
+          <t>08/10/2026 04:51</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -13375,7 +13430,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08/03/2026 13:58</t>
+          <t>08/09/2026 14:04</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
@@ -13398,7 +13453,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08/04/2026 05:23</t>
+          <t>08/10/2026 05:32</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -13421,7 +13476,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/04/2026 12:52</t>
+          <t>08/10/2026 12:58</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -13444,7 +13499,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08/03/2026 20:52</t>
+          <t>08/09/2026 21:23</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -13467,7 +13522,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/04/2026 14:59</t>
+          <t>08/10/2026 15:10</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -13490,7 +13545,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08/03/2026 20:00</t>
+          <t>08/06/2026 20:06</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
@@ -13536,7 +13591,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/05/2026 06:35</t>
+          <t>08/08/2026 06:39</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -13559,7 +13614,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/05/2026 06:25</t>
+          <t>08/08/2026 06:30</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -13582,7 +13637,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08/03/2026 22:01</t>
+          <t>08/09/2026 22:52</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -13605,7 +13660,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>07/31/2026 14:03</t>
+          <t>08/09/2026 15:08</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
@@ -13628,7 +13683,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/05/2026 23:19</t>
+          <t>08/10/2026 10:54</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -13651,7 +13706,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08/03/2026 21:10</t>
+          <t>08/09/2026 21:35</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -13674,11 +13729,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/05/2026 21:13</t>
+          <t>08/10/2026 07:00</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20114.42</v>
+        <v>20082.4</v>
       </c>
     </row>
     <row r="24">
@@ -13720,11 +13775,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/05/2026 21:51</t>
+          <t>08/10/2026 07:54</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19260.19</v>
+        <v>19546.98</v>
       </c>
     </row>
     <row r="26">
@@ -13743,11 +13798,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/05/2026 21:33</t>
+          <t>08/10/2026 07:14</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21776.68</v>
+        <v>21739.79</v>
       </c>
     </row>
     <row r="27">
@@ -13766,11 +13821,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/05/2026 18:25</t>
+          <t>08/10/2026 14:38</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>17989.59</v>
+        <v>18401.17</v>
       </c>
     </row>
     <row r="28">
@@ -13789,7 +13844,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/05/2026 18:42</t>
+          <t>08/10/2026 04:21</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -13812,7 +13867,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/05/2026 18:45</t>
+          <t>08/10/2026 04:31</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -13835,7 +13890,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/05/2026 18:17</t>
+          <t>08/10/2026 13:37</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -13858,7 +13913,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/05/2026 18:43</t>
+          <t>08/10/2026 04:22</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -13881,7 +13936,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/05/2026 18:20</t>
+          <t>08/10/2026 13:51</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -13904,7 +13959,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/05/2026 23:41</t>
+          <t>08/10/2026 12:23</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -13927,7 +13982,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/05/2026 22:15</t>
+          <t>08/10/2026 09:02</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
@@ -13950,7 +14005,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>08/05/2026 22:19</t>
+          <t>08/10/2026 08:39</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
@@ -13973,11 +14028,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/05/2026 21:12</t>
+          <t>08/10/2026 07:45</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>20642.59</v>
+        <v>20682.12</v>
       </c>
     </row>
     <row r="37">
@@ -14019,7 +14074,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/03/2026 20:00</t>
+          <t>08/09/2026 20:25</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -14042,7 +14097,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/03/2026 20:01</t>
+          <t>08/06/2026 20:21</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -14065,7 +14120,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/03/2026 23:06</t>
+          <t>08/09/2026 23:53</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
@@ -14088,7 +14143,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>08/05/2026 09:14</t>
+          <t>08/10/2026 09:22</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-12
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -1000,19 +1000,19 @@
         <v>28.07</v>
       </c>
       <c r="T2" t="n">
-        <v>3321</v>
+        <v>3326</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>25145.10999999999</v>
+        <v>28937.96</v>
       </c>
       <c r="V2" t="n">
-        <v>2095</v>
+        <v>2098</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.0834086118639</v>
+        <v>63.07877330126278</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -3728,7 +3728,7 @@
         <v>96</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>487.5299999999999</v>
+        <v>481.6799999999999</v>
       </c>
       <c r="V27" t="n">
         <v>44</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>08/09/2026 21:26</t>
+          <t>08/12/2026 21:51</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -5442,22 +5442,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>-50.87</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>0.2037877602128658</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
         <v>4278</v>
@@ -5551,22 +5542,13 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-1124.46</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>0.4043290318479436</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>5.73</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5660,22 +5642,13 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-361.12</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.1572658747753845</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>1.97</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
         <v>440</v>
@@ -5769,22 +5742,13 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>19979.66</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q46" s="7" t="n">
-        <v>29.41176470588236</v>
-      </c>
-      <c r="R46" s="7" t="n">
-        <v>326.7199217476361</v>
-      </c>
-      <c r="S46" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="T46" t="n">
         <v>33</v>
@@ -5816,7 +5780,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -6887,19 +6851,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-266.64</v>
+        <v>-261.41</v>
       </c>
       <c r="V57" t="n">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.98395721925134</v>
+        <v>44.13333333333333</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -8478,22 +8442,13 @@
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O73" s="7" t="n">
-        <v>28.34</v>
+        <v>0</v>
       </c>
       <c r="P73" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q73" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R73" s="7" t="n">
-        <v>1.110036886041545</v>
-      </c>
-      <c r="S73" s="7" t="n">
-        <v>0.73</v>
+        <v>0</v>
       </c>
       <c r="T73" t="n">
         <v>329</v>
@@ -8696,16 +8651,16 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>-88.36000000000013</v>
+        <v>-61.21000000000004</v>
       </c>
       <c r="V75" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>53.2258064516129</v>
+        <v>53.6</v>
       </c>
       <c r="X75" s="7" t="n">
         <v>0.98</v>
@@ -8796,16 +8751,16 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>1016.91</v>
+        <v>1011.24</v>
       </c>
       <c r="V76" t="n">
         <v>639</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>60.11288805268109</v>
+        <v>60.05639097744361</v>
       </c>
       <c r="X76" s="7" t="n">
         <v>1.2</v>
@@ -8896,16 +8851,16 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>284.1899999999999</v>
+        <v>289.4799999999998</v>
       </c>
       <c r="V77" t="n">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>51.52792413066386</v>
+        <v>51.62986330178759</v>
       </c>
       <c r="X77" s="7" t="n">
         <v>1.05</v>
@@ -9096,19 +9051,19 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>-442.6600000000008</v>
+        <v>-339.2900000000009</v>
       </c>
       <c r="V79" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>52.96442687747036</v>
+        <v>53.33333333333334</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="Y79" s="7" t="n">
         <v>17</v>
@@ -9196,16 +9151,16 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>1839</v>
+        <v>1840</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>329.1399999999992</v>
+        <v>317.0899999999992</v>
       </c>
       <c r="V80" t="n">
         <v>1141</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>62.04458945078846</v>
+        <v>62.01086956521738</v>
       </c>
       <c r="X80" s="7" t="n">
         <v>1.01</v>
@@ -9296,7 +9251,7 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>883</v>
+        <v>885</v>
       </c>
       <c r="U81" s="7" t="n">
         <v>189.1600000000003</v>
@@ -9305,7 +9260,7 @@
         <v>457</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>51.75537938844847</v>
+        <v>51.63841807909605</v>
       </c>
       <c r="X81" s="7" t="n">
         <v>1.01</v>
@@ -9793,16 +9748,16 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>763.4899999999999</v>
+        <v>763.4699999999999</v>
       </c>
       <c r="V86" t="n">
         <v>28</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>47.45762711864407</v>
+        <v>46.66666666666666</v>
       </c>
       <c r="X86" s="7" t="n">
         <v>2.11</v>
@@ -10193,13 +10148,13 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>74.56</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="V90" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W90" s="7" t="n">
         <v>100</v>
@@ -10290,13 +10245,13 @@
         <v>0</v>
       </c>
       <c r="T91" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U91" s="7" t="n">
-        <v>68.13</v>
+        <v>90.04999999999998</v>
       </c>
       <c r="V91" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W91" s="7" t="n">
         <v>100</v>
@@ -10584,20 +10539,20 @@
         <v>3</v>
       </c>
       <c r="U94" s="7" t="n">
-        <v>50.26</v>
+        <v>82.94</v>
       </c>
       <c r="V94" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W94" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>100</v>
       </c>
       <c r="Y94" s="7" t="n">
         <v>0</v>
       </c>
       <c r="Z94" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="AA94" t="inlineStr">
@@ -10678,19 +10633,19 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="U95" s="7" t="n">
-        <v>142.52</v>
+        <v>179.78</v>
       </c>
       <c r="V95" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="W95" s="7" t="n">
-        <v>65.625</v>
+        <v>63.1578947368421</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>3.05</v>
+        <v>3.58</v>
       </c>
       <c r="Y95" s="7" t="n">
         <v>0.02</v>
@@ -10712,7 +10667,7 @@
       </c>
       <c r="AC95" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro</t>
+          <t>T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10778,19 +10733,19 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="U96" s="7" t="n">
-        <v>428.5000000000001</v>
+        <v>584.9000000000001</v>
       </c>
       <c r="V96" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="W96" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>64.1025641025641</v>
       </c>
       <c r="X96" s="7" t="n">
-        <v>2.97</v>
+        <v>3.69</v>
       </c>
       <c r="Y96" s="7" t="n">
         <v>0.07000000000000001</v>
@@ -10812,7 +10767,7 @@
       </c>
       <c r="AC96" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro</t>
+          <t>T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10878,19 +10833,19 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="U97" s="7" t="n">
-        <v>737.65</v>
+        <v>1066.09</v>
       </c>
       <c r="V97" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="W97" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>64.1025641025641</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>3</v>
+        <v>3.89</v>
       </c>
       <c r="Y97" s="7" t="n">
         <v>0.12</v>
@@ -10912,7 +10867,7 @@
       </c>
       <c r="AC97" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro</t>
+          <t>T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10978,19 +10933,19 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="U98" s="7" t="n">
-        <v>91.63000000000002</v>
+        <v>144.74</v>
       </c>
       <c r="V98" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W98" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>40</v>
       </c>
       <c r="X98" s="7" t="n">
-        <v>2.67</v>
+        <v>3.65</v>
       </c>
       <c r="Y98" s="7" t="n">
         <v>0.04</v>
@@ -11012,7 +10967,7 @@
       </c>
       <c r="AC98" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | USDCAD.pro</t>
+          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11078,7 +11033,7 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="U99" s="7" t="n">
         <v>-271.2000000000001</v>
@@ -11087,7 +11042,7 @@
         <v>40</v>
       </c>
       <c r="W99" s="7" t="n">
-        <v>52.63157894736842</v>
+        <v>51.94805194805194</v>
       </c>
       <c r="X99" s="7" t="n">
         <v>0.7</v>
@@ -11514,16 +11469,16 @@
         <v>0.96</v>
       </c>
       <c r="T103" t="n">
-        <v>3375</v>
+        <v>3417</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-7382.309999999999</v>
+        <v>-7422.57</v>
       </c>
       <c r="V103" t="n">
-        <v>2054</v>
+        <v>2062</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>60.85925925925926</v>
+        <v>60.34533216271583</v>
       </c>
       <c r="X103" s="7" t="n">
         <v>0.77</v>
@@ -11538,7 +11493,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -12515,23 +12470,17 @@
         <v>0</v>
       </c>
       <c r="N114" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O114" s="9" t="n">
-        <v>-27.2</v>
+        <v>0</v>
       </c>
       <c r="P114" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q114" s="9" t="n">
-        <v>60</v>
-      </c>
-      <c r="R114" s="9" t="n">
-        <v>0.9300015440835864</v>
-      </c>
-      <c r="S114" s="9" t="n">
-        <v>0.72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q114" s="8" t="n"/>
+      <c r="R114" s="8" t="n"/>
+      <c r="S114" s="8" t="n"/>
       <c r="T114" s="8" t="n">
         <v>0</v>
       </c>
@@ -14217,7 +14166,7 @@
         <v>2.91</v>
       </c>
       <c r="I15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -15963,7 +15912,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08/09/2026 21:23</t>
+          <t>08/12/2026 21:50</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -16170,7 +16119,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08/09/2026 21:35</t>
+          <t>08/12/2026 21:56</t>
         </is>
       </c>
       <c r="E22" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-13
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-12 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-13 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/12/2026 08:23</t>
+          <t>08/13/2026 20:00</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>55345.31</v>
+        <v>55619.4</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>153.79</v>
+        <v>154.23</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>35573.48</v>
+        <v>37022.48</v>
       </c>
       <c r="P2" t="n">
         <v>36</v>
@@ -994,22 +994,22 @@
         <v>90</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>5.537757799026461</v>
+        <v>5.875497459696216</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>28.07</v>
+        <v>8.41</v>
       </c>
       <c r="T2" t="n">
-        <v>3326</v>
+        <v>3331</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>28937.96</v>
+        <v>30619.39999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2098</v>
+        <v>2102</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.07877330126278</v>
+        <v>63.10417292104474</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.07</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,11 +1178,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/10/2026 19:19</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="n">
-        <v>23788.13</v>
+          <t>08/13/2026 19:21</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
       </c>
       <c r="I4" s="7" t="n">
         <v>14.67</v>
@@ -1197,31 +1197,31 @@
         <v>50545.04</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>26858.3</v>
+        <v>50646.43</v>
       </c>
       <c r="N4" t="n">
         <v>40</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>-7626.92</v>
+        <v>-31339.33</v>
       </c>
       <c r="P4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Q4" s="7" t="n">
-        <v>52.5</v>
+        <v>50</v>
       </c>
       <c r="R4" s="7" t="n">
-        <v>0.7350524707215493</v>
+        <v>0.4020916555470635</v>
       </c>
       <c r="S4" s="7" t="n">
-        <v>116.25</v>
+        <v>300.52</v>
       </c>
       <c r="T4" t="n">
         <v>1000</v>
       </c>
       <c r="U4" s="7" t="n">
-        <v>101.3900000000008</v>
+        <v>101.3899999999999</v>
       </c>
       <c r="V4" t="n">
         <v>601</v>
@@ -1233,7 +1233,7 @@
         <v>1</v>
       </c>
       <c r="Y4" s="7" t="n">
-        <v>12.52</v>
+        <v>25.2</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/12/2026 19:58</t>
+          <t>08/13/2026 18:56</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08/10/2026 09:38</t>
+          <t>08/13/2026 09:40</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/10/2026 14:53</t>
+          <t>08/13/2026 15:03</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08/09/2026 22:16</t>
+          <t>08/12/2026 22:38</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>08/09/2026 23:30</t>
+          <t>08/12/2026 23:53</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>08/09/2026 23:36</t>
+          <t>08/12/2026 23:53</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,14 +2159,14 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/12/2026 08:09</t>
+          <t>08/13/2026 19:51</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>5187.94</v>
+        <v>5192.94</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>-1.27</v>
+        <v>-1.17</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>8.949999999999999</v>
@@ -2184,7 +2184,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>-4802.53</v>
+        <v>-4829.63</v>
       </c>
       <c r="P13" t="n">
         <v>29</v>
@@ -2193,22 +2193,22 @@
         <v>72.5</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>0.6952136949579363</v>
+        <v>0.6934938287901788</v>
       </c>
       <c r="S13" s="7" t="n">
-        <v>98.29000000000001</v>
+        <v>98.48</v>
       </c>
       <c r="T13" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>121.44</v>
+        <v>126.4399999999999</v>
       </c>
       <c r="V13" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>67.21311475409836</v>
       </c>
       <c r="X13" s="7" t="n">
         <v>1.13</v>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2377,11 +2377,11 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/12/2026 10:03</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>19022.8</v>
+          <t>08/13/2026 05:44</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>-9.83</v>
@@ -2395,14 +2395,14 @@
       <c r="L15" s="7" t="n">
         <v>26775.1</v>
       </c>
-      <c r="M15" t="n">
-        <v>6000</v>
+      <c r="M15" s="7" t="n">
+        <v>25022.8</v>
       </c>
       <c r="N15" t="n">
         <v>40</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>4720.440000000001</v>
+        <v>-14301.96</v>
       </c>
       <c r="P15" t="n">
         <v>14</v>
@@ -2411,10 +2411,10 @@
         <v>35</v>
       </c>
       <c r="R15" s="7" t="n">
-        <v>1.615467659667678</v>
+        <v>0.4641871296654289</v>
       </c>
       <c r="S15" s="7" t="n">
-        <v>21.5</v>
+        <v>193.26</v>
       </c>
       <c r="T15" t="n">
         <v>174</v>
@@ -2432,7 +2432,7 @@
         <v>0.73</v>
       </c>
       <c r="Y15" s="7" t="n">
-        <v>9.32</v>
+        <v>100</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/12/2026 06:52</t>
+          <t>08/13/2026 19:04</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/12/2026 17:59</t>
+          <t>08/13/2026 21:59</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/12/2026 10:08</t>
+          <t>08/13/2026 20:56</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3183,7 +3183,7 @@
         <v>22</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-2200.229999999999</v>
+        <v>-2200.23</v>
       </c>
       <c r="V22" t="n">
         <v>6</v>
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/12/2026 08:59</t>
+          <t>08/13/2026 20:19</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19999.32</v>
+        <v>19867.23</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0</v>
+        <v>-0.66</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.1</v>
       </c>
-      <c r="K23" t="n">
-        <v>1</v>
+      <c r="K23" s="7" t="n">
+        <v>0.97</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>237.94</v>
+        <v>245.92</v>
       </c>
       <c r="P23" t="n">
         <v>22</v>
@@ -3283,25 +3283,25 @@
         <v>55.00000000000001</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.114630104252982</v>
+        <v>1.11893178059137</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.24</v>
+        <v>4.21</v>
       </c>
       <c r="T23" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-0.6799999999995778</v>
+        <v>-132.7699999999999</v>
       </c>
       <c r="V23" t="n">
         <v>42</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>53.84615384615385</v>
+        <v>53.16455696202531</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>6.11</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/12/2026 09:34</t>
-        </is>
-      </c>
-      <c r="H25" t="n">
-        <v>16555</v>
+          <t>08/13/2026 20:38</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>16557.78</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-16.91</v>
+        <v>-16.89</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,31 +3492,31 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>447.45</v>
+        <v>325.55</v>
       </c>
       <c r="P25" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>52.5</v>
+        <v>62.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>2.962069721552291</v>
+        <v>2.572173661080794</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.6</v>
+        <v>0.43</v>
       </c>
       <c r="T25" t="n">
-        <v>649</v>
+        <v>657</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3443.199999999999</v>
+        <v>-3442.22</v>
       </c>
       <c r="V25" t="n">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>39.59938366718028</v>
+        <v>39.5738203957382</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>0.67</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/12/2026 07:38</t>
+          <t>08/13/2026 19:33</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,14 +3685,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/12/2026 09:19</t>
+          <t>08/13/2026 20:30</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20487.53</v>
+        <v>20481.68</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-2.03</v>
+        <v>-2.06</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>7.39</v>
@@ -3710,25 +3710,25 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-343.09</v>
+        <v>-640.9599999999999</v>
       </c>
       <c r="P27" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>52.5</v>
+        <v>50</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.8265557858551136</v>
+        <v>0.6769273419188991</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>6.57</v>
+        <v>6.66</v>
       </c>
       <c r="T27" t="n">
         <v>96</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>481.6799999999999</v>
+        <v>481.68</v>
       </c>
       <c r="V27" t="n">
         <v>44</v>
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/12/2026 09:19</t>
+          <t>08/13/2026 20:29</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19561.99</v>
+        <v>19579.62</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-2.2</v>
+        <v>-2.11</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,34 +3928,34 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-798.54</v>
+        <v>-779.26</v>
       </c>
       <c r="P29" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>27.5</v>
+        <v>30</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.08545970956067617</v>
+        <v>0.1060148909564399</v>
       </c>
       <c r="S29" s="7" t="n">
         <v>4.02</v>
       </c>
       <c r="T29" t="n">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-438.01</v>
+        <v>-420.3800000000002</v>
       </c>
       <c r="V29" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>46.61016949152542</v>
+        <v>46.28099173553719</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08/10/2026 10:00</t>
+          <t>08/13/2026 10:15</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/12/2026 09:44</t>
+          <t>08/13/2026 20:41</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4164,7 +4164,7 @@
         <v>66</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>681.2099999999999</v>
+        <v>681.2099999999998</v>
       </c>
       <c r="V31" t="n">
         <v>19</v>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/12/2026 09:00</t>
+          <t>08/13/2026 20:19</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4448,14 +4448,14 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/12/2026 18:04</t>
+          <t>08/13/2026 22:04</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>19991.51</v>
+        <v>20012.3</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>-0.04</v>
+        <v>0.06</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>3.42</v>
@@ -4473,7 +4473,7 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-63.00999999999999</v>
+        <v>-189.39</v>
       </c>
       <c r="P34" t="n">
         <v>14</v>
@@ -4482,25 +4482,25 @@
         <v>35</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.9441370994911077</v>
+        <v>0.8318103103769815</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>2.85</v>
+        <v>2.87</v>
       </c>
       <c r="T34" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>-8.489999999999952</v>
+        <v>42.39000000000005</v>
       </c>
       <c r="V34" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>40</v>
+        <v>40.19607843137255</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>3.43</v>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/12/2026 11:10</t>
+          <t>08/13/2026 18:11</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19935.93</v>
+        <v>19813.9</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.31</v>
+        <v>-0.93</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>134.0399999999998</v>
+        <v>-186.1000000000001</v>
       </c>
       <c r="V36" t="n">
         <v>40</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>50.63291139240506</v>
+        <v>48.78048780487805</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>1.03</v>
+        <v>0.96</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.83</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/12/2026 10:26</t>
+          <t>08/13/2026 21:07</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/12/2026 11:10</t>
+          <t>08/13/2026 21:30</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>08/10/2026 09:21</t>
+          <t>08/13/2026 09:24</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>08/10/2026 07:22</t>
+          <t>08/13/2026 07:24</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/12/2026 09:16</t>
+          <t>08/13/2026 20:30</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/12/2026 09:53</t>
+          <t>08/13/2026 20:48</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,13 +5442,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T43" t="n">
         <v>4278</v>
@@ -5520,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/12/2026 09:13</t>
+          <t>08/13/2026 20:28</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5542,13 +5551,22 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5620,17 +5638,17 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/12/2026 09:34</t>
+          <t>08/13/2026 20:36</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19632.97</v>
+        <v>19636.01</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-1.82</v>
+        <v>-1.8</v>
       </c>
       <c r="J45" s="7" t="n">
-        <v>4.34</v>
+        <v>4.38</v>
       </c>
       <c r="K45" s="7" t="n">
         <v>0.88</v>
@@ -5642,25 +5660,34 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-370.61</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.1500550408219429</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>2.01</v>
       </c>
       <c r="T45" t="n">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-380.64</v>
+        <v>-373.4599999999999</v>
       </c>
       <c r="V45" t="n">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>54.54545454545454</v>
+        <v>54.7085201793722</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0.88</v>
@@ -5675,7 +5702,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5720,7 +5747,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/12/2026 08:46</t>
+          <t>08/13/2026 20:13</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5742,13 +5769,22 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>19979.66</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q46" s="7" t="n">
+        <v>29.41176470588236</v>
+      </c>
+      <c r="R46" s="7" t="n">
+        <v>326.7199217476361</v>
+      </c>
+      <c r="S46" s="7" t="n">
+        <v>0.1</v>
       </c>
       <c r="T46" t="n">
         <v>33</v>
@@ -5780,7 +5816,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5820,20 +5856,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/12/2026 09:02</t>
+          <t>08/13/2026 20:23</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>19254.74</v>
+        <v>19146.11</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-3.71</v>
+        <v>-4.25</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5851,19 +5887,19 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-841.3500000000001</v>
+        <v>-902.8500000000001</v>
       </c>
       <c r="V47" t="n">
         <v>24</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>41.37931034482759</v>
+        <v>40</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5875,7 +5911,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5920,7 +5956,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/12/2026 08:52</t>
+          <t>08/13/2026 20:19</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6020,7 +6056,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/12/2026 09:35</t>
+          <t>08/13/2026 20:38</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6120,7 +6156,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/12/2026 09:31</t>
+          <t>08/13/2026 20:35</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6220,7 +6256,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/12/2026 09:05</t>
+          <t>08/13/2026 20:21</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6320,20 +6356,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/12/2026 09:00</t>
+          <t>08/13/2026 20:20</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19289.44</v>
+        <v>19520.45</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-3.55</v>
+        <v>-2.39</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.78</v>
+        <v>0.85</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6354,16 +6390,16 @@
         <v>38</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-710.5600000000002</v>
+        <v>-479.5500000000002</v>
       </c>
       <c r="V52" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>26.31578947368421</v>
+        <v>28.94736842105263</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.78</v>
+        <v>0.85</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>10.19</v>
@@ -6375,7 +6411,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6420,20 +6456,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/12/2026 09:49</t>
+          <t>08/13/2026 20:44</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19794.17</v>
+        <v>19740.55</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.05</v>
+        <v>-1.32</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6451,19 +6487,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-231.5200000000001</v>
+        <v>-259.45</v>
       </c>
       <c r="V53" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.9098712446352</v>
+        <v>36.25</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6475,7 +6511,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6520,7 +6556,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/12/2026 10:04</t>
+          <t>08/13/2026 20:54</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6620,7 +6656,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/12/2026 09:34</t>
+          <t>08/13/2026 20:36</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6720,7 +6756,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/12/2026 10:06</t>
+          <t>08/13/2026 20:54</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6820,14 +6856,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/12/2026 09:02</t>
+          <t>08/13/2026 20:19</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19741.04</v>
+        <v>19737.71</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.31</v>
+        <v>-1.32</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6851,16 +6887,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>750</v>
+        <v>761</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-261.41</v>
+        <v>-262.29</v>
       </c>
       <c r="V57" t="n">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.13333333333333</v>
+        <v>44.2838370565046</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.8</v>
@@ -6875,7 +6911,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6920,20 +6956,20 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/12/2026 09:26</t>
+          <t>08/13/2026 20:35</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
-        <v>16883.07</v>
+        <v>16865.67</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>-15.59</v>
+        <v>-15.68</v>
       </c>
       <c r="J58" s="7" t="n">
-        <v>15.65</v>
+        <v>15.68</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="L58" t="n">
         <v>20000</v>
@@ -7020,7 +7056,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/12/2026 09:09</t>
+          <t>08/13/2026 20:23</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7120,14 +7156,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/12/2026 09:18</t>
+          <t>08/13/2026 20:29</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>20456.01</v>
+        <v>20442.76</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-3.82</v>
+        <v>-3.89</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
@@ -7220,7 +7256,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/12/2026 09:53</t>
+          <t>08/13/2026 20:51</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7320,7 +7356,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/12/2026 09:52</t>
+          <t>08/13/2026 20:47</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7420,20 +7456,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/12/2026 09:48</t>
+          <t>08/13/2026 20:43</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18796.69</v>
+        <v>18670.29</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.03</v>
+        <v>-6.66</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>6.74</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.33</v>
+        <v>0.31</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7451,16 +7487,16 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1275.61</v>
+        <v>-1329.71</v>
       </c>
       <c r="V63" t="n">
         <v>3</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>8.571428571428571</v>
+        <v>8.108108108108109</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>0.31</v>
@@ -7475,7 +7511,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7520,7 +7556,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/12/2026 10:10</t>
+          <t>08/13/2026 20:58</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7620,20 +7656,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/12/2026 09:41</t>
+          <t>08/13/2026 20:40</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19398.06</v>
+        <v>19197.65</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-3.02</v>
+        <v>-4.02</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>11.64</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7720,7 +7756,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/12/2026 09:34</t>
+          <t>08/13/2026 20:35</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7820,7 +7856,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/12/2026 10:22</t>
+          <t>08/13/2026 21:08</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -8220,7 +8256,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/12/2026 09:43</t>
+          <t>08/13/2026 20:44</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8320,7 +8356,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/12/2026 10:35</t>
+          <t>08/13/2026 21:11</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8420,7 +8456,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/12/2026 09:49</t>
+          <t>08/13/2026 20:45</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8520,20 +8556,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/12/2026 10:15</t>
+          <t>08/13/2026 21:03</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20633.89</v>
+        <v>20671.54</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>3.18</v>
+        <v>3.37</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>1.73</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.46</v>
+        <v>1.48</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8551,19 +8587,19 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>686.09</v>
+        <v>671.5400000000001</v>
       </c>
       <c r="V74" t="n">
         <v>62</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>68.13186813186813</v>
+        <v>67.39130434782609</v>
       </c>
       <c r="X74" s="7" t="n">
-        <v>1.5</v>
+        <v>1.48</v>
       </c>
       <c r="Y74" s="7" t="n">
         <v>1.73</v>
@@ -8575,7 +8611,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8620,20 +8656,20 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/12/2026 09:23</t>
+          <t>08/13/2026 20:34</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>19849.14</v>
+        <v>20036.74</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>-0.72</v>
+        <v>0.22</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K75" s="7" t="n">
-        <v>0.96</v>
+        <v>1.01</v>
       </c>
       <c r="L75" t="n">
         <v>20000</v>
@@ -8651,19 +8687,19 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>-61.21000000000004</v>
+        <v>36.74000000000007</v>
       </c>
       <c r="V75" t="n">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>53.6</v>
+        <v>54.26356589147287</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>0.98</v>
+        <v>1.01</v>
       </c>
       <c r="Y75" s="7" t="n">
         <v>4.5</v>
@@ -8675,7 +8711,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8720,20 +8756,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/12/2026 10:06</t>
+          <t>08/13/2026 20:54</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>21085.29</v>
-      </c>
-      <c r="I76" s="7" t="n">
-        <v>5.43</v>
+        <v>20798.51</v>
+      </c>
+      <c r="I76" t="n">
+        <v>4</v>
       </c>
       <c r="J76" s="7" t="n">
-        <v>2.92</v>
+        <v>3.36</v>
       </c>
       <c r="K76" s="7" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="L76" t="n">
         <v>20000</v>
@@ -8751,22 +8787,22 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1064</v>
+        <v>1104</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>1011.24</v>
+        <v>832.1400000000003</v>
       </c>
       <c r="V76" t="n">
-        <v>639</v>
+        <v>662</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>60.05639097744361</v>
+        <v>59.96376811594203</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.2</v>
+        <v>1.15</v>
       </c>
       <c r="Y76" s="7" t="n">
-        <v>2.93</v>
+        <v>3.35</v>
       </c>
       <c r="Z76" t="inlineStr">
         <is>
@@ -8775,7 +8811,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8820,20 +8856,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/12/2026 09:55</t>
+          <t>08/13/2026 20:48</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>20333.92</v>
+        <v>20095.35</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>1.66</v>
+        <v>0.46</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="K77" s="7" t="n">
-        <v>1.05</v>
+        <v>1.01</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8851,19 +8887,19 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>951</v>
+        <v>990</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>289.4799999999998</v>
+        <v>105.8200000000001</v>
       </c>
       <c r="V77" t="n">
-        <v>491</v>
+        <v>507</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>51.62986330178759</v>
+        <v>51.21212121212121</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>1.05</v>
+        <v>1.02</v>
       </c>
       <c r="Y77" s="7" t="n">
         <v>4.48</v>
@@ -8875,7 +8911,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8920,20 +8956,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/12/2026 10:02</t>
+          <t>08/13/2026 20:53</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>20287.91</v>
+        <v>20269.57</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>1.44</v>
+        <v>1.35</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -8951,19 +8987,19 @@
         <v>0</v>
       </c>
       <c r="T78" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="U78" s="7" t="n">
-        <v>287.91</v>
+        <v>269.5699999999999</v>
       </c>
       <c r="V78" t="n">
         <v>29</v>
       </c>
       <c r="W78" s="7" t="n">
-        <v>40.84507042253522</v>
+        <v>40.27777777777778</v>
       </c>
       <c r="X78" s="7" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="Y78" s="7" t="n">
         <v>5.5</v>
@@ -9020,20 +9056,20 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/12/2026 10:00</t>
+          <t>08/13/2026 20:53</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>19306.09</v>
+        <v>20043.76</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>-3.44</v>
+        <v>0.26</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>16.96</v>
       </c>
-      <c r="K79" s="7" t="n">
-        <v>0.96</v>
+      <c r="K79" t="n">
+        <v>1</v>
       </c>
       <c r="L79" t="n">
         <v>20000</v>
@@ -9051,19 +9087,19 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>-339.2900000000009</v>
+        <v>43.75999999999976</v>
       </c>
       <c r="V79" t="n">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>53.33333333333334</v>
+        <v>53.99239543726235</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="Y79" s="7" t="n">
         <v>17</v>
@@ -9075,7 +9111,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9120,20 +9156,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/12/2026 09:35</t>
+          <t>08/13/2026 20:36</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>20411.73</v>
+        <v>20373.31</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>2.09</v>
+        <v>1.9</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9151,19 +9187,19 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>1840</v>
+        <v>1904</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>317.0899999999992</v>
+        <v>392.8400000000004</v>
       </c>
       <c r="V80" t="n">
-        <v>1141</v>
+        <v>1181</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>62.01086956521738</v>
+        <v>62.02731092436975</v>
       </c>
       <c r="X80" s="7" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="Y80" s="7" t="n">
         <v>17.52</v>
@@ -9175,7 +9211,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9220,20 +9256,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/12/2026 10:19</t>
+          <t>08/13/2026 21:03</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>20176.05</v>
+        <v>19704.56</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>0.9</v>
+        <v>-1.45</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>1.01</v>
+        <v>0.98</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9251,19 +9287,19 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>885</v>
+        <v>925</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>189.1600000000003</v>
+        <v>-255.2100000000003</v>
       </c>
       <c r="V81" t="n">
-        <v>457</v>
+        <v>474</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>51.63841807909605</v>
+        <v>51.24324324324324</v>
       </c>
       <c r="X81" s="7" t="n">
-        <v>1.01</v>
+        <v>0.98</v>
       </c>
       <c r="Y81" s="7" t="n">
         <v>12.38</v>
@@ -9275,7 +9311,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9320,14 +9356,14 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/12/2026 10:03</t>
+          <t>08/13/2026 20:56</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>20064.15</v>
+        <v>20047.14</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>0.35</v>
+        <v>0.26</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
@@ -9420,7 +9456,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/12/2026 11:30</t>
+          <t>08/13/2026 21:44</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9517,7 +9553,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/12/2026 11:17</t>
+          <t>08/13/2026 21:37</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9617,20 +9653,20 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/12/2026 10:16</t>
+          <t>08/13/2026 21:00</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
-        <v>3276.54</v>
+        <v>3095.33</v>
       </c>
       <c r="I85" s="7" t="n">
-        <v>9.220000000000001</v>
+        <v>3.18</v>
       </c>
       <c r="J85" s="7" t="n">
-        <v>3.02</v>
+        <v>5.53</v>
       </c>
       <c r="K85" s="7" t="n">
-        <v>4.03</v>
+        <v>1.35</v>
       </c>
       <c r="L85" t="n">
         <v>3000</v>
@@ -9717,20 +9753,20 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/12/2026 10:31</t>
+          <t>08/13/2026 21:11</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20768.09</v>
+        <v>20775.94</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>3.85</v>
+        <v>3.89</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>2.18</v>
       </c>
       <c r="K86" s="7" t="n">
-        <v>2.12</v>
+        <v>2.13</v>
       </c>
       <c r="L86" t="n">
         <v>20000</v>
@@ -9748,19 +9784,19 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>763.4699999999999</v>
+        <v>775.9399999999999</v>
       </c>
       <c r="V86" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>46.66666666666666</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="X86" s="7" t="n">
-        <v>2.11</v>
+        <v>2.13</v>
       </c>
       <c r="Y86" s="7" t="n">
         <v>2.17</v>
@@ -9772,7 +9808,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9817,20 +9853,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/12/2026 10:04</t>
+          <t>08/13/2026 20:54</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>20283.8</v>
+        <v>20364.8</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>1.42</v>
+        <v>1.83</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>1.07</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>4.33</v>
+        <v>4.52</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9848,19 +9884,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="U87" s="7" t="n">
-        <v>282.6</v>
+        <v>364.8</v>
       </c>
       <c r="V87" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W87" s="7" t="n">
-        <v>72.72727272727273</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>4.27</v>
+        <v>4.46</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>0.33</v>
@@ -9872,7 +9908,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9917,20 +9953,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/12/2026 10:09</t>
+          <t>08/13/2026 20:56</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20202.2</v>
+        <v>20392.52</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>1.01</v>
+        <v>1.96</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>1.98</v>
+        <v>2.9</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -9948,19 +9984,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="U88" s="7" t="n">
-        <v>226</v>
+        <v>343.2</v>
       </c>
       <c r="V88" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="W88" s="7" t="n">
-        <v>91.30434782608695</v>
+        <v>92.5925925925926</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>2.09</v>
+        <v>2.66</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -9972,7 +10008,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10017,20 +10053,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/12/2026 10:08</t>
+          <t>08/13/2026 20:58</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>21078.6</v>
+        <v>21288.9</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="J89" t="n">
-        <v>0</v>
-      </c>
-      <c r="K89" t="n">
-        <v>0</v>
+        <v>6.46</v>
+      </c>
+      <c r="J89" s="7" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="K89" s="7" t="n">
+        <v>4.06</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10048,19 +10084,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>662.2200000000003</v>
+        <v>1288.9</v>
       </c>
       <c r="V89" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>83.33333333333334</v>
+        <v>87.5</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>2.57</v>
+        <v>4.06</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>1.99</v>
@@ -10072,7 +10108,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10117,20 +10153,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/12/2026 09:01</t>
+          <t>08/13/2026 20:22</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>20042.04</v>
+        <v>20119.27</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="J90" t="n">
-        <v>0</v>
-      </c>
-      <c r="K90" t="n">
-        <v>0</v>
+        <v>0.6</v>
+      </c>
+      <c r="J90" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K90" s="7" t="n">
+        <v>3.38</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10148,19 +10184,22 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>82.90000000000001</v>
+        <v>119.27</v>
       </c>
       <c r="V90" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>100</v>
+        <v>85.71428571428571</v>
+      </c>
+      <c r="X90" s="7" t="n">
+        <v>3.38</v>
       </c>
       <c r="Y90" s="7" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10169,7 +10208,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10179,7 +10218,7 @@
       </c>
       <c r="AC90" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 MOL | EURUSD.pro, T&amp;D19L13 L8 MOL | US500, T&amp;D19L13 L8 MOL | USTECH</t>
+          <t>T&amp;D19L13 L8 MOL | AUDJPY.pro, T&amp;D19L13 L8 MOL | EURUSD.pro, T&amp;D19L13 L8 MOL | US30, T&amp;D19L13 L8 MOL | US500, T&amp;D19L13 L8 MOL | USTECH, T&amp;D19L13 L8 MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10214,20 +10253,20 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/12/2026 09:04</t>
+          <t>08/13/2026 20:20</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
-        <v>20000.6</v>
+        <v>20176.99</v>
       </c>
       <c r="I91" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J91" t="n">
-        <v>0</v>
-      </c>
-      <c r="K91" t="n">
-        <v>0</v>
+        <v>0.89</v>
+      </c>
+      <c r="J91" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K91" s="7" t="n">
+        <v>2.76</v>
       </c>
       <c r="L91" t="n">
         <v>20000</v>
@@ -10245,19 +10284,22 @@
         <v>0</v>
       </c>
       <c r="T91" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="U91" s="7" t="n">
-        <v>90.04999999999998</v>
+        <v>176.99</v>
       </c>
       <c r="V91" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="W91" s="7" t="n">
-        <v>100</v>
+        <v>84.61538461538461</v>
+      </c>
+      <c r="X91" s="7" t="n">
+        <v>2.76</v>
       </c>
       <c r="Y91" s="7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Z91" t="inlineStr">
         <is>
@@ -10266,7 +10308,7 @@
       </c>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB91" t="inlineStr">
@@ -10276,7 +10318,7 @@
       </c>
       <c r="AC91" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L8 Agg | EURUSD.pro, T&amp;D19L13 L8 Agg | US500, T&amp;D19L13 L8 Agg | USTECH</t>
+          <t>T&amp;D19L13 L8 Agg | AUDJPY.pro, T&amp;D19L13 L8 Agg | EURUSD.pro, T&amp;D19L13 L8 Agg | US30, T&amp;D19L13 L8 Agg | US500, T&amp;D19L13 L8 Agg | USTECH, T&amp;D19L13 L8 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10311,20 +10353,20 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/12/2026 09:02</t>
+          <t>08/13/2026 20:20</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
-        <v>20007.89</v>
+        <v>20005.68</v>
       </c>
       <c r="I92" s="7" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="J92" t="n">
-        <v>0</v>
-      </c>
-      <c r="K92" t="n">
-        <v>0</v>
+        <v>0.03</v>
+      </c>
+      <c r="J92" s="7" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K92" s="7" t="n">
+        <v>3.57</v>
       </c>
       <c r="L92" t="n">
         <v>20000</v>
@@ -10342,19 +10384,22 @@
         <v>0</v>
       </c>
       <c r="T92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U92" s="7" t="n">
-        <v>7.890000000000001</v>
+        <v>5.680000000000001</v>
       </c>
       <c r="V92" t="n">
         <v>2</v>
       </c>
       <c r="W92" s="7" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
+      </c>
+      <c r="X92" s="7" t="n">
+        <v>3.57</v>
       </c>
       <c r="Y92" s="7" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="Z92" t="inlineStr">
         <is>
@@ -10373,7 +10418,7 @@
       </c>
       <c r="AC92" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Prop | AUDUSD.pro, T&amp;D19L13 L11 Prop | GBPCHF.pro</t>
+          <t>T&amp;D19L13 L11 Prop | AUDJPY.pro, T&amp;D19L13 L11 Prop | AUDUSD.pro, T&amp;D19L13 L11 Prop | GBPCHF.pro</t>
         </is>
       </c>
     </row>
@@ -10408,20 +10453,20 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/12/2026 09:01</t>
+          <t>08/13/2026 20:20</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
-        <v>20024.65</v>
+        <v>20017.75</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="J93" t="n">
-        <v>0</v>
-      </c>
-      <c r="K93" t="n">
-        <v>0</v>
+        <v>0.09</v>
+      </c>
+      <c r="J93" s="7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K93" s="7" t="n">
+        <v>3.57</v>
       </c>
       <c r="L93" t="n">
         <v>20000</v>
@@ -10439,19 +10484,22 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U93" s="7" t="n">
-        <v>24.65</v>
+        <v>17.75</v>
       </c>
       <c r="V93" t="n">
         <v>2</v>
       </c>
       <c r="W93" s="7" t="n">
-        <v>100</v>
+        <v>66.66666666666666</v>
+      </c>
+      <c r="X93" s="7" t="n">
+        <v>3.57</v>
       </c>
       <c r="Y93" s="7" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="Z93" t="inlineStr">
         <is>
@@ -10470,7 +10518,7 @@
       </c>
       <c r="AC93" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 MOL | AUDUSD.pro, T&amp;D19L13 L11 MOL | GBPCHF.pro</t>
+          <t>T&amp;D19L13 L11 MOL | AUDJPY.pro, T&amp;D19L13 L11 MOL | AUDUSD.pro, T&amp;D19L13 L11 MOL | GBPCHF.pro</t>
         </is>
       </c>
     </row>
@@ -10505,20 +10553,20 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/12/2026 09:04</t>
+          <t>08/13/2026 20:21</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
-        <v>20050.26</v>
+        <v>20069.14</v>
       </c>
       <c r="I94" s="7" t="n">
-        <v>0.25</v>
+        <v>0.34</v>
       </c>
       <c r="J94" s="7" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="K94" t="n">
-        <v>0</v>
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="K94" s="7" t="n">
+        <v>6.01</v>
       </c>
       <c r="L94" t="n">
         <v>20000</v>
@@ -10536,19 +10584,22 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U94" s="7" t="n">
-        <v>82.94</v>
+        <v>69.14</v>
       </c>
       <c r="V94" t="n">
         <v>3</v>
       </c>
       <c r="W94" s="7" t="n">
-        <v>100</v>
+        <v>75</v>
+      </c>
+      <c r="X94" s="7" t="n">
+        <v>6.01</v>
       </c>
       <c r="Y94" s="7" t="n">
-        <v>0</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z94" t="inlineStr">
         <is>
@@ -10567,7 +10618,7 @@
       </c>
       <c r="AC94" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Agg | AUDUSD.pro, T&amp;D19L13 L11 Agg | GBPCHF.pro, T&amp;D19L13 L11 Agg | XAUUSD</t>
+          <t>T&amp;D19L13 L11 Agg | AUDJPY.pro, T&amp;D19L13 L11 Agg | AUDUSD.pro, T&amp;D19L13 L11 Agg | GBPCHF.pro, T&amp;D19L13 L11 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10602,20 +10653,20 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/12/2026 08:53</t>
+          <t>08/13/2026 20:16</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
-        <v>100094.63</v>
+        <v>99821.64999999999</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>0.1</v>
+        <v>-0.17</v>
       </c>
       <c r="J95" s="7" t="n">
-        <v>0.02</v>
+        <v>0.47</v>
       </c>
       <c r="K95" s="7" t="n">
-        <v>3.37</v>
+        <v>0.85</v>
       </c>
       <c r="L95" t="n">
         <v>100000</v>
@@ -10633,22 +10684,22 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>38</v>
+        <v>149</v>
       </c>
       <c r="U95" s="7" t="n">
-        <v>179.78</v>
+        <v>-169.06</v>
       </c>
       <c r="V95" t="n">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="W95" s="7" t="n">
-        <v>63.1578947368421</v>
+        <v>52.34899328859061</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>3.58</v>
+        <v>0.86</v>
       </c>
       <c r="Y95" s="7" t="n">
-        <v>0.02</v>
+        <v>0.47</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -10657,7 +10708,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
@@ -10667,7 +10718,7 @@
       </c>
       <c r="AC95" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | US30, T&amp;D19L13 Meta4 Prop | US500, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10702,20 +10753,20 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/12/2026 08:55</t>
+          <t>08/13/2026 20:19</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
-        <v>100288.57</v>
+        <v>99976.53</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>0.28</v>
+        <v>-0.03</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.12</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>3.09</v>
+        <v>0.99</v>
       </c>
       <c r="L96" t="n">
         <v>100000</v>
@@ -10733,22 +10784,22 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>39</v>
+        <v>165</v>
       </c>
       <c r="U96" s="7" t="n">
-        <v>584.9000000000001</v>
+        <v>-1.340000000000032</v>
       </c>
       <c r="V96" t="n">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="W96" s="7" t="n">
-        <v>64.1025641025641</v>
+        <v>53.33333333333334</v>
       </c>
       <c r="X96" s="7" t="n">
-        <v>3.69</v>
+        <v>1</v>
       </c>
       <c r="Y96" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.11</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -10757,7 +10808,7 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr">
@@ -10767,7 +10818,7 @@
       </c>
       <c r="AC96" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | US30, T&amp;D19L13 Meta4 MOL | US500, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10802,20 +10853,20 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/12/2026 09:07</t>
+          <t>08/13/2026 20:22</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
-        <v>100518.39</v>
+        <v>100196.16</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>0.52</v>
+        <v>0.2</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>0.12</v>
+        <v>1.81</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>3.01</v>
+        <v>1.04</v>
       </c>
       <c r="L97" t="n">
         <v>100000</v>
@@ -10833,22 +10884,22 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>39</v>
+        <v>165</v>
       </c>
       <c r="U97" s="7" t="n">
-        <v>1066.09</v>
+        <v>247.3000000000002</v>
       </c>
       <c r="V97" t="n">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="W97" s="7" t="n">
-        <v>64.1025641025641</v>
+        <v>53.33333333333334</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>3.89</v>
+        <v>1.06</v>
       </c>
       <c r="Y97" s="7" t="n">
-        <v>0.12</v>
+        <v>1.81</v>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
@@ -10857,7 +10908,7 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB97" t="inlineStr">
@@ -10867,7 +10918,7 @@
       </c>
       <c r="AC97" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | US30, T&amp;D19L13 Meta4 Agg | US500, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10902,20 +10953,20 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/12/2026 08:56</t>
+          <t>08/13/2026 20:16</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
-        <v>100087.63</v>
+        <v>99857.37</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>0.08</v>
+        <v>-0.15</v>
       </c>
       <c r="J98" s="7" t="n">
-        <v>0.05</v>
+        <v>0.49</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>3.07</v>
+        <v>0.83</v>
       </c>
       <c r="L98" t="n">
         <v>100000</v>
@@ -10933,22 +10984,22 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="U98" s="7" t="n">
-        <v>144.74</v>
+        <v>-124.0499999999999</v>
       </c>
       <c r="V98" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="W98" s="7" t="n">
-        <v>40</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="X98" s="7" t="n">
-        <v>3.65</v>
+        <v>0.85</v>
       </c>
       <c r="Y98" s="7" t="n">
-        <v>0.04</v>
+        <v>0.49</v>
       </c>
       <c r="Z98" t="inlineStr">
         <is>
@@ -10957,7 +11008,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
@@ -10967,7 +11018,7 @@
       </c>
       <c r="AC98" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11002,20 +11053,20 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/12/2026 09:02</t>
+          <t>08/13/2026 20:21</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
-        <v>99669.13</v>
+        <v>99489.06</v>
       </c>
       <c r="I99" s="7" t="n">
-        <v>-0.33</v>
+        <v>-0.52</v>
       </c>
       <c r="J99" s="7" t="n">
         <v>0.67</v>
       </c>
       <c r="K99" s="7" t="n">
-        <v>0.62</v>
+        <v>0.72</v>
       </c>
       <c r="L99" t="n">
         <v>100000</v>
@@ -11033,19 +11084,19 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>77</v>
+        <v>134</v>
       </c>
       <c r="U99" s="7" t="n">
-        <v>-271.2000000000001</v>
+        <v>-508.8100000000001</v>
       </c>
       <c r="V99" t="n">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="W99" s="7" t="n">
-        <v>51.94805194805194</v>
+        <v>51.49253731343284</v>
       </c>
       <c r="X99" s="7" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="Y99" s="7" t="n">
         <v>0.67</v>
@@ -11057,7 +11108,7 @@
       </c>
       <c r="AA99" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB99" t="inlineStr">
@@ -11067,7 +11118,7 @@
       </c>
       <c r="AC99" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 Prop | AUDJPY.pro, T&amp;D19L13 L9 Prop | AUDNZD.pro, T&amp;D19L13 L9 Prop | AUDUSD.pro, T&amp;D19L13 L9 Prop | CHFJPY.pro, T&amp;D19L13 L9 Prop | EURCHF.pro, T&amp;D19L13 L9 Prop | EURJPY.pro, T&amp;D19L13 L9 Prop | EURUSD.pro, T&amp;D19L13 L9 Prop | GBPCHF.pro, T&amp;D19L13 L9 Prop | GBPJPY.pro, T&amp;D19L13 L9 Prop | GBPNZD.pro, T&amp;D19L13 L9 Prop | NZDUSD.pro, T&amp;D19L13 L9 Prop | US30, T&amp;D19L13 L9 Prop | US500, T&amp;D19L13 L9 Prop | USDCHF.pro, T&amp;D19L13 L9 Prop | USTECH, T&amp;D19L13 L9 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 L9 Prop | AUDJPY.pro, T&amp;D19L13 L9 Prop | AUDNZD.pro, T&amp;D19L13 L9 Prop | AUDUSD.pro, T&amp;D19L13 L9 Prop | CHFJPY.pro, T&amp;D19L13 L9 Prop | EURCHF.pro, T&amp;D19L13 L9 Prop | EURJPY.pro, T&amp;D19L13 L9 Prop | EURUSD.pro, T&amp;D19L13 L9 Prop | GBPCHF.pro, T&amp;D19L13 L9 Prop | GBPJPY.pro, T&amp;D19L13 L9 Prop | GBPNZD.pro, T&amp;D19L13 L9 Prop | NZDUSD.pro, T&amp;D19L13 L9 Prop | US30, T&amp;D19L13 L9 Prop | US500, T&amp;D19L13 L9 Prop | USDCAD.pro, T&amp;D19L13 L9 Prop | USDCHF.pro, T&amp;D19L13 L9 Prop | USTECH, T&amp;D19L13 L9 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11102,17 +11153,17 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/12/2026 09:59</t>
+          <t>08/13/2026 20:52</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
-        <v>368.46</v>
+        <v>300.95</v>
       </c>
       <c r="I100" s="7" t="n">
-        <v>-99.7</v>
+        <v>-99.76000000000001</v>
       </c>
       <c r="J100" s="7" t="n">
-        <v>99.94</v>
+        <v>99.95</v>
       </c>
       <c r="K100" s="7" t="n">
         <v>0.82</v>
@@ -11127,19 +11178,19 @@
         <v>40</v>
       </c>
       <c r="O100" s="7" t="n">
-        <v>-1505.78</v>
+        <v>-1564.07</v>
       </c>
       <c r="P100" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q100" s="7" t="n">
-        <v>30</v>
+        <v>27.5</v>
       </c>
       <c r="R100" s="7" t="n">
-        <v>0.1853955682506708</v>
+        <v>0.1431959988386553</v>
       </c>
       <c r="S100" s="7" t="n">
-        <v>7.9</v>
+        <v>8.26</v>
       </c>
       <c r="T100" t="n">
         <v>631</v>
@@ -11251,26 +11302,26 @@
         <v>9.640000000000001</v>
       </c>
       <c r="T101" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="U101" s="7" t="n">
-        <v>272.14</v>
+        <v>-43.44999999999997</v>
       </c>
       <c r="V101" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="W101" s="7" t="n">
-        <v>45.71428571428572</v>
+        <v>40.98360655737705</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>1.29</v>
+        <v>0.98</v>
       </c>
       <c r="Y101" s="7" t="n">
-        <v>1.08</v>
+        <v>2.56</v>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="AA101" t="inlineStr">
@@ -11280,12 +11331,12 @@
       </c>
       <c r="AB101" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC101" t="inlineStr">
         <is>
-          <t>Gold Talon | XAUUSD.PRO</t>
+          <t>Gold Talon | EURUSD.PRO, Gold Talon | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
@@ -11320,7 +11371,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>08/09/2026 22:10</t>
+          <t>08/12/2026 22:38</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11429,14 +11480,14 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/12/2026 08:01</t>
+          <t>08/13/2026 19:45</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>26838.83</v>
+        <v>26875.34</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-30.11</v>
+        <v>-30.01</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
@@ -11454,7 +11505,7 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>17.97000000000001</v>
+        <v>16.5</v>
       </c>
       <c r="P103" t="n">
         <v>30</v>
@@ -11463,22 +11514,22 @@
         <v>75</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>1.053595395031167</v>
+        <v>1.049211130663008</v>
       </c>
       <c r="S103" s="7" t="n">
         <v>0.96</v>
       </c>
       <c r="T103" t="n">
-        <v>3417</v>
+        <v>3433</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-7422.57</v>
+        <v>-7406.660000000001</v>
       </c>
       <c r="V103" t="n">
-        <v>2062</v>
+        <v>2065</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>60.34533216271583</v>
+        <v>60.15147101660355</v>
       </c>
       <c r="X103" s="7" t="n">
         <v>0.77</v>
@@ -11493,7 +11544,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11629,7 +11680,7 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>08/10/2026 20:01</t>
+          <t>08/13/2026 20:03</t>
         </is>
       </c>
       <c r="H105" s="9" t="n">
@@ -11811,7 +11862,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>08/10/2026 09:42</t>
+          <t>08/13/2026 09:52</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -11902,7 +11953,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>08/10/2026 01:17</t>
+          <t>08/13/2026 01:44</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -11993,7 +12044,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>08/09/2026 22:04</t>
+          <t>08/12/2026 22:37</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12084,7 +12135,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:34</t>
+          <t>08/13/2026 20:36</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12266,7 +12317,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>08/10/2026 14:33</t>
+          <t>08/13/2026 14:50</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12357,7 +12408,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 10:00</t>
+          <t>08/13/2026 20:53</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12448,7 +12499,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 03:41</t>
+          <t>08/13/2026 20:27</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12533,7 +12584,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:16</t>
+          <t>08/13/2026 20:30</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12618,7 +12669,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:11</t>
+          <t>08/13/2026 20:25</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12788,20 +12839,20 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:06</t>
+          <t>08/13/2026 20:22</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
-        <v>50072.49</v>
+        <v>49693.02</v>
       </c>
       <c r="I118" s="9" t="n">
-        <v>0.15</v>
+        <v>-0.6</v>
       </c>
       <c r="J118" s="9" t="n">
-        <v>1.24</v>
+        <v>1.79</v>
       </c>
       <c r="K118" s="9" t="n">
-        <v>1.05</v>
+        <v>0.88</v>
       </c>
       <c r="L118" s="8" t="n">
         <v>50000</v>
@@ -12873,20 +12924,20 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:08</t>
+          <t>08/13/2026 20:24</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
-        <v>98308.98</v>
+        <v>97124.75</v>
       </c>
       <c r="I119" s="9" t="n">
-        <v>-1.69</v>
+        <v>-2.88</v>
       </c>
       <c r="J119" s="9" t="n">
-        <v>2.46</v>
+        <v>3.59</v>
       </c>
       <c r="K119" s="9" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="L119" s="8" t="n">
         <v>100000</v>
@@ -12958,20 +13009,20 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:09</t>
+          <t>08/13/2026 20:23</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
-        <v>99685.03999999999</v>
+        <v>98626.98</v>
       </c>
       <c r="I120" s="9" t="n">
-        <v>-0.31</v>
+        <v>-1.37</v>
       </c>
       <c r="J120" s="9" t="n">
-        <v>1.62</v>
+        <v>2.18</v>
       </c>
       <c r="K120" s="9" t="n">
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
       <c r="L120" s="8" t="n">
         <v>100000</v>
@@ -13043,20 +13094,20 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:07</t>
+          <t>08/13/2026 20:23</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
-        <v>98937.42</v>
+        <v>97089.92</v>
       </c>
       <c r="I121" s="9" t="n">
-        <v>-1.07</v>
+        <v>-2.92</v>
       </c>
       <c r="J121" s="9" t="n">
-        <v>3.26</v>
+        <v>5.44</v>
       </c>
       <c r="K121" s="9" t="n">
-        <v>0.84</v>
+        <v>0.79</v>
       </c>
       <c r="L121" s="8" t="n">
         <v>100000</v>
@@ -13128,20 +13179,20 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:13</t>
+          <t>08/13/2026 20:26</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
-        <v>91072.89</v>
+        <v>88781.78999999999</v>
       </c>
       <c r="I122" s="9" t="n">
-        <v>-8.93</v>
+        <v>-11.22</v>
       </c>
       <c r="J122" s="9" t="n">
-        <v>9.279999999999999</v>
+        <v>11.5</v>
       </c>
       <c r="K122" s="9" t="n">
-        <v>0.45</v>
+        <v>0.64</v>
       </c>
       <c r="L122" s="8" t="n">
         <v>100000</v>
@@ -13213,20 +13264,20 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 09:16</t>
+          <t>08/13/2026 20:27</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
-        <v>98477.35000000001</v>
+        <v>97787.39</v>
       </c>
       <c r="I123" s="9" t="n">
-        <v>-1.52</v>
+        <v>-2.21</v>
       </c>
       <c r="J123" s="9" t="n">
-        <v>1.62</v>
+        <v>2.26</v>
       </c>
       <c r="K123" s="9" t="n">
-        <v>0.61</v>
+        <v>0.7</v>
       </c>
       <c r="L123" s="8" t="n">
         <v>100000</v>
@@ -13235,17 +13286,23 @@
         <v>0</v>
       </c>
       <c r="N123" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O123" s="9" t="n">
-        <v>0</v>
+        <v>-525.47</v>
       </c>
       <c r="P123" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q123" s="8" t="n"/>
-      <c r="R123" s="8" t="n"/>
-      <c r="S123" s="8" t="n"/>
+        <v>25</v>
+      </c>
+      <c r="Q123" s="9" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="R123" s="9" t="n">
+        <v>0.522108843537415</v>
+      </c>
+      <c r="S123" s="9" t="n">
+        <v>0.58</v>
+      </c>
       <c r="T123" s="8" t="n">
         <v>0</v>
       </c>
@@ -13571,7 +13628,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>08/09/2026 23:59</t>
+          <t>08/13/2026 00:16</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13787,7 +13844,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08/10/2026 20:01</t>
+          <t>08/13/2026 20:03</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -13869,7 +13926,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08/10/2026 09:42</t>
+          <t>08/13/2026 09:52</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -13910,7 +13967,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08/10/2026 01:17</t>
+          <t>08/13/2026 01:44</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -13951,7 +14008,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08/09/2026 22:04</t>
+          <t>08/12/2026 22:37</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -13992,7 +14049,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/12/2026 09:34</t>
+          <t>08/13/2026 20:36</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14074,7 +14131,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/10/2026 14:33</t>
+          <t>08/13/2026 14:50</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14115,7 +14172,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/12/2026 10:00</t>
+          <t>08/13/2026 20:53</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14156,7 +14213,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/12/2026 03:41</t>
+          <t>08/13/2026 20:27</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14197,7 +14254,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/12/2026 09:16</t>
+          <t>08/13/2026 20:30</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14238,7 +14295,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/12/2026 09:11</t>
+          <t>08/13/2026 20:25</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14320,14 +14377,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/12/2026 09:06</t>
+          <t>08/13/2026 20:22</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>50072.49</v>
+        <v>49693.02</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.15</v>
+        <v>-0.6</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -14361,14 +14418,14 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/12/2026 09:08</t>
+          <t>08/13/2026 20:24</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>98308.98</v>
+        <v>97124.75</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>-1.69</v>
+        <v>-2.88</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -14402,14 +14459,14 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/12/2026 09:09</t>
+          <t>08/13/2026 20:23</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>99685.03999999999</v>
+        <v>98626.98</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>-0.31</v>
+        <v>-1.37</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -14443,14 +14500,14 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/12/2026 09:07</t>
+          <t>08/13/2026 20:23</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>98937.42</v>
+        <v>97089.92</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>-1.07</v>
+        <v>-2.92</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -14484,14 +14541,14 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/12/2026 09:13</t>
+          <t>08/13/2026 20:26</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>91072.89</v>
+        <v>88781.78999999999</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>-8.93</v>
+        <v>-11.22</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -14525,17 +14582,17 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/12/2026 09:16</t>
+          <t>08/13/2026 20:27</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>98477.35000000001</v>
+        <v>97787.39</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>-1.52</v>
+        <v>-2.21</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25">
@@ -14689,7 +14746,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>08/09/2026 23:59</t>
+          <t>08/13/2026 00:16</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
@@ -15728,7 +15785,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/10/2026 10:11</t>
+          <t>08/13/2026 10:19</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -15820,7 +15877,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08/10/2026 04:51</t>
+          <t>08/13/2026 04:53</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -15866,7 +15923,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08/10/2026 05:32</t>
+          <t>08/13/2026 05:35</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -15889,7 +15946,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/10/2026 12:58</t>
+          <t>08/13/2026 13:00</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -15935,7 +15992,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/10/2026 15:10</t>
+          <t>08/13/2026 15:15</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -16050,7 +16107,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08/09/2026 22:52</t>
+          <t>08/12/2026 23:06</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -16096,7 +16153,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/12/2026 11:50</t>
+          <t>08/13/2026 21:50</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16142,11 +16199,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/12/2026 09:37</t>
+          <t>08/13/2026 20:39</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20270.5</v>
+        <v>20180.43</v>
       </c>
     </row>
     <row r="24">
@@ -16188,11 +16245,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/12/2026 10:26</t>
+          <t>08/13/2026 21:10</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19709.98</v>
+        <v>19696.99</v>
       </c>
     </row>
     <row r="26">
@@ -16211,11 +16268,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/12/2026 09:52</t>
+          <t>08/13/2026 20:48</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21502.35</v>
+        <v>21890.48</v>
       </c>
     </row>
     <row r="27">
@@ -16234,7 +16291,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/12/2026 01:27</t>
+          <t>08/13/2026 19:12</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16257,7 +16314,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/12/2026 07:05</t>
+          <t>08/13/2026 19:13</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16280,7 +16337,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/12/2026 07:12</t>
+          <t>08/13/2026 19:20</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16303,7 +16360,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/12/2026 06:48</t>
+          <t>08/13/2026 18:59</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16326,7 +16383,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/12/2026 07:04</t>
+          <t>08/13/2026 19:13</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16349,7 +16406,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/12/2026 06:54</t>
+          <t>08/13/2026 19:07</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16372,7 +16429,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/12/2026 20:02</t>
+          <t>08/13/2026 15:00</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -16395,7 +16452,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/12/2026 08:55</t>
+          <t>08/13/2026 20:19</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -16418,7 +16475,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>08/12/2026 09:03</t>
+          <t>08/13/2026 20:20</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -16510,7 +16567,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/09/2026 23:53</t>
+          <t>08/13/2026 00:13</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
@@ -16533,7 +16590,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/12/2026 09:38</t>
+          <t>08/13/2026 09:46</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-14
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-13 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-14 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/13/2026 20:00</t>
+          <t>08/14/2026 21:06</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>55619.4</v>
+        <v>57291.6</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>154.23</v>
+        <v>161.87</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>37022.48</v>
+        <v>36615.64</v>
       </c>
       <c r="P2" t="n">
         <v>36</v>
@@ -994,25 +994,25 @@
         <v>90</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>5.875497459696216</v>
+        <v>5.821920622420518</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>8.41</v>
+        <v>8.69</v>
       </c>
       <c r="T2" t="n">
         <v>3331</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>30619.39999999999</v>
+        <v>32291.59999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2102</v>
+        <v>2103</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.10417292104474</v>
+        <v>63.13419393575502</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/13/2026 18:56</t>
+          <t>08/14/2026 20:15</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -2159,20 +2159,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/13/2026 19:51</t>
+          <t>08/14/2026 21:01</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>5192.94</v>
+        <v>5198.67</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>-1.17</v>
+        <v>-1.06</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>8.949999999999999</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="L13" t="n">
         <v>20000</v>
@@ -2184,34 +2184,34 @@
         <v>40</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>-4829.63</v>
+        <v>-4788.8</v>
       </c>
       <c r="P13" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>72.5</v>
+        <v>75</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>0.6934938287901788</v>
+        <v>0.6953612051197231</v>
       </c>
       <c r="S13" s="7" t="n">
-        <v>98.48</v>
+        <v>98.2</v>
       </c>
       <c r="T13" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>126.4399999999999</v>
+        <v>132.1699999999999</v>
       </c>
       <c r="V13" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>67.21311475409836</v>
+        <v>67.74193548387096</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="Y13" s="7" t="n">
         <v>12.26</v>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/13/2026 19:04</t>
+          <t>08/14/2026 20:19</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/11/2026 14:53</t>
+          <t>08/14/2026 14:56</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/13/2026 21:59</t>
+          <t>08/14/2026 20:02</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/13/2026 20:56</t>
+          <t>08/14/2026 18:48</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/13/2026 20:19</t>
+          <t>08/14/2026 21:25</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/13/2026 20:38</t>
+          <t>08/14/2026 21:44</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16557.78</v>
+        <v>16468.45</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-16.89</v>
+        <v>-17.34</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,34 +3492,34 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>325.55</v>
+        <v>104.57</v>
       </c>
       <c r="P25" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>62.5</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>2.572173661080794</v>
+        <v>1.364368096449354</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.43</v>
+        <v>0.87</v>
       </c>
       <c r="T25" t="n">
-        <v>657</v>
+        <v>664</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3442.22</v>
+        <v>-3531.55</v>
       </c>
       <c r="V25" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>39.5738203957382</v>
+        <v>39.45783132530121</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>21.17</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/13/2026 19:33</t>
+          <t>08/14/2026 20:44</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/13/2026 20:30</t>
+          <t>08/14/2026 21:35</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3725,7 +3725,7 @@
         <v>6.66</v>
       </c>
       <c r="T27" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="U27" s="7" t="n">
         <v>481.68</v>
@@ -3734,7 +3734,7 @@
         <v>44</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>45.83333333333333</v>
+        <v>44</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>1.11</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/13/2026 20:29</t>
+          <t>08/14/2026 21:36</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19579.62</v>
+        <v>19610.1</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-2.11</v>
+        <v>-1.96</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,16 +3928,16 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-779.26</v>
+        <v>-747.61</v>
       </c>
       <c r="P29" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>30</v>
+        <v>32.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.1060148909564399</v>
+        <v>0.1408559148681882</v>
       </c>
       <c r="S29" s="7" t="n">
         <v>4.02</v>
@@ -3946,16 +3946,16 @@
         <v>121</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-420.3800000000002</v>
+        <v>-389.9000000000002</v>
       </c>
       <c r="V29" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>46.28099173553719</v>
+        <v>47.10743801652892</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/13/2026 20:41</t>
+          <t>08/14/2026 21:46</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/13/2026 20:19</t>
+          <t>08/14/2026 21:25</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/13/2026 22:04</t>
+          <t>08/14/2026 20:05</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20012.3</v>
+        <v>20055.94</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.06</v>
+        <v>0.28</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>3.42</v>
       </c>
-      <c r="K34" t="n">
-        <v>1</v>
+      <c r="K34" s="7" t="n">
+        <v>1.02</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,7 +4473,7 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-189.39</v>
+        <v>-203.4</v>
       </c>
       <c r="P34" t="n">
         <v>14</v>
@@ -4482,25 +4482,25 @@
         <v>35</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.8318103103769815</v>
+        <v>0.8193685893166378</v>
       </c>
       <c r="S34" s="7" t="n">
         <v>2.87</v>
       </c>
       <c r="T34" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>42.39000000000005</v>
+        <v>12.30000000000005</v>
       </c>
       <c r="V34" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>40.19607843137255</v>
+        <v>40.77669902912621</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>3.43</v>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/13/2026 18:11</t>
+          <t>08/14/2026 19:33</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/13/2026 21:07</t>
+          <t>08/14/2026 18:59</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/11/2026 17:26</t>
+          <t>08/14/2026 17:27</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/13/2026 21:30</t>
+          <t>08/14/2026 19:35</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/13/2026 20:30</t>
+          <t>08/14/2026 21:35</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/13/2026 20:48</t>
+          <t>08/14/2026 18:41</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/13/2026 20:28</t>
+          <t>08/14/2026 21:34</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/13/2026 20:36</t>
+          <t>08/14/2026 18:31</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5681,13 +5681,13 @@
         <v>446</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-373.4599999999999</v>
+        <v>-363.9899999999999</v>
       </c>
       <c r="V45" t="n">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>54.7085201793722</v>
+        <v>55.15695067264574</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0.88</v>
@@ -5747,7 +5747,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/13/2026 20:13</t>
+          <t>08/14/2026 21:20</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/13/2026 20:23</t>
+          <t>08/14/2026 21:29</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5890,16 +5890,16 @@
         <v>60</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-902.8500000000001</v>
+        <v>-853.8900000000002</v>
       </c>
       <c r="V47" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>40</v>
+        <v>41.66666666666667</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.65</v>
+        <v>0.67</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5956,7 +5956,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/13/2026 20:19</t>
+          <t>08/14/2026 21:25</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/13/2026 20:38</t>
+          <t>08/14/2026 21:43</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/13/2026 20:35</t>
+          <t>08/14/2026 21:41</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6256,7 +6256,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/13/2026 20:21</t>
+          <t>08/14/2026 21:28</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/13/2026 20:20</t>
+          <t>08/14/2026 21:28</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6387,7 +6387,7 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="U52" s="7" t="n">
         <v>-479.5500000000002</v>
@@ -6396,7 +6396,7 @@
         <v>11</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>28.94736842105263</v>
+        <v>28.2051282051282</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>0.85</v>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6456,14 +6456,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/13/2026 20:44</t>
+          <t>08/14/2026 18:39</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19740.55</v>
+        <v>19735.7</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.32</v>
+        <v>-1.35</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6487,16 +6487,16 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-259.45</v>
+        <v>-264.3</v>
       </c>
       <c r="V53" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.25</v>
+        <v>36.17886178861789</v>
       </c>
       <c r="X53" s="7" t="n">
         <v>0.71</v>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/13/2026 20:54</t>
+          <t>08/14/2026 18:49</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/13/2026 20:36</t>
+          <t>08/14/2026 21:44</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/13/2026 20:54</t>
+          <t>08/14/2026 18:48</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6856,20 +6856,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/13/2026 20:19</t>
+          <t>08/14/2026 21:26</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19737.71</v>
+        <v>19748.72</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.32</v>
+        <v>-1.27</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6887,16 +6887,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-262.29</v>
+        <v>-255.55</v>
       </c>
       <c r="V57" t="n">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.2838370565046</v>
+        <v>44.12903225806451</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.8</v>
@@ -6911,7 +6911,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/13/2026 20:35</t>
+          <t>08/14/2026 21:41</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/13/2026 20:23</t>
+          <t>08/14/2026 21:30</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7156,7 +7156,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/13/2026 20:29</t>
+          <t>08/14/2026 21:35</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7256,14 +7256,14 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/13/2026 20:51</t>
+          <t>08/14/2026 18:44</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>20922.87</v>
+        <v>20926.01</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-2.33</v>
+        <v>-2.32</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>13.96</v>
@@ -7356,7 +7356,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/13/2026 20:47</t>
+          <t>08/14/2026 18:40</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7456,20 +7456,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/13/2026 20:43</t>
+          <t>08/14/2026 18:37</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18670.29</v>
+        <v>18649.39</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.66</v>
+        <v>-6.76</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>6.74</v>
+        <v>6.76</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7487,22 +7487,22 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1329.71</v>
+        <v>-1350.61</v>
       </c>
       <c r="V63" t="n">
         <v>3</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>8.108108108108109</v>
+        <v>7.894736842105263</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="Y63" s="7" t="n">
-        <v>6.73</v>
+        <v>6.75</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7511,7 +7511,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7556,20 +7556,20 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/13/2026 20:58</t>
+          <t>08/14/2026 18:50</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
-        <v>19395.57</v>
+        <v>19414.44</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>-3.01</v>
+        <v>-2.92</v>
       </c>
       <c r="J64" s="7" t="n">
         <v>3.87</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="L64" t="n">
         <v>20000</v>
@@ -7656,14 +7656,14 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/13/2026 20:40</t>
+          <t>08/14/2026 21:46</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19197.65</v>
+        <v>19276.92</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-4.02</v>
+        <v>-3.62</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>11.64</v>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/13/2026 20:35</t>
+          <t>08/14/2026 21:42</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7856,7 +7856,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/13/2026 21:08</t>
+          <t>08/14/2026 19:00</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/11/2026 13:03</t>
+          <t>08/14/2026 13:05</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/11/2026 13:02</t>
+          <t>08/14/2026 13:05</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8156,7 +8156,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/11/2026 13:14</t>
+          <t>08/14/2026 13:15</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8256,7 +8256,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/13/2026 20:44</t>
+          <t>08/14/2026 15:37</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/13/2026 21:11</t>
+          <t>08/14/2026 19:15</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8456,7 +8456,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/13/2026 20:45</t>
+          <t>08/14/2026 18:40</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8556,20 +8556,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/13/2026 21:03</t>
+          <t>08/14/2026 18:55</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20671.54</v>
+        <v>20681.14</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>3.37</v>
+        <v>3.42</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>1.73</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8587,19 +8587,19 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>671.5400000000001</v>
+        <v>681.1400000000001</v>
       </c>
       <c r="V74" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>67.39130434782609</v>
+        <v>67.74193548387096</v>
       </c>
       <c r="X74" s="7" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
       <c r="Y74" s="7" t="n">
         <v>1.73</v>
@@ -8611,7 +8611,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8656,20 +8656,20 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/13/2026 20:34</t>
+          <t>08/14/2026 21:41</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20036.74</v>
+        <v>20128.61</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>0.22</v>
+        <v>0.68</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K75" s="7" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="L75" t="n">
         <v>20000</v>
@@ -8687,19 +8687,19 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>36.74000000000007</v>
+        <v>128.6100000000001</v>
       </c>
       <c r="V75" t="n">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>54.26356589147287</v>
+        <v>55.22388059701493</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="Y75" s="7" t="n">
         <v>4.5</v>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8756,20 +8756,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/13/2026 20:54</t>
+          <t>08/14/2026 18:47</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>20798.51</v>
-      </c>
-      <c r="I76" t="n">
-        <v>4</v>
+        <v>20598.79</v>
+      </c>
+      <c r="I76" s="7" t="n">
+        <v>3.01</v>
       </c>
       <c r="J76" s="7" t="n">
-        <v>3.36</v>
+        <v>4.28</v>
       </c>
       <c r="K76" s="7" t="n">
-        <v>1.14</v>
+        <v>1.1</v>
       </c>
       <c r="L76" t="n">
         <v>20000</v>
@@ -8787,22 +8787,22 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1104</v>
+        <v>1148</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>832.1400000000003</v>
+        <v>644.3099999999998</v>
       </c>
       <c r="V76" t="n">
-        <v>662</v>
+        <v>684</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>59.96376811594203</v>
+        <v>59.58188153310105</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.15</v>
+        <v>1.11</v>
       </c>
       <c r="Y76" s="7" t="n">
-        <v>3.35</v>
+        <v>4.29</v>
       </c>
       <c r="Z76" t="inlineStr">
         <is>
@@ -8811,7 +8811,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8856,20 +8856,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/13/2026 20:48</t>
+          <t>08/14/2026 18:40</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>20095.35</v>
+        <v>19976.14</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>0.46</v>
+        <v>-0.14</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
       </c>
-      <c r="K77" s="7" t="n">
-        <v>1.01</v>
+      <c r="K77" t="n">
+        <v>1</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8887,19 +8887,19 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>990</v>
+        <v>1028</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>105.8200000000001</v>
+        <v>-23.86000000000013</v>
       </c>
       <c r="V77" t="n">
-        <v>507</v>
+        <v>527</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>51.21212121212121</v>
+        <v>51.26459143968872</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="Y77" s="7" t="n">
         <v>4.48</v>
@@ -8911,7 +8911,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8956,7 +8956,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/13/2026 20:53</t>
+          <t>08/14/2026 18:46</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9056,20 +9056,20 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/13/2026 20:53</t>
+          <t>08/14/2026 18:47</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>20043.76</v>
+        <v>20414.49</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>0.26</v>
+        <v>2.11</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>16.96</v>
       </c>
-      <c r="K79" t="n">
-        <v>1</v>
+      <c r="K79" s="7" t="n">
+        <v>1.02</v>
       </c>
       <c r="L79" t="n">
         <v>20000</v>
@@ -9087,19 +9087,19 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>43.75999999999976</v>
+        <v>414.489999999999</v>
       </c>
       <c r="V79" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>53.99239543726235</v>
+        <v>54.94505494505495</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="Y79" s="7" t="n">
         <v>17</v>
@@ -9111,7 +9111,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9156,20 +9156,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/13/2026 20:36</t>
+          <t>08/14/2026 21:41</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>20373.31</v>
+        <v>19810.93</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>1.9</v>
+        <v>-0.93</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>1.01</v>
+        <v>0.99</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9187,19 +9187,19 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>1904</v>
+        <v>1967</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>392.8400000000004</v>
+        <v>44.48999999999887</v>
       </c>
       <c r="V80" t="n">
-        <v>1181</v>
+        <v>1212</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>62.02731092436975</v>
+        <v>61.61667513980681</v>
       </c>
       <c r="X80" s="7" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="Y80" s="7" t="n">
         <v>17.52</v>
@@ -9211,7 +9211,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9256,20 +9256,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/13/2026 21:03</t>
+          <t>08/14/2026 18:56</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>19704.56</v>
+        <v>19364.77</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-1.45</v>
+        <v>-3.16</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9287,19 +9287,19 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>925</v>
+        <v>965</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>-255.2100000000003</v>
+        <v>-635.230000000001</v>
       </c>
       <c r="V81" t="n">
-        <v>474</v>
+        <v>495</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>51.24324324324324</v>
+        <v>51.29533678756477</v>
       </c>
       <c r="X81" s="7" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
       <c r="Y81" s="7" t="n">
         <v>12.38</v>
@@ -9311,7 +9311,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9356,7 +9356,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/13/2026 20:56</t>
+          <t>08/14/2026 18:49</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9553,20 +9553,20 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/13/2026 21:37</t>
+          <t>08/14/2026 19:38</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
-        <v>20005.28</v>
+        <v>20151.68</v>
       </c>
       <c r="I84" s="7" t="n">
-        <v>0.03</v>
+        <v>0.76</v>
       </c>
       <c r="J84" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="K84" s="7" t="n">
-        <v>1.11</v>
+        <v>4.05</v>
       </c>
       <c r="L84" t="n">
         <v>20000</v>
@@ -9584,19 +9584,19 @@
         <v>0</v>
       </c>
       <c r="T84" t="n">
+        <v>3</v>
+      </c>
+      <c r="U84" s="7" t="n">
+        <v>151.68</v>
+      </c>
+      <c r="V84" t="n">
         <v>2</v>
       </c>
-      <c r="U84" s="7" t="n">
-        <v>5.280000000000001</v>
-      </c>
-      <c r="V84" t="n">
-        <v>1</v>
-      </c>
       <c r="W84" s="7" t="n">
-        <v>50</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X84" s="7" t="n">
-        <v>1.11</v>
+        <v>4.05</v>
       </c>
       <c r="Y84" s="7" t="n">
         <v>0.25</v>
@@ -9608,7 +9608,7 @@
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr">
@@ -9653,7 +9653,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/13/2026 21:00</t>
+          <t>08/14/2026 18:53</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9753,14 +9753,14 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/13/2026 21:11</t>
+          <t>08/14/2026 19:16</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20775.94</v>
+        <v>20780.54</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>3.89</v>
+        <v>3.91</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>2.18</v>
@@ -9784,16 +9784,16 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>775.9399999999999</v>
+        <v>780.54</v>
       </c>
       <c r="V86" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>48.38709677419355</v>
+        <v>49.2063492063492</v>
       </c>
       <c r="X86" s="7" t="n">
         <v>2.13</v>
@@ -9808,7 +9808,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9853,20 +9853,20 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/13/2026 20:54</t>
+          <t>08/14/2026 18:46</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
-        <v>20364.8</v>
+        <v>20490.8</v>
       </c>
       <c r="I87" s="7" t="n">
-        <v>1.83</v>
+        <v>2.46</v>
       </c>
       <c r="J87" s="7" t="n">
         <v>1.07</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>4.52</v>
+        <v>5.71</v>
       </c>
       <c r="L87" t="n">
         <v>20000</v>
@@ -9884,19 +9884,19 @@
         <v>0</v>
       </c>
       <c r="T87" t="n">
+        <v>17</v>
+      </c>
+      <c r="U87" s="7" t="n">
+        <v>490.8</v>
+      </c>
+      <c r="V87" t="n">
         <v>14</v>
       </c>
-      <c r="U87" s="7" t="n">
-        <v>364.8</v>
-      </c>
-      <c r="V87" t="n">
-        <v>10</v>
-      </c>
       <c r="W87" s="7" t="n">
-        <v>71.42857142857143</v>
+        <v>82.35294117647058</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>4.46</v>
+        <v>5.71</v>
       </c>
       <c r="Y87" s="7" t="n">
         <v>0.33</v>
@@ -9908,7 +9908,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -9953,20 +9953,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/13/2026 20:56</t>
+          <t>08/14/2026 18:51</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20392.52</v>
+        <v>20427.32</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>1.96</v>
+        <v>2.13</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>2.9</v>
+        <v>3.06</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -9984,19 +9984,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="U88" s="7" t="n">
-        <v>343.2</v>
+        <v>427.32</v>
       </c>
       <c r="V88" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="W88" s="7" t="n">
-        <v>92.5925925925926</v>
+        <v>93.33333333333333</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>2.66</v>
+        <v>3.06</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -10008,7 +10008,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10053,20 +10053,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/13/2026 20:58</t>
+          <t>08/14/2026 18:51</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>21288.9</v>
+        <v>21496.1</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>6.46</v>
+        <v>7.5</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>1.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>4.06</v>
+        <v>4.56</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10084,19 +10084,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
+        <v>18</v>
+      </c>
+      <c r="U89" s="7" t="n">
+        <v>1496.1</v>
+      </c>
+      <c r="V89" t="n">
         <v>16</v>
       </c>
-      <c r="U89" s="7" t="n">
-        <v>1288.9</v>
-      </c>
-      <c r="V89" t="n">
-        <v>14</v>
-      </c>
       <c r="W89" s="7" t="n">
-        <v>87.5</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>4.06</v>
+        <v>4.56</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>1.99</v>
@@ -10108,7 +10108,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10153,20 +10153,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/13/2026 20:22</t>
+          <t>08/14/2026 21:29</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>20119.27</v>
+        <v>20159.92</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="J90" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>3.38</v>
+        <v>3.98</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10184,19 +10184,19 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>119.27</v>
+        <v>145.88</v>
       </c>
       <c r="V90" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>85.71428571428571</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>3.38</v>
+        <v>3.72</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>0.25</v>
@@ -10208,7 +10208,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10253,20 +10253,20 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/13/2026 20:20</t>
+          <t>08/14/2026 21:26</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
-        <v>20176.99</v>
+        <v>20269.59</v>
       </c>
       <c r="I91" s="7" t="n">
-        <v>0.89</v>
+        <v>1.36</v>
       </c>
       <c r="J91" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="K91" s="7" t="n">
-        <v>2.76</v>
+        <v>3.5</v>
       </c>
       <c r="L91" t="n">
         <v>20000</v>
@@ -10284,19 +10284,19 @@
         <v>0</v>
       </c>
       <c r="T91" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="U91" s="7" t="n">
-        <v>176.99</v>
+        <v>237.26</v>
       </c>
       <c r="V91" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="W91" s="7" t="n">
-        <v>84.61538461538461</v>
+        <v>65.21739130434783</v>
       </c>
       <c r="X91" s="7" t="n">
-        <v>2.76</v>
+        <v>3.2</v>
       </c>
       <c r="Y91" s="7" t="n">
         <v>0.5</v>
@@ -10308,7 +10308,7 @@
       </c>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB91" t="inlineStr">
@@ -10353,20 +10353,20 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/13/2026 20:20</t>
+          <t>08/14/2026 21:25</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
-        <v>20005.68</v>
+        <v>20003.27</v>
       </c>
       <c r="I92" s="7" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="J92" s="7" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="K92" s="7" t="n">
-        <v>3.57</v>
+        <v>1.71</v>
       </c>
       <c r="L92" t="n">
         <v>20000</v>
@@ -10453,20 +10453,20 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/13/2026 20:20</t>
+          <t>08/14/2026 21:27</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
-        <v>20017.75</v>
+        <v>20010.22</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
       <c r="J93" s="7" t="n">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K93" s="7" t="n">
-        <v>3.57</v>
+        <v>1.71</v>
       </c>
       <c r="L93" t="n">
         <v>20000</v>
@@ -10553,20 +10553,20 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/13/2026 20:21</t>
+          <t>08/14/2026 21:26</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
-        <v>20069.14</v>
+        <v>20054.08</v>
       </c>
       <c r="I94" s="7" t="n">
-        <v>0.34</v>
+        <v>0.26</v>
       </c>
       <c r="J94" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="K94" s="7" t="n">
-        <v>6.01</v>
+        <v>2.87</v>
       </c>
       <c r="L94" t="n">
         <v>20000</v>
@@ -10653,20 +10653,20 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/13/2026 20:16</t>
+          <t>08/14/2026 21:24</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
-        <v>99821.64999999999</v>
+        <v>99225.28</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>-0.17</v>
+        <v>-0.76</v>
       </c>
       <c r="J95" s="7" t="n">
-        <v>0.47</v>
+        <v>0.95</v>
       </c>
       <c r="K95" s="7" t="n">
-        <v>0.85</v>
+        <v>0.65</v>
       </c>
       <c r="L95" t="n">
         <v>100000</v>
@@ -10684,22 +10684,22 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>149</v>
+        <v>260</v>
       </c>
       <c r="U95" s="7" t="n">
-        <v>-169.06</v>
+        <v>-631.25</v>
       </c>
       <c r="V95" t="n">
-        <v>78</v>
+        <v>135</v>
       </c>
       <c r="W95" s="7" t="n">
-        <v>52.34899328859061</v>
+        <v>51.92307692307693</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>0.86</v>
+        <v>0.7</v>
       </c>
       <c r="Y95" s="7" t="n">
-        <v>0.47</v>
+        <v>0.84</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -10708,7 +10708,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
@@ -10718,7 +10718,7 @@
       </c>
       <c r="AC95" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | US30, T&amp;D19L13 Meta4 Prop | US500, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | GBPUSD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | US30, T&amp;D19L13 Meta4 Prop | US500, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10753,20 +10753,20 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/13/2026 20:19</t>
+          <t>08/14/2026 21:25</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
-        <v>99976.53</v>
+        <v>98386.59</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>-0.03</v>
+        <v>-1.61</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>1.12</v>
+        <v>2.17</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>0.99</v>
+        <v>0.73</v>
       </c>
       <c r="L96" t="n">
         <v>100000</v>
@@ -10784,22 +10784,22 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>165</v>
+        <v>289</v>
       </c>
       <c r="U96" s="7" t="n">
-        <v>-1.340000000000032</v>
+        <v>-1214.24</v>
       </c>
       <c r="V96" t="n">
-        <v>88</v>
+        <v>153</v>
       </c>
       <c r="W96" s="7" t="n">
-        <v>53.33333333333334</v>
+        <v>52.94117647058824</v>
       </c>
       <c r="X96" s="7" t="n">
-        <v>1</v>
+        <v>0.78</v>
       </c>
       <c r="Y96" s="7" t="n">
-        <v>1.11</v>
+        <v>1.88</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -10808,7 +10808,7 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr">
@@ -10818,7 +10818,7 @@
       </c>
       <c r="AC96" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | US30, T&amp;D19L13 Meta4 MOL | US500, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | GBPUSD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | US30, T&amp;D19L13 Meta4 MOL | US500, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10853,20 +10853,20 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/13/2026 20:22</t>
+          <t>08/14/2026 21:30</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
-        <v>100196.16</v>
+        <v>98228.64999999999</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>0.2</v>
+        <v>-1.77</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>1.81</v>
+        <v>2.81</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>1.04</v>
+        <v>0.79</v>
       </c>
       <c r="L97" t="n">
         <v>100000</v>
@@ -10884,22 +10884,22 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>165</v>
+        <v>289</v>
       </c>
       <c r="U97" s="7" t="n">
-        <v>247.3000000000002</v>
+        <v>-1142.24</v>
       </c>
       <c r="V97" t="n">
-        <v>88</v>
+        <v>153</v>
       </c>
       <c r="W97" s="7" t="n">
-        <v>53.33333333333334</v>
+        <v>52.94117647058824</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>1.06</v>
+        <v>0.85</v>
       </c>
       <c r="Y97" s="7" t="n">
-        <v>1.81</v>
+        <v>2.37</v>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
@@ -10908,7 +10908,7 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB97" t="inlineStr">
@@ -10918,7 +10918,7 @@
       </c>
       <c r="AC97" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | US30, T&amp;D19L13 Meta4 Agg | US500, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | GBPUSD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | US30, T&amp;D19L13 Meta4 Agg | US500, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10953,20 +10953,20 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/13/2026 20:16</t>
+          <t>08/14/2026 21:23</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
-        <v>99857.37</v>
+        <v>99511.98</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>-0.15</v>
+        <v>-0.5</v>
       </c>
       <c r="J98" s="7" t="n">
-        <v>0.49</v>
+        <v>0.67</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>0.83</v>
+        <v>0.66</v>
       </c>
       <c r="L98" t="n">
         <v>100000</v>
@@ -10984,22 +10984,22 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>56</v>
+        <v>97</v>
       </c>
       <c r="U98" s="7" t="n">
-        <v>-124.0499999999999</v>
+        <v>-467.6999999999999</v>
       </c>
       <c r="V98" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="W98" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>45.36082474226804</v>
       </c>
       <c r="X98" s="7" t="n">
-        <v>0.85</v>
+        <v>0.67</v>
       </c>
       <c r="Y98" s="7" t="n">
-        <v>0.49</v>
+        <v>0.67</v>
       </c>
       <c r="Z98" t="inlineStr">
         <is>
@@ -11008,7 +11008,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
@@ -11053,20 +11053,20 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/13/2026 20:21</t>
+          <t>08/14/2026 21:28</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
-        <v>99489.06</v>
+        <v>98886.05</v>
       </c>
       <c r="I99" s="7" t="n">
-        <v>-0.52</v>
+        <v>-1.12</v>
       </c>
       <c r="J99" s="7" t="n">
-        <v>0.67</v>
+        <v>1.12</v>
       </c>
       <c r="K99" s="7" t="n">
-        <v>0.72</v>
+        <v>0.61</v>
       </c>
       <c r="L99" t="n">
         <v>100000</v>
@@ -11084,22 +11084,22 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>134</v>
+        <v>197</v>
       </c>
       <c r="U99" s="7" t="n">
-        <v>-508.8100000000001</v>
+        <v>-948.48</v>
       </c>
       <c r="V99" t="n">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="W99" s="7" t="n">
-        <v>51.49253731343284</v>
+        <v>49.74619289340102</v>
       </c>
       <c r="X99" s="7" t="n">
-        <v>0.72</v>
+        <v>0.65</v>
       </c>
       <c r="Y99" s="7" t="n">
-        <v>0.67</v>
+        <v>0.95</v>
       </c>
       <c r="Z99" t="inlineStr">
         <is>
@@ -11108,7 +11108,7 @@
       </c>
       <c r="AA99" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB99" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="AC99" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L9 Prop | AUDJPY.pro, T&amp;D19L13 L9 Prop | AUDNZD.pro, T&amp;D19L13 L9 Prop | AUDUSD.pro, T&amp;D19L13 L9 Prop | CHFJPY.pro, T&amp;D19L13 L9 Prop | EURCHF.pro, T&amp;D19L13 L9 Prop | EURJPY.pro, T&amp;D19L13 L9 Prop | EURUSD.pro, T&amp;D19L13 L9 Prop | GBPCHF.pro, T&amp;D19L13 L9 Prop | GBPJPY.pro, T&amp;D19L13 L9 Prop | GBPNZD.pro, T&amp;D19L13 L9 Prop | NZDUSD.pro, T&amp;D19L13 L9 Prop | US30, T&amp;D19L13 L9 Prop | US500, T&amp;D19L13 L9 Prop | USDCAD.pro, T&amp;D19L13 L9 Prop | USDCHF.pro, T&amp;D19L13 L9 Prop | USTECH, T&amp;D19L13 L9 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 L9 Prop | AUDJPY.pro, T&amp;D19L13 L9 Prop | AUDNZD.pro, T&amp;D19L13 L9 Prop | AUDUSD.pro, T&amp;D19L13 L9 Prop | CHFJPY.pro, T&amp;D19L13 L9 Prop | EURCHF.pro, T&amp;D19L13 L9 Prop | EURJPY.pro, T&amp;D19L13 L9 Prop | EURUSD.pro, T&amp;D19L13 L9 Prop | GBPCHF.pro, T&amp;D19L13 L9 Prop | GBPJPY.pro, T&amp;D19L13 L9 Prop | GBPNZD.pro, T&amp;D19L13 L9 Prop | GBPUSD.pro, T&amp;D19L13 L9 Prop | NZDUSD.pro, T&amp;D19L13 L9 Prop | US30, T&amp;D19L13 L9 Prop | US500, T&amp;D19L13 L9 Prop | USDCAD.pro, T&amp;D19L13 L9 Prop | USDCHF.pro, T&amp;D19L13 L9 Prop | USTECH, T&amp;D19L13 L9 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11153,7 +11153,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/13/2026 20:52</t>
+          <t>08/14/2026 18:45</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11262,7 +11262,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>08/11/2026 03:34</t>
+          <t>08/14/2026 03:35</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11480,20 +11480,20 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/13/2026 19:45</t>
+          <t>08/14/2026 20:56</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>26875.34</v>
+        <v>27037.49</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-30.01</v>
+        <v>-29.59</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
       </c>
       <c r="K103" s="7" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="L103" t="n">
         <v>25000</v>
@@ -11505,7 +11505,7 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>16.5</v>
+        <v>133.56</v>
       </c>
       <c r="P103" t="n">
         <v>30</v>
@@ -11514,25 +11514,25 @@
         <v>75</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>1.049211130663008</v>
+        <v>1.398341734021295</v>
       </c>
       <c r="S103" s="7" t="n">
         <v>0.96</v>
       </c>
       <c r="T103" t="n">
-        <v>3433</v>
+        <v>3448</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-7406.660000000001</v>
+        <v>-7244.51</v>
       </c>
       <c r="V103" t="n">
-        <v>2065</v>
+        <v>2073</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>60.15147101660355</v>
+        <v>60.12180974477958</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="Y103" s="7" t="n">
         <v>37.71</v>
@@ -11544,7 +11544,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -12135,7 +12135,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:36</t>
+          <t>08/14/2026 21:42</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12408,7 +12408,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:53</t>
+          <t>08/14/2026 18:46</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12499,7 +12499,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:27</t>
+          <t>08/14/2026 21:32</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12521,17 +12521,23 @@
         <v>0</v>
       </c>
       <c r="N114" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O114" s="9" t="n">
-        <v>0</v>
+        <v>-27.2</v>
       </c>
       <c r="P114" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q114" s="8" t="n"/>
-      <c r="R114" s="8" t="n"/>
-      <c r="S114" s="8" t="n"/>
+        <v>24</v>
+      </c>
+      <c r="Q114" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="R114" s="9" t="n">
+        <v>0.9300015440835864</v>
+      </c>
+      <c r="S114" s="9" t="n">
+        <v>0.72</v>
+      </c>
       <c r="T114" s="8" t="n">
         <v>0</v>
       </c>
@@ -12584,7 +12590,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:30</t>
+          <t>08/14/2026 18:25</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12669,7 +12675,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:25</t>
+          <t>08/14/2026 21:31</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12754,7 +12760,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>08/11/2026 13:06</t>
+          <t>08/14/2026 13:08</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12839,20 +12845,20 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:22</t>
+          <t>08/14/2026 21:28</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
-        <v>49693.02</v>
+        <v>49357.3</v>
       </c>
       <c r="I118" s="9" t="n">
-        <v>-0.6</v>
-      </c>
-      <c r="J118" s="9" t="n">
-        <v>1.79</v>
+        <v>-1.27</v>
+      </c>
+      <c r="J118" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="K118" s="9" t="n">
-        <v>0.88</v>
+        <v>0.79</v>
       </c>
       <c r="L118" s="8" t="n">
         <v>50000</v>
@@ -12924,20 +12930,20 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:24</t>
+          <t>08/14/2026 21:30</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
-        <v>97124.75</v>
+        <v>94848.16</v>
       </c>
       <c r="I119" s="9" t="n">
-        <v>-2.88</v>
+        <v>-5.16</v>
       </c>
       <c r="J119" s="9" t="n">
-        <v>3.59</v>
+        <v>5.74</v>
       </c>
       <c r="K119" s="9" t="n">
-        <v>0.74</v>
+        <v>0.65</v>
       </c>
       <c r="L119" s="8" t="n">
         <v>100000</v>
@@ -13009,20 +13015,20 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:23</t>
+          <t>08/14/2026 21:28</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
-        <v>98626.98</v>
+        <v>97685.21000000001</v>
       </c>
       <c r="I120" s="9" t="n">
-        <v>-1.37</v>
+        <v>-2.31</v>
       </c>
       <c r="J120" s="9" t="n">
-        <v>2.18</v>
+        <v>2.65</v>
       </c>
       <c r="K120" s="9" t="n">
-        <v>0.79</v>
+        <v>0.72</v>
       </c>
       <c r="L120" s="8" t="n">
         <v>100000</v>
@@ -13094,20 +13100,20 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:23</t>
+          <t>08/14/2026 21:30</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
-        <v>97089.92</v>
+        <v>93342.05</v>
       </c>
       <c r="I121" s="9" t="n">
-        <v>-2.92</v>
+        <v>-6.66</v>
       </c>
       <c r="J121" s="9" t="n">
-        <v>5.44</v>
+        <v>8.26</v>
       </c>
       <c r="K121" s="9" t="n">
-        <v>0.79</v>
+        <v>0.65</v>
       </c>
       <c r="L121" s="8" t="n">
         <v>100000</v>
@@ -13179,20 +13185,20 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:26</t>
+          <t>08/14/2026 21:33</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
-        <v>88781.78999999999</v>
+        <v>79769.78</v>
       </c>
       <c r="I122" s="9" t="n">
-        <v>-11.22</v>
+        <v>-20.23</v>
       </c>
       <c r="J122" s="9" t="n">
-        <v>11.5</v>
+        <v>20.23</v>
       </c>
       <c r="K122" s="9" t="n">
-        <v>0.64</v>
+        <v>0.55</v>
       </c>
       <c r="L122" s="8" t="n">
         <v>100000</v>
@@ -13264,20 +13270,20 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:27</t>
+          <t>08/14/2026 21:32</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
-        <v>97787.39</v>
+        <v>96074.11</v>
       </c>
       <c r="I123" s="9" t="n">
-        <v>-2.21</v>
+        <v>-3.92</v>
       </c>
       <c r="J123" s="9" t="n">
-        <v>2.26</v>
+        <v>3.92</v>
       </c>
       <c r="K123" s="9" t="n">
-        <v>0.7</v>
+        <v>0.61</v>
       </c>
       <c r="L123" s="8" t="n">
         <v>100000</v>
@@ -13286,23 +13292,17 @@
         <v>0</v>
       </c>
       <c r="N123" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O123" s="9" t="n">
-        <v>-525.47</v>
+        <v>0</v>
       </c>
       <c r="P123" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="Q123" s="9" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="R123" s="9" t="n">
-        <v>0.522108843537415</v>
-      </c>
-      <c r="S123" s="9" t="n">
-        <v>0.58</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q123" s="8" t="n"/>
+      <c r="R123" s="8" t="n"/>
+      <c r="S123" s="8" t="n"/>
       <c r="T123" s="8" t="n">
         <v>0</v>
       </c>
@@ -14049,7 +14049,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/13/2026 20:36</t>
+          <t>08/14/2026 21:42</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/13/2026 20:53</t>
+          <t>08/14/2026 18:46</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14213,7 +14213,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/13/2026 20:27</t>
+          <t>08/14/2026 21:32</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14223,7 +14223,7 @@
         <v>2.91</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
@@ -14254,7 +14254,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/13/2026 20:30</t>
+          <t>08/14/2026 18:25</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14295,7 +14295,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/13/2026 20:25</t>
+          <t>08/14/2026 21:31</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14336,7 +14336,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/11/2026 13:06</t>
+          <t>08/14/2026 13:08</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14377,14 +14377,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/13/2026 20:22</t>
+          <t>08/14/2026 21:28</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>49693.02</v>
+        <v>49357.3</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>-0.6</v>
+        <v>-1.27</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -14418,14 +14418,14 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/13/2026 20:24</t>
+          <t>08/14/2026 21:30</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>97124.75</v>
+        <v>94848.16</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>-2.88</v>
+        <v>-5.16</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -14459,14 +14459,14 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/13/2026 20:23</t>
+          <t>08/14/2026 21:28</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>98626.98</v>
+        <v>97685.21000000001</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>-1.37</v>
+        <v>-2.31</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -14500,14 +14500,14 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/13/2026 20:23</t>
+          <t>08/14/2026 21:30</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>97089.92</v>
+        <v>93342.05</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>-2.92</v>
+        <v>-6.66</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
@@ -14541,14 +14541,14 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/13/2026 20:26</t>
+          <t>08/14/2026 21:33</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>88781.78999999999</v>
+        <v>79769.78</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>-11.22</v>
+        <v>-20.23</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -14582,17 +14582,17 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/13/2026 20:27</t>
+          <t>08/14/2026 21:32</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>97787.39</v>
+        <v>96074.11</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>-2.21</v>
+        <v>-3.92</v>
       </c>
       <c r="I24" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -15854,7 +15854,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/08/2026 06:34</t>
+          <t>08/14/2026 06:51</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -16061,7 +16061,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/08/2026 06:39</t>
+          <t>08/14/2026 07:22</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -16084,7 +16084,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/08/2026 06:30</t>
+          <t>08/14/2026 06:54</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -16153,11 +16153,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/13/2026 21:50</t>
+          <t>08/14/2026 19:52</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>20005.61</v>
+        <v>19985.7</v>
       </c>
     </row>
     <row r="22">
@@ -16199,11 +16199,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/13/2026 20:39</t>
+          <t>08/14/2026 21:43</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20180.43</v>
+        <v>20179.79</v>
       </c>
     </row>
     <row r="24">
@@ -16245,11 +16245,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/13/2026 21:10</t>
+          <t>08/14/2026 19:02</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19696.99</v>
+        <v>19694.69</v>
       </c>
     </row>
     <row r="26">
@@ -16268,11 +16268,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/13/2026 20:48</t>
+          <t>08/14/2026 18:41</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21890.48</v>
+        <v>21623.86</v>
       </c>
     </row>
     <row r="27">
@@ -16291,7 +16291,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/13/2026 19:12</t>
+          <t>08/14/2026 20:26</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16314,7 +16314,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/13/2026 19:13</t>
+          <t>08/14/2026 20:27</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16337,7 +16337,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/13/2026 19:20</t>
+          <t>08/14/2026 20:32</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16360,7 +16360,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/13/2026 18:59</t>
+          <t>08/14/2026 20:16</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16383,7 +16383,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/13/2026 19:13</t>
+          <t>08/14/2026 20:26</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16406,7 +16406,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/13/2026 19:07</t>
+          <t>08/14/2026 20:22</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16452,7 +16452,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/13/2026 20:19</t>
+          <t>08/14/2026 21:25</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -16475,7 +16475,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>08/13/2026 20:20</t>
+          <t>08/14/2026 21:27</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -16590,7 +16590,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/13/2026 09:46</t>
+          <t>08/14/2026 09:48</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-17
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-14 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-17 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/14/2026 21:06</t>
+          <t>08/17/2026 20:11</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>57291.6</v>
+        <v>58137.43</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>161.87</v>
+        <v>165.74</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>36615.64</v>
+        <v>35399.86</v>
       </c>
       <c r="P2" t="n">
         <v>36</v>
@@ -994,22 +994,22 @@
         <v>90</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>5.821920622420518</v>
+        <v>5.661814322098405</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>8.69</v>
+        <v>8.99</v>
       </c>
       <c r="T2" t="n">
-        <v>3331</v>
+        <v>3334</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>32291.59999999999</v>
+        <v>33137.42999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2103</v>
+        <v>2105</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.13419393575502</v>
+        <v>63.1373725254949</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.08</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>08/12/2026 17:24</t>
+          <t>08/15/2026 17:24</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/13/2026 19:21</t>
+          <t>08/16/2026 19:23</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/14/2026 20:15</t>
+          <t>08/17/2026 19:23</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08/13/2026 09:40</t>
+          <t>08/16/2026 09:42</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/13/2026 15:03</t>
+          <t>08/16/2026 14:57</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08/12/2026 22:38</t>
+          <t>08/15/2026 22:40</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>08/12/2026 23:53</t>
+          <t>08/15/2026 23:55</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>08/12/2026 23:53</t>
+          <t>08/15/2026 23:55</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/14/2026 21:01</t>
+          <t>08/17/2026 19:57</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>08/12/2026 18:22</t>
+          <t>08/15/2026 18:24</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/13/2026 05:44</t>
+          <t>08/15/2026 10:05</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/14/2026 20:19</t>
+          <t>08/17/2026 16:04</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/14/2026 14:56</t>
+          <t>08/17/2026 14:59</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>08/12/2026 12:22</t>
+          <t>08/15/2026 12:36</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>08/12/2026 05:41</t>
+          <t>08/15/2026 05:43</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>08/12/2026 05:39</t>
+          <t>08/15/2026 05:41</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/14/2026 20:02</t>
+          <t>08/17/2026 19:03</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/14/2026 18:48</t>
+          <t>08/17/2026 21:02</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/14/2026 21:25</t>
+          <t>08/17/2026 20:30</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>08/12/2026 18:11</t>
+          <t>08/15/2026 18:13</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/14/2026 21:44</t>
+          <t>08/17/2026 20:46</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16468.45</v>
+        <v>16431.85</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-17.34</v>
+        <v>-17.53</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,31 +3492,31 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>104.57</v>
+        <v>22.94999999999998</v>
       </c>
       <c r="P25" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>50</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.364368096449354</v>
+        <v>1.067979857819905</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.87</v>
+        <v>1.06</v>
       </c>
       <c r="T25" t="n">
-        <v>664</v>
+        <v>673</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3531.55</v>
+        <v>-3568.15</v>
       </c>
       <c r="V25" t="n">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>39.45783132530121</v>
+        <v>39.52451708766716</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>0.66</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/14/2026 20:44</t>
+          <t>08/17/2026 19:44</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/14/2026 21:35</t>
+          <t>08/17/2026 20:40</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20481.68</v>
+        <v>20431.27</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-2.06</v>
+        <v>-2.3</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>7.39</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,7 +3710,7 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-640.9599999999999</v>
+        <v>-212.98</v>
       </c>
       <c r="P27" t="n">
         <v>20</v>
@@ -3719,25 +3719,25 @@
         <v>50</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.6769273419188991</v>
+        <v>0.8680298664683831</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>6.66</v>
+        <v>4.21</v>
       </c>
       <c r="T27" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>481.68</v>
+        <v>431.27</v>
       </c>
       <c r="V27" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>44</v>
+        <v>45.54455445544555</v>
       </c>
       <c r="X27" s="7" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="Y27" s="7" t="n">
         <v>7.39</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>08/12/2026 21:51</t>
+          <t>08/15/2026 21:53</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/14/2026 21:36</t>
+          <t>08/17/2026 20:40</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19610.1</v>
+        <v>19646.46</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-1.96</v>
+        <v>-1.78</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,7 +3928,7 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-747.61</v>
+        <v>-674.53</v>
       </c>
       <c r="P29" t="n">
         <v>13</v>
@@ -3937,25 +3937,25 @@
         <v>32.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.1408559148681882</v>
+        <v>0.2003106142337194</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>4.02</v>
+        <v>3.79</v>
       </c>
       <c r="T29" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-389.9000000000002</v>
+        <v>-353.5400000000002</v>
       </c>
       <c r="V29" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>47.10743801652892</v>
+        <v>47.54098360655738</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08/13/2026 10:15</t>
+          <t>08/16/2026 10:18</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/14/2026 21:46</t>
+          <t>08/17/2026 20:46</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/14/2026 21:25</t>
+          <t>08/17/2026 20:32</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>08/12/2026 11:00</t>
+          <t>08/15/2026 11:02</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/14/2026 20:05</t>
+          <t>08/17/2026 19:13</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4491,16 +4491,16 @@
         <v>103</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>12.30000000000005</v>
+        <v>55.94000000000005</v>
       </c>
       <c r="V34" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>40.77669902912621</v>
+        <v>41.74757281553398</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>3.43</v>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/12/2026 00:11</t>
+          <t>08/15/2026 00:13</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/14/2026 19:33</t>
+          <t>08/17/2026 21:30</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/14/2026 18:59</t>
+          <t>08/17/2026 21:08</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/14/2026 17:27</t>
+          <t>08/17/2026 17:30</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/14/2026 19:35</t>
+          <t>08/17/2026 21:26</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>08/13/2026 09:24</t>
+          <t>08/16/2026 09:26</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>08/13/2026 07:24</t>
+          <t>08/16/2026 07:27</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/14/2026 21:35</t>
+          <t>08/17/2026 20:41</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/14/2026 18:41</t>
+          <t>08/17/2026 21:02</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,22 +5442,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>-50.87</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>0.2037877602128658</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
         <v>4278</v>
@@ -5529,7 +5520,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/14/2026 21:34</t>
+          <t>08/17/2026 20:41</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5551,22 +5542,13 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-1124.46</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>0.4043290318479436</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>5.73</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5638,14 +5620,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/14/2026 18:31</t>
+          <t>08/17/2026 20:46</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19636.01</v>
+        <v>19632.66</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-1.8</v>
+        <v>-1.82</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>4.38</v>
@@ -5660,34 +5642,25 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-370.61</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.1500550408219429</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>2.01</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-363.9899999999999</v>
+        <v>-367.34</v>
       </c>
       <c r="V45" t="n">
         <v>246</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>55.15695067264574</v>
+        <v>54.91071428571429</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0.88</v>
@@ -5702,7 +5675,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5747,7 +5720,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/14/2026 21:20</t>
+          <t>08/17/2026 20:30</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5769,22 +5742,13 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>19979.66</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q46" s="7" t="n">
-        <v>29.41176470588236</v>
-      </c>
-      <c r="R46" s="7" t="n">
-        <v>326.7199217476361</v>
-      </c>
-      <c r="S46" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="T46" t="n">
         <v>33</v>
@@ -5816,7 +5780,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5856,7 +5820,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/14/2026 21:29</t>
+          <t>08/17/2026 20:33</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5956,7 +5920,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/14/2026 21:25</t>
+          <t>08/17/2026 20:29</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6056,7 +6020,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/14/2026 21:43</t>
+          <t>08/17/2026 20:48</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6156,7 +6120,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/14/2026 21:41</t>
+          <t>08/17/2026 20:45</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6256,7 +6220,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/14/2026 21:28</t>
+          <t>08/17/2026 20:33</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6356,7 +6320,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/14/2026 21:28</t>
+          <t>08/17/2026 20:33</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6456,20 +6420,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/14/2026 18:39</t>
+          <t>08/17/2026 20:56</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19735.7</v>
+        <v>19717.49</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.35</v>
+        <v>-1.44</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6487,19 +6451,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-264.3</v>
+        <v>-282.51</v>
       </c>
       <c r="V53" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.17886178861789</v>
+        <v>37.15415019762846</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6511,7 +6475,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6556,7 +6520,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/14/2026 18:49</t>
+          <t>08/17/2026 21:03</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6656,7 +6620,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/14/2026 21:44</t>
+          <t>08/17/2026 20:48</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6756,7 +6720,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/14/2026 18:48</t>
+          <t>08/17/2026 20:59</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6856,14 +6820,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/14/2026 21:26</t>
+          <t>08/17/2026 20:30</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19748.72</v>
+        <v>19746.37</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.27</v>
+        <v>-1.28</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6887,16 +6851,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>775</v>
+        <v>780</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-255.55</v>
+        <v>-254.42</v>
       </c>
       <c r="V57" t="n">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.12903225806451</v>
+        <v>44.48717948717948</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.8</v>
@@ -6911,7 +6875,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6956,7 +6920,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/14/2026 21:41</t>
+          <t>08/17/2026 20:44</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7056,7 +7020,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/14/2026 21:30</t>
+          <t>08/17/2026 20:35</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7156,14 +7120,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/14/2026 21:35</t>
+          <t>08/17/2026 20:38</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>20442.76</v>
+        <v>20446.56</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-3.89</v>
+        <v>-3.87</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
@@ -7256,7 +7220,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/14/2026 18:44</t>
+          <t>08/17/2026 20:56</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7356,7 +7320,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/14/2026 18:40</t>
+          <t>08/17/2026 20:54</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7456,20 +7420,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/14/2026 18:37</t>
+          <t>08/17/2026 20:53</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18649.39</v>
+        <v>18583.89</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.76</v>
+        <v>-7.09</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>6.76</v>
+        <v>7.09</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7487,22 +7451,22 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1350.61</v>
+        <v>-1416.11</v>
       </c>
       <c r="V63" t="n">
         <v>3</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>7.894736842105263</v>
+        <v>7.5</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="Y63" s="7" t="n">
-        <v>6.75</v>
+        <v>7.08</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7511,7 +7475,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7556,7 +7520,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/14/2026 18:50</t>
+          <t>08/17/2026 21:00</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7656,7 +7620,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/14/2026 21:46</t>
+          <t>08/17/2026 20:46</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7756,7 +7720,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/14/2026 21:42</t>
+          <t>08/17/2026 20:43</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7856,7 +7820,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/14/2026 19:00</t>
+          <t>08/17/2026 21:09</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7956,7 +7920,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/14/2026 13:05</t>
+          <t>08/17/2026 13:07</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8056,7 +8020,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/14/2026 13:05</t>
+          <t>08/17/2026 13:06</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8156,7 +8120,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/14/2026 13:15</t>
+          <t>08/17/2026 13:16</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8256,7 +8220,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/14/2026 15:37</t>
+          <t>08/17/2026 20:54</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8356,7 +8320,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/14/2026 19:15</t>
+          <t>08/17/2026 21:15</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8456,7 +8420,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/14/2026 18:40</t>
+          <t>08/17/2026 20:54</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8556,7 +8520,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/14/2026 18:55</t>
+          <t>08/17/2026 21:13</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8656,14 +8620,14 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/14/2026 21:41</t>
+          <t>08/17/2026 20:44</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20128.61</v>
+        <v>20118.47</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>0.68</v>
+        <v>0.63</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>4.48</v>
@@ -8687,16 +8651,16 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>128.6100000000001</v>
+        <v>118.4699999999999</v>
       </c>
       <c r="V75" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>55.22388059701493</v>
+        <v>54.94505494505495</v>
       </c>
       <c r="X75" s="7" t="n">
         <v>1.03</v>
@@ -8711,7 +8675,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8756,17 +8720,17 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/14/2026 18:47</t>
+          <t>08/17/2026 21:01</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>20598.79</v>
+        <v>20581.52</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>3.01</v>
+        <v>2.92</v>
       </c>
       <c r="J76" s="7" t="n">
-        <v>4.28</v>
+        <v>4.57</v>
       </c>
       <c r="K76" s="7" t="n">
         <v>1.1</v>
@@ -8787,22 +8751,22 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1148</v>
+        <v>1201</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>644.3099999999998</v>
+        <v>576.8900000000003</v>
       </c>
       <c r="V76" t="n">
-        <v>684</v>
+        <v>710</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>59.58188153310105</v>
+        <v>59.11740216486261</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="Y76" s="7" t="n">
-        <v>4.29</v>
+        <v>4.59</v>
       </c>
       <c r="Z76" t="inlineStr">
         <is>
@@ -8811,7 +8775,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8856,20 +8820,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/14/2026 18:40</t>
+          <t>08/17/2026 20:55</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>19976.14</v>
+        <v>19887.77</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>-0.14</v>
+        <v>-0.58</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
       </c>
-      <c r="K77" t="n">
-        <v>1</v>
+      <c r="K77" s="7" t="n">
+        <v>0.98</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8887,19 +8851,19 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>1028</v>
+        <v>1066</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>-23.86000000000013</v>
+        <v>-121.8199999999999</v>
       </c>
       <c r="V77" t="n">
-        <v>527</v>
+        <v>547</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>51.26459143968872</v>
+        <v>51.31332082551595</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Y77" s="7" t="n">
         <v>4.48</v>
@@ -8911,7 +8875,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8956,20 +8920,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/14/2026 18:46</t>
+          <t>08/17/2026 20:58</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>20269.57</v>
+        <v>20088.4</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>1.35</v>
+        <v>0.45</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>1.1</v>
+        <v>1.03</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -8987,19 +8951,19 @@
         <v>0</v>
       </c>
       <c r="T78" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="U78" s="7" t="n">
-        <v>269.5699999999999</v>
+        <v>88.39999999999993</v>
       </c>
       <c r="V78" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="W78" s="7" t="n">
-        <v>40.27777777777778</v>
+        <v>40.25974025974026</v>
       </c>
       <c r="X78" s="7" t="n">
-        <v>1.1</v>
+        <v>1.03</v>
       </c>
       <c r="Y78" s="7" t="n">
         <v>5.5</v>
@@ -9011,7 +8975,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -9056,14 +9020,14 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/14/2026 18:47</t>
+          <t>08/17/2026 21:01</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>20414.49</v>
+        <v>20374.32</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>2.11</v>
+        <v>1.91</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>16.96</v>
@@ -9087,16 +9051,16 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>414.489999999999</v>
+        <v>374.319999999999</v>
       </c>
       <c r="V79" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>54.94505494505495</v>
+        <v>54.67625899280576</v>
       </c>
       <c r="X79" s="7" t="n">
         <v>1.02</v>
@@ -9111,7 +9075,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9156,14 +9120,14 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/14/2026 21:41</t>
+          <t>08/17/2026 20:46</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>19810.93</v>
+        <v>19843.08</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>-0.93</v>
+        <v>-0.77</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
@@ -9187,16 +9151,16 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>1967</v>
+        <v>2043</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>44.48999999999887</v>
+        <v>-77.51000000000113</v>
       </c>
       <c r="V80" t="n">
-        <v>1212</v>
+        <v>1255</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>61.61667513980681</v>
+        <v>61.42927068037201</v>
       </c>
       <c r="X80" s="7" t="n">
         <v>1</v>
@@ -9211,7 +9175,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9256,20 +9220,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/14/2026 18:56</t>
+          <t>08/17/2026 21:07</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>19364.77</v>
+        <v>19138.79</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-3.16</v>
+        <v>-4.29</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9287,19 +9251,19 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>965</v>
+        <v>1004</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>-635.230000000001</v>
+        <v>-890.0100000000006</v>
       </c>
       <c r="V81" t="n">
-        <v>495</v>
+        <v>515</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>51.29533678756477</v>
+        <v>51.29482071713147</v>
       </c>
       <c r="X81" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="Y81" s="7" t="n">
         <v>12.38</v>
@@ -9311,7 +9275,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9356,20 +9320,20 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/14/2026 18:49</t>
+          <t>08/17/2026 21:04</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>20047.14</v>
+        <v>19879.03</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>0.26</v>
+        <v>-0.57</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>1.02</v>
+        <v>0.96</v>
       </c>
       <c r="L82" t="n">
         <v>20000</v>
@@ -9456,7 +9420,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/13/2026 21:44</t>
+          <t>08/16/2026 21:49</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9553,20 +9517,20 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/14/2026 19:38</t>
+          <t>08/17/2026 21:34</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
-        <v>20151.68</v>
+        <v>20105.63</v>
       </c>
       <c r="I84" s="7" t="n">
-        <v>0.76</v>
+        <v>0.53</v>
       </c>
       <c r="J84" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="K84" s="7" t="n">
-        <v>4.05</v>
+        <v>2.1</v>
       </c>
       <c r="L84" t="n">
         <v>20000</v>
@@ -9584,19 +9548,19 @@
         <v>0</v>
       </c>
       <c r="T84" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U84" s="7" t="n">
-        <v>151.68</v>
+        <v>105.63</v>
       </c>
       <c r="V84" t="n">
         <v>2</v>
       </c>
       <c r="W84" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>50</v>
       </c>
       <c r="X84" s="7" t="n">
-        <v>4.05</v>
+        <v>2.1</v>
       </c>
       <c r="Y84" s="7" t="n">
         <v>0.25</v>
@@ -9608,7 +9572,7 @@
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr">
@@ -9653,7 +9617,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/14/2026 18:53</t>
+          <t>08/17/2026 21:06</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9753,20 +9717,20 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/14/2026 19:16</t>
+          <t>08/17/2026 21:14</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20780.54</v>
+        <v>20899.75</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>3.91</v>
+        <v>4.51</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>2.18</v>
       </c>
       <c r="K86" s="7" t="n">
-        <v>2.13</v>
+        <v>2.28</v>
       </c>
       <c r="L86" t="n">
         <v>20000</v>
@@ -9784,19 +9748,19 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>780.54</v>
+        <v>899.7500000000001</v>
       </c>
       <c r="V86" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>49.2063492063492</v>
+        <v>49.29577464788733</v>
       </c>
       <c r="X86" s="7" t="n">
-        <v>2.13</v>
+        <v>2.28</v>
       </c>
       <c r="Y86" s="7" t="n">
         <v>2.17</v>
@@ -9808,7 +9772,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9853,7 +9817,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/14/2026 18:46</t>
+          <t>08/17/2026 20:58</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9953,20 +9917,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/14/2026 18:51</t>
+          <t>08/17/2026 21:06</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20427.32</v>
+        <v>20476.42</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>2.13</v>
+        <v>2.37</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>3.06</v>
+        <v>3.3</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -9984,19 +9948,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="U88" s="7" t="n">
-        <v>427.32</v>
+        <v>476.42</v>
       </c>
       <c r="V88" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="W88" s="7" t="n">
-        <v>93.33333333333333</v>
+        <v>93.93939393939394</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>3.06</v>
+        <v>3.3</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -10008,7 +9972,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10053,20 +10017,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/14/2026 18:51</t>
+          <t>08/17/2026 21:06</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>21496.1</v>
+        <v>22458.33</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>7.5</v>
+        <v>12.32</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>1.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>4.56</v>
+        <v>6.85</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10084,19 +10048,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>1496.1</v>
+        <v>2458.33</v>
       </c>
       <c r="V89" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>88.88888888888889</v>
+        <v>91.30434782608695</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>4.56</v>
+        <v>6.85</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>1.99</v>
@@ -10108,7 +10072,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10118,7 +10082,7 @@
       </c>
       <c r="AC89" t="inlineStr">
         <is>
-          <t>MOL XAUUSD M15 Pass16 | USTECH, MOL XAUUSD M15 Pass16 | XAUUSD</t>
+          <t>MOL XAUUSD M15 Pass16 | US30, MOL XAUUSD M15 Pass16 | USTECH, MOL XAUUSD M15 Pass16 | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10153,7 +10117,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/14/2026 21:29</t>
+          <t>08/17/2026 20:34</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
@@ -10187,16 +10151,16 @@
         <v>24</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>145.88</v>
+        <v>159.92</v>
       </c>
       <c r="V90" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>87.5</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>3.72</v>
+        <v>3.98</v>
       </c>
       <c r="Y90" s="7" t="n">
         <v>0.25</v>
@@ -10253,7 +10217,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/14/2026 21:26</t>
+          <t>08/17/2026 20:34</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10287,16 +10251,16 @@
         <v>23</v>
       </c>
       <c r="U91" s="7" t="n">
-        <v>237.26</v>
+        <v>269.59</v>
       </c>
       <c r="V91" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="W91" s="7" t="n">
-        <v>65.21739130434783</v>
+        <v>86.95652173913044</v>
       </c>
       <c r="X91" s="7" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="Y91" s="7" t="n">
         <v>0.5</v>
@@ -10353,7 +10317,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/14/2026 21:25</t>
+          <t>08/17/2026 20:32</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10384,22 +10348,22 @@
         <v>0</v>
       </c>
       <c r="T92" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U92" s="7" t="n">
-        <v>5.680000000000001</v>
+        <v>3.27</v>
       </c>
       <c r="V92" t="n">
         <v>2</v>
       </c>
       <c r="W92" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>50</v>
       </c>
       <c r="X92" s="7" t="n">
-        <v>3.57</v>
+        <v>1.71</v>
       </c>
       <c r="Y92" s="7" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="Z92" t="inlineStr">
         <is>
@@ -10408,7 +10372,7 @@
       </c>
       <c r="AA92" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB92" t="inlineStr">
@@ -10453,7 +10417,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/14/2026 21:27</t>
+          <t>08/17/2026 20:37</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10484,22 +10448,22 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U93" s="7" t="n">
-        <v>17.75</v>
+        <v>10.22</v>
       </c>
       <c r="V93" t="n">
         <v>2</v>
       </c>
       <c r="W93" s="7" t="n">
-        <v>66.66666666666666</v>
+        <v>50</v>
       </c>
       <c r="X93" s="7" t="n">
-        <v>3.57</v>
+        <v>1.71</v>
       </c>
       <c r="Y93" s="7" t="n">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z93" t="inlineStr">
         <is>
@@ -10508,7 +10472,7 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB93" t="inlineStr">
@@ -10553,7 +10517,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/14/2026 21:26</t>
+          <t>08/17/2026 20:32</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10584,22 +10548,22 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U94" s="7" t="n">
-        <v>69.14</v>
+        <v>54.08</v>
       </c>
       <c r="V94" t="n">
         <v>3</v>
       </c>
       <c r="W94" s="7" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="X94" s="7" t="n">
-        <v>6.01</v>
+        <v>2.87</v>
       </c>
       <c r="Y94" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="Z94" t="inlineStr">
         <is>
@@ -10608,7 +10572,7 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AB94" t="inlineStr">
@@ -10653,14 +10617,14 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/14/2026 21:24</t>
+          <t>08/17/2026 20:31</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
-        <v>99225.28</v>
+        <v>99220.14999999999</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>-0.76</v>
+        <v>-0.77</v>
       </c>
       <c r="J95" s="7" t="n">
         <v>0.95</v>
@@ -10684,22 +10648,22 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="U95" s="7" t="n">
-        <v>-631.25</v>
+        <v>-779.8499999999999</v>
       </c>
       <c r="V95" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="W95" s="7" t="n">
-        <v>51.92307692307693</v>
+        <v>51.8796992481203</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="Y95" s="7" t="n">
-        <v>0.84</v>
+        <v>0.96</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -10708,7 +10672,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
@@ -10753,20 +10717,20 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/14/2026 21:25</t>
+          <t>08/17/2026 20:32</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
-        <v>98386.59</v>
+        <v>98048.10000000001</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>-1.61</v>
+        <v>-1.95</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>2.17</v>
+        <v>2.52</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>0.73</v>
+        <v>0.7</v>
       </c>
       <c r="L96" t="n">
         <v>100000</v>
@@ -10784,22 +10748,22 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>289</v>
+        <v>321</v>
       </c>
       <c r="U96" s="7" t="n">
-        <v>-1214.24</v>
+        <v>-1951.9</v>
       </c>
       <c r="V96" t="n">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="W96" s="7" t="n">
-        <v>52.94117647058824</v>
+        <v>51.71339563862928</v>
       </c>
       <c r="X96" s="7" t="n">
-        <v>0.78</v>
+        <v>0.7</v>
       </c>
       <c r="Y96" s="7" t="n">
-        <v>1.88</v>
+        <v>2.52</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -10808,7 +10772,7 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr">
@@ -10853,20 +10817,20 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/14/2026 21:30</t>
+          <t>08/17/2026 20:37</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
-        <v>98228.64999999999</v>
+        <v>97781.53</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>-1.77</v>
+        <v>-2.22</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>2.81</v>
+        <v>3.26</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>0.79</v>
+        <v>0.76</v>
       </c>
       <c r="L97" t="n">
         <v>100000</v>
@@ -10884,22 +10848,22 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>289</v>
+        <v>321</v>
       </c>
       <c r="U97" s="7" t="n">
-        <v>-1142.24</v>
+        <v>-2158.92</v>
       </c>
       <c r="V97" t="n">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="W97" s="7" t="n">
-        <v>52.94117647058824</v>
+        <v>51.71339563862928</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>0.85</v>
+        <v>0.76</v>
       </c>
       <c r="Y97" s="7" t="n">
-        <v>2.37</v>
+        <v>3.19</v>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
@@ -10908,7 +10872,7 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB97" t="inlineStr">
@@ -10953,20 +10917,20 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/14/2026 21:23</t>
+          <t>08/17/2026 20:31</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
-        <v>99511.98</v>
+        <v>99585.02</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>-0.5</v>
+        <v>-0.43</v>
       </c>
       <c r="J98" s="7" t="n">
         <v>0.67</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>0.66</v>
+        <v>0.71</v>
       </c>
       <c r="L98" t="n">
         <v>100000</v>
@@ -10984,19 +10948,19 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="U98" s="7" t="n">
-        <v>-467.6999999999999</v>
+        <v>-414.9799999999999</v>
       </c>
       <c r="V98" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="W98" s="7" t="n">
-        <v>45.36082474226804</v>
+        <v>47.16981132075472</v>
       </c>
       <c r="X98" s="7" t="n">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="Y98" s="7" t="n">
         <v>0.67</v>
@@ -11008,7 +10972,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
@@ -11018,7 +10982,7 @@
       </c>
       <c r="AC98" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | GBPJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USDCHF.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11053,7 +11017,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/14/2026 21:28</t>
+          <t>08/17/2026 20:34</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11084,22 +11048,22 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="U99" s="7" t="n">
-        <v>-948.48</v>
+        <v>-1113.95</v>
       </c>
       <c r="V99" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="W99" s="7" t="n">
-        <v>49.74619289340102</v>
+        <v>50.25125628140703</v>
       </c>
       <c r="X99" s="7" t="n">
-        <v>0.65</v>
+        <v>0.61</v>
       </c>
       <c r="Y99" s="7" t="n">
-        <v>0.95</v>
+        <v>1.11</v>
       </c>
       <c r="Z99" t="inlineStr">
         <is>
@@ -11153,7 +11117,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/14/2026 18:45</t>
+          <t>08/17/2026 20:58</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11262,7 +11226,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>08/14/2026 03:35</t>
+          <t>08/17/2026 04:05</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11371,7 +11335,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>08/12/2026 22:38</t>
+          <t>08/15/2026 22:40</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11480,14 +11444,14 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/14/2026 20:56</t>
+          <t>08/17/2026 20:03</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>27037.49</v>
+        <v>27079.51</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-29.59</v>
+        <v>-29.48</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
@@ -11505,7 +11469,7 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>133.56</v>
+        <v>162.25</v>
       </c>
       <c r="P103" t="n">
         <v>30</v>
@@ -11514,22 +11478,22 @@
         <v>75</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>1.398341734021295</v>
+        <v>1.48390945151958</v>
       </c>
       <c r="S103" s="7" t="n">
         <v>0.96</v>
       </c>
       <c r="T103" t="n">
-        <v>3448</v>
+        <v>3468</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-7244.51</v>
+        <v>-7224.77</v>
       </c>
       <c r="V103" t="n">
-        <v>2073</v>
+        <v>2074</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>60.12180974477958</v>
+        <v>59.80392156862745</v>
       </c>
       <c r="X103" s="7" t="n">
         <v>0.78</v>
@@ -11544,7 +11508,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11589,7 +11553,7 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 21:29</t>
+          <t>08/15/2026 21:31</t>
         </is>
       </c>
       <c r="H104" s="9" t="n">
@@ -11771,7 +11735,7 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 14:27</t>
+          <t>08/15/2026 14:30</t>
         </is>
       </c>
       <c r="H106" s="9" t="n">
@@ -11862,7 +11826,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 09:52</t>
+          <t>08/16/2026 09:53</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -11953,7 +11917,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 01:44</t>
+          <t>08/16/2026 01:46</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12044,7 +12008,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 22:37</t>
+          <t>08/15/2026 22:39</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12135,7 +12099,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:42</t>
+          <t>08/17/2026 20:44</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12226,7 +12190,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 18:01</t>
+          <t>08/15/2026 18:02</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12317,7 +12281,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 14:50</t>
+          <t>08/16/2026 14:39</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12408,14 +12372,14 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 18:46</t>
+          <t>08/17/2026 21:01</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
-        <v>19085.51</v>
+        <v>19059.58</v>
       </c>
       <c r="I113" s="9" t="n">
-        <v>-4.57</v>
+        <v>-4.7</v>
       </c>
       <c r="J113" s="9" t="n">
         <v>9.16</v>
@@ -12433,7 +12397,7 @@
         <v>40</v>
       </c>
       <c r="O113" s="9" t="n">
-        <v>871.4499999999999</v>
+        <v>845.0699999999999</v>
       </c>
       <c r="P113" s="8" t="n">
         <v>26</v>
@@ -12442,10 +12406,10 @@
         <v>65</v>
       </c>
       <c r="R113" s="9" t="n">
-        <v>22.28083028083028</v>
+        <v>13.55116589930195</v>
       </c>
       <c r="S113" s="9" t="n">
-        <v>0.19</v>
+        <v>0.31</v>
       </c>
       <c r="T113" s="8" t="n">
         <v>0</v>
@@ -12499,7 +12463,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:32</t>
+          <t>08/17/2026 20:40</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12521,23 +12485,17 @@
         <v>0</v>
       </c>
       <c r="N114" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O114" s="9" t="n">
-        <v>-27.2</v>
+        <v>0</v>
       </c>
       <c r="P114" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q114" s="9" t="n">
-        <v>60</v>
-      </c>
-      <c r="R114" s="9" t="n">
-        <v>0.9300015440835864</v>
-      </c>
-      <c r="S114" s="9" t="n">
-        <v>0.72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q114" s="8" t="n"/>
+      <c r="R114" s="8" t="n"/>
+      <c r="S114" s="8" t="n"/>
       <c r="T114" s="8" t="n">
         <v>0</v>
       </c>
@@ -12590,7 +12548,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 18:25</t>
+          <t>08/17/2026 20:46</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12675,7 +12633,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:31</t>
+          <t>08/15/2026 13:43</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12760,7 +12718,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 13:08</t>
+          <t>08/17/2026 13:10</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12845,7 +12803,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:28</t>
+          <t>08/17/2026 20:40</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12930,7 +12888,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:30</t>
+          <t>08/17/2026 20:39</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13015,7 +12973,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:28</t>
+          <t>08/17/2026 20:35</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13100,7 +13058,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:30</t>
+          <t>08/17/2026 20:40</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13185,7 +13143,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:33</t>
+          <t>08/17/2026 20:43</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13270,7 +13228,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/14/2026 21:32</t>
+          <t>08/17/2026 20:39</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13355,7 +13313,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 19:23</t>
+          <t>08/15/2026 19:26</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13446,7 +13404,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>08/12/2026 19:06</t>
+          <t>08/15/2026 19:07</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13628,7 +13586,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 00:16</t>
+          <t>08/16/2026 00:18</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13803,7 +13761,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>08/12/2026 21:29</t>
+          <t>08/15/2026 21:31</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -13885,7 +13843,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08/12/2026 14:27</t>
+          <t>08/15/2026 14:30</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -13926,7 +13884,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08/13/2026 09:52</t>
+          <t>08/16/2026 09:53</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -13967,7 +13925,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08/13/2026 01:44</t>
+          <t>08/16/2026 01:46</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14008,7 +13966,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08/12/2026 22:37</t>
+          <t>08/15/2026 22:39</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14049,7 +14007,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/14/2026 21:42</t>
+          <t>08/17/2026 20:44</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14090,7 +14048,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>08/12/2026 18:01</t>
+          <t>08/15/2026 18:02</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14131,7 +14089,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/13/2026 14:50</t>
+          <t>08/16/2026 14:39</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14172,14 +14130,14 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/14/2026 18:46</t>
+          <t>08/17/2026 21:01</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>19085.51</v>
+        <v>19059.58</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>-4.57</v>
+        <v>-4.7</v>
       </c>
       <c r="I14" t="n">
         <v>40</v>
@@ -14213,7 +14171,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/14/2026 21:32</t>
+          <t>08/17/2026 20:40</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14223,7 +14181,7 @@
         <v>2.91</v>
       </c>
       <c r="I15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -14254,7 +14212,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/14/2026 18:25</t>
+          <t>08/17/2026 20:46</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14295,7 +14253,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/14/2026 21:31</t>
+          <t>08/15/2026 13:43</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14336,7 +14294,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/14/2026 13:08</t>
+          <t>08/17/2026 13:10</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14377,7 +14335,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/14/2026 21:28</t>
+          <t>08/17/2026 20:40</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14418,7 +14376,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/14/2026 21:30</t>
+          <t>08/17/2026 20:39</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14459,7 +14417,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/14/2026 21:28</t>
+          <t>08/17/2026 20:35</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14500,7 +14458,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/14/2026 21:30</t>
+          <t>08/17/2026 20:40</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14541,7 +14499,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/14/2026 21:33</t>
+          <t>08/17/2026 20:43</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14582,7 +14540,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/14/2026 21:32</t>
+          <t>08/17/2026 20:39</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -14623,7 +14581,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>08/12/2026 19:23</t>
+          <t>08/15/2026 19:26</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -14664,7 +14622,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>08/12/2026 19:06</t>
+          <t>08/15/2026 19:07</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
@@ -14746,7 +14704,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>08/13/2026 00:16</t>
+          <t>08/16/2026 00:18</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
@@ -15762,7 +15720,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08/12/2026 20:48</t>
+          <t>08/15/2026 20:50</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -15785,7 +15743,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/13/2026 10:19</t>
+          <t>08/16/2026 10:22</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -15808,7 +15766,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08/09/2026 20:31</t>
+          <t>08/15/2026 20:38</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -15831,7 +15789,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08/12/2026 16:26</t>
+          <t>08/15/2026 16:28</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -15854,7 +15812,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/14/2026 06:51</t>
+          <t>08/17/2026 07:54</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -15877,7 +15835,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08/13/2026 04:53</t>
+          <t>08/16/2026 04:55</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -15900,7 +15858,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08/12/2026 15:52</t>
+          <t>08/15/2026 15:54</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -15923,7 +15881,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08/13/2026 05:35</t>
+          <t>08/16/2026 05:38</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -15946,7 +15904,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/13/2026 13:00</t>
+          <t>08/16/2026 13:01</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -15969,7 +15927,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08/12/2026 21:50</t>
+          <t>08/15/2026 21:53</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -15992,7 +15950,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/13/2026 15:15</t>
+          <t>08/16/2026 15:13</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -16015,7 +15973,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08/12/2026 20:35</t>
+          <t>08/15/2026 20:35</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -16061,7 +16019,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/14/2026 07:22</t>
+          <t>08/17/2026 09:02</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -16084,7 +16042,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/14/2026 06:54</t>
+          <t>08/17/2026 07:41</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -16107,7 +16065,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08/12/2026 23:06</t>
+          <t>08/15/2026 23:08</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -16153,11 +16111,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/14/2026 19:52</t>
+          <t>08/17/2026 21:40</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>19985.7</v>
+        <v>19946.87</v>
       </c>
     </row>
     <row r="22">
@@ -16176,7 +16134,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08/12/2026 21:56</t>
+          <t>08/15/2026 21:58</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -16199,11 +16157,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/14/2026 21:43</t>
+          <t>08/17/2026 20:45</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20179.79</v>
+        <v>20434.06</v>
       </c>
     </row>
     <row r="24">
@@ -16245,11 +16203,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/14/2026 19:02</t>
+          <t>08/17/2026 21:10</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19694.69</v>
+        <v>19734.69</v>
       </c>
     </row>
     <row r="26">
@@ -16268,11 +16226,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/14/2026 18:41</t>
+          <t>08/17/2026 20:54</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21623.86</v>
+        <v>21621.74</v>
       </c>
     </row>
     <row r="27">
@@ -16291,7 +16249,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/14/2026 20:26</t>
+          <t>08/17/2026 19:31</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16314,7 +16272,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/14/2026 20:27</t>
+          <t>08/17/2026 19:30</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16337,7 +16295,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/14/2026 20:32</t>
+          <t>08/17/2026 19:34</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16360,7 +16318,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/14/2026 20:16</t>
+          <t>08/17/2026 19:23</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16383,7 +16341,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/14/2026 20:26</t>
+          <t>08/17/2026 19:28</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16406,7 +16364,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/14/2026 20:22</t>
+          <t>08/17/2026 19:28</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16429,7 +16387,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/13/2026 15:00</t>
+          <t>08/16/2026 14:53</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -16452,7 +16410,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/14/2026 21:25</t>
+          <t>08/17/2026 20:32</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -16475,7 +16433,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>08/14/2026 21:27</t>
+          <t>08/17/2026 20:34</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -16521,7 +16479,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/12/2026 20:31</t>
+          <t>08/15/2026 20:34</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -16544,7 +16502,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/12/2026 21:13</t>
+          <t>08/15/2026 21:16</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -16567,7 +16525,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/13/2026 00:13</t>
+          <t>08/16/2026 00:15</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
@@ -16590,7 +16548,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/14/2026 09:48</t>
+          <t>08/17/2026 11:33</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-18
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-17 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-18 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/17/2026 20:11</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="n">
-        <v>58137.43</v>
+          <t>08/18/2026 18:21</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>59950</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>165.74</v>
+        <v>174.03</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>35399.86</v>
+        <v>35099.36</v>
       </c>
       <c r="P2" t="n">
         <v>36</v>
@@ -994,22 +994,22 @@
         <v>90</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>5.661814322098405</v>
+        <v>5.622241419725611</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>8.99</v>
+        <v>9.32</v>
       </c>
       <c r="T2" t="n">
         <v>3334</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>33137.42999999999</v>
+        <v>34949.99999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2105</v>
+        <v>2106</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.1373725254949</v>
+        <v>63.16736652669466</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.08</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>08/15/2026 17:24</t>
+          <t>08/18/2026 17:49</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/17/2026 19:23</t>
+          <t>08/18/2026 21:44</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/17/2026 19:57</t>
+          <t>08/18/2026 18:06</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>08/15/2026 18:24</t>
+          <t>08/18/2026 19:00</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/15/2026 10:05</t>
+          <t>08/18/2026 10:06</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/17/2026 16:04</t>
+          <t>08/18/2026 16:40</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>08/15/2026 12:36</t>
+          <t>08/18/2026 12:38</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>08/15/2026 05:43</t>
+          <t>08/18/2026 05:45</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>08/15/2026 05:41</t>
+          <t>08/18/2026 05:43</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/17/2026 19:03</t>
+          <t>08/18/2026 21:25</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/17/2026 21:02</t>
+          <t>08/18/2026 19:48</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/17/2026 20:30</t>
+          <t>08/18/2026 18:48</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>08/15/2026 18:13</t>
+          <t>08/18/2026 18:43</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/17/2026 20:46</t>
+          <t>08/18/2026 19:20</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16431.85</v>
+        <v>16445.5</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-17.53</v>
+        <v>-17.46</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,34 +3492,34 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>22.94999999999998</v>
+        <v>48.76999999999998</v>
       </c>
       <c r="P25" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>50</v>
+        <v>57.49999999999999</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.067979857819905</v>
+        <v>1.146817990246252</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>1.06</v>
+        <v>1.19</v>
       </c>
       <c r="T25" t="n">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3568.15</v>
+        <v>-3554.5</v>
       </c>
       <c r="V25" t="n">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>39.52451708766716</v>
+        <v>39.82300884955752</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>21.17</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/17/2026 19:44</t>
+          <t>08/18/2026 17:37</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,14 +3685,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/17/2026 20:40</t>
+          <t>08/18/2026 19:06</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20431.27</v>
+        <v>20425.62</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-2.3</v>
+        <v>-2.33</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>7.39</v>
@@ -3710,7 +3710,7 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-212.98</v>
+        <v>-127.22</v>
       </c>
       <c r="P27" t="n">
         <v>20</v>
@@ -3719,16 +3719,16 @@
         <v>50</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.8680298664683831</v>
+        <v>0.9167457414157543</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>4.21</v>
+        <v>3.75</v>
       </c>
       <c r="T27" t="n">
         <v>101</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>431.27</v>
+        <v>425.62</v>
       </c>
       <c r="V27" t="n">
         <v>46</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/17/2026 20:40</t>
+          <t>08/18/2026 19:07</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/17/2026 20:46</t>
+          <t>08/18/2026 19:23</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/17/2026 20:32</t>
+          <t>08/18/2026 18:54</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>08/15/2026 11:02</t>
+          <t>08/18/2026 11:04</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/17/2026 19:13</t>
+          <t>08/18/2026 21:34</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20055.94</v>
+        <v>20090.73</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.28</v>
+        <v>0.45</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>3.42</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,34 +4473,34 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-203.4</v>
+        <v>-433.67</v>
       </c>
       <c r="P34" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.8193685893166378</v>
+        <v>0.6417253230230329</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>2.87</v>
+        <v>2.91</v>
       </c>
       <c r="T34" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>55.94000000000005</v>
+        <v>124.93</v>
       </c>
       <c r="V34" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>41.74757281553398</v>
+        <v>41.50943396226415</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>3.43</v>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/15/2026 00:13</t>
+          <t>08/18/2026 00:14</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,14 +4666,14 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/17/2026 21:30</t>
+          <t>08/18/2026 20:48</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19813.9</v>
+        <v>19816.79</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.93</v>
+        <v>-0.91</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
@@ -4697,16 +4697,16 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-186.1000000000001</v>
+        <v>-183.2100000000001</v>
       </c>
       <c r="V36" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>48.78048780487805</v>
+        <v>48.80952380952381</v>
       </c>
       <c r="X36" s="7" t="n">
         <v>0.96</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/17/2026 21:08</t>
+          <t>08/18/2026 20:06</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/17/2026 21:26</t>
+          <t>08/18/2026 20:43</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/17/2026 20:41</t>
+          <t>08/18/2026 19:07</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/17/2026 21:02</t>
+          <t>08/18/2026 19:50</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/17/2026 20:41</t>
+          <t>08/18/2026 19:08</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/17/2026 20:46</t>
+          <t>08/18/2026 19:25</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5720,7 +5720,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/17/2026 20:30</t>
+          <t>08/18/2026 18:52</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5820,20 +5820,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/17/2026 20:33</t>
+          <t>08/18/2026 19:00</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>19146.11</v>
+        <v>19082.59</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-4.25</v>
+        <v>-4.57</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5851,19 +5851,19 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-853.8900000000002</v>
+        <v>-917.4100000000002</v>
       </c>
       <c r="V47" t="n">
         <v>25</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>41.66666666666667</v>
+        <v>40.98360655737705</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5875,7 +5875,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/17/2026 20:29</t>
+          <t>08/18/2026 18:49</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/17/2026 20:48</t>
+          <t>08/18/2026 19:27</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/17/2026 20:45</t>
+          <t>08/18/2026 19:20</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/17/2026 20:33</t>
+          <t>08/18/2026 19:01</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/17/2026 20:33</t>
+          <t>08/18/2026 18:52</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6420,14 +6420,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/17/2026 20:56</t>
+          <t>08/18/2026 19:38</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19717.49</v>
+        <v>19703.78</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.44</v>
+        <v>-1.5</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6451,19 +6451,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-282.51</v>
+        <v>-296.2199999999999</v>
       </c>
       <c r="V53" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>37.15415019762846</v>
+        <v>37.06563706563706</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6520,7 +6520,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/17/2026 21:03</t>
+          <t>08/18/2026 19:52</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/17/2026 20:48</t>
+          <t>08/18/2026 19:27</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6720,7 +6720,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/17/2026 20:59</t>
+          <t>08/18/2026 19:46</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6820,14 +6820,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/17/2026 20:30</t>
+          <t>08/18/2026 18:50</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19746.37</v>
+        <v>19748.58</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.28</v>
+        <v>-1.26</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6851,19 +6851,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>780</v>
+        <v>791</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-254.42</v>
+        <v>-251.42</v>
       </c>
       <c r="V57" t="n">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.48717948717948</v>
+        <v>44.62705436156764</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6875,7 +6875,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/17/2026 20:44</t>
+          <t>08/18/2026 19:18</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7020,7 +7020,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/17/2026 20:35</t>
+          <t>08/18/2026 19:00</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/17/2026 20:38</t>
+          <t>08/18/2026 19:05</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/17/2026 20:56</t>
+          <t>08/18/2026 19:42</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/17/2026 20:54</t>
+          <t>08/18/2026 19:41</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7420,17 +7420,17 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/17/2026 20:53</t>
+          <t>08/18/2026 19:36</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18583.89</v>
+        <v>18557.89</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-7.09</v>
+        <v>-7.22</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>7.09</v>
+        <v>7.22</v>
       </c>
       <c r="K63" s="7" t="n">
         <v>0.29</v>
@@ -7451,22 +7451,22 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1416.11</v>
+        <v>-1442.11</v>
       </c>
       <c r="V63" t="n">
         <v>3</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>7.5</v>
+        <v>7.317073170731707</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>0.29</v>
       </c>
       <c r="Y63" s="7" t="n">
-        <v>7.08</v>
+        <v>7.21</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7475,7 +7475,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/17/2026 21:00</t>
+          <t>08/18/2026 19:46</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/17/2026 20:46</t>
+          <t>08/18/2026 19:22</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/17/2026 20:43</t>
+          <t>08/18/2026 19:17</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/17/2026 21:09</t>
+          <t>08/18/2026 20:09</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/17/2026 20:54</t>
+          <t>08/18/2026 19:30</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8320,7 +8320,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/17/2026 21:15</t>
+          <t>08/18/2026 20:19</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/17/2026 20:54</t>
+          <t>08/18/2026 19:37</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8520,7 +8520,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/17/2026 21:13</t>
+          <t>08/18/2026 20:09</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8620,11 +8620,11 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/17/2026 20:44</t>
+          <t>08/18/2026 19:21</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20118.47</v>
+        <v>20119.91</v>
       </c>
       <c r="I75" s="7" t="n">
         <v>0.63</v>
@@ -8651,16 +8651,16 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>118.4699999999999</v>
+        <v>133.2299999999999</v>
       </c>
       <c r="V75" t="n">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>54.94505494505495</v>
+        <v>54.64285714285714</v>
       </c>
       <c r="X75" s="7" t="n">
         <v>1.03</v>
@@ -8675,7 +8675,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8720,20 +8720,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/17/2026 21:01</t>
+          <t>08/18/2026 19:53</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>20581.52</v>
+        <v>20334.68</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>2.92</v>
+        <v>1.7</v>
       </c>
       <c r="J76" s="7" t="n">
-        <v>4.57</v>
+        <v>5.53</v>
       </c>
       <c r="K76" s="7" t="n">
-        <v>1.1</v>
+        <v>1.05</v>
       </c>
       <c r="L76" t="n">
         <v>20000</v>
@@ -8751,22 +8751,22 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1201</v>
+        <v>1225</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>576.8900000000003</v>
+        <v>334.6800000000003</v>
       </c>
       <c r="V76" t="n">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>59.11740216486261</v>
+        <v>58.61224489795919</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.09</v>
+        <v>1.05</v>
       </c>
       <c r="Y76" s="7" t="n">
-        <v>4.59</v>
+        <v>5.56</v>
       </c>
       <c r="Z76" t="inlineStr">
         <is>
@@ -8775,7 +8775,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8820,20 +8820,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/17/2026 20:55</t>
+          <t>08/18/2026 19:42</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>19887.77</v>
+        <v>19790.91</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>-0.58</v>
+        <v>-1.06</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="K77" s="7" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8851,19 +8851,19 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>1066</v>
+        <v>1097</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>-121.8199999999999</v>
+        <v>-209.0900000000002</v>
       </c>
       <c r="V77" t="n">
-        <v>547</v>
+        <v>558</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>51.31332082551595</v>
+        <v>50.86599817684594</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="Y77" s="7" t="n">
         <v>4.48</v>
@@ -8875,7 +8875,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8920,20 +8920,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/17/2026 20:58</t>
+          <t>08/18/2026 19:46</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>20088.4</v>
+        <v>19906.67</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>0.45</v>
+        <v>-0.46</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>1.03</v>
+        <v>0.97</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -8951,19 +8951,19 @@
         <v>0</v>
       </c>
       <c r="T78" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="U78" s="7" t="n">
-        <v>88.39999999999993</v>
+        <v>-93.3300000000002</v>
       </c>
       <c r="V78" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W78" s="7" t="n">
-        <v>40.25974025974026</v>
+        <v>39.50617283950617</v>
       </c>
       <c r="X78" s="7" t="n">
-        <v>1.03</v>
+        <v>0.97</v>
       </c>
       <c r="Y78" s="7" t="n">
         <v>5.5</v>
@@ -8975,7 +8975,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -9020,11 +9020,11 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/17/2026 21:01</t>
+          <t>08/18/2026 19:51</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>20374.32</v>
+        <v>20374.38</v>
       </c>
       <c r="I79" s="7" t="n">
         <v>1.91</v>
@@ -9051,16 +9051,16 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>374.319999999999</v>
+        <v>374.3799999999994</v>
       </c>
       <c r="V79" t="n">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>54.67625899280576</v>
+        <v>54.38596491228071</v>
       </c>
       <c r="X79" s="7" t="n">
         <v>1.02</v>
@@ -9075,7 +9075,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9120,20 +9120,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/17/2026 20:46</t>
+          <t>08/18/2026 19:23</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>19843.08</v>
+        <v>19389.95</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>-0.77</v>
+        <v>-3.03</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9151,19 +9151,19 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>2043</v>
+        <v>2095</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>-77.51000000000113</v>
+        <v>-610.0500000000011</v>
       </c>
       <c r="V80" t="n">
-        <v>1255</v>
+        <v>1281</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>61.42927068037201</v>
+        <v>61.14558472553699</v>
       </c>
       <c r="X80" s="7" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Y80" s="7" t="n">
         <v>17.52</v>
@@ -9175,7 +9175,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9220,20 +9220,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/17/2026 21:07</t>
+          <t>08/18/2026 20:05</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>19138.79</v>
+        <v>18895.97</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-4.29</v>
+        <v>-5.5</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9251,19 +9251,19 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>1004</v>
+        <v>1035</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>-890.0100000000006</v>
+        <v>-1104.030000000001</v>
       </c>
       <c r="V81" t="n">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>51.29482071713147</v>
+        <v>50.82125603864734</v>
       </c>
       <c r="X81" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y81" s="7" t="n">
         <v>12.38</v>
@@ -9275,7 +9275,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9320,20 +9320,20 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/17/2026 21:04</t>
+          <t>08/18/2026 19:54</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>19879.03</v>
+        <v>19710.63</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>-0.57</v>
+        <v>-1.41</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>0.96</v>
+        <v>0.9</v>
       </c>
       <c r="L82" t="n">
         <v>20000</v>
@@ -9451,19 +9451,22 @@
         <v>0</v>
       </c>
       <c r="T83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U83" s="7" t="n">
-        <v>42.78</v>
+        <v>-6.659999999999997</v>
       </c>
       <c r="V83" t="n">
         <v>1</v>
       </c>
       <c r="W83" s="7" t="n">
-        <v>100</v>
+        <v>50</v>
+      </c>
+      <c r="X83" s="7" t="n">
+        <v>0.87</v>
       </c>
       <c r="Y83" s="7" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Z83" t="inlineStr">
         <is>
@@ -9472,7 +9475,7 @@
       </c>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB83" t="inlineStr">
@@ -9517,7 +9520,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/17/2026 21:34</t>
+          <t>08/18/2026 20:54</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9617,7 +9620,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/17/2026 21:06</t>
+          <t>08/18/2026 20:02</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9717,14 +9720,14 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/17/2026 21:14</t>
+          <t>08/18/2026 20:17</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20899.75</v>
+        <v>20901.95</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>4.51</v>
+        <v>4.52</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>2.18</v>
@@ -9748,16 +9751,16 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>899.7500000000001</v>
+        <v>901.95</v>
       </c>
       <c r="V86" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>49.29577464788733</v>
+        <v>49.31506849315068</v>
       </c>
       <c r="X86" s="7" t="n">
         <v>2.28</v>
@@ -9772,7 +9775,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9817,7 +9820,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/17/2026 20:58</t>
+          <t>08/18/2026 19:45</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9917,20 +9920,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/17/2026 21:06</t>
+          <t>08/18/2026 20:02</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20476.42</v>
+        <v>20497.82</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>2.37</v>
+        <v>2.48</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -9948,19 +9951,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
+        <v>35</v>
+      </c>
+      <c r="U88" s="7" t="n">
+        <v>497.8199999999999</v>
+      </c>
+      <c r="V88" t="n">
         <v>33</v>
       </c>
-      <c r="U88" s="7" t="n">
-        <v>476.42</v>
-      </c>
-      <c r="V88" t="n">
-        <v>31</v>
-      </c>
       <c r="W88" s="7" t="n">
-        <v>93.93939393939394</v>
+        <v>94.28571428571428</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -9972,7 +9975,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10017,20 +10020,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/17/2026 21:06</t>
+          <t>08/18/2026 14:52</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>22458.33</v>
+        <v>22010.81</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>12.32</v>
+        <v>10.08</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>1.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>6.85</v>
+        <v>2.84</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10048,19 +10051,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>2458.33</v>
+        <v>2010.81</v>
       </c>
       <c r="V89" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>91.30434782608695</v>
+        <v>81.48148148148148</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>6.85</v>
+        <v>2.84</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>1.99</v>
@@ -10072,7 +10075,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10117,7 +10120,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/17/2026 20:34</t>
+          <t>08/18/2026 18:56</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
@@ -10148,22 +10151,22 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>159.92</v>
+        <v>58.40999999999998</v>
       </c>
       <c r="V90" t="n">
         <v>21</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>87.5</v>
+        <v>84</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>3.98</v>
+        <v>1.38</v>
       </c>
       <c r="Y90" s="7" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10172,7 +10175,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10217,7 +10220,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/17/2026 20:34</t>
+          <t>08/18/2026 18:52</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10317,20 +10320,20 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/17/2026 20:32</t>
+          <t>08/18/2026 18:52</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
-        <v>20003.27</v>
+        <v>19979.06</v>
       </c>
       <c r="I92" s="7" t="n">
-        <v>0.02</v>
+        <v>-0.1</v>
       </c>
       <c r="J92" s="7" t="n">
-        <v>0.02</v>
+        <v>0.14</v>
       </c>
       <c r="K92" s="7" t="n">
-        <v>1.71</v>
+        <v>0.27</v>
       </c>
       <c r="L92" t="n">
         <v>20000</v>
@@ -10348,22 +10351,22 @@
         <v>0</v>
       </c>
       <c r="T92" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="U92" s="7" t="n">
-        <v>3.27</v>
+        <v>-20.94</v>
       </c>
       <c r="V92" t="n">
         <v>2</v>
       </c>
       <c r="W92" s="7" t="n">
-        <v>50</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="X92" s="7" t="n">
-        <v>1.71</v>
+        <v>0.27</v>
       </c>
       <c r="Y92" s="7" t="n">
-        <v>0.02</v>
+        <v>0.14</v>
       </c>
       <c r="Z92" t="inlineStr">
         <is>
@@ -10372,7 +10375,7 @@
       </c>
       <c r="AA92" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB92" t="inlineStr">
@@ -10382,7 +10385,7 @@
       </c>
       <c r="AC92" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Prop | AUDJPY.pro, T&amp;D19L13 L11 Prop | AUDUSD.pro, T&amp;D19L13 L11 Prop | GBPCHF.pro</t>
+          <t>T&amp;D19L13 L11 Prop | AUDJPY.pro, T&amp;D19L13 L11 Prop | AUDUSD.pro, T&amp;D19L13 L11 Prop | EURUSD.pro, T&amp;D19L13 L11 Prop | GBPAUD.pro, T&amp;D19L13 L11 Prop | GBPCHF.pro</t>
         </is>
       </c>
     </row>
@@ -10417,20 +10420,20 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/17/2026 20:37</t>
+          <t>08/18/2026 18:52</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
-        <v>20010.22</v>
+        <v>19935.43</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>0.05</v>
+        <v>-0.32</v>
       </c>
       <c r="J93" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.44</v>
       </c>
       <c r="K93" s="7" t="n">
-        <v>1.71</v>
+        <v>0.28</v>
       </c>
       <c r="L93" t="n">
         <v>20000</v>
@@ -10448,22 +10451,22 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="U93" s="7" t="n">
-        <v>10.22</v>
+        <v>-64.56999999999999</v>
       </c>
       <c r="V93" t="n">
         <v>2</v>
       </c>
       <c r="W93" s="7" t="n">
-        <v>50</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="X93" s="7" t="n">
-        <v>1.71</v>
+        <v>0.28</v>
       </c>
       <c r="Y93" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="Z93" t="inlineStr">
         <is>
@@ -10472,7 +10475,7 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB93" t="inlineStr">
@@ -10482,7 +10485,7 @@
       </c>
       <c r="AC93" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 MOL | AUDJPY.pro, T&amp;D19L13 L11 MOL | AUDUSD.pro, T&amp;D19L13 L11 MOL | GBPCHF.pro</t>
+          <t>T&amp;D19L13 L11 MOL | AUDJPY.pro, T&amp;D19L13 L11 MOL | AUDUSD.pro, T&amp;D19L13 L11 MOL | EURUSD.pro, T&amp;D19L13 L11 MOL | GBPAUD.pro, T&amp;D19L13 L11 MOL | GBPCHF.pro</t>
         </is>
       </c>
     </row>
@@ -10517,20 +10520,20 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/17/2026 20:32</t>
+          <t>08/18/2026 18:52</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
-        <v>20054.08</v>
+        <v>19900.96</v>
       </c>
       <c r="I94" s="7" t="n">
-        <v>0.26</v>
+        <v>-0.5</v>
       </c>
       <c r="J94" s="7" t="n">
-        <v>0.14</v>
+        <v>0.91</v>
       </c>
       <c r="K94" s="7" t="n">
-        <v>2.87</v>
+        <v>0.46</v>
       </c>
       <c r="L94" t="n">
         <v>20000</v>
@@ -10548,22 +10551,22 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="U94" s="7" t="n">
-        <v>54.08</v>
+        <v>-99.04000000000002</v>
       </c>
       <c r="V94" t="n">
         <v>3</v>
       </c>
       <c r="W94" s="7" t="n">
-        <v>60</v>
+        <v>37.5</v>
       </c>
       <c r="X94" s="7" t="n">
-        <v>2.87</v>
+        <v>0.46</v>
       </c>
       <c r="Y94" s="7" t="n">
-        <v>0.14</v>
+        <v>0.91</v>
       </c>
       <c r="Z94" t="inlineStr">
         <is>
@@ -10572,7 +10575,7 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB94" t="inlineStr">
@@ -10582,7 +10585,7 @@
       </c>
       <c r="AC94" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Agg | AUDJPY.pro, T&amp;D19L13 L11 Agg | AUDUSD.pro, T&amp;D19L13 L11 Agg | GBPCHF.pro, T&amp;D19L13 L11 Agg | XAUUSD</t>
+          <t>T&amp;D19L13 L11 Agg | AUDJPY.pro, T&amp;D19L13 L11 Agg | AUDUSD.pro, T&amp;D19L13 L11 Agg | EURUSD.pro, T&amp;D19L13 L11 Agg | GBPAUD.pro, T&amp;D19L13 L11 Agg | GBPCHF.pro, T&amp;D19L13 L11 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10617,20 +10620,20 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/17/2026 20:31</t>
+          <t>08/18/2026 18:45</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
-        <v>99220.14999999999</v>
+        <v>99227.49000000001</v>
       </c>
       <c r="I95" s="7" t="n">
         <v>-0.77</v>
       </c>
       <c r="J95" s="7" t="n">
-        <v>0.95</v>
+        <v>1.01</v>
       </c>
       <c r="K95" s="7" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="L95" t="n">
         <v>100000</v>
@@ -10648,22 +10651,22 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>266</v>
+        <v>291</v>
       </c>
       <c r="U95" s="7" t="n">
-        <v>-779.8499999999999</v>
+        <v>-772.5099999999999</v>
       </c>
       <c r="V95" t="n">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="W95" s="7" t="n">
-        <v>51.8796992481203</v>
+        <v>52.23367697594502</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="Y95" s="7" t="n">
-        <v>0.96</v>
+        <v>1.01</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -10672,7 +10675,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
@@ -10682,7 +10685,7 @@
       </c>
       <c r="AC95" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | GBPUSD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | US30, T&amp;D19L13 Meta4 Prop | US500, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 Prop | AUDCAD.pro, T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURAUD.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPAUD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | GBPUSD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | US30, T&amp;D19L13 Meta4 Prop | US500, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10717,20 +10720,20 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/17/2026 20:32</t>
+          <t>08/18/2026 18:56</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
-        <v>98048.10000000001</v>
+        <v>97936.66</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>-1.95</v>
+        <v>-2.07</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>2.52</v>
+        <v>2.77</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="L96" t="n">
         <v>100000</v>
@@ -10748,22 +10751,22 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>321</v>
+        <v>346</v>
       </c>
       <c r="U96" s="7" t="n">
-        <v>-1951.9</v>
+        <v>-2063.34</v>
       </c>
       <c r="V96" t="n">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="W96" s="7" t="n">
-        <v>51.71339563862928</v>
+        <v>52.02312138728323</v>
       </c>
       <c r="X96" s="7" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="Y96" s="7" t="n">
-        <v>2.52</v>
+        <v>2.78</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -10772,7 +10775,7 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr">
@@ -10782,7 +10785,7 @@
       </c>
       <c r="AC96" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | GBPUSD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | US30, T&amp;D19L13 Meta4 MOL | US500, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 MOL | AUDCAD.pro, T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURAUD.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPAUD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | GBPUSD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | US30, T&amp;D19L13 Meta4 MOL | US500, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10817,17 +10820,17 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/17/2026 20:37</t>
+          <t>08/18/2026 18:59</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
-        <v>97781.53</v>
+        <v>97652.64</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>-2.22</v>
+        <v>-2.35</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>3.26</v>
+        <v>3.59</v>
       </c>
       <c r="K97" s="7" t="n">
         <v>0.76</v>
@@ -10848,22 +10851,22 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>321</v>
+        <v>346</v>
       </c>
       <c r="U97" s="7" t="n">
-        <v>-2158.92</v>
+        <v>-2347.36</v>
       </c>
       <c r="V97" t="n">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="W97" s="7" t="n">
-        <v>51.71339563862928</v>
+        <v>52.02312138728323</v>
       </c>
       <c r="X97" s="7" t="n">
         <v>0.76</v>
       </c>
       <c r="Y97" s="7" t="n">
-        <v>3.19</v>
+        <v>3.58</v>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
@@ -10872,7 +10875,7 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB97" t="inlineStr">
@@ -10882,7 +10885,7 @@
       </c>
       <c r="AC97" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | GBPUSD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | US30, T&amp;D19L13 Meta4 Agg | US500, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 Agg | AUDCAD.pro, T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURAUD.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPAUD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | GBPUSD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | US30, T&amp;D19L13 Meta4 Agg | US500, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10917,20 +10920,20 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/17/2026 20:31</t>
+          <t>08/18/2026 18:45</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
-        <v>99585.02</v>
+        <v>99537.8</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>-0.43</v>
+        <v>-0.49</v>
       </c>
       <c r="J98" s="7" t="n">
-        <v>0.67</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="L98" t="n">
         <v>100000</v>
@@ -10948,22 +10951,22 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="U98" s="7" t="n">
-        <v>-414.9799999999999</v>
+        <v>-462.1999999999999</v>
       </c>
       <c r="V98" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="W98" s="7" t="n">
-        <v>47.16981132075472</v>
+        <v>46.42857142857143</v>
       </c>
       <c r="X98" s="7" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="Y98" s="7" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="Z98" t="inlineStr">
         <is>
@@ -10972,7 +10975,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
@@ -10982,7 +10985,7 @@
       </c>
       <c r="AC98" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | GBPJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USDCHF.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | EURUSD.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | GBPJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USDCHF.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11017,7 +11020,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/17/2026 20:34</t>
+          <t>08/18/2026 18:56</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11117,7 +11120,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/17/2026 20:58</t>
+          <t>08/18/2026 19:44</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11444,14 +11447,14 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/17/2026 20:03</t>
+          <t>08/18/2026 18:11</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>27079.51</v>
+        <v>27084.78</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-29.48</v>
+        <v>-29.47</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
@@ -11469,31 +11472,31 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>162.25</v>
+        <v>188.87</v>
       </c>
       <c r="P103" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>1.48390945151958</v>
+        <v>1.831769938785397</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>0.96</v>
+        <v>0.59</v>
       </c>
       <c r="T103" t="n">
-        <v>3468</v>
+        <v>3469</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-7224.77</v>
+        <v>-7191.75</v>
       </c>
       <c r="V103" t="n">
-        <v>2074</v>
+        <v>2086</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>59.80392156862745</v>
+        <v>60.13260305563563</v>
       </c>
       <c r="X103" s="7" t="n">
         <v>0.78</v>
@@ -11508,7 +11511,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11735,7 +11738,7 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>08/15/2026 14:30</t>
+          <t>08/18/2026 14:31</t>
         </is>
       </c>
       <c r="H106" s="9" t="n">
@@ -12099,7 +12102,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:44</t>
+          <t>08/18/2026 19:20</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12190,7 +12193,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>08/15/2026 18:02</t>
+          <t>08/18/2026 18:31</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12372,7 +12375,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 21:01</t>
+          <t>08/18/2026 19:51</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12463,7 +12466,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:40</t>
+          <t>08/18/2026 19:00</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12548,7 +12551,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:46</t>
+          <t>08/18/2026 19:15</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12633,7 +12636,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>08/15/2026 13:43</t>
+          <t>08/18/2026 13:44</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12803,7 +12806,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:40</t>
+          <t>08/18/2026 19:04</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12888,7 +12891,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:39</t>
+          <t>08/18/2026 19:06</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12973,7 +12976,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:35</t>
+          <t>08/18/2026 18:59</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13058,7 +13061,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:40</t>
+          <t>08/18/2026 19:06</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13143,7 +13146,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:43</t>
+          <t>08/18/2026 19:14</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13228,7 +13231,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 20:39</t>
+          <t>08/18/2026 19:06</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13313,7 +13316,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>08/15/2026 19:26</t>
+          <t>08/18/2026 20:13</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13404,7 +13407,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>08/15/2026 19:07</t>
+          <t>08/18/2026 19:52</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13843,7 +13846,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08/15/2026 14:30</t>
+          <t>08/18/2026 14:31</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14007,7 +14010,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/17/2026 20:44</t>
+          <t>08/18/2026 19:20</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14048,7 +14051,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>08/15/2026 18:02</t>
+          <t>08/18/2026 18:31</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14130,7 +14133,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/17/2026 21:01</t>
+          <t>08/18/2026 19:51</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14171,7 +14174,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/17/2026 20:40</t>
+          <t>08/18/2026 19:00</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14212,7 +14215,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/17/2026 20:46</t>
+          <t>08/18/2026 19:15</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14253,7 +14256,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/15/2026 13:43</t>
+          <t>08/18/2026 13:44</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14335,7 +14338,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/17/2026 20:40</t>
+          <t>08/18/2026 19:04</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14376,7 +14379,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/17/2026 20:39</t>
+          <t>08/18/2026 19:06</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14417,7 +14420,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/17/2026 20:35</t>
+          <t>08/18/2026 18:59</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14458,7 +14461,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/17/2026 20:40</t>
+          <t>08/18/2026 19:06</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14499,7 +14502,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/17/2026 20:43</t>
+          <t>08/18/2026 19:14</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14540,7 +14543,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/17/2026 20:39</t>
+          <t>08/18/2026 19:06</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -14581,7 +14584,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>08/15/2026 19:26</t>
+          <t>08/18/2026 20:13</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -14622,7 +14625,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>08/15/2026 19:07</t>
+          <t>08/18/2026 19:52</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
@@ -15720,7 +15723,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08/15/2026 20:50</t>
+          <t>08/18/2026 21:43</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -15766,7 +15769,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08/15/2026 20:38</t>
+          <t>08/18/2026 21:29</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -15789,7 +15792,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08/15/2026 16:28</t>
+          <t>08/18/2026 16:31</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -15858,7 +15861,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08/15/2026 15:54</t>
+          <t>08/18/2026 15:55</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -15973,7 +15976,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08/15/2026 20:35</t>
+          <t>08/18/2026 21:29</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -16088,7 +16091,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08/12/2026 16:18</t>
+          <t>08/18/2026 16:22</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -16111,7 +16114,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/17/2026 21:40</t>
+          <t>08/18/2026 21:13</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16157,11 +16160,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/17/2026 20:45</t>
+          <t>08/18/2026 19:20</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20434.06</v>
+        <v>20364.54</v>
       </c>
     </row>
     <row r="24">
@@ -16203,11 +16206,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/17/2026 21:10</t>
+          <t>08/18/2026 20:13</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19734.69</v>
+        <v>19838.33</v>
       </c>
     </row>
     <row r="26">
@@ -16226,11 +16229,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/17/2026 20:54</t>
+          <t>08/18/2026 19:40</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21621.74</v>
+        <v>21395.6</v>
       </c>
     </row>
     <row r="27">
@@ -16249,7 +16252,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/17/2026 19:31</t>
+          <t>08/18/2026 16:52</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16272,7 +16275,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/17/2026 19:30</t>
+          <t>08/18/2026 16:53</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16295,7 +16298,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/17/2026 19:34</t>
+          <t>08/18/2026 17:05</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16318,7 +16321,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/17/2026 19:23</t>
+          <t>08/18/2026 16:37</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16341,7 +16344,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/17/2026 19:28</t>
+          <t>08/18/2026 16:50</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16364,7 +16367,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/17/2026 19:28</t>
+          <t>08/18/2026 16:43</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16410,7 +16413,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/17/2026 20:32</t>
+          <t>08/18/2026 18:52</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -16433,7 +16436,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>08/17/2026 20:34</t>
+          <t>08/18/2026 18:56</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -16479,7 +16482,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/15/2026 20:34</t>
+          <t>08/18/2026 21:32</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -16548,7 +16551,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/17/2026 11:33</t>
+          <t>08/18/2026 11:40</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-19
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-18 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-19 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/18/2026 18:21</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>59950</v>
+          <t>08/19/2026 17:32</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>49845.7</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>174.03</v>
+        <v>127.84</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.1</v>
+        <v>1.08</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>35099.36</v>
+        <v>20109.34</v>
       </c>
       <c r="P2" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>5.622241419725611</v>
+        <v>2.040253600528473</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>9.32</v>
+        <v>21.24</v>
       </c>
       <c r="T2" t="n">
-        <v>3334</v>
+        <v>3338</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>34949.99999999999</v>
+        <v>24845.69999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2106</v>
+        <v>2109</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.16736652669466</v>
+        <v>63.18154583582983</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.08</v>
+        <v>1.06</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/16/2026 19:23</t>
+          <t>08/19/2026 19:25</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/18/2026 21:44</t>
+          <t>08/19/2026 19:43</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08/16/2026 09:42</t>
+          <t>08/19/2026 09:44</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/16/2026 14:57</t>
+          <t>08/19/2026 14:59</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08/15/2026 22:40</t>
+          <t>08/18/2026 23:32</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>08/15/2026 23:55</t>
+          <t>08/19/2026 00:40</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>08/15/2026 23:55</t>
+          <t>08/19/2026 00:40</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/18/2026 18:06</t>
+          <t>08/19/2026 20:31</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/18/2026 16:40</t>
+          <t>08/19/2026 19:49</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/18/2026 21:25</t>
+          <t>08/19/2026 19:34</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/18/2026 19:48</t>
+          <t>08/19/2026 21:29</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/18/2026 18:48</t>
+          <t>08/19/2026 20:59</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3289,16 +3289,16 @@
         <v>4.21</v>
       </c>
       <c r="T23" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-132.7699999999999</v>
+        <v>-132.7699999999998</v>
       </c>
       <c r="V23" t="n">
         <v>42</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>53.16455696202531</v>
+        <v>52.5</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>0.97</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3467,20 +3467,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/18/2026 19:20</t>
+          <t>08/19/2026 21:15</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16445.5</v>
+        <v>16615.3</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-17.46</v>
+        <v>-16.6</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.67</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3492,34 +3492,34 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>48.76999999999998</v>
+        <v>41.65000000000002</v>
       </c>
       <c r="P25" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>57.49999999999999</v>
+        <v>45</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.146817990246252</v>
+        <v>1.093010272443055</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>1.19</v>
+        <v>1.34</v>
       </c>
       <c r="T25" t="n">
-        <v>678</v>
+        <v>687</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3554.5</v>
+        <v>-3599.15</v>
       </c>
       <c r="V25" t="n">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>39.82300884955752</v>
+        <v>39.5924308588064</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>21.17</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/18/2026 17:37</t>
+          <t>08/19/2026 20:13</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/18/2026 19:06</t>
+          <t>08/19/2026 21:06</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3725,7 +3725,7 @@
         <v>3.75</v>
       </c>
       <c r="T27" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="U27" s="7" t="n">
         <v>425.62</v>
@@ -3734,7 +3734,7 @@
         <v>46</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>45.54455445544555</v>
+        <v>44.66019417475729</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>1.1</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>08/15/2026 21:53</t>
+          <t>08/18/2026 22:43</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,14 +3903,14 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/18/2026 19:07</t>
+          <t>08/19/2026 21:08</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19646.46</v>
+        <v>19637.38</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-1.78</v>
+        <v>-1.83</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
@@ -3928,31 +3928,31 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-674.53</v>
+        <v>-657.92</v>
       </c>
       <c r="P29" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>32.5</v>
+        <v>35</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.2003106142337194</v>
+        <v>0.240189398313893</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>3.79</v>
+        <v>3.66</v>
       </c>
       <c r="T29" t="n">
         <v>122</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-353.5400000000002</v>
+        <v>-362.6200000000002</v>
       </c>
       <c r="V29" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>47.54098360655738</v>
+        <v>48.36065573770492</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>0.87</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08/16/2026 10:18</t>
+          <t>08/19/2026 10:19</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/18/2026 19:23</t>
+          <t>08/19/2026 21:16</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/18/2026 18:54</t>
+          <t>08/19/2026 21:01</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/18/2026 21:34</t>
+          <t>08/19/2026 19:37</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20090.73</v>
+        <v>20040.77</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.45</v>
+        <v>0.2</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>3.42</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,7 +4473,7 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-433.67</v>
+        <v>-432.08</v>
       </c>
       <c r="P34" t="n">
         <v>12</v>
@@ -4482,25 +4482,25 @@
         <v>30</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.6417253230230329</v>
+        <v>0.6425693841254084</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>2.91</v>
+        <v>2.66</v>
       </c>
       <c r="T34" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U34" s="7" t="n">
-        <v>124.93</v>
+        <v>40.77000000000005</v>
       </c>
       <c r="V34" t="n">
         <v>44</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>41.50943396226415</v>
+        <v>41.1214953271028</v>
       </c>
       <c r="X34" s="7" t="n">
-        <v>1.05</v>
+        <v>1.02</v>
       </c>
       <c r="Y34" s="7" t="n">
         <v>3.43</v>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/18/2026 20:48</t>
+          <t>08/19/2026 19:03</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19816.79</v>
+        <v>19915.68</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.91</v>
+        <v>-0.42</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-183.2100000000001</v>
+        <v>-84.32000000000009</v>
       </c>
       <c r="V36" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>48.80952380952381</v>
+        <v>49.41176470588236</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.83</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/18/2026 20:06</t>
+          <t>08/19/2026 21:41</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/18/2026 20:43</t>
+          <t>08/19/2026 19:03</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>08/16/2026 09:26</t>
+          <t>08/19/2026 09:29</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>08/16/2026 07:27</t>
+          <t>08/19/2026 07:28</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/18/2026 19:07</t>
+          <t>08/19/2026 21:07</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/18/2026 19:50</t>
+          <t>08/19/2026 21:27</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,13 +5442,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T43" t="n">
         <v>4278</v>
@@ -5520,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/18/2026 19:08</t>
+          <t>08/19/2026 21:07</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5542,13 +5551,22 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5620,20 +5638,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/18/2026 19:25</t>
+          <t>08/19/2026 21:14</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19632.66</v>
+        <v>19772.33</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-1.82</v>
+        <v>-1.12</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>4.38</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.88</v>
+        <v>0.93</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5642,28 +5660,37 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>-4.869999999999998</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>0.9739836529729152</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>0.77</v>
       </c>
       <c r="T45" t="n">
-        <v>448</v>
+        <v>467</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-367.34</v>
+        <v>-217.2</v>
       </c>
       <c r="V45" t="n">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>54.91071428571429</v>
+        <v>55.46038543897216</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.88</v>
+        <v>0.93</v>
       </c>
       <c r="Y45" s="7" t="n">
         <v>4.39</v>
@@ -5675,7 +5702,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5720,20 +5747,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/18/2026 18:52</t>
+          <t>08/19/2026 20:54</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19983.62</v>
+        <v>19982.08</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>-0.08</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5742,31 +5769,40 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>19977.76</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q46" s="7" t="n">
+        <v>32.43243243243244</v>
+      </c>
+      <c r="R46" s="7" t="n">
+        <v>311.8411389450754</v>
+      </c>
+      <c r="S46" s="7" t="n">
+        <v>0.11</v>
       </c>
       <c r="T46" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-16.38</v>
+        <v>-17.92</v>
       </c>
       <c r="V46" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>27.27272727272727</v>
+        <v>30.55555555555556</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="Y46" s="7" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5775,12 +5811,12 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5820,7 +5856,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/18/2026 19:00</t>
+          <t>08/19/2026 21:00</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5842,13 +5878,22 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>82.33999999999995</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q47" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R47" s="7" t="n">
+        <v>1.059591960802762</v>
+      </c>
+      <c r="S47" s="7" t="n">
+        <v>2.1</v>
       </c>
       <c r="T47" t="n">
         <v>61</v>
@@ -5920,7 +5965,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/18/2026 18:49</t>
+          <t>08/19/2026 20:55</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -5942,13 +5987,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>504.68</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>2.47982641332395</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>1.7</v>
       </c>
       <c r="T48" t="n">
         <v>193</v>
@@ -6020,7 +6074,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/18/2026 19:27</t>
+          <t>08/19/2026 21:17</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6042,13 +6096,22 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>0</v>
+        <v>698.46</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="Q49" s="7" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="R49" s="7" t="n">
+        <v>7.636199524940618</v>
+      </c>
+      <c r="S49" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T49" t="n">
         <v>410</v>
@@ -6120,7 +6183,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/18/2026 19:20</t>
+          <t>08/19/2026 21:14</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6142,13 +6205,22 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>0</v>
+        <v>13.93999999999999</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q50" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R50" s="7" t="n">
+        <v>1.066618876941458</v>
+      </c>
+      <c r="S50" s="7" t="n">
+        <v>0.89</v>
       </c>
       <c r="T50" t="n">
         <v>1161</v>
@@ -6220,7 +6292,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/18/2026 19:01</t>
+          <t>08/19/2026 20:59</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6242,13 +6314,22 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>0</v>
+        <v>-52.41999999999999</v>
       </c>
       <c r="P51" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q51" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R51" s="7" t="n">
+        <v>0.8051952878219183</v>
+      </c>
+      <c r="S51" s="7" t="n">
+        <v>1.3</v>
       </c>
       <c r="T51" t="n">
         <v>1978</v>
@@ -6320,20 +6401,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/18/2026 18:52</t>
+          <t>08/19/2026 21:01</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19520.45</v>
+        <v>19322.78</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-2.39</v>
+        <v>-3.38</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.85</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6342,28 +6423,37 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>0</v>
+        <v>19223.51</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q52" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R52" s="7" t="n">
+        <v>6.415057985752154</v>
+      </c>
+      <c r="S52" s="7" t="n">
+        <v>5.22</v>
       </c>
       <c r="T52" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-479.5500000000002</v>
+        <v>-677.22</v>
       </c>
       <c r="V52" t="n">
         <v>11</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>28.2051282051282</v>
+        <v>27.5</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.85</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>10.19</v>
@@ -6375,7 +6465,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6420,20 +6510,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/18/2026 19:38</t>
+          <t>08/19/2026 21:24</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19703.78</v>
+        <v>19794.62</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.5</v>
+        <v>-1.05</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.78</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6442,28 +6532,37 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>0</v>
+        <v>-5.350000000000002</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q53" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R53" s="7" t="n">
+        <v>0.956813044882144</v>
+      </c>
+      <c r="S53" s="7" t="n">
+        <v>0.51</v>
       </c>
       <c r="T53" t="n">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-296.2199999999999</v>
+        <v>-281.52</v>
       </c>
       <c r="V53" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>37.06563706563706</v>
+        <v>36.9811320754717</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6475,7 +6574,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6520,7 +6619,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/18/2026 19:52</t>
+          <t>08/19/2026 21:33</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6542,13 +6641,22 @@
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>0</v>
+        <v>-149.77</v>
       </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q54" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R54" s="7" t="n">
+        <v>0.4112351599968551</v>
+      </c>
+      <c r="S54" s="7" t="n">
+        <v>0.83</v>
       </c>
       <c r="T54" t="n">
         <v>229</v>
@@ -6620,7 +6728,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/18/2026 19:27</t>
+          <t>08/19/2026 21:17</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6642,13 +6750,22 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>0</v>
+        <v>-54.22</v>
       </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="Q55" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="R55" s="7" t="n">
+        <v>0.506462770799199</v>
+      </c>
+      <c r="S55" s="7" t="n">
+        <v>0.27</v>
       </c>
       <c r="T55" t="n">
         <v>1920</v>
@@ -6720,7 +6837,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/18/2026 19:46</t>
+          <t>08/19/2026 21:31</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6742,13 +6859,22 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O56" s="7" t="n">
-        <v>0</v>
+        <v>4.35</v>
       </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q56" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R56" s="7" t="n">
+        <v>1.066564651874522</v>
+      </c>
+      <c r="S56" s="7" t="n">
+        <v>0.16</v>
       </c>
       <c r="T56" t="n">
         <v>1272</v>
@@ -6820,14 +6946,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/18/2026 18:50</t>
+          <t>08/19/2026 20:58</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19748.58</v>
+        <v>19750.95</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.26</v>
+        <v>-1.25</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6842,25 +6968,34 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>0</v>
+        <v>3.939999999999999</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q57" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R57" s="7" t="n">
+        <v>1.183000464468184</v>
+      </c>
+      <c r="S57" s="7" t="n">
+        <v>0.06</v>
       </c>
       <c r="T57" t="n">
-        <v>791</v>
+        <v>808</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-251.42</v>
+        <v>-249.7200000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.62705436156764</v>
+        <v>44.3069306930693</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.8100000000000001</v>
@@ -6875,7 +7010,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6920,7 +7055,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/18/2026 19:18</t>
+          <t>08/19/2026 21:12</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -6942,13 +7077,22 @@
         <v>0</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O58" s="7" t="n">
-        <v>0</v>
+        <v>-83.65000000000001</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q58" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R58" s="7" t="n">
+        <v>0.3526042875938395</v>
+      </c>
+      <c r="S58" s="7" t="n">
+        <v>0.46</v>
       </c>
       <c r="T58" t="n">
         <v>4426</v>
@@ -7020,7 +7164,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/18/2026 19:00</t>
+          <t>08/19/2026 21:04</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7042,13 +7186,22 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>0</v>
+        <v>-80.78999999999999</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="Q59" s="7" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="R59" s="7" t="n">
+        <v>0.32387647501883</v>
+      </c>
+      <c r="S59" s="7" t="n">
+        <v>0.43</v>
       </c>
       <c r="T59" t="n">
         <v>304</v>
@@ -7120,14 +7273,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/18/2026 19:05</t>
+          <t>08/19/2026 21:08</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>20446.56</v>
+        <v>20418.34</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-3.87</v>
+        <v>-4.01</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
@@ -7142,13 +7295,22 @@
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O60" s="7" t="n">
-        <v>0</v>
+        <v>326.88</v>
       </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q60" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R60" s="7" t="n">
+        <v>6.042887997531627</v>
+      </c>
+      <c r="S60" s="7" t="n">
+        <v>0.19</v>
       </c>
       <c r="T60" t="n">
         <v>7019</v>
@@ -7220,7 +7382,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/18/2026 19:42</t>
+          <t>08/19/2026 21:26</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7242,13 +7404,22 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O61" s="7" t="n">
-        <v>0</v>
+        <v>343.99</v>
       </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>21</v>
+      </c>
+      <c r="Q61" s="7" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="R61" s="7" t="n">
+        <v>5.804329608938549</v>
+      </c>
+      <c r="S61" s="7" t="n">
+        <v>0.28</v>
       </c>
       <c r="T61" t="n">
         <v>3982</v>
@@ -7320,7 +7491,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/18/2026 19:41</t>
+          <t>08/19/2026 18:23</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7342,13 +7513,22 @@
         <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O62" s="7" t="n">
-        <v>0</v>
+        <v>-353.59</v>
       </c>
       <c r="P62" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q62" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R62" s="7" t="n">
+        <v>0.3361931402181462</v>
+      </c>
+      <c r="S62" s="7" t="n">
+        <v>2.17</v>
       </c>
       <c r="T62" t="n">
         <v>170</v>
@@ -7420,20 +7600,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/18/2026 19:36</t>
+          <t>08/19/2026 21:23</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18557.89</v>
+        <v>18748.23</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-7.22</v>
+        <v>-6.27</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>7.22</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.29</v>
+        <v>0.38</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7442,16 +7622,25 @@
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>0</v>
+        <v>-737.4599999999999</v>
       </c>
       <c r="P63" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="Q63" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="R63" s="7" t="n">
+        <v>0.5123199619092965</v>
+      </c>
+      <c r="S63" s="7" t="n">
+        <v>4.64</v>
       </c>
       <c r="T63" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="U63" s="7" t="n">
         <v>-1442.11</v>
@@ -7460,7 +7649,7 @@
         <v>3</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>7.317073170731707</v>
+        <v>7.142857142857142</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>0.29</v>
@@ -7475,7 +7664,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7520,7 +7709,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/18/2026 19:46</t>
+          <t>08/19/2026 21:29</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7542,13 +7731,22 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>0</v>
+        <v>-3.710000000000004</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q64" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R64" s="7" t="n">
+        <v>0.9861323963667626</v>
+      </c>
+      <c r="S64" s="7" t="n">
+        <v>0.95</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7620,11 +7818,11 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/18/2026 19:22</t>
+          <t>08/19/2026 18:13</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19276.92</v>
+        <v>18879.58</v>
       </c>
       <c r="I65" s="7" t="n">
         <v>-3.62</v>
@@ -7642,13 +7840,22 @@
         <v>0</v>
       </c>
       <c r="N65" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O65" s="7" t="n">
-        <v>0</v>
+        <v>88.81000000000003</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="Q65" s="7" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="R65" s="7" t="n">
+        <v>1.163430926924422</v>
+      </c>
+      <c r="S65" s="7" t="n">
+        <v>2.24</v>
       </c>
       <c r="T65" t="n">
         <v>3298</v>
@@ -7720,7 +7927,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/18/2026 19:17</t>
+          <t>08/19/2026 21:12</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7742,13 +7949,22 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>0</v>
+        <v>-116.23</v>
       </c>
       <c r="P66" t="n">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="Q66" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="R66" s="7" t="n">
+        <v>0.317217881689479</v>
+      </c>
+      <c r="S66" s="7" t="n">
+        <v>0.66</v>
       </c>
       <c r="T66" t="n">
         <v>262</v>
@@ -7820,7 +8036,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/18/2026 20:09</t>
+          <t>08/19/2026 21:41</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7842,13 +8058,22 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>0</v>
+        <v>-51.36999999999998</v>
       </c>
       <c r="P67" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q67" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R67" s="7" t="n">
+        <v>0.9115149427267248</v>
+      </c>
+      <c r="S67" s="7" t="n">
+        <v>2.12</v>
       </c>
       <c r="T67" t="n">
         <v>215</v>
@@ -7942,13 +8167,22 @@
         <v>0</v>
       </c>
       <c r="N68" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O68" s="7" t="n">
-        <v>0</v>
+        <v>-35.83</v>
       </c>
       <c r="P68" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q68" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R68" s="7" t="n">
+        <v>0.5722812462695476</v>
+      </c>
+      <c r="S68" s="7" t="n">
+        <v>0.2</v>
       </c>
       <c r="T68" t="n">
         <v>55</v>
@@ -8042,13 +8276,22 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>0</v>
+        <v>71.06</v>
       </c>
       <c r="P69" t="n">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="Q69" s="7" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R69" s="7" t="n">
+        <v>2.289187227866473</v>
+      </c>
+      <c r="S69" s="7" t="n">
+        <v>0.14</v>
       </c>
       <c r="T69" t="n">
         <v>271</v>
@@ -8142,13 +8385,22 @@
         <v>0</v>
       </c>
       <c r="N70" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O70" s="7" t="n">
-        <v>0</v>
+        <v>19946.4</v>
       </c>
       <c r="P70" t="n">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="Q70" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R70" s="7" t="n">
+        <v>278.6503340757238</v>
+      </c>
+      <c r="S70" s="7" t="n">
+        <v>0.17</v>
       </c>
       <c r="T70" t="n">
         <v>7</v>
@@ -8180,7 +8432,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC70" t="inlineStr">
@@ -8220,7 +8472,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/18/2026 19:30</t>
+          <t>08/19/2026 21:19</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8242,13 +8494,22 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O71" s="7" t="n">
-        <v>0</v>
+        <v>10.11</v>
       </c>
       <c r="P71" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q71" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R71" s="7" t="n">
+        <v>1.117407966554407</v>
+      </c>
+      <c r="S71" s="7" t="n">
+        <v>0.23</v>
       </c>
       <c r="T71" t="n">
         <v>326</v>
@@ -8320,7 +8581,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/18/2026 20:19</t>
+          <t>08/19/2026 18:46</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8342,13 +8603,22 @@
         <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O72" s="7" t="n">
-        <v>0</v>
+        <v>17.22000000000001</v>
       </c>
       <c r="P72" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q72" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R72" s="7" t="n">
+        <v>1.101198871650211</v>
+      </c>
+      <c r="S72" s="7" t="n">
+        <v>0.49</v>
       </c>
       <c r="T72" t="n">
         <v>329</v>
@@ -8420,7 +8690,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/18/2026 19:37</t>
+          <t>08/19/2026 21:22</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8442,13 +8712,22 @@
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O73" s="7" t="n">
-        <v>0</v>
+        <v>28.34</v>
       </c>
       <c r="P73" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q73" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R73" s="7" t="n">
+        <v>1.110036886041545</v>
+      </c>
+      <c r="S73" s="7" t="n">
+        <v>0.73</v>
       </c>
       <c r="T73" t="n">
         <v>329</v>
@@ -8520,20 +8799,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/18/2026 20:09</t>
+          <t>08/19/2026 21:39</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20681.14</v>
+        <v>20666.64</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>3.42</v>
+        <v>3.36</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>1.73</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.49</v>
+        <v>1.47</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8542,28 +8821,37 @@
         <v>0</v>
       </c>
       <c r="N74" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O74" s="7" t="n">
-        <v>0</v>
+        <v>140.88</v>
       </c>
       <c r="P74" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="Q74" s="7" t="n">
+        <v>57.49999999999999</v>
+      </c>
+      <c r="R74" s="7" t="n">
+        <v>1.240290641150284</v>
+      </c>
+      <c r="S74" s="7" t="n">
+        <v>1.57</v>
       </c>
       <c r="T74" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>681.1400000000001</v>
+        <v>669.2400000000001</v>
       </c>
       <c r="V74" t="n">
         <v>63</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>67.74193548387096</v>
+        <v>67.02127659574468</v>
       </c>
       <c r="X74" s="7" t="n">
-        <v>1.49</v>
+        <v>1.47</v>
       </c>
       <c r="Y74" s="7" t="n">
         <v>1.73</v>
@@ -8575,7 +8863,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8620,20 +8908,20 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/18/2026 19:21</t>
+          <t>08/19/2026 21:12</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20119.91</v>
+        <v>20221.62</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>0.63</v>
+        <v>1.14</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K75" s="7" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="L75" t="n">
         <v>20000</v>
@@ -8642,28 +8930,37 @@
         <v>0</v>
       </c>
       <c r="N75" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O75" s="7" t="n">
-        <v>0</v>
+        <v>248.55</v>
       </c>
       <c r="P75" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q75" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R75" s="7" t="n">
+        <v>2.072214313446357</v>
+      </c>
+      <c r="S75" s="7" t="n">
+        <v>0.53</v>
       </c>
       <c r="T75" t="n">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>133.2299999999999</v>
+        <v>221.6200000000001</v>
       </c>
       <c r="V75" t="n">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>54.64285714285714</v>
+        <v>54.63917525773196</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="Y75" s="7" t="n">
         <v>4.5</v>
@@ -8675,7 +8972,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8720,20 +9017,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/18/2026 19:53</t>
+          <t>08/19/2026 21:33</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>20334.68</v>
+        <v>20529.59</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>1.7</v>
+        <v>2.68</v>
       </c>
       <c r="J76" s="7" t="n">
-        <v>5.53</v>
+        <v>5.69</v>
       </c>
       <c r="K76" s="7" t="n">
-        <v>1.05</v>
+        <v>1.08</v>
       </c>
       <c r="L76" t="n">
         <v>20000</v>
@@ -8742,31 +9039,40 @@
         <v>0</v>
       </c>
       <c r="N76" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O76" s="7" t="n">
-        <v>0</v>
+        <v>155.39</v>
       </c>
       <c r="P76" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q76" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R76" s="7" t="n">
+        <v>1.816595722318566</v>
+      </c>
+      <c r="S76" s="7" t="n">
+        <v>0.45</v>
       </c>
       <c r="T76" t="n">
-        <v>1225</v>
+        <v>1254</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>334.6800000000003</v>
+        <v>393.67</v>
       </c>
       <c r="V76" t="n">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>58.61224489795919</v>
+        <v>58.0542264752791</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="Y76" s="7" t="n">
-        <v>5.56</v>
+        <v>5.72</v>
       </c>
       <c r="Z76" t="inlineStr">
         <is>
@@ -8775,7 +9081,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8820,14 +9126,14 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/18/2026 19:42</t>
+          <t>08/19/2026 21:24</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>19790.91</v>
-      </c>
-      <c r="I77" s="7" t="n">
-        <v>-1.06</v>
+        <v>19804.49</v>
+      </c>
+      <c r="I77" t="n">
+        <v>-1</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
@@ -8842,25 +9148,34 @@
         <v>0</v>
       </c>
       <c r="N77" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O77" s="7" t="n">
-        <v>0</v>
+        <v>24.35</v>
       </c>
       <c r="P77" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q77" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R77" s="7" t="n">
+        <v>1.160927896371687</v>
+      </c>
+      <c r="S77" s="7" t="n">
+        <v>0.4</v>
       </c>
       <c r="T77" t="n">
-        <v>1097</v>
+        <v>1128</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>-209.0900000000002</v>
+        <v>-222.3199999999999</v>
       </c>
       <c r="V77" t="n">
-        <v>558</v>
+        <v>577</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>50.86599817684594</v>
+        <v>51.15248226950354</v>
       </c>
       <c r="X77" s="7" t="n">
         <v>0.97</v>
@@ -8875,7 +9190,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8920,20 +9235,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/18/2026 19:46</t>
+          <t>08/19/2026 18:27</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>19906.67</v>
+        <v>19948.56</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>-0.46</v>
+        <v>-0.25</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -8942,28 +9257,37 @@
         <v>0</v>
       </c>
       <c r="N78" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O78" s="7" t="n">
-        <v>0</v>
+        <v>528.8599999999998</v>
       </c>
       <c r="P78" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q78" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R78" s="7" t="n">
+        <v>1.291633580377625</v>
+      </c>
+      <c r="S78" s="7" t="n">
+        <v>4.01</v>
       </c>
       <c r="T78" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="U78" s="7" t="n">
-        <v>-93.3300000000002</v>
+        <v>-51.4400000000002</v>
       </c>
       <c r="V78" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="W78" s="7" t="n">
-        <v>39.50617283950617</v>
+        <v>39.75903614457831</v>
       </c>
       <c r="X78" s="7" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="Y78" s="7" t="n">
         <v>5.5</v>
@@ -8975,7 +9299,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -9020,14 +9344,14 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/18/2026 19:51</t>
+          <t>08/19/2026 18:27</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>20374.38</v>
+        <v>20315.65</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>1.91</v>
+        <v>1.62</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>16.96</v>
@@ -9051,19 +9375,19 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>374.3799999999994</v>
+        <v>806.7199999999993</v>
       </c>
       <c r="V79" t="n">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>54.38596491228071</v>
+        <v>54.39189189189189</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>1.02</v>
+        <v>1.04</v>
       </c>
       <c r="Y79" s="7" t="n">
         <v>17</v>
@@ -9075,7 +9399,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9120,20 +9444,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/18/2026 19:23</t>
+          <t>08/19/2026 21:13</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>19389.95</v>
+        <v>20009.48</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>-3.03</v>
+        <v>0.08</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
-      <c r="K80" s="7" t="n">
-        <v>0.98</v>
+      <c r="K80" t="n">
+        <v>1</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9151,19 +9475,19 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>2095</v>
+        <v>2148</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>-610.0500000000011</v>
+        <v>-319.8900000000009</v>
       </c>
       <c r="V80" t="n">
-        <v>1281</v>
+        <v>1306</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>61.14558472553699</v>
+        <v>60.80074487895717</v>
       </c>
       <c r="X80" s="7" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="Y80" s="7" t="n">
         <v>17.52</v>
@@ -9175,7 +9499,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9220,20 +9544,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/18/2026 20:05</t>
+          <t>08/19/2026 21:38</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>18895.97</v>
+        <v>19014.41</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-5.5</v>
+        <v>-4.91</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9251,16 +9575,16 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>1035</v>
+        <v>1067</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>-1104.030000000001</v>
+        <v>-1063.61</v>
       </c>
       <c r="V81" t="n">
-        <v>526</v>
+        <v>546</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>50.82125603864734</v>
+        <v>51.17150890346767</v>
       </c>
       <c r="X81" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -9275,7 +9599,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9320,20 +9644,20 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/18/2026 19:54</t>
+          <t>08/19/2026 21:32</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>19710.63</v>
+        <v>19749.75</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>-1.41</v>
+        <v>-1.21</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="L82" t="n">
         <v>20000</v>
@@ -9442,12 +9766,18 @@
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O83" s="7" t="n">
-        <v>0</v>
+        <v>20042.78</v>
       </c>
       <c r="P83" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q83" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="S83" s="7" t="n">
         <v>0</v>
       </c>
       <c r="T83" t="n">
@@ -9520,7 +9850,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/18/2026 20:54</t>
+          <t>08/19/2026 15:36</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9620,7 +9950,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/18/2026 20:02</t>
+          <t>08/19/2026 21:36</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9720,11 +10050,11 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/18/2026 20:17</t>
+          <t>08/19/2026 18:46</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20901.95</v>
+        <v>20902.55</v>
       </c>
       <c r="I86" s="7" t="n">
         <v>4.52</v>
@@ -9742,25 +10072,34 @@
         <v>0</v>
       </c>
       <c r="N86" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O86" s="7" t="n">
-        <v>0</v>
+        <v>591.4000000000001</v>
       </c>
       <c r="P86" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q86" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R86" s="7" t="n">
+        <v>5.740681362725452</v>
+      </c>
+      <c r="S86" s="7" t="n">
+        <v>0.27</v>
       </c>
       <c r="T86" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>901.95</v>
+        <v>902.5500000000001</v>
       </c>
       <c r="V86" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>49.31506849315068</v>
+        <v>50</v>
       </c>
       <c r="X86" s="7" t="n">
         <v>2.28</v>
@@ -9775,7 +10114,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9820,7 +10159,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/18/2026 19:45</t>
+          <t>08/19/2026 21:27</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9920,20 +10259,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/18/2026 20:02</t>
+          <t>08/19/2026 21:36</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20497.82</v>
+        <v>20541.66</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>2.48</v>
+        <v>2.7</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>3.4</v>
+        <v>3.62</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -9951,19 +10290,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="U88" s="7" t="n">
-        <v>497.8199999999999</v>
+        <v>541.6599999999999</v>
       </c>
       <c r="V88" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="W88" s="7" t="n">
-        <v>94.28571428571428</v>
+        <v>94.87179487179486</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>3.4</v>
+        <v>3.62</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -9975,7 +10314,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10020,20 +10359,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/18/2026 14:52</t>
+          <t>08/19/2026 21:36</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>22010.81</v>
+        <v>22753.64</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>10.08</v>
+        <v>13.8</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>1.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>2.84</v>
+        <v>3.08</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10051,19 +10390,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>2010.81</v>
+        <v>2753.64</v>
       </c>
       <c r="V89" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>81.48148148148148</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>2.84</v>
+        <v>3.08</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>1.99</v>
@@ -10075,7 +10414,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10120,20 +10459,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/18/2026 18:56</t>
+          <t>08/19/2026 21:00</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>20159.92</v>
+        <v>20008.29</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>0.8</v>
+        <v>0.04</v>
       </c>
       <c r="J90" s="7" t="n">
-        <v>0.25</v>
+        <v>0.97</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>3.98</v>
+        <v>1.03</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10142,31 +10481,40 @@
         <v>0</v>
       </c>
       <c r="N90" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="O90" s="7" t="n">
-        <v>0</v>
+        <v>20008.29</v>
       </c>
       <c r="P90" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q90" s="7" t="n">
+        <v>82.75862068965517</v>
+      </c>
+      <c r="R90" s="7" t="n">
+        <v>81.43533668341709</v>
+      </c>
+      <c r="S90" s="7" t="n">
+        <v>0.49</v>
       </c>
       <c r="T90" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>58.40999999999998</v>
+        <v>8.289999999999978</v>
       </c>
       <c r="V90" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>84</v>
+        <v>82.14285714285714</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.38</v>
+        <v>1.03</v>
       </c>
       <c r="Y90" s="7" t="n">
-        <v>0.5</v>
+        <v>0.97</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10175,12 +10523,12 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC90" t="inlineStr">
@@ -10220,7 +10568,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/18/2026 18:52</t>
+          <t>08/19/2026 20:59</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10320,7 +10668,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/18/2026 18:52</t>
+          <t>08/19/2026 20:59</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10342,13 +10690,22 @@
         <v>0</v>
       </c>
       <c r="N92" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O92" s="7" t="n">
-        <v>0</v>
+        <v>19979.06</v>
       </c>
       <c r="P92" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="Q92" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R92" s="7" t="n">
+        <v>693.995490808186</v>
+      </c>
+      <c r="S92" s="7" t="n">
+        <v>0.07000000000000001</v>
       </c>
       <c r="T92" t="n">
         <v>7</v>
@@ -10380,7 +10737,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC92" t="inlineStr">
@@ -10420,7 +10777,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/18/2026 18:52</t>
+          <t>08/19/2026 21:00</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10520,7 +10877,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/18/2026 18:52</t>
+          <t>08/19/2026 20:59</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10620,20 +10977,20 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/18/2026 18:45</t>
+          <t>08/19/2026 20:54</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
-        <v>99227.49000000001</v>
+        <v>99151.36</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>-0.77</v>
+        <v>-0.84</v>
       </c>
       <c r="J95" s="7" t="n">
-        <v>1.01</v>
+        <v>1.09</v>
       </c>
       <c r="K95" s="7" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="L95" t="n">
         <v>100000</v>
@@ -10642,31 +10999,40 @@
         <v>0</v>
       </c>
       <c r="N95" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O95" s="7" t="n">
-        <v>0</v>
+        <v>-34.16</v>
       </c>
       <c r="P95" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q95" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R95" s="7" t="n">
+        <v>0.8046437149719776</v>
+      </c>
+      <c r="S95" s="7" t="n">
+        <v>0.14</v>
       </c>
       <c r="T95" t="n">
-        <v>291</v>
+        <v>318</v>
       </c>
       <c r="U95" s="7" t="n">
-        <v>-772.5099999999999</v>
+        <v>-873.0500000000001</v>
       </c>
       <c r="V95" t="n">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="W95" s="7" t="n">
-        <v>52.23367697594502</v>
+        <v>51.25786163522012</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="Y95" s="7" t="n">
-        <v>1.01</v>
+        <v>1.09</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -10675,7 +11041,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
@@ -10720,20 +11086,20 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/18/2026 18:56</t>
+          <t>08/19/2026 20:58</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
-        <v>97936.66</v>
+        <v>97735.67999999999</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>-2.07</v>
+        <v>-2.27</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>2.77</v>
+        <v>2.99</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="L96" t="n">
         <v>100000</v>
@@ -10751,22 +11117,22 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>346</v>
+        <v>373</v>
       </c>
       <c r="U96" s="7" t="n">
-        <v>-2063.34</v>
+        <v>-2325.14</v>
       </c>
       <c r="V96" t="n">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="W96" s="7" t="n">
-        <v>52.02312138728323</v>
+        <v>51.20643431635389</v>
       </c>
       <c r="X96" s="7" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y96" s="7" t="n">
-        <v>2.78</v>
+        <v>2.99</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -10775,7 +11141,7 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr">
@@ -10820,20 +11186,20 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/18/2026 18:59</t>
+          <t>08/19/2026 21:04</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
-        <v>97652.64</v>
+        <v>97349.57000000001</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>-2.35</v>
+        <v>-2.65</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>3.59</v>
+        <v>3.87</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>0.76</v>
+        <v>0.74</v>
       </c>
       <c r="L97" t="n">
         <v>100000</v>
@@ -10851,22 +11217,22 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>346</v>
+        <v>373</v>
       </c>
       <c r="U97" s="7" t="n">
-        <v>-2347.36</v>
+        <v>-2726.91</v>
       </c>
       <c r="V97" t="n">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="W97" s="7" t="n">
-        <v>52.02312138728323</v>
+        <v>51.20643431635389</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>0.76</v>
+        <v>0.73</v>
       </c>
       <c r="Y97" s="7" t="n">
-        <v>3.58</v>
+        <v>3.87</v>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
@@ -10875,7 +11241,7 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB97" t="inlineStr">
@@ -10920,20 +11286,20 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/18/2026 18:45</t>
+          <t>08/19/2026 20:53</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
-        <v>99537.8</v>
+        <v>99491.22</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>-0.49</v>
+        <v>-0.54</v>
       </c>
       <c r="J98" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.71</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="L98" t="n">
         <v>100000</v>
@@ -10942,31 +11308,40 @@
         <v>0</v>
       </c>
       <c r="N98" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O98" s="7" t="n">
-        <v>0</v>
+        <v>-83.91000000000001</v>
       </c>
       <c r="P98" t="n">
-        <v>0</v>
+        <v>22</v>
+      </c>
+      <c r="Q98" s="7" t="n">
+        <v>55.00000000000001</v>
+      </c>
+      <c r="R98" s="7" t="n">
+        <v>0.7519070427532375</v>
+      </c>
+      <c r="S98" s="7" t="n">
+        <v>0.1</v>
       </c>
       <c r="T98" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="U98" s="7" t="n">
-        <v>-462.1999999999999</v>
+        <v>-508.78</v>
       </c>
       <c r="V98" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="W98" s="7" t="n">
-        <v>46.42857142857143</v>
+        <v>46.49122807017544</v>
       </c>
       <c r="X98" s="7" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="Y98" s="7" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Z98" t="inlineStr">
         <is>
@@ -10975,7 +11350,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
@@ -11020,7 +11395,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/18/2026 18:56</t>
+          <t>08/19/2026 21:01</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11042,13 +11417,22 @@
         <v>0</v>
       </c>
       <c r="N99" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O99" s="7" t="n">
-        <v>0</v>
+        <v>-304.44</v>
       </c>
       <c r="P99" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q99" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R99" s="7" t="n">
+        <v>0.4682177854635016</v>
+      </c>
+      <c r="S99" s="7" t="n">
+        <v>0.41</v>
       </c>
       <c r="T99" t="n">
         <v>199</v>
@@ -11120,7 +11504,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/18/2026 19:44</t>
+          <t>08/19/2026 21:27</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11338,7 +11722,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>08/15/2026 22:40</t>
+          <t>08/18/2026 23:31</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11447,20 +11831,20 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/18/2026 18:11</t>
+          <t>08/19/2026 20:36</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>27084.78</v>
+        <v>28815.73</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-29.47</v>
+        <v>-24.97</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
       </c>
       <c r="K103" s="7" t="n">
-        <v>0.78</v>
+        <v>0.83</v>
       </c>
       <c r="L103" t="n">
         <v>25000</v>
@@ -11472,34 +11856,34 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>188.87</v>
+        <v>1015.09</v>
       </c>
       <c r="P103" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>1.831769938785397</v>
+        <v>32.93111041207927</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>0.59</v>
+        <v>0.06</v>
       </c>
       <c r="T103" t="n">
-        <v>3469</v>
+        <v>3473</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-7191.75</v>
+        <v>-5466.27</v>
       </c>
       <c r="V103" t="n">
-        <v>2086</v>
+        <v>2149</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>60.13260305563563</v>
+        <v>61.87733947595738</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>0.78</v>
+        <v>0.83</v>
       </c>
       <c r="Y103" s="7" t="n">
         <v>37.71</v>
@@ -11511,7 +11895,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11556,7 +11940,7 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>08/15/2026 21:31</t>
+          <t>08/18/2026 22:24</t>
         </is>
       </c>
       <c r="H104" s="9" t="n">
@@ -11647,7 +12031,7 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>08/13/2026 20:03</t>
+          <t>08/19/2026 20:07</t>
         </is>
       </c>
       <c r="H105" s="9" t="n">
@@ -11829,7 +12213,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>08/16/2026 09:53</t>
+          <t>08/19/2026 09:55</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -11920,7 +12304,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>08/16/2026 01:46</t>
+          <t>08/19/2026 02:04</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12011,7 +12395,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>08/15/2026 22:39</t>
+          <t>08/18/2026 23:30</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12102,7 +12486,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:20</t>
+          <t>08/19/2026 21:12</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12284,7 +12668,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>08/16/2026 14:39</t>
+          <t>08/19/2026 14:40</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12375,7 +12759,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:51</t>
+          <t>08/19/2026 21:29</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12466,7 +12850,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:00</t>
+          <t>08/19/2026 21:04</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12488,17 +12872,23 @@
         <v>0</v>
       </c>
       <c r="N114" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O114" s="9" t="n">
-        <v>0</v>
+        <v>-27.2</v>
       </c>
       <c r="P114" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q114" s="8" t="n"/>
-      <c r="R114" s="8" t="n"/>
-      <c r="S114" s="8" t="n"/>
+        <v>24</v>
+      </c>
+      <c r="Q114" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="R114" s="9" t="n">
+        <v>0.9300015440835864</v>
+      </c>
+      <c r="S114" s="9" t="n">
+        <v>0.72</v>
+      </c>
       <c r="T114" s="8" t="n">
         <v>0</v>
       </c>
@@ -12551,7 +12941,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:15</t>
+          <t>08/19/2026 21:11</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12573,17 +12963,23 @@
         <v>0</v>
       </c>
       <c r="N115" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O115" s="9" t="n">
-        <v>0</v>
+        <v>-6156.77</v>
       </c>
       <c r="P115" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q115" s="8" t="n"/>
-      <c r="R115" s="8" t="n"/>
-      <c r="S115" s="8" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="Q115" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="R115" s="9" t="n">
+        <v>0.01160528233794505</v>
+      </c>
+      <c r="S115" s="9" t="n">
+        <v>31.03</v>
+      </c>
       <c r="T115" s="8" t="n">
         <v>0</v>
       </c>
@@ -12658,17 +13054,23 @@
         <v>0</v>
       </c>
       <c r="N116" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O116" s="9" t="n">
-        <v>0</v>
+        <v>3326.65</v>
       </c>
       <c r="P116" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q116" s="8" t="n"/>
-      <c r="R116" s="8" t="n"/>
-      <c r="S116" s="8" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="Q116" s="9" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="R116" s="9" t="n">
+        <v>8.896717069812709</v>
+      </c>
+      <c r="S116" s="9" t="n">
+        <v>1.04</v>
+      </c>
       <c r="T116" s="8" t="n">
         <v>0</v>
       </c>
@@ -12743,17 +13145,23 @@
         <v>0</v>
       </c>
       <c r="N117" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O117" s="9" t="n">
-        <v>0</v>
+        <v>-58.49</v>
       </c>
       <c r="P117" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q117" s="8" t="n"/>
-      <c r="R117" s="8" t="n"/>
-      <c r="S117" s="8" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="Q117" s="9" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R117" s="9" t="n">
+        <v>0.2666750250752257</v>
+      </c>
+      <c r="S117" s="9" t="n">
+        <v>0.32</v>
+      </c>
       <c r="T117" s="8" t="n">
         <v>0</v>
       </c>
@@ -12806,7 +13214,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:04</t>
+          <t>08/19/2026 21:02</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12891,7 +13299,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:06</t>
+          <t>08/19/2026 21:03</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12913,17 +13321,23 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>0</v>
+        <v>-1491.15</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q119" s="8" t="n"/>
-      <c r="R119" s="8" t="n"/>
-      <c r="S119" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q119" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R119" s="9" t="n">
+        <v>0.2217786128072648</v>
+      </c>
+      <c r="S119" s="9" t="n">
+        <v>1.64</v>
+      </c>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -12976,7 +13390,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 18:59</t>
+          <t>08/19/2026 21:00</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13061,7 +13475,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:06</t>
+          <t>08/19/2026 21:03</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13083,17 +13497,23 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>0</v>
+        <v>-3715.63</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q121" s="8" t="n"/>
-      <c r="R121" s="8" t="n"/>
-      <c r="S121" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q121" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R121" s="9" t="n">
+        <v>0.2438039067238144</v>
+      </c>
+      <c r="S121" s="9" t="n">
+        <v>3.72</v>
+      </c>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13146,7 +13566,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:14</t>
+          <t>08/19/2026 21:08</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13168,17 +13588,23 @@
         <v>0</v>
       </c>
       <c r="N122" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O122" s="9" t="n">
-        <v>0</v>
+        <v>-4944.48</v>
       </c>
       <c r="P122" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q122" s="8" t="n"/>
-      <c r="R122" s="8" t="n"/>
-      <c r="S122" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q122" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R122" s="9" t="n">
+        <v>0.2385997385250534</v>
+      </c>
+      <c r="S122" s="9" t="n">
+        <v>5.42</v>
+      </c>
       <c r="T122" s="8" t="n">
         <v>0</v>
       </c>
@@ -13231,7 +13657,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:06</t>
+          <t>08/19/2026 21:04</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13589,7 +14015,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>08/16/2026 00:18</t>
+          <t>08/19/2026 01:03</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13764,7 +14190,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>08/15/2026 21:31</t>
+          <t>08/18/2026 22:24</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -13805,7 +14231,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08/13/2026 20:03</t>
+          <t>08/19/2026 20:07</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -13887,7 +14313,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08/16/2026 09:53</t>
+          <t>08/19/2026 09:55</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -13928,7 +14354,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08/16/2026 01:46</t>
+          <t>08/19/2026 02:04</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -13969,7 +14395,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08/15/2026 22:39</t>
+          <t>08/18/2026 23:30</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14010,7 +14436,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/18/2026 19:20</t>
+          <t>08/19/2026 21:12</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14092,7 +14518,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/16/2026 14:39</t>
+          <t>08/19/2026 14:40</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14133,7 +14559,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/18/2026 19:51</t>
+          <t>08/19/2026 21:29</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14174,7 +14600,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/18/2026 19:00</t>
+          <t>08/19/2026 21:04</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14184,7 +14610,7 @@
         <v>2.91</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
@@ -14215,7 +14641,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/18/2026 19:15</t>
+          <t>08/19/2026 21:11</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14225,7 +14651,7 @@
         <v>-33.06</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -14266,7 +14692,7 @@
         <v>-5.87</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18">
@@ -14307,7 +14733,7 @@
         <v>-0.16</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -14338,7 +14764,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/18/2026 19:04</t>
+          <t>08/19/2026 21:02</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14379,7 +14805,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/18/2026 19:06</t>
+          <t>08/19/2026 21:03</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14389,7 +14815,7 @@
         <v>-5.16</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21">
@@ -14420,7 +14846,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/18/2026 18:59</t>
+          <t>08/19/2026 21:00</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14461,7 +14887,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/18/2026 19:06</t>
+          <t>08/19/2026 21:03</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14471,7 +14897,7 @@
         <v>-6.66</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -14502,7 +14928,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/18/2026 19:14</t>
+          <t>08/19/2026 21:08</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14512,7 +14938,7 @@
         <v>-20.23</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -14543,7 +14969,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/18/2026 19:06</t>
+          <t>08/19/2026 21:04</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -14707,7 +15133,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>08/16/2026 00:18</t>
+          <t>08/19/2026 01:03</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
@@ -15662,7 +16088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -15746,7 +16172,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/16/2026 10:22</t>
+          <t>08/19/2026 10:25</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -15838,7 +16264,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08/16/2026 04:55</t>
+          <t>08/19/2026 04:57</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -15884,7 +16310,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08/16/2026 05:38</t>
+          <t>08/19/2026 05:40</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -15907,7 +16333,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/16/2026 13:01</t>
+          <t>08/19/2026 13:03</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -15930,7 +16356,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08/15/2026 21:53</t>
+          <t>08/18/2026 22:45</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -15953,7 +16379,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/16/2026 15:13</t>
+          <t>08/19/2026 15:27</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -16068,7 +16494,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08/15/2026 23:08</t>
+          <t>08/19/2026 00:02</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -16114,11 +16540,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/18/2026 21:13</t>
+          <t>08/19/2026 19:23</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
-        <v>19946.87</v>
+        <v>19899.9</v>
       </c>
     </row>
     <row r="22">
@@ -16137,7 +16563,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08/15/2026 21:58</t>
+          <t>08/18/2026 22:47</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -16160,11 +16586,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/18/2026 19:20</t>
+          <t>08/19/2026 21:14</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20364.54</v>
+        <v>19977.05</v>
       </c>
     </row>
     <row r="24">
@@ -16206,11 +16632,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/18/2026 20:13</t>
+          <t>08/19/2026 21:43</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>19838.33</v>
+        <v>19722.24</v>
       </c>
     </row>
     <row r="26">
@@ -16229,11 +16655,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/18/2026 19:40</t>
+          <t>08/19/2026 21:25</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21395.6</v>
+        <v>20768.26</v>
       </c>
     </row>
     <row r="27">
@@ -16252,7 +16678,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/18/2026 16:52</t>
+          <t>08/19/2026 19:56</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16275,7 +16701,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/18/2026 16:53</t>
+          <t>08/19/2026 19:59</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16298,7 +16724,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/18/2026 17:05</t>
+          <t>08/19/2026 20:01</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16321,7 +16747,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/18/2026 16:37</t>
+          <t>08/19/2026 19:48</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16344,7 +16770,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/18/2026 16:50</t>
+          <t>08/19/2026 19:56</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16367,7 +16793,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/18/2026 16:43</t>
+          <t>08/19/2026 19:53</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16390,7 +16816,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/16/2026 14:53</t>
+          <t>08/19/2026 14:55</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -16400,150 +16826,150 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>57576</t>
+          <t>55955</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>57576 T&amp;D19L13 Meta Agg</t>
+          <t>LIVE 55955 Dream Catcher Gold</t>
         </is>
       </c>
       <c r="C34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/18/2026 18:52</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>20000</v>
+          <t>08/19/2026 21:22</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>2944.12</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>57577</t>
+          <t>55956</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>57577 T&amp;D19L13 Meta RCLOCK</t>
+          <t>LIVE 55956 Time and Day Cells</t>
         </is>
       </c>
       <c r="C35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>08/18/2026 18:56</t>
+          <t>08/19/2026 14:02</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>20000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>647831</t>
+          <t>57576</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>A MOL Argos</t>
+          <t>57576 T&amp;D19L13 Meta Agg</t>
         </is>
       </c>
       <c r="C36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>03/30/2026 11:54</t>
+          <t>08/19/2026 20:55</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>648289</t>
+          <t>57577</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">A-MOL Medallion </t>
+          <t>57577 T&amp;D19L13 Meta RCLOCK</t>
         </is>
       </c>
       <c r="C37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/18/2026 21:32</t>
+          <t>08/19/2026 20:59</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>3038308</t>
+          <t>57704</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>A-MOL inactive Maven</t>
+          <t>57704 Demo Full Throttle</t>
         </is>
       </c>
       <c r="C38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/15/2026 21:16</t>
+          <t>08/19/2026 21:17</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>52428846</t>
+          <t>57825</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EA The5ers Low DD Dual Breakout</t>
+          <t>LIVE 57825 Portfolio 30k Raven+Reaper+Aurang</t>
         </is>
       </c>
       <c r="C39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/16/2026 00:15</t>
+          <t>08/19/2026 21:21</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>41224.86</v>
+        <v>31932.56</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>80059994</t>
+          <t>647831</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>A-MOL Denali Plus</t>
+          <t>A MOL Argos</t>
         </is>
       </c>
       <c r="C40" t="b">
@@ -16551,33 +16977,125 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/18/2026 11:40</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>0.43</v>
+          <t>03/30/2026 11:54</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>648289</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A-MOL Medallion </t>
+        </is>
+      </c>
+      <c r="C41" t="b">
+        <v>0</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>08/18/2026 21:32</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>3038308</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>A-MOL inactive Maven</t>
+        </is>
+      </c>
+      <c r="C42" t="b">
+        <v>0</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>08/15/2026 21:16</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>52428846</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>EA The5ers Low DD Dual Breakout</t>
+        </is>
+      </c>
+      <c r="C43" t="b">
+        <v>1</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>08/19/2026 01:02</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>41224.86</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>80059994</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>A-MOL Denali Plus</t>
+        </is>
+      </c>
+      <c r="C44" t="b">
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>08/19/2026 11:44</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>5035285664</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Manual Trades (Rvg)</t>
         </is>
       </c>
-      <c r="C41" t="b">
+      <c r="C45" t="b">
         <v>1</v>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>07/24/2025 16:40</t>
         </is>
       </c>
-      <c r="E41" s="7" t="n">
+      <c r="E45" s="7" t="n">
         <v>5331.24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboards — 2026-08-20
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-19 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-20 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/19/2026 17:32</t>
+          <t>08/20/2026 19:37</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>49845.7</v>
+        <v>57192.47</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>127.84</v>
+        <v>161.43</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>20109.34</v>
+        <v>19802.88</v>
       </c>
       <c r="P2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>85</v>
+        <v>82.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>2.040253600528473</v>
+        <v>1.936790502136565</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>21.24</v>
+        <v>24.59</v>
       </c>
       <c r="T2" t="n">
-        <v>3338</v>
+        <v>3346</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>24845.69999999999</v>
+        <v>32192.46999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2109</v>
+        <v>2115</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.18154583582983</v>
+        <v>63.2098027495517</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/19/2026 19:43</t>
+          <t>08/20/2026 21:41</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/19/2026 20:31</t>
+          <t>08/20/2026 19:26</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/19/2026 19:49</t>
+          <t>08/20/2026 21:46</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/17/2026 14:59</t>
+          <t>08/20/2026 15:01</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/19/2026 19:34</t>
+          <t>08/20/2026 21:33</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,20 +3140,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/19/2026 21:29</t>
+          <t>08/20/2026 20:23</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>17799.77</v>
+        <v>17734.85</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>-11.03</v>
+        <v>-11.35</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>18.8</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="L22" t="n">
         <v>20000</v>
@@ -3162,34 +3162,34 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>17913.07</v>
+        <v>17848.15</v>
       </c>
       <c r="P22" t="n">
         <v>7</v>
       </c>
       <c r="Q22" s="7" t="n">
-        <v>30.43478260869566</v>
+        <v>29.16666666666667</v>
       </c>
       <c r="R22" s="7" t="n">
-        <v>3.43913023349546</v>
+        <v>3.408995324579968</v>
       </c>
       <c r="S22" s="7" t="n">
         <v>9.119999999999999</v>
       </c>
       <c r="T22" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="U22" s="7" t="n">
-        <v>-2200.23</v>
+        <v>-2265.15</v>
       </c>
       <c r="V22" t="n">
         <v>6</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>27.27272727272727</v>
+        <v>26.08695652173913</v>
       </c>
       <c r="X22" s="7" t="n">
         <v>0.7</v>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3249,14 +3249,14 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/19/2026 20:59</t>
+          <t>08/20/2026 19:53</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19867.23</v>
+        <v>19882.68</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-0.66</v>
+        <v>-0.58</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.1</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>245.92</v>
+        <v>193.89</v>
       </c>
       <c r="P23" t="n">
         <v>22</v>
@@ -3283,22 +3283,22 @@
         <v>55.00000000000001</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.11893178059137</v>
+        <v>1.093769042529525</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.21</v>
+        <v>4.22</v>
       </c>
       <c r="T23" t="n">
         <v>80</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-132.7699999999998</v>
+        <v>-117.3199999999999</v>
       </c>
       <c r="V23" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>52.5</v>
+        <v>53.75</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>0.97</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/19/2026 21:15</t>
+          <t>08/20/2026 20:09</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16615.3</v>
+        <v>16578.09</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-16.6</v>
+        <v>-16.79</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,34 +3492,34 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>41.65000000000002</v>
+        <v>-66.10999999999997</v>
       </c>
       <c r="P25" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>45</v>
+        <v>42.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.093010272443055</v>
+        <v>0.8610083256244219</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="T25" t="n">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3599.15</v>
+        <v>-3421.91</v>
       </c>
       <c r="V25" t="n">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>39.5924308588064</v>
+        <v>39.85611510791367</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>21.17</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/19/2026 20:13</t>
+          <t>08/20/2026 19:10</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/19/2026 21:06</t>
+          <t>08/20/2026 20:00</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20425.62</v>
+        <v>20262.11</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-2.33</v>
+        <v>-3.11</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>7.39</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.89</v>
+        <v>0.85</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,7 +3710,7 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-127.22</v>
+        <v>-226.24</v>
       </c>
       <c r="P27" t="n">
         <v>20</v>
@@ -3719,25 +3719,25 @@
         <v>50</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.9167457414157543</v>
+        <v>0.8609559279950342</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>3.75</v>
+        <v>3.43</v>
       </c>
       <c r="T27" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>425.62</v>
+        <v>262.1100000000001</v>
       </c>
       <c r="V27" t="n">
         <v>46</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>44.66019417475729</v>
+        <v>43.39622641509434</v>
       </c>
       <c r="X27" s="7" t="n">
-        <v>1.1</v>
+        <v>1.06</v>
       </c>
       <c r="Y27" s="7" t="n">
         <v>7.39</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/19/2026 21:08</t>
+          <t>08/20/2026 20:03</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19637.38</v>
+        <v>19701.94</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-1.83</v>
+        <v>-1.51</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,34 +3928,34 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-657.92</v>
+        <v>-469.9</v>
       </c>
       <c r="P29" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>35</v>
+        <v>37.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.240189398313893</v>
+        <v>0.3668139923462513</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>3.66</v>
+        <v>3.04</v>
       </c>
       <c r="T29" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-362.6200000000002</v>
+        <v>-298.0600000000002</v>
       </c>
       <c r="V29" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>48.36065573770492</v>
+        <v>48.78048780487805</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/19/2026 21:16</t>
+          <t>08/20/2026 20:10</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/19/2026 21:01</t>
+          <t>08/20/2026 19:56</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/19/2026 19:37</t>
+          <t>08/20/2026 21:34</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4666,14 +4666,14 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/19/2026 19:03</t>
+          <t>08/20/2026 20:59</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19915.68</v>
+        <v>19907.5</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.42</v>
+        <v>-0.46</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
@@ -4697,16 +4697,16 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-84.32000000000009</v>
+        <v>-92.50000000000009</v>
       </c>
       <c r="V36" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>49.41176470588236</v>
+        <v>49.42528735632184</v>
       </c>
       <c r="X36" s="7" t="n">
         <v>0.98</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,20 +4766,20 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/19/2026 21:41</t>
+          <t>08/20/2026 20:37</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>19807.61</v>
+        <v>19608.67</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-0.97</v>
+        <v>-1.96</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>9.82</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="L37" t="n">
         <v>20000</v>
@@ -4791,34 +4791,34 @@
         <v>40</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>-1415.82</v>
+        <v>-2116.51</v>
       </c>
       <c r="P37" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q37" s="7" t="n">
-        <v>37.5</v>
+        <v>35</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>0.6604015255091027</v>
+        <v>0.5154554445472112</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>11.16</v>
+        <v>11.44</v>
       </c>
       <c r="T37" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="U37" s="7" t="n">
-        <v>-192.3899999999998</v>
+        <v>-391.3299999999998</v>
       </c>
       <c r="V37" t="n">
         <v>22</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>41.50943396226415</v>
+        <v>40.74074074074074</v>
       </c>
       <c r="X37" s="7" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="Y37" s="7" t="n">
         <v>9.83</v>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/17/2026 17:30</t>
+          <t>08/20/2026 17:31</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/19/2026 19:03</t>
+          <t>08/20/2026 20:59</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/19/2026 21:07</t>
+          <t>08/20/2026 20:00</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/19/2026 21:27</t>
+          <t>08/20/2026 20:20</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/19/2026 21:07</t>
+          <t>08/20/2026 20:00</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5551,22 +5551,13 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-1124.46</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>0.4043290318479436</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>5.73</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5638,14 +5629,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/19/2026 21:14</t>
+          <t>08/20/2026 20:09</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19772.33</v>
+        <v>19776.9</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-1.12</v>
+        <v>-1.11</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>4.38</v>
@@ -5660,34 +5651,25 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>-4.869999999999998</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>0.9739836529729152</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-217.2</v>
+        <v>-223.1</v>
       </c>
       <c r="V45" t="n">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>55.46038543897216</v>
+        <v>55.83864118895966</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0.93</v>
@@ -5702,7 +5684,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5747,7 +5729,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/19/2026 20:54</t>
+          <t>08/20/2026 19:49</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5769,22 +5751,13 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>19977.76</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q46" s="7" t="n">
-        <v>32.43243243243244</v>
-      </c>
-      <c r="R46" s="7" t="n">
-        <v>311.8411389450754</v>
-      </c>
-      <c r="S46" s="7" t="n">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="T46" t="n">
         <v>36</v>
@@ -5816,7 +5789,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5856,20 +5829,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/19/2026 21:00</t>
+          <t>08/20/2026 19:55</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>19082.59</v>
+        <v>19153.21</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-4.57</v>
+        <v>-4.21</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5878,37 +5851,28 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>82.33999999999995</v>
+        <v>0</v>
       </c>
       <c r="P47" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q47" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R47" s="7" t="n">
-        <v>1.059591960802762</v>
-      </c>
-      <c r="S47" s="7" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-917.4100000000002</v>
+        <v>-846.7900000000002</v>
       </c>
       <c r="V47" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>40.98360655737705</v>
+        <v>41.26984126984127</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5920,7 +5884,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5965,7 +5929,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/19/2026 20:55</t>
+          <t>08/20/2026 19:49</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -5987,22 +5951,13 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>504.68</v>
+        <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q48" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="R48" s="7" t="n">
-        <v>2.47982641332395</v>
-      </c>
-      <c r="S48" s="7" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="T48" t="n">
         <v>193</v>
@@ -6074,7 +6029,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/19/2026 21:17</t>
+          <t>08/20/2026 20:12</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6096,22 +6051,13 @@
         <v>0</v>
       </c>
       <c r="N49" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>698.46</v>
+        <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q49" s="7" t="n">
-        <v>67.5</v>
-      </c>
-      <c r="R49" s="7" t="n">
-        <v>7.636199524940618</v>
-      </c>
-      <c r="S49" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T49" t="n">
         <v>410</v>
@@ -6183,7 +6129,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/19/2026 21:14</t>
+          <t>08/20/2026 20:09</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6205,22 +6151,13 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>13.93999999999999</v>
+        <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q50" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R50" s="7" t="n">
-        <v>1.066618876941458</v>
-      </c>
-      <c r="S50" s="7" t="n">
-        <v>0.89</v>
+        <v>0</v>
       </c>
       <c r="T50" t="n">
         <v>1161</v>
@@ -6292,7 +6229,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/19/2026 20:59</t>
+          <t>08/20/2026 19:53</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6314,22 +6251,13 @@
         <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>-52.41999999999999</v>
+        <v>0</v>
       </c>
       <c r="P51" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q51" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R51" s="7" t="n">
-        <v>0.8051952878219183</v>
-      </c>
-      <c r="S51" s="7" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="T51" t="n">
         <v>1978</v>
@@ -6401,7 +6329,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/19/2026 21:01</t>
+          <t>08/20/2026 19:54</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6423,22 +6351,13 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>19223.51</v>
+        <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q52" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="R52" s="7" t="n">
-        <v>6.415057985752154</v>
-      </c>
-      <c r="S52" s="7" t="n">
-        <v>5.22</v>
+        <v>0</v>
       </c>
       <c r="T52" t="n">
         <v>40</v>
@@ -6510,14 +6429,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/19/2026 21:24</t>
+          <t>08/20/2026 20:18</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19794.62</v>
+        <v>19789.51</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.05</v>
+        <v>-1.08</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6535,34 +6454,34 @@
         <v>40</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>-5.350000000000002</v>
+        <v>19.86</v>
       </c>
       <c r="P53" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q53" s="7" t="n">
-        <v>40</v>
+        <v>42.5</v>
       </c>
       <c r="R53" s="7" t="n">
-        <v>0.956813044882144</v>
+        <v>1.18964858670741</v>
       </c>
       <c r="S53" s="7" t="n">
-        <v>0.51</v>
+        <v>0.36</v>
       </c>
       <c r="T53" t="n">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-281.52</v>
+        <v>-210.49</v>
       </c>
       <c r="V53" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.9811320754717</v>
+        <v>37.63837638376384</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.7</v>
+        <v>0.78</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6574,7 +6493,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6619,7 +6538,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/19/2026 21:33</t>
+          <t>08/20/2026 20:29</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6641,22 +6560,13 @@
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>-149.77</v>
+        <v>0</v>
       </c>
       <c r="P54" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q54" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R54" s="7" t="n">
-        <v>0.4112351599968551</v>
-      </c>
-      <c r="S54" s="7" t="n">
-        <v>0.83</v>
+        <v>0</v>
       </c>
       <c r="T54" t="n">
         <v>229</v>
@@ -6728,20 +6638,20 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/19/2026 21:17</t>
+          <t>08/20/2026 20:12</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
-        <v>19605.46</v>
+        <v>19575.33</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>-1.92</v>
+        <v>-2.07</v>
       </c>
       <c r="J55" s="7" t="n">
         <v>2.83</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="L55" t="n">
         <v>20000</v>
@@ -6750,22 +6660,13 @@
         <v>0</v>
       </c>
       <c r="N55" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>-54.22</v>
+        <v>0</v>
       </c>
       <c r="P55" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q55" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="R55" s="7" t="n">
-        <v>0.506462770799199</v>
-      </c>
-      <c r="S55" s="7" t="n">
-        <v>0.27</v>
+        <v>0</v>
       </c>
       <c r="T55" t="n">
         <v>1920</v>
@@ -6837,7 +6738,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/19/2026 21:31</t>
+          <t>08/20/2026 20:27</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6859,22 +6760,13 @@
         <v>0</v>
       </c>
       <c r="N56" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O56" s="7" t="n">
-        <v>4.35</v>
+        <v>0</v>
       </c>
       <c r="P56" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q56" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R56" s="7" t="n">
-        <v>1.066564651874522</v>
-      </c>
-      <c r="S56" s="7" t="n">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="T56" t="n">
         <v>1272</v>
@@ -6946,20 +6838,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/19/2026 20:58</t>
+          <t>08/20/2026 19:52</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19750.95</v>
+        <v>19728.35</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.25</v>
+        <v>-1.37</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6968,37 +6860,28 @@
         <v>0</v>
       </c>
       <c r="N57" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>3.939999999999999</v>
+        <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q57" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R57" s="7" t="n">
-        <v>1.183000464468184</v>
-      </c>
-      <c r="S57" s="7" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>808</v>
+        <v>819</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-249.7200000000001</v>
+        <v>-271.65</v>
       </c>
       <c r="V57" t="n">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.3069306930693</v>
+        <v>44.2002442002442</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -7010,7 +6893,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -7055,7 +6938,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/19/2026 21:12</t>
+          <t>08/20/2026 20:06</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7077,22 +6960,13 @@
         <v>0</v>
       </c>
       <c r="N58" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O58" s="7" t="n">
-        <v>-83.65000000000001</v>
+        <v>0</v>
       </c>
       <c r="P58" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q58" s="7" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R58" s="7" t="n">
-        <v>0.3526042875938395</v>
-      </c>
-      <c r="S58" s="7" t="n">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="T58" t="n">
         <v>4426</v>
@@ -7164,7 +7038,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/19/2026 21:04</t>
+          <t>08/20/2026 19:59</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7186,22 +7060,13 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>-80.78999999999999</v>
+        <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q59" s="7" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="R59" s="7" t="n">
-        <v>0.32387647501883</v>
-      </c>
-      <c r="S59" s="7" t="n">
-        <v>0.43</v>
+        <v>0</v>
       </c>
       <c r="T59" t="n">
         <v>304</v>
@@ -7273,7 +7138,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/19/2026 21:08</t>
+          <t>08/20/2026 20:02</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7295,22 +7160,13 @@
         <v>0</v>
       </c>
       <c r="N60" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O60" s="7" t="n">
-        <v>326.88</v>
+        <v>0</v>
       </c>
       <c r="P60" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q60" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R60" s="7" t="n">
-        <v>6.042887997531627</v>
-      </c>
-      <c r="S60" s="7" t="n">
-        <v>0.19</v>
+        <v>0</v>
       </c>
       <c r="T60" t="n">
         <v>7019</v>
@@ -7382,7 +7238,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/19/2026 21:26</t>
+          <t>08/20/2026 20:19</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7404,22 +7260,13 @@
         <v>0</v>
       </c>
       <c r="N61" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O61" s="7" t="n">
-        <v>343.99</v>
+        <v>0</v>
       </c>
       <c r="P61" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q61" s="7" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="R61" s="7" t="n">
-        <v>5.804329608938549</v>
-      </c>
-      <c r="S61" s="7" t="n">
-        <v>0.28</v>
+        <v>0</v>
       </c>
       <c r="T61" t="n">
         <v>3982</v>
@@ -7491,7 +7338,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/19/2026 18:23</t>
+          <t>08/20/2026 20:21</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7513,22 +7360,13 @@
         <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O62" s="7" t="n">
-        <v>-353.59</v>
+        <v>0</v>
       </c>
       <c r="P62" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q62" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R62" s="7" t="n">
-        <v>0.3361931402181462</v>
-      </c>
-      <c r="S62" s="7" t="n">
-        <v>2.17</v>
+        <v>0</v>
       </c>
       <c r="T62" t="n">
         <v>170</v>
@@ -7600,14 +7438,14 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/19/2026 21:23</t>
+          <t>08/20/2026 20:16</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18748.23</v>
+        <v>18720.59</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.27</v>
+        <v>-6.41</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>7.22</v>
@@ -7622,37 +7460,28 @@
         <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>-737.4599999999999</v>
+        <v>0</v>
       </c>
       <c r="P63" t="n">
+        <v>0</v>
+      </c>
+      <c r="T63" t="n">
+        <v>43</v>
+      </c>
+      <c r="U63" s="7" t="n">
+        <v>-1279.41</v>
+      </c>
+      <c r="V63" t="n">
         <v>4</v>
       </c>
-      <c r="Q63" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="R63" s="7" t="n">
-        <v>0.5123199619092965</v>
-      </c>
-      <c r="S63" s="7" t="n">
-        <v>4.64</v>
-      </c>
-      <c r="T63" t="n">
-        <v>42</v>
-      </c>
-      <c r="U63" s="7" t="n">
-        <v>-1442.11</v>
-      </c>
-      <c r="V63" t="n">
-        <v>3</v>
-      </c>
       <c r="W63" s="7" t="n">
-        <v>7.142857142857142</v>
+        <v>9.302325581395349</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.29</v>
+        <v>0.38</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>7.21</v>
@@ -7664,7 +7493,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7709,7 +7538,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/19/2026 21:29</t>
+          <t>08/20/2026 20:24</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7731,22 +7560,13 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>-3.710000000000004</v>
+        <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q64" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R64" s="7" t="n">
-        <v>0.9861323963667626</v>
-      </c>
-      <c r="S64" s="7" t="n">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7818,20 +7638,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/19/2026 18:13</t>
+          <t>08/20/2026 20:13</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>18879.58</v>
+        <v>18913.15</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-3.62</v>
+        <v>-5.48</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>11.64</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7840,22 +7660,13 @@
         <v>0</v>
       </c>
       <c r="N65" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O65" s="7" t="n">
-        <v>88.81000000000003</v>
+        <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>25</v>
-      </c>
-      <c r="Q65" s="7" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="R65" s="7" t="n">
-        <v>1.163430926924422</v>
-      </c>
-      <c r="S65" s="7" t="n">
-        <v>2.24</v>
+        <v>0</v>
       </c>
       <c r="T65" t="n">
         <v>3298</v>
@@ -7927,7 +7738,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/19/2026 21:12</t>
+          <t>08/20/2026 20:06</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7949,22 +7760,13 @@
         <v>0</v>
       </c>
       <c r="N66" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O66" s="7" t="n">
-        <v>-116.23</v>
+        <v>0</v>
       </c>
       <c r="P66" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q66" s="7" t="n">
-        <v>40</v>
-      </c>
-      <c r="R66" s="7" t="n">
-        <v>0.317217881689479</v>
-      </c>
-      <c r="S66" s="7" t="n">
-        <v>0.66</v>
+        <v>0</v>
       </c>
       <c r="T66" t="n">
         <v>262</v>
@@ -8036,7 +7838,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/19/2026 21:41</t>
+          <t>08/20/2026 20:36</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -8058,22 +7860,13 @@
         <v>0</v>
       </c>
       <c r="N67" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O67" s="7" t="n">
-        <v>-51.36999999999998</v>
+        <v>0</v>
       </c>
       <c r="P67" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q67" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R67" s="7" t="n">
-        <v>0.9115149427267248</v>
-      </c>
-      <c r="S67" s="7" t="n">
-        <v>2.12</v>
+        <v>0</v>
       </c>
       <c r="T67" t="n">
         <v>215</v>
@@ -8145,7 +7938,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/17/2026 13:07</t>
+          <t>08/20/2026 13:09</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8167,22 +7960,13 @@
         <v>0</v>
       </c>
       <c r="N68" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O68" s="7" t="n">
-        <v>-35.83</v>
+        <v>0</v>
       </c>
       <c r="P68" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q68" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R68" s="7" t="n">
-        <v>0.5722812462695476</v>
-      </c>
-      <c r="S68" s="7" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="T68" t="n">
         <v>55</v>
@@ -8254,7 +8038,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/17/2026 13:06</t>
+          <t>08/20/2026 13:08</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8276,22 +8060,13 @@
         <v>0</v>
       </c>
       <c r="N69" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O69" s="7" t="n">
-        <v>71.06</v>
+        <v>0</v>
       </c>
       <c r="P69" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q69" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R69" s="7" t="n">
-        <v>2.289187227866473</v>
-      </c>
-      <c r="S69" s="7" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="T69" t="n">
         <v>271</v>
@@ -8363,7 +8138,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/17/2026 13:16</t>
+          <t>08/20/2026 13:17</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8385,22 +8160,13 @@
         <v>0</v>
       </c>
       <c r="N70" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O70" s="7" t="n">
-        <v>19946.4</v>
+        <v>0</v>
       </c>
       <c r="P70" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q70" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R70" s="7" t="n">
-        <v>278.6503340757238</v>
-      </c>
-      <c r="S70" s="7" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="T70" t="n">
         <v>7</v>
@@ -8432,7 +8198,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC70" t="inlineStr">
@@ -8472,7 +8238,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/19/2026 21:19</t>
+          <t>08/20/2026 20:13</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8494,22 +8260,13 @@
         <v>0</v>
       </c>
       <c r="N71" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O71" s="7" t="n">
-        <v>10.11</v>
+        <v>0</v>
       </c>
       <c r="P71" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q71" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R71" s="7" t="n">
-        <v>1.117407966554407</v>
-      </c>
-      <c r="S71" s="7" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="T71" t="n">
         <v>326</v>
@@ -8581,7 +8338,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/19/2026 18:46</t>
+          <t>08/20/2026 20:43</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8603,22 +8360,13 @@
         <v>0</v>
       </c>
       <c r="N72" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O72" s="7" t="n">
-        <v>17.22000000000001</v>
+        <v>0</v>
       </c>
       <c r="P72" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q72" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R72" s="7" t="n">
-        <v>1.101198871650211</v>
-      </c>
-      <c r="S72" s="7" t="n">
-        <v>0.49</v>
+        <v>0</v>
       </c>
       <c r="T72" t="n">
         <v>329</v>
@@ -8690,7 +8438,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/19/2026 21:22</t>
+          <t>08/20/2026 20:18</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8712,22 +8460,13 @@
         <v>0</v>
       </c>
       <c r="N73" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O73" s="7" t="n">
-        <v>28.34</v>
+        <v>0</v>
       </c>
       <c r="P73" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q73" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R73" s="7" t="n">
-        <v>1.110036886041545</v>
-      </c>
-      <c r="S73" s="7" t="n">
-        <v>0.73</v>
+        <v>0</v>
       </c>
       <c r="T73" t="n">
         <v>329</v>
@@ -8799,20 +8538,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/19/2026 21:39</t>
+          <t>08/20/2026 20:33</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20666.64</v>
+        <v>20501.6</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>3.36</v>
+        <v>2.53</v>
       </c>
       <c r="J74" s="7" t="n">
         <v>1.73</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.47</v>
+        <v>1.31</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8821,37 +8560,28 @@
         <v>0</v>
       </c>
       <c r="N74" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O74" s="7" t="n">
-        <v>140.88</v>
+        <v>0</v>
       </c>
       <c r="P74" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q74" s="7" t="n">
-        <v>57.49999999999999</v>
-      </c>
-      <c r="R74" s="7" t="n">
-        <v>1.240290641150284</v>
-      </c>
-      <c r="S74" s="7" t="n">
-        <v>1.57</v>
+        <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>669.2400000000001</v>
+        <v>501.6</v>
       </c>
       <c r="V74" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>67.02127659574468</v>
+        <v>65.30612244897959</v>
       </c>
       <c r="X74" s="7" t="n">
-        <v>1.47</v>
+        <v>1.31</v>
       </c>
       <c r="Y74" s="7" t="n">
         <v>1.73</v>
@@ -8863,7 +8593,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8908,20 +8638,20 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/19/2026 21:12</t>
+          <t>08/20/2026 20:06</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20221.62</v>
+        <v>20028.02</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>1.14</v>
+        <v>0.18</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K75" s="7" t="n">
-        <v>1.05</v>
+        <v>1.01</v>
       </c>
       <c r="L75" t="n">
         <v>20000</v>
@@ -8930,37 +8660,28 @@
         <v>0</v>
       </c>
       <c r="N75" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O75" s="7" t="n">
-        <v>248.55</v>
+        <v>0</v>
       </c>
       <c r="P75" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q75" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="R75" s="7" t="n">
-        <v>2.072214313446357</v>
-      </c>
-      <c r="S75" s="7" t="n">
-        <v>0.53</v>
+        <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>221.6200000000001</v>
+        <v>28.02000000000004</v>
       </c>
       <c r="V75" t="n">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>54.63917525773196</v>
+        <v>53.66666666666666</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>1.05</v>
+        <v>1.01</v>
       </c>
       <c r="Y75" s="7" t="n">
         <v>4.5</v>
@@ -8972,7 +8693,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -9017,14 +8738,14 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/19/2026 21:33</t>
+          <t>08/20/2026 20:27</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>20529.59</v>
+        <v>20515.87</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>2.68</v>
+        <v>2.62</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>5.69</v>
@@ -9039,37 +8760,28 @@
         <v>0</v>
       </c>
       <c r="N76" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O76" s="7" t="n">
-        <v>155.39</v>
+        <v>0</v>
       </c>
       <c r="P76" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q76" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R76" s="7" t="n">
-        <v>1.816595722318566</v>
-      </c>
-      <c r="S76" s="7" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1254</v>
+        <v>1305</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>393.67</v>
+        <v>517.1500000000001</v>
       </c>
       <c r="V76" t="n">
-        <v>728</v>
+        <v>752</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>58.0542264752791</v>
+        <v>57.62452107279693</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="Y76" s="7" t="n">
         <v>5.72</v>
@@ -9081,7 +8793,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -9126,14 +8838,14 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/19/2026 21:24</t>
+          <t>08/20/2026 20:17</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>19804.49</v>
-      </c>
-      <c r="I77" t="n">
-        <v>-1</v>
+        <v>19741.61</v>
+      </c>
+      <c r="I77" s="7" t="n">
+        <v>-1.3</v>
       </c>
       <c r="J77" s="7" t="n">
         <v>4.5</v>
@@ -9148,37 +8860,28 @@
         <v>0</v>
       </c>
       <c r="N77" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O77" s="7" t="n">
-        <v>24.35</v>
+        <v>0</v>
       </c>
       <c r="P77" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q77" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="R77" s="7" t="n">
-        <v>1.160927896371687</v>
-      </c>
-      <c r="S77" s="7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>1128</v>
+        <v>1167</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>-222.3199999999999</v>
+        <v>-284.9100000000002</v>
       </c>
       <c r="V77" t="n">
-        <v>577</v>
+        <v>593</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>51.15248226950354</v>
+        <v>50.8140531276778</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="Y77" s="7" t="n">
         <v>4.48</v>
@@ -9190,7 +8893,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -9235,20 +8938,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/19/2026 18:27</t>
+          <t>08/20/2026 20:25</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>19948.56</v>
+        <v>20295.57</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>-0.25</v>
+        <v>1.48</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>0.98</v>
+        <v>1.1</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -9257,37 +8960,28 @@
         <v>0</v>
       </c>
       <c r="N78" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O78" s="7" t="n">
-        <v>528.8599999999998</v>
+        <v>0</v>
       </c>
       <c r="P78" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q78" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R78" s="7" t="n">
-        <v>1.291633580377625</v>
-      </c>
-      <c r="S78" s="7" t="n">
-        <v>4.01</v>
+        <v>0</v>
       </c>
       <c r="T78" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="U78" s="7" t="n">
-        <v>-51.4400000000002</v>
+        <v>295.5699999999999</v>
       </c>
       <c r="V78" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="W78" s="7" t="n">
-        <v>39.75903614457831</v>
+        <v>43.82022471910113</v>
       </c>
       <c r="X78" s="7" t="n">
-        <v>0.98</v>
+        <v>1.1</v>
       </c>
       <c r="Y78" s="7" t="n">
         <v>5.5</v>
@@ -9299,7 +8993,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -9344,20 +9038,20 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/19/2026 18:27</t>
+          <t>08/20/2026 20:26</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>20315.65</v>
+        <v>20006.15</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>1.62</v>
+        <v>0.08</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>16.96</v>
       </c>
-      <c r="K79" s="7" t="n">
-        <v>1.02</v>
+      <c r="K79" t="n">
+        <v>1</v>
       </c>
       <c r="L79" t="n">
         <v>20000</v>
@@ -9375,19 +9069,19 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>806.7199999999993</v>
+        <v>6.149999999999636</v>
       </c>
       <c r="V79" t="n">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>54.39189189189189</v>
+        <v>53.44262295081968</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>1.04</v>
+        <v>1</v>
       </c>
       <c r="Y79" s="7" t="n">
         <v>17</v>
@@ -9399,7 +9093,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9444,20 +9138,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/19/2026 21:13</t>
+          <t>08/20/2026 20:06</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>20009.48</v>
+        <v>19647.03</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>0.08</v>
+        <v>-1.7</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
-      <c r="K80" t="n">
-        <v>1</v>
+      <c r="K80" s="7" t="n">
+        <v>0.99</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9475,16 +9169,16 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>2148</v>
+        <v>2228</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>-319.8900000000009</v>
+        <v>-292.9800000000014</v>
       </c>
       <c r="V80" t="n">
-        <v>1306</v>
+        <v>1349</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>60.80074487895717</v>
+        <v>60.54757630161581</v>
       </c>
       <c r="X80" s="7" t="n">
         <v>0.99</v>
@@ -9499,7 +9193,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9544,20 +9238,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/19/2026 21:38</t>
+          <t>08/20/2026 20:35</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>19014.41</v>
+        <v>18852.81</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-4.91</v>
+        <v>-5.71</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9575,16 +9269,16 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>1067</v>
+        <v>1107</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>-1063.61</v>
+        <v>-1222.06</v>
       </c>
       <c r="V81" t="n">
-        <v>546</v>
+        <v>563</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>51.17150890346767</v>
+        <v>50.85817524841914</v>
       </c>
       <c r="X81" s="7" t="n">
         <v>0.9399999999999999</v>
@@ -9599,7 +9293,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9644,20 +9338,20 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/19/2026 21:32</t>
+          <t>08/20/2026 20:25</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>19749.75</v>
+        <v>20073.33</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>-1.21</v>
+        <v>0.42</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
       </c>
       <c r="K82" s="7" t="n">
-        <v>0.92</v>
+        <v>1.02</v>
       </c>
       <c r="L82" t="n">
         <v>20000</v>
@@ -9744,20 +9438,20 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/16/2026 21:49</t>
+          <t>08/20/2026 20:42</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
-        <v>20042.78</v>
+        <v>19993.34</v>
       </c>
       <c r="I83" s="7" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="J83" t="n">
-        <v>0</v>
-      </c>
-      <c r="K83" t="n">
-        <v>0</v>
+        <v>-0.04</v>
+      </c>
+      <c r="J83" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K83" s="7" t="n">
+        <v>0.87</v>
       </c>
       <c r="L83" t="n">
         <v>20000</v>
@@ -9766,18 +9460,12 @@
         <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O83" s="7" t="n">
-        <v>20042.78</v>
+        <v>0</v>
       </c>
       <c r="P83" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q83" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="S83" s="7" t="n">
         <v>0</v>
       </c>
       <c r="T83" t="n">
@@ -9850,7 +9538,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/19/2026 15:36</t>
+          <t>08/20/2026 21:07</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9950,7 +9638,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/19/2026 21:36</t>
+          <t>08/20/2026 20:33</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -10050,20 +9738,20 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/19/2026 18:46</t>
+          <t>08/20/2026 20:43</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20902.55</v>
+        <v>20881.33</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>4.52</v>
+        <v>4.42</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>2.18</v>
       </c>
       <c r="K86" s="7" t="n">
-        <v>2.28</v>
+        <v>2.2</v>
       </c>
       <c r="L86" t="n">
         <v>20000</v>
@@ -10072,37 +9760,28 @@
         <v>0</v>
       </c>
       <c r="N86" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O86" s="7" t="n">
-        <v>591.4000000000001</v>
+        <v>0</v>
       </c>
       <c r="P86" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q86" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R86" s="7" t="n">
-        <v>5.740681362725452</v>
-      </c>
-      <c r="S86" s="7" t="n">
-        <v>0.27</v>
+        <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>902.5500000000001</v>
+        <v>881.3300000000002</v>
       </c>
       <c r="V86" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>50</v>
+        <v>50.64935064935064</v>
       </c>
       <c r="X86" s="7" t="n">
-        <v>2.28</v>
+        <v>2.2</v>
       </c>
       <c r="Y86" s="7" t="n">
         <v>2.17</v>
@@ -10114,7 +9793,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -10159,7 +9838,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/19/2026 21:27</t>
+          <t>08/20/2026 20:22</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -10259,20 +9938,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/19/2026 21:36</t>
+          <t>08/20/2026 20:31</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20541.66</v>
+        <v>20559.26</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>2.7</v>
+        <v>2.79</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>3.62</v>
+        <v>3.7</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -10290,19 +9969,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
+        <v>41</v>
+      </c>
+      <c r="U88" s="7" t="n">
+        <v>559.26</v>
+      </c>
+      <c r="V88" t="n">
         <v>39</v>
       </c>
-      <c r="U88" s="7" t="n">
-        <v>541.6599999999999</v>
-      </c>
-      <c r="V88" t="n">
-        <v>37</v>
-      </c>
       <c r="W88" s="7" t="n">
-        <v>94.87179487179486</v>
+        <v>95.1219512195122</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>3.62</v>
+        <v>3.7</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -10314,7 +9993,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10359,20 +10038,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/19/2026 21:36</t>
+          <t>08/20/2026 20:30</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>22753.64</v>
+        <v>23012.64</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>13.8</v>
+        <v>15.09</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>1.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>3.08</v>
+        <v>2.94</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10390,19 +10069,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>2753.64</v>
+        <v>3012.64</v>
       </c>
       <c r="V89" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>80.64516129032258</v>
+        <v>80</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>3.08</v>
+        <v>2.94</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>1.99</v>
@@ -10414,7 +10093,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10424,7 +10103,7 @@
       </c>
       <c r="AC89" t="inlineStr">
         <is>
-          <t>MOL XAUUSD M15 Pass16 | US30, MOL XAUUSD M15 Pass16 | USTECH, MOL XAUUSD M15 Pass16 | XAUUSD</t>
+          <t>MOL XAUUSD M15 Pass16 | US30, MOL XAUUSD M15 Pass16 | USDJPY.pro, MOL XAUUSD M15 Pass16 | USTECH, MOL XAUUSD M15 Pass16 | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10459,20 +10138,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/19/2026 21:00</t>
+          <t>08/20/2026 19:55</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
-        <v>20008.29</v>
+        <v>19852.15</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>0.04</v>
+        <v>-0.74</v>
       </c>
       <c r="J90" s="7" t="n">
-        <v>0.97</v>
+        <v>1.53</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>1.03</v>
+        <v>0.63</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10481,40 +10160,31 @@
         <v>0</v>
       </c>
       <c r="N90" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="O90" s="7" t="n">
-        <v>20008.29</v>
+        <v>0</v>
       </c>
       <c r="P90" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q90" s="7" t="n">
-        <v>82.75862068965517</v>
-      </c>
-      <c r="R90" s="7" t="n">
-        <v>81.43533668341709</v>
-      </c>
-      <c r="S90" s="7" t="n">
-        <v>0.49</v>
+        <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>8.289999999999978</v>
+        <v>-147.85</v>
       </c>
       <c r="V90" t="n">
         <v>23</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>82.14285714285714</v>
+        <v>74.19354838709677</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>1.03</v>
+        <v>0.63</v>
       </c>
       <c r="Y90" s="7" t="n">
-        <v>0.97</v>
+        <v>1.53</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10523,12 +10193,12 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC90" t="inlineStr">
@@ -10568,7 +10238,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/19/2026 20:59</t>
+          <t>08/20/2026 19:54</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10668,20 +10338,20 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/19/2026 20:59</t>
+          <t>08/20/2026 19:54</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
-        <v>19979.06</v>
+        <v>19986.77</v>
       </c>
       <c r="I92" s="7" t="n">
-        <v>-0.1</v>
+        <v>-0.06</v>
       </c>
       <c r="J92" s="7" t="n">
         <v>0.14</v>
       </c>
       <c r="K92" s="7" t="n">
-        <v>0.27</v>
+        <v>0.54</v>
       </c>
       <c r="L92" t="n">
         <v>20000</v>
@@ -10690,37 +10360,28 @@
         <v>0</v>
       </c>
       <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P92" t="n">
+        <v>0</v>
+      </c>
+      <c r="T92" t="n">
         <v>8</v>
       </c>
-      <c r="O92" s="7" t="n">
-        <v>19979.06</v>
-      </c>
-      <c r="P92" t="n">
+      <c r="U92" s="7" t="n">
+        <v>-13.23</v>
+      </c>
+      <c r="V92" t="n">
         <v>3</v>
       </c>
-      <c r="Q92" s="7" t="n">
+      <c r="W92" s="7" t="n">
         <v>37.5</v>
       </c>
-      <c r="R92" s="7" t="n">
-        <v>693.995490808186</v>
-      </c>
-      <c r="S92" s="7" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="T92" t="n">
-        <v>7</v>
-      </c>
-      <c r="U92" s="7" t="n">
-        <v>-20.94</v>
-      </c>
-      <c r="V92" t="n">
-        <v>2</v>
-      </c>
-      <c r="W92" s="7" t="n">
-        <v>28.57142857142857</v>
-      </c>
       <c r="X92" s="7" t="n">
-        <v>0.27</v>
+        <v>0.54</v>
       </c>
       <c r="Y92" s="7" t="n">
         <v>0.14</v>
@@ -10732,12 +10393,12 @@
       </c>
       <c r="AA92" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC92" t="inlineStr">
@@ -10777,20 +10438,20 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/19/2026 21:00</t>
+          <t>08/20/2026 19:54</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
-        <v>19935.43</v>
+        <v>19959.51</v>
       </c>
       <c r="I93" s="7" t="n">
-        <v>-0.32</v>
+        <v>-0.2</v>
       </c>
       <c r="J93" s="7" t="n">
         <v>0.44</v>
       </c>
       <c r="K93" s="7" t="n">
-        <v>0.28</v>
+        <v>0.55</v>
       </c>
       <c r="L93" t="n">
         <v>20000</v>
@@ -10808,19 +10469,19 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U93" s="7" t="n">
-        <v>-64.56999999999999</v>
+        <v>-40.49</v>
       </c>
       <c r="V93" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W93" s="7" t="n">
-        <v>28.57142857142857</v>
+        <v>37.5</v>
       </c>
       <c r="X93" s="7" t="n">
-        <v>0.28</v>
+        <v>0.55</v>
       </c>
       <c r="Y93" s="7" t="n">
         <v>0.45</v>
@@ -10832,7 +10493,7 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB93" t="inlineStr">
@@ -10877,20 +10538,20 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/19/2026 20:59</t>
+          <t>08/20/2026 19:52</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
-        <v>19900.96</v>
+        <v>19949.13</v>
       </c>
       <c r="I94" s="7" t="n">
-        <v>-0.5</v>
+        <v>-0.26</v>
       </c>
       <c r="J94" s="7" t="n">
         <v>0.91</v>
       </c>
       <c r="K94" s="7" t="n">
-        <v>0.46</v>
+        <v>0.72</v>
       </c>
       <c r="L94" t="n">
         <v>20000</v>
@@ -10908,19 +10569,19 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U94" s="7" t="n">
-        <v>-99.04000000000002</v>
+        <v>-50.87000000000002</v>
       </c>
       <c r="V94" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W94" s="7" t="n">
-        <v>37.5</v>
+        <v>44.44444444444444</v>
       </c>
       <c r="X94" s="7" t="n">
-        <v>0.46</v>
+        <v>0.72</v>
       </c>
       <c r="Y94" s="7" t="n">
         <v>0.91</v>
@@ -10932,7 +10593,7 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB94" t="inlineStr">
@@ -10977,20 +10638,20 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/19/2026 20:54</t>
+          <t>08/20/2026 19:51</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
-        <v>99151.36</v>
+        <v>98985.63</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>-0.84</v>
+        <v>-0.99</v>
       </c>
       <c r="J95" s="7" t="n">
-        <v>1.09</v>
+        <v>1.18</v>
       </c>
       <c r="K95" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="L95" t="n">
         <v>100000</v>
@@ -10999,40 +10660,31 @@
         <v>0</v>
       </c>
       <c r="N95" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O95" s="7" t="n">
-        <v>-34.16</v>
+        <v>0</v>
       </c>
       <c r="P95" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q95" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="R95" s="7" t="n">
-        <v>0.8046437149719776</v>
-      </c>
-      <c r="S95" s="7" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>318</v>
+        <v>371</v>
       </c>
       <c r="U95" s="7" t="n">
-        <v>-873.0500000000001</v>
+        <v>-973.74</v>
       </c>
       <c r="V95" t="n">
-        <v>163</v>
+        <v>196</v>
       </c>
       <c r="W95" s="7" t="n">
-        <v>51.25786163522012</v>
+        <v>52.83018867924528</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="Y95" s="7" t="n">
-        <v>1.09</v>
+        <v>1.15</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -11041,7 +10693,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
@@ -11051,7 +10703,7 @@
       </c>
       <c r="AC95" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Prop | AUDCAD.pro, T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURAUD.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPAUD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | GBPUSD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | US30, T&amp;D19L13 Meta4 Prop | US500, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 Prop | AUDCAD.pro, T&amp;D19L13 Meta4 Prop | AUDJPY.pro, T&amp;D19L13 Meta4 Prop | AUDNZD.pro, T&amp;D19L13 Meta4 Prop | AUDUSD.pro, T&amp;D19L13 Meta4 Prop | CADJPY.pro, T&amp;D19L13 Meta4 Prop | CHFJPY.pro, T&amp;D19L13 Meta4 Prop | EURAUD.pro, T&amp;D19L13 Meta4 Prop | EURCHF.pro, T&amp;D19L13 Meta4 Prop | EURJPY.pro, T&amp;D19L13 Meta4 Prop | EURUSD.pro, T&amp;D19L13 Meta4 Prop | GBPAUD.pro, T&amp;D19L13 Meta4 Prop | GBPCHF.pro, T&amp;D19L13 Meta4 Prop | GBPJPY.pro, T&amp;D19L13 Meta4 Prop | GBPNZD.pro, T&amp;D19L13 Meta4 Prop | GBPUSD.pro, T&amp;D19L13 Meta4 Prop | NZDUSD.pro, T&amp;D19L13 Meta4 Prop | US30, T&amp;D19L13 Meta4 Prop | US500, T&amp;D19L13 Meta4 Prop | USDCAD.pro, T&amp;D19L13 Meta4 Prop | USDCHF.pro, T&amp;D19L13 Meta4 Prop | USDJPY.pro, T&amp;D19L13 Meta4 Prop | USTECH, T&amp;D19L13 Meta4 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11086,20 +10738,20 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/19/2026 20:58</t>
+          <t>08/20/2026 19:54</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
-        <v>97735.67999999999</v>
+        <v>97207.08</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>-2.27</v>
+        <v>-2.79</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>2.99</v>
+        <v>3.35</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L96" t="n">
         <v>100000</v>
@@ -11117,22 +10769,22 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>373</v>
+        <v>426</v>
       </c>
       <c r="U96" s="7" t="n">
-        <v>-2325.14</v>
+        <v>-2695.5</v>
       </c>
       <c r="V96" t="n">
-        <v>191</v>
+        <v>224</v>
       </c>
       <c r="W96" s="7" t="n">
-        <v>51.20643431635389</v>
+        <v>52.58215962441315</v>
       </c>
       <c r="X96" s="7" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="Y96" s="7" t="n">
-        <v>2.99</v>
+        <v>3.27</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -11141,7 +10793,7 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr">
@@ -11151,7 +10803,7 @@
       </c>
       <c r="AC96" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 MOL | AUDCAD.pro, T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURAUD.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPAUD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | GBPUSD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | US30, T&amp;D19L13 Meta4 MOL | US500, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 MOL | AUDCAD.pro, T&amp;D19L13 Meta4 MOL | AUDJPY.pro, T&amp;D19L13 Meta4 MOL | AUDNZD.pro, T&amp;D19L13 Meta4 MOL | AUDUSD.pro, T&amp;D19L13 Meta4 MOL | CADJPY.pro, T&amp;D19L13 Meta4 MOL | CHFJPY.pro, T&amp;D19L13 Meta4 MOL | EURAUD.pro, T&amp;D19L13 Meta4 MOL | EURCHF.pro, T&amp;D19L13 Meta4 MOL | EURJPY.pro, T&amp;D19L13 Meta4 MOL | EURUSD.pro, T&amp;D19L13 Meta4 MOL | GBPAUD.pro, T&amp;D19L13 Meta4 MOL | GBPCHF.pro, T&amp;D19L13 Meta4 MOL | GBPJPY.pro, T&amp;D19L13 Meta4 MOL | GBPNZD.pro, T&amp;D19L13 Meta4 MOL | GBPUSD.pro, T&amp;D19L13 Meta4 MOL | NZDUSD.pro, T&amp;D19L13 Meta4 MOL | US30, T&amp;D19L13 Meta4 MOL | US500, T&amp;D19L13 Meta4 MOL | USDCAD.pro, T&amp;D19L13 Meta4 MOL | USDCHF.pro, T&amp;D19L13 Meta4 MOL | USDJPY.pro, T&amp;D19L13 Meta4 MOL | USTECH, T&amp;D19L13 Meta4 MOL | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11186,20 +10838,20 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/19/2026 21:04</t>
+          <t>08/20/2026 20:01</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
-        <v>97349.57000000001</v>
+        <v>96262.02</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>-2.65</v>
+        <v>-3.74</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>3.87</v>
+        <v>4.76</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="L97" t="n">
         <v>100000</v>
@@ -11217,22 +10869,22 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>373</v>
+        <v>426</v>
       </c>
       <c r="U97" s="7" t="n">
-        <v>-2726.91</v>
+        <v>-3616.09</v>
       </c>
       <c r="V97" t="n">
-        <v>191</v>
+        <v>224</v>
       </c>
       <c r="W97" s="7" t="n">
-        <v>51.20643431635389</v>
+        <v>52.58215962441315</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="Y97" s="7" t="n">
-        <v>3.87</v>
+        <v>4.65</v>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
@@ -11241,7 +10893,7 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB97" t="inlineStr">
@@ -11251,7 +10903,7 @@
       </c>
       <c r="AC97" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 Meta4 Agg | AUDCAD.pro, T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURAUD.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPAUD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | GBPUSD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | US30, T&amp;D19L13 Meta4 Agg | US500, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
+          <t>T&amp;D19L13 Meta4 Agg | AUDCAD.pro, T&amp;D19L13 Meta4 Agg | AUDJPY.pro, T&amp;D19L13 Meta4 Agg | AUDNZD.pro, T&amp;D19L13 Meta4 Agg | AUDUSD.pro, T&amp;D19L13 Meta4 Agg | CADJPY.pro, T&amp;D19L13 Meta4 Agg | CHFJPY.pro, T&amp;D19L13 Meta4 Agg | EURAUD.pro, T&amp;D19L13 Meta4 Agg | EURCHF.pro, T&amp;D19L13 Meta4 Agg | EURJPY.pro, T&amp;D19L13 Meta4 Agg | EURUSD.pro, T&amp;D19L13 Meta4 Agg | GBPAUD.pro, T&amp;D19L13 Meta4 Agg | GBPCHF.pro, T&amp;D19L13 Meta4 Agg | GBPJPY.pro, T&amp;D19L13 Meta4 Agg | GBPNZD.pro, T&amp;D19L13 Meta4 Agg | GBPUSD.pro, T&amp;D19L13 Meta4 Agg | NZDUSD.pro, T&amp;D19L13 Meta4 Agg | US30, T&amp;D19L13 Meta4 Agg | US500, T&amp;D19L13 Meta4 Agg | USDCAD.pro, T&amp;D19L13 Meta4 Agg | USDCHF.pro, T&amp;D19L13 Meta4 Agg | USDJPY.pro, T&amp;D19L13 Meta4 Agg | USTECH, T&amp;D19L13 Meta4 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11286,20 +10938,20 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/19/2026 20:53</t>
+          <t>08/20/2026 19:48</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
-        <v>99491.22</v>
+        <v>99589.60000000001</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>-0.54</v>
+        <v>-0.45</v>
       </c>
       <c r="J98" s="7" t="n">
         <v>0.71</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>0.68</v>
+        <v>0.75</v>
       </c>
       <c r="L98" t="n">
         <v>100000</v>
@@ -11308,37 +10960,28 @@
         <v>0</v>
       </c>
       <c r="N98" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O98" s="7" t="n">
-        <v>-83.91000000000001</v>
+        <v>0</v>
       </c>
       <c r="P98" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q98" s="7" t="n">
-        <v>55.00000000000001</v>
-      </c>
-      <c r="R98" s="7" t="n">
-        <v>0.7519070427532375</v>
-      </c>
-      <c r="S98" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="U98" s="7" t="n">
-        <v>-508.78</v>
+        <v>-410.3999999999999</v>
       </c>
       <c r="V98" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="W98" s="7" t="n">
-        <v>46.49122807017544</v>
+        <v>48</v>
       </c>
       <c r="X98" s="7" t="n">
-        <v>0.68</v>
+        <v>0.75</v>
       </c>
       <c r="Y98" s="7" t="n">
         <v>0.6899999999999999</v>
@@ -11350,7 +10993,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
@@ -11360,7 +11003,7 @@
       </c>
       <c r="AC98" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | EURUSD.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | GBPJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USDCHF.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | CHFJPY.pro, T&amp;D19L13 L10 Prop | EURUSD.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | GBPJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USDCHF.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11395,7 +11038,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/19/2026 21:01</t>
+          <t>08/20/2026 19:57</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11417,22 +11060,13 @@
         <v>0</v>
       </c>
       <c r="N99" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O99" s="7" t="n">
-        <v>-304.44</v>
+        <v>0</v>
       </c>
       <c r="P99" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q99" s="7" t="n">
-        <v>45</v>
-      </c>
-      <c r="R99" s="7" t="n">
-        <v>0.4682177854635016</v>
-      </c>
-      <c r="S99" s="7" t="n">
-        <v>0.41</v>
+        <v>0</v>
       </c>
       <c r="T99" t="n">
         <v>199</v>
@@ -11504,7 +11138,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/19/2026 21:27</t>
+          <t>08/20/2026 20:20</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11613,7 +11247,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>08/17/2026 04:05</t>
+          <t>08/20/2026 04:06</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11831,14 +11465,14 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/19/2026 20:36</t>
+          <t>08/20/2026 19:27</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>28815.73</v>
+        <v>28668.37</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-24.97</v>
+        <v>-25.36</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
@@ -11856,31 +11490,31 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>1015.09</v>
+        <v>690.4599999999999</v>
       </c>
       <c r="P103" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>90</v>
+        <v>72.5</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>32.93111041207927</v>
+        <v>4.019328319048451</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>0.06</v>
+        <v>0.64</v>
       </c>
       <c r="T103" t="n">
-        <v>3473</v>
+        <v>3491</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-5466.27</v>
+        <v>-5613.630000000002</v>
       </c>
       <c r="V103" t="n">
-        <v>2149</v>
+        <v>2151</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>61.87733947595738</v>
+        <v>61.61558292752793</v>
       </c>
       <c r="X103" s="7" t="n">
         <v>0.83</v>
@@ -11895,7 +11529,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -12486,7 +12120,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:12</t>
+          <t>08/20/2026 20:06</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12759,7 +12393,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:29</t>
+          <t>08/20/2026 20:23</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12850,20 +12484,20 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:04</t>
+          <t>08/20/2026 19:59</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
-        <v>20582.53</v>
+        <v>20592.66</v>
       </c>
       <c r="I114" s="9" t="n">
-        <v>2.91</v>
+        <v>2.96</v>
       </c>
       <c r="J114" s="9" t="n">
         <v>3.12</v>
       </c>
       <c r="K114" s="9" t="n">
-        <v>1.21</v>
+        <v>1.22</v>
       </c>
       <c r="L114" s="8" t="n">
         <v>20000</v>
@@ -12872,23 +12506,17 @@
         <v>0</v>
       </c>
       <c r="N114" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O114" s="9" t="n">
-        <v>-27.2</v>
+        <v>0</v>
       </c>
       <c r="P114" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q114" s="9" t="n">
-        <v>60</v>
-      </c>
-      <c r="R114" s="9" t="n">
-        <v>0.9300015440835864</v>
-      </c>
-      <c r="S114" s="9" t="n">
-        <v>0.72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q114" s="8" t="n"/>
+      <c r="R114" s="8" t="n"/>
+      <c r="S114" s="8" t="n"/>
       <c r="T114" s="8" t="n">
         <v>0</v>
       </c>
@@ -12941,7 +12569,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:11</t>
+          <t>08/20/2026 20:06</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12963,23 +12591,17 @@
         <v>0</v>
       </c>
       <c r="N115" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O115" s="9" t="n">
-        <v>-6156.77</v>
+        <v>0</v>
       </c>
       <c r="P115" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q115" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="R115" s="9" t="n">
-        <v>0.01160528233794505</v>
-      </c>
-      <c r="S115" s="9" t="n">
-        <v>31.03</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q115" s="8" t="n"/>
+      <c r="R115" s="8" t="n"/>
+      <c r="S115" s="8" t="n"/>
       <c r="T115" s="8" t="n">
         <v>0</v>
       </c>
@@ -13054,23 +12676,17 @@
         <v>0</v>
       </c>
       <c r="N116" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O116" s="9" t="n">
-        <v>3326.65</v>
+        <v>0</v>
       </c>
       <c r="P116" s="8" t="n">
-        <v>31</v>
-      </c>
-      <c r="Q116" s="9" t="n">
-        <v>77.5</v>
-      </c>
-      <c r="R116" s="9" t="n">
-        <v>8.896717069812709</v>
-      </c>
-      <c r="S116" s="9" t="n">
-        <v>1.04</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q116" s="8" t="n"/>
+      <c r="R116" s="8" t="n"/>
+      <c r="S116" s="8" t="n"/>
       <c r="T116" s="8" t="n">
         <v>0</v>
       </c>
@@ -13123,7 +12739,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>08/17/2026 13:10</t>
+          <t>08/20/2026 13:11</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -13145,23 +12761,17 @@
         <v>0</v>
       </c>
       <c r="N117" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O117" s="9" t="n">
-        <v>-58.49</v>
+        <v>0</v>
       </c>
       <c r="P117" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q117" s="9" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R117" s="9" t="n">
-        <v>0.2666750250752257</v>
-      </c>
-      <c r="S117" s="9" t="n">
-        <v>0.32</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q117" s="8" t="n"/>
+      <c r="R117" s="8" t="n"/>
+      <c r="S117" s="8" t="n"/>
       <c r="T117" s="8" t="n">
         <v>0</v>
       </c>
@@ -13214,7 +12824,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:02</t>
+          <t>08/20/2026 19:57</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -13299,7 +12909,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:03</t>
+          <t>08/20/2026 19:57</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13321,23 +12931,17 @@
         <v>0</v>
       </c>
       <c r="N119" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O119" s="9" t="n">
-        <v>-1491.15</v>
+        <v>0</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q119" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R119" s="9" t="n">
-        <v>0.2217786128072648</v>
-      </c>
-      <c r="S119" s="9" t="n">
-        <v>1.64</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q119" s="8" t="n"/>
+      <c r="R119" s="8" t="n"/>
+      <c r="S119" s="8" t="n"/>
       <c r="T119" s="8" t="n">
         <v>0</v>
       </c>
@@ -13390,7 +12994,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:00</t>
+          <t>08/20/2026 19:55</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13475,7 +13079,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:03</t>
+          <t>08/20/2026 19:58</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13497,23 +13101,17 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>-3715.63</v>
+        <v>0</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q121" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R121" s="9" t="n">
-        <v>0.2438039067238144</v>
-      </c>
-      <c r="S121" s="9" t="n">
-        <v>3.72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q121" s="8" t="n"/>
+      <c r="R121" s="8" t="n"/>
+      <c r="S121" s="8" t="n"/>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13566,7 +13164,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:08</t>
+          <t>08/20/2026 20:02</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13588,23 +13186,17 @@
         <v>0</v>
       </c>
       <c r="N122" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O122" s="9" t="n">
-        <v>-4944.48</v>
+        <v>0</v>
       </c>
       <c r="P122" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q122" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R122" s="9" t="n">
-        <v>0.2385997385250534</v>
-      </c>
-      <c r="S122" s="9" t="n">
-        <v>5.42</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q122" s="8" t="n"/>
+      <c r="R122" s="8" t="n"/>
+      <c r="S122" s="8" t="n"/>
       <c r="T122" s="8" t="n">
         <v>0</v>
       </c>
@@ -13657,7 +13249,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 21:04</t>
+          <t>08/20/2026 19:59</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -14436,7 +14028,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/19/2026 21:12</t>
+          <t>08/20/2026 20:06</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14559,7 +14151,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/19/2026 21:29</t>
+          <t>08/20/2026 20:23</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14600,17 +14192,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/19/2026 21:04</t>
+          <t>08/20/2026 19:59</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>20582.53</v>
+        <v>20592.66</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>2.91</v>
+        <v>2.96</v>
       </c>
       <c r="I15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -14641,7 +14233,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/19/2026 21:11</t>
+          <t>08/20/2026 20:06</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14651,7 +14243,7 @@
         <v>-33.06</v>
       </c>
       <c r="I16" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -14692,7 +14284,7 @@
         <v>-5.87</v>
       </c>
       <c r="I17" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -14723,7 +14315,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/17/2026 13:10</t>
+          <t>08/20/2026 13:11</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14733,7 +14325,7 @@
         <v>-0.16</v>
       </c>
       <c r="I18" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -14764,7 +14356,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/19/2026 21:02</t>
+          <t>08/20/2026 19:57</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14805,7 +14397,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/19/2026 21:03</t>
+          <t>08/20/2026 19:57</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14815,7 +14407,7 @@
         <v>-5.16</v>
       </c>
       <c r="I20" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -14846,7 +14438,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/19/2026 21:00</t>
+          <t>08/20/2026 19:55</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14887,7 +14479,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/19/2026 21:03</t>
+          <t>08/20/2026 19:58</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14897,7 +14489,7 @@
         <v>-6.66</v>
       </c>
       <c r="I22" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -14928,7 +14520,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/19/2026 21:08</t>
+          <t>08/20/2026 20:02</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14938,7 +14530,7 @@
         <v>-20.23</v>
       </c>
       <c r="I23" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -14969,7 +14561,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/19/2026 21:04</t>
+          <t>08/20/2026 19:59</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -16088,7 +15680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -16241,7 +15833,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/17/2026 07:54</t>
+          <t>08/20/2026 07:56</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -16448,7 +16040,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/17/2026 09:02</t>
+          <t>08/20/2026 09:06</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -16471,7 +16063,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/17/2026 07:41</t>
+          <t>08/20/2026 07:42</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -16540,7 +16132,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/19/2026 19:23</t>
+          <t>08/20/2026 21:19</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16586,11 +16178,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/19/2026 21:14</t>
+          <t>08/20/2026 20:07</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>19977.05</v>
+        <v>20106.35</v>
       </c>
     </row>
     <row r="24">
@@ -16632,7 +16224,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/19/2026 21:43</t>
+          <t>08/20/2026 20:37</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -16655,7 +16247,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/19/2026 21:25</t>
+          <t>08/20/2026 20:18</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -16678,7 +16270,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/19/2026 19:56</t>
+          <t>08/20/2026 18:55</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16701,7 +16293,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/19/2026 19:59</t>
+          <t>08/20/2026 18:57</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16724,7 +16316,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/19/2026 20:01</t>
+          <t>08/20/2026 18:59</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16747,7 +16339,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/19/2026 19:48</t>
+          <t>08/20/2026 21:46</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16770,7 +16362,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/19/2026 19:56</t>
+          <t>08/20/2026 15:57</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16793,7 +16385,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/19/2026 19:53</t>
+          <t>08/20/2026 18:52</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16839,7 +16431,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/19/2026 21:22</t>
+          <t>08/20/2026 20:17</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
@@ -16885,7 +16477,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/19/2026 20:55</t>
+          <t>08/20/2026 19:50</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -16908,7 +16500,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/19/2026 20:59</t>
+          <t>08/20/2026 19:54</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -16918,12 +16510,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>57704</t>
+          <t>57699</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>57704 Demo Full Throttle</t>
+          <t>57699 Demo Gold Snap</t>
         </is>
       </c>
       <c r="C38" t="b">
@@ -16931,7 +16523,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/19/2026 21:17</t>
+          <t>08/20/2026 20:59</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -16941,35 +16533,35 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>57825</t>
+          <t>57704</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>LIVE 57825 Portfolio 30k Raven+Reaper+Aurang</t>
+          <t>57704 Demo Full Throttle</t>
         </is>
       </c>
       <c r="C39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/19/2026 21:21</t>
+          <t>08/20/2026 20:10</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>31932.56</v>
+        <v>19985.75</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>647831</t>
+          <t>57825</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>A MOL Argos</t>
+          <t>LIVE 57825 Portfolio 30k Raven+Reaper+Aurang</t>
         </is>
       </c>
       <c r="C40" t="b">
@@ -16977,22 +16569,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>03/30/2026 11:54</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>0</v>
+          <t>08/20/2026 20:15</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>31954.16</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>648289</t>
+          <t>647831</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">A-MOL Medallion </t>
+          <t>A MOL Argos</t>
         </is>
       </c>
       <c r="C41" t="b">
@@ -17000,7 +16592,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>08/18/2026 21:32</t>
+          <t>03/30/2026 11:54</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -17010,12 +16602,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>3038308</t>
+          <t>648289</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>A-MOL inactive Maven</t>
+          <t xml:space="preserve">A-MOL Medallion </t>
         </is>
       </c>
       <c r="C42" t="b">
@@ -17023,7 +16615,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>08/15/2026 21:16</t>
+          <t>08/18/2026 21:32</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -17033,69 +16625,92 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>52428846</t>
+          <t>3038308</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EA The5ers Low DD Dual Breakout</t>
+          <t>A-MOL inactive Maven</t>
         </is>
       </c>
       <c r="C43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>08/19/2026 01:02</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="n">
-        <v>41224.86</v>
+          <t>08/15/2026 21:16</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>80059994</t>
+          <t>52428846</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>A-MOL Denali Plus</t>
+          <t>EA The5ers Low DD Dual Breakout</t>
         </is>
       </c>
       <c r="C44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>08/19/2026 11:44</t>
+          <t>08/19/2026 01:02</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>0.43</v>
+        <v>41224.86</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>80059994</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>A-MOL Denali Plus</t>
+        </is>
+      </c>
+      <c r="C45" t="b">
+        <v>0</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>08/20/2026 11:46</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>5035285664</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Manual Trades (Rvg)</t>
         </is>
       </c>
-      <c r="C45" t="b">
+      <c r="C46" t="b">
         <v>1</v>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>07/24/2025 16:40</t>
         </is>
       </c>
-      <c r="E45" s="7" t="n">
+      <c r="E46" s="7" t="n">
         <v>5331.24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboards — 2026-08-21
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-20 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-21 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/20/2026 19:37</t>
+          <t>08/21/2026 09:50</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>57192.47</v>
+        <v>52448.1</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>161.43</v>
+        <v>139.75</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.09</v>
+        <v>1.08</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>19802.88</v>
+        <v>12719.53</v>
       </c>
       <c r="P2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>82.5</v>
+        <v>80</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.936790502136565</v>
+        <v>1.475681386408174</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>24.59</v>
+        <v>25.81</v>
       </c>
       <c r="T2" t="n">
-        <v>3346</v>
+        <v>3350</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>32192.46999999999</v>
+        <v>31156.28999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2115</v>
+        <v>2119</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.2098027495517</v>
+        <v>63.25373134328358</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.07</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/20/2026 21:41</t>
+          <t>08/21/2026 08:57</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/20/2026 19:26</t>
+          <t>08/21/2026 09:41</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/18/2026 10:06</t>
+          <t>08/21/2026 10:09</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/20/2026 21:46</t>
+          <t>08/21/2026 09:01</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>08/18/2026 12:38</t>
+          <t>08/21/2026 13:01</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>08/18/2026 05:45</t>
+          <t>08/21/2026 05:47</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>08/18/2026 05:43</t>
+          <t>08/21/2026 05:45</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/20/2026 21:33</t>
+          <t>08/21/2026 08:47</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/20/2026 20:23</t>
+          <t>08/21/2026 11:38</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/20/2026 19:53</t>
+          <t>08/21/2026 10:14</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/20/2026 20:09</t>
+          <t>08/21/2026 11:01</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16578.09</v>
+        <v>16597.1</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-16.79</v>
+        <v>-16.69</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,34 +3492,34 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>-66.10999999999997</v>
+        <v>64.88000000000002</v>
       </c>
       <c r="P25" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>42.5</v>
+        <v>47.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>0.8610083256244219</v>
+        <v>1.157151507811554</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>1.35</v>
+        <v>0.84</v>
       </c>
       <c r="T25" t="n">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>-3421.91</v>
+        <v>-3411.74</v>
       </c>
       <c r="V25" t="n">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>39.85611510791367</v>
+        <v>39.97155049786629</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y25" s="7" t="n">
         <v>21.17</v>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/20/2026 19:10</t>
+          <t>08/21/2026 09:24</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/20/2026 20:00</t>
+          <t>08/21/2026 10:30</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20262.11</v>
+        <v>20173.69</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-3.11</v>
+        <v>-3.53</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>7.39</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,7 +3710,7 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-226.24</v>
+        <v>-260.4399999999999</v>
       </c>
       <c r="P27" t="n">
         <v>20</v>
@@ -3719,28 +3719,28 @@
         <v>50</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.8609559279950342</v>
+        <v>0.8425697567580638</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>3.43</v>
+        <v>3.22</v>
       </c>
       <c r="T27" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="U27" s="7" t="n">
-        <v>262.1100000000001</v>
+        <v>-200.05</v>
       </c>
       <c r="V27" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="W27" s="7" t="n">
-        <v>43.39622641509434</v>
+        <v>42.72727272727273</v>
       </c>
       <c r="X27" s="7" t="n">
-        <v>1.06</v>
+        <v>0.96</v>
       </c>
       <c r="Y27" s="7" t="n">
-        <v>7.39</v>
+        <v>7.4</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/20/2026 20:03</t>
+          <t>08/21/2026 10:35</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19701.94</v>
+        <v>19541.42</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-1.51</v>
+        <v>-2.31</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,7 +3928,7 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-469.9</v>
+        <v>-624.87</v>
       </c>
       <c r="P29" t="n">
         <v>15</v>
@@ -3937,16 +3937,16 @@
         <v>37.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.3668139923462513</v>
+        <v>0.3034478146005418</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>3.04</v>
+        <v>3.14</v>
       </c>
       <c r="T29" t="n">
         <v>123</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-298.0600000000002</v>
+        <v>-458.5800000000003</v>
       </c>
       <c r="V29" t="n">
         <v>60</v>
@@ -3955,7 +3955,7 @@
         <v>48.78048780487805</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/20/2026 20:10</t>
+          <t>08/21/2026 11:03</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/20/2026 19:56</t>
+          <t>08/21/2026 10:20</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>08/18/2026 11:04</t>
+          <t>08/21/2026 11:09</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/20/2026 21:34</t>
+          <t>08/21/2026 08:49</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4488,7 +4488,7 @@
         <v>2.66</v>
       </c>
       <c r="T34" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="U34" s="7" t="n">
         <v>40.77000000000005</v>
@@ -4497,7 +4497,7 @@
         <v>44</v>
       </c>
       <c r="W34" s="7" t="n">
-        <v>41.1214953271028</v>
+        <v>40.74074074074074</v>
       </c>
       <c r="X34" s="7" t="n">
         <v>1.02</v>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/18/2026 00:14</t>
+          <t>08/21/2026 00:15</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/20/2026 20:59</t>
+          <t>08/21/2026 08:19</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-92.50000000000009</v>
+        <v>0.3999999999998636</v>
       </c>
       <c r="V36" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>49.42528735632184</v>
+        <v>50</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.83</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/20/2026 20:37</t>
+          <t>08/21/2026 07:57</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/20/2026 20:59</t>
+          <t>08/21/2026 08:18</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/20/2026 20:00</t>
+          <t>08/21/2026 10:32</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/20/2026 20:20</t>
+          <t>08/21/2026 11:32</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,22 +5442,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>-50.87</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>0.2037877602128658</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
         <v>4278</v>
@@ -5529,7 +5520,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/20/2026 20:00</t>
+          <t>08/21/2026 10:29</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5629,7 +5620,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/20/2026 20:09</t>
+          <t>08/21/2026 11:03</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5729,7 +5720,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/20/2026 19:49</t>
+          <t>08/21/2026 10:09</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5829,20 +5820,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/20/2026 19:55</t>
+          <t>08/21/2026 10:18</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>19153.21</v>
+        <v>19058.66</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-4.21</v>
+        <v>-4.69</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5863,7 +5854,7 @@
         <v>63</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-846.7900000000002</v>
+        <v>-941.3400000000001</v>
       </c>
       <c r="V47" t="n">
         <v>26</v>
@@ -5872,7 +5863,7 @@
         <v>41.26984126984127</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5884,7 +5875,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5929,7 +5920,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/20/2026 19:49</t>
+          <t>08/21/2026 10:07</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6029,7 +6020,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/20/2026 20:12</t>
+          <t>08/21/2026 11:05</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6129,7 +6120,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/20/2026 20:09</t>
+          <t>08/21/2026 11:00</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6229,7 +6220,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/20/2026 19:53</t>
+          <t>08/21/2026 10:17</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6329,7 +6320,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/20/2026 19:54</t>
+          <t>08/21/2026 10:15</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6429,14 +6420,14 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/20/2026 20:18</t>
+          <t>08/21/2026 11:28</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19789.51</v>
+        <v>19784.06</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.08</v>
+        <v>-1.11</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
@@ -6451,37 +6442,28 @@
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>19.86</v>
+        <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q53" s="7" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R53" s="7" t="n">
-        <v>1.18964858670741</v>
-      </c>
-      <c r="S53" s="7" t="n">
-        <v>0.36</v>
+        <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-210.49</v>
+        <v>-218.54</v>
       </c>
       <c r="V53" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>37.63837638376384</v>
+        <v>37.18411552346571</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6493,7 +6475,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6538,7 +6520,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/20/2026 20:29</t>
+          <t>08/21/2026 11:59</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6638,7 +6620,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/20/2026 20:12</t>
+          <t>08/21/2026 11:04</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6738,7 +6720,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/20/2026 20:27</t>
+          <t>08/21/2026 11:51</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6838,14 +6820,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/20/2026 19:52</t>
+          <t>08/21/2026 10:15</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19728.35</v>
+        <v>19724.15</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.37</v>
+        <v>-1.39</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6869,19 +6851,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>819</v>
+        <v>835</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-271.65</v>
+        <v>-280.2200000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.2002442002442</v>
+        <v>43.83233532934131</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6893,7 +6875,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6938,7 +6920,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/20/2026 20:06</t>
+          <t>08/21/2026 10:55</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7038,7 +7020,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/20/2026 19:59</t>
+          <t>08/21/2026 10:27</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7138,20 +7120,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/20/2026 20:02</t>
+          <t>08/21/2026 10:34</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>20418.34</v>
+        <v>20199.39</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-4.01</v>
+        <v>-5.04</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="L60" s="7" t="n">
         <v>21100.65</v>
@@ -7238,20 +7220,20 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/20/2026 20:19</t>
+          <t>08/21/2026 11:28</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
-        <v>20926.01</v>
+        <v>20707.06</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>-2.32</v>
+        <v>-3.34</v>
       </c>
       <c r="J61" s="7" t="n">
         <v>13.96</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="L61" s="7" t="n">
         <v>21292.1</v>
@@ -7338,7 +7320,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/20/2026 20:21</t>
+          <t>08/21/2026 11:32</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7438,7 +7420,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/20/2026 20:16</t>
+          <t>08/21/2026 11:23</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7469,7 +7451,7 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="U63" s="7" t="n">
         <v>-1279.41</v>
@@ -7478,7 +7460,7 @@
         <v>4</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>9.302325581395349</v>
+        <v>9.090909090909092</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>0.38</v>
@@ -7493,7 +7475,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7538,7 +7520,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/20/2026 20:24</t>
+          <t>08/21/2026 11:41</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7638,7 +7620,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/20/2026 20:13</t>
+          <t>08/21/2026 07:35</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7738,7 +7720,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/20/2026 20:06</t>
+          <t>08/21/2026 10:57</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7838,7 +7820,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/20/2026 20:36</t>
+          <t>08/21/2026 07:57</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -8238,7 +8220,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/20/2026 20:13</t>
+          <t>08/21/2026 11:11</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8338,7 +8320,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/20/2026 20:43</t>
+          <t>08/21/2026 08:03</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8438,7 +8420,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/20/2026 20:18</t>
+          <t>08/21/2026 11:24</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8538,20 +8520,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/20/2026 20:33</t>
+          <t>08/21/2026 07:55</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20501.6</v>
+        <v>20328.13</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>2.53</v>
+        <v>1.66</v>
       </c>
       <c r="J74" s="7" t="n">
-        <v>1.73</v>
+        <v>1.78</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.31</v>
+        <v>1.18</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8569,22 +8551,22 @@
         <v>0</v>
       </c>
       <c r="T74" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="U74" s="7" t="n">
-        <v>501.6</v>
+        <v>324.21</v>
       </c>
       <c r="V74" t="n">
         <v>64</v>
       </c>
       <c r="W74" s="7" t="n">
-        <v>65.30612244897959</v>
+        <v>63.36633663366337</v>
       </c>
       <c r="X74" s="7" t="n">
-        <v>1.31</v>
+        <v>1.18</v>
       </c>
       <c r="Y74" s="7" t="n">
-        <v>1.73</v>
+        <v>1.82</v>
       </c>
       <c r="Z74" t="inlineStr">
         <is>
@@ -8593,7 +8575,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8638,20 +8620,20 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/20/2026 20:06</t>
+          <t>08/21/2026 07:28</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>20028.02</v>
+        <v>19941.62</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>0.18</v>
+        <v>-0.25</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K75" s="7" t="n">
-        <v>1.01</v>
+        <v>0.99</v>
       </c>
       <c r="L75" t="n">
         <v>20000</v>
@@ -8669,19 +8651,19 @@
         <v>0</v>
       </c>
       <c r="T75" t="n">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="U75" s="7" t="n">
-        <v>28.02000000000004</v>
+        <v>-74.06999999999991</v>
       </c>
       <c r="V75" t="n">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="W75" s="7" t="n">
-        <v>53.66666666666666</v>
+        <v>53.35463258785943</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>1.01</v>
+        <v>0.98</v>
       </c>
       <c r="Y75" s="7" t="n">
         <v>4.5</v>
@@ -8693,7 +8675,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8738,20 +8720,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/20/2026 20:27</t>
+          <t>08/21/2026 11:57</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>20515.87</v>
+        <v>20899.24</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>2.62</v>
+        <v>4.55</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>5.69</v>
       </c>
       <c r="K76" s="7" t="n">
-        <v>1.08</v>
+        <v>1.13</v>
       </c>
       <c r="L76" t="n">
         <v>20000</v>
@@ -8769,19 +8751,19 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1305</v>
+        <v>1343</v>
       </c>
       <c r="U76" s="7" t="n">
-        <v>517.1500000000001</v>
+        <v>982.8800000000001</v>
       </c>
       <c r="V76" t="n">
-        <v>752</v>
+        <v>787</v>
       </c>
       <c r="W76" s="7" t="n">
-        <v>57.62452107279693</v>
+        <v>58.60014892032762</v>
       </c>
       <c r="X76" s="7" t="n">
-        <v>1.08</v>
+        <v>1.15</v>
       </c>
       <c r="Y76" s="7" t="n">
         <v>5.72</v>
@@ -8793,7 +8775,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8838,20 +8820,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/20/2026 20:17</t>
+          <t>08/21/2026 11:22</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>19741.61</v>
+        <v>19620.27</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>-1.3</v>
+        <v>-1.91</v>
       </c>
       <c r="J77" s="7" t="n">
-        <v>4.5</v>
+        <v>4.69</v>
       </c>
       <c r="K77" s="7" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8869,22 +8851,22 @@
         <v>0</v>
       </c>
       <c r="T77" t="n">
-        <v>1167</v>
+        <v>1216</v>
       </c>
       <c r="U77" s="7" t="n">
-        <v>-284.9100000000002</v>
+        <v>-464.0500000000001</v>
       </c>
       <c r="V77" t="n">
-        <v>593</v>
+        <v>619</v>
       </c>
       <c r="W77" s="7" t="n">
-        <v>50.8140531276778</v>
+        <v>50.9046052631579</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y77" s="7" t="n">
-        <v>4.48</v>
+        <v>5.06</v>
       </c>
       <c r="Z77" t="inlineStr">
         <is>
@@ -8893,7 +8875,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8938,20 +8920,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/20/2026 20:25</t>
+          <t>08/21/2026 11:55</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>20295.57</v>
+        <v>20268.7</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>1.48</v>
+        <v>1.34</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>1.1</v>
+        <v>1.08</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -8969,19 +8951,19 @@
         <v>0</v>
       </c>
       <c r="T78" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="U78" s="7" t="n">
-        <v>295.5699999999999</v>
+        <v>275.7599999999999</v>
       </c>
       <c r="V78" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="W78" s="7" t="n">
-        <v>43.82022471910113</v>
+        <v>45.74468085106383</v>
       </c>
       <c r="X78" s="7" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="Y78" s="7" t="n">
         <v>5.5</v>
@@ -8993,7 +8975,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -9038,20 +9020,20 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/20/2026 20:26</t>
+          <t>08/21/2026 11:46</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>20006.15</v>
+        <v>19294.83</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>0.08</v>
+        <v>-3.49</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>16.96</v>
       </c>
-      <c r="K79" t="n">
-        <v>1</v>
+      <c r="K79" s="7" t="n">
+        <v>0.97</v>
       </c>
       <c r="L79" t="n">
         <v>20000</v>
@@ -9069,19 +9051,19 @@
         <v>0</v>
       </c>
       <c r="T79" t="n">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="U79" s="7" t="n">
-        <v>6.149999999999636</v>
+        <v>-420.4200000000003</v>
       </c>
       <c r="V79" t="n">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="W79" s="7" t="n">
-        <v>53.44262295081968</v>
+        <v>53.14465408805032</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Y79" s="7" t="n">
         <v>17</v>
@@ -9093,7 +9075,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -9138,20 +9120,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/20/2026 20:06</t>
+          <t>08/21/2026 10:55</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>19647.03</v>
+        <v>21265.6</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>-1.7</v>
+        <v>6.37</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>0.99</v>
+        <v>1.04</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9169,19 +9151,19 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>2228</v>
+        <v>2303</v>
       </c>
       <c r="U80" s="7" t="n">
-        <v>-292.9800000000014</v>
+        <v>1660.71</v>
       </c>
       <c r="V80" t="n">
-        <v>1349</v>
+        <v>1408</v>
       </c>
       <c r="W80" s="7" t="n">
-        <v>60.54757630161581</v>
+        <v>61.13764654798089</v>
       </c>
       <c r="X80" s="7" t="n">
-        <v>0.99</v>
+        <v>1.05</v>
       </c>
       <c r="Y80" s="7" t="n">
         <v>17.52</v>
@@ -9193,7 +9175,7 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
@@ -9238,20 +9220,20 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/20/2026 20:35</t>
+          <t>08/21/2026 07:55</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>18852.81</v>
+        <v>18521.65</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-5.71</v>
+        <v>-7.37</v>
       </c>
       <c r="J81" s="7" t="n">
         <v>12.36</v>
       </c>
       <c r="K81" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="L81" t="n">
         <v>20000</v>
@@ -9269,22 +9251,22 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>1107</v>
+        <v>1156</v>
       </c>
       <c r="U81" s="7" t="n">
-        <v>-1222.06</v>
+        <v>-1647.77</v>
       </c>
       <c r="V81" t="n">
-        <v>563</v>
+        <v>589</v>
       </c>
       <c r="W81" s="7" t="n">
-        <v>50.85817524841914</v>
+        <v>50.95155709342561</v>
       </c>
       <c r="X81" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="Y81" s="7" t="n">
-        <v>12.38</v>
+        <v>12.62</v>
       </c>
       <c r="Z81" t="inlineStr">
         <is>
@@ -9293,7 +9275,7 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
@@ -9338,14 +9320,14 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/20/2026 20:25</t>
+          <t>08/21/2026 11:49</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>20073.33</v>
+        <v>20048.59</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>0.42</v>
+        <v>0.29</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
@@ -9438,7 +9420,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/20/2026 20:42</t>
+          <t>08/21/2026 08:03</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9538,7 +9520,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/20/2026 21:07</t>
+          <t>08/21/2026 08:26</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9638,7 +9620,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/20/2026 20:33</t>
+          <t>08/21/2026 07:55</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9738,7 +9720,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/20/2026 20:43</t>
+          <t>08/21/2026 08:03</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
@@ -9769,19 +9751,19 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>881.3300000000002</v>
+        <v>877.8300000000002</v>
       </c>
       <c r="V86" t="n">
         <v>39</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>50.64935064935064</v>
+        <v>50</v>
       </c>
       <c r="X86" s="7" t="n">
-        <v>2.2</v>
+        <v>2.19</v>
       </c>
       <c r="Y86" s="7" t="n">
         <v>2.17</v>
@@ -9793,7 +9775,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9838,7 +9820,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/20/2026 20:22</t>
+          <t>08/21/2026 11:32</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9938,7 +9920,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/20/2026 20:31</t>
+          <t>08/21/2026 07:52</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
@@ -9969,19 +9951,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="U88" s="7" t="n">
-        <v>559.26</v>
+        <v>576.16</v>
       </c>
       <c r="V88" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W88" s="7" t="n">
-        <v>95.1219512195122</v>
+        <v>95.23809523809523</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>3.7</v>
+        <v>3.78</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -9993,7 +9975,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10038,20 +10020,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/20/2026 20:30</t>
+          <t>08/21/2026 07:53</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>23012.64</v>
+        <v>22762.4</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>15.09</v>
+        <v>13.84</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>1.99</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>2.94</v>
+        <v>2.53</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10069,22 +10051,22 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>3012.64</v>
+        <v>2515.89</v>
       </c>
       <c r="V89" t="n">
         <v>28</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>80</v>
+        <v>75.67567567567568</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>2.94</v>
+        <v>2.23</v>
       </c>
       <c r="Y89" s="7" t="n">
-        <v>1.99</v>
+        <v>2.9</v>
       </c>
       <c r="Z89" t="inlineStr">
         <is>
@@ -10093,7 +10075,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10138,7 +10120,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/20/2026 19:55</t>
+          <t>08/21/2026 10:19</t>
         </is>
       </c>
       <c r="H90" s="7" t="n">
@@ -10169,22 +10151,22 @@
         <v>0</v>
       </c>
       <c r="T90" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="U90" s="7" t="n">
-        <v>-147.85</v>
+        <v>-254.0000000000001</v>
       </c>
       <c r="V90" t="n">
         <v>23</v>
       </c>
       <c r="W90" s="7" t="n">
-        <v>74.19354838709677</v>
+        <v>71.875</v>
       </c>
       <c r="X90" s="7" t="n">
-        <v>0.63</v>
+        <v>0.5</v>
       </c>
       <c r="Y90" s="7" t="n">
-        <v>1.53</v>
+        <v>2.05</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10193,7 +10175,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -10238,7 +10220,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/20/2026 19:54</t>
+          <t>08/21/2026 10:17</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10338,11 +10320,11 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/20/2026 19:54</t>
+          <t>08/21/2026 10:18</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
-        <v>19986.77</v>
+        <v>19987.07</v>
       </c>
       <c r="I92" s="7" t="n">
         <v>-0.06</v>
@@ -10351,7 +10333,7 @@
         <v>0.14</v>
       </c>
       <c r="K92" s="7" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="L92" t="n">
         <v>20000</v>
@@ -10369,19 +10351,19 @@
         <v>0</v>
       </c>
       <c r="T92" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U92" s="7" t="n">
-        <v>-13.23</v>
+        <v>-13.13</v>
       </c>
       <c r="V92" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W92" s="7" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
       <c r="X92" s="7" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="Y92" s="7" t="n">
         <v>0.14</v>
@@ -10393,7 +10375,7 @@
       </c>
       <c r="AA92" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB92" t="inlineStr">
@@ -10403,7 +10385,7 @@
       </c>
       <c r="AC92" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Prop | AUDJPY.pro, T&amp;D19L13 L11 Prop | AUDUSD.pro, T&amp;D19L13 L11 Prop | EURUSD.pro, T&amp;D19L13 L11 Prop | GBPAUD.pro, T&amp;D19L13 L11 Prop | GBPCHF.pro</t>
+          <t>T&amp;D19L13 L11 Prop | AUDJPY.pro, T&amp;D19L13 L11 Prop | AUDUSD.pro, T&amp;D19L13 L11 Prop | EURUSD.pro, T&amp;D19L13 L11 Prop | GBPAUD.pro, T&amp;D19L13 L11 Prop | GBPCHF.pro, T&amp;D19L13 L11 Prop | GBPUSD.pro</t>
         </is>
       </c>
     </row>
@@ -10438,11 +10420,11 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/20/2026 19:54</t>
+          <t>08/21/2026 10:15</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
-        <v>19959.51</v>
+        <v>19960.45</v>
       </c>
       <c r="I93" s="7" t="n">
         <v>-0.2</v>
@@ -10451,7 +10433,7 @@
         <v>0.44</v>
       </c>
       <c r="K93" s="7" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="L93" t="n">
         <v>20000</v>
@@ -10469,16 +10451,16 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U93" s="7" t="n">
-        <v>-40.49</v>
+        <v>-40.23</v>
       </c>
       <c r="V93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W93" s="7" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
       <c r="X93" s="7" t="n">
         <v>0.55</v>
@@ -10493,7 +10475,7 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB93" t="inlineStr">
@@ -10503,7 +10485,7 @@
       </c>
       <c r="AC93" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 MOL | AUDJPY.pro, T&amp;D19L13 L11 MOL | AUDUSD.pro, T&amp;D19L13 L11 MOL | EURUSD.pro, T&amp;D19L13 L11 MOL | GBPAUD.pro, T&amp;D19L13 L11 MOL | GBPCHF.pro</t>
+          <t>T&amp;D19L13 L11 MOL | AUDJPY.pro, T&amp;D19L13 L11 MOL | AUDUSD.pro, T&amp;D19L13 L11 MOL | EURUSD.pro, T&amp;D19L13 L11 MOL | GBPAUD.pro, T&amp;D19L13 L11 MOL | GBPCHF.pro, T&amp;D19L13 L11 MOL | GBPUSD.pro</t>
         </is>
       </c>
     </row>
@@ -10538,20 +10520,20 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/20/2026 19:52</t>
+          <t>08/21/2026 10:14</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
-        <v>19949.13</v>
+        <v>19951.04</v>
       </c>
       <c r="I94" s="7" t="n">
-        <v>-0.26</v>
+        <v>-0.25</v>
       </c>
       <c r="J94" s="7" t="n">
         <v>0.91</v>
       </c>
       <c r="K94" s="7" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="L94" t="n">
         <v>20000</v>
@@ -10569,19 +10551,19 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="U94" s="7" t="n">
-        <v>-50.87000000000002</v>
+        <v>-50.32000000000002</v>
       </c>
       <c r="V94" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W94" s="7" t="n">
-        <v>44.44444444444444</v>
+        <v>45.45454545454545</v>
       </c>
       <c r="X94" s="7" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="Y94" s="7" t="n">
         <v>0.91</v>
@@ -10593,7 +10575,7 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB94" t="inlineStr">
@@ -10603,7 +10585,7 @@
       </c>
       <c r="AC94" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L11 Agg | AUDJPY.pro, T&amp;D19L13 L11 Agg | AUDUSD.pro, T&amp;D19L13 L11 Agg | EURUSD.pro, T&amp;D19L13 L11 Agg | GBPAUD.pro, T&amp;D19L13 L11 Agg | GBPCHF.pro, T&amp;D19L13 L11 Agg | XAUUSD</t>
+          <t>T&amp;D19L13 L11 Agg | AUDJPY.pro, T&amp;D19L13 L11 Agg | AUDUSD.pro, T&amp;D19L13 L11 Agg | EURUSD.pro, T&amp;D19L13 L11 Agg | GBPAUD.pro, T&amp;D19L13 L11 Agg | GBPCHF.pro, T&amp;D19L13 L11 Agg | GBPUSD.pro, T&amp;D19L13 L11 Agg | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -10638,20 +10620,20 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/20/2026 19:51</t>
+          <t>08/21/2026 10:08</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
-        <v>98985.63</v>
+        <v>98922.03999999999</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>-0.99</v>
+        <v>-1.06</v>
       </c>
       <c r="J95" s="7" t="n">
-        <v>1.18</v>
+        <v>1.25</v>
       </c>
       <c r="K95" s="7" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="L95" t="n">
         <v>100000</v>
@@ -10669,22 +10651,22 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>371</v>
+        <v>393</v>
       </c>
       <c r="U95" s="7" t="n">
-        <v>-973.74</v>
+        <v>-1097.76</v>
       </c>
       <c r="V95" t="n">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="W95" s="7" t="n">
-        <v>52.83018867924528</v>
+        <v>51.90839694656488</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
       <c r="Y95" s="7" t="n">
-        <v>1.15</v>
+        <v>1.28</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -10693,7 +10675,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
@@ -10738,20 +10720,20 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/20/2026 19:54</t>
+          <t>08/21/2026 10:15</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
-        <v>97207.08</v>
+        <v>97031.89</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>-2.79</v>
+        <v>-2.97</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>3.35</v>
+        <v>3.53</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="L96" t="n">
         <v>100000</v>
@@ -10769,22 +10751,22 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>426</v>
+        <v>448</v>
       </c>
       <c r="U96" s="7" t="n">
-        <v>-2695.5</v>
+        <v>-3017.03</v>
       </c>
       <c r="V96" t="n">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="W96" s="7" t="n">
-        <v>52.58215962441315</v>
+        <v>51.78571428571429</v>
       </c>
       <c r="X96" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="Y96" s="7" t="n">
-        <v>3.27</v>
+        <v>3.59</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -10793,7 +10775,7 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr">
@@ -10838,20 +10820,20 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/20/2026 20:01</t>
+          <t>08/21/2026 10:31</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
-        <v>96262.02</v>
+        <v>95974.97</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>-3.74</v>
+        <v>-4.02</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>4.76</v>
+        <v>5.05</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="L97" t="n">
         <v>100000</v>
@@ -10869,22 +10851,22 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>426</v>
+        <v>448</v>
       </c>
       <c r="U97" s="7" t="n">
-        <v>-3616.09</v>
+        <v>-4085.89</v>
       </c>
       <c r="V97" t="n">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="W97" s="7" t="n">
-        <v>52.58215962441315</v>
+        <v>51.78571428571429</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>0.72</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y97" s="7" t="n">
-        <v>4.65</v>
+        <v>5.11</v>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
@@ -10893,7 +10875,7 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB97" t="inlineStr">
@@ -10938,20 +10920,20 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/20/2026 19:48</t>
+          <t>08/21/2026 10:03</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
-        <v>99589.60000000001</v>
+        <v>99497.42</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>-0.45</v>
+        <v>-0.54</v>
       </c>
       <c r="J98" s="7" t="n">
         <v>0.71</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="L98" t="n">
         <v>100000</v>
@@ -10969,19 +10951,19 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="U98" s="7" t="n">
-        <v>-410.3999999999999</v>
+        <v>-506.1599999999999</v>
       </c>
       <c r="V98" t="n">
         <v>60</v>
       </c>
       <c r="W98" s="7" t="n">
-        <v>48</v>
+        <v>45.80152671755725</v>
       </c>
       <c r="X98" s="7" t="n">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="Y98" s="7" t="n">
         <v>0.6899999999999999</v>
@@ -10993,7 +10975,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
@@ -11003,7 +10985,7 @@
       </c>
       <c r="AC98" t="inlineStr">
         <is>
-          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | CHFJPY.pro, T&amp;D19L13 L10 Prop | EURUSD.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | GBPJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USDCHF.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
+          <t>T&amp;D19L13 L10 Prop | AUDJPY.pro, T&amp;D19L13 L10 Prop | AUDUSD.pro, T&amp;D19L13 L10 Prop | CADJPY.pro, T&amp;D19L13 L10 Prop | CHFJPY.pro, T&amp;D19L13 L10 Prop | EURJPY.pro, T&amp;D19L13 L10 Prop | EURUSD.pro, T&amp;D19L13 L10 Prop | GBPCHF.pro, T&amp;D19L13 L10 Prop | GBPJPY.pro, T&amp;D19L13 L10 Prop | NZDUSD.pro, T&amp;D19L13 L10 Prop | US30, T&amp;D19L13 L10 Prop | US500, T&amp;D19L13 L10 Prop | USDCAD.pro, T&amp;D19L13 L10 Prop | USDCHF.pro, T&amp;D19L13 L10 Prop | USTECH, T&amp;D19L13 L10 Prop | XAUUSD</t>
         </is>
       </c>
     </row>
@@ -11038,7 +11020,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/20/2026 19:57</t>
+          <t>08/21/2026 10:19</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11138,7 +11120,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/20/2026 20:20</t>
+          <t>08/21/2026 11:31</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11465,20 +11447,20 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/20/2026 19:27</t>
+          <t>08/21/2026 09:40</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>28668.37</v>
+        <v>28140.86</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-25.36</v>
+        <v>-26.72</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
       </c>
       <c r="K103" s="7" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="L103" t="n">
         <v>25000</v>
@@ -11490,34 +11472,34 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>690.4599999999999</v>
+        <v>-684.8099999999999</v>
       </c>
       <c r="P103" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>72.5</v>
+        <v>15</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>4.019328319048451</v>
+        <v>0.158492977303727</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>0.64</v>
+        <v>2.74</v>
       </c>
       <c r="T103" t="n">
-        <v>3491</v>
+        <v>3512</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-5613.630000000002</v>
+        <v>-6256.16</v>
       </c>
       <c r="V103" t="n">
-        <v>2151</v>
+        <v>2155</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>61.61558292752793</v>
+        <v>61.36104783599089</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y103" s="7" t="n">
         <v>37.71</v>
@@ -11529,7 +11511,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11756,7 +11738,7 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 14:31</t>
+          <t>08/21/2026 16:21</t>
         </is>
       </c>
       <c r="H106" s="9" t="n">
@@ -12120,7 +12102,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 20:06</t>
+          <t>08/21/2026 10:52</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12393,7 +12375,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 20:23</t>
+          <t>08/21/2026 11:37</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12484,7 +12466,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 19:59</t>
+          <t>08/21/2026 10:26</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12569,7 +12551,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 20:06</t>
+          <t>08/21/2026 10:56</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12654,7 +12636,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 13:44</t>
+          <t>08/21/2026 14:55</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12824,7 +12806,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 19:57</t>
+          <t>08/21/2026 10:21</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12909,7 +12891,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 19:57</t>
+          <t>08/21/2026 10:22</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12994,7 +12976,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 19:55</t>
+          <t>08/21/2026 10:18</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13079,7 +13061,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 19:58</t>
+          <t>08/21/2026 10:24</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13164,7 +13146,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 20:02</t>
+          <t>08/21/2026 10:33</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13249,7 +13231,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 19:59</t>
+          <t>08/21/2026 10:26</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13864,7 +13846,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08/18/2026 14:31</t>
+          <t>08/21/2026 16:21</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14028,7 +14010,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/20/2026 20:06</t>
+          <t>08/21/2026 10:52</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14151,7 +14133,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/20/2026 20:23</t>
+          <t>08/21/2026 11:37</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14192,7 +14174,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/20/2026 19:59</t>
+          <t>08/21/2026 10:26</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14233,7 +14215,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/20/2026 20:06</t>
+          <t>08/21/2026 10:56</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14274,7 +14256,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/18/2026 13:44</t>
+          <t>08/21/2026 14:55</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14356,7 +14338,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/20/2026 19:57</t>
+          <t>08/21/2026 10:21</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14397,7 +14379,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/20/2026 19:57</t>
+          <t>08/21/2026 10:22</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14438,7 +14420,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/20/2026 19:55</t>
+          <t>08/21/2026 10:18</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14479,7 +14461,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/20/2026 19:58</t>
+          <t>08/21/2026 10:24</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14520,7 +14502,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/20/2026 20:02</t>
+          <t>08/21/2026 10:33</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14561,7 +14543,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/20/2026 19:59</t>
+          <t>08/21/2026 10:26</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -16132,7 +16114,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/20/2026 21:19</t>
+          <t>08/21/2026 08:38</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16178,11 +16160,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/20/2026 20:07</t>
+          <t>08/21/2026 10:57</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20106.35</v>
+        <v>20230.4</v>
       </c>
     </row>
     <row r="24">
@@ -16224,7 +16206,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/20/2026 20:37</t>
+          <t>08/21/2026 07:59</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -16247,7 +16229,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/20/2026 20:18</t>
+          <t>08/21/2026 11:25</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
@@ -16270,7 +16252,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/20/2026 18:55</t>
+          <t>08/21/2026 09:09</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16293,7 +16275,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/20/2026 18:57</t>
+          <t>08/21/2026 09:12</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16316,7 +16298,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/20/2026 18:59</t>
+          <t>08/21/2026 09:13</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16339,7 +16321,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/20/2026 21:46</t>
+          <t>08/21/2026 09:09</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16362,7 +16344,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/20/2026 15:57</t>
+          <t>08/21/2026 09:08</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16385,7 +16367,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/20/2026 18:52</t>
+          <t>08/21/2026 09:05</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16431,11 +16413,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/20/2026 20:17</t>
+          <t>08/21/2026 11:25</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>2944.12</v>
+        <v>2922.36</v>
       </c>
     </row>
     <row r="35">
@@ -16477,7 +16459,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/20/2026 19:50</t>
+          <t>08/21/2026 10:07</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -16500,7 +16482,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/20/2026 19:54</t>
+          <t>08/21/2026 10:17</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -16523,7 +16505,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/20/2026 20:59</t>
+          <t>08/21/2026 08:18</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -16546,7 +16528,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/20/2026 20:10</t>
+          <t>08/21/2026 07:33</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
@@ -16569,7 +16551,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/20/2026 20:15</t>
+          <t>08/21/2026 07:37</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
@@ -16684,7 +16666,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>08/20/2026 11:46</t>
+          <t>08/21/2026 12:03</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-24
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-21 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-24 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/21/2026 09:50</t>
+          <t>08/24/2026 21:12</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>52448.1</v>
+        <v>63616.48</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>139.75</v>
+        <v>190.8</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.08</v>
+        <v>1.11</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>12719.53</v>
+        <v>16243.8</v>
       </c>
       <c r="P2" t="n">
         <v>32</v>
@@ -994,25 +994,25 @@
         <v>80</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.475681386408174</v>
+        <v>1.607481039357358</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>25.81</v>
+        <v>30.8</v>
       </c>
       <c r="T2" t="n">
-        <v>3350</v>
+        <v>3354</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>31156.28999999999</v>
+        <v>38616.47999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2119</v>
+        <v>2123</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.25373134328358</v>
+        <v>63.29755515802027</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.07</v>
+        <v>1.09</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>08/18/2026 17:49</t>
+          <t>08/22/2026 01:38</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/19/2026 19:25</t>
+          <t>08/23/2026 19:11</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/21/2026 08:57</t>
+          <t>08/24/2026 09:00</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08/19/2026 09:44</t>
+          <t>08/22/2026 17:18</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/19/2026 14:59</t>
+          <t>08/23/2026 17:03</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08/18/2026 23:32</t>
+          <t>08/22/2026 08:47</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>08/19/2026 00:40</t>
+          <t>08/22/2026 10:31</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>08/19/2026 00:40</t>
+          <t>08/22/2026 10:33</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/21/2026 09:41</t>
+          <t>08/24/2026 21:20</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>08/18/2026 19:00</t>
+          <t>08/22/2026 02:27</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/21/2026 10:09</t>
+          <t>08/24/2026 10:17</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/21/2026 09:01</t>
+          <t>08/24/2026 19:55</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/20/2026 15:01</t>
+          <t>08/23/2026 21:56</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>08/21/2026 13:01</t>
+          <t>08/24/2026 13:03</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>08/21/2026 05:47</t>
+          <t>08/24/2026 05:49</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>08/21/2026 05:45</t>
+          <t>08/24/2026 05:49</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/21/2026 08:47</t>
+          <t>08/24/2026 19:41</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/21/2026 11:38</t>
+          <t>08/24/2026 17:47</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/21/2026 10:14</t>
+          <t>08/24/2026 21:19</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>08/18/2026 18:43</t>
+          <t>08/22/2026 02:16</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/21/2026 11:01</t>
+          <t>08/24/2026 21:35</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16597.1</v>
+        <v>16588.26</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-16.69</v>
+        <v>-16.73</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,7 +3492,7 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>64.88000000000002</v>
+        <v>71.06000000000003</v>
       </c>
       <c r="P25" t="n">
         <v>19</v>
@@ -3501,10 +3501,10 @@
         <v>47.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.157151507811554</v>
+        <v>1.174252084355076</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.84</v>
+        <v>0.71</v>
       </c>
       <c r="T25" t="n">
         <v>703</v>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/21/2026 09:24</t>
+          <t>08/24/2026 20:30</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/21/2026 10:30</t>
+          <t>08/24/2026 21:28</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>20173.69</v>
+        <v>19994.53</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-3.53</v>
+        <v>-4.39</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>7.39</v>
+        <v>7.4</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,7 +3710,7 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-260.4399999999999</v>
+        <v>-453.3899999999999</v>
       </c>
       <c r="P27" t="n">
         <v>20</v>
@@ -3719,10 +3719,10 @@
         <v>50</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.8425697567580638</v>
+        <v>0.7730019576134139</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>3.22</v>
+        <v>3.43</v>
       </c>
       <c r="T27" t="n">
         <v>110</v>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>08/18/2026 22:43</t>
+          <t>08/22/2026 08:13</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/21/2026 10:35</t>
+          <t>08/24/2026 21:29</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08/19/2026 10:19</t>
+          <t>08/22/2026 17:43</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/21/2026 11:03</t>
+          <t>08/24/2026 21:36</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/21/2026 10:20</t>
+          <t>08/24/2026 10:21</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>08/21/2026 11:09</t>
+          <t>08/24/2026 11:12</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,20 +4448,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/21/2026 08:49</t>
+          <t>08/24/2026 19:47</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
-        <v>20040.77</v>
+        <v>20151.55</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.2</v>
+        <v>0.75</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>3.42</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>1.02</v>
+        <v>1.06</v>
       </c>
       <c r="L34" t="n">
         <v>20000</v>
@@ -4473,19 +4473,19 @@
         <v>40</v>
       </c>
       <c r="O34" s="7" t="n">
-        <v>-432.08</v>
+        <v>-250.43</v>
       </c>
       <c r="P34" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q34" s="7" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="R34" s="7" t="n">
-        <v>0.6425693841254084</v>
+        <v>0.7799346209950966</v>
       </c>
       <c r="S34" s="7" t="n">
-        <v>2.66</v>
+        <v>2.5</v>
       </c>
       <c r="T34" t="n">
         <v>108</v>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/21/2026 00:15</t>
+          <t>08/24/2026 00:17</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/21/2026 08:19</t>
+          <t>08/24/2026 19:07</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19907.5</v>
+        <v>19997.1</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.46</v>
+        <v>-0.01</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
       </c>
-      <c r="K36" s="7" t="n">
-        <v>0.98</v>
+      <c r="K36" t="n">
+        <v>1</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,13 +4697,13 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>0.3999999999998636</v>
+        <v>-2.900000000000134</v>
       </c>
       <c r="V36" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="W36" s="7" t="n">
         <v>50</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,20 +4766,20 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/21/2026 07:57</t>
+          <t>08/24/2026 18:29</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
-        <v>19608.67</v>
+        <v>19407.85</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>-1.96</v>
+        <v>-2.96</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>9.82</v>
+        <v>10.38</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>0.93</v>
+        <v>0.89</v>
       </c>
       <c r="L37" t="n">
         <v>20000</v>
@@ -4791,7 +4791,7 @@
         <v>40</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>-2116.51</v>
+        <v>-2109.12</v>
       </c>
       <c r="P37" t="n">
         <v>14</v>
@@ -4800,10 +4800,10 @@
         <v>35</v>
       </c>
       <c r="R37" s="7" t="n">
-        <v>0.5154554445472112</v>
+        <v>0.5163289876509237</v>
       </c>
       <c r="S37" s="7" t="n">
-        <v>11.44</v>
+        <v>11.98</v>
       </c>
       <c r="T37" t="n">
         <v>54</v>
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/20/2026 17:31</t>
+          <t>08/23/2026 22:05</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/21/2026 08:18</t>
+          <t>08/24/2026 18:59</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>08/19/2026 09:29</t>
+          <t>08/22/2026 17:04</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>08/19/2026 07:28</t>
+          <t>08/22/2026 16:31</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/21/2026 10:32</t>
+          <t>08/24/2026 21:29</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/21/2026 11:32</t>
+          <t>08/24/2026 21:45</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,13 +5442,22 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>0</v>
+        <v>-50.87</v>
       </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="Q43" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="R43" s="7" t="n">
+        <v>0.2037877602128658</v>
+      </c>
+      <c r="S43" s="7" t="n">
+        <v>0.25</v>
       </c>
       <c r="T43" t="n">
         <v>4278</v>
@@ -5520,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/21/2026 10:29</t>
+          <t>08/24/2026 21:29</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5542,13 +5551,22 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>0</v>
+        <v>-1124.46</v>
       </c>
       <c r="P44" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="Q44" s="7" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="R44" s="7" t="n">
+        <v>0.4043290318479436</v>
+      </c>
+      <c r="S44" s="7" t="n">
+        <v>5.73</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5620,14 +5638,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/21/2026 11:03</t>
+          <t>08/24/2026 21:37</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19776.9</v>
+        <v>19782.46</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-1.11</v>
+        <v>-1.08</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>4.38</v>
@@ -5642,25 +5660,34 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>0</v>
+        <v>144.05</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>25</v>
+      </c>
+      <c r="Q45" s="7" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="R45" s="7" t="n">
+        <v>3.717924528301887</v>
+      </c>
+      <c r="S45" s="7" t="n">
+        <v>0.1</v>
       </c>
       <c r="T45" t="n">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-223.1</v>
+        <v>-217.5400000000001</v>
       </c>
       <c r="V45" t="n">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>55.83864118895966</v>
+        <v>56.02536997885835</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0.93</v>
@@ -5675,7 +5702,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5720,7 +5747,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/21/2026 10:09</t>
+          <t>08/24/2026 21:20</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5742,13 +5769,22 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>0</v>
+        <v>19977.76</v>
       </c>
       <c r="P46" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q46" s="7" t="n">
+        <v>32.43243243243244</v>
+      </c>
+      <c r="R46" s="7" t="n">
+        <v>311.8411389450754</v>
+      </c>
+      <c r="S46" s="7" t="n">
+        <v>0.11</v>
       </c>
       <c r="T46" t="n">
         <v>36</v>
@@ -5780,7 +5816,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>RECONCILE</t>
+          <t>OK (small account, full sample)</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5820,7 +5856,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/21/2026 10:18</t>
+          <t>08/24/2026 21:23</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5920,7 +5956,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/21/2026 10:07</t>
+          <t>08/24/2026 21:17</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6020,7 +6056,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/21/2026 11:05</t>
+          <t>08/24/2026 21:37</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6120,7 +6156,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/21/2026 11:00</t>
+          <t>08/24/2026 21:36</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6220,7 +6256,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/21/2026 10:17</t>
+          <t>08/24/2026 21:23</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6320,20 +6356,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/21/2026 10:15</t>
+          <t>08/24/2026 21:23</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>19322.78</v>
+        <v>20632.26</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>-3.38</v>
+        <v>3.17</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.18</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6354,16 +6390,16 @@
         <v>40</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>-677.22</v>
+        <v>632.2599999999998</v>
       </c>
       <c r="V52" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>27.5</v>
+        <v>30</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.18</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>10.19</v>
@@ -6375,7 +6411,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6420,20 +6456,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/21/2026 11:28</t>
+          <t>08/24/2026 21:41</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19784.06</v>
+        <v>19763.85</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.11</v>
+        <v>-1.21</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6451,16 +6487,16 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-218.54</v>
+        <v>-236.15</v>
       </c>
       <c r="V53" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>37.18411552346571</v>
+        <v>36.61971830985916</v>
       </c>
       <c r="X53" s="7" t="n">
         <v>0.77</v>
@@ -6475,7 +6511,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6520,7 +6556,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/21/2026 11:59</t>
+          <t>08/24/2026 17:58</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6620,7 +6656,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/21/2026 11:04</t>
+          <t>08/24/2026 21:36</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6720,7 +6756,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/21/2026 11:51</t>
+          <t>08/24/2026 17:55</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6820,20 +6856,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/21/2026 10:15</t>
+          <t>08/24/2026 21:19</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19724.15</v>
+        <v>19711.53</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.39</v>
+        <v>-1.45</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6851,16 +6887,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>835</v>
+        <v>845</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-280.2200000000001</v>
+        <v>-288.4700000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.83233532934131</v>
+        <v>44.02366863905326</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.79</v>
@@ -6875,7 +6911,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6920,7 +6956,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/21/2026 10:55</t>
+          <t>08/24/2026 21:32</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7020,7 +7056,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/21/2026 10:27</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7120,20 +7156,20 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/21/2026 10:34</t>
+          <t>08/24/2026 21:29</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>20199.39</v>
+        <v>19931.35</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-5.04</v>
+        <v>-6.3</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L60" s="7" t="n">
         <v>21100.65</v>
@@ -7220,7 +7256,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/21/2026 11:28</t>
+          <t>08/24/2026 21:42</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7320,7 +7356,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/21/2026 11:32</t>
+          <t>08/24/2026 21:45</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7420,20 +7456,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/21/2026 11:23</t>
+          <t>08/24/2026 21:40</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18720.59</v>
+        <v>18705.13</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.41</v>
+        <v>-6.49</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>7.22</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7451,19 +7487,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1279.41</v>
+        <v>-1294.87</v>
       </c>
       <c r="V63" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>9.090909090909092</v>
+        <v>10.8695652173913</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>7.21</v>
@@ -7475,7 +7511,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7520,7 +7556,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/21/2026 11:41</t>
+          <t>08/24/2026 21:46</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7542,13 +7578,22 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>0</v>
+        <v>-3.710000000000004</v>
       </c>
       <c r="P64" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q64" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R64" s="7" t="n">
+        <v>0.9861323963667626</v>
+      </c>
+      <c r="S64" s="7" t="n">
+        <v>0.95</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7620,20 +7665,20 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/21/2026 07:35</t>
+          <t>08/24/2026 21:37</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>18913.15</v>
+        <v>19301.2</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-5.48</v>
+        <v>-3.54</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>11.64</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="L65" t="n">
         <v>20000</v>
@@ -7720,7 +7765,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/21/2026 10:57</t>
+          <t>08/24/2026 21:33</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7820,7 +7865,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/21/2026 07:57</t>
+          <t>08/24/2026 18:26</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7920,7 +7965,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/20/2026 13:09</t>
+          <t>08/23/2026 21:48</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8020,7 +8065,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/20/2026 13:08</t>
+          <t>08/23/2026 21:47</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8120,7 +8165,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/20/2026 13:17</t>
+          <t>08/23/2026 21:48</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8220,7 +8265,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/21/2026 11:11</t>
+          <t>08/24/2026 21:39</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8320,7 +8365,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/21/2026 08:03</t>
+          <t>08/24/2026 18:38</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8420,7 +8465,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/21/2026 11:24</t>
+          <t>08/24/2026 21:43</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8520,20 +8565,20 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/21/2026 07:55</t>
+          <t>08/24/2026 18:25</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
-        <v>20328.13</v>
+        <v>20255.8</v>
       </c>
       <c r="I74" s="7" t="n">
-        <v>1.66</v>
+        <v>1.3</v>
       </c>
       <c r="J74" s="7" t="n">
-        <v>1.78</v>
+        <v>2.13</v>
       </c>
       <c r="K74" s="7" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="L74" t="n">
         <v>20000</v>
@@ -8620,20 +8665,20 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/21/2026 07:28</t>
+          <t>08/24/2026 21:33</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
-        <v>19941.62</v>
+        <v>19925.93</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>-0.25</v>
+        <v>-0.33</v>
       </c>
       <c r="J75" s="7" t="n">
         <v>4.48</v>
       </c>
       <c r="K75" s="7" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="L75" t="n">
         <v>20000</v>
@@ -8720,14 +8765,14 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/21/2026 11:57</t>
+          <t>08/24/2026 17:53</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
-        <v>20899.24</v>
+        <v>20904.09</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>4.55</v>
+        <v>4.57</v>
       </c>
       <c r="J76" s="7" t="n">
         <v>5.69</v>
@@ -8820,20 +8865,20 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/21/2026 11:22</t>
+          <t>08/24/2026 21:43</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
-        <v>19620.27</v>
+        <v>19533.82</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>-1.91</v>
+        <v>-2.34</v>
       </c>
       <c r="J77" s="7" t="n">
-        <v>4.69</v>
+        <v>5.07</v>
       </c>
       <c r="K77" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L77" t="n">
         <v>20000</v>
@@ -8920,20 +8965,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/21/2026 11:55</t>
+          <t>08/24/2026 17:54</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
-        <v>20268.7</v>
+        <v>20275.76</v>
       </c>
       <c r="I78" s="7" t="n">
-        <v>1.34</v>
+        <v>1.38</v>
       </c>
       <c r="J78" s="7" t="n">
         <v>5.5</v>
       </c>
       <c r="K78" s="7" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="L78" t="n">
         <v>20000</v>
@@ -9020,20 +9065,20 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/21/2026 11:46</t>
+          <t>08/24/2026 21:50</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
-        <v>19294.83</v>
+        <v>19579.58</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>-3.49</v>
+        <v>-2.07</v>
       </c>
       <c r="J79" s="7" t="n">
         <v>16.96</v>
       </c>
       <c r="K79" s="7" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="L79" t="n">
         <v>20000</v>
@@ -9120,20 +9165,20 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/21/2026 10:55</t>
+          <t>08/24/2026 21:33</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
-        <v>21265.6</v>
+        <v>21651.25</v>
       </c>
       <c r="I80" s="7" t="n">
-        <v>6.37</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="J80" s="7" t="n">
         <v>17.52</v>
       </c>
       <c r="K80" s="7" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
       <c r="L80" t="n">
         <v>20000</v>
@@ -9220,17 +9265,17 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/21/2026 07:55</t>
+          <t>08/24/2026 18:31</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
-        <v>18521.65</v>
+        <v>18347.58</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>-7.37</v>
+        <v>-8.24</v>
       </c>
       <c r="J81" s="7" t="n">
-        <v>12.36</v>
+        <v>12.64</v>
       </c>
       <c r="K81" s="7" t="n">
         <v>0.92</v>
@@ -9320,14 +9365,14 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/21/2026 11:49</t>
+          <t>08/24/2026 17:53</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
-        <v>20048.59</v>
+        <v>20055.23</v>
       </c>
       <c r="I82" s="7" t="n">
-        <v>0.29</v>
+        <v>0.32</v>
       </c>
       <c r="J82" s="7" t="n">
         <v>5.82</v>
@@ -9420,20 +9465,20 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/21/2026 08:03</t>
+          <t>08/24/2026 18:40</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
-        <v>19993.34</v>
+        <v>20136.49</v>
       </c>
       <c r="I83" s="7" t="n">
-        <v>-0.04</v>
+        <v>0.68</v>
       </c>
       <c r="J83" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="K83" s="7" t="n">
-        <v>0.87</v>
+        <v>3.76</v>
       </c>
       <c r="L83" t="n">
         <v>20000</v>
@@ -9451,19 +9496,19 @@
         <v>0</v>
       </c>
       <c r="T83" t="n">
+        <v>3</v>
+      </c>
+      <c r="U83" s="7" t="n">
+        <v>136.49</v>
+      </c>
+      <c r="V83" t="n">
         <v>2</v>
       </c>
-      <c r="U83" s="7" t="n">
-        <v>-6.659999999999997</v>
-      </c>
-      <c r="V83" t="n">
-        <v>1</v>
-      </c>
       <c r="W83" s="7" t="n">
-        <v>50</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="X83" s="7" t="n">
-        <v>0.87</v>
+        <v>3.76</v>
       </c>
       <c r="Y83" s="7" t="n">
         <v>0.25</v>
@@ -9475,7 +9520,7 @@
       </c>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB83" t="inlineStr">
@@ -9520,7 +9565,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/21/2026 08:26</t>
+          <t>08/24/2026 19:16</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9620,7 +9665,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/21/2026 07:55</t>
+          <t>08/24/2026 18:25</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9720,20 +9765,20 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/21/2026 08:03</t>
+          <t>08/24/2026 18:35</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20881.33</v>
+        <v>20715.24</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>4.42</v>
+        <v>3.59</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>2.18</v>
       </c>
       <c r="K86" s="7" t="n">
-        <v>2.2</v>
+        <v>1.72</v>
       </c>
       <c r="L86" t="n">
         <v>20000</v>
@@ -9751,19 +9796,19 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>877.8300000000002</v>
+        <v>715.2400000000001</v>
       </c>
       <c r="V86" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="W86" s="7" t="n">
         <v>50</v>
       </c>
       <c r="X86" s="7" t="n">
-        <v>2.19</v>
+        <v>1.72</v>
       </c>
       <c r="Y86" s="7" t="n">
         <v>2.17</v>
@@ -9775,7 +9820,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9820,7 +9865,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/21/2026 11:32</t>
+          <t>08/24/2026 21:46</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9920,20 +9965,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/21/2026 07:52</t>
+          <t>08/24/2026 18:24</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20559.26</v>
+        <v>20600.46</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>2.79</v>
+        <v>2.99</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -9951,19 +9996,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
+        <v>44</v>
+      </c>
+      <c r="U88" s="7" t="n">
+        <v>600.46</v>
+      </c>
+      <c r="V88" t="n">
         <v>42</v>
       </c>
-      <c r="U88" s="7" t="n">
-        <v>576.16</v>
-      </c>
-      <c r="V88" t="n">
-        <v>40</v>
-      </c>
       <c r="W88" s="7" t="n">
-        <v>95.23809523809523</v>
+        <v>95.45454545454545</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>3.78</v>
+        <v>3.9</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -9975,7 +10020,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10020,20 +10065,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/21/2026 07:53</t>
+          <t>08/24/2026 18:20</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>22762.4</v>
+        <v>22700.91</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>13.84</v>
+        <v>13.54</v>
       </c>
       <c r="J89" s="7" t="n">
-        <v>1.99</v>
+        <v>3.08</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>2.53</v>
+        <v>2.29</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10051,22 +10096,22 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>2515.89</v>
+        <v>2700.91</v>
       </c>
       <c r="V89" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>75.67567567567568</v>
+        <v>74.35897435897436</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>2.23</v>
+        <v>2.29</v>
       </c>
       <c r="Y89" s="7" t="n">
-        <v>2.9</v>
+        <v>3.08</v>
       </c>
       <c r="Z89" t="inlineStr">
         <is>
@@ -10075,7 +10120,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10120,20 +10165,20 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/21/2026 10:19</t>
-        </is>
-      </c>
-      <c r="H90" s="7" t="n">
-        <v>19852.15</v>
+          <t>08/24/2026 21:27</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>19746</v>
       </c>
       <c r="I90" s="7" t="n">
-        <v>-0.74</v>
+        <v>-1.27</v>
       </c>
       <c r="J90" s="7" t="n">
-        <v>1.53</v>
+        <v>2.05</v>
       </c>
       <c r="K90" s="7" t="n">
-        <v>0.63</v>
+        <v>0.5</v>
       </c>
       <c r="L90" t="n">
         <v>20000</v>
@@ -10220,7 +10265,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/21/2026 10:17</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10320,11 +10365,11 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/21/2026 10:18</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
-        <v>19987.07</v>
+        <v>19986.87</v>
       </c>
       <c r="I92" s="7" t="n">
         <v>-0.06</v>
@@ -10420,11 +10465,11 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/21/2026 10:15</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
-        <v>19960.45</v>
+        <v>19959.77</v>
       </c>
       <c r="I93" s="7" t="n">
         <v>-0.2</v>
@@ -10433,7 +10478,7 @@
         <v>0.44</v>
       </c>
       <c r="K93" s="7" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="L93" t="n">
         <v>20000</v>
@@ -10520,14 +10565,14 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/21/2026 10:14</t>
+          <t>08/24/2026 21:24</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
-        <v>19951.04</v>
+        <v>19949.68</v>
       </c>
       <c r="I94" s="7" t="n">
-        <v>-0.25</v>
+        <v>-0.26</v>
       </c>
       <c r="J94" s="7" t="n">
         <v>0.91</v>
@@ -10620,20 +10665,20 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/21/2026 10:08</t>
+          <t>08/24/2026 21:19</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
-        <v>98922.03999999999</v>
+        <v>98853.85000000001</v>
       </c>
       <c r="I95" s="7" t="n">
-        <v>-1.06</v>
+        <v>-1.13</v>
       </c>
       <c r="J95" s="7" t="n">
-        <v>1.25</v>
+        <v>1.32</v>
       </c>
       <c r="K95" s="7" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="L95" t="n">
         <v>100000</v>
@@ -10720,20 +10765,20 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/21/2026 10:15</t>
+          <t>08/24/2026 21:27</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
-        <v>97031.89</v>
+        <v>96865.77</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>-2.97</v>
+        <v>-3.14</v>
       </c>
       <c r="J96" s="7" t="n">
-        <v>3.53</v>
+        <v>3.69</v>
       </c>
       <c r="K96" s="7" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="L96" t="n">
         <v>100000</v>
@@ -10820,20 +10865,20 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/21/2026 10:31</t>
+          <t>08/24/2026 21:31</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
-        <v>95974.97</v>
+        <v>95768.78999999999</v>
       </c>
       <c r="I97" s="7" t="n">
-        <v>-4.02</v>
+        <v>-4.23</v>
       </c>
       <c r="J97" s="7" t="n">
-        <v>5.05</v>
+        <v>5.24</v>
       </c>
       <c r="K97" s="7" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L97" t="n">
         <v>100000</v>
@@ -10920,20 +10965,20 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/21/2026 10:03</t>
+          <t>08/24/2026 21:19</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
-        <v>99497.42</v>
+        <v>99477.8</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>-0.54</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="J98" s="7" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="K98" s="7" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="L98" t="n">
         <v>100000</v>
@@ -11020,7 +11065,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/21/2026 10:19</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11120,7 +11165,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/21/2026 11:31</t>
+          <t>08/24/2026 21:48</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11229,7 +11274,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>08/20/2026 04:06</t>
+          <t>08/23/2026 20:59</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11338,7 +11383,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>08/18/2026 23:31</t>
+          <t>08/22/2026 08:47</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11447,14 +11492,14 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/21/2026 09:40</t>
+          <t>08/24/2026 20:59</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>28140.86</v>
+        <v>28075.4</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-26.72</v>
+        <v>-26.89</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
@@ -11472,34 +11517,34 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>-684.8099999999999</v>
+        <v>-437.15</v>
       </c>
       <c r="P103" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>15</v>
+        <v>32.5</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>0.158492977303727</v>
+        <v>0.2340377067563779</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>2.74</v>
+        <v>1.94</v>
       </c>
       <c r="T103" t="n">
-        <v>3512</v>
+        <v>3530</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-6256.16</v>
+        <v>-6206.600000000002</v>
       </c>
       <c r="V103" t="n">
-        <v>2155</v>
+        <v>2164</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>61.36104783599089</v>
+        <v>61.30311614730878</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="Y103" s="7" t="n">
         <v>37.71</v>
@@ -11511,7 +11556,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11556,7 +11601,7 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 22:24</t>
+          <t>08/22/2026 07:56</t>
         </is>
       </c>
       <c r="H104" s="9" t="n">
@@ -11647,7 +11692,7 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 20:07</t>
+          <t>08/23/2026 19:21</t>
         </is>
       </c>
       <c r="H105" s="9" t="n">
@@ -11738,7 +11783,7 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 16:21</t>
+          <t>08/24/2026 16:30</t>
         </is>
       </c>
       <c r="H106" s="9" t="n">
@@ -11829,7 +11874,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 09:55</t>
+          <t>08/22/2026 17:25</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -12011,7 +12056,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 23:30</t>
+          <t>08/22/2026 08:46</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12102,7 +12147,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:52</t>
+          <t>08/24/2026 21:33</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12193,7 +12238,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 18:31</t>
+          <t>08/22/2026 02:08</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12284,7 +12329,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 14:40</t>
+          <t>08/23/2026 16:44</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12375,7 +12420,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 11:37</t>
+          <t>08/24/2026 21:47</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12466,7 +12511,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:26</t>
+          <t>08/24/2026 21:29</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12488,17 +12533,23 @@
         <v>0</v>
       </c>
       <c r="N114" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O114" s="9" t="n">
-        <v>0</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="P114" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q114" s="8" t="n"/>
-      <c r="R114" s="8" t="n"/>
-      <c r="S114" s="8" t="n"/>
+        <v>26</v>
+      </c>
+      <c r="Q114" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="R114" s="9" t="n">
+        <v>1.223174978645115</v>
+      </c>
+      <c r="S114" s="9" t="n">
+        <v>0.57</v>
+      </c>
       <c r="T114" s="8" t="n">
         <v>0</v>
       </c>
@@ -12551,7 +12602,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:56</t>
+          <t>08/24/2026 21:34</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12636,7 +12687,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 14:55</t>
+          <t>08/24/2026 14:57</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12721,7 +12772,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>08/20/2026 13:11</t>
+          <t>08/23/2026 21:48</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12743,17 +12794,23 @@
         <v>0</v>
       </c>
       <c r="N117" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O117" s="9" t="n">
-        <v>0</v>
+        <v>-58.49</v>
       </c>
       <c r="P117" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q117" s="8" t="n"/>
-      <c r="R117" s="8" t="n"/>
-      <c r="S117" s="8" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="Q117" s="9" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R117" s="9" t="n">
+        <v>0.2666750250752257</v>
+      </c>
+      <c r="S117" s="9" t="n">
+        <v>0.32</v>
+      </c>
       <c r="T117" s="8" t="n">
         <v>0</v>
       </c>
@@ -12806,7 +12863,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:21</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12891,7 +12948,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:22</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12976,7 +13033,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:18</t>
+          <t>08/24/2026 21:25</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13061,7 +13118,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:24</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13083,17 +13140,23 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>0</v>
+        <v>-3715.63</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q121" s="8" t="n"/>
-      <c r="R121" s="8" t="n"/>
-      <c r="S121" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q121" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R121" s="9" t="n">
+        <v>0.2438039067238144</v>
+      </c>
+      <c r="S121" s="9" t="n">
+        <v>3.72</v>
+      </c>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13146,7 +13209,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:33</t>
+          <t>08/24/2026 21:31</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13231,7 +13294,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/21/2026 10:26</t>
+          <t>08/24/2026 21:30</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13316,7 +13379,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 20:13</t>
+          <t>08/22/2026 05:52</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13407,7 +13470,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>08/18/2026 19:52</t>
+          <t>08/22/2026 04:12</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13589,7 +13652,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 01:03</t>
+          <t>08/22/2026 10:52</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13764,7 +13827,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>08/18/2026 22:24</t>
+          <t>08/22/2026 07:56</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -13805,7 +13868,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08/19/2026 20:07</t>
+          <t>08/23/2026 19:21</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -13846,7 +13909,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08/21/2026 16:21</t>
+          <t>08/24/2026 16:30</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -13887,7 +13950,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08/19/2026 09:55</t>
+          <t>08/22/2026 17:25</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -13969,7 +14032,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08/18/2026 23:30</t>
+          <t>08/22/2026 08:46</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14010,7 +14073,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/21/2026 10:52</t>
+          <t>08/24/2026 21:33</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14051,7 +14114,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>08/18/2026 18:31</t>
+          <t>08/22/2026 02:08</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14092,7 +14155,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/19/2026 14:40</t>
+          <t>08/23/2026 16:44</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14133,7 +14196,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/21/2026 11:37</t>
+          <t>08/24/2026 21:47</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14174,7 +14237,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/21/2026 10:26</t>
+          <t>08/24/2026 21:29</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14184,7 +14247,7 @@
         <v>2.96</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
@@ -14215,7 +14278,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/21/2026 10:56</t>
+          <t>08/24/2026 21:34</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14256,7 +14319,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/21/2026 14:55</t>
+          <t>08/24/2026 14:57</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14297,7 +14360,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/20/2026 13:11</t>
+          <t>08/23/2026 21:48</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14307,7 +14370,7 @@
         <v>-0.16</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19">
@@ -14338,7 +14401,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/21/2026 10:21</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14379,7 +14442,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/21/2026 10:22</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14420,7 +14483,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/21/2026 10:18</t>
+          <t>08/24/2026 21:25</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14461,7 +14524,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/21/2026 10:24</t>
+          <t>08/24/2026 21:26</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14471,7 +14534,7 @@
         <v>-6.66</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -14502,7 +14565,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/21/2026 10:33</t>
+          <t>08/24/2026 21:31</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14543,7 +14606,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/21/2026 10:26</t>
+          <t>08/24/2026 21:30</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -14584,7 +14647,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>08/18/2026 20:13</t>
+          <t>08/22/2026 05:52</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -14625,7 +14688,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>08/18/2026 19:52</t>
+          <t>08/22/2026 04:12</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
@@ -14707,7 +14770,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>08/19/2026 01:03</t>
+          <t>08/22/2026 10:52</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
@@ -15723,7 +15786,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08/18/2026 21:43</t>
+          <t>08/22/2026 07:14</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -15746,7 +15809,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/19/2026 10:25</t>
+          <t>08/23/2026 12:52</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -15769,7 +15832,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08/18/2026 21:29</t>
+          <t>08/22/2026 07:00</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -15792,7 +15855,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08/18/2026 16:31</t>
+          <t>08/22/2026 00:26</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -15815,7 +15878,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/20/2026 07:56</t>
+          <t>08/23/2026 21:11</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -15838,7 +15901,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08/19/2026 04:57</t>
+          <t>08/22/2026 15:07</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -15861,7 +15924,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08/18/2026 15:55</t>
+          <t>08/21/2026 23:40</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -15884,7 +15947,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08/19/2026 05:40</t>
+          <t>08/22/2026 15:16</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -15907,7 +15970,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/19/2026 13:03</t>
+          <t>08/23/2026 15:22</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -15930,7 +15993,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08/18/2026 22:45</t>
+          <t>08/22/2026 08:12</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -15953,7 +16016,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/19/2026 15:27</t>
+          <t>08/23/2026 17:20</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -15976,7 +16039,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08/18/2026 21:29</t>
+          <t>08/22/2026 06:55</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -16022,7 +16085,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/20/2026 09:06</t>
+          <t>08/23/2026 21:20</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -16045,7 +16108,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/20/2026 07:42</t>
+          <t>08/23/2026 21:10</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -16068,7 +16131,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08/19/2026 00:02</t>
+          <t>08/22/2026 09:18</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -16091,7 +16154,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08/18/2026 16:22</t>
+          <t>08/22/2026 00:12</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -16114,7 +16177,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/21/2026 08:38</t>
+          <t>08/24/2026 19:29</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16137,7 +16200,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08/18/2026 22:47</t>
+          <t>08/22/2026 08:17</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -16160,11 +16223,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/21/2026 10:57</t>
+          <t>08/24/2026 21:36</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20230.4</v>
+        <v>20228.52</v>
       </c>
     </row>
     <row r="24">
@@ -16206,7 +16269,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/21/2026 07:59</t>
+          <t>08/24/2026 18:28</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -16229,11 +16292,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/21/2026 11:25</t>
+          <t>08/24/2026 21:40</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20768.26</v>
+        <v>21419.57</v>
       </c>
     </row>
     <row r="27">
@@ -16252,7 +16315,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/21/2026 09:09</t>
+          <t>08/24/2026 20:20</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16275,7 +16338,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/21/2026 09:12</t>
+          <t>08/24/2026 20:11</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16298,7 +16361,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/21/2026 09:13</t>
+          <t>08/24/2026 20:14</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16321,7 +16384,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/21/2026 09:09</t>
+          <t>08/24/2026 19:55</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16344,7 +16407,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/21/2026 09:08</t>
+          <t>08/24/2026 20:06</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16367,7 +16430,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/21/2026 09:05</t>
+          <t>08/24/2026 20:02</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16390,7 +16453,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/19/2026 14:55</t>
+          <t>08/23/2026 16:59</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -16413,11 +16476,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/21/2026 11:25</t>
+          <t>08/24/2026 21:40</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>2922.36</v>
+        <v>2914.73</v>
       </c>
     </row>
     <row r="35">
@@ -16459,7 +16522,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/21/2026 10:07</t>
+          <t>08/24/2026 21:19</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -16482,7 +16545,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/21/2026 10:17</t>
+          <t>08/24/2026 21:27</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -16505,7 +16568,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/21/2026 08:18</t>
+          <t>08/24/2026 18:56</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -16528,11 +16591,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/21/2026 07:33</t>
+          <t>08/24/2026 21:37</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>19985.75</v>
+        <v>19975.38</v>
       </c>
     </row>
     <row r="40">
@@ -16551,11 +16614,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/21/2026 07:37</t>
+          <t>08/24/2026 21:39</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>31954.16</v>
+        <v>32004.41</v>
       </c>
     </row>
     <row r="41">
@@ -16597,7 +16660,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>08/18/2026 21:32</t>
+          <t>08/22/2026 06:52</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -16620,7 +16683,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>08/15/2026 21:16</t>
+          <t>08/22/2026 07:42</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -16643,7 +16706,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>08/19/2026 01:02</t>
+          <t>08/22/2026 10:49</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
@@ -16666,7 +16729,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>08/21/2026 12:03</t>
+          <t>08/24/2026 12:36</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-25
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-24 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-25 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/24/2026 21:12</t>
+          <t>08/25/2026 18:50</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>63616.48</v>
-      </c>
-      <c r="I2" s="7" t="n">
-        <v>190.8</v>
+        <v>57753.37</v>
+      </c>
+      <c r="I2" t="n">
+        <v>164</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.11</v>
+        <v>1.09</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>16243.8</v>
+        <v>9503.240000000002</v>
       </c>
       <c r="P2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>80</v>
+        <v>77.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.607481039357358</v>
+        <v>1.291486198539937</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>30.8</v>
+        <v>31.5</v>
       </c>
       <c r="T2" t="n">
-        <v>3354</v>
+        <v>3356</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>38616.47999999999</v>
+        <v>32753.36999999999</v>
       </c>
       <c r="V2" t="n">
         <v>2123</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.29755515802027</v>
+        <v>63.25983313468415</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.09</v>
+        <v>1.07</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>08/22/2026 01:38</t>
+          <t>08/25/2026 04:11</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08/22/2026 17:18</t>
+          <t>08/25/2026 17:19</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08/22/2026 08:47</t>
+          <t>08/25/2026 08:49</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>08/22/2026 10:31</t>
+          <t>08/25/2026 10:34</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>08/22/2026 10:33</t>
+          <t>08/25/2026 10:36</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/24/2026 21:20</t>
+          <t>08/25/2026 21:45</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>08/22/2026 02:27</t>
+          <t>08/25/2026 04:44</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/24/2026 19:55</t>
+          <t>08/25/2026 21:08</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/24/2026 19:41</t>
+          <t>08/25/2026 20:59</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/24/2026 17:47</t>
+          <t>08/25/2026 19:34</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/24/2026 21:19</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>08/22/2026 02:16</t>
+          <t>08/25/2026 04:36</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/24/2026 21:35</t>
+          <t>08/25/2026 19:17</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/24/2026 20:30</t>
+          <t>08/25/2026 21:27</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/24/2026 21:28</t>
+          <t>08/25/2026 19:11</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>08/22/2026 08:13</t>
+          <t>08/25/2026 08:15</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/24/2026 21:29</t>
+          <t>08/25/2026 19:13</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08/22/2026 17:43</t>
+          <t>08/25/2026 17:51</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/24/2026 21:36</t>
+          <t>08/25/2026 19:19</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/24/2026 19:47</t>
+          <t>08/25/2026 21:02</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/24/2026 19:07</t>
+          <t>08/25/2026 20:35</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19997.1</v>
+        <v>19904.3</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.01</v>
+        <v>-0.47</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
       </c>
-      <c r="K36" t="n">
-        <v>1</v>
+      <c r="K36" s="7" t="n">
+        <v>0.98</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-2.900000000000134</v>
+        <v>-95.70000000000013</v>
       </c>
       <c r="V36" t="n">
         <v>46</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>50</v>
+        <v>49.46236559139785</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.83</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/24/2026 18:29</t>
+          <t>08/25/2026 20:06</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/24/2026 18:59</t>
+          <t>08/25/2026 20:27</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>08/22/2026 17:04</t>
+          <t>08/25/2026 17:06</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/24/2026 21:29</t>
+          <t>08/25/2026 19:10</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/24/2026 21:45</t>
+          <t>08/25/2026 19:42</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/24/2026 21:29</t>
+          <t>08/25/2026 19:09</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/24/2026 21:37</t>
+          <t>08/25/2026 19:22</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/24/2026 21:20</t>
+          <t>08/25/2026 18:59</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/24/2026 21:23</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/24/2026 21:17</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -5978,13 +5978,22 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>0</v>
+        <v>504.68</v>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="Q48" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="R48" s="7" t="n">
+        <v>2.47982641332395</v>
+      </c>
+      <c r="S48" s="7" t="n">
+        <v>1.7</v>
       </c>
       <c r="T48" t="n">
         <v>193</v>
@@ -6056,7 +6065,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/24/2026 21:37</t>
+          <t>08/25/2026 19:21</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6156,7 +6165,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/24/2026 21:36</t>
+          <t>08/25/2026 19:17</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6178,13 +6187,22 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>0</v>
+        <v>13.93999999999999</v>
       </c>
       <c r="P50" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q50" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R50" s="7" t="n">
+        <v>1.066618876941458</v>
+      </c>
+      <c r="S50" s="7" t="n">
+        <v>0.89</v>
       </c>
       <c r="T50" t="n">
         <v>1161</v>
@@ -6256,7 +6274,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/24/2026 21:23</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6356,7 +6374,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/24/2026 21:23</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6456,20 +6474,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/24/2026 21:41</t>
-        </is>
-      </c>
-      <c r="H53" s="7" t="n">
-        <v>19763.85</v>
+          <t>08/25/2026 19:28</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>19747</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.21</v>
+        <v>-1.29</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6487,19 +6505,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-236.15</v>
+        <v>-253.0000000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.61971830985916</v>
+        <v>36.20689655172414</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6511,7 +6529,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6556,7 +6574,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/24/2026 17:58</t>
+          <t>08/25/2026 19:40</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6656,7 +6674,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/24/2026 21:36</t>
+          <t>08/25/2026 19:20</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6756,7 +6774,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/24/2026 17:55</t>
+          <t>08/25/2026 19:35</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6856,14 +6874,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/24/2026 21:19</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19711.53</v>
+        <v>19716.74</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.45</v>
+        <v>-1.42</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6887,16 +6905,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>845</v>
+        <v>853</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-288.4700000000001</v>
+        <v>-283.26</v>
       </c>
       <c r="V57" t="n">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.02366863905326</v>
+        <v>43.96248534583822</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.79</v>
@@ -6911,7 +6929,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6956,7 +6974,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/24/2026 21:32</t>
+          <t>08/25/2026 19:14</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7056,7 +7074,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:05</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7156,7 +7174,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/24/2026 21:29</t>
+          <t>08/25/2026 19:13</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7256,7 +7274,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/24/2026 21:42</t>
+          <t>08/25/2026 19:28</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7356,7 +7374,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/24/2026 21:45</t>
+          <t>08/25/2026 19:30</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7456,14 +7474,14 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/24/2026 21:40</t>
+          <t>08/25/2026 19:24</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18705.13</v>
+        <v>18680.7</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.49</v>
+        <v>-6.61</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>7.22</v>
@@ -7487,16 +7505,16 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1294.87</v>
+        <v>-1319.3</v>
       </c>
       <c r="V63" t="n">
         <v>5</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>10.8695652173913</v>
+        <v>10.63829787234043</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>0.39</v>
@@ -7511,7 +7529,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7556,7 +7574,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/24/2026 21:46</t>
+          <t>08/25/2026 19:32</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7578,22 +7596,13 @@
         <v>0</v>
       </c>
       <c r="N64" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O64" s="7" t="n">
-        <v>-3.710000000000004</v>
+        <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q64" s="7" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="R64" s="7" t="n">
-        <v>0.9861323963667626</v>
-      </c>
-      <c r="S64" s="7" t="n">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="T64" t="n">
         <v>228</v>
@@ -7665,7 +7674,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/24/2026 21:37</t>
+          <t>08/25/2026 19:21</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7765,7 +7774,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/24/2026 21:33</t>
+          <t>08/25/2026 19:15</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7865,7 +7874,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/24/2026 18:26</t>
+          <t>08/25/2026 20:08</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -8265,7 +8274,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/24/2026 21:39</t>
+          <t>08/25/2026 19:23</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8365,7 +8374,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/24/2026 18:38</t>
+          <t>08/25/2026 20:14</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8465,7 +8474,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/24/2026 21:43</t>
+          <t>08/25/2026 19:28</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8565,7 +8574,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/24/2026 18:25</t>
+          <t>08/25/2026 20:03</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8665,7 +8674,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/24/2026 21:33</t>
+          <t>08/25/2026 19:21</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8765,7 +8774,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/24/2026 17:53</t>
+          <t>08/25/2026 19:39</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8865,7 +8874,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/24/2026 21:43</t>
+          <t>08/25/2026 19:25</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8965,7 +8974,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/24/2026 17:54</t>
+          <t>08/25/2026 19:39</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9065,7 +9074,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/24/2026 21:50</t>
+          <t>08/25/2026 19:38</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9165,7 +9174,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/24/2026 21:33</t>
+          <t>08/25/2026 19:21</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9265,7 +9274,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/24/2026 18:31</t>
+          <t>08/25/2026 20:16</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9365,7 +9374,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/24/2026 17:53</t>
+          <t>08/25/2026 19:39</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9465,7 +9474,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/24/2026 18:40</t>
+          <t>08/25/2026 20:13</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9565,7 +9574,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/24/2026 19:16</t>
+          <t>08/25/2026 20:48</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9665,7 +9674,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/24/2026 18:25</t>
+          <t>08/25/2026 20:02</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9765,14 +9774,14 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/24/2026 18:35</t>
+          <t>08/25/2026 20:12</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20715.24</v>
+        <v>20713.74</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>3.59</v>
+        <v>3.58</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>2.18</v>
@@ -9796,13 +9805,13 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>715.2400000000001</v>
+        <v>713.7400000000001</v>
       </c>
       <c r="V86" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="W86" s="7" t="n">
         <v>50</v>
@@ -9820,7 +9829,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9865,7 +9874,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/24/2026 21:46</t>
+          <t>08/25/2026 19:33</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9965,20 +9974,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/24/2026 18:24</t>
+          <t>08/25/2026 20:02</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20600.46</v>
+        <v>20703.02</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>2.99</v>
+        <v>3.5</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>3.9</v>
+        <v>4.39</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -9996,19 +10005,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
+        <v>46</v>
+      </c>
+      <c r="U88" s="7" t="n">
+        <v>700.26</v>
+      </c>
+      <c r="V88" t="n">
         <v>44</v>
       </c>
-      <c r="U88" s="7" t="n">
-        <v>600.46</v>
-      </c>
-      <c r="V88" t="n">
-        <v>42</v>
-      </c>
       <c r="W88" s="7" t="n">
-        <v>95.45454545454545</v>
+        <v>95.65217391304348</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>3.9</v>
+        <v>4.38</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -10020,7 +10029,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10065,20 +10074,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/24/2026 18:20</t>
+          <t>08/25/2026 20:17</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>22700.91</v>
+        <v>22841.48</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>13.54</v>
+        <v>14.25</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>3.08</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>2.29</v>
+        <v>2.23</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10087,28 +10096,37 @@
         <v>0</v>
       </c>
       <c r="N89" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O89" s="7" t="n">
-        <v>0</v>
+        <v>2495.88</v>
       </c>
       <c r="P89" t="n">
-        <v>0</v>
+        <v>29</v>
+      </c>
+      <c r="Q89" s="7" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="R89" s="7" t="n">
+        <v>2.076209284476142</v>
+      </c>
+      <c r="S89" s="7" t="n">
+        <v>3.13</v>
       </c>
       <c r="T89" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>2700.91</v>
+        <v>2841.48</v>
       </c>
       <c r="V89" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>74.35897435897436</v>
+        <v>73.80952380952381</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>2.29</v>
+        <v>2.23</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3.08</v>
@@ -10120,7 +10138,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10165,7 +10183,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/24/2026 21:27</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -10265,7 +10283,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:03</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10365,7 +10383,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:03</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10465,7 +10483,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:03</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10565,7 +10583,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/24/2026 21:24</t>
+          <t>08/25/2026 19:03</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10665,7 +10683,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/24/2026 21:19</t>
+          <t>08/25/2026 18:58</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10765,7 +10783,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/24/2026 21:27</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10865,7 +10883,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/24/2026 21:31</t>
+          <t>08/25/2026 19:11</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10965,7 +10983,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/24/2026 21:19</t>
+          <t>08/25/2026 18:56</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11065,7 +11083,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11165,7 +11183,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/24/2026 21:48</t>
+          <t>08/25/2026 19:33</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11383,7 +11401,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>08/22/2026 08:47</t>
+          <t>08/25/2026 08:49</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11492,14 +11510,14 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/24/2026 20:59</t>
+          <t>08/25/2026 21:45</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>28075.4</v>
+        <v>28108.64</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-26.89</v>
+        <v>-26.8</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
@@ -11517,31 +11535,31 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>-437.15</v>
+        <v>-271.17</v>
       </c>
       <c r="P103" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>32.5</v>
+        <v>47.5</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>0.2340377067563779</v>
+        <v>0.3800978419897586</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>1.94</v>
+        <v>1.57</v>
       </c>
       <c r="T103" t="n">
-        <v>3530</v>
+        <v>3542</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-6206.600000000002</v>
+        <v>-6173.360000000001</v>
       </c>
       <c r="V103" t="n">
-        <v>2164</v>
+        <v>2170</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>61.30311614730878</v>
+        <v>61.26482213438735</v>
       </c>
       <c r="X103" s="7" t="n">
         <v>0.82</v>
@@ -11556,7 +11574,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11601,7 +11619,7 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>08/22/2026 07:56</t>
+          <t>08/25/2026 08:04</t>
         </is>
       </c>
       <c r="H104" s="9" t="n">
@@ -11874,7 +11892,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>08/22/2026 17:25</t>
+          <t>08/25/2026 17:28</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -11965,7 +11983,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>08/19/2026 02:04</t>
+          <t>08/25/2026 12:52</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12056,7 +12074,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>08/22/2026 08:46</t>
+          <t>08/25/2026 08:49</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12147,7 +12165,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:33</t>
+          <t>08/25/2026 19:18</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12238,7 +12256,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>08/22/2026 02:08</t>
+          <t>08/25/2026 04:45</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12420,7 +12438,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:47</t>
+          <t>08/25/2026 19:41</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12511,7 +12529,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:29</t>
+          <t>08/25/2026 19:12</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12602,7 +12620,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:34</t>
+          <t>08/25/2026 19:26</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12624,17 +12642,23 @@
         <v>0</v>
       </c>
       <c r="N115" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O115" s="9" t="n">
-        <v>0</v>
+        <v>-6156.77</v>
       </c>
       <c r="P115" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q115" s="8" t="n"/>
-      <c r="R115" s="8" t="n"/>
-      <c r="S115" s="8" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="Q115" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="R115" s="9" t="n">
+        <v>0.01160528233794505</v>
+      </c>
+      <c r="S115" s="9" t="n">
+        <v>31.03</v>
+      </c>
       <c r="T115" s="8" t="n">
         <v>0</v>
       </c>
@@ -12794,23 +12818,17 @@
         <v>0</v>
       </c>
       <c r="N117" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O117" s="9" t="n">
-        <v>-58.49</v>
+        <v>0</v>
       </c>
       <c r="P117" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q117" s="9" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="R117" s="9" t="n">
-        <v>0.2666750250752257</v>
-      </c>
-      <c r="S117" s="9" t="n">
-        <v>0.32</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q117" s="8" t="n"/>
+      <c r="R117" s="8" t="n"/>
+      <c r="S117" s="8" t="n"/>
       <c r="T117" s="8" t="n">
         <v>0</v>
       </c>
@@ -12863,7 +12881,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:09</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12948,7 +12966,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:09</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13033,7 +13051,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:25</t>
+          <t>08/25/2026 19:24</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13118,7 +13136,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:09</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13140,23 +13158,17 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>-3715.63</v>
+        <v>0</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q121" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R121" s="9" t="n">
-        <v>0.2438039067238144</v>
-      </c>
-      <c r="S121" s="9" t="n">
-        <v>3.72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q121" s="8" t="n"/>
+      <c r="R121" s="8" t="n"/>
+      <c r="S121" s="8" t="n"/>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13209,7 +13221,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:31</t>
+          <t>08/25/2026 19:12</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13294,7 +13306,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 21:30</t>
+          <t>08/25/2026 19:08</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13379,7 +13391,7 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>08/22/2026 05:52</t>
+          <t>08/25/2026 06:23</t>
         </is>
       </c>
       <c r="H124" s="9" t="n">
@@ -13470,7 +13482,7 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>08/22/2026 04:12</t>
+          <t>08/25/2026 04:59</t>
         </is>
       </c>
       <c r="H125" s="9" t="n">
@@ -13652,7 +13664,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>08/22/2026 10:52</t>
+          <t>08/25/2026 10:54</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13827,7 +13839,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>08/22/2026 07:56</t>
+          <t>08/25/2026 08:04</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -13950,7 +13962,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08/22/2026 17:25</t>
+          <t>08/25/2026 17:28</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -13991,7 +14003,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08/19/2026 02:04</t>
+          <t>08/25/2026 12:52</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14032,7 +14044,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08/22/2026 08:46</t>
+          <t>08/25/2026 08:49</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14073,7 +14085,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/24/2026 21:33</t>
+          <t>08/25/2026 19:18</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14114,7 +14126,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>08/22/2026 02:08</t>
+          <t>08/25/2026 04:45</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14196,7 +14208,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/24/2026 21:47</t>
+          <t>08/25/2026 19:41</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14237,7 +14249,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/24/2026 21:29</t>
+          <t>08/25/2026 19:12</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14278,7 +14290,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/24/2026 21:34</t>
+          <t>08/25/2026 19:26</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14288,7 +14300,7 @@
         <v>-33.06</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -14370,7 +14382,7 @@
         <v>-0.16</v>
       </c>
       <c r="I18" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -14401,7 +14413,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:09</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14442,7 +14454,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:09</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14483,7 +14495,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/24/2026 21:25</t>
+          <t>08/25/2026 19:24</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14524,7 +14536,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/24/2026 21:26</t>
+          <t>08/25/2026 19:09</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14534,7 +14546,7 @@
         <v>-6.66</v>
       </c>
       <c r="I22" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -14565,7 +14577,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/24/2026 21:31</t>
+          <t>08/25/2026 19:12</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14606,7 +14618,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/24/2026 21:30</t>
+          <t>08/25/2026 19:08</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -14647,7 +14659,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>08/22/2026 05:52</t>
+          <t>08/25/2026 06:23</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
@@ -14688,7 +14700,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>08/22/2026 04:12</t>
+          <t>08/25/2026 04:59</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
@@ -14770,7 +14782,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>08/22/2026 10:52</t>
+          <t>08/25/2026 10:54</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
@@ -15786,7 +15798,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08/22/2026 07:14</t>
+          <t>08/25/2026 07:28</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -15832,7 +15844,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08/22/2026 07:00</t>
+          <t>08/25/2026 07:22</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -15855,7 +15867,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08/22/2026 00:26</t>
+          <t>08/25/2026 03:39</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -15901,7 +15913,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08/22/2026 15:07</t>
+          <t>08/25/2026 15:11</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -15924,7 +15936,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08/21/2026 23:40</t>
+          <t>08/25/2026 03:20</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -15947,7 +15959,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08/22/2026 15:16</t>
+          <t>08/25/2026 15:18</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -15993,7 +16005,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08/22/2026 08:12</t>
+          <t>08/25/2026 08:15</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -16039,7 +16051,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08/22/2026 06:55</t>
+          <t>08/25/2026 07:13</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -16131,7 +16143,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08/22/2026 09:18</t>
+          <t>08/25/2026 09:20</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -16154,7 +16166,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08/22/2026 00:12</t>
+          <t>08/25/2026 03:33</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -16177,7 +16189,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/24/2026 19:29</t>
+          <t>08/25/2026 20:54</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16200,7 +16212,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08/22/2026 08:17</t>
+          <t>08/25/2026 08:19</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -16223,11 +16235,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/24/2026 21:36</t>
+          <t>08/25/2026 19:18</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20228.52</v>
+        <v>20136.42</v>
       </c>
     </row>
     <row r="24">
@@ -16269,7 +16281,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/24/2026 18:28</t>
+          <t>08/25/2026 20:09</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -16292,11 +16304,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/24/2026 21:40</t>
+          <t>08/25/2026 19:27</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21419.57</v>
+        <v>21542.07</v>
       </c>
     </row>
     <row r="27">
@@ -16315,7 +16327,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/24/2026 20:20</t>
+          <t>08/25/2026 21:21</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16338,7 +16350,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/24/2026 20:11</t>
+          <t>08/25/2026 21:17</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16361,7 +16373,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/24/2026 20:14</t>
+          <t>08/25/2026 21:18</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16384,7 +16396,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/24/2026 19:55</t>
+          <t>08/25/2026 21:07</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16407,7 +16419,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/24/2026 20:06</t>
+          <t>08/25/2026 21:13</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16430,7 +16442,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/24/2026 20:02</t>
+          <t>08/25/2026 21:11</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16476,11 +16488,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/24/2026 21:40</t>
+          <t>08/25/2026 19:28</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>2914.73</v>
+        <v>2958.29</v>
       </c>
     </row>
     <row r="35">
@@ -16522,7 +16534,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/24/2026 21:19</t>
+          <t>08/25/2026 18:58</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -16545,7 +16557,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/24/2026 21:27</t>
+          <t>08/25/2026 19:02</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -16568,7 +16580,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/24/2026 18:56</t>
+          <t>08/25/2026 20:34</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -16591,11 +16603,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/24/2026 21:37</t>
+          <t>08/25/2026 19:18</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>19975.38</v>
+        <v>19970.13</v>
       </c>
     </row>
     <row r="40">
@@ -16614,11 +16626,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/24/2026 21:39</t>
+          <t>08/25/2026 19:28</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>32004.41</v>
+        <v>32133.53</v>
       </c>
     </row>
     <row r="41">
@@ -16660,7 +16672,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>08/22/2026 06:52</t>
+          <t>08/25/2026 07:16</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -16683,7 +16695,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>08/22/2026 07:42</t>
+          <t>08/25/2026 07:46</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -16706,7 +16718,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>08/22/2026 10:49</t>
+          <t>08/25/2026 10:51</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
@@ -16729,7 +16741,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>08/24/2026 12:36</t>
+          <t>08/25/2026 12:39</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-08-27
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-25 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-26 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/25/2026 18:50</t>
+          <t>08/26/2026 22:50</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>57753.37</v>
-      </c>
-      <c r="I2" t="n">
-        <v>164</v>
+        <v>59600.6</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>172.44</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>9503.240000000002</v>
+        <v>10698</v>
       </c>
       <c r="P2" t="n">
         <v>31</v>
@@ -994,25 +994,25 @@
         <v>77.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.291486198539937</v>
+        <v>1.328132231952497</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>31.5</v>
+        <v>32.04</v>
       </c>
       <c r="T2" t="n">
-        <v>3356</v>
+        <v>3357</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>32753.36999999999</v>
+        <v>34600.59999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2123</v>
+        <v>2124</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.25983313468415</v>
+        <v>63.27077747989276</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/23/2026 19:11</t>
+          <t>08/26/2026 19:13</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/23/2026 17:03</t>
+          <t>08/26/2026 17:05</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/25/2026 21:45</t>
+          <t>08/26/2026 22:35</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/25/2026 21:08</t>
+          <t>08/26/2026 21:22</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/23/2026 21:56</t>
+          <t>08/26/2026 21:59</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/25/2026 20:59</t>
+          <t>08/26/2026 20:59</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/25/2026 19:34</t>
+          <t>08/26/2026 23:37</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:09</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/25/2026 19:17</t>
+          <t>08/26/2026 23:23</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16588.26</v>
+        <v>16542.07</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-16.73</v>
+        <v>-16.96</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,7 +3492,7 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>71.06000000000003</v>
+        <v>54.48000000000003</v>
       </c>
       <c r="P25" t="n">
         <v>19</v>
@@ -3501,10 +3501,10 @@
         <v>47.5</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.174252084355076</v>
+        <v>1.128375512512371</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.71</v>
+        <v>0.66</v>
       </c>
       <c r="T25" t="n">
         <v>703</v>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/25/2026 21:27</t>
+          <t>08/26/2026 22:12</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/25/2026 19:11</t>
+          <t>08/26/2026 23:15</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>19994.53</v>
+        <v>19460.25</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-4.39</v>
+        <v>-6.94</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>7.4</v>
+        <v>8.99</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.74</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,7 +3710,7 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-453.3899999999999</v>
+        <v>-912.1399999999999</v>
       </c>
       <c r="P27" t="n">
         <v>20</v>
@@ -3719,10 +3719,10 @@
         <v>50</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.7730019576134139</v>
+        <v>0.6286195889384711</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>3.43</v>
+        <v>5.11</v>
       </c>
       <c r="T27" t="n">
         <v>110</v>
@@ -3903,11 +3903,11 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/25/2026 19:13</t>
+          <t>08/26/2026 23:16</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19541.42</v>
+        <v>19541.18</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>-2.31</v>
@@ -3943,16 +3943,16 @@
         <v>3.14</v>
       </c>
       <c r="T29" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-458.5800000000003</v>
+        <v>-458.8200000000002</v>
       </c>
       <c r="V29" t="n">
         <v>60</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>48.78048780487805</v>
+        <v>47.61904761904761</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>0.84</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/25/2026 19:19</t>
+          <t>08/26/2026 23:22</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/25/2026 21:02</t>
+          <t>08/26/2026 21:24</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/24/2026 00:17</t>
+          <t>08/27/2026 00:20</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/25/2026 20:35</t>
+          <t>08/27/2026 00:34</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>19904.3</v>
+        <v>20090.8</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>-0.47</v>
+        <v>0.46</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>-95.70000000000013</v>
+        <v>90.79999999999987</v>
       </c>
       <c r="V36" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>49.46236559139785</v>
+        <v>50.52631578947368</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>0.98</v>
+        <v>1.02</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.83</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/25/2026 20:06</t>
+          <t>08/27/2026 00:12</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/23/2026 22:05</t>
+          <t>08/26/2026 22:08</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/25/2026 20:27</t>
+          <t>08/27/2026 00:35</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/25/2026 19:10</t>
+          <t>08/26/2026 23:17</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/25/2026 19:42</t>
+          <t>08/26/2026 23:44</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/25/2026 19:09</t>
+          <t>08/26/2026 23:17</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5638,11 +5638,11 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/25/2026 19:22</t>
+          <t>08/26/2026 23:24</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19782.46</v>
+        <v>19781.72</v>
       </c>
       <c r="I45" s="7" t="n">
         <v>-1.08</v>
@@ -5663,7 +5663,7 @@
         <v>40</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>144.05</v>
+        <v>150.78</v>
       </c>
       <c r="P45" t="n">
         <v>25</v>
@@ -5672,22 +5672,22 @@
         <v>62.5</v>
       </c>
       <c r="R45" s="7" t="n">
-        <v>3.717924528301887</v>
+        <v>4.258698940998487</v>
       </c>
       <c r="S45" s="7" t="n">
         <v>0.1</v>
       </c>
       <c r="T45" t="n">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-217.5400000000001</v>
+        <v>-218.2800000000001</v>
       </c>
       <c r="V45" t="n">
         <v>265</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>56.02536997885835</v>
+        <v>55.78947368421052</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0.93</v>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5747,20 +5747,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/25/2026 18:59</t>
+          <t>08/26/2026 23:00</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19982.08</v>
+        <v>19978.68</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-0.08</v>
+        <v>-0.1</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5769,40 +5769,40 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>19977.76</v>
+        <v>-23.38000000000001</v>
       </c>
       <c r="P46" t="n">
         <v>12</v>
       </c>
       <c r="Q46" s="7" t="n">
-        <v>32.43243243243244</v>
+        <v>30</v>
       </c>
       <c r="R46" s="7" t="n">
-        <v>311.8411389450754</v>
+        <v>0.6648028673835125</v>
       </c>
       <c r="S46" s="7" t="n">
-        <v>0.11</v>
+        <v>0.26</v>
       </c>
       <c r="T46" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-17.92</v>
+        <v>-21.32</v>
       </c>
       <c r="V46" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>30.55555555555556</v>
+        <v>29.26829268292683</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y46" s="7" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5811,12 +5811,12 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC46" t="inlineStr">
@@ -5856,20 +5856,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:06</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>19058.66</v>
+        <v>18891.49</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-4.69</v>
+        <v>-5.52</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.66</v>
+        <v>0.62</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5887,19 +5887,19 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-941.3400000000001</v>
+        <v>-1108.51</v>
       </c>
       <c r="V47" t="n">
         <v>26</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>41.26984126984127</v>
+        <v>39.39393939393939</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.66</v>
+        <v>0.62</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5911,7 +5911,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 22:59</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/25/2026 19:21</t>
+          <t>08/26/2026 23:22</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/25/2026 19:17</t>
+          <t>08/26/2026 23:22</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6187,22 +6187,13 @@
         <v>0</v>
       </c>
       <c r="N50" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>13.93999999999999</v>
+        <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q50" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="R50" s="7" t="n">
-        <v>1.066618876941458</v>
-      </c>
-      <c r="S50" s="7" t="n">
-        <v>0.89</v>
+        <v>0</v>
       </c>
       <c r="T50" t="n">
         <v>1161</v>
@@ -6274,7 +6265,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:09</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6374,20 +6365,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:09</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>20632.26</v>
+        <v>20430.27</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>3.17</v>
+        <v>2.16</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6405,19 +6396,19 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>632.2599999999998</v>
+        <v>430.2699999999998</v>
       </c>
       <c r="V52" t="n">
         <v>12</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>30</v>
+        <v>29.26829268292683</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>10.19</v>
@@ -6429,7 +6420,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6474,20 +6465,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/25/2026 19:28</t>
-        </is>
-      </c>
-      <c r="H53" t="n">
-        <v>19747</v>
+          <t>08/26/2026 23:36</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="n">
+        <v>19752.37</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.29</v>
+        <v>-1.26</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6505,19 +6496,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-253.0000000000001</v>
+        <v>-247.6300000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.20689655172414</v>
+        <v>36.27118644067797</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6529,7 +6520,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6574,7 +6565,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/25/2026 19:40</t>
+          <t>08/26/2026 23:44</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6674,7 +6665,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/25/2026 19:20</t>
+          <t>08/26/2026 23:22</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6774,7 +6765,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/25/2026 19:35</t>
+          <t>08/26/2026 23:41</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6874,14 +6865,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:07</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19716.74</v>
+        <v>19702.92</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.42</v>
+        <v>-1.48</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6905,16 +6896,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>853</v>
+        <v>858</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-283.26</v>
+        <v>-294.1</v>
       </c>
       <c r="V57" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.96248534583822</v>
+        <v>43.82284382284382</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.79</v>
@@ -6929,7 +6920,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6974,7 +6965,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/25/2026 19:14</t>
+          <t>08/26/2026 23:21</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7074,7 +7065,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/25/2026 19:05</t>
+          <t>08/26/2026 23:12</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7096,13 +7087,22 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>0</v>
+        <v>-80.78999999999999</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="Q59" s="7" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="R59" s="7" t="n">
+        <v>0.32387647501883</v>
+      </c>
+      <c r="S59" s="7" t="n">
+        <v>0.43</v>
       </c>
       <c r="T59" t="n">
         <v>304</v>
@@ -7174,7 +7174,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/25/2026 19:13</t>
+          <t>08/26/2026 23:16</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7274,7 +7274,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/25/2026 19:28</t>
+          <t>08/26/2026 23:33</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/25/2026 19:30</t>
+          <t>08/26/2026 23:35</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/25/2026 19:24</t>
+          <t>08/26/2026 23:34</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/25/2026 19:32</t>
+          <t>08/26/2026 23:36</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/25/2026 19:21</t>
+          <t>08/26/2026 23:28</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/25/2026 19:15</t>
+          <t>08/26/2026 23:20</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/25/2026 20:08</t>
+          <t>08/27/2026 00:11</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7974,7 +7974,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/23/2026 21:48</t>
+          <t>08/26/2026 21:50</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/23/2026 21:47</t>
+          <t>08/26/2026 21:50</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/23/2026 21:48</t>
+          <t>08/26/2026 21:50</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/25/2026 19:23</t>
+          <t>08/26/2026 23:28</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8374,7 +8374,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/25/2026 20:14</t>
+          <t>08/27/2026 00:19</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/25/2026 19:28</t>
+          <t>08/26/2026 23:40</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8574,7 +8574,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/25/2026 20:03</t>
+          <t>08/27/2026 00:06</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8674,7 +8674,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/25/2026 19:21</t>
+          <t>08/26/2026 23:24</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/25/2026 19:39</t>
+          <t>08/26/2026 23:44</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8874,7 +8874,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/25/2026 19:25</t>
+          <t>08/26/2026 23:39</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8974,7 +8974,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/25/2026 19:39</t>
+          <t>08/26/2026 23:44</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/25/2026 19:38</t>
+          <t>08/26/2026 23:54</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/25/2026 19:21</t>
+          <t>08/26/2026 23:25</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9274,7 +9274,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/25/2026 20:16</t>
+          <t>08/27/2026 00:16</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9374,7 +9374,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/25/2026 19:39</t>
+          <t>08/26/2026 23:41</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/25/2026 20:13</t>
+          <t>08/27/2026 00:18</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9574,7 +9574,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/25/2026 20:48</t>
+          <t>08/27/2026 00:42</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9674,7 +9674,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/25/2026 20:02</t>
+          <t>08/27/2026 00:11</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9774,20 +9774,20 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/25/2026 20:12</t>
+          <t>08/27/2026 00:17</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20713.74</v>
+        <v>20710.34</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>3.58</v>
+        <v>3.56</v>
       </c>
       <c r="J86" s="7" t="n">
         <v>2.18</v>
       </c>
       <c r="K86" s="7" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="L86" t="n">
         <v>20000</v>
@@ -9805,19 +9805,19 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>713.7400000000001</v>
+        <v>710.3400000000001</v>
       </c>
       <c r="V86" t="n">
         <v>44</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>50</v>
+        <v>48.88888888888889</v>
       </c>
       <c r="X86" s="7" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="Y86" s="7" t="n">
         <v>2.17</v>
@@ -9829,7 +9829,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9874,7 +9874,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/25/2026 19:33</t>
+          <t>08/26/2026 23:35</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9974,20 +9974,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/25/2026 20:02</t>
+          <t>08/27/2026 00:02</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20703.02</v>
+        <v>20702.32</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>3.5</v>
+        <v>3.49</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>0.52</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>4.39</v>
+        <v>3.25</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -10005,19 +10005,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="U88" s="7" t="n">
-        <v>700.26</v>
+        <v>702.3200000000001</v>
       </c>
       <c r="V88" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="W88" s="7" t="n">
-        <v>95.65217391304348</v>
+        <v>94.11764705882352</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>4.38</v>
+        <v>3.25</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>0.52</v>
@@ -10029,7 +10029,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10074,20 +10074,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/25/2026 20:17</t>
+          <t>08/27/2026 00:05</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>22841.48</v>
+        <v>23122.63</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>14.25</v>
+        <v>15.66</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>3.08</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10096,37 +10096,28 @@
         <v>0</v>
       </c>
       <c r="N89" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O89" s="7" t="n">
-        <v>2495.88</v>
+        <v>0</v>
       </c>
       <c r="P89" t="n">
-        <v>29</v>
-      </c>
-      <c r="Q89" s="7" t="n">
-        <v>72.5</v>
-      </c>
-      <c r="R89" s="7" t="n">
-        <v>2.076209284476142</v>
-      </c>
-      <c r="S89" s="7" t="n">
-        <v>3.13</v>
+        <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>2841.48</v>
+        <v>3325.13</v>
       </c>
       <c r="V89" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>73.80952380952381</v>
+        <v>75.55555555555556</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>2.23</v>
+        <v>2.43</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3.08</v>
@@ -10138,7 +10129,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10183,7 +10174,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:07</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -10283,7 +10274,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/25/2026 19:03</t>
+          <t>08/26/2026 23:04</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10383,7 +10374,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/25/2026 19:03</t>
+          <t>08/26/2026 23:07</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10483,7 +10474,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/25/2026 19:03</t>
+          <t>08/26/2026 23:04</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10583,7 +10574,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/25/2026 19:03</t>
+          <t>08/26/2026 23:04</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10679,11 +10670,11 @@
         </is>
       </c>
       <c r="F95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/25/2026 18:58</t>
+          <t>08/26/2026 23:00</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10779,11 +10770,11 @@
         </is>
       </c>
       <c r="F96" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:03</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10879,11 +10870,11 @@
         </is>
       </c>
       <c r="F97" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/25/2026 19:11</t>
+          <t>08/26/2026 23:16</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10979,11 +10970,11 @@
         </is>
       </c>
       <c r="F98" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/25/2026 18:56</t>
+          <t>08/26/2026 22:57</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11079,11 +11070,11 @@
         </is>
       </c>
       <c r="F99" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:07</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11183,7 +11174,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/25/2026 19:33</t>
+          <t>08/26/2026 23:39</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11292,7 +11283,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>08/23/2026 20:59</t>
+          <t>08/26/2026 21:04</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11510,20 +11501,20 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/25/2026 21:45</t>
+          <t>08/26/2026 22:36</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>28108.64</v>
+        <v>28011.47</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-26.8</v>
+        <v>-27.05</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
       </c>
       <c r="K103" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L103" t="n">
         <v>25000</v>
@@ -11535,34 +11526,34 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>-271.17</v>
+        <v>-391.13</v>
       </c>
       <c r="P103" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>47.5</v>
+        <v>40</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>0.3800978419897586</v>
+        <v>0.2096148405609667</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>1.57</v>
+        <v>1.65</v>
       </c>
       <c r="T103" t="n">
-        <v>3542</v>
+        <v>3556</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-6173.360000000001</v>
+        <v>-6270.530000000001</v>
       </c>
       <c r="V103" t="n">
         <v>2170</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>61.26482213438735</v>
+        <v>61.0236220472441</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y103" s="7" t="n">
         <v>37.71</v>
@@ -11574,7 +11565,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11710,7 +11701,7 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>08/23/2026 19:21</t>
+          <t>08/26/2026 19:26</t>
         </is>
       </c>
       <c r="H105" s="9" t="n">
@@ -12165,7 +12156,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:18</t>
+          <t>08/26/2026 23:19</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12347,7 +12338,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>08/23/2026 16:44</t>
+          <t>08/26/2026 16:46</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12438,7 +12429,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:41</t>
+          <t>08/26/2026 23:44</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12529,7 +12520,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:12</t>
+          <t>08/26/2026 23:11</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12620,7 +12611,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:26</t>
+          <t>08/26/2026 23:35</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12796,7 +12787,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>08/23/2026 21:48</t>
+          <t>08/26/2026 21:51</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12881,7 +12872,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:09</t>
+          <t>08/26/2026 23:07</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12966,7 +12957,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:09</t>
+          <t>08/26/2026 23:12</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13051,7 +13042,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:24</t>
+          <t>08/26/2026 23:10</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13136,7 +13127,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:09</t>
+          <t>08/26/2026 23:12</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13158,17 +13149,23 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>0</v>
+        <v>-3715.63</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q121" s="8" t="n"/>
-      <c r="R121" s="8" t="n"/>
-      <c r="S121" s="8" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="Q121" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="R121" s="9" t="n">
+        <v>0.2438039067238144</v>
+      </c>
+      <c r="S121" s="9" t="n">
+        <v>3.72</v>
+      </c>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13221,7 +13218,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:12</t>
+          <t>08/26/2026 23:16</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13306,7 +13303,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 19:08</t>
+          <t>08/26/2026 23:11</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13880,7 +13877,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08/23/2026 19:21</t>
+          <t>08/26/2026 19:26</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -14085,7 +14082,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/25/2026 19:18</t>
+          <t>08/26/2026 23:19</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14167,7 +14164,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/23/2026 16:44</t>
+          <t>08/26/2026 16:46</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14208,7 +14205,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/25/2026 19:41</t>
+          <t>08/26/2026 23:44</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14249,7 +14246,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/25/2026 19:12</t>
+          <t>08/26/2026 23:11</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14290,7 +14287,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/25/2026 19:26</t>
+          <t>08/26/2026 23:35</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14372,7 +14369,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/23/2026 21:48</t>
+          <t>08/26/2026 21:51</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14413,7 +14410,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/25/2026 19:09</t>
+          <t>08/26/2026 23:07</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14454,7 +14451,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/25/2026 19:09</t>
+          <t>08/26/2026 23:12</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14495,7 +14492,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/25/2026 19:24</t>
+          <t>08/26/2026 23:10</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14536,7 +14533,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/25/2026 19:09</t>
+          <t>08/26/2026 23:12</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14546,7 +14543,7 @@
         <v>-6.66</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -14577,7 +14574,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/25/2026 19:12</t>
+          <t>08/26/2026 23:16</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14618,7 +14615,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/25/2026 19:08</t>
+          <t>08/26/2026 23:11</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -14806,7 +14803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -15618,7 +15615,7 @@
         </is>
       </c>
       <c r="D34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -15654,42 +15651,42 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>662434</t>
+          <t>58303</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>EA FX RSI AUDUSD</t>
+          <t>T&amp;D19L13 L8 Prop</t>
         </is>
       </c>
       <c r="D36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>662435</t>
+          <t>58304</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>demo</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Aggv1 Pro Filter 60</t>
+          <t>T&amp;D19L13 L8 MOL</t>
         </is>
       </c>
       <c r="D37" t="b">
@@ -15697,30 +15694,480 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>VPS92t2</t>
+          <t>VPS204</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>58305</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L8 Agg</t>
+        </is>
+      </c>
+      <c r="D38" t="b">
+        <v>0</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>58306</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L11 Prop</t>
+        </is>
+      </c>
+      <c r="D39" t="b">
+        <v>0</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>58307</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L11 MOL</t>
+        </is>
+      </c>
+      <c r="D40" t="b">
+        <v>0</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>58308</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L11 Agg</t>
+        </is>
+      </c>
+      <c r="D41" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>VPS204</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>58318</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L10 Agg</t>
+        </is>
+      </c>
+      <c r="D42" t="b">
+        <v>0</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>58319</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta4 Prop</t>
+        </is>
+      </c>
+      <c r="D43" t="b">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>58320</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta4 MOL</t>
+        </is>
+      </c>
+      <c r="D44" t="b">
+        <v>0</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>58321</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta4 Agg</t>
+        </is>
+      </c>
+      <c r="D45" t="b">
+        <v>0</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>58322</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 Meta4 RCLOCK</t>
+        </is>
+      </c>
+      <c r="D46" t="b">
+        <v>0</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>58323</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 Prop</t>
+        </is>
+      </c>
+      <c r="D47" t="b">
+        <v>0</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>58324</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L10 Prop</t>
+        </is>
+      </c>
+      <c r="D48" t="b">
+        <v>0</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>58325</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 Agg</t>
+        </is>
+      </c>
+      <c r="D49" t="b">
+        <v>0</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>58326</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 Agg Control</t>
+        </is>
+      </c>
+      <c r="D50" t="b">
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>58327</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 MOL</t>
+        </is>
+      </c>
+      <c r="D51" t="b">
+        <v>0</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>58328</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L9 RCLOCK</t>
+        </is>
+      </c>
+      <c r="D52" t="b">
+        <v>0</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>58329</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>T&amp;D19L13 L10 MOL</t>
+        </is>
+      </c>
+      <c r="D53" t="b">
+        <v>0</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>VPS242t3</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>662434</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>EA FX RSI AUDUSD</t>
+        </is>
+      </c>
+      <c r="D54" t="b">
+        <v>1</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>662435</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Aggv1 Pro Filter 60</t>
+        </is>
+      </c>
+      <c r="D55" t="b">
+        <v>0</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>VPS92t2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>600025868</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>demo</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
         <is>
           <t>FTMO Manual Trading</t>
         </is>
       </c>
-      <c r="D38" t="b">
+      <c r="D56" t="b">
         <v>1</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>VPS149</t>
         </is>
@@ -15821,7 +16268,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/23/2026 12:52</t>
+          <t>08/26/2026 12:54</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -15890,7 +16337,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/23/2026 21:11</t>
+          <t>08/26/2026 21:14</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -15982,7 +16429,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/23/2026 15:22</t>
+          <t>08/26/2026 15:24</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -16028,7 +16475,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/23/2026 17:20</t>
+          <t>08/26/2026 17:23</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -16097,7 +16544,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/23/2026 21:20</t>
+          <t>08/26/2026 21:23</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -16120,7 +16567,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/23/2026 21:10</t>
+          <t>08/26/2026 21:15</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -16189,7 +16636,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/25/2026 20:54</t>
+          <t>08/26/2026 20:42</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16235,7 +16682,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/25/2026 19:18</t>
+          <t>08/26/2026 23:23</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
@@ -16281,7 +16728,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/25/2026 20:09</t>
+          <t>08/27/2026 00:15</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -16304,11 +16751,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/25/2026 19:27</t>
+          <t>08/26/2026 23:34</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21542.07</v>
+        <v>21329.83</v>
       </c>
     </row>
     <row r="27">
@@ -16327,7 +16774,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/25/2026 21:21</t>
+          <t>08/26/2026 21:46</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16350,7 +16797,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/25/2026 21:17</t>
+          <t>08/26/2026 21:43</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16373,7 +16820,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/25/2026 21:18</t>
+          <t>08/26/2026 21:51</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16396,7 +16843,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/25/2026 21:07</t>
+          <t>08/26/2026 21:23</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16419,7 +16866,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/25/2026 21:13</t>
+          <t>08/26/2026 21:36</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16442,7 +16889,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/25/2026 21:11</t>
+          <t>08/26/2026 21:32</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16465,7 +16912,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/23/2026 16:59</t>
+          <t>08/26/2026 17:01</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -16488,11 +16935,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/25/2026 19:28</t>
+          <t>08/26/2026 23:34</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>2958.29</v>
+        <v>2999.64</v>
       </c>
     </row>
     <row r="35">
@@ -16534,7 +16981,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/25/2026 18:58</t>
+          <t>08/26/2026 23:00</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -16557,7 +17004,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/25/2026 19:02</t>
+          <t>08/26/2026 23:04</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -16580,11 +17027,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/25/2026 20:34</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>20000</v>
+          <t>08/27/2026 00:34</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>19800.9</v>
       </c>
     </row>
     <row r="39">
@@ -16603,11 +17050,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/25/2026 19:18</t>
+          <t>08/26/2026 23:21</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>19970.13</v>
+        <v>19979.35</v>
       </c>
     </row>
     <row r="40">
@@ -16626,11 +17073,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/25/2026 19:28</t>
+          <t>08/26/2026 23:29</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>32133.53</v>
+        <v>32372.74</v>
       </c>
     </row>
     <row r="41">
@@ -16741,7 +17188,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>08/25/2026 12:39</t>
+          <t>08/26/2026 12:42</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-01
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-26 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-08-31 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/26/2026 22:50</t>
+          <t>08/31/2026 23:53</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>59600.6</v>
+        <v>56588.78</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>172.44</v>
+        <v>158.67</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.1</v>
+        <v>1.09</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,7 +985,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>10698</v>
+        <v>4312.130000000001</v>
       </c>
       <c r="P2" t="n">
         <v>31</v>
@@ -994,25 +994,25 @@
         <v>77.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.328132231952497</v>
+        <v>1.115612560529206</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>32.04</v>
+        <v>34.95</v>
       </c>
       <c r="T2" t="n">
-        <v>3357</v>
+        <v>3364</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>34600.59999999999</v>
+        <v>31588.77999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2124</v>
+        <v>2131</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.27077747989276</v>
+        <v>63.34720570749109</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>08/25/2026 04:11</t>
+          <t>08/31/2026 04:12</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/26/2026 19:13</t>
+          <t>08/29/2026 19:15</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/24/2026 09:00</t>
+          <t>08/30/2026 09:10</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08/25/2026 17:19</t>
+          <t>08/31/2026 17:41</t>
         </is>
       </c>
       <c r="H7" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/26/2026 17:05</t>
+          <t>08/29/2026 17:07</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08/25/2026 08:49</t>
+          <t>08/31/2026 08:53</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>08/25/2026 10:34</t>
+          <t>08/31/2026 10:37</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>08/25/2026 10:36</t>
+          <t>08/31/2026 10:40</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2159,20 +2159,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/26/2026 22:35</t>
+          <t>08/31/2026 23:31</t>
         </is>
       </c>
       <c r="H13" s="7" t="n">
-        <v>5198.67</v>
+        <v>5105.06</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>-1.06</v>
+        <v>-2.84</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>8.949999999999999</v>
+        <v>10.41</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>1.14</v>
+        <v>1.04</v>
       </c>
       <c r="L13" t="n">
         <v>20000</v>
@@ -2184,7 +2184,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>-4788.8</v>
+        <v>-4917.41</v>
       </c>
       <c r="P13" t="n">
         <v>30</v>
@@ -2193,28 +2193,28 @@
         <v>75</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>0.6953612051197231</v>
+        <v>0.6894156865791646</v>
       </c>
       <c r="S13" s="7" t="n">
-        <v>98.2</v>
+        <v>99.09</v>
       </c>
       <c r="T13" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>132.1699999999999</v>
+        <v>38.55999999999992</v>
       </c>
       <c r="V13" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>67.74193548387096</v>
+        <v>67.69230769230769</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>1.14</v>
+        <v>1.04</v>
       </c>
       <c r="Y13" s="7" t="n">
-        <v>12.26</v>
+        <v>13.67</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>08/25/2026 04:44</t>
+          <t>08/31/2026 04:40</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/24/2026 10:17</t>
+          <t>08/30/2026 10:23</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/26/2026 21:22</t>
+          <t>08/31/2026 22:49</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/26/2026 21:59</t>
+          <t>08/29/2026 22:00</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>08/24/2026 13:03</t>
+          <t>08/30/2026 13:06</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>08/24/2026 05:49</t>
+          <t>08/30/2026 05:52</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>08/24/2026 05:49</t>
+          <t>08/30/2026 05:52</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/26/2026 20:59</t>
+          <t>08/31/2026 22:32</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>08/26/2026 23:37</t>
+          <t>09/01/2026 00:27</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/26/2026 23:09</t>
+          <t>08/31/2026 23:59</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19882.68</v>
+        <v>19736.81</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-0.58</v>
+        <v>-1.31</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.1</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,34 +3274,34 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>193.89</v>
+        <v>33.27</v>
       </c>
       <c r="P23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="Q23" s="7" t="n">
-        <v>55.00000000000001</v>
+        <v>52.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.093769042529525</v>
+        <v>1.015014418715899</v>
       </c>
       <c r="S23" s="7" t="n">
         <v>4.22</v>
       </c>
       <c r="T23" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-117.3199999999999</v>
+        <v>-263.1899999999999</v>
       </c>
       <c r="V23" t="n">
         <v>43</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>53.75</v>
+        <v>53.08641975308642</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>6.11</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>08/25/2026 04:36</t>
+          <t>08/31/2026 04:34</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
@@ -3398,7 +3398,7 @@
         <v>0.7</v>
       </c>
       <c r="T24" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="U24" s="7" t="n">
         <v>-195.13</v>
@@ -3407,7 +3407,7 @@
         <v>14</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>35.8974358974359</v>
+        <v>31.81818181818182</v>
       </c>
       <c r="X24" s="7" t="n">
         <v>0.5</v>
@@ -3422,17 +3422,17 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>OK (small account, full sample)</t>
+          <t>RECONCILE</t>
         </is>
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>Bar Reversal MOL Bots | AUDUSD.pro, Bar Reversal MOL Bots | CHFJPY.pro, Bar Reversal MOL Bots | EURCAD.pro, Bar Reversal MOL Bots | EURUSD.pro, Bar Reversal MOL Bots | GBPJPY.pro, Bar Reversal MOL Bots | GBPNZD.pro, Bar Reversal MOL Bots | USDCAD.pro</t>
+          <t>Bar Reversal MOL Bots | AUDUSD.pro, Bar Reversal MOL Bots | CHFJPY.pro, Bar Reversal MOL Bots | EURCAD.pro, Bar Reversal MOL Bots | EURJPY.pro, Bar Reversal MOL Bots | EURUSD.pro, Bar Reversal MOL Bots | GBPJPY.pro, Bar Reversal MOL Bots | GBPNZD.pro, Bar Reversal MOL Bots | USDCAD.pro</t>
         </is>
       </c>
     </row>
@@ -3467,14 +3467,14 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>08/26/2026 23:23</t>
+          <t>09/01/2026 00:12</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16542.07</v>
+        <v>16571.33</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-16.96</v>
+        <v>-16.81</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
@@ -3492,19 +3492,19 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>54.48000000000003</v>
+        <v>104.52</v>
       </c>
       <c r="P25" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>47.5</v>
+        <v>50</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.128375512512371</v>
+        <v>1.258969276511397</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="T25" t="n">
         <v>703</v>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/26/2026 22:12</t>
+          <t>08/30/2026 22:50</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>08/26/2026 23:15</t>
+          <t>09/01/2026 00:04</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>08/25/2026 08:15</t>
+          <t>08/31/2026 08:20</t>
         </is>
       </c>
       <c r="H28" s="7" t="n">
@@ -3903,14 +3903,14 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>08/26/2026 23:16</t>
+          <t>09/01/2026 00:09</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19541.18</v>
+        <v>19537.07</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-2.31</v>
+        <v>-2.33</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
@@ -3928,7 +3928,7 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-624.87</v>
+        <v>-617.73</v>
       </c>
       <c r="P29" t="n">
         <v>15</v>
@@ -3937,22 +3937,22 @@
         <v>37.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.3034478146005418</v>
+        <v>0.3058823529411765</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>3.14</v>
+        <v>3.15</v>
       </c>
       <c r="T29" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-458.8200000000002</v>
+        <v>-462.9300000000001</v>
       </c>
       <c r="V29" t="n">
         <v>60</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>47.61904761904761</v>
+        <v>46.51162790697674</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>0.84</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>08/25/2026 17:51</t>
+          <t>08/31/2026 17:54</t>
         </is>
       </c>
       <c r="H30" s="7" t="n">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>08/26/2026 23:22</t>
+          <t>09/01/2026 00:12</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/24/2026 10:21</t>
+          <t>08/30/2026 10:26</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>08/24/2026 11:12</t>
+          <t>08/30/2026 11:16</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/26/2026 21:24</t>
+          <t>08/31/2026 22:40</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/27/2026 00:20</t>
+          <t>08/30/2026 00:21</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/27/2026 00:34</t>
+          <t>08/31/2026 22:05</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>20090.8</v>
+        <v>20284.45</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>0.46</v>
+        <v>1.43</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>1.02</v>
+        <v>1.06</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>90.79999999999987</v>
+        <v>284.4499999999999</v>
       </c>
       <c r="V36" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>50.52631578947368</v>
+        <v>51.51515151515152</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>1.02</v>
+        <v>1.06</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.83</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/27/2026 00:12</t>
+          <t>08/31/2026 21:45</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/26/2026 22:08</t>
+          <t>08/29/2026 22:10</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/27/2026 00:35</t>
+          <t>08/29/2026 14:33</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>08/25/2026 17:06</t>
+          <t>08/31/2026 17:11</t>
         </is>
       </c>
       <c r="H40" s="7" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>08/22/2026 16:31</t>
+          <t>08/31/2026 16:39</t>
         </is>
       </c>
       <c r="H41" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08/26/2026 23:17</t>
+          <t>09/01/2026 00:08</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08/26/2026 23:44</t>
+          <t>09/01/2026 00:27</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5442,22 +5442,13 @@
         <v>0</v>
       </c>
       <c r="N43" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>-50.87</v>
+        <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q43" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="R43" s="7" t="n">
-        <v>0.2037877602128658</v>
-      </c>
-      <c r="S43" s="7" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="T43" t="n">
         <v>4278</v>
@@ -5529,7 +5520,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08/26/2026 23:17</t>
+          <t>09/01/2026 00:05</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5551,22 +5542,13 @@
         <v>0</v>
       </c>
       <c r="N44" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>-1124.46</v>
+        <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q44" s="7" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="R44" s="7" t="n">
-        <v>0.4043290318479436</v>
-      </c>
-      <c r="S44" s="7" t="n">
-        <v>5.73</v>
+        <v>0</v>
       </c>
       <c r="T44" t="n">
         <v>57</v>
@@ -5638,14 +5620,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>08/26/2026 23:24</t>
+          <t>09/01/2026 00:16</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19781.72</v>
+        <v>19794.87</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-1.08</v>
+        <v>-1.01</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>4.38</v>
@@ -5660,34 +5642,25 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>150.78</v>
+        <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>25</v>
-      </c>
-      <c r="Q45" s="7" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="R45" s="7" t="n">
-        <v>4.258698940998487</v>
-      </c>
-      <c r="S45" s="7" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-218.2800000000001</v>
+        <v>-205.1300000000001</v>
       </c>
       <c r="V45" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>55.78947368421052</v>
+        <v>55.9748427672956</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0.93</v>
@@ -5702,7 +5675,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5747,20 +5720,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>08/26/2026 23:00</t>
+          <t>09/01/2026 00:08</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19978.68</v>
+        <v>19982.25</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-0.1</v>
+        <v>-0.08</v>
       </c>
       <c r="J46" s="7" t="n">
         <v>0.23</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.74</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5769,37 +5742,28 @@
         <v>0</v>
       </c>
       <c r="N46" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>-23.38000000000001</v>
+        <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q46" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="R46" s="7" t="n">
-        <v>0.6648028673835125</v>
-      </c>
-      <c r="S46" s="7" t="n">
-        <v>0.26</v>
+        <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-21.32</v>
+        <v>-17.75</v>
       </c>
       <c r="V46" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>29.26829268292683</v>
+        <v>30.95238095238095</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.74</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>0.24</v>
@@ -5811,7 +5775,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5856,20 +5820,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>08/26/2026 23:06</t>
+          <t>09/01/2026 00:00</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>18891.49</v>
+        <v>18812.85</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-5.52</v>
+        <v>-5.91</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5887,19 +5851,19 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-1108.51</v>
+        <v>-1187.15</v>
       </c>
       <c r="V47" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>39.39393939393939</v>
+        <v>38.57142857142858</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5911,7 +5875,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5956,7 +5920,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/26/2026 22:59</t>
+          <t>08/31/2026 23:54</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -5978,22 +5942,13 @@
         <v>0</v>
       </c>
       <c r="N48" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>504.68</v>
+        <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>24</v>
-      </c>
-      <c r="Q48" s="7" t="n">
-        <v>60</v>
-      </c>
-      <c r="R48" s="7" t="n">
-        <v>2.47982641332395</v>
-      </c>
-      <c r="S48" s="7" t="n">
-        <v>1.7</v>
+        <v>0</v>
       </c>
       <c r="T48" t="n">
         <v>193</v>
@@ -6065,7 +6020,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>08/26/2026 23:22</t>
+          <t>09/01/2026 00:20</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6165,7 +6120,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>08/26/2026 23:22</t>
+          <t>09/01/2026 00:13</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6265,7 +6220,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>08/26/2026 23:09</t>
+          <t>09/01/2026 00:00</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6365,20 +6320,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/26/2026 23:09</t>
+          <t>08/31/2026 23:54</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>20430.27</v>
+        <v>20497.37</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>2.16</v>
+        <v>2.5</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6396,19 +6351,19 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>430.2699999999998</v>
+        <v>497.3699999999997</v>
       </c>
       <c r="V52" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>29.26829268292683</v>
+        <v>30.23255813953488</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>10.19</v>
@@ -6420,7 +6375,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6465,20 +6420,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>08/26/2026 23:36</t>
+          <t>09/01/2026 00:32</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19752.37</v>
+        <v>19697.63</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.26</v>
+        <v>-1.54</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.76</v>
+        <v>0.72</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6496,19 +6451,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>295</v>
+        <v>313</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-247.6300000000001</v>
+        <v>-302.3700000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>36.27118644067797</v>
+        <v>35.14376996805112</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.76</v>
+        <v>0.72</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6520,7 +6475,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6565,7 +6520,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>08/26/2026 23:44</t>
+          <t>09/01/2026 00:33</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6665,7 +6620,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>08/26/2026 23:22</t>
+          <t>09/01/2026 00:14</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6765,7 +6720,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>08/26/2026 23:41</t>
+          <t>09/01/2026 00:32</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6865,14 +6820,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/26/2026 23:07</t>
+          <t>08/31/2026 23:54</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19702.92</v>
+        <v>19708.39</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.48</v>
+        <v>-1.44</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6896,16 +6851,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>858</v>
+        <v>881</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-294.1</v>
+        <v>-290.6500000000001</v>
       </c>
       <c r="V57" t="n">
-        <v>376</v>
+        <v>387</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.82284382284382</v>
+        <v>43.92735527809307</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.79</v>
@@ -6920,7 +6875,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6965,7 +6920,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>08/26/2026 23:21</t>
+          <t>09/01/2026 00:11</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7065,7 +7020,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>08/26/2026 23:12</t>
+          <t>09/01/2026 00:07</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7087,22 +7042,13 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>-80.78999999999999</v>
+        <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q59" s="7" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="R59" s="7" t="n">
-        <v>0.32387647501883</v>
-      </c>
-      <c r="S59" s="7" t="n">
-        <v>0.43</v>
+        <v>0</v>
       </c>
       <c r="T59" t="n">
         <v>304</v>
@@ -7174,7 +7120,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>08/26/2026 23:16</t>
+          <t>09/01/2026 00:08</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7274,7 +7220,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>08/26/2026 23:33</t>
+          <t>09/01/2026 00:26</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7374,7 +7320,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/26/2026 23:35</t>
+          <t>08/30/2026 20:53</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7474,20 +7420,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>08/26/2026 23:34</t>
+          <t>09/01/2026 00:20</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
-        <v>18680.7</v>
+        <v>18592.24</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>-6.61</v>
+        <v>-7.06</v>
       </c>
       <c r="J63" s="7" t="n">
         <v>7.22</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="L63" t="n">
         <v>20000</v>
@@ -7505,19 +7451,19 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="U63" s="7" t="n">
-        <v>-1319.3</v>
+        <v>-1407.76</v>
       </c>
       <c r="V63" t="n">
         <v>5</v>
       </c>
       <c r="W63" s="7" t="n">
-        <v>10.63829787234043</v>
+        <v>10</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="Y63" s="7" t="n">
         <v>7.21</v>
@@ -7529,7 +7475,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7574,7 +7520,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>08/26/2026 23:36</t>
+          <t>09/01/2026 00:27</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
@@ -7674,7 +7620,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>08/26/2026 23:28</t>
+          <t>09/01/2026 00:21</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
@@ -7774,7 +7720,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>08/26/2026 23:20</t>
+          <t>09/01/2026 00:10</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
@@ -7874,7 +7820,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/27/2026 00:11</t>
+          <t>08/31/2026 21:43</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7974,7 +7920,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/26/2026 21:50</t>
+          <t>08/29/2026 21:52</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8074,7 +8020,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/26/2026 21:50</t>
+          <t>08/29/2026 21:52</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8174,7 +8120,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/26/2026 21:50</t>
+          <t>08/29/2026 21:52</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8274,7 +8220,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>08/26/2026 23:28</t>
+          <t>09/01/2026 00:21</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8374,7 +8320,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/27/2026 00:19</t>
+          <t>08/31/2026 21:50</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8474,7 +8420,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>08/26/2026 23:40</t>
+          <t>09/01/2026 00:23</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8574,7 +8520,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/27/2026 00:06</t>
+          <t>08/31/2026 21:55</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8674,7 +8620,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>08/26/2026 23:24</t>
+          <t>09/01/2026 00:19</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8774,7 +8720,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>08/26/2026 23:44</t>
+          <t>09/01/2026 00:34</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8874,7 +8820,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08/26/2026 23:39</t>
+          <t>09/01/2026 00:37</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8974,7 +8920,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08/26/2026 23:44</t>
+          <t>09/01/2026 00:34</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9074,7 +9020,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>08/26/2026 23:54</t>
+          <t>09/01/2026 00:31</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9174,7 +9120,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>08/26/2026 23:25</t>
+          <t>09/01/2026 00:19</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9274,7 +9220,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/27/2026 00:16</t>
+          <t>08/31/2026 21:44</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9374,7 +9320,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>08/26/2026 23:41</t>
+          <t>09/01/2026 00:34</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9474,7 +9420,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/27/2026 00:18</t>
+          <t>08/31/2026 21:53</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9574,7 +9520,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/27/2026 00:42</t>
+          <t>08/31/2026 22:20</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9674,7 +9620,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/27/2026 00:11</t>
+          <t>08/31/2026 21:41</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9774,20 +9720,20 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/27/2026 00:17</t>
+          <t>08/31/2026 21:45</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20710.34</v>
+        <v>20388.17</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>3.56</v>
+        <v>1.95</v>
       </c>
       <c r="J86" s="7" t="n">
-        <v>2.18</v>
+        <v>2.51</v>
       </c>
       <c r="K86" s="7" t="n">
-        <v>1.71</v>
+        <v>1.29</v>
       </c>
       <c r="L86" t="n">
         <v>20000</v>
@@ -9805,22 +9751,22 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>710.3400000000001</v>
+        <v>388.1700000000001</v>
       </c>
       <c r="V86" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>48.88888888888889</v>
+        <v>46.53465346534654</v>
       </c>
       <c r="X86" s="7" t="n">
-        <v>1.71</v>
+        <v>1.29</v>
       </c>
       <c r="Y86" s="7" t="n">
-        <v>2.17</v>
+        <v>2.51</v>
       </c>
       <c r="Z86" t="inlineStr">
         <is>
@@ -9829,7 +9775,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9874,7 +9820,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>08/26/2026 23:35</t>
+          <t>09/01/2026 00:25</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9974,20 +9920,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/27/2026 00:02</t>
+          <t>08/31/2026 21:41</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20702.32</v>
+        <v>20177.38</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>3.49</v>
+        <v>0.87</v>
       </c>
       <c r="J88" s="7" t="n">
-        <v>0.52</v>
+        <v>2.69</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>3.25</v>
+        <v>1.19</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -10005,22 +9951,22 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="U88" s="7" t="n">
-        <v>702.3200000000001</v>
+        <v>177.38</v>
       </c>
       <c r="V88" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="W88" s="7" t="n">
-        <v>94.11764705882352</v>
+        <v>85.48387096774194</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>3.25</v>
+        <v>1.19</v>
       </c>
       <c r="Y88" s="7" t="n">
-        <v>0.52</v>
+        <v>2.7</v>
       </c>
       <c r="Z88" t="inlineStr">
         <is>
@@ -10029,7 +9975,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10074,20 +10020,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/27/2026 00:05</t>
+          <t>08/31/2026 21:41</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>23122.63</v>
+        <v>23570.7</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>15.66</v>
+        <v>17.91</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>3.08</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>2.24</v>
+        <v>2.28</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10105,19 +10051,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>3325.13</v>
+        <v>3570.7</v>
       </c>
       <c r="V89" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>75.55555555555556</v>
+        <v>72.72727272727273</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>2.43</v>
+        <v>2.28</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3.08</v>
@@ -10129,7 +10075,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10174,7 +10120,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>08/26/2026 23:07</t>
+          <t>09/01/2026 00:01</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -10274,7 +10220,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>08/26/2026 23:04</t>
+          <t>09/01/2026 00:01</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10374,7 +10320,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>08/26/2026 23:07</t>
+          <t>09/01/2026 00:03</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10474,7 +10420,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/26/2026 23:04</t>
+          <t>08/31/2026 23:57</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10574,7 +10520,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/26/2026 23:04</t>
+          <t>08/31/2026 23:57</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10674,7 +10620,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/26/2026 23:00</t>
+          <t>08/31/2026 23:54</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10774,7 +10720,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>08/26/2026 23:03</t>
+          <t>09/01/2026 00:00</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10874,7 +10820,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>08/26/2026 23:16</t>
+          <t>09/01/2026 00:09</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10974,7 +10920,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/26/2026 22:57</t>
+          <t>08/31/2026 23:51</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11074,7 +11020,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>08/26/2026 23:07</t>
+          <t>09/01/2026 00:01</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11174,7 +11120,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>08/26/2026 23:39</t>
+          <t>09/01/2026 00:29</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11283,7 +11229,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>08/26/2026 21:04</t>
+          <t>08/29/2026 21:03</t>
         </is>
       </c>
       <c r="H101" s="7" t="n">
@@ -11357,7 +11303,7 @@
       </c>
       <c r="AC101" t="inlineStr">
         <is>
-          <t>Gold Talon | EURUSD.PRO, Gold Talon | XAUUSD.PRO</t>
+          <t>Gold Talon V1.2 | EURUSD.PRO, Gold Talon V1.2 | XAUUSD.PRO</t>
         </is>
       </c>
     </row>
@@ -11392,7 +11338,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>08/25/2026 08:49</t>
+          <t>08/31/2026 08:53</t>
         </is>
       </c>
       <c r="H102" s="7" t="n">
@@ -11501,20 +11447,20 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/26/2026 22:36</t>
+          <t>08/31/2026 23:30</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>28011.47</v>
+        <v>28245.15</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-27.05</v>
+        <v>-26.44</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
       </c>
       <c r="K103" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="L103" t="n">
         <v>25000</v>
@@ -11526,34 +11472,34 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>-391.13</v>
+        <v>203.53</v>
       </c>
       <c r="P103" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>0.2096148405609667</v>
+        <v>3.769115646258503</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>1.65</v>
+        <v>0.29</v>
       </c>
       <c r="T103" t="n">
-        <v>3556</v>
+        <v>3602</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-6270.530000000001</v>
+        <v>-6036.85</v>
       </c>
       <c r="V103" t="n">
-        <v>2170</v>
+        <v>2207</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>61.0236220472441</v>
+        <v>61.27151582454192</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="Y103" s="7" t="n">
         <v>37.71</v>
@@ -11565,7 +11511,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11610,7 +11556,7 @@
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 08:04</t>
+          <t>08/31/2026 08:03</t>
         </is>
       </c>
       <c r="H104" s="9" t="n">
@@ -11701,7 +11647,7 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 19:26</t>
+          <t>08/29/2026 19:33</t>
         </is>
       </c>
       <c r="H105" s="9" t="n">
@@ -11792,7 +11738,7 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 16:30</t>
+          <t>08/30/2026 16:33</t>
         </is>
       </c>
       <c r="H106" s="9" t="n">
@@ -11883,7 +11829,7 @@
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 17:28</t>
+          <t>08/31/2026 17:44</t>
         </is>
       </c>
       <c r="H107" s="9" t="n">
@@ -11974,7 +11920,7 @@
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 12:52</t>
+          <t>08/31/2026 12:55</t>
         </is>
       </c>
       <c r="H108" s="9" t="n">
@@ -12065,7 +12011,7 @@
       </c>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 08:49</t>
+          <t>08/31/2026 08:52</t>
         </is>
       </c>
       <c r="H109" s="9" t="n">
@@ -12156,7 +12102,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:19</t>
+          <t>08/29/2026 12:49</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12247,7 +12193,7 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 04:45</t>
+          <t>08/31/2026 04:29</t>
         </is>
       </c>
       <c r="H111" s="9" t="n">
@@ -12338,7 +12284,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 16:46</t>
+          <t>08/29/2026 16:48</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12429,7 +12375,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:44</t>
+          <t>09/01/2026 00:30</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12520,7 +12466,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:11</t>
+          <t>09/01/2026 00:05</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12542,23 +12488,17 @@
         <v>0</v>
       </c>
       <c r="N114" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O114" s="9" t="n">
-        <v>67.93000000000001</v>
+        <v>0</v>
       </c>
       <c r="P114" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q114" s="9" t="n">
-        <v>65</v>
-      </c>
-      <c r="R114" s="9" t="n">
-        <v>1.223174978645115</v>
-      </c>
-      <c r="S114" s="9" t="n">
-        <v>0.57</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q114" s="8" t="n"/>
+      <c r="R114" s="8" t="n"/>
+      <c r="S114" s="8" t="n"/>
       <c r="T114" s="8" t="n">
         <v>0</v>
       </c>
@@ -12611,7 +12551,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:35</t>
+          <t>08/30/2026 20:39</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12633,23 +12573,17 @@
         <v>0</v>
       </c>
       <c r="N115" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O115" s="9" t="n">
-        <v>-6156.77</v>
+        <v>0</v>
       </c>
       <c r="P115" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q115" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="R115" s="9" t="n">
-        <v>0.01160528233794505</v>
-      </c>
-      <c r="S115" s="9" t="n">
-        <v>31.03</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q115" s="8" t="n"/>
+      <c r="R115" s="8" t="n"/>
+      <c r="S115" s="8" t="n"/>
       <c r="T115" s="8" t="n">
         <v>0</v>
       </c>
@@ -12702,7 +12636,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>08/24/2026 14:57</t>
+          <t>08/30/2026 15:00</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12787,7 +12721,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 21:51</t>
+          <t>08/29/2026 21:52</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12872,7 +12806,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:07</t>
+          <t>09/01/2026 00:01</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12957,7 +12891,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:12</t>
+          <t>09/01/2026 00:02</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -13042,7 +12976,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:10</t>
+          <t>09/01/2026 00:01</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13127,7 +13061,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:12</t>
+          <t>09/01/2026 00:03</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13149,23 +13083,17 @@
         <v>0</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O121" s="9" t="n">
-        <v>-3715.63</v>
+        <v>0</v>
       </c>
       <c r="P121" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q121" s="9" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="R121" s="9" t="n">
-        <v>0.2438039067238144</v>
-      </c>
-      <c r="S121" s="9" t="n">
-        <v>3.72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q121" s="8" t="n"/>
+      <c r="R121" s="8" t="n"/>
+      <c r="S121" s="8" t="n"/>
       <c r="T121" s="8" t="n">
         <v>0</v>
       </c>
@@ -13218,7 +13146,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:16</t>
+          <t>09/01/2026 00:14</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13303,7 +13231,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>08/26/2026 23:11</t>
+          <t>09/01/2026 00:21</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13388,11 +13316,11 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 06:23</t>
-        </is>
-      </c>
-      <c r="H124" s="9" t="n">
-        <v>5027.65</v>
+          <t>08/31/2026 06:10</t>
+        </is>
+      </c>
+      <c r="H124" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="I124" s="9" t="n">
         <v>42.67</v>
@@ -13407,25 +13335,25 @@
         <v>570933.12</v>
       </c>
       <c r="M124" s="9" t="n">
-        <v>600632.65</v>
+        <v>605660.3</v>
       </c>
       <c r="N124" s="8" t="n">
         <v>40</v>
       </c>
       <c r="O124" s="9" t="n">
-        <v>-74273.92</v>
+        <v>-79301.63</v>
       </c>
       <c r="P124" s="8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Q124" s="9" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="R124" s="9" t="n">
-        <v>0.06452367787659215</v>
+        <v>0.06068045373057955</v>
       </c>
       <c r="S124" s="9" t="n">
-        <v>788.87</v>
+        <v>838.85</v>
       </c>
       <c r="T124" s="8" t="n">
         <v>0</v>
@@ -13479,11 +13407,11 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 04:59</t>
-        </is>
-      </c>
-      <c r="H125" s="9" t="n">
-        <v>4879.61</v>
+          <t>08/31/2026 04:54</t>
+        </is>
+      </c>
+      <c r="H125" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="I125" s="9" t="n">
         <v>-27.8</v>
@@ -13498,13 +13426,13 @@
         <v>95000</v>
       </c>
       <c r="M125" s="9" t="n">
-        <v>75748.57000000001</v>
+        <v>80628.17999999999</v>
       </c>
       <c r="N125" s="8" t="n">
         <v>40</v>
       </c>
       <c r="O125" s="9" t="n">
-        <v>-40619.29</v>
+        <v>-44109.12</v>
       </c>
       <c r="P125" s="8" t="n">
         <v>16</v>
@@ -13513,10 +13441,10 @@
         <v>40</v>
       </c>
       <c r="R125" s="9" t="n">
-        <v>0.1140036762292105</v>
+        <v>0.105939469414858</v>
       </c>
       <c r="S125" s="9" t="n">
-        <v>236.08</v>
+        <v>306.91</v>
       </c>
       <c r="T125" s="8" t="n">
         <v>0</v>
@@ -13661,7 +13589,7 @@
       </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t>08/25/2026 10:54</t>
+          <t>08/31/2026 10:59</t>
         </is>
       </c>
       <c r="H127" s="9" t="n">
@@ -13836,7 +13764,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>08/25/2026 08:04</t>
+          <t>08/31/2026 08:03</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
@@ -13877,7 +13805,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08/26/2026 19:26</t>
+          <t>08/29/2026 19:33</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -13918,7 +13846,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08/24/2026 16:30</t>
+          <t>08/30/2026 16:33</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -13959,7 +13887,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>08/25/2026 17:28</t>
+          <t>08/31/2026 17:44</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -14000,7 +13928,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>08/25/2026 12:52</t>
+          <t>08/31/2026 12:55</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
@@ -14041,7 +13969,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>08/25/2026 08:49</t>
+          <t>08/31/2026 08:52</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -14082,7 +14010,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/26/2026 23:19</t>
+          <t>08/29/2026 12:49</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14123,7 +14051,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>08/25/2026 04:45</t>
+          <t>08/31/2026 04:29</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -14164,7 +14092,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/26/2026 16:46</t>
+          <t>08/29/2026 16:48</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14205,7 +14133,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>08/26/2026 23:44</t>
+          <t>09/01/2026 00:30</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14246,7 +14174,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>08/26/2026 23:11</t>
+          <t>09/01/2026 00:05</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14256,7 +14184,7 @@
         <v>2.96</v>
       </c>
       <c r="I15" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -14287,7 +14215,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/26/2026 23:35</t>
+          <t>08/30/2026 20:39</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14297,7 +14225,7 @@
         <v>-33.06</v>
       </c>
       <c r="I16" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -14328,7 +14256,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/24/2026 14:57</t>
+          <t>08/30/2026 15:00</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14369,7 +14297,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/26/2026 21:51</t>
+          <t>08/29/2026 21:52</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14410,7 +14338,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>08/26/2026 23:07</t>
+          <t>09/01/2026 00:01</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14451,7 +14379,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>08/26/2026 23:12</t>
+          <t>09/01/2026 00:02</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14492,7 +14420,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>08/26/2026 23:10</t>
+          <t>09/01/2026 00:01</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14533,7 +14461,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>08/26/2026 23:12</t>
+          <t>09/01/2026 00:03</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14543,7 +14471,7 @@
         <v>-6.66</v>
       </c>
       <c r="I22" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -14574,7 +14502,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>08/26/2026 23:16</t>
+          <t>09/01/2026 00:14</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14615,7 +14543,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>08/26/2026 23:11</t>
+          <t>09/01/2026 00:21</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -14656,11 +14584,11 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>08/25/2026 06:23</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="n">
-        <v>5027.65</v>
+          <t>08/31/2026 06:10</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
       </c>
       <c r="H25" s="7" t="n">
         <v>42.67</v>
@@ -14697,11 +14625,11 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>08/25/2026 04:59</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>4879.61</v>
+          <t>08/31/2026 04:54</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
       </c>
       <c r="H26" s="7" t="n">
         <v>-27.8</v>
@@ -14779,7 +14707,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>08/25/2026 10:54</t>
+          <t>08/31/2026 10:59</t>
         </is>
       </c>
       <c r="G28" s="7" t="n">
@@ -16245,7 +16173,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>08/25/2026 07:28</t>
+          <t>08/31/2026 07:21</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -16268,7 +16196,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/26/2026 12:54</t>
+          <t>08/29/2026 12:56</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -16291,7 +16219,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>08/25/2026 07:22</t>
+          <t>08/31/2026 07:11</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -16314,7 +16242,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>08/25/2026 03:39</t>
+          <t>08/31/2026 03:45</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -16337,7 +16265,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/26/2026 21:14</t>
+          <t>08/29/2026 21:16</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -16360,7 +16288,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>08/25/2026 15:11</t>
+          <t>08/31/2026 15:14</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -16383,7 +16311,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>08/25/2026 03:20</t>
+          <t>08/31/2026 03:26</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -16406,7 +16334,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>08/25/2026 15:18</t>
+          <t>08/31/2026 15:22</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -16429,7 +16357,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/26/2026 15:24</t>
+          <t>08/29/2026 15:27</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -16452,7 +16380,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>08/25/2026 08:15</t>
+          <t>08/31/2026 08:20</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -16475,7 +16403,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/26/2026 17:23</t>
+          <t>08/29/2026 17:24</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -16498,7 +16426,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>08/25/2026 07:13</t>
+          <t>08/31/2026 07:08</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -16544,7 +16472,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/26/2026 21:23</t>
+          <t>08/29/2026 21:24</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -16567,7 +16495,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/26/2026 21:15</t>
+          <t>08/29/2026 21:15</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -16590,7 +16518,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>08/25/2026 09:20</t>
+          <t>08/31/2026 09:23</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -16613,7 +16541,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>08/25/2026 03:33</t>
+          <t>08/31/2026 03:40</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -16636,7 +16564,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/26/2026 20:42</t>
+          <t>08/31/2026 22:33</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16659,7 +16587,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>08/25/2026 08:19</t>
+          <t>08/31/2026 08:23</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -16682,11 +16610,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>08/26/2026 23:23</t>
+          <t>09/01/2026 00:13</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20136.42</v>
+        <v>20364.32</v>
       </c>
     </row>
     <row r="24">
@@ -16728,7 +16656,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/27/2026 00:15</t>
+          <t>08/31/2026 21:46</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -16751,11 +16679,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08/26/2026 23:34</t>
+          <t>09/01/2026 00:24</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>21329.83</v>
+        <v>20987.56</v>
       </c>
     </row>
     <row r="27">
@@ -16774,7 +16702,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/26/2026 21:46</t>
+          <t>08/31/2026 23:01</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16797,7 +16725,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/26/2026 21:43</t>
+          <t>08/29/2026 16:27</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16820,7 +16748,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/26/2026 21:51</t>
+          <t>08/29/2026 16:27</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16843,7 +16771,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/26/2026 21:23</t>
+          <t>08/30/2026 22:45</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16866,7 +16794,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/26/2026 21:36</t>
+          <t>08/30/2026 22:52</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16889,7 +16817,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/26/2026 21:32</t>
+          <t>08/29/2026 16:16</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16912,7 +16840,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/26/2026 17:01</t>
+          <t>08/29/2026 17:03</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -16935,11 +16863,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>08/26/2026 23:34</t>
+          <t>09/01/2026 00:22</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>2999.64</v>
+        <v>10597.56</v>
       </c>
     </row>
     <row r="35">
@@ -16981,7 +16909,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/26/2026 23:00</t>
+          <t>08/31/2026 23:51</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -17004,7 +16932,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>08/26/2026 23:04</t>
+          <t>09/01/2026 00:01</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -17027,11 +16955,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/27/2026 00:34</t>
+          <t>08/31/2026 22:02</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>19800.9</v>
+        <v>20438.68</v>
       </c>
     </row>
     <row r="39">
@@ -17050,11 +16978,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>08/26/2026 23:21</t>
+          <t>09/01/2026 00:16</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>19979.35</v>
+        <v>20134.75</v>
       </c>
     </row>
     <row r="40">
@@ -17073,11 +17001,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>08/26/2026 23:29</t>
+          <t>09/01/2026 00:20</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>32372.74</v>
+        <v>41483.68</v>
       </c>
     </row>
     <row r="41">
@@ -17119,7 +17047,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>08/25/2026 07:16</t>
+          <t>08/31/2026 07:07</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -17142,7 +17070,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>08/25/2026 07:46</t>
+          <t>08/31/2026 07:48</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -17165,7 +17093,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>08/25/2026 10:51</t>
+          <t>08/31/2026 10:55</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
@@ -17188,7 +17116,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>08/26/2026 12:42</t>
+          <t>08/31/2026 13:04</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-02
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-08-31 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-02 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>08/31/2026 23:53</t>
+          <t>09/02/2026 23:07</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>56588.78</v>
+        <v>49148.85</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>158.67</v>
+        <v>124.65</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.09</v>
+        <v>1.07</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,34 +985,34 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>4312.130000000001</v>
+        <v>-6294.339999999998</v>
       </c>
       <c r="P2" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>77.5</v>
+        <v>72.5</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>1.115612560529206</v>
+        <v>0.8741457962387742</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>34.95</v>
+        <v>52.43</v>
       </c>
       <c r="T2" t="n">
-        <v>3364</v>
+        <v>3376</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>31588.77999999999</v>
+        <v>24148.84999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2131</v>
+        <v>2138</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.34720570749109</v>
+        <v>63.32938388625592</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="Y2" s="7" t="n">
         <v>80.69</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>08/29/2026 19:15</t>
+          <t>09/01/2026 19:23</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>08/30/2026 09:10</t>
+          <t>09/02/2026 09:11</t>
         </is>
       </c>
       <c r="H5" s="7" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>08/29/2026 17:07</t>
+          <t>09/01/2026 17:11</t>
         </is>
       </c>
       <c r="H8" s="7" t="n">
@@ -2159,14 +2159,14 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>08/31/2026 23:31</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>5105.06</v>
+          <t>09/01/2026 21:40</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>-2.84</v>
+        <v>-2.77</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>10.41</v>
@@ -2178,25 +2178,25 @@
         <v>20000</v>
       </c>
       <c r="M13" s="7" t="n">
-        <v>14933.5</v>
+        <v>20042.05</v>
       </c>
       <c r="N13" t="n">
         <v>40</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>-4917.41</v>
+        <v>-1544.79</v>
       </c>
       <c r="P13" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>75</v>
+        <v>77.5</v>
       </c>
       <c r="R13" s="7" t="n">
-        <v>0.6894156865791646</v>
+        <v>0.8760331971251842</v>
       </c>
       <c r="S13" s="7" t="n">
-        <v>99.09</v>
+        <v>56.48</v>
       </c>
       <c r="T13" t="n">
         <v>65</v>
@@ -2214,7 +2214,7 @@
         <v>1.04</v>
       </c>
       <c r="Y13" s="7" t="n">
-        <v>13.67</v>
+        <v>7.45</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>08/30/2026 10:23</t>
+          <t>09/02/2026 10:25</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>08/31/2026 22:49</t>
+          <t>09/02/2026 22:14</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>08/29/2026 22:00</t>
+          <t>09/01/2026 22:03</t>
         </is>
       </c>
       <c r="H17" s="7" t="n">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>08/30/2026 13:06</t>
+          <t>09/02/2026 13:08</t>
         </is>
       </c>
       <c r="H18" s="7" t="n">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>08/30/2026 05:52</t>
+          <t>09/02/2026 06:08</t>
         </is>
       </c>
       <c r="H19" s="7" t="n">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>08/30/2026 05:52</t>
+          <t>09/02/2026 06:07</t>
         </is>
       </c>
       <c r="H20" s="7" t="n">
@@ -3031,20 +3031,20 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>08/31/2026 22:32</t>
+          <t>09/02/2026 21:57</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
-        <v>15086.78</v>
+        <v>14814.83</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>-24.55</v>
+        <v>-25.92</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>37.21</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="L21" t="n">
         <v>20000</v>
@@ -3056,7 +3056,7 @@
         <v>40</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>-1651.52</v>
+        <v>-1897.99</v>
       </c>
       <c r="P21" t="n">
         <v>15</v>
@@ -3065,7 +3065,7 @@
         <v>37.5</v>
       </c>
       <c r="R21" s="7" t="n">
-        <v>0.538533327744946</v>
+        <v>0.5038349732832809</v>
       </c>
       <c r="S21" s="7" t="n">
         <v>12.31</v>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/01/2026 00:27</t>
+          <t>09/02/2026 20:44</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>08/31/2026 23:59</t>
+          <t>09/02/2026 20:16</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>19736.81</v>
+        <v>20216.06</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>-1.31</v>
+        <v>1.09</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.1</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>33.27</v>
+        <v>133.5899999999999</v>
       </c>
       <c r="P23" t="n">
         <v>21</v>
@@ -3283,25 +3283,25 @@
         <v>52.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.015014418715899</v>
+        <v>1.06096075129711</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.22</v>
+        <v>4.3</v>
       </c>
       <c r="T23" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>-263.1899999999999</v>
+        <v>216.0600000000001</v>
       </c>
       <c r="V23" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>53.08641975308642</v>
+        <v>54.11764705882353</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>6.11</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3398,22 +3398,22 @@
         <v>0.7</v>
       </c>
       <c r="T24" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>-195.13</v>
+        <v>-347.89</v>
       </c>
       <c r="V24" t="n">
         <v>14</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>31.81818181818182</v>
+        <v>29.16666666666667</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>0.5</v>
+        <v>0.36</v>
       </c>
       <c r="Y24" s="7" t="n">
-        <v>1.39</v>
+        <v>1.8</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>Bar Reversal MOL Bots | AUDUSD.pro, Bar Reversal MOL Bots | CHFJPY.pro, Bar Reversal MOL Bots | EURCAD.pro, Bar Reversal MOL Bots | EURJPY.pro, Bar Reversal MOL Bots | EURUSD.pro, Bar Reversal MOL Bots | GBPJPY.pro, Bar Reversal MOL Bots | GBPNZD.pro, Bar Reversal MOL Bots | USDCAD.pro</t>
+          <t>Bar Reversal MOL Bots | AUDUSD.pro, Bar Reversal MOL Bots | CADJPY.pro, Bar Reversal MOL Bots | CHFJPY.pro, Bar Reversal MOL Bots | EURCAD.pro, Bar Reversal MOL Bots | EURJPY.pro, Bar Reversal MOL Bots | EURUSD.pro, Bar Reversal MOL Bots | GBPJPY.pro, Bar Reversal MOL Bots | GBPNZD.pro, Bar Reversal MOL Bots | USDCAD.pro</t>
         </is>
       </c>
     </row>
@@ -3467,20 +3467,20 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>09/01/2026 00:12</t>
+          <t>09/02/2026 20:30</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
-        <v>16571.33</v>
+        <v>16421.59</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>-16.81</v>
+        <v>-17.57</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>20.92</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="L25" t="n">
         <v>20000</v>
@@ -3492,19 +3492,19 @@
         <v>40</v>
       </c>
       <c r="O25" s="7" t="n">
-        <v>104.52</v>
+        <v>-73.73999999999997</v>
       </c>
       <c r="P25" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="Q25" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="R25" s="7" t="n">
-        <v>1.258969276511397</v>
+        <v>0.8663622030120155</v>
       </c>
       <c r="S25" s="7" t="n">
-        <v>0.65</v>
+        <v>1.19</v>
       </c>
       <c r="T25" t="n">
         <v>703</v>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>08/30/2026 22:50</t>
+          <t>09/02/2026 22:49</t>
         </is>
       </c>
       <c r="H26" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/01/2026 00:04</t>
+          <t>09/02/2026 20:22</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>19460.25</v>
+        <v>19855.55</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-6.94</v>
+        <v>-5.05</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.74</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,19 +3710,19 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-912.1399999999999</v>
+        <v>-385.8299999999999</v>
       </c>
       <c r="P27" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="Q27" s="7" t="n">
-        <v>50</v>
+        <v>52.5</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.6286195889384711</v>
+        <v>0.8338443650144266</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>5.11</v>
+        <v>5.07</v>
       </c>
       <c r="T27" t="n">
         <v>110</v>
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>09/01/2026 00:09</t>
+          <t>09/02/2026 20:21</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19537.07</v>
+        <v>19432.85</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-2.33</v>
+        <v>-2.85</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,34 +3928,34 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-617.73</v>
+        <v>-660.73</v>
       </c>
       <c r="P29" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>37.5</v>
+        <v>32.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.3058823529411765</v>
+        <v>0.2728203209262398</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>3.15</v>
+        <v>3.3</v>
       </c>
       <c r="T29" t="n">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-462.9300000000001</v>
+        <v>-567.1500000000003</v>
       </c>
       <c r="V29" t="n">
         <v>60</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>46.51162790697674</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4121,20 +4121,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>09/01/2026 00:12</t>
+          <t>09/02/2026 20:29</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20681.21</v>
+        <v>20625.45</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>3.43</v>
+        <v>3.15</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="K31" t="n">
-        <v>2</v>
+        <v>1.29</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>1.85</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -4146,7 +4146,7 @@
         <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>-157.92</v>
+        <v>-192</v>
       </c>
       <c r="P31" t="n">
         <v>13</v>
@@ -4155,28 +4155,28 @@
         <v>32.5</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>0.7079503633976291</v>
+        <v>0.6659765835667438</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>1.14</v>
+        <v>1.39</v>
       </c>
       <c r="T31" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>681.2099999999998</v>
+        <v>625.4499999999998</v>
       </c>
       <c r="V31" t="n">
         <v>19</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>28.78787878787879</v>
+        <v>27.53623188405797</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>2</v>
+        <v>1.85</v>
       </c>
       <c r="Y31" s="7" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -4185,7 +4185,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>08/30/2026 10:26</t>
+          <t>09/02/2026 10:28</t>
         </is>
       </c>
       <c r="H32" s="7" t="n">
@@ -4339,7 +4339,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>08/30/2026 11:16</t>
+          <t>09/02/2026 11:18</t>
         </is>
       </c>
       <c r="H33" s="7" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>08/31/2026 22:40</t>
+          <t>09/02/2026 22:03</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4557,7 +4557,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>08/30/2026 00:21</t>
+          <t>09/02/2026 00:23</t>
         </is>
       </c>
       <c r="H35" s="7" t="n">
@@ -4666,20 +4666,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>08/31/2026 22:05</t>
+          <t>09/02/2026 21:32</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
-        <v>20284.45</v>
+        <v>20112.96</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>1.43</v>
+        <v>0.57</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>8.84</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>1.06</v>
+        <v>1.02</v>
       </c>
       <c r="L36" t="n">
         <v>20000</v>
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>284.4499999999999</v>
+        <v>112.9599999999998</v>
       </c>
       <c r="V36" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>51.51515151515152</v>
+        <v>50.48543689320388</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>1.06</v>
+        <v>1.02</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.83</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>08/31/2026 21:45</t>
+          <t>09/02/2026 21:10</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>08/29/2026 22:10</t>
+          <t>09/01/2026 22:12</t>
         </is>
       </c>
       <c r="H38" s="7" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>08/29/2026 14:33</t>
+          <t>09/01/2026 14:36</t>
         </is>
       </c>
       <c r="H39" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/01/2026 00:08</t>
+          <t>09/02/2026 20:22</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/01/2026 00:27</t>
+          <t>09/02/2026 20:42</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/01/2026 00:05</t>
+          <t>09/02/2026 20:20</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5620,20 +5620,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/01/2026 00:16</t>
+          <t>09/02/2026 20:32</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19794.87</v>
+        <v>19803.09</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-1.01</v>
+        <v>-0.96</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>4.38</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5651,19 +5651,19 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>477</v>
+        <v>496</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-205.1300000000001</v>
+        <v>-196.9100000000001</v>
       </c>
       <c r="V45" t="n">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>55.9748427672956</v>
+        <v>56.04838709677419</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Y45" s="7" t="n">
         <v>4.39</v>
@@ -5675,7 +5675,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5720,7 +5720,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/01/2026 00:08</t>
+          <t>09/02/2026 23:22</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
@@ -5820,20 +5820,20 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>09/01/2026 00:00</t>
+          <t>09/02/2026 23:27</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
-        <v>18812.85</v>
+        <v>19014.1</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>-5.91</v>
+        <v>-4.9</v>
       </c>
       <c r="J47" s="7" t="n">
         <v>7.43</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>0.61</v>
+        <v>0.67</v>
       </c>
       <c r="L47" t="n">
         <v>20000</v>
@@ -5851,19 +5851,19 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="U47" s="7" t="n">
-        <v>-1187.15</v>
+        <v>-985.9</v>
       </c>
       <c r="V47" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>38.57142857142858</v>
+        <v>40.27777777777778</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>0.61</v>
+        <v>0.67</v>
       </c>
       <c r="Y47" s="7" t="n">
         <v>7.43</v>
@@ -5875,7 +5875,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5920,7 +5920,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>08/31/2026 23:54</t>
+          <t>09/02/2026 23:18</t>
         </is>
       </c>
       <c r="H48" s="7" t="n">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/01/2026 00:20</t>
+          <t>09/02/2026 20:36</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>09/01/2026 00:13</t>
+          <t>09/02/2026 20:31</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/01/2026 00:00</t>
+          <t>09/02/2026 23:26</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6320,20 +6320,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>08/31/2026 23:54</t>
+          <t>09/02/2026 23:24</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
-        <v>20497.37</v>
+        <v>20608.97</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>2.5</v>
+        <v>3.06</v>
       </c>
       <c r="J52" s="7" t="n">
         <v>10.18</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>1.13</v>
+        <v>1.15</v>
       </c>
       <c r="L52" t="n">
         <v>20000</v>
@@ -6351,19 +6351,19 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="U52" s="7" t="n">
-        <v>497.3699999999997</v>
+        <v>608.9699999999996</v>
       </c>
       <c r="V52" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>30.23255813953488</v>
+        <v>31.91489361702128</v>
       </c>
       <c r="X52" s="7" t="n">
-        <v>1.13</v>
+        <v>1.15</v>
       </c>
       <c r="Y52" s="7" t="n">
         <v>10.19</v>
@@ -6375,7 +6375,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6420,20 +6420,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/01/2026 00:32</t>
+          <t>09/02/2026 20:43</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19697.63</v>
+        <v>19669.05</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>-1.54</v>
+        <v>-1.68</v>
       </c>
       <c r="J53" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="L53" t="n">
         <v>20000</v>
@@ -6451,19 +6451,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>313</v>
+        <v>323</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-302.3700000000001</v>
+        <v>-330.9500000000001</v>
       </c>
       <c r="V53" t="n">
         <v>110</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>35.14376996805112</v>
+        <v>34.05572755417957</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6520,7 +6520,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>09/01/2026 00:33</t>
+          <t>09/02/2026 20:50</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/01/2026 00:14</t>
+          <t>09/02/2026 20:32</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6720,7 +6720,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>09/01/2026 00:32</t>
+          <t>09/02/2026 20:55</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6820,20 +6820,20 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>08/31/2026 23:54</t>
+          <t>09/02/2026 23:25</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19708.39</v>
+        <v>19717.48</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.44</v>
+        <v>-1.39</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="L57" t="n">
         <v>20000</v>
@@ -6851,19 +6851,19 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>881</v>
+        <v>900</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-290.6500000000001</v>
+        <v>-281.86</v>
       </c>
       <c r="V57" t="n">
-        <v>387</v>
+        <v>398</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>43.92735527809307</v>
+        <v>44.22222222222222</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="Y57" s="7" t="n">
         <v>1.95</v>
@@ -6875,7 +6875,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/01/2026 00:11</t>
+          <t>09/02/2026 20:28</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -7020,7 +7020,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>09/01/2026 00:07</t>
+          <t>09/02/2026 20:23</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7120,14 +7120,14 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/01/2026 00:08</t>
+          <t>09/02/2026 20:22</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
-        <v>19931.35</v>
+        <v>19913.31</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>-6.3</v>
+        <v>-6.39</v>
       </c>
       <c r="J60" s="7" t="n">
         <v>19.42</v>
@@ -7220,7 +7220,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/01/2026 00:26</t>
+          <t>09/02/2026 20:45</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>08/30/2026 20:53</t>
+          <t>09/02/2026 20:57</t>
         </is>
       </c>
       <c r="H62" s="7" t="n">
@@ -7420,7 +7420,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>09/01/2026 00:20</t>
+          <t>09/02/2026 20:38</t>
         </is>
       </c>
       <c r="H63" s="7" t="n">
@@ -7520,20 +7520,20 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>09/01/2026 00:27</t>
+          <t>09/02/2026 20:44</t>
         </is>
       </c>
       <c r="H64" s="7" t="n">
-        <v>19414.44</v>
+        <v>19342.33</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>-2.92</v>
+        <v>-3.28</v>
       </c>
       <c r="J64" s="7" t="n">
         <v>3.87</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>0.72</v>
+        <v>0.7</v>
       </c>
       <c r="L64" t="n">
         <v>20000</v>
@@ -7620,14 +7620,14 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>09/01/2026 00:21</t>
+          <t>09/02/2026 20:39</t>
         </is>
       </c>
       <c r="H65" s="7" t="n">
-        <v>19301.2</v>
+        <v>19346.13</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>-3.54</v>
+        <v>-3.32</v>
       </c>
       <c r="J65" s="7" t="n">
         <v>11.64</v>
@@ -7720,14 +7720,14 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>09/01/2026 00:10</t>
+          <t>09/02/2026 20:27</t>
         </is>
       </c>
       <c r="H66" s="7" t="n">
-        <v>19976.23</v>
+        <v>19971.98</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>-0.11</v>
+        <v>-0.13</v>
       </c>
       <c r="J66" s="7" t="n">
         <v>2.86</v>
@@ -7820,7 +7820,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>08/31/2026 21:43</t>
+          <t>09/02/2026 21:08</t>
         </is>
       </c>
       <c r="H67" s="7" t="n">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>08/29/2026 21:52</t>
+          <t>09/01/2026 21:54</t>
         </is>
       </c>
       <c r="H68" s="7" t="n">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>08/29/2026 21:52</t>
+          <t>09/01/2026 21:54</t>
         </is>
       </c>
       <c r="H69" s="7" t="n">
@@ -8120,7 +8120,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>08/29/2026 21:52</t>
+          <t>09/01/2026 21:54</t>
         </is>
       </c>
       <c r="H70" s="7" t="n">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>09/01/2026 00:21</t>
+          <t>09/02/2026 20:32</t>
         </is>
       </c>
       <c r="H71" s="7" t="n">
@@ -8320,7 +8320,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>08/31/2026 21:50</t>
+          <t>09/02/2026 21:16</t>
         </is>
       </c>
       <c r="H72" s="7" t="n">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>09/01/2026 00:23</t>
+          <t>09/02/2026 20:36</t>
         </is>
       </c>
       <c r="H73" s="7" t="n">
@@ -8520,7 +8520,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>08/31/2026 21:55</t>
+          <t>09/02/2026 21:10</t>
         </is>
       </c>
       <c r="H74" s="7" t="n">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>09/01/2026 00:19</t>
+          <t>09/02/2026 20:28</t>
         </is>
       </c>
       <c r="H75" s="7" t="n">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>09/01/2026 00:34</t>
+          <t>09/02/2026 20:48</t>
         </is>
       </c>
       <c r="H76" s="7" t="n">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>09/01/2026 00:37</t>
+          <t>09/02/2026 20:39</t>
         </is>
       </c>
       <c r="H77" s="7" t="n">
@@ -8920,7 +8920,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>09/01/2026 00:34</t>
+          <t>09/02/2026 20:53</t>
         </is>
       </c>
       <c r="H78" s="7" t="n">
@@ -9020,7 +9020,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>09/01/2026 00:31</t>
+          <t>09/02/2026 20:48</t>
         </is>
       </c>
       <c r="H79" s="7" t="n">
@@ -9120,7 +9120,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09/01/2026 00:19</t>
+          <t>09/02/2026 20:26</t>
         </is>
       </c>
       <c r="H80" s="7" t="n">
@@ -9220,7 +9220,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>08/31/2026 21:44</t>
+          <t>09/02/2026 21:07</t>
         </is>
       </c>
       <c r="H81" s="7" t="n">
@@ -9320,7 +9320,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>09/01/2026 00:34</t>
+          <t>09/02/2026 20:48</t>
         </is>
       </c>
       <c r="H82" s="7" t="n">
@@ -9420,7 +9420,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>08/31/2026 21:53</t>
+          <t>09/02/2026 21:16</t>
         </is>
       </c>
       <c r="H83" s="7" t="n">
@@ -9520,7 +9520,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08/31/2026 22:20</t>
+          <t>09/02/2026 21:42</t>
         </is>
       </c>
       <c r="H84" s="7" t="n">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>08/31/2026 21:41</t>
+          <t>09/02/2026 21:05</t>
         </is>
       </c>
       <c r="H85" s="7" t="n">
@@ -9720,17 +9720,17 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>08/31/2026 21:45</t>
+          <t>09/02/2026 21:13</t>
         </is>
       </c>
       <c r="H86" s="7" t="n">
-        <v>20388.17</v>
+        <v>20381.8</v>
       </c>
       <c r="I86" s="7" t="n">
-        <v>1.95</v>
+        <v>1.91</v>
       </c>
       <c r="J86" s="7" t="n">
-        <v>2.51</v>
+        <v>2.55</v>
       </c>
       <c r="K86" s="7" t="n">
         <v>1.29</v>
@@ -9751,22 +9751,22 @@
         <v>0</v>
       </c>
       <c r="T86" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="U86" s="7" t="n">
-        <v>388.1700000000001</v>
+        <v>381.8000000000002</v>
       </c>
       <c r="V86" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="W86" s="7" t="n">
-        <v>46.53465346534654</v>
+        <v>45.71428571428572</v>
       </c>
       <c r="X86" s="7" t="n">
         <v>1.29</v>
       </c>
       <c r="Y86" s="7" t="n">
-        <v>2.51</v>
+        <v>2.54</v>
       </c>
       <c r="Z86" t="inlineStr">
         <is>
@@ -9775,7 +9775,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -9820,7 +9820,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>09/01/2026 00:25</t>
+          <t>09/02/2026 20:40</t>
         </is>
       </c>
       <c r="H87" s="7" t="n">
@@ -9920,20 +9920,20 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>08/31/2026 21:41</t>
+          <t>09/02/2026 21:02</t>
         </is>
       </c>
       <c r="H88" s="7" t="n">
-        <v>20177.38</v>
+        <v>20273.18</v>
       </c>
       <c r="I88" s="7" t="n">
-        <v>0.87</v>
+        <v>1.35</v>
       </c>
       <c r="J88" s="7" t="n">
         <v>2.69</v>
       </c>
       <c r="K88" s="7" t="n">
-        <v>1.19</v>
+        <v>1.29</v>
       </c>
       <c r="L88" t="n">
         <v>20000</v>
@@ -9951,19 +9951,19 @@
         <v>0</v>
       </c>
       <c r="T88" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="U88" s="7" t="n">
-        <v>177.38</v>
+        <v>273.18</v>
       </c>
       <c r="V88" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="W88" s="7" t="n">
-        <v>85.48387096774194</v>
+        <v>87.14285714285714</v>
       </c>
       <c r="X88" s="7" t="n">
-        <v>1.19</v>
+        <v>1.29</v>
       </c>
       <c r="Y88" s="7" t="n">
         <v>2.7</v>
@@ -9975,7 +9975,7 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
@@ -10020,20 +10020,20 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>08/31/2026 21:41</t>
+          <t>09/02/2026 21:03</t>
         </is>
       </c>
       <c r="H89" s="7" t="n">
-        <v>23570.7</v>
+        <v>23371.37</v>
       </c>
       <c r="I89" s="7" t="n">
-        <v>17.91</v>
+        <v>16.91</v>
       </c>
       <c r="J89" s="7" t="n">
         <v>3.08</v>
       </c>
       <c r="K89" s="7" t="n">
-        <v>2.28</v>
+        <v>1.98</v>
       </c>
       <c r="L89" t="n">
         <v>20000</v>
@@ -10051,19 +10051,19 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="U89" s="7" t="n">
-        <v>3570.7</v>
+        <v>3371.37</v>
       </c>
       <c r="V89" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="W89" s="7" t="n">
-        <v>72.72727272727273</v>
+        <v>69.84126984126983</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>2.28</v>
+        <v>1.98</v>
       </c>
       <c r="Y89" s="7" t="n">
         <v>3.08</v>
@@ -10075,7 +10075,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -10120,7 +10120,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>09/01/2026 00:01</t>
+          <t>09/02/2026 23:27</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09/01/2026 00:01</t>
+          <t>09/02/2026 20:15</t>
         </is>
       </c>
       <c r="H91" s="7" t="n">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>09/01/2026 00:03</t>
+          <t>09/02/2026 20:16</t>
         </is>
       </c>
       <c r="H92" s="7" t="n">
@@ -10420,7 +10420,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>08/31/2026 23:57</t>
+          <t>09/02/2026 23:25</t>
         </is>
       </c>
       <c r="H93" s="7" t="n">
@@ -10520,7 +10520,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>08/31/2026 23:57</t>
+          <t>09/02/2026 23:24</t>
         </is>
       </c>
       <c r="H94" s="7" t="n">
@@ -10620,7 +10620,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>08/31/2026 23:54</t>
+          <t>09/02/2026 23:22</t>
         </is>
       </c>
       <c r="H95" s="7" t="n">
@@ -10720,7 +10720,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>09/01/2026 00:00</t>
+          <t>09/02/2026 23:24</t>
         </is>
       </c>
       <c r="H96" s="7" t="n">
@@ -10820,7 +10820,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>09/01/2026 00:09</t>
+          <t>09/02/2026 20:22</t>
         </is>
       </c>
       <c r="H97" s="7" t="n">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>08/31/2026 23:51</t>
+          <t>09/02/2026 23:17</t>
         </is>
       </c>
       <c r="H98" s="7" t="n">
@@ -11020,7 +11020,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>09/01/2026 00:01</t>
+          <t>09/02/2026 20:18</t>
         </is>
       </c>
       <c r="H99" s="7" t="n">
@@ -11120,7 +11120,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>09/01/2026 00:29</t>
+          <t>09/02/2026 20:44</t>
         </is>
       </c>
       <c r="H100" s="7" t="n">
@@ -11160,22 +11160,22 @@
         <v>8.26</v>
       </c>
       <c r="T100" t="n">
-        <v>631</v>
+        <v>640</v>
       </c>
       <c r="U100" s="7" t="n">
-        <v>-20600.09</v>
+        <v>-20642.16</v>
       </c>
       <c r="V100" t="n">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="W100" s="7" t="n">
-        <v>41.67987321711568</v>
+        <v>41.875</v>
       </c>
       <c r="X100" s="7" t="n">
         <v>0.82</v>
       </c>
       <c r="Y100" s="7" t="n">
-        <v>99.06999999999999</v>
+        <v>99.23999999999999</v>
       </c>
       <c r="Z100" t="inlineStr">
         <is>
@@ -11184,7 +11184,7 @@
       </c>
       <c r="AA100" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB100" t="inlineStr">
@@ -11229,11 +11229,11 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>08/29/2026 21:03</t>
-        </is>
-      </c>
-      <c r="H101" s="7" t="n">
-        <v>25956.55</v>
+          <t>09/01/2026 21:06</t>
+        </is>
+      </c>
+      <c r="H101" t="n">
+        <v>0</v>
       </c>
       <c r="I101" s="7" t="n">
         <v>0.02</v>
@@ -11247,14 +11247,14 @@
       <c r="L101" t="n">
         <v>30000</v>
       </c>
-      <c r="M101" t="n">
-        <v>4000</v>
+      <c r="M101" s="7" t="n">
+        <v>29956.55</v>
       </c>
       <c r="N101" t="n">
         <v>40</v>
       </c>
       <c r="O101" s="7" t="n">
-        <v>16192.62</v>
+        <v>-9691.929999999998</v>
       </c>
       <c r="P101" t="n">
         <v>17</v>
@@ -11263,10 +11263,10 @@
         <v>42.5</v>
       </c>
       <c r="R101" s="7" t="n">
-        <v>4.221713101038779</v>
+        <v>0.6864532730477272</v>
       </c>
       <c r="S101" s="7" t="n">
-        <v>9.640000000000001</v>
+        <v>158.14</v>
       </c>
       <c r="T101" t="n">
         <v>61</v>
@@ -11284,7 +11284,7 @@
         <v>0.98</v>
       </c>
       <c r="Y101" s="7" t="n">
-        <v>2.56</v>
+        <v>233.96</v>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
@@ -11447,20 +11447,20 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>08/31/2026 23:30</t>
+          <t>09/02/2026 22:59</t>
         </is>
       </c>
       <c r="H103" s="7" t="n">
-        <v>28245.15</v>
+        <v>27727.62</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>-26.44</v>
+        <v>-27.8</v>
       </c>
       <c r="J103" s="7" t="n">
         <v>37.71</v>
       </c>
       <c r="K103" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L103" t="n">
         <v>25000</v>
@@ -11472,34 +11472,34 @@
         <v>40</v>
       </c>
       <c r="O103" s="7" t="n">
-        <v>203.53</v>
+        <v>-559.39</v>
       </c>
       <c r="P103" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="Q103" s="7" t="n">
-        <v>90</v>
+        <v>55.00000000000001</v>
       </c>
       <c r="R103" s="7" t="n">
-        <v>3.769115646258503</v>
+        <v>0.2095550311577103</v>
       </c>
       <c r="S103" s="7" t="n">
-        <v>0.29</v>
+        <v>2.71</v>
       </c>
       <c r="T103" t="n">
-        <v>3602</v>
+        <v>3632</v>
       </c>
       <c r="U103" s="7" t="n">
-        <v>-6036.85</v>
+        <v>-6554.379999999999</v>
       </c>
       <c r="V103" t="n">
-        <v>2207</v>
+        <v>2240</v>
       </c>
       <c r="W103" s="7" t="n">
-        <v>61.27151582454192</v>
+        <v>61.67400881057269</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>0.82</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y103" s="7" t="n">
         <v>37.71</v>
@@ -11511,7 +11511,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -11647,7 +11647,7 @@
       </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t>08/29/2026 19:33</t>
+          <t>09/01/2026 19:40</t>
         </is>
       </c>
       <c r="H105" s="9" t="n">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>08/30/2026 16:33</t>
+          <t>09/02/2026 16:43</t>
         </is>
       </c>
       <c r="H106" s="9" t="n">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t>08/29/2026 12:49</t>
+          <t>09/01/2026 12:51</t>
         </is>
       </c>
       <c r="H110" s="9" t="n">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t>08/29/2026 16:48</t>
+          <t>09/01/2026 16:51</t>
         </is>
       </c>
       <c r="H112" s="9" t="n">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t>09/01/2026 00:30</t>
+          <t>09/02/2026 20:42</t>
         </is>
       </c>
       <c r="H113" s="9" t="n">
@@ -12466,7 +12466,7 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t>09/01/2026 00:05</t>
+          <t>09/02/2026 20:17</t>
         </is>
       </c>
       <c r="H114" s="9" t="n">
@@ -12551,7 +12551,7 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>08/30/2026 20:39</t>
+          <t>09/02/2026 20:41</t>
         </is>
       </c>
       <c r="H115" s="9" t="n">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t>08/30/2026 15:00</t>
+          <t>09/02/2026 15:02</t>
         </is>
       </c>
       <c r="H116" s="9" t="n">
@@ -12721,7 +12721,7 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t>08/29/2026 21:52</t>
+          <t>09/01/2026 21:55</t>
         </is>
       </c>
       <c r="H117" s="9" t="n">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t>09/01/2026 00:01</t>
+          <t>09/02/2026 20:16</t>
         </is>
       </c>
       <c r="H118" s="9" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t>09/01/2026 00:02</t>
+          <t>09/02/2026 20:19</t>
         </is>
       </c>
       <c r="H119" s="9" t="n">
@@ -12976,7 +12976,7 @@
       </c>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t>09/01/2026 00:01</t>
+          <t>09/02/2026 20:18</t>
         </is>
       </c>
       <c r="H120" s="9" t="n">
@@ -13061,7 +13061,7 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>09/01/2026 00:03</t>
+          <t>09/02/2026 20:18</t>
         </is>
       </c>
       <c r="H121" s="9" t="n">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t>09/01/2026 00:14</t>
+          <t>09/02/2026 20:24</t>
         </is>
       </c>
       <c r="H122" s="9" t="n">
@@ -13231,7 +13231,7 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>09/01/2026 00:21</t>
+          <t>09/02/2026 20:19</t>
         </is>
       </c>
       <c r="H123" s="9" t="n">
@@ -13805,7 +13805,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>08/29/2026 19:33</t>
+          <t>09/01/2026 19:40</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -13846,7 +13846,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08/30/2026 16:33</t>
+          <t>09/02/2026 16:43</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
@@ -14010,7 +14010,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08/29/2026 12:49</t>
+          <t>09/01/2026 12:51</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
@@ -14092,7 +14092,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>08/29/2026 16:48</t>
+          <t>09/01/2026 16:51</t>
         </is>
       </c>
       <c r="G13" s="7" t="n">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>09/01/2026 00:30</t>
+          <t>09/02/2026 20:42</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -14174,7 +14174,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>09/01/2026 00:05</t>
+          <t>09/02/2026 20:17</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -14215,7 +14215,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>08/30/2026 20:39</t>
+          <t>09/02/2026 20:41</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
@@ -14256,7 +14256,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>08/30/2026 15:00</t>
+          <t>09/02/2026 15:02</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
@@ -14297,7 +14297,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>08/29/2026 21:52</t>
+          <t>09/01/2026 21:55</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -14338,7 +14338,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>09/01/2026 00:01</t>
+          <t>09/02/2026 20:16</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
@@ -14379,7 +14379,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>09/01/2026 00:02</t>
+          <t>09/02/2026 20:19</t>
         </is>
       </c>
       <c r="G20" s="7" t="n">
@@ -14420,7 +14420,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>09/01/2026 00:01</t>
+          <t>09/02/2026 20:18</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
@@ -14461,7 +14461,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>09/01/2026 00:03</t>
+          <t>09/02/2026 20:18</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
@@ -14502,7 +14502,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>09/01/2026 00:14</t>
+          <t>09/02/2026 20:24</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
@@ -14543,7 +14543,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>09/01/2026 00:21</t>
+          <t>09/02/2026 20:19</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
@@ -16196,7 +16196,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>08/29/2026 12:56</t>
+          <t>09/01/2026 13:11</t>
         </is>
       </c>
       <c r="E5" s="7" t="n">
@@ -16265,7 +16265,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>08/29/2026 21:16</t>
+          <t>09/01/2026 21:18</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -16357,7 +16357,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>08/29/2026 15:27</t>
+          <t>09/01/2026 15:28</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
@@ -16403,7 +16403,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>08/29/2026 17:24</t>
+          <t>09/01/2026 17:27</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -16472,7 +16472,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>08/29/2026 21:24</t>
+          <t>09/01/2026 21:26</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -16495,7 +16495,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>08/29/2026 21:15</t>
+          <t>09/01/2026 21:16</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -16564,7 +16564,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>08/31/2026 22:33</t>
+          <t>09/02/2026 21:52</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
@@ -16610,11 +16610,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>09/01/2026 00:13</t>
+          <t>09/02/2026 20:29</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>20364.32</v>
+        <v>20194.74</v>
       </c>
     </row>
     <row r="24">
@@ -16656,7 +16656,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08/31/2026 21:46</t>
+          <t>09/02/2026 21:11</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
@@ -16679,11 +16679,11 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09/01/2026 00:24</t>
+          <t>09/02/2026 20:42</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>20987.56</v>
+        <v>20643.75</v>
       </c>
     </row>
     <row r="27">
@@ -16702,7 +16702,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08/31/2026 23:01</t>
+          <t>09/02/2026 22:28</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
@@ -16725,7 +16725,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>08/29/2026 16:27</t>
+          <t>09/01/2026 16:29</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -16748,7 +16748,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>08/29/2026 16:27</t>
+          <t>09/01/2026 16:30</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
@@ -16771,7 +16771,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>08/30/2026 22:45</t>
+          <t>09/02/2026 22:47</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
@@ -16794,7 +16794,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>08/30/2026 22:52</t>
+          <t>09/02/2026 22:54</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -16817,7 +16817,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>08/29/2026 16:16</t>
+          <t>09/01/2026 16:18</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -16840,7 +16840,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>08/29/2026 17:03</t>
+          <t>09/01/2026 17:06</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -16863,11 +16863,11 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>09/01/2026 00:22</t>
+          <t>09/02/2026 20:39</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>10597.56</v>
+        <v>17819.36</v>
       </c>
     </row>
     <row r="35">
@@ -16909,7 +16909,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>08/31/2026 23:51</t>
+          <t>09/02/2026 23:21</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -16932,7 +16932,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>09/01/2026 00:01</t>
+          <t>09/02/2026 23:27</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -16955,11 +16955,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>08/31/2026 22:02</t>
+          <t>09/02/2026 21:30</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>20438.68</v>
+        <v>20071.24</v>
       </c>
     </row>
     <row r="39">
@@ -16978,11 +16978,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>09/01/2026 00:16</t>
+          <t>09/02/2026 20:29</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>20134.75</v>
+        <v>19989.47</v>
       </c>
     </row>
     <row r="40">
@@ -17001,11 +17001,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>09/01/2026 00:20</t>
+          <t>09/02/2026 20:35</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>41483.68</v>
+        <v>48809.71</v>
       </c>
     </row>
     <row r="41">
@@ -17116,7 +17116,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>08/31/2026 13:04</t>
+          <t>09/01/2026 13:05</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">

</xml_diff>

<commit_message>
Update dashboards — 2026-09-03
</commit_message>
<xml_diff>
--- a/MFB_Bachelier_Reconciliation_latest.xlsx
+++ b/MFB_Bachelier_Reconciliation_latest.xlsx
@@ -500,7 +500,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot: 2026-09-02 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
+          <t>Snapshot: 2026-09-03 • Data pulled live from MyFXBook API + ~/bachelier_data/consolidated/all_trades.parquet</t>
         </is>
       </c>
     </row>
@@ -960,20 +960,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>09/02/2026 23:07</t>
+          <t>09/03/2026 13:27</t>
         </is>
       </c>
       <c r="H2" s="7" t="n">
-        <v>49148.85</v>
+        <v>54618.68</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>124.65</v>
+        <v>149.66</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>80.69</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="L2" t="n">
         <v>25000</v>
@@ -985,31 +985,31 @@
         <v>40</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>-6294.339999999998</v>
+        <v>32.09000000000111</v>
       </c>
       <c r="P2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q2" s="7" t="n">
-        <v>72.5</v>
+        <v>75</v>
       </c>
       <c r="R2" s="7" t="n">
-        <v>0.8741457962387742</v>
+        <v>1.000749155828148</v>
       </c>
       <c r="S2" s="7" t="n">
-        <v>52.43</v>
+        <v>50.25</v>
       </c>
       <c r="T2" t="n">
-        <v>3376</v>
+        <v>3385</v>
       </c>
       <c r="U2" s="7" t="n">
-        <v>24148.84999999999</v>
+        <v>25846.72999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>2138</v>
+        <v>2145</v>
       </c>
       <c r="W2" s="7" t="n">
-        <v>63.32938388625592</v>
+        <v>63.36779911373708</v>
       </c>
       <c r="X2" s="7" t="n">
         <v>1.05</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>08/31/2026 04:12</t>
+          <t>09/03/2026 04:17</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1545,22 +1545,22 @@
         <v>1.26</v>
       </c>
       <c r="T7" t="n">
-        <v>1007</v>
+        <v>477</v>
       </c>
       <c r="U7" s="7" t="n">
-        <v>-16616.73</v>
+        <v>-3430.57</v>
       </c>
       <c r="V7" t="n">
-        <v>650</v>
+        <v>398</v>
       </c>
       <c r="W7" s="7" t="n">
-        <v>64.54816285998014</v>
+        <v>83.43815513626835</v>
       </c>
       <c r="X7" s="7" t="n">
-        <v>0.57</v>
+        <v>0.66</v>
       </c>
       <c r="Y7" s="7" t="n">
-        <v>54.53</v>
+        <v>12.06</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>T&amp;D Low Drawdown | AUDUSD.pro, T&amp;D Low Drawdown | BTCUSD, T&amp;D Low Drawdown | EURUSD.pro, T&amp;D Low Drawdown | GBPUSD.pro, T&amp;D Low Drawdown | NZDUSD.pro, T&amp;D Low Drawdown | USDCAD.pro, T&amp;D Low Drawdown | USDJPY.pro, T&amp;D Low Drawdown | XAUAUD, T&amp;D Low Drawdown | XAUUSD, T&amp;D60 | AUDUSD.pro, T&amp;D60 | EURUSD.pro, T&amp;D60 | GBPUSD.pro, T&amp;D60 | NZDUSD.pro, T&amp;D60 | USDJPY.pro</t>
+          <t>T&amp;D Low Drawdown | AUDUSD.pro, T&amp;D Low Drawdown | EURUSD.pro, T&amp;D Low Drawdown | GBPUSD.pro, T&amp;D Low Drawdown | NZDUSD.pro, T&amp;D Low Drawdown | USDCAD.pro, T&amp;D Low Drawdown | USDJPY.pro</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>08/31/2026 08:53</t>
+          <t>09/03/2026 08:55</t>
         </is>
       </c>
       <c r="H9" s="7" t="n">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>08/31/2026 10:37</t>
+          <t>09/03/2026 10:38</t>
         </is>
       </c>
       <c r="H10" s="7" t="n">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>08/31/2026 10:40</t>
+          <t>09/03/2026 10:41</t>
         </is>
       </c>
       <c r="H12" s="7" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>08/31/2026 04:40</t>
+          <t>09/03/2026 04:41</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>09/02/2026 22:14</t>
+          <t>09/03/2026 12:23</t>
         </is>
       </c>
       <c r="H16" s="7" t="n">
@@ -3031,7 +3031,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>09/02/2026 21:57</t>
+          <t>09/03/2026 11:56</t>
         </is>
       </c>
       <c r="H21" s="7" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>09/02/2026 20:44</t>
+          <t>09/03/2026 09:46</t>
         </is>
       </c>
       <c r="H22" s="7" t="n">
@@ -3249,20 +3249,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>09/02/2026 20:16</t>
+          <t>09/03/2026 08:55</t>
         </is>
       </c>
       <c r="H23" s="7" t="n">
-        <v>20216.06</v>
+        <v>20110.16</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>1.09</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>6.1</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>1.05</v>
+        <v>1.02</v>
       </c>
       <c r="L23" t="n">
         <v>20000</v>
@@ -3274,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>133.5899999999999</v>
+        <v>131.9999999999999</v>
       </c>
       <c r="P23" t="n">
         <v>21</v>
@@ -3283,25 +3283,25 @@
         <v>52.5</v>
       </c>
       <c r="R23" s="7" t="n">
-        <v>1.06096075129711</v>
+        <v>1.060191518467852</v>
       </c>
       <c r="S23" s="7" t="n">
-        <v>4.3</v>
+        <v>4.28</v>
       </c>
       <c r="T23" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>216.0600000000001</v>
+        <v>-104.1899999999999</v>
       </c>
       <c r="V23" t="n">
         <v>46</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>54.11764705882353</v>
+        <v>51.68539325842697</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>1.05</v>
+        <v>0.98</v>
       </c>
       <c r="Y23" s="7" t="n">
         <v>6.11</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3358,20 +3358,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>08/31/2026 04:34</t>
+          <t>09/03/2026 10:10</t>
         </is>
       </c>
       <c r="H24" s="7" t="n">
-        <v>19804.87</v>
+        <v>19624.27</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>-1.16</v>
+        <v>-2.06</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>1.41</v>
+        <v>2.12</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>0.41</v>
+        <v>0.28</v>
       </c>
       <c r="L24" t="n">
         <v>20000</v>
@@ -3383,37 +3383,37 @@
         <v>40</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>19764.42</v>
+        <v>-400.97</v>
       </c>
       <c r="P24" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="Q24" s="7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="R24" s="7" t="n">
-        <v>50.65435634609587</v>
+        <v>0.2833294607589055</v>
       </c>
       <c r="S24" s="7" t="n">
-        <v>0.7</v>
+        <v>2.11</v>
       </c>
       <c r="T24" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U24" s="7" t="n">
-        <v>-347.89</v>
+        <v>-375.73</v>
       </c>
       <c r="V24" t="n">
         <v>14</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>29.16666666666667</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="Y24" s="7" t="n">
-        <v>1.8</v>
+        <v>1.94</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>09/02/2026 20:30</t>
+          <t>09/03/2026 09:23</t>
         </is>
       </c>
       <c r="H25" s="7" t="n">
@@ -3685,20 +3685,20 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>09/02/2026 20:22</t>
+          <t>09/03/2026 09:00</t>
         </is>
       </c>
       <c r="H27" s="7" t="n">
-        <v>19855.55</v>
+        <v>20618.97</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>-5.05</v>
+        <v>-1.4</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>8.99</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L27" t="n">
         <v>20000</v>
@@ -3710,7 +3710,7 @@
         <v>40</v>
       </c>
       <c r="O27" s="7" t="n">
-        <v>-385.8299999999999</v>
+        <v>321.57</v>
       </c>
       <c r="P27" t="n">
         <v>21</v>
@@ -3719,10 +3719,10 @@
         <v>52.5</v>
       </c>
       <c r="R27" s="7" t="n">
-        <v>0.8338443650144266</v>
+        <v>1.138482408165023</v>
       </c>
       <c r="S27" s="7" t="n">
-        <v>5.07</v>
+        <v>5.08</v>
       </c>
       <c r="T27" t="n">
         <v>110</v>
@@ -3903,20 +3903,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>09/02/2026 20:21</t>
+          <t>09/03/2026 09:02</t>
         </is>
       </c>
       <c r="H29" s="7" t="n">
-        <v>19432.85</v>
+        <v>19364.34</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>-2.85</v>
+        <v>-3.2</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>7.56</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="L29" t="n">
         <v>20000</v>
@@ -3928,34 +3928,34 @@
         <v>40</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>-660.73</v>
+        <v>-597.28</v>
       </c>
       <c r="P29" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Q29" s="7" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>0.2728203209262398</v>
+        <v>0.3055852671720226</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="T29" t="n">
         <v>140</v>
       </c>
       <c r="U29" s="7" t="n">
-        <v>-567.1500000000003</v>
+        <v>-635.6600000000002</v>
       </c>
       <c r="V29" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="W29" s="7" t="n">
-        <v>42.85714285714285</v>
+        <v>43.57142857142857</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="Y29" s="7" t="n">
         <v>7.56</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4121,20 +4121,20 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>09/02/2026 20:29</t>
+          <t>09/03/2026 09:21</t>
         </is>
       </c>
       <c r="H31" s="7" t="n">
-        <v>20625.45</v>
+        <v>20609.32</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>3.15</v>
+        <v>3.07</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>1.29</v>
+        <v>1.36</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>1.85</v>
+        <v>1.81</v>
       </c>
       <c r="L31" t="n">
         <v>20000</v>
@@ -4146,37 +4146,37 @@
         <v>40</v>
       </c>
       <c r="O31" s="7" t="n">
-        <v>-192</v>
+        <v>-238.14</v>
       </c>
       <c r="P31" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Q31" s="7" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="R31" s="7" t="n">
-        <v>0.6659765835667438</v>
+        <v>0.59033201445037</v>
       </c>
       <c r="S31" s="7" t="n">
-        <v>1.39</v>
+        <v>1.47</v>
       </c>
       <c r="T31" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="U31" s="7" t="n">
-        <v>625.4499999999998</v>
+        <v>609.3199999999998</v>
       </c>
       <c r="V31" t="n">
         <v>19</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>27.53623188405797</v>
+        <v>26.76056338028169</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>1.85</v>
+        <v>1.81</v>
       </c>
       <c r="Y31" s="7" t="n">
-        <v>1.3</v>
+        <v>1.37</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -4185,7 +4185,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>09/02/2026 22:03</t>
+          <t>09/03/2026 12:07</t>
         </is>
       </c>
       <c r="H34" s="7" t="n">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>09/02/2026 21:32</t>
+          <t>09/03/2026 11:03</t>
         </is>
       </c>
       <c r="H36" s="7" t="n">
@@ -4697,19 +4697,19 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="U36" s="7" t="n">
-        <v>112.9599999999998</v>
+        <v>13.29999999999995</v>
       </c>
       <c r="V36" t="n">
         <v>52</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>50.48543689320388</v>
+        <v>50</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="Y36" s="7" t="n">
         <v>8.83</v>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>09/02/2026 21:10</t>
+          <t>09/03/2026 10:23</t>
         </is>
       </c>
       <c r="H37" s="7" t="n">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>09/02/2026 20:22</t>
+          <t>09/03/2026 09:04</t>
         </is>
       </c>
       <c r="H42" s="7" t="n">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>09/02/2026 20:42</t>
+          <t>09/03/2026 09:44</t>
         </is>
       </c>
       <c r="H43" s="7" t="n">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>09/02/2026 20:20</t>
+          <t>09/03/2026 02:43</t>
         </is>
       </c>
       <c r="H44" s="7" t="n">
@@ -5620,20 +5620,20 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>09/02/2026 20:32</t>
+          <t>09/03/2026 09:28</t>
         </is>
       </c>
       <c r="H45" s="7" t="n">
-        <v>19803.09</v>
+        <v>19685.5</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>-0.96</v>
+        <v>-1.54</v>
       </c>
       <c r="J45" s="7" t="n">
         <v>4.38</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="L45" t="n">
         <v>20000</v>
@@ -5651,19 +5651,19 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>496</v>
+        <v>526</v>
       </c>
       <c r="U45" s="7" t="n">
-        <v>-196.9100000000001</v>
+        <v>-235.97</v>
       </c>
       <c r="V45" t="n">
-        <v>278</v>
+        <v>297</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>56.04838709677419</v>
+        <v>56.46387832699619</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="Y45" s="7" t="n">
         <v>4.39</v>
@@ -5675,7 +5675,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5720,20 +5720,20 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>09/02/2026 23:22</t>
+          <t>09/03/2026 08:39</t>
         </is>
       </c>
       <c r="H46" s="7" t="n">
-        <v>19982.25</v>
+        <v>19971.45</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>-0.08</v>
+        <v>-0.13</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>0.74</v>
+        <v>0.64</v>
       </c>
       <c r="L46" t="n">
         <v>20000</v>
@@ -5751,22 +5751,22 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="U46" s="7" t="n">
-        <v>-17.75</v>
+        <v>-28.55000000000001</v>
       </c>
       <c r="V46" t="n">
         <v>13</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>30.95238095238095</v>
+        <v>28.88888888888889</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>0.74</v>
+        <v>0.64</v>
       </c>
       <c r="Y46" s="7" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>09/02/2026 23:27</t>
+          <t>09/03/2026 08:52</t>
         </is>
       </c>
       <c r="H47" s="7" t="n">
@@ -5842,13 +5842,22 @@
         <v>0</v>
       </c>
       <c r="N47" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>0</v>
+        <v>118.1899999999999</v>
       </c>
       <c r="P47" t="n">
-        <v>0</v>
+        <v>20</v>
+      </c>
+      <c r="Q47" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="R47" s="7" t="n">
+        <v>1.083207197820378</v>
+      </c>
+      <c r="S47" s="7" t="n">
+        <v>2.38</v>
       </c>
       <c r="T47" t="n">
         <v>72</v>
@@ -6020,7 +6029,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>09/02/2026 20:36</t>
+          <t>09/03/2026 09:31</t>
         </is>
       </c>
       <c r="H49" s="7" t="n">
@@ -6120,7 +6129,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>09/02/2026 20:31</t>
+          <t>09/03/2026 09:27</t>
         </is>
       </c>
       <c r="H50" s="7" t="n">
@@ -6220,7 +6229,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>09/02/2026 23:26</t>
+          <t>09/03/2026 08:51</t>
         </is>
       </c>
       <c r="H51" s="7" t="n">
@@ -6320,7 +6329,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>09/02/2026 23:24</t>
+          <t>09/03/2026 08:44</t>
         </is>
       </c>
       <c r="H52" s="7" t="n">
@@ -6342,16 +6351,25 @@
         <v>0</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>0</v>
+        <v>558.41</v>
       </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="Q52" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="R52" s="7" t="n">
+        <v>1.157700617066042</v>
+      </c>
+      <c r="S52" s="7" t="n">
+        <v>10.16</v>
       </c>
       <c r="T52" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="U52" s="7" t="n">
         <v>608.9699999999996</v>
@@ -6360,7 +6378,7 @@
         <v>15</v>
       </c>
       <c r="W52" s="7" t="n">
-        <v>31.91489361702128</v>
+        <v>31.25</v>
       </c>
       <c r="X52" s="7" t="n">
         <v>1.15</v>
@@ -6375,7 +6393,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6420,11 +6438,11 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>09/02/2026 20:43</t>
+          <t>09/03/2026 09:41</t>
         </is>
       </c>
       <c r="H53" s="7" t="n">
-        <v>19669.05</v>
+        <v>19668.81</v>
       </c>
       <c r="I53" s="7" t="n">
         <v>-1.68</v>
@@ -6451,19 +6469,19 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="U53" s="7" t="n">
-        <v>-330.9500000000001</v>
+        <v>-170.0200000000001</v>
       </c>
       <c r="V53" t="n">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="W53" s="7" t="n">
-        <v>34.05572755417957</v>
+        <v>34.95440729483283</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>0.71</v>
+        <v>0.85</v>
       </c>
       <c r="Y53" s="7" t="n">
         <v>1.89</v>
@@ -6475,7 +6493,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6520,7 +6538,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>09/02/2026 20:50</t>
+          <t>09/03/2026 09:55</t>
         </is>
       </c>
       <c r="H54" s="7" t="n">
@@ -6542,13 +6560,22 @@
         <v>0</v>
       </c>
       <c r="N54" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>0</v>
+        <v>-149.77</v>
       </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="Q54" s="7" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="R54" s="7" t="n">
+        <v>0.4112351599968551</v>
+      </c>
+      <c r="S54" s="7" t="n">
+        <v>0.83</v>
       </c>
       <c r="T54" t="n">
         <v>229</v>
@@ -6620,7 +6647,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>09/02/2026 20:32</t>
+          <t>09/03/2026 09:26</t>
         </is>
       </c>
       <c r="H55" s="7" t="n">
@@ -6720,7 +6747,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>09/02/2026 20:55</t>
+          <t>09/03/2026 09:58</t>
         </is>
       </c>
       <c r="H56" s="7" t="n">
@@ -6820,14 +6847,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>09/02/2026 23:25</t>
+          <t>09/03/2026 08:48</t>
         </is>
       </c>
       <c r="H57" s="7" t="n">
-        <v>19717.48</v>
+        <v>19722.29</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>-1.39</v>
+        <v>-1.37</v>
       </c>
       <c r="J57" s="7" t="n">
         <v>1.95</v>
@@ -6851,16 +6878,16 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>900</v>
+        <v>906</v>
       </c>
       <c r="U57" s="7" t="n">
-        <v>-281.86</v>
+        <v>-280</v>
       </c>
       <c r="V57" t="n">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>44.22222222222222</v>
+        <v>44.15011037527594</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>0.8</v>
@@ -6875,7 +6902,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6920,7 +6947,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>09/02/2026 20:28</t>
+          <t>09/03/2026 09:19</t>
         </is>
       </c>
       <c r="H58" s="7" t="n">
@@ -6942,13 +6969,22 @@
         <v>0</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O58" s="7" t="n">
-        <v>0</v>
+        <v>-83.65000000000001</v>
       </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="Q58" s="7" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="R58" s="7" t="n">
+        <v>0.3526042875938395</v>
+      </c>
+      <c r="S58" s="7" t="n">
+        <v>0.46</v>
       </c>
       <c r="T58" t="n">
         <v>4426</v>
@@ -7020,7 +7056,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>09/02/2026 20:23</t>
+          <t>09/03/2026 09:08</t>
         </is>
       </c>
       <c r="H59" s="7" t="n">
@@ -7042,13 +7078,22 @@
         <v>0</v>
       </c>
       <c r="N59" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>0</v>
+        <v>-80.78999999999999</v>
       </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="Q59" s="7" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="R59" s="7" t="n">
+        <v>0.32387647501883</v>
+      </c>
+      <c r="S59" s="7" t="n">
+        <v>0.43</v>
       </c>
       <c r="T59" t="n">
         <v>304</v>
@@ -7120,7 +7165,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>09/02/2026 20:22</t>
+          <t>09/03/2026 09:04</t>
         </is>
       </c>
       <c r="H60" s="7" t="n">
@@ -7220,7 +7265,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>09/02/2026 20:45</t>
+          <t>09/03/2026 09:45</t>
         </is>
       </c>
       <c r="H61" s="7" t="n">
@@ -7342,13 +7387,22 @@
         <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O62" s="7" t="n">
-        <v>0</v>
+        <v>-353.59</v>
       </c>
       <c r="P62" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="Q62" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="R62" s="7" t="n">
+        <v>0.3361931402181462</v>
+      </c>
+      <c r="S62" s="7" t="n">
+        <v>2.17</v>
       </c>
       <c r="T62" t="n">
         <v>170</v>
@@ -7420,7 +7474,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <